<commit_message>
Daily price update — 2026-06-21
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF67"/>
+  <dimension ref="A1:AF103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -5834,6 +5834,2836 @@
         <v>1</v>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D68" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E68" s="4" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="F68" s="4" t="n"/>
+      <c r="G68" s="4" t="n"/>
+      <c r="H68" s="4" t="n">
+        <v>53.16</v>
+      </c>
+      <c r="I68" s="4" t="inlineStr"/>
+      <c r="J68" s="4" t="inlineStr"/>
+      <c r="K68" s="4" t="inlineStr"/>
+      <c r="L68" s="4" t="n">
+        <v>73.83</v>
+      </c>
+      <c r="M68" s="4" t="n">
+        <v>2.215</v>
+      </c>
+      <c r="N68" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O68" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P68" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q68" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R68" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S68" s="4" t="n"/>
+      <c r="T68" s="4" t="n"/>
+      <c r="U68" s="4" t="n"/>
+      <c r="V68" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W68" s="4" t="inlineStr"/>
+      <c r="X68" s="4" t="n"/>
+      <c r="Y68" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z68" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA68" s="4" t="n"/>
+      <c r="AB68" s="4" t="n"/>
+      <c r="AC68" s="4" t="n"/>
+      <c r="AD68" s="4" t="n"/>
+      <c r="AE68" s="4" t="n"/>
+      <c r="AF68" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B69" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C69" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="F69" s="6" t="n"/>
+      <c r="G69" s="6" t="n"/>
+      <c r="H69" s="6" t="n">
+        <v>55.04</v>
+      </c>
+      <c r="I69" s="6" t="inlineStr"/>
+      <c r="J69" s="6" t="inlineStr"/>
+      <c r="K69" s="6" t="inlineStr"/>
+      <c r="L69" s="6" t="n">
+        <v>76.44</v>
+      </c>
+      <c r="M69" s="6" t="n">
+        <v>2.293</v>
+      </c>
+      <c r="N69" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O69" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P69" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q69" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R69" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S69" s="6" t="n"/>
+      <c r="T69" s="6" t="n"/>
+      <c r="U69" s="6" t="n"/>
+      <c r="V69" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W69" s="6" t="inlineStr"/>
+      <c r="X69" s="6" t="n"/>
+      <c r="Y69" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z69" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA69" s="6" t="n"/>
+      <c r="AB69" s="6" t="n"/>
+      <c r="AC69" s="6" t="n"/>
+      <c r="AD69" s="6" t="n"/>
+      <c r="AE69" s="6" t="n"/>
+      <c r="AF69" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D70" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E70" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F70" s="4" t="n"/>
+      <c r="G70" s="4" t="n"/>
+      <c r="H70" s="4" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="I70" s="4" t="inlineStr"/>
+      <c r="J70" s="4" t="inlineStr"/>
+      <c r="K70" s="4" t="inlineStr"/>
+      <c r="L70" s="4" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="M70" s="4" t="n">
+        <v>1.749</v>
+      </c>
+      <c r="N70" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O70" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P70" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q70" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R70" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S70" s="4" t="n"/>
+      <c r="T70" s="4" t="n"/>
+      <c r="U70" s="4" t="n"/>
+      <c r="V70" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W70" s="4" t="inlineStr"/>
+      <c r="X70" s="4" t="n"/>
+      <c r="Y70" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z70" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA70" s="4" t="n"/>
+      <c r="AB70" s="4" t="n"/>
+      <c r="AC70" s="4" t="n"/>
+      <c r="AD70" s="4" t="n"/>
+      <c r="AE70" s="4" t="n"/>
+      <c r="AF70" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B71" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C71" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D71" s="6" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E71" s="6" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="F71" s="6" t="n"/>
+      <c r="G71" s="6" t="n"/>
+      <c r="H71" s="6" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="I71" s="6" t="inlineStr"/>
+      <c r="J71" s="6" t="inlineStr"/>
+      <c r="K71" s="6" t="inlineStr"/>
+      <c r="L71" s="6" t="n">
+        <v>57.75</v>
+      </c>
+      <c r="M71" s="6" t="n">
+        <v>1.732</v>
+      </c>
+      <c r="N71" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O71" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P71" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q71" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R71" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S71" s="6" t="n"/>
+      <c r="T71" s="6" t="n"/>
+      <c r="U71" s="6" t="n"/>
+      <c r="V71" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W71" s="6" t="inlineStr"/>
+      <c r="X71" s="6" t="n"/>
+      <c r="Y71" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z71" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA71" s="6" t="n"/>
+      <c r="AB71" s="6" t="n"/>
+      <c r="AC71" s="6" t="n"/>
+      <c r="AD71" s="6" t="n"/>
+      <c r="AE71" s="6" t="n"/>
+      <c r="AF71" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B72" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C72" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D72" s="4" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E72" s="4" t="n">
+        <v>30.99</v>
+      </c>
+      <c r="F72" s="4" t="n"/>
+      <c r="G72" s="4" t="n"/>
+      <c r="H72" s="4" t="n">
+        <v>41.32</v>
+      </c>
+      <c r="I72" s="4" t="inlineStr"/>
+      <c r="J72" s="4" t="inlineStr"/>
+      <c r="K72" s="4" t="inlineStr"/>
+      <c r="L72" s="4" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="M72" s="4" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="N72" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O72" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P72" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q72" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R72" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S72" s="4" t="n"/>
+      <c r="T72" s="4" t="n"/>
+      <c r="U72" s="4" t="n"/>
+      <c r="V72" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W72" s="4" t="inlineStr"/>
+      <c r="X72" s="4" t="n"/>
+      <c r="Y72" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z72" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA72" s="4" t="n"/>
+      <c r="AB72" s="4" t="n"/>
+      <c r="AC72" s="4" t="n"/>
+      <c r="AD72" s="4" t="n"/>
+      <c r="AE72" s="4" t="n"/>
+      <c r="AF72" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B73" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C73" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D73" s="6" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E73" s="6" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="F73" s="6" t="n"/>
+      <c r="G73" s="6" t="n"/>
+      <c r="H73" s="6" t="n">
+        <v>38.01</v>
+      </c>
+      <c r="I73" s="6" t="inlineStr"/>
+      <c r="J73" s="6" t="inlineStr"/>
+      <c r="K73" s="6" t="inlineStr"/>
+      <c r="L73" s="6" t="n">
+        <v>52.79</v>
+      </c>
+      <c r="M73" s="6" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="N73" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O73" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P73" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q73" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R73" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S73" s="6" t="n"/>
+      <c r="T73" s="6" t="n"/>
+      <c r="U73" s="6" t="n"/>
+      <c r="V73" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W73" s="6" t="inlineStr"/>
+      <c r="X73" s="6" t="n"/>
+      <c r="Y73" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z73" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA73" s="6" t="n"/>
+      <c r="AB73" s="6" t="n"/>
+      <c r="AC73" s="6" t="n"/>
+      <c r="AD73" s="6" t="n"/>
+      <c r="AE73" s="6" t="n"/>
+      <c r="AF73" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B74" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C74" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D74" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E74" s="4" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="F74" s="4" t="n"/>
+      <c r="G74" s="4" t="n"/>
+      <c r="H74" s="4" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="I74" s="4" t="inlineStr"/>
+      <c r="J74" s="4" t="inlineStr"/>
+      <c r="K74" s="4" t="inlineStr"/>
+      <c r="L74" s="4" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M74" s="4" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="N74" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O74" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P74" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q74" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R74" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S74" s="4" t="n"/>
+      <c r="T74" s="4" t="n"/>
+      <c r="U74" s="4" t="n"/>
+      <c r="V74" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W74" s="4" t="inlineStr"/>
+      <c r="X74" s="4" t="n"/>
+      <c r="Y74" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z74" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA74" s="4" t="n"/>
+      <c r="AB74" s="4" t="n"/>
+      <c r="AC74" s="4" t="n"/>
+      <c r="AD74" s="4" t="n"/>
+      <c r="AE74" s="4" t="n"/>
+      <c r="AF74" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D75" s="6" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E75" s="6" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="F75" s="6" t="n"/>
+      <c r="G75" s="6" t="n"/>
+      <c r="H75" s="6" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="I75" s="6" t="inlineStr"/>
+      <c r="J75" s="6" t="inlineStr"/>
+      <c r="K75" s="6" t="inlineStr"/>
+      <c r="L75" s="6" t="n">
+        <v>50.63</v>
+      </c>
+      <c r="M75" s="6" t="n">
+        <v>1.519</v>
+      </c>
+      <c r="N75" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O75" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P75" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q75" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R75" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S75" s="6" t="n"/>
+      <c r="T75" s="6" t="n"/>
+      <c r="U75" s="6" t="n"/>
+      <c r="V75" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W75" s="6" t="inlineStr"/>
+      <c r="X75" s="6" t="n"/>
+      <c r="Y75" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z75" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA75" s="6" t="n"/>
+      <c r="AB75" s="6" t="n"/>
+      <c r="AC75" s="6" t="n"/>
+      <c r="AD75" s="6" t="n"/>
+      <c r="AE75" s="6" t="n"/>
+      <c r="AF75" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B76" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C76" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D76" s="4" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E76" s="4" t="n">
+        <v>85.98999999999999</v>
+      </c>
+      <c r="F76" s="4" t="n"/>
+      <c r="G76" s="4" t="n"/>
+      <c r="H76" s="4" t="n">
+        <v>41.54</v>
+      </c>
+      <c r="I76" s="4" t="inlineStr"/>
+      <c r="J76" s="4" t="inlineStr"/>
+      <c r="K76" s="4" t="inlineStr"/>
+      <c r="L76" s="4" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="M76" s="4" t="n">
+        <v>1.731</v>
+      </c>
+      <c r="N76" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O76" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P76" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q76" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R76" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S76" s="4" t="n"/>
+      <c r="T76" s="4" t="n"/>
+      <c r="U76" s="4" t="n"/>
+      <c r="V76" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W76" s="4" t="inlineStr"/>
+      <c r="X76" s="4" t="n"/>
+      <c r="Y76" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z76" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA76" s="4" t="n"/>
+      <c r="AB76" s="4" t="n"/>
+      <c r="AC76" s="4" t="n"/>
+      <c r="AD76" s="4" t="n"/>
+      <c r="AE76" s="4" t="n"/>
+      <c r="AF76" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C77" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D77" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E77" s="6" t="n">
+        <v>137.99</v>
+      </c>
+      <c r="F77" s="6" t="n"/>
+      <c r="G77" s="6" t="n"/>
+      <c r="H77" s="6" t="n">
+        <v>38.33</v>
+      </c>
+      <c r="I77" s="6" t="inlineStr"/>
+      <c r="J77" s="6" t="inlineStr"/>
+      <c r="K77" s="6" t="inlineStr"/>
+      <c r="L77" s="6" t="n">
+        <v>53.24</v>
+      </c>
+      <c r="M77" s="6" t="n">
+        <v>1.597</v>
+      </c>
+      <c r="N77" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O77" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P77" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q77" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R77" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S77" s="6" t="n"/>
+      <c r="T77" s="6" t="n"/>
+      <c r="U77" s="6" t="n"/>
+      <c r="V77" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W77" s="6" t="inlineStr"/>
+      <c r="X77" s="6" t="n"/>
+      <c r="Y77" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z77" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA77" s="6" t="n"/>
+      <c r="AB77" s="6" t="n"/>
+      <c r="AC77" s="6" t="n"/>
+      <c r="AD77" s="6" t="n"/>
+      <c r="AE77" s="6" t="n"/>
+      <c r="AF77" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B78" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C78" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D78" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E78" s="4" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="F78" s="4" t="n"/>
+      <c r="G78" s="4" t="n"/>
+      <c r="H78" s="4" t="n">
+        <v>89.72</v>
+      </c>
+      <c r="I78" s="4" t="inlineStr"/>
+      <c r="J78" s="4" t="inlineStr"/>
+      <c r="K78" s="4" t="inlineStr"/>
+      <c r="L78" s="4" t="n">
+        <v>109.41</v>
+      </c>
+      <c r="M78" s="4" t="n">
+        <v>3.282</v>
+      </c>
+      <c r="N78" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O78" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P78" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q78" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R78" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S78" s="4" t="n"/>
+      <c r="T78" s="4" t="n"/>
+      <c r="U78" s="4" t="n"/>
+      <c r="V78" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W78" s="4" t="inlineStr"/>
+      <c r="X78" s="4" t="n"/>
+      <c r="Y78" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z78" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA78" s="4" t="n"/>
+      <c r="AB78" s="4" t="n"/>
+      <c r="AC78" s="4" t="n"/>
+      <c r="AD78" s="4" t="n"/>
+      <c r="AE78" s="4" t="n"/>
+      <c r="AF78" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B79" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C79" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D79" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E79" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F79" s="6" t="n"/>
+      <c r="G79" s="6" t="n"/>
+      <c r="H79" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I79" s="6" t="inlineStr"/>
+      <c r="J79" s="6" t="inlineStr"/>
+      <c r="K79" s="6" t="inlineStr"/>
+      <c r="L79" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M79" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N79" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O79" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P79" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q79" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R79" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S79" s="6" t="n"/>
+      <c r="T79" s="6" t="n"/>
+      <c r="U79" s="6" t="n"/>
+      <c r="V79" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W79" s="6" t="inlineStr"/>
+      <c r="X79" s="6" t="n"/>
+      <c r="Y79" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z79" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA79" s="6" t="n"/>
+      <c r="AB79" s="6" t="n"/>
+      <c r="AC79" s="6" t="n"/>
+      <c r="AD79" s="6" t="n"/>
+      <c r="AE79" s="6" t="n"/>
+      <c r="AF79" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D80" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E80" s="4" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="F80" s="4" t="n"/>
+      <c r="G80" s="4" t="n"/>
+      <c r="H80" s="4" t="n">
+        <v>71.78</v>
+      </c>
+      <c r="I80" s="4" t="inlineStr"/>
+      <c r="J80" s="4" t="inlineStr"/>
+      <c r="K80" s="4" t="inlineStr"/>
+      <c r="L80" s="4" t="n">
+        <v>87.54000000000001</v>
+      </c>
+      <c r="M80" s="4" t="n">
+        <v>2.626</v>
+      </c>
+      <c r="N80" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O80" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P80" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q80" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R80" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S80" s="4" t="n"/>
+      <c r="T80" s="4" t="n"/>
+      <c r="U80" s="4" t="n"/>
+      <c r="V80" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W80" s="4" t="inlineStr"/>
+      <c r="X80" s="4" t="n"/>
+      <c r="Y80" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z80" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA80" s="4" t="n"/>
+      <c r="AB80" s="4" t="n"/>
+      <c r="AC80" s="4" t="n"/>
+      <c r="AD80" s="4" t="n"/>
+      <c r="AE80" s="4" t="n"/>
+      <c r="AF80" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="F81" s="6" t="n"/>
+      <c r="G81" s="6" t="n"/>
+      <c r="H81" s="6" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="I81" s="6" t="inlineStr"/>
+      <c r="J81" s="6" t="inlineStr"/>
+      <c r="K81" s="6" t="inlineStr"/>
+      <c r="L81" s="6" t="n">
+        <v>80.48</v>
+      </c>
+      <c r="M81" s="6" t="n">
+        <v>2.414</v>
+      </c>
+      <c r="N81" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O81" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P81" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q81" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R81" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S81" s="6" t="n"/>
+      <c r="T81" s="6" t="n"/>
+      <c r="U81" s="6" t="n"/>
+      <c r="V81" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W81" s="6" t="inlineStr"/>
+      <c r="X81" s="6" t="n"/>
+      <c r="Y81" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z81" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA81" s="6" t="n"/>
+      <c r="AB81" s="6" t="n"/>
+      <c r="AC81" s="6" t="n"/>
+      <c r="AD81" s="6" t="n"/>
+      <c r="AE81" s="6" t="n"/>
+      <c r="AF81" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D82" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E82" s="4" t="n">
+        <v>132.99</v>
+      </c>
+      <c r="F82" s="4" t="n"/>
+      <c r="G82" s="4" t="n"/>
+      <c r="H82" s="4" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="I82" s="4" t="inlineStr"/>
+      <c r="J82" s="4" t="inlineStr"/>
+      <c r="K82" s="4" t="inlineStr"/>
+      <c r="L82" s="4" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="M82" s="4" t="n">
+        <v>1.946</v>
+      </c>
+      <c r="N82" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O82" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P82" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q82" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R82" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S82" s="4" t="n"/>
+      <c r="T82" s="4" t="n"/>
+      <c r="U82" s="4" t="n"/>
+      <c r="V82" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W82" s="4" t="inlineStr"/>
+      <c r="X82" s="4" t="n"/>
+      <c r="Y82" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z82" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA82" s="4" t="n"/>
+      <c r="AB82" s="4" t="n"/>
+      <c r="AC82" s="4" t="n"/>
+      <c r="AD82" s="4" t="n"/>
+      <c r="AE82" s="4" t="n"/>
+      <c r="AF82" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B83" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C83" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="n">
+        <v>155.99</v>
+      </c>
+      <c r="F83" s="6" t="n"/>
+      <c r="G83" s="6" t="n"/>
+      <c r="H83" s="6" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="I83" s="6" t="inlineStr"/>
+      <c r="J83" s="6" t="inlineStr"/>
+      <c r="K83" s="6" t="inlineStr"/>
+      <c r="L83" s="6" t="n">
+        <v>70.45</v>
+      </c>
+      <c r="M83" s="6" t="n">
+        <v>2.114</v>
+      </c>
+      <c r="N83" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O83" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P83" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q83" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R83" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S83" s="6" t="n"/>
+      <c r="T83" s="6" t="n"/>
+      <c r="U83" s="6" t="n"/>
+      <c r="V83" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W83" s="6" t="inlineStr"/>
+      <c r="X83" s="6" t="n"/>
+      <c r="Y83" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z83" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA83" s="6" t="n"/>
+      <c r="AB83" s="6" t="n"/>
+      <c r="AC83" s="6" t="n"/>
+      <c r="AD83" s="6" t="n"/>
+      <c r="AE83" s="6" t="n"/>
+      <c r="AF83" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D84" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E84" s="4" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="F84" s="4" t="n"/>
+      <c r="G84" s="4" t="n"/>
+      <c r="H84" s="4" t="n">
+        <v>59.52</v>
+      </c>
+      <c r="I84" s="4" t="inlineStr"/>
+      <c r="J84" s="4" t="inlineStr"/>
+      <c r="K84" s="4" t="inlineStr"/>
+      <c r="L84" s="4" t="n">
+        <v>72.59</v>
+      </c>
+      <c r="M84" s="4" t="n">
+        <v>2.178</v>
+      </c>
+      <c r="N84" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O84" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P84" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q84" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R84" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S84" s="4" t="n"/>
+      <c r="T84" s="4" t="n"/>
+      <c r="U84" s="4" t="n"/>
+      <c r="V84" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W84" s="4" t="inlineStr"/>
+      <c r="X84" s="4" t="n"/>
+      <c r="Y84" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z84" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA84" s="4" t="n"/>
+      <c r="AB84" s="4" t="n"/>
+      <c r="AC84" s="4" t="n"/>
+      <c r="AD84" s="4" t="n"/>
+      <c r="AE84" s="4" t="n"/>
+      <c r="AF84" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B85" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C85" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="n">
+        <v>30.39</v>
+      </c>
+      <c r="F85" s="6" t="n"/>
+      <c r="G85" s="6" t="n"/>
+      <c r="H85" s="6" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="I85" s="6" t="inlineStr"/>
+      <c r="J85" s="6" t="inlineStr"/>
+      <c r="K85" s="6" t="inlineStr"/>
+      <c r="L85" s="6" t="n">
+        <v>91.59</v>
+      </c>
+      <c r="M85" s="6" t="n">
+        <v>2.748</v>
+      </c>
+      <c r="N85" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O85" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P85" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q85" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S85" s="6" t="n"/>
+      <c r="T85" s="6" t="n"/>
+      <c r="U85" s="6" t="n"/>
+      <c r="V85" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W85" s="6" t="inlineStr"/>
+      <c r="X85" s="6" t="n"/>
+      <c r="Y85" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z85" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA85" s="6" t="n"/>
+      <c r="AB85" s="6" t="n"/>
+      <c r="AC85" s="6" t="n"/>
+      <c r="AD85" s="6" t="n"/>
+      <c r="AE85" s="6" t="n"/>
+      <c r="AF85" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D86" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E86" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="F86" s="4" t="n"/>
+      <c r="G86" s="4" t="n"/>
+      <c r="H86" s="4" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="I86" s="4" t="inlineStr"/>
+      <c r="J86" s="4" t="inlineStr"/>
+      <c r="K86" s="4" t="inlineStr"/>
+      <c r="L86" s="4" t="n">
+        <v>70.86</v>
+      </c>
+      <c r="M86" s="4" t="n">
+        <v>2.126</v>
+      </c>
+      <c r="N86" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O86" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P86" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S86" s="4" t="n"/>
+      <c r="T86" s="4" t="n"/>
+      <c r="U86" s="4" t="n"/>
+      <c r="V86" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W86" s="4" t="inlineStr"/>
+      <c r="X86" s="4" t="n"/>
+      <c r="Y86" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z86" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA86" s="4" t="n"/>
+      <c r="AB86" s="4" t="n"/>
+      <c r="AC86" s="4" t="n"/>
+      <c r="AD86" s="4" t="n"/>
+      <c r="AE86" s="4" t="n"/>
+      <c r="AF86" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B87" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C87" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>910g</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F87" s="6" t="n"/>
+      <c r="G87" s="6" t="n"/>
+      <c r="H87" s="6" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="I87" s="6" t="inlineStr"/>
+      <c r="J87" s="6" t="inlineStr"/>
+      <c r="K87" s="6" t="inlineStr"/>
+      <c r="L87" s="6" t="n">
+        <v>69.53</v>
+      </c>
+      <c r="M87" s="6" t="n">
+        <v>2.086</v>
+      </c>
+      <c r="N87" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O87" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P87" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q87" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S87" s="6" t="n"/>
+      <c r="T87" s="6" t="n"/>
+      <c r="U87" s="6" t="n"/>
+      <c r="V87" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W87" s="6" t="inlineStr"/>
+      <c r="X87" s="6" t="n"/>
+      <c r="Y87" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z87" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA87" s="6" t="n"/>
+      <c r="AB87" s="6" t="n"/>
+      <c r="AC87" s="6" t="n"/>
+      <c r="AD87" s="6" t="n"/>
+      <c r="AE87" s="6" t="n"/>
+      <c r="AF87" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D88" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E88" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F88" s="4" t="n"/>
+      <c r="G88" s="4" t="n"/>
+      <c r="H88" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="I88" s="4" t="inlineStr"/>
+      <c r="J88" s="4" t="inlineStr"/>
+      <c r="K88" s="4" t="inlineStr"/>
+      <c r="L88" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M88" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N88" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O88" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P88" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q88" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S88" s="4" t="n"/>
+      <c r="T88" s="4" t="n"/>
+      <c r="U88" s="4" t="n"/>
+      <c r="V88" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W88" s="4" t="inlineStr"/>
+      <c r="X88" s="4" t="n"/>
+      <c r="Y88" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z88" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA88" s="4" t="n"/>
+      <c r="AB88" s="4" t="n"/>
+      <c r="AC88" s="4" t="n"/>
+      <c r="AD88" s="4" t="n"/>
+      <c r="AE88" s="4" t="n"/>
+      <c r="AF88" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B89" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C89" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="F89" s="6" t="n"/>
+      <c r="G89" s="6" t="n"/>
+      <c r="H89" s="6" t="n">
+        <v>37.12</v>
+      </c>
+      <c r="I89" s="6" t="inlineStr"/>
+      <c r="J89" s="6" t="inlineStr"/>
+      <c r="K89" s="6" t="inlineStr"/>
+      <c r="L89" s="6" t="n">
+        <v>62.92</v>
+      </c>
+      <c r="M89" s="6" t="n">
+        <v>1.888</v>
+      </c>
+      <c r="N89" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O89" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P89" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q89" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R89" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S89" s="6" t="n"/>
+      <c r="T89" s="6" t="n"/>
+      <c r="U89" s="6" t="n"/>
+      <c r="V89" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W89" s="6" t="inlineStr"/>
+      <c r="X89" s="6" t="n"/>
+      <c r="Y89" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z89" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA89" s="6" t="n"/>
+      <c r="AB89" s="6" t="n"/>
+      <c r="AC89" s="6" t="n"/>
+      <c r="AD89" s="6" t="n"/>
+      <c r="AE89" s="6" t="n"/>
+      <c r="AF89" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D90" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E90" s="4" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="F90" s="4" t="n"/>
+      <c r="G90" s="4" t="n"/>
+      <c r="H90" s="4" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="I90" s="4" t="inlineStr"/>
+      <c r="J90" s="4" t="inlineStr"/>
+      <c r="K90" s="4" t="inlineStr"/>
+      <c r="L90" s="4" t="n">
+        <v>56.17</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>1.685</v>
+      </c>
+      <c r="N90" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O90" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P90" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q90" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R90" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S90" s="4" t="n"/>
+      <c r="T90" s="4" t="n"/>
+      <c r="U90" s="4" t="n"/>
+      <c r="V90" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W90" s="4" t="inlineStr"/>
+      <c r="X90" s="4" t="n"/>
+      <c r="Y90" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z90" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA90" s="4" t="n"/>
+      <c r="AB90" s="4" t="n"/>
+      <c r="AC90" s="4" t="n"/>
+      <c r="AD90" s="4" t="n"/>
+      <c r="AE90" s="4" t="n"/>
+      <c r="AF90" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="n">
+        <v>74.73999999999999</v>
+      </c>
+      <c r="F91" s="6" t="n"/>
+      <c r="G91" s="6" t="n"/>
+      <c r="H91" s="6" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I91" s="6" t="inlineStr"/>
+      <c r="J91" s="6" t="inlineStr"/>
+      <c r="K91" s="6" t="inlineStr"/>
+      <c r="L91" s="6" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M91" s="6" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="N91" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O91" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P91" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q91" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R91" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S91" s="6" t="n"/>
+      <c r="T91" s="6" t="n"/>
+      <c r="U91" s="6" t="n"/>
+      <c r="V91" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W91" s="6" t="inlineStr"/>
+      <c r="X91" s="6" t="n"/>
+      <c r="Y91" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z91" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA91" s="6" t="n"/>
+      <c r="AB91" s="6" t="n"/>
+      <c r="AC91" s="6" t="n"/>
+      <c r="AD91" s="6" t="n"/>
+      <c r="AE91" s="6" t="n"/>
+      <c r="AF91" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D92" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E92" s="4" t="n">
+        <v>139.74</v>
+      </c>
+      <c r="F92" s="4" t="n"/>
+      <c r="G92" s="4" t="n"/>
+      <c r="H92" s="4" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="I92" s="4" t="inlineStr"/>
+      <c r="J92" s="4" t="inlineStr"/>
+      <c r="K92" s="4" t="inlineStr"/>
+      <c r="L92" s="4" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="M92" s="4" t="n">
+        <v>1.421</v>
+      </c>
+      <c r="N92" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O92" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P92" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q92" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R92" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S92" s="4" t="n"/>
+      <c r="T92" s="4" t="n"/>
+      <c r="U92" s="4" t="n"/>
+      <c r="V92" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W92" s="4" t="inlineStr"/>
+      <c r="X92" s="4" t="n"/>
+      <c r="Y92" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z92" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA92" s="4" t="n"/>
+      <c r="AB92" s="4" t="n"/>
+      <c r="AC92" s="4" t="n"/>
+      <c r="AD92" s="4" t="n"/>
+      <c r="AE92" s="4" t="n"/>
+      <c r="AF92" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B93" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="F93" s="6" t="n"/>
+      <c r="G93" s="6" t="n"/>
+      <c r="H93" s="6" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="I93" s="6" t="inlineStr"/>
+      <c r="J93" s="6" t="inlineStr"/>
+      <c r="K93" s="6" t="inlineStr"/>
+      <c r="L93" s="6" t="n"/>
+      <c r="M93" s="6" t="n"/>
+      <c r="N93" s="6" t="n"/>
+      <c r="O93" s="6" t="n"/>
+      <c r="P93" s="6" t="n"/>
+      <c r="Q93" s="6" t="n"/>
+      <c r="R93" s="6" t="n"/>
+      <c r="S93" s="6" t="n"/>
+      <c r="T93" s="6" t="n"/>
+      <c r="U93" s="6" t="n"/>
+      <c r="V93" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W93" s="6" t="inlineStr"/>
+      <c r="X93" s="6" t="n"/>
+      <c r="Y93" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z93" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA93" s="6" t="n"/>
+      <c r="AB93" s="6" t="n"/>
+      <c r="AC93" s="6" t="n"/>
+      <c r="AD93" s="6" t="n"/>
+      <c r="AE93" s="6" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="AF93" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D94" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E94" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="F94" s="4" t="n"/>
+      <c r="G94" s="4" t="n"/>
+      <c r="H94" s="4" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="I94" s="4" t="inlineStr"/>
+      <c r="J94" s="4" t="inlineStr"/>
+      <c r="K94" s="4" t="inlineStr"/>
+      <c r="L94" s="4" t="n"/>
+      <c r="M94" s="4" t="n"/>
+      <c r="N94" s="4" t="n"/>
+      <c r="O94" s="4" t="n"/>
+      <c r="P94" s="4" t="n"/>
+      <c r="Q94" s="4" t="n"/>
+      <c r="R94" s="4" t="n"/>
+      <c r="S94" s="4" t="n"/>
+      <c r="T94" s="4" t="n"/>
+      <c r="U94" s="4" t="n"/>
+      <c r="V94" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W94" s="4" t="inlineStr"/>
+      <c r="X94" s="4" t="n"/>
+      <c r="Y94" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z94" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA94" s="4" t="n"/>
+      <c r="AB94" s="4" t="n"/>
+      <c r="AC94" s="4" t="n"/>
+      <c r="AD94" s="4" t="n"/>
+      <c r="AE94" s="4" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="AF94" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B95" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C95" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="F95" s="6" t="n"/>
+      <c r="G95" s="6" t="n"/>
+      <c r="H95" s="6" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="I95" s="6" t="inlineStr"/>
+      <c r="J95" s="6" t="inlineStr"/>
+      <c r="K95" s="6" t="inlineStr"/>
+      <c r="L95" s="6" t="n"/>
+      <c r="M95" s="6" t="n"/>
+      <c r="N95" s="6" t="n"/>
+      <c r="O95" s="6" t="n"/>
+      <c r="P95" s="6" t="n"/>
+      <c r="Q95" s="6" t="n"/>
+      <c r="R95" s="6" t="n"/>
+      <c r="S95" s="6" t="n"/>
+      <c r="T95" s="6" t="n"/>
+      <c r="U95" s="6" t="n"/>
+      <c r="V95" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W95" s="6" t="inlineStr"/>
+      <c r="X95" s="6" t="n"/>
+      <c r="Y95" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z95" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA95" s="6" t="n"/>
+      <c r="AB95" s="6" t="n"/>
+      <c r="AC95" s="6" t="n"/>
+      <c r="AD95" s="6" t="n"/>
+      <c r="AE95" s="6" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="AF95" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B96" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C96" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D96" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E96" s="4" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="F96" s="4" t="n"/>
+      <c r="G96" s="4" t="n"/>
+      <c r="H96" s="4" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="I96" s="4" t="inlineStr"/>
+      <c r="J96" s="4" t="inlineStr"/>
+      <c r="K96" s="4" t="inlineStr"/>
+      <c r="L96" s="4" t="n"/>
+      <c r="M96" s="4" t="n"/>
+      <c r="N96" s="4" t="n"/>
+      <c r="O96" s="4" t="n"/>
+      <c r="P96" s="4" t="n"/>
+      <c r="Q96" s="4" t="n"/>
+      <c r="R96" s="4" t="n"/>
+      <c r="S96" s="4" t="n"/>
+      <c r="T96" s="4" t="n"/>
+      <c r="U96" s="4" t="n"/>
+      <c r="V96" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W96" s="4" t="inlineStr"/>
+      <c r="X96" s="4" t="n"/>
+      <c r="Y96" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z96" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA96" s="4" t="n"/>
+      <c r="AB96" s="4" t="n"/>
+      <c r="AC96" s="4" t="n"/>
+      <c r="AD96" s="4" t="n"/>
+      <c r="AE96" s="4" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="AF96" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B97" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C97" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D97" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E97" s="6" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="F97" s="6" t="n"/>
+      <c r="G97" s="6" t="n"/>
+      <c r="H97" s="6" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="I97" s="6" t="inlineStr"/>
+      <c r="J97" s="6" t="inlineStr"/>
+      <c r="K97" s="6" t="inlineStr"/>
+      <c r="L97" s="6" t="n"/>
+      <c r="M97" s="6" t="n"/>
+      <c r="N97" s="6" t="n"/>
+      <c r="O97" s="6" t="n"/>
+      <c r="P97" s="6" t="n"/>
+      <c r="Q97" s="6" t="n"/>
+      <c r="R97" s="6" t="n"/>
+      <c r="S97" s="6" t="n"/>
+      <c r="T97" s="6" t="n"/>
+      <c r="U97" s="6" t="n"/>
+      <c r="V97" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W97" s="6" t="inlineStr"/>
+      <c r="X97" s="6" t="n"/>
+      <c r="Y97" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z97" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA97" s="6" t="n"/>
+      <c r="AB97" s="6" t="n"/>
+      <c r="AC97" s="6" t="n"/>
+      <c r="AD97" s="6" t="n"/>
+      <c r="AE97" s="6" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="AF97" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D98" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E98" s="4" t="n">
+        <v>42.99</v>
+      </c>
+      <c r="F98" s="4" t="n"/>
+      <c r="G98" s="4" t="n"/>
+      <c r="H98" s="4" t="n">
+        <v>85.98</v>
+      </c>
+      <c r="I98" s="4" t="inlineStr"/>
+      <c r="J98" s="4" t="inlineStr"/>
+      <c r="K98" s="4" t="inlineStr"/>
+      <c r="L98" s="4" t="n"/>
+      <c r="M98" s="4" t="n"/>
+      <c r="N98" s="4" t="n"/>
+      <c r="O98" s="4" t="n"/>
+      <c r="P98" s="4" t="n"/>
+      <c r="Q98" s="4" t="n"/>
+      <c r="R98" s="4" t="n"/>
+      <c r="S98" s="4" t="n"/>
+      <c r="T98" s="4" t="n"/>
+      <c r="U98" s="4" t="n"/>
+      <c r="V98" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W98" s="4" t="inlineStr"/>
+      <c r="X98" s="4" t="n"/>
+      <c r="Y98" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z98" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA98" s="4" t="n"/>
+      <c r="AB98" s="4" t="n"/>
+      <c r="AC98" s="4" t="n"/>
+      <c r="AD98" s="4" t="n"/>
+      <c r="AE98" s="4" t="n">
+        <v>85.98</v>
+      </c>
+      <c r="AF98" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B99" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C99" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D99" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E99" s="6" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="F99" s="6" t="n"/>
+      <c r="G99" s="6" t="n"/>
+      <c r="H99" s="6" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="I99" s="6" t="inlineStr"/>
+      <c r="J99" s="6" t="inlineStr"/>
+      <c r="K99" s="6" t="inlineStr"/>
+      <c r="L99" s="6" t="n"/>
+      <c r="M99" s="6" t="n"/>
+      <c r="N99" s="6" t="n"/>
+      <c r="O99" s="6" t="n"/>
+      <c r="P99" s="6" t="n"/>
+      <c r="Q99" s="6" t="n"/>
+      <c r="R99" s="6" t="n"/>
+      <c r="S99" s="6" t="n"/>
+      <c r="T99" s="6" t="n"/>
+      <c r="U99" s="6" t="n"/>
+      <c r="V99" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W99" s="6" t="inlineStr"/>
+      <c r="X99" s="6" t="n"/>
+      <c r="Y99" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z99" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA99" s="6" t="n"/>
+      <c r="AB99" s="6" t="n"/>
+      <c r="AC99" s="6" t="n"/>
+      <c r="AD99" s="6" t="n"/>
+      <c r="AE99" s="6" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="AF99" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B100" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C100" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D100" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E100" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F100" s="4" t="n"/>
+      <c r="G100" s="4" t="n"/>
+      <c r="H100" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I100" s="4" t="inlineStr"/>
+      <c r="J100" s="4" t="inlineStr"/>
+      <c r="K100" s="4" t="inlineStr"/>
+      <c r="L100" s="4" t="n"/>
+      <c r="M100" s="4" t="n"/>
+      <c r="N100" s="4" t="n"/>
+      <c r="O100" s="4" t="n"/>
+      <c r="P100" s="4" t="n"/>
+      <c r="Q100" s="4" t="n"/>
+      <c r="R100" s="4" t="n"/>
+      <c r="S100" s="4" t="n"/>
+      <c r="T100" s="4" t="n"/>
+      <c r="U100" s="4" t="n"/>
+      <c r="V100" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W100" s="4" t="inlineStr"/>
+      <c r="X100" s="4" t="n"/>
+      <c r="Y100" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z100" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA100" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB100" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC100" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD100" s="4" t="n"/>
+      <c r="AE100" s="4" t="n"/>
+      <c r="AF100" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B101" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C101" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D101" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E101" s="6" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="F101" s="6" t="n"/>
+      <c r="G101" s="6" t="n"/>
+      <c r="H101" s="6" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="I101" s="6" t="inlineStr"/>
+      <c r="J101" s="6" t="inlineStr"/>
+      <c r="K101" s="6" t="inlineStr"/>
+      <c r="L101" s="6" t="n"/>
+      <c r="M101" s="6" t="n"/>
+      <c r="N101" s="6" t="n"/>
+      <c r="O101" s="6" t="n"/>
+      <c r="P101" s="6" t="n"/>
+      <c r="Q101" s="6" t="n"/>
+      <c r="R101" s="6" t="n"/>
+      <c r="S101" s="6" t="n"/>
+      <c r="T101" s="6" t="n"/>
+      <c r="U101" s="6" t="n"/>
+      <c r="V101" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W101" s="6" t="inlineStr"/>
+      <c r="X101" s="6" t="n"/>
+      <c r="Y101" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z101" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA101" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB101" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC101" s="6" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AD101" s="6" t="n"/>
+      <c r="AE101" s="6" t="n"/>
+      <c r="AF101" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B102" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C102" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D102" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E102" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F102" s="4" t="n"/>
+      <c r="G102" s="4" t="n"/>
+      <c r="H102" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I102" s="4" t="inlineStr"/>
+      <c r="J102" s="4" t="inlineStr"/>
+      <c r="K102" s="4" t="inlineStr"/>
+      <c r="L102" s="4" t="n"/>
+      <c r="M102" s="4" t="n"/>
+      <c r="N102" s="4" t="n"/>
+      <c r="O102" s="4" t="n"/>
+      <c r="P102" s="4" t="n"/>
+      <c r="Q102" s="4" t="n"/>
+      <c r="R102" s="4" t="n"/>
+      <c r="S102" s="4" t="n"/>
+      <c r="T102" s="4" t="n"/>
+      <c r="U102" s="4" t="n"/>
+      <c r="V102" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W102" s="4" t="inlineStr"/>
+      <c r="X102" s="4" t="n"/>
+      <c r="Y102" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z102" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA102" s="4" t="n"/>
+      <c r="AB102" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC102" s="4" t="n"/>
+      <c r="AD102" s="4" t="n"/>
+      <c r="AE102" s="4" t="n"/>
+      <c r="AF102" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-21</t>
+        </is>
+      </c>
+      <c r="B103" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D103" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E103" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F103" s="6" t="n"/>
+      <c r="G103" s="6" t="n"/>
+      <c r="H103" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I103" s="6" t="inlineStr"/>
+      <c r="J103" s="6" t="inlineStr"/>
+      <c r="K103" s="6" t="inlineStr"/>
+      <c r="L103" s="6" t="n"/>
+      <c r="M103" s="6" t="n"/>
+      <c r="N103" s="6" t="n"/>
+      <c r="O103" s="6" t="n"/>
+      <c r="P103" s="6" t="n"/>
+      <c r="Q103" s="6" t="n"/>
+      <c r="R103" s="6" t="n"/>
+      <c r="S103" s="6" t="n"/>
+      <c r="T103" s="6" t="n"/>
+      <c r="U103" s="6" t="n"/>
+      <c r="V103" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W103" s="6" t="inlineStr"/>
+      <c r="X103" s="6" t="n"/>
+      <c r="Y103" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z103" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA103" s="6" t="n"/>
+      <c r="AB103" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC103" s="6" t="n"/>
+      <c r="AD103" s="6" t="n"/>
+      <c r="AE103" s="6" t="n"/>
+      <c r="AF103" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-22
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF103"/>
+  <dimension ref="A1:AF141"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -8664,6 +8664,3000 @@
         <v>1</v>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B104" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C104" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D104" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E104" s="4" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="F104" s="4" t="n"/>
+      <c r="G104" s="4" t="n"/>
+      <c r="H104" s="4" t="n">
+        <v>53.16</v>
+      </c>
+      <c r="I104" s="4" t="inlineStr"/>
+      <c r="J104" s="4" t="inlineStr"/>
+      <c r="K104" s="4" t="inlineStr"/>
+      <c r="L104" s="4" t="n">
+        <v>73.83</v>
+      </c>
+      <c r="M104" s="4" t="n">
+        <v>2.215</v>
+      </c>
+      <c r="N104" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O104" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P104" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q104" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R104" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S104" s="4" t="n"/>
+      <c r="T104" s="4" t="n"/>
+      <c r="U104" s="4" t="n"/>
+      <c r="V104" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W104" s="4" t="inlineStr"/>
+      <c r="X104" s="4" t="n"/>
+      <c r="Y104" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z104" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA104" s="4" t="n"/>
+      <c r="AB104" s="4" t="n"/>
+      <c r="AC104" s="4" t="n"/>
+      <c r="AD104" s="4" t="n"/>
+      <c r="AE104" s="4" t="n"/>
+      <c r="AF104" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B105" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C105" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D105" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E105" s="6" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="F105" s="6" t="n"/>
+      <c r="G105" s="6" t="n"/>
+      <c r="H105" s="6" t="n">
+        <v>55.04</v>
+      </c>
+      <c r="I105" s="6" t="inlineStr"/>
+      <c r="J105" s="6" t="inlineStr"/>
+      <c r="K105" s="6" t="inlineStr"/>
+      <c r="L105" s="6" t="n">
+        <v>76.44</v>
+      </c>
+      <c r="M105" s="6" t="n">
+        <v>2.293</v>
+      </c>
+      <c r="N105" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O105" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P105" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q105" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R105" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S105" s="6" t="n"/>
+      <c r="T105" s="6" t="n"/>
+      <c r="U105" s="6" t="n"/>
+      <c r="V105" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W105" s="6" t="inlineStr"/>
+      <c r="X105" s="6" t="n"/>
+      <c r="Y105" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z105" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA105" s="6" t="n"/>
+      <c r="AB105" s="6" t="n"/>
+      <c r="AC105" s="6" t="n"/>
+      <c r="AD105" s="6" t="n"/>
+      <c r="AE105" s="6" t="n"/>
+      <c r="AF105" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B106" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C106" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D106" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E106" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F106" s="4" t="n"/>
+      <c r="G106" s="4" t="n"/>
+      <c r="H106" s="4" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="I106" s="4" t="inlineStr"/>
+      <c r="J106" s="4" t="inlineStr"/>
+      <c r="K106" s="4" t="inlineStr"/>
+      <c r="L106" s="4" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="M106" s="4" t="n">
+        <v>1.749</v>
+      </c>
+      <c r="N106" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O106" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P106" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q106" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R106" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S106" s="4" t="n"/>
+      <c r="T106" s="4" t="n"/>
+      <c r="U106" s="4" t="n"/>
+      <c r="V106" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W106" s="4" t="inlineStr"/>
+      <c r="X106" s="4" t="n"/>
+      <c r="Y106" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z106" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA106" s="4" t="n"/>
+      <c r="AB106" s="4" t="n"/>
+      <c r="AC106" s="4" t="n"/>
+      <c r="AD106" s="4" t="n"/>
+      <c r="AE106" s="4" t="n"/>
+      <c r="AF106" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B107" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C107" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D107" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E107" s="6" t="n">
+        <v>25.19</v>
+      </c>
+      <c r="F107" s="6" t="n"/>
+      <c r="G107" s="6" t="n"/>
+      <c r="H107" s="6" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="I107" s="6" t="inlineStr"/>
+      <c r="J107" s="6" t="inlineStr"/>
+      <c r="K107" s="6" t="inlineStr"/>
+      <c r="L107" s="6" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="M107" s="6" t="n">
+        <v>1.749</v>
+      </c>
+      <c r="N107" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O107" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P107" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q107" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R107" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S107" s="6" t="n"/>
+      <c r="T107" s="6" t="n"/>
+      <c r="U107" s="6" t="n"/>
+      <c r="V107" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W107" s="6" t="inlineStr"/>
+      <c r="X107" s="6" t="n"/>
+      <c r="Y107" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z107" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA107" s="6" t="n"/>
+      <c r="AB107" s="6" t="n"/>
+      <c r="AC107" s="6" t="n"/>
+      <c r="AD107" s="6" t="n"/>
+      <c r="AE107" s="6" t="n"/>
+      <c r="AF107" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B108" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C108" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D108" s="4" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E108" s="4" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="F108" s="4" t="n"/>
+      <c r="G108" s="4" t="n"/>
+      <c r="H108" s="4" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="I108" s="4" t="inlineStr"/>
+      <c r="J108" s="4" t="inlineStr"/>
+      <c r="K108" s="4" t="inlineStr"/>
+      <c r="L108" s="4" t="n">
+        <v>57.75</v>
+      </c>
+      <c r="M108" s="4" t="n">
+        <v>1.732</v>
+      </c>
+      <c r="N108" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O108" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P108" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q108" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R108" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S108" s="4" t="n"/>
+      <c r="T108" s="4" t="n"/>
+      <c r="U108" s="4" t="n"/>
+      <c r="V108" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W108" s="4" t="inlineStr"/>
+      <c r="X108" s="4" t="n"/>
+      <c r="Y108" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z108" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA108" s="4" t="n"/>
+      <c r="AB108" s="4" t="n"/>
+      <c r="AC108" s="4" t="n"/>
+      <c r="AD108" s="4" t="n"/>
+      <c r="AE108" s="4" t="n"/>
+      <c r="AF108" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B109" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C109" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D109" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E109" s="6" t="n">
+        <v>30.99</v>
+      </c>
+      <c r="F109" s="6" t="n"/>
+      <c r="G109" s="6" t="n"/>
+      <c r="H109" s="6" t="n">
+        <v>41.32</v>
+      </c>
+      <c r="I109" s="6" t="inlineStr"/>
+      <c r="J109" s="6" t="inlineStr"/>
+      <c r="K109" s="6" t="inlineStr"/>
+      <c r="L109" s="6" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="M109" s="6" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="N109" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O109" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P109" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q109" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R109" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S109" s="6" t="n"/>
+      <c r="T109" s="6" t="n"/>
+      <c r="U109" s="6" t="n"/>
+      <c r="V109" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W109" s="6" t="inlineStr"/>
+      <c r="X109" s="6" t="n"/>
+      <c r="Y109" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z109" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA109" s="6" t="n"/>
+      <c r="AB109" s="6" t="n"/>
+      <c r="AC109" s="6" t="n"/>
+      <c r="AD109" s="6" t="n"/>
+      <c r="AE109" s="6" t="n"/>
+      <c r="AF109" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B110" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C110" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D110" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E110" s="4" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="F110" s="4" t="n"/>
+      <c r="G110" s="4" t="n"/>
+      <c r="H110" s="4" t="n">
+        <v>38.01</v>
+      </c>
+      <c r="I110" s="4" t="inlineStr"/>
+      <c r="J110" s="4" t="inlineStr"/>
+      <c r="K110" s="4" t="inlineStr"/>
+      <c r="L110" s="4" t="n">
+        <v>52.79</v>
+      </c>
+      <c r="M110" s="4" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="N110" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O110" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P110" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q110" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R110" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S110" s="4" t="n"/>
+      <c r="T110" s="4" t="n"/>
+      <c r="U110" s="4" t="n"/>
+      <c r="V110" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W110" s="4" t="inlineStr"/>
+      <c r="X110" s="4" t="n"/>
+      <c r="Y110" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z110" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA110" s="4" t="n"/>
+      <c r="AB110" s="4" t="n"/>
+      <c r="AC110" s="4" t="n"/>
+      <c r="AD110" s="4" t="n"/>
+      <c r="AE110" s="4" t="n"/>
+      <c r="AF110" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C111" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D111" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E111" s="6" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="F111" s="6" t="n"/>
+      <c r="G111" s="6" t="n"/>
+      <c r="H111" s="6" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="I111" s="6" t="inlineStr"/>
+      <c r="J111" s="6" t="inlineStr"/>
+      <c r="K111" s="6" t="inlineStr"/>
+      <c r="L111" s="6" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M111" s="6" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="N111" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O111" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P111" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q111" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R111" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S111" s="6" t="n"/>
+      <c r="T111" s="6" t="n"/>
+      <c r="U111" s="6" t="n"/>
+      <c r="V111" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W111" s="6" t="inlineStr"/>
+      <c r="X111" s="6" t="n"/>
+      <c r="Y111" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z111" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA111" s="6" t="n"/>
+      <c r="AB111" s="6" t="n"/>
+      <c r="AC111" s="6" t="n"/>
+      <c r="AD111" s="6" t="n"/>
+      <c r="AE111" s="6" t="n"/>
+      <c r="AF111" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B112" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C112" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D112" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E112" s="4" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="F112" s="4" t="n"/>
+      <c r="G112" s="4" t="n"/>
+      <c r="H112" s="4" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="I112" s="4" t="inlineStr"/>
+      <c r="J112" s="4" t="inlineStr"/>
+      <c r="K112" s="4" t="inlineStr"/>
+      <c r="L112" s="4" t="n">
+        <v>50.63</v>
+      </c>
+      <c r="M112" s="4" t="n">
+        <v>1.519</v>
+      </c>
+      <c r="N112" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O112" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P112" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q112" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R112" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S112" s="4" t="n"/>
+      <c r="T112" s="4" t="n"/>
+      <c r="U112" s="4" t="n"/>
+      <c r="V112" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W112" s="4" t="inlineStr"/>
+      <c r="X112" s="4" t="n"/>
+      <c r="Y112" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z112" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA112" s="4" t="n"/>
+      <c r="AB112" s="4" t="n"/>
+      <c r="AC112" s="4" t="n"/>
+      <c r="AD112" s="4" t="n"/>
+      <c r="AE112" s="4" t="n"/>
+      <c r="AF112" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B113" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D113" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E113" s="6" t="n">
+        <v>85.98999999999999</v>
+      </c>
+      <c r="F113" s="6" t="n"/>
+      <c r="G113" s="6" t="n"/>
+      <c r="H113" s="6" t="n">
+        <v>41.54</v>
+      </c>
+      <c r="I113" s="6" t="inlineStr"/>
+      <c r="J113" s="6" t="inlineStr"/>
+      <c r="K113" s="6" t="inlineStr"/>
+      <c r="L113" s="6" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="M113" s="6" t="n">
+        <v>1.731</v>
+      </c>
+      <c r="N113" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O113" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P113" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q113" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R113" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S113" s="6" t="n"/>
+      <c r="T113" s="6" t="n"/>
+      <c r="U113" s="6" t="n"/>
+      <c r="V113" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W113" s="6" t="inlineStr"/>
+      <c r="X113" s="6" t="n"/>
+      <c r="Y113" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z113" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA113" s="6" t="n"/>
+      <c r="AB113" s="6" t="n"/>
+      <c r="AC113" s="6" t="n"/>
+      <c r="AD113" s="6" t="n"/>
+      <c r="AE113" s="6" t="n"/>
+      <c r="AF113" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B114" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C114" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D114" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E114" s="4" t="n">
+        <v>87.98999999999999</v>
+      </c>
+      <c r="F114" s="4" t="n"/>
+      <c r="G114" s="4" t="n"/>
+      <c r="H114" s="4" t="n">
+        <v>35.2</v>
+      </c>
+      <c r="I114" s="4" t="inlineStr"/>
+      <c r="J114" s="4" t="inlineStr"/>
+      <c r="K114" s="4" t="inlineStr"/>
+      <c r="L114" s="4" t="n">
+        <v>48.89</v>
+      </c>
+      <c r="M114" s="4" t="n">
+        <v>1.467</v>
+      </c>
+      <c r="N114" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O114" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P114" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q114" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R114" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S114" s="4" t="n"/>
+      <c r="T114" s="4" t="n"/>
+      <c r="U114" s="4" t="n"/>
+      <c r="V114" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W114" s="4" t="inlineStr"/>
+      <c r="X114" s="4" t="n"/>
+      <c r="Y114" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z114" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA114" s="4" t="n"/>
+      <c r="AB114" s="4" t="n"/>
+      <c r="AC114" s="4" t="n"/>
+      <c r="AD114" s="4" t="n"/>
+      <c r="AE114" s="4" t="n"/>
+      <c r="AF114" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B115" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D115" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E115" s="6" t="n">
+        <v>137.99</v>
+      </c>
+      <c r="F115" s="6" t="n"/>
+      <c r="G115" s="6" t="n"/>
+      <c r="H115" s="6" t="n">
+        <v>38.33</v>
+      </c>
+      <c r="I115" s="6" t="inlineStr"/>
+      <c r="J115" s="6" t="inlineStr"/>
+      <c r="K115" s="6" t="inlineStr"/>
+      <c r="L115" s="6" t="n">
+        <v>53.24</v>
+      </c>
+      <c r="M115" s="6" t="n">
+        <v>1.597</v>
+      </c>
+      <c r="N115" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O115" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P115" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q115" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R115" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S115" s="6" t="n"/>
+      <c r="T115" s="6" t="n"/>
+      <c r="U115" s="6" t="n"/>
+      <c r="V115" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W115" s="6" t="inlineStr"/>
+      <c r="X115" s="6" t="n"/>
+      <c r="Y115" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z115" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA115" s="6" t="n"/>
+      <c r="AB115" s="6" t="n"/>
+      <c r="AC115" s="6" t="n"/>
+      <c r="AD115" s="6" t="n"/>
+      <c r="AE115" s="6" t="n"/>
+      <c r="AF115" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B116" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C116" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D116" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E116" s="4" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="F116" s="4" t="n"/>
+      <c r="G116" s="4" t="n"/>
+      <c r="H116" s="4" t="n">
+        <v>89.72</v>
+      </c>
+      <c r="I116" s="4" t="inlineStr"/>
+      <c r="J116" s="4" t="inlineStr"/>
+      <c r="K116" s="4" t="inlineStr"/>
+      <c r="L116" s="4" t="n">
+        <v>109.41</v>
+      </c>
+      <c r="M116" s="4" t="n">
+        <v>3.282</v>
+      </c>
+      <c r="N116" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O116" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P116" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q116" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R116" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S116" s="4" t="n"/>
+      <c r="T116" s="4" t="n"/>
+      <c r="U116" s="4" t="n"/>
+      <c r="V116" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W116" s="4" t="inlineStr"/>
+      <c r="X116" s="4" t="n"/>
+      <c r="Y116" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z116" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA116" s="4" t="n"/>
+      <c r="AB116" s="4" t="n"/>
+      <c r="AC116" s="4" t="n"/>
+      <c r="AD116" s="4" t="n"/>
+      <c r="AE116" s="4" t="n"/>
+      <c r="AF116" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B117" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C117" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D117" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E117" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F117" s="6" t="n"/>
+      <c r="G117" s="6" t="n"/>
+      <c r="H117" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I117" s="6" t="inlineStr"/>
+      <c r="J117" s="6" t="inlineStr"/>
+      <c r="K117" s="6" t="inlineStr"/>
+      <c r="L117" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M117" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N117" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O117" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P117" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q117" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R117" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S117" s="6" t="n"/>
+      <c r="T117" s="6" t="n"/>
+      <c r="U117" s="6" t="n"/>
+      <c r="V117" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W117" s="6" t="inlineStr"/>
+      <c r="X117" s="6" t="n"/>
+      <c r="Y117" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z117" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA117" s="6" t="n"/>
+      <c r="AB117" s="6" t="n"/>
+      <c r="AC117" s="6" t="n"/>
+      <c r="AD117" s="6" t="n"/>
+      <c r="AE117" s="6" t="n"/>
+      <c r="AF117" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B118" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C118" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D118" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E118" s="4" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="F118" s="4" t="n"/>
+      <c r="G118" s="4" t="n"/>
+      <c r="H118" s="4" t="n">
+        <v>71.78</v>
+      </c>
+      <c r="I118" s="4" t="inlineStr"/>
+      <c r="J118" s="4" t="inlineStr"/>
+      <c r="K118" s="4" t="inlineStr"/>
+      <c r="L118" s="4" t="n">
+        <v>87.54000000000001</v>
+      </c>
+      <c r="M118" s="4" t="n">
+        <v>2.626</v>
+      </c>
+      <c r="N118" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O118" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P118" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q118" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R118" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S118" s="4" t="n"/>
+      <c r="T118" s="4" t="n"/>
+      <c r="U118" s="4" t="n"/>
+      <c r="V118" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W118" s="4" t="inlineStr"/>
+      <c r="X118" s="4" t="n"/>
+      <c r="Y118" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z118" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA118" s="4" t="n"/>
+      <c r="AB118" s="4" t="n"/>
+      <c r="AC118" s="4" t="n"/>
+      <c r="AD118" s="4" t="n"/>
+      <c r="AE118" s="4" t="n"/>
+      <c r="AF118" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B119" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C119" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D119" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E119" s="6" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="F119" s="6" t="n"/>
+      <c r="G119" s="6" t="n"/>
+      <c r="H119" s="6" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="I119" s="6" t="inlineStr"/>
+      <c r="J119" s="6" t="inlineStr"/>
+      <c r="K119" s="6" t="inlineStr"/>
+      <c r="L119" s="6" t="n">
+        <v>80.48</v>
+      </c>
+      <c r="M119" s="6" t="n">
+        <v>2.414</v>
+      </c>
+      <c r="N119" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O119" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P119" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q119" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R119" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S119" s="6" t="n"/>
+      <c r="T119" s="6" t="n"/>
+      <c r="U119" s="6" t="n"/>
+      <c r="V119" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W119" s="6" t="inlineStr"/>
+      <c r="X119" s="6" t="n"/>
+      <c r="Y119" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z119" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA119" s="6" t="n"/>
+      <c r="AB119" s="6" t="n"/>
+      <c r="AC119" s="6" t="n"/>
+      <c r="AD119" s="6" t="n"/>
+      <c r="AE119" s="6" t="n"/>
+      <c r="AF119" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D120" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E120" s="4" t="n">
+        <v>132.99</v>
+      </c>
+      <c r="F120" s="4" t="n"/>
+      <c r="G120" s="4" t="n"/>
+      <c r="H120" s="4" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="I120" s="4" t="inlineStr"/>
+      <c r="J120" s="4" t="inlineStr"/>
+      <c r="K120" s="4" t="inlineStr"/>
+      <c r="L120" s="4" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="M120" s="4" t="n">
+        <v>1.946</v>
+      </c>
+      <c r="N120" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O120" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P120" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q120" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R120" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S120" s="4" t="n"/>
+      <c r="T120" s="4" t="n"/>
+      <c r="U120" s="4" t="n"/>
+      <c r="V120" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W120" s="4" t="inlineStr"/>
+      <c r="X120" s="4" t="n"/>
+      <c r="Y120" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z120" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA120" s="4" t="n"/>
+      <c r="AB120" s="4" t="n"/>
+      <c r="AC120" s="4" t="n"/>
+      <c r="AD120" s="4" t="n"/>
+      <c r="AE120" s="4" t="n"/>
+      <c r="AF120" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B121" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C121" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D121" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E121" s="6" t="n">
+        <v>155.99</v>
+      </c>
+      <c r="F121" s="6" t="n"/>
+      <c r="G121" s="6" t="n"/>
+      <c r="H121" s="6" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="I121" s="6" t="inlineStr"/>
+      <c r="J121" s="6" t="inlineStr"/>
+      <c r="K121" s="6" t="inlineStr"/>
+      <c r="L121" s="6" t="n">
+        <v>70.45</v>
+      </c>
+      <c r="M121" s="6" t="n">
+        <v>2.114</v>
+      </c>
+      <c r="N121" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O121" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P121" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q121" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R121" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S121" s="6" t="n"/>
+      <c r="T121" s="6" t="n"/>
+      <c r="U121" s="6" t="n"/>
+      <c r="V121" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W121" s="6" t="inlineStr"/>
+      <c r="X121" s="6" t="n"/>
+      <c r="Y121" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z121" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA121" s="6" t="n"/>
+      <c r="AB121" s="6" t="n"/>
+      <c r="AC121" s="6" t="n"/>
+      <c r="AD121" s="6" t="n"/>
+      <c r="AE121" s="6" t="n"/>
+      <c r="AF121" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B122" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C122" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D122" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E122" s="4" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="F122" s="4" t="n"/>
+      <c r="G122" s="4" t="n"/>
+      <c r="H122" s="4" t="n">
+        <v>59.52</v>
+      </c>
+      <c r="I122" s="4" t="inlineStr"/>
+      <c r="J122" s="4" t="inlineStr"/>
+      <c r="K122" s="4" t="inlineStr"/>
+      <c r="L122" s="4" t="n">
+        <v>72.59</v>
+      </c>
+      <c r="M122" s="4" t="n">
+        <v>2.178</v>
+      </c>
+      <c r="N122" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O122" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P122" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q122" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R122" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S122" s="4" t="n"/>
+      <c r="T122" s="4" t="n"/>
+      <c r="U122" s="4" t="n"/>
+      <c r="V122" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W122" s="4" t="inlineStr"/>
+      <c r="X122" s="4" t="n"/>
+      <c r="Y122" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z122" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA122" s="4" t="n"/>
+      <c r="AB122" s="4" t="n"/>
+      <c r="AC122" s="4" t="n"/>
+      <c r="AD122" s="4" t="n"/>
+      <c r="AE122" s="4" t="n"/>
+      <c r="AF122" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B123" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C123" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D123" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E123" s="6" t="n">
+        <v>30.39</v>
+      </c>
+      <c r="F123" s="6" t="n"/>
+      <c r="G123" s="6" t="n"/>
+      <c r="H123" s="6" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="I123" s="6" t="inlineStr"/>
+      <c r="J123" s="6" t="inlineStr"/>
+      <c r="K123" s="6" t="inlineStr"/>
+      <c r="L123" s="6" t="n">
+        <v>91.59</v>
+      </c>
+      <c r="M123" s="6" t="n">
+        <v>2.748</v>
+      </c>
+      <c r="N123" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O123" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P123" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q123" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R123" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S123" s="6" t="n"/>
+      <c r="T123" s="6" t="n"/>
+      <c r="U123" s="6" t="n"/>
+      <c r="V123" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W123" s="6" t="inlineStr"/>
+      <c r="X123" s="6" t="n"/>
+      <c r="Y123" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z123" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA123" s="6" t="n"/>
+      <c r="AB123" s="6" t="n"/>
+      <c r="AC123" s="6" t="n"/>
+      <c r="AD123" s="6" t="n"/>
+      <c r="AE123" s="6" t="n"/>
+      <c r="AF123" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B124" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C124" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D124" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E124" s="4" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="F124" s="4" t="n"/>
+      <c r="G124" s="4" t="n"/>
+      <c r="H124" s="4" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="I124" s="4" t="inlineStr"/>
+      <c r="J124" s="4" t="inlineStr"/>
+      <c r="K124" s="4" t="inlineStr"/>
+      <c r="L124" s="4" t="n">
+        <v>70.86</v>
+      </c>
+      <c r="M124" s="4" t="n">
+        <v>2.126</v>
+      </c>
+      <c r="N124" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O124" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P124" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q124" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R124" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S124" s="4" t="n"/>
+      <c r="T124" s="4" t="n"/>
+      <c r="U124" s="4" t="n"/>
+      <c r="V124" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W124" s="4" t="inlineStr"/>
+      <c r="X124" s="4" t="n"/>
+      <c r="Y124" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z124" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA124" s="4" t="n"/>
+      <c r="AB124" s="4" t="n"/>
+      <c r="AC124" s="4" t="n"/>
+      <c r="AD124" s="4" t="n"/>
+      <c r="AE124" s="4" t="n"/>
+      <c r="AF124" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D125" s="6" t="inlineStr">
+        <is>
+          <t>910g</t>
+        </is>
+      </c>
+      <c r="E125" s="6" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F125" s="6" t="n"/>
+      <c r="G125" s="6" t="n"/>
+      <c r="H125" s="6" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="I125" s="6" t="inlineStr"/>
+      <c r="J125" s="6" t="inlineStr"/>
+      <c r="K125" s="6" t="inlineStr"/>
+      <c r="L125" s="6" t="n">
+        <v>69.53</v>
+      </c>
+      <c r="M125" s="6" t="n">
+        <v>2.086</v>
+      </c>
+      <c r="N125" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O125" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P125" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q125" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R125" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S125" s="6" t="n"/>
+      <c r="T125" s="6" t="n"/>
+      <c r="U125" s="6" t="n"/>
+      <c r="V125" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W125" s="6" t="inlineStr"/>
+      <c r="X125" s="6" t="n"/>
+      <c r="Y125" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z125" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA125" s="6" t="n"/>
+      <c r="AB125" s="6" t="n"/>
+      <c r="AC125" s="6" t="n"/>
+      <c r="AD125" s="6" t="n"/>
+      <c r="AE125" s="6" t="n"/>
+      <c r="AF125" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B126" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C126" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D126" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E126" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F126" s="4" t="n"/>
+      <c r="G126" s="4" t="n"/>
+      <c r="H126" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="I126" s="4" t="inlineStr"/>
+      <c r="J126" s="4" t="inlineStr"/>
+      <c r="K126" s="4" t="inlineStr"/>
+      <c r="L126" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M126" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N126" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O126" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P126" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q126" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R126" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S126" s="4" t="n"/>
+      <c r="T126" s="4" t="n"/>
+      <c r="U126" s="4" t="n"/>
+      <c r="V126" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W126" s="4" t="inlineStr"/>
+      <c r="X126" s="4" t="n"/>
+      <c r="Y126" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z126" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA126" s="4" t="n"/>
+      <c r="AB126" s="4" t="n"/>
+      <c r="AC126" s="4" t="n"/>
+      <c r="AD126" s="4" t="n"/>
+      <c r="AE126" s="4" t="n"/>
+      <c r="AF126" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B127" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C127" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D127" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E127" s="6" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="F127" s="6" t="n"/>
+      <c r="G127" s="6" t="n"/>
+      <c r="H127" s="6" t="n">
+        <v>37.12</v>
+      </c>
+      <c r="I127" s="6" t="inlineStr"/>
+      <c r="J127" s="6" t="inlineStr"/>
+      <c r="K127" s="6" t="inlineStr"/>
+      <c r="L127" s="6" t="n">
+        <v>62.92</v>
+      </c>
+      <c r="M127" s="6" t="n">
+        <v>1.888</v>
+      </c>
+      <c r="N127" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O127" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P127" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q127" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R127" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S127" s="6" t="n"/>
+      <c r="T127" s="6" t="n"/>
+      <c r="U127" s="6" t="n"/>
+      <c r="V127" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W127" s="6" t="inlineStr"/>
+      <c r="X127" s="6" t="n"/>
+      <c r="Y127" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z127" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA127" s="6" t="n"/>
+      <c r="AB127" s="6" t="n"/>
+      <c r="AC127" s="6" t="n"/>
+      <c r="AD127" s="6" t="n"/>
+      <c r="AE127" s="6" t="n"/>
+      <c r="AF127" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B128" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C128" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D128" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E128" s="4" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="F128" s="4" t="n"/>
+      <c r="G128" s="4" t="n"/>
+      <c r="H128" s="4" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="I128" s="4" t="inlineStr"/>
+      <c r="J128" s="4" t="inlineStr"/>
+      <c r="K128" s="4" t="inlineStr"/>
+      <c r="L128" s="4" t="n">
+        <v>56.17</v>
+      </c>
+      <c r="M128" s="4" t="n">
+        <v>1.685</v>
+      </c>
+      <c r="N128" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O128" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P128" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q128" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R128" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S128" s="4" t="n"/>
+      <c r="T128" s="4" t="n"/>
+      <c r="U128" s="4" t="n"/>
+      <c r="V128" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W128" s="4" t="inlineStr"/>
+      <c r="X128" s="4" t="n"/>
+      <c r="Y128" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z128" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA128" s="4" t="n"/>
+      <c r="AB128" s="4" t="n"/>
+      <c r="AC128" s="4" t="n"/>
+      <c r="AD128" s="4" t="n"/>
+      <c r="AE128" s="4" t="n"/>
+      <c r="AF128" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B129" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C129" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D129" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E129" s="6" t="n">
+        <v>74.73999999999999</v>
+      </c>
+      <c r="F129" s="6" t="n"/>
+      <c r="G129" s="6" t="n"/>
+      <c r="H129" s="6" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I129" s="6" t="inlineStr"/>
+      <c r="J129" s="6" t="inlineStr"/>
+      <c r="K129" s="6" t="inlineStr"/>
+      <c r="L129" s="6" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M129" s="6" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="N129" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O129" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P129" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q129" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R129" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S129" s="6" t="n"/>
+      <c r="T129" s="6" t="n"/>
+      <c r="U129" s="6" t="n"/>
+      <c r="V129" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W129" s="6" t="inlineStr"/>
+      <c r="X129" s="6" t="n"/>
+      <c r="Y129" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z129" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA129" s="6" t="n"/>
+      <c r="AB129" s="6" t="n"/>
+      <c r="AC129" s="6" t="n"/>
+      <c r="AD129" s="6" t="n"/>
+      <c r="AE129" s="6" t="n"/>
+      <c r="AF129" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B130" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C130" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D130" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E130" s="4" t="n">
+        <v>139.74</v>
+      </c>
+      <c r="F130" s="4" t="n"/>
+      <c r="G130" s="4" t="n"/>
+      <c r="H130" s="4" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="I130" s="4" t="inlineStr"/>
+      <c r="J130" s="4" t="inlineStr"/>
+      <c r="K130" s="4" t="inlineStr"/>
+      <c r="L130" s="4" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="M130" s="4" t="n">
+        <v>1.421</v>
+      </c>
+      <c r="N130" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O130" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P130" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q130" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R130" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S130" s="4" t="n"/>
+      <c r="T130" s="4" t="n"/>
+      <c r="U130" s="4" t="n"/>
+      <c r="V130" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W130" s="4" t="inlineStr"/>
+      <c r="X130" s="4" t="n"/>
+      <c r="Y130" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z130" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA130" s="4" t="n"/>
+      <c r="AB130" s="4" t="n"/>
+      <c r="AC130" s="4" t="n"/>
+      <c r="AD130" s="4" t="n"/>
+      <c r="AE130" s="4" t="n"/>
+      <c r="AF130" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C131" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D131" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E131" s="6" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="F131" s="6" t="n"/>
+      <c r="G131" s="6" t="n"/>
+      <c r="H131" s="6" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="I131" s="6" t="inlineStr"/>
+      <c r="J131" s="6" t="inlineStr"/>
+      <c r="K131" s="6" t="inlineStr"/>
+      <c r="L131" s="6" t="n"/>
+      <c r="M131" s="6" t="n"/>
+      <c r="N131" s="6" t="n"/>
+      <c r="O131" s="6" t="n"/>
+      <c r="P131" s="6" t="n"/>
+      <c r="Q131" s="6" t="n"/>
+      <c r="R131" s="6" t="n"/>
+      <c r="S131" s="6" t="n"/>
+      <c r="T131" s="6" t="n"/>
+      <c r="U131" s="6" t="n"/>
+      <c r="V131" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W131" s="6" t="inlineStr"/>
+      <c r="X131" s="6" t="n"/>
+      <c r="Y131" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z131" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA131" s="6" t="n"/>
+      <c r="AB131" s="6" t="n"/>
+      <c r="AC131" s="6" t="n"/>
+      <c r="AD131" s="6" t="n"/>
+      <c r="AE131" s="6" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="AF131" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B132" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C132" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D132" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E132" s="4" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="F132" s="4" t="n"/>
+      <c r="G132" s="4" t="n"/>
+      <c r="H132" s="4" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="I132" s="4" t="inlineStr"/>
+      <c r="J132" s="4" t="inlineStr"/>
+      <c r="K132" s="4" t="inlineStr"/>
+      <c r="L132" s="4" t="n"/>
+      <c r="M132" s="4" t="n"/>
+      <c r="N132" s="4" t="n"/>
+      <c r="O132" s="4" t="n"/>
+      <c r="P132" s="4" t="n"/>
+      <c r="Q132" s="4" t="n"/>
+      <c r="R132" s="4" t="n"/>
+      <c r="S132" s="4" t="n"/>
+      <c r="T132" s="4" t="n"/>
+      <c r="U132" s="4" t="n"/>
+      <c r="V132" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W132" s="4" t="inlineStr"/>
+      <c r="X132" s="4" t="n"/>
+      <c r="Y132" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z132" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA132" s="4" t="n"/>
+      <c r="AB132" s="4" t="n"/>
+      <c r="AC132" s="4" t="n"/>
+      <c r="AD132" s="4" t="n"/>
+      <c r="AE132" s="4" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="AF132" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B133" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C133" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D133" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E133" s="6" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="F133" s="6" t="n"/>
+      <c r="G133" s="6" t="n"/>
+      <c r="H133" s="6" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="I133" s="6" t="inlineStr"/>
+      <c r="J133" s="6" t="inlineStr"/>
+      <c r="K133" s="6" t="inlineStr"/>
+      <c r="L133" s="6" t="n"/>
+      <c r="M133" s="6" t="n"/>
+      <c r="N133" s="6" t="n"/>
+      <c r="O133" s="6" t="n"/>
+      <c r="P133" s="6" t="n"/>
+      <c r="Q133" s="6" t="n"/>
+      <c r="R133" s="6" t="n"/>
+      <c r="S133" s="6" t="n"/>
+      <c r="T133" s="6" t="n"/>
+      <c r="U133" s="6" t="n"/>
+      <c r="V133" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W133" s="6" t="inlineStr"/>
+      <c r="X133" s="6" t="n"/>
+      <c r="Y133" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z133" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA133" s="6" t="n"/>
+      <c r="AB133" s="6" t="n"/>
+      <c r="AC133" s="6" t="n"/>
+      <c r="AD133" s="6" t="n"/>
+      <c r="AE133" s="6" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="AF133" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B134" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C134" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D134" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E134" s="4" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="F134" s="4" t="n"/>
+      <c r="G134" s="4" t="n"/>
+      <c r="H134" s="4" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="I134" s="4" t="inlineStr"/>
+      <c r="J134" s="4" t="inlineStr"/>
+      <c r="K134" s="4" t="inlineStr"/>
+      <c r="L134" s="4" t="n"/>
+      <c r="M134" s="4" t="n"/>
+      <c r="N134" s="4" t="n"/>
+      <c r="O134" s="4" t="n"/>
+      <c r="P134" s="4" t="n"/>
+      <c r="Q134" s="4" t="n"/>
+      <c r="R134" s="4" t="n"/>
+      <c r="S134" s="4" t="n"/>
+      <c r="T134" s="4" t="n"/>
+      <c r="U134" s="4" t="n"/>
+      <c r="V134" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W134" s="4" t="inlineStr"/>
+      <c r="X134" s="4" t="n"/>
+      <c r="Y134" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z134" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA134" s="4" t="n"/>
+      <c r="AB134" s="4" t="n"/>
+      <c r="AC134" s="4" t="n"/>
+      <c r="AD134" s="4" t="n"/>
+      <c r="AE134" s="4" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="AF134" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B135" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C135" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D135" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E135" s="6" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="F135" s="6" t="n"/>
+      <c r="G135" s="6" t="n"/>
+      <c r="H135" s="6" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="I135" s="6" t="inlineStr"/>
+      <c r="J135" s="6" t="inlineStr"/>
+      <c r="K135" s="6" t="inlineStr"/>
+      <c r="L135" s="6" t="n"/>
+      <c r="M135" s="6" t="n"/>
+      <c r="N135" s="6" t="n"/>
+      <c r="O135" s="6" t="n"/>
+      <c r="P135" s="6" t="n"/>
+      <c r="Q135" s="6" t="n"/>
+      <c r="R135" s="6" t="n"/>
+      <c r="S135" s="6" t="n"/>
+      <c r="T135" s="6" t="n"/>
+      <c r="U135" s="6" t="n"/>
+      <c r="V135" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W135" s="6" t="inlineStr"/>
+      <c r="X135" s="6" t="n"/>
+      <c r="Y135" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z135" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA135" s="6" t="n"/>
+      <c r="AB135" s="6" t="n"/>
+      <c r="AC135" s="6" t="n"/>
+      <c r="AD135" s="6" t="n"/>
+      <c r="AE135" s="6" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="AF135" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B136" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C136" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D136" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E136" s="4" t="n">
+        <v>42.99</v>
+      </c>
+      <c r="F136" s="4" t="n"/>
+      <c r="G136" s="4" t="n"/>
+      <c r="H136" s="4" t="n">
+        <v>85.98</v>
+      </c>
+      <c r="I136" s="4" t="inlineStr"/>
+      <c r="J136" s="4" t="inlineStr"/>
+      <c r="K136" s="4" t="inlineStr"/>
+      <c r="L136" s="4" t="n"/>
+      <c r="M136" s="4" t="n"/>
+      <c r="N136" s="4" t="n"/>
+      <c r="O136" s="4" t="n"/>
+      <c r="P136" s="4" t="n"/>
+      <c r="Q136" s="4" t="n"/>
+      <c r="R136" s="4" t="n"/>
+      <c r="S136" s="4" t="n"/>
+      <c r="T136" s="4" t="n"/>
+      <c r="U136" s="4" t="n"/>
+      <c r="V136" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W136" s="4" t="inlineStr"/>
+      <c r="X136" s="4" t="n"/>
+      <c r="Y136" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z136" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA136" s="4" t="n"/>
+      <c r="AB136" s="4" t="n"/>
+      <c r="AC136" s="4" t="n"/>
+      <c r="AD136" s="4" t="n"/>
+      <c r="AE136" s="4" t="n">
+        <v>85.98</v>
+      </c>
+      <c r="AF136" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B137" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C137" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D137" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E137" s="6" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="F137" s="6" t="n"/>
+      <c r="G137" s="6" t="n"/>
+      <c r="H137" s="6" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="I137" s="6" t="inlineStr"/>
+      <c r="J137" s="6" t="inlineStr"/>
+      <c r="K137" s="6" t="inlineStr"/>
+      <c r="L137" s="6" t="n"/>
+      <c r="M137" s="6" t="n"/>
+      <c r="N137" s="6" t="n"/>
+      <c r="O137" s="6" t="n"/>
+      <c r="P137" s="6" t="n"/>
+      <c r="Q137" s="6" t="n"/>
+      <c r="R137" s="6" t="n"/>
+      <c r="S137" s="6" t="n"/>
+      <c r="T137" s="6" t="n"/>
+      <c r="U137" s="6" t="n"/>
+      <c r="V137" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W137" s="6" t="inlineStr"/>
+      <c r="X137" s="6" t="n"/>
+      <c r="Y137" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z137" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA137" s="6" t="n"/>
+      <c r="AB137" s="6" t="n"/>
+      <c r="AC137" s="6" t="n"/>
+      <c r="AD137" s="6" t="n"/>
+      <c r="AE137" s="6" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="AF137" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B138" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C138" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D138" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E138" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F138" s="4" t="n"/>
+      <c r="G138" s="4" t="n"/>
+      <c r="H138" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I138" s="4" t="inlineStr"/>
+      <c r="J138" s="4" t="inlineStr"/>
+      <c r="K138" s="4" t="inlineStr"/>
+      <c r="L138" s="4" t="n"/>
+      <c r="M138" s="4" t="n"/>
+      <c r="N138" s="4" t="n"/>
+      <c r="O138" s="4" t="n"/>
+      <c r="P138" s="4" t="n"/>
+      <c r="Q138" s="4" t="n"/>
+      <c r="R138" s="4" t="n"/>
+      <c r="S138" s="4" t="n"/>
+      <c r="T138" s="4" t="n"/>
+      <c r="U138" s="4" t="n"/>
+      <c r="V138" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W138" s="4" t="inlineStr"/>
+      <c r="X138" s="4" t="n"/>
+      <c r="Y138" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z138" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA138" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB138" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC138" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD138" s="4" t="n"/>
+      <c r="AE138" s="4" t="n"/>
+      <c r="AF138" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B139" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C139" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D139" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E139" s="6" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="F139" s="6" t="n"/>
+      <c r="G139" s="6" t="n"/>
+      <c r="H139" s="6" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="I139" s="6" t="inlineStr"/>
+      <c r="J139" s="6" t="inlineStr"/>
+      <c r="K139" s="6" t="inlineStr"/>
+      <c r="L139" s="6" t="n"/>
+      <c r="M139" s="6" t="n"/>
+      <c r="N139" s="6" t="n"/>
+      <c r="O139" s="6" t="n"/>
+      <c r="P139" s="6" t="n"/>
+      <c r="Q139" s="6" t="n"/>
+      <c r="R139" s="6" t="n"/>
+      <c r="S139" s="6" t="n"/>
+      <c r="T139" s="6" t="n"/>
+      <c r="U139" s="6" t="n"/>
+      <c r="V139" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W139" s="6" t="inlineStr"/>
+      <c r="X139" s="6" t="n"/>
+      <c r="Y139" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z139" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA139" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB139" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC139" s="6" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AD139" s="6" t="n"/>
+      <c r="AE139" s="6" t="n"/>
+      <c r="AF139" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B140" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C140" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D140" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E140" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F140" s="4" t="n"/>
+      <c r="G140" s="4" t="n"/>
+      <c r="H140" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I140" s="4" t="inlineStr"/>
+      <c r="J140" s="4" t="inlineStr"/>
+      <c r="K140" s="4" t="inlineStr"/>
+      <c r="L140" s="4" t="n"/>
+      <c r="M140" s="4" t="n"/>
+      <c r="N140" s="4" t="n"/>
+      <c r="O140" s="4" t="n"/>
+      <c r="P140" s="4" t="n"/>
+      <c r="Q140" s="4" t="n"/>
+      <c r="R140" s="4" t="n"/>
+      <c r="S140" s="4" t="n"/>
+      <c r="T140" s="4" t="n"/>
+      <c r="U140" s="4" t="n"/>
+      <c r="V140" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W140" s="4" t="inlineStr"/>
+      <c r="X140" s="4" t="n"/>
+      <c r="Y140" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z140" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA140" s="4" t="n"/>
+      <c r="AB140" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC140" s="4" t="n"/>
+      <c r="AD140" s="4" t="n"/>
+      <c r="AE140" s="4" t="n"/>
+      <c r="AF140" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-22</t>
+        </is>
+      </c>
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D141" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E141" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F141" s="6" t="n"/>
+      <c r="G141" s="6" t="n"/>
+      <c r="H141" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I141" s="6" t="inlineStr"/>
+      <c r="J141" s="6" t="inlineStr"/>
+      <c r="K141" s="6" t="inlineStr"/>
+      <c r="L141" s="6" t="n"/>
+      <c r="M141" s="6" t="n"/>
+      <c r="N141" s="6" t="n"/>
+      <c r="O141" s="6" t="n"/>
+      <c r="P141" s="6" t="n"/>
+      <c r="Q141" s="6" t="n"/>
+      <c r="R141" s="6" t="n"/>
+      <c r="S141" s="6" t="n"/>
+      <c r="T141" s="6" t="n"/>
+      <c r="U141" s="6" t="n"/>
+      <c r="V141" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W141" s="6" t="inlineStr"/>
+      <c r="X141" s="6" t="n"/>
+      <c r="Y141" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z141" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA141" s="6" t="n"/>
+      <c r="AB141" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC141" s="6" t="n"/>
+      <c r="AD141" s="6" t="n"/>
+      <c r="AE141" s="6" t="n"/>
+      <c r="AF141" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-23
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF141"/>
+  <dimension ref="A1:AF178"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11658,6 +11658,2918 @@
         <v>1</v>
       </c>
     </row>
+    <row r="142">
+      <c r="A142" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B142" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C142" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D142" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E142" s="4" t="n">
+        <v>13.29</v>
+      </c>
+      <c r="F142" s="4" t="n"/>
+      <c r="G142" s="4" t="n"/>
+      <c r="H142" s="4" t="n">
+        <v>53.16</v>
+      </c>
+      <c r="I142" s="4" t="inlineStr"/>
+      <c r="J142" s="4" t="inlineStr"/>
+      <c r="K142" s="4" t="inlineStr"/>
+      <c r="L142" s="4" t="n">
+        <v>73.83</v>
+      </c>
+      <c r="M142" s="4" t="n">
+        <v>2.215</v>
+      </c>
+      <c r="N142" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O142" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P142" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q142" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R142" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S142" s="4" t="n"/>
+      <c r="T142" s="4" t="n"/>
+      <c r="U142" s="4" t="n"/>
+      <c r="V142" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W142" s="4" t="inlineStr"/>
+      <c r="X142" s="4" t="n"/>
+      <c r="Y142" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z142" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA142" s="4" t="n"/>
+      <c r="AB142" s="4" t="n"/>
+      <c r="AC142" s="4" t="n"/>
+      <c r="AD142" s="4" t="n"/>
+      <c r="AE142" s="4" t="n"/>
+      <c r="AF142" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B143" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D143" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E143" s="6" t="n">
+        <v>18.99</v>
+      </c>
+      <c r="F143" s="6" t="n"/>
+      <c r="G143" s="6" t="n"/>
+      <c r="H143" s="6" t="n">
+        <v>55.04</v>
+      </c>
+      <c r="I143" s="6" t="inlineStr"/>
+      <c r="J143" s="6" t="inlineStr"/>
+      <c r="K143" s="6" t="inlineStr"/>
+      <c r="L143" s="6" t="n">
+        <v>76.44</v>
+      </c>
+      <c r="M143" s="6" t="n">
+        <v>2.293</v>
+      </c>
+      <c r="N143" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O143" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P143" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q143" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R143" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S143" s="6" t="n"/>
+      <c r="T143" s="6" t="n"/>
+      <c r="U143" s="6" t="n"/>
+      <c r="V143" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W143" s="6" t="inlineStr"/>
+      <c r="X143" s="6" t="n"/>
+      <c r="Y143" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z143" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA143" s="6" t="n"/>
+      <c r="AB143" s="6" t="n"/>
+      <c r="AC143" s="6" t="n"/>
+      <c r="AD143" s="6" t="n"/>
+      <c r="AE143" s="6" t="n"/>
+      <c r="AF143" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B144" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C144" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D144" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E144" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F144" s="4" t="n"/>
+      <c r="G144" s="4" t="n"/>
+      <c r="H144" s="4" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="I144" s="4" t="inlineStr"/>
+      <c r="J144" s="4" t="inlineStr"/>
+      <c r="K144" s="4" t="inlineStr"/>
+      <c r="L144" s="4" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="M144" s="4" t="n">
+        <v>1.749</v>
+      </c>
+      <c r="N144" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O144" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P144" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q144" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R144" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S144" s="4" t="n"/>
+      <c r="T144" s="4" t="n"/>
+      <c r="U144" s="4" t="n"/>
+      <c r="V144" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W144" s="4" t="inlineStr"/>
+      <c r="X144" s="4" t="n"/>
+      <c r="Y144" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z144" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA144" s="4" t="n"/>
+      <c r="AB144" s="4" t="n"/>
+      <c r="AC144" s="4" t="n"/>
+      <c r="AD144" s="4" t="n"/>
+      <c r="AE144" s="4" t="n"/>
+      <c r="AF144" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B145" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C145" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D145" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E145" s="6" t="n">
+        <v>25.19</v>
+      </c>
+      <c r="F145" s="6" t="n"/>
+      <c r="G145" s="6" t="n"/>
+      <c r="H145" s="6" t="n">
+        <v>41.98</v>
+      </c>
+      <c r="I145" s="6" t="inlineStr"/>
+      <c r="J145" s="6" t="inlineStr"/>
+      <c r="K145" s="6" t="inlineStr"/>
+      <c r="L145" s="6" t="n">
+        <v>58.31</v>
+      </c>
+      <c r="M145" s="6" t="n">
+        <v>1.749</v>
+      </c>
+      <c r="N145" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O145" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P145" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q145" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R145" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S145" s="6" t="n"/>
+      <c r="T145" s="6" t="n"/>
+      <c r="U145" s="6" t="n"/>
+      <c r="V145" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W145" s="6" t="inlineStr"/>
+      <c r="X145" s="6" t="n"/>
+      <c r="Y145" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z145" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA145" s="6" t="n"/>
+      <c r="AB145" s="6" t="n"/>
+      <c r="AC145" s="6" t="n"/>
+      <c r="AD145" s="6" t="n"/>
+      <c r="AE145" s="6" t="n"/>
+      <c r="AF145" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B146" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C146" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D146" s="4" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E146" s="4" t="n">
+        <v>25.99</v>
+      </c>
+      <c r="F146" s="4" t="n"/>
+      <c r="G146" s="4" t="n"/>
+      <c r="H146" s="4" t="n">
+        <v>41.58</v>
+      </c>
+      <c r="I146" s="4" t="inlineStr"/>
+      <c r="J146" s="4" t="inlineStr"/>
+      <c r="K146" s="4" t="inlineStr"/>
+      <c r="L146" s="4" t="n">
+        <v>57.75</v>
+      </c>
+      <c r="M146" s="4" t="n">
+        <v>1.732</v>
+      </c>
+      <c r="N146" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O146" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P146" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q146" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R146" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S146" s="4" t="n"/>
+      <c r="T146" s="4" t="n"/>
+      <c r="U146" s="4" t="n"/>
+      <c r="V146" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W146" s="4" t="inlineStr"/>
+      <c r="X146" s="4" t="n"/>
+      <c r="Y146" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z146" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA146" s="4" t="n"/>
+      <c r="AB146" s="4" t="n"/>
+      <c r="AC146" s="4" t="n"/>
+      <c r="AD146" s="4" t="n"/>
+      <c r="AE146" s="4" t="n"/>
+      <c r="AF146" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B147" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C147" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D147" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E147" s="6" t="n">
+        <v>30.99</v>
+      </c>
+      <c r="F147" s="6" t="n"/>
+      <c r="G147" s="6" t="n"/>
+      <c r="H147" s="6" t="n">
+        <v>41.32</v>
+      </c>
+      <c r="I147" s="6" t="inlineStr"/>
+      <c r="J147" s="6" t="inlineStr"/>
+      <c r="K147" s="6" t="inlineStr"/>
+      <c r="L147" s="6" t="n">
+        <v>57.39</v>
+      </c>
+      <c r="M147" s="6" t="n">
+        <v>1.722</v>
+      </c>
+      <c r="N147" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O147" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P147" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q147" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R147" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S147" s="6" t="n"/>
+      <c r="T147" s="6" t="n"/>
+      <c r="U147" s="6" t="n"/>
+      <c r="V147" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W147" s="6" t="inlineStr"/>
+      <c r="X147" s="6" t="n"/>
+      <c r="Y147" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z147" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA147" s="6" t="n"/>
+      <c r="AB147" s="6" t="n"/>
+      <c r="AC147" s="6" t="n"/>
+      <c r="AD147" s="6" t="n"/>
+      <c r="AE147" s="6" t="n"/>
+      <c r="AF147" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B148" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C148" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D148" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E148" s="4" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="F148" s="4" t="n"/>
+      <c r="G148" s="4" t="n"/>
+      <c r="H148" s="4" t="n">
+        <v>38.01</v>
+      </c>
+      <c r="I148" s="4" t="inlineStr"/>
+      <c r="J148" s="4" t="inlineStr"/>
+      <c r="K148" s="4" t="inlineStr"/>
+      <c r="L148" s="4" t="n">
+        <v>52.79</v>
+      </c>
+      <c r="M148" s="4" t="n">
+        <v>1.584</v>
+      </c>
+      <c r="N148" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O148" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P148" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q148" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R148" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S148" s="4" t="n"/>
+      <c r="T148" s="4" t="n"/>
+      <c r="U148" s="4" t="n"/>
+      <c r="V148" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W148" s="4" t="inlineStr"/>
+      <c r="X148" s="4" t="n"/>
+      <c r="Y148" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z148" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA148" s="4" t="n"/>
+      <c r="AB148" s="4" t="n"/>
+      <c r="AC148" s="4" t="n"/>
+      <c r="AD148" s="4" t="n"/>
+      <c r="AE148" s="4" t="n"/>
+      <c r="AF148" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B149" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C149" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D149" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E149" s="6" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="F149" s="6" t="n"/>
+      <c r="G149" s="6" t="n"/>
+      <c r="H149" s="6" t="n">
+        <v>36.49</v>
+      </c>
+      <c r="I149" s="6" t="inlineStr"/>
+      <c r="J149" s="6" t="inlineStr"/>
+      <c r="K149" s="6" t="inlineStr"/>
+      <c r="L149" s="6" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M149" s="6" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="N149" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O149" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P149" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q149" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R149" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S149" s="6" t="n"/>
+      <c r="T149" s="6" t="n"/>
+      <c r="U149" s="6" t="n"/>
+      <c r="V149" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W149" s="6" t="inlineStr"/>
+      <c r="X149" s="6" t="n"/>
+      <c r="Y149" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z149" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA149" s="6" t="n"/>
+      <c r="AB149" s="6" t="n"/>
+      <c r="AC149" s="6" t="n"/>
+      <c r="AD149" s="6" t="n"/>
+      <c r="AE149" s="6" t="n"/>
+      <c r="AF149" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B150" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C150" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D150" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E150" s="4" t="n">
+        <v>69.98999999999999</v>
+      </c>
+      <c r="F150" s="4" t="n"/>
+      <c r="G150" s="4" t="n"/>
+      <c r="H150" s="4" t="n">
+        <v>36.45</v>
+      </c>
+      <c r="I150" s="4" t="inlineStr"/>
+      <c r="J150" s="4" t="inlineStr"/>
+      <c r="K150" s="4" t="inlineStr"/>
+      <c r="L150" s="4" t="n">
+        <v>50.63</v>
+      </c>
+      <c r="M150" s="4" t="n">
+        <v>1.519</v>
+      </c>
+      <c r="N150" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O150" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P150" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q150" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R150" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S150" s="4" t="n"/>
+      <c r="T150" s="4" t="n"/>
+      <c r="U150" s="4" t="n"/>
+      <c r="V150" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W150" s="4" t="inlineStr"/>
+      <c r="X150" s="4" t="n"/>
+      <c r="Y150" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z150" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA150" s="4" t="n"/>
+      <c r="AB150" s="4" t="n"/>
+      <c r="AC150" s="4" t="n"/>
+      <c r="AD150" s="4" t="n"/>
+      <c r="AE150" s="4" t="n"/>
+      <c r="AF150" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B151" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C151" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D151" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E151" s="6" t="n">
+        <v>85.98999999999999</v>
+      </c>
+      <c r="F151" s="6" t="n"/>
+      <c r="G151" s="6" t="n"/>
+      <c r="H151" s="6" t="n">
+        <v>41.54</v>
+      </c>
+      <c r="I151" s="6" t="inlineStr"/>
+      <c r="J151" s="6" t="inlineStr"/>
+      <c r="K151" s="6" t="inlineStr"/>
+      <c r="L151" s="6" t="n">
+        <v>57.69</v>
+      </c>
+      <c r="M151" s="6" t="n">
+        <v>1.731</v>
+      </c>
+      <c r="N151" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O151" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P151" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q151" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R151" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S151" s="6" t="n"/>
+      <c r="T151" s="6" t="n"/>
+      <c r="U151" s="6" t="n"/>
+      <c r="V151" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W151" s="6" t="inlineStr"/>
+      <c r="X151" s="6" t="n"/>
+      <c r="Y151" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z151" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA151" s="6" t="n"/>
+      <c r="AB151" s="6" t="n"/>
+      <c r="AC151" s="6" t="n"/>
+      <c r="AD151" s="6" t="n"/>
+      <c r="AE151" s="6" t="n"/>
+      <c r="AF151" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B152" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C152" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D152" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E152" s="4" t="n">
+        <v>137.99</v>
+      </c>
+      <c r="F152" s="4" t="n"/>
+      <c r="G152" s="4" t="n"/>
+      <c r="H152" s="4" t="n">
+        <v>38.33</v>
+      </c>
+      <c r="I152" s="4" t="inlineStr"/>
+      <c r="J152" s="4" t="inlineStr"/>
+      <c r="K152" s="4" t="inlineStr"/>
+      <c r="L152" s="4" t="n">
+        <v>53.24</v>
+      </c>
+      <c r="M152" s="4" t="n">
+        <v>1.597</v>
+      </c>
+      <c r="N152" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O152" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P152" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q152" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R152" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S152" s="4" t="n"/>
+      <c r="T152" s="4" t="n"/>
+      <c r="U152" s="4" t="n"/>
+      <c r="V152" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W152" s="4" t="inlineStr"/>
+      <c r="X152" s="4" t="n"/>
+      <c r="Y152" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z152" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA152" s="4" t="n"/>
+      <c r="AB152" s="4" t="n"/>
+      <c r="AC152" s="4" t="n"/>
+      <c r="AD152" s="4" t="n"/>
+      <c r="AE152" s="4" t="n"/>
+      <c r="AF152" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B153" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C153" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D153" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E153" s="6" t="n">
+        <v>34.99</v>
+      </c>
+      <c r="F153" s="6" t="n"/>
+      <c r="G153" s="6" t="n"/>
+      <c r="H153" s="6" t="n">
+        <v>89.72</v>
+      </c>
+      <c r="I153" s="6" t="inlineStr"/>
+      <c r="J153" s="6" t="inlineStr"/>
+      <c r="K153" s="6" t="inlineStr"/>
+      <c r="L153" s="6" t="n">
+        <v>109.41</v>
+      </c>
+      <c r="M153" s="6" t="n">
+        <v>3.282</v>
+      </c>
+      <c r="N153" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O153" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P153" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q153" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R153" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S153" s="6" t="n"/>
+      <c r="T153" s="6" t="n"/>
+      <c r="U153" s="6" t="n"/>
+      <c r="V153" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W153" s="6" t="inlineStr"/>
+      <c r="X153" s="6" t="n"/>
+      <c r="Y153" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z153" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA153" s="6" t="n"/>
+      <c r="AB153" s="6" t="n"/>
+      <c r="AC153" s="6" t="n"/>
+      <c r="AD153" s="6" t="n"/>
+      <c r="AE153" s="6" t="n"/>
+      <c r="AF153" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B154" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C154" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D154" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E154" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F154" s="4" t="n"/>
+      <c r="G154" s="4" t="n"/>
+      <c r="H154" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I154" s="4" t="inlineStr"/>
+      <c r="J154" s="4" t="inlineStr"/>
+      <c r="K154" s="4" t="inlineStr"/>
+      <c r="L154" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M154" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N154" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O154" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P154" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q154" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R154" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S154" s="4" t="n"/>
+      <c r="T154" s="4" t="n"/>
+      <c r="U154" s="4" t="n"/>
+      <c r="V154" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W154" s="4" t="inlineStr"/>
+      <c r="X154" s="4" t="n"/>
+      <c r="Y154" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z154" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA154" s="4" t="n"/>
+      <c r="AB154" s="4" t="n"/>
+      <c r="AC154" s="4" t="n"/>
+      <c r="AD154" s="4" t="n"/>
+      <c r="AE154" s="4" t="n"/>
+      <c r="AF154" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B155" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C155" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D155" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E155" s="6" t="n">
+        <v>55.99</v>
+      </c>
+      <c r="F155" s="6" t="n"/>
+      <c r="G155" s="6" t="n"/>
+      <c r="H155" s="6" t="n">
+        <v>71.78</v>
+      </c>
+      <c r="I155" s="6" t="inlineStr"/>
+      <c r="J155" s="6" t="inlineStr"/>
+      <c r="K155" s="6" t="inlineStr"/>
+      <c r="L155" s="6" t="n">
+        <v>87.54000000000001</v>
+      </c>
+      <c r="M155" s="6" t="n">
+        <v>2.626</v>
+      </c>
+      <c r="N155" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O155" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P155" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q155" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R155" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S155" s="6" t="n"/>
+      <c r="T155" s="6" t="n"/>
+      <c r="U155" s="6" t="n"/>
+      <c r="V155" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W155" s="6" t="inlineStr"/>
+      <c r="X155" s="6" t="n"/>
+      <c r="Y155" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z155" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA155" s="6" t="n"/>
+      <c r="AB155" s="6" t="n"/>
+      <c r="AC155" s="6" t="n"/>
+      <c r="AD155" s="6" t="n"/>
+      <c r="AE155" s="6" t="n"/>
+      <c r="AF155" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B156" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C156" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D156" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E156" s="4" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="F156" s="4" t="n"/>
+      <c r="G156" s="4" t="n"/>
+      <c r="H156" s="4" t="n">
+        <v>65.98999999999999</v>
+      </c>
+      <c r="I156" s="4" t="inlineStr"/>
+      <c r="J156" s="4" t="inlineStr"/>
+      <c r="K156" s="4" t="inlineStr"/>
+      <c r="L156" s="4" t="n">
+        <v>80.48</v>
+      </c>
+      <c r="M156" s="4" t="n">
+        <v>2.414</v>
+      </c>
+      <c r="N156" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O156" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P156" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q156" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R156" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S156" s="4" t="n"/>
+      <c r="T156" s="4" t="n"/>
+      <c r="U156" s="4" t="n"/>
+      <c r="V156" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W156" s="4" t="inlineStr"/>
+      <c r="X156" s="4" t="n"/>
+      <c r="Y156" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z156" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA156" s="4" t="n"/>
+      <c r="AB156" s="4" t="n"/>
+      <c r="AC156" s="4" t="n"/>
+      <c r="AD156" s="4" t="n"/>
+      <c r="AE156" s="4" t="n"/>
+      <c r="AF156" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B157" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C157" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D157" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E157" s="6" t="n">
+        <v>132.99</v>
+      </c>
+      <c r="F157" s="6" t="n"/>
+      <c r="G157" s="6" t="n"/>
+      <c r="H157" s="6" t="n">
+        <v>53.2</v>
+      </c>
+      <c r="I157" s="6" t="inlineStr"/>
+      <c r="J157" s="6" t="inlineStr"/>
+      <c r="K157" s="6" t="inlineStr"/>
+      <c r="L157" s="6" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="M157" s="6" t="n">
+        <v>1.946</v>
+      </c>
+      <c r="N157" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O157" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P157" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q157" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R157" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S157" s="6" t="n"/>
+      <c r="T157" s="6" t="n"/>
+      <c r="U157" s="6" t="n"/>
+      <c r="V157" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W157" s="6" t="inlineStr"/>
+      <c r="X157" s="6" t="n"/>
+      <c r="Y157" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z157" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA157" s="6" t="n"/>
+      <c r="AB157" s="6" t="n"/>
+      <c r="AC157" s="6" t="n"/>
+      <c r="AD157" s="6" t="n"/>
+      <c r="AE157" s="6" t="n"/>
+      <c r="AF157" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="158">
+      <c r="A158" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B158" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C158" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D158" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E158" s="4" t="n">
+        <v>155.99</v>
+      </c>
+      <c r="F158" s="4" t="n"/>
+      <c r="G158" s="4" t="n"/>
+      <c r="H158" s="4" t="n">
+        <v>57.77</v>
+      </c>
+      <c r="I158" s="4" t="inlineStr"/>
+      <c r="J158" s="4" t="inlineStr"/>
+      <c r="K158" s="4" t="inlineStr"/>
+      <c r="L158" s="4" t="n">
+        <v>70.45</v>
+      </c>
+      <c r="M158" s="4" t="n">
+        <v>2.114</v>
+      </c>
+      <c r="N158" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O158" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P158" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q158" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R158" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S158" s="4" t="n"/>
+      <c r="T158" s="4" t="n"/>
+      <c r="U158" s="4" t="n"/>
+      <c r="V158" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W158" s="4" t="inlineStr"/>
+      <c r="X158" s="4" t="n"/>
+      <c r="Y158" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z158" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA158" s="4" t="n"/>
+      <c r="AB158" s="4" t="n"/>
+      <c r="AC158" s="4" t="n"/>
+      <c r="AD158" s="4" t="n"/>
+      <c r="AE158" s="4" t="n"/>
+      <c r="AF158" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="159">
+      <c r="A159" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B159" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C159" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D159" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E159" s="6" t="n">
+        <v>249.99</v>
+      </c>
+      <c r="F159" s="6" t="n"/>
+      <c r="G159" s="6" t="n"/>
+      <c r="H159" s="6" t="n">
+        <v>59.52</v>
+      </c>
+      <c r="I159" s="6" t="inlineStr"/>
+      <c r="J159" s="6" t="inlineStr"/>
+      <c r="K159" s="6" t="inlineStr"/>
+      <c r="L159" s="6" t="n">
+        <v>72.59</v>
+      </c>
+      <c r="M159" s="6" t="n">
+        <v>2.178</v>
+      </c>
+      <c r="N159" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O159" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P159" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q159" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R159" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S159" s="6" t="n"/>
+      <c r="T159" s="6" t="n"/>
+      <c r="U159" s="6" t="n"/>
+      <c r="V159" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W159" s="6" t="inlineStr"/>
+      <c r="X159" s="6" t="n"/>
+      <c r="Y159" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z159" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA159" s="6" t="n"/>
+      <c r="AB159" s="6" t="n"/>
+      <c r="AC159" s="6" t="n"/>
+      <c r="AD159" s="6" t="n"/>
+      <c r="AE159" s="6" t="n"/>
+      <c r="AF159" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="160">
+      <c r="A160" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B160" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C160" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D160" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E160" s="4" t="n">
+        <v>30.39</v>
+      </c>
+      <c r="F160" s="4" t="n"/>
+      <c r="G160" s="4" t="n"/>
+      <c r="H160" s="4" t="n">
+        <v>72.36</v>
+      </c>
+      <c r="I160" s="4" t="inlineStr"/>
+      <c r="J160" s="4" t="inlineStr"/>
+      <c r="K160" s="4" t="inlineStr"/>
+      <c r="L160" s="4" t="n">
+        <v>91.59</v>
+      </c>
+      <c r="M160" s="4" t="n">
+        <v>2.748</v>
+      </c>
+      <c r="N160" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O160" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P160" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q160" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R160" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S160" s="4" t="n"/>
+      <c r="T160" s="4" t="n"/>
+      <c r="U160" s="4" t="n"/>
+      <c r="V160" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W160" s="4" t="inlineStr"/>
+      <c r="X160" s="4" t="n"/>
+      <c r="Y160" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z160" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA160" s="4" t="n"/>
+      <c r="AB160" s="4" t="n"/>
+      <c r="AC160" s="4" t="n"/>
+      <c r="AD160" s="4" t="n"/>
+      <c r="AE160" s="4" t="n"/>
+      <c r="AF160" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="161">
+      <c r="A161" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B161" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C161" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D161" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E161" s="6" t="n">
+        <v>27.99</v>
+      </c>
+      <c r="F161" s="6" t="n"/>
+      <c r="G161" s="6" t="n"/>
+      <c r="H161" s="6" t="n">
+        <v>55.98</v>
+      </c>
+      <c r="I161" s="6" t="inlineStr"/>
+      <c r="J161" s="6" t="inlineStr"/>
+      <c r="K161" s="6" t="inlineStr"/>
+      <c r="L161" s="6" t="n">
+        <v>70.86</v>
+      </c>
+      <c r="M161" s="6" t="n">
+        <v>2.126</v>
+      </c>
+      <c r="N161" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O161" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P161" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q161" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R161" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S161" s="6" t="n"/>
+      <c r="T161" s="6" t="n"/>
+      <c r="U161" s="6" t="n"/>
+      <c r="V161" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W161" s="6" t="inlineStr"/>
+      <c r="X161" s="6" t="n"/>
+      <c r="Y161" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z161" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA161" s="6" t="n"/>
+      <c r="AB161" s="6" t="n"/>
+      <c r="AC161" s="6" t="n"/>
+      <c r="AD161" s="6" t="n"/>
+      <c r="AE161" s="6" t="n"/>
+      <c r="AF161" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="162">
+      <c r="A162" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B162" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C162" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D162" s="4" t="inlineStr">
+        <is>
+          <t>910g</t>
+        </is>
+      </c>
+      <c r="E162" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F162" s="4" t="n"/>
+      <c r="G162" s="4" t="n"/>
+      <c r="H162" s="4" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="I162" s="4" t="inlineStr"/>
+      <c r="J162" s="4" t="inlineStr"/>
+      <c r="K162" s="4" t="inlineStr"/>
+      <c r="L162" s="4" t="n">
+        <v>69.53</v>
+      </c>
+      <c r="M162" s="4" t="n">
+        <v>2.086</v>
+      </c>
+      <c r="N162" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O162" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P162" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q162" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R162" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S162" s="4" t="n"/>
+      <c r="T162" s="4" t="n"/>
+      <c r="U162" s="4" t="n"/>
+      <c r="V162" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W162" s="4" t="inlineStr"/>
+      <c r="X162" s="4" t="n"/>
+      <c r="Y162" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z162" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA162" s="4" t="n"/>
+      <c r="AB162" s="4" t="n"/>
+      <c r="AC162" s="4" t="n"/>
+      <c r="AD162" s="4" t="n"/>
+      <c r="AE162" s="4" t="n"/>
+      <c r="AF162" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="163">
+      <c r="A163" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B163" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C163" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D163" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E163" s="6" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F163" s="6" t="n"/>
+      <c r="G163" s="6" t="n"/>
+      <c r="H163" s="6" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="I163" s="6" t="inlineStr"/>
+      <c r="J163" s="6" t="inlineStr"/>
+      <c r="K163" s="6" t="inlineStr"/>
+      <c r="L163" s="6" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M163" s="6" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N163" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O163" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P163" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q163" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R163" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S163" s="6" t="n"/>
+      <c r="T163" s="6" t="n"/>
+      <c r="U163" s="6" t="n"/>
+      <c r="V163" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W163" s="6" t="inlineStr"/>
+      <c r="X163" s="6" t="n"/>
+      <c r="Y163" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z163" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA163" s="6" t="n"/>
+      <c r="AB163" s="6" t="n"/>
+      <c r="AC163" s="6" t="n"/>
+      <c r="AD163" s="6" t="n"/>
+      <c r="AE163" s="6" t="n"/>
+      <c r="AF163" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="164">
+      <c r="A164" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B164" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C164" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D164" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E164" s="4" t="n">
+        <v>15.59</v>
+      </c>
+      <c r="F164" s="4" t="n"/>
+      <c r="G164" s="4" t="n"/>
+      <c r="H164" s="4" t="n">
+        <v>37.12</v>
+      </c>
+      <c r="I164" s="4" t="inlineStr"/>
+      <c r="J164" s="4" t="inlineStr"/>
+      <c r="K164" s="4" t="inlineStr"/>
+      <c r="L164" s="4" t="n">
+        <v>62.92</v>
+      </c>
+      <c r="M164" s="4" t="n">
+        <v>1.888</v>
+      </c>
+      <c r="N164" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O164" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P164" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q164" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R164" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S164" s="4" t="n"/>
+      <c r="T164" s="4" t="n"/>
+      <c r="U164" s="4" t="n"/>
+      <c r="V164" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W164" s="4" t="inlineStr"/>
+      <c r="X164" s="4" t="n"/>
+      <c r="Y164" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z164" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA164" s="4" t="n"/>
+      <c r="AB164" s="4" t="n"/>
+      <c r="AC164" s="4" t="n"/>
+      <c r="AD164" s="4" t="n"/>
+      <c r="AE164" s="4" t="n"/>
+      <c r="AF164" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="165">
+      <c r="A165" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B165" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C165" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D165" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E165" s="6" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="F165" s="6" t="n"/>
+      <c r="G165" s="6" t="n"/>
+      <c r="H165" s="6" t="n">
+        <v>33.14</v>
+      </c>
+      <c r="I165" s="6" t="inlineStr"/>
+      <c r="J165" s="6" t="inlineStr"/>
+      <c r="K165" s="6" t="inlineStr"/>
+      <c r="L165" s="6" t="n">
+        <v>56.17</v>
+      </c>
+      <c r="M165" s="6" t="n">
+        <v>1.685</v>
+      </c>
+      <c r="N165" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O165" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P165" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q165" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R165" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S165" s="6" t="n"/>
+      <c r="T165" s="6" t="n"/>
+      <c r="U165" s="6" t="n"/>
+      <c r="V165" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W165" s="6" t="inlineStr"/>
+      <c r="X165" s="6" t="n"/>
+      <c r="Y165" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z165" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA165" s="6" t="n"/>
+      <c r="AB165" s="6" t="n"/>
+      <c r="AC165" s="6" t="n"/>
+      <c r="AD165" s="6" t="n"/>
+      <c r="AE165" s="6" t="n"/>
+      <c r="AF165" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="166">
+      <c r="A166" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B166" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C166" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D166" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E166" s="4" t="n">
+        <v>74.73999999999999</v>
+      </c>
+      <c r="F166" s="4" t="n"/>
+      <c r="G166" s="4" t="n"/>
+      <c r="H166" s="4" t="n">
+        <v>29.9</v>
+      </c>
+      <c r="I166" s="4" t="inlineStr"/>
+      <c r="J166" s="4" t="inlineStr"/>
+      <c r="K166" s="4" t="inlineStr"/>
+      <c r="L166" s="4" t="n">
+        <v>50.68</v>
+      </c>
+      <c r="M166" s="4" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="N166" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O166" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P166" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q166" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R166" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S166" s="4" t="n"/>
+      <c r="T166" s="4" t="n"/>
+      <c r="U166" s="4" t="n"/>
+      <c r="V166" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W166" s="4" t="inlineStr"/>
+      <c r="X166" s="4" t="n"/>
+      <c r="Y166" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z166" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA166" s="4" t="n"/>
+      <c r="AB166" s="4" t="n"/>
+      <c r="AC166" s="4" t="n"/>
+      <c r="AD166" s="4" t="n"/>
+      <c r="AE166" s="4" t="n"/>
+      <c r="AF166" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="167">
+      <c r="A167" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B167" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C167" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D167" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E167" s="6" t="n">
+        <v>139.74</v>
+      </c>
+      <c r="F167" s="6" t="n"/>
+      <c r="G167" s="6" t="n"/>
+      <c r="H167" s="6" t="n">
+        <v>27.95</v>
+      </c>
+      <c r="I167" s="6" t="inlineStr"/>
+      <c r="J167" s="6" t="inlineStr"/>
+      <c r="K167" s="6" t="inlineStr"/>
+      <c r="L167" s="6" t="n">
+        <v>47.37</v>
+      </c>
+      <c r="M167" s="6" t="n">
+        <v>1.421</v>
+      </c>
+      <c r="N167" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O167" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P167" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q167" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R167" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S167" s="6" t="n"/>
+      <c r="T167" s="6" t="n"/>
+      <c r="U167" s="6" t="n"/>
+      <c r="V167" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W167" s="6" t="inlineStr"/>
+      <c r="X167" s="6" t="n"/>
+      <c r="Y167" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z167" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA167" s="6" t="n"/>
+      <c r="AB167" s="6" t="n"/>
+      <c r="AC167" s="6" t="n"/>
+      <c r="AD167" s="6" t="n"/>
+      <c r="AE167" s="6" t="n"/>
+      <c r="AF167" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="168">
+      <c r="A168" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B168" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C168" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D168" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E168" s="4" t="n">
+        <v>7.99</v>
+      </c>
+      <c r="F168" s="4" t="n"/>
+      <c r="G168" s="4" t="n"/>
+      <c r="H168" s="4" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="I168" s="4" t="inlineStr"/>
+      <c r="J168" s="4" t="inlineStr"/>
+      <c r="K168" s="4" t="inlineStr"/>
+      <c r="L168" s="4" t="n"/>
+      <c r="M168" s="4" t="n"/>
+      <c r="N168" s="4" t="n"/>
+      <c r="O168" s="4" t="n"/>
+      <c r="P168" s="4" t="n"/>
+      <c r="Q168" s="4" t="n"/>
+      <c r="R168" s="4" t="n"/>
+      <c r="S168" s="4" t="n"/>
+      <c r="T168" s="4" t="n"/>
+      <c r="U168" s="4" t="n"/>
+      <c r="V168" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W168" s="4" t="inlineStr"/>
+      <c r="X168" s="4" t="n"/>
+      <c r="Y168" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z168" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA168" s="4" t="n"/>
+      <c r="AB168" s="4" t="n"/>
+      <c r="AC168" s="4" t="n"/>
+      <c r="AD168" s="4" t="n"/>
+      <c r="AE168" s="4" t="n">
+        <v>79.90000000000001</v>
+      </c>
+      <c r="AF168" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="169">
+      <c r="A169" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B169" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C169" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D169" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E169" s="6" t="n">
+        <v>14.99</v>
+      </c>
+      <c r="F169" s="6" t="n"/>
+      <c r="G169" s="6" t="n"/>
+      <c r="H169" s="6" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="I169" s="6" t="inlineStr"/>
+      <c r="J169" s="6" t="inlineStr"/>
+      <c r="K169" s="6" t="inlineStr"/>
+      <c r="L169" s="6" t="n"/>
+      <c r="M169" s="6" t="n"/>
+      <c r="N169" s="6" t="n"/>
+      <c r="O169" s="6" t="n"/>
+      <c r="P169" s="6" t="n"/>
+      <c r="Q169" s="6" t="n"/>
+      <c r="R169" s="6" t="n"/>
+      <c r="S169" s="6" t="n"/>
+      <c r="T169" s="6" t="n"/>
+      <c r="U169" s="6" t="n"/>
+      <c r="V169" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W169" s="6" t="inlineStr"/>
+      <c r="X169" s="6" t="n"/>
+      <c r="Y169" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z169" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA169" s="6" t="n"/>
+      <c r="AB169" s="6" t="n"/>
+      <c r="AC169" s="6" t="n"/>
+      <c r="AD169" s="6" t="n"/>
+      <c r="AE169" s="6" t="n">
+        <v>59.96</v>
+      </c>
+      <c r="AF169" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="170">
+      <c r="A170" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B170" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C170" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D170" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E170" s="4" t="n">
+        <v>24.99</v>
+      </c>
+      <c r="F170" s="4" t="n"/>
+      <c r="G170" s="4" t="n"/>
+      <c r="H170" s="4" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="I170" s="4" t="inlineStr"/>
+      <c r="J170" s="4" t="inlineStr"/>
+      <c r="K170" s="4" t="inlineStr"/>
+      <c r="L170" s="4" t="n"/>
+      <c r="M170" s="4" t="n"/>
+      <c r="N170" s="4" t="n"/>
+      <c r="O170" s="4" t="n"/>
+      <c r="P170" s="4" t="n"/>
+      <c r="Q170" s="4" t="n"/>
+      <c r="R170" s="4" t="n"/>
+      <c r="S170" s="4" t="n"/>
+      <c r="T170" s="4" t="n"/>
+      <c r="U170" s="4" t="n"/>
+      <c r="V170" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W170" s="4" t="inlineStr"/>
+      <c r="X170" s="4" t="n"/>
+      <c r="Y170" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z170" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA170" s="4" t="n"/>
+      <c r="AB170" s="4" t="n"/>
+      <c r="AC170" s="4" t="n"/>
+      <c r="AD170" s="4" t="n"/>
+      <c r="AE170" s="4" t="n">
+        <v>49.98</v>
+      </c>
+      <c r="AF170" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="A171" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B171" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C171" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D171" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E171" s="6" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="F171" s="6" t="n"/>
+      <c r="G171" s="6" t="n"/>
+      <c r="H171" s="6" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="I171" s="6" t="inlineStr"/>
+      <c r="J171" s="6" t="inlineStr"/>
+      <c r="K171" s="6" t="inlineStr"/>
+      <c r="L171" s="6" t="n"/>
+      <c r="M171" s="6" t="n"/>
+      <c r="N171" s="6" t="n"/>
+      <c r="O171" s="6" t="n"/>
+      <c r="P171" s="6" t="n"/>
+      <c r="Q171" s="6" t="n"/>
+      <c r="R171" s="6" t="n"/>
+      <c r="S171" s="6" t="n"/>
+      <c r="T171" s="6" t="n"/>
+      <c r="U171" s="6" t="n"/>
+      <c r="V171" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W171" s="6" t="inlineStr"/>
+      <c r="X171" s="6" t="n"/>
+      <c r="Y171" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z171" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA171" s="6" t="n"/>
+      <c r="AB171" s="6" t="n"/>
+      <c r="AC171" s="6" t="n"/>
+      <c r="AD171" s="6" t="n"/>
+      <c r="AE171" s="6" t="n">
+        <v>45.99</v>
+      </c>
+      <c r="AF171" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="A172" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B172" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C172" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D172" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E172" s="4" t="n">
+        <v>28.99</v>
+      </c>
+      <c r="F172" s="4" t="n"/>
+      <c r="G172" s="4" t="n"/>
+      <c r="H172" s="4" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="I172" s="4" t="inlineStr"/>
+      <c r="J172" s="4" t="inlineStr"/>
+      <c r="K172" s="4" t="inlineStr"/>
+      <c r="L172" s="4" t="n"/>
+      <c r="M172" s="4" t="n"/>
+      <c r="N172" s="4" t="n"/>
+      <c r="O172" s="4" t="n"/>
+      <c r="P172" s="4" t="n"/>
+      <c r="Q172" s="4" t="n"/>
+      <c r="R172" s="4" t="n"/>
+      <c r="S172" s="4" t="n"/>
+      <c r="T172" s="4" t="n"/>
+      <c r="U172" s="4" t="n"/>
+      <c r="V172" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W172" s="4" t="inlineStr"/>
+      <c r="X172" s="4" t="n"/>
+      <c r="Y172" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z172" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA172" s="4" t="n"/>
+      <c r="AB172" s="4" t="n"/>
+      <c r="AC172" s="4" t="n"/>
+      <c r="AD172" s="4" t="n"/>
+      <c r="AE172" s="4" t="n">
+        <v>115.96</v>
+      </c>
+      <c r="AF172" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B173" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C173" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D173" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E173" s="6" t="n">
+        <v>42.99</v>
+      </c>
+      <c r="F173" s="6" t="n"/>
+      <c r="G173" s="6" t="n"/>
+      <c r="H173" s="6" t="n">
+        <v>85.98</v>
+      </c>
+      <c r="I173" s="6" t="inlineStr"/>
+      <c r="J173" s="6" t="inlineStr"/>
+      <c r="K173" s="6" t="inlineStr"/>
+      <c r="L173" s="6" t="n"/>
+      <c r="M173" s="6" t="n"/>
+      <c r="N173" s="6" t="n"/>
+      <c r="O173" s="6" t="n"/>
+      <c r="P173" s="6" t="n"/>
+      <c r="Q173" s="6" t="n"/>
+      <c r="R173" s="6" t="n"/>
+      <c r="S173" s="6" t="n"/>
+      <c r="T173" s="6" t="n"/>
+      <c r="U173" s="6" t="n"/>
+      <c r="V173" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W173" s="6" t="inlineStr"/>
+      <c r="X173" s="6" t="n"/>
+      <c r="Y173" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z173" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA173" s="6" t="n"/>
+      <c r="AB173" s="6" t="n"/>
+      <c r="AC173" s="6" t="n"/>
+      <c r="AD173" s="6" t="n"/>
+      <c r="AE173" s="6" t="n">
+        <v>85.98</v>
+      </c>
+      <c r="AF173" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B174" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C174" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D174" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E174" s="4" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="F174" s="4" t="n"/>
+      <c r="G174" s="4" t="n"/>
+      <c r="H174" s="4" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="I174" s="4" t="inlineStr"/>
+      <c r="J174" s="4" t="inlineStr"/>
+      <c r="K174" s="4" t="inlineStr"/>
+      <c r="L174" s="4" t="n"/>
+      <c r="M174" s="4" t="n"/>
+      <c r="N174" s="4" t="n"/>
+      <c r="O174" s="4" t="n"/>
+      <c r="P174" s="4" t="n"/>
+      <c r="Q174" s="4" t="n"/>
+      <c r="R174" s="4" t="n"/>
+      <c r="S174" s="4" t="n"/>
+      <c r="T174" s="4" t="n"/>
+      <c r="U174" s="4" t="n"/>
+      <c r="V174" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W174" s="4" t="inlineStr"/>
+      <c r="X174" s="4" t="n"/>
+      <c r="Y174" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z174" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA174" s="4" t="n"/>
+      <c r="AB174" s="4" t="n"/>
+      <c r="AC174" s="4" t="n"/>
+      <c r="AD174" s="4" t="n"/>
+      <c r="AE174" s="4" t="n">
+        <v>83.98999999999999</v>
+      </c>
+      <c r="AF174" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B175" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C175" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D175" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E175" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F175" s="6" t="n"/>
+      <c r="G175" s="6" t="n"/>
+      <c r="H175" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I175" s="6" t="inlineStr"/>
+      <c r="J175" s="6" t="inlineStr"/>
+      <c r="K175" s="6" t="inlineStr"/>
+      <c r="L175" s="6" t="n"/>
+      <c r="M175" s="6" t="n"/>
+      <c r="N175" s="6" t="n"/>
+      <c r="O175" s="6" t="n"/>
+      <c r="P175" s="6" t="n"/>
+      <c r="Q175" s="6" t="n"/>
+      <c r="R175" s="6" t="n"/>
+      <c r="S175" s="6" t="n"/>
+      <c r="T175" s="6" t="n"/>
+      <c r="U175" s="6" t="n"/>
+      <c r="V175" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W175" s="6" t="inlineStr"/>
+      <c r="X175" s="6" t="n"/>
+      <c r="Y175" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z175" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA175" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB175" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC175" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD175" s="6" t="n"/>
+      <c r="AE175" s="6" t="n"/>
+      <c r="AF175" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B176" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C176" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D176" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E176" s="4" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="F176" s="4" t="n"/>
+      <c r="G176" s="4" t="n"/>
+      <c r="H176" s="4" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="I176" s="4" t="inlineStr"/>
+      <c r="J176" s="4" t="inlineStr"/>
+      <c r="K176" s="4" t="inlineStr"/>
+      <c r="L176" s="4" t="n"/>
+      <c r="M176" s="4" t="n"/>
+      <c r="N176" s="4" t="n"/>
+      <c r="O176" s="4" t="n"/>
+      <c r="P176" s="4" t="n"/>
+      <c r="Q176" s="4" t="n"/>
+      <c r="R176" s="4" t="n"/>
+      <c r="S176" s="4" t="n"/>
+      <c r="T176" s="4" t="n"/>
+      <c r="U176" s="4" t="n"/>
+      <c r="V176" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W176" s="4" t="inlineStr"/>
+      <c r="X176" s="4" t="n"/>
+      <c r="Y176" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z176" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA176" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB176" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC176" s="4" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AD176" s="4" t="n"/>
+      <c r="AE176" s="4" t="n"/>
+      <c r="AF176" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B177" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C177" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D177" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E177" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F177" s="6" t="n"/>
+      <c r="G177" s="6" t="n"/>
+      <c r="H177" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I177" s="6" t="inlineStr"/>
+      <c r="J177" s="6" t="inlineStr"/>
+      <c r="K177" s="6" t="inlineStr"/>
+      <c r="L177" s="6" t="n"/>
+      <c r="M177" s="6" t="n"/>
+      <c r="N177" s="6" t="n"/>
+      <c r="O177" s="6" t="n"/>
+      <c r="P177" s="6" t="n"/>
+      <c r="Q177" s="6" t="n"/>
+      <c r="R177" s="6" t="n"/>
+      <c r="S177" s="6" t="n"/>
+      <c r="T177" s="6" t="n"/>
+      <c r="U177" s="6" t="n"/>
+      <c r="V177" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W177" s="6" t="inlineStr"/>
+      <c r="X177" s="6" t="n"/>
+      <c r="Y177" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z177" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA177" s="6" t="n"/>
+      <c r="AB177" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC177" s="6" t="n"/>
+      <c r="AD177" s="6" t="n"/>
+      <c r="AE177" s="6" t="n"/>
+      <c r="AF177" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-23</t>
+        </is>
+      </c>
+      <c r="B178" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C178" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D178" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E178" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F178" s="4" t="n"/>
+      <c r="G178" s="4" t="n"/>
+      <c r="H178" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I178" s="4" t="inlineStr"/>
+      <c r="J178" s="4" t="inlineStr"/>
+      <c r="K178" s="4" t="inlineStr"/>
+      <c r="L178" s="4" t="n"/>
+      <c r="M178" s="4" t="n"/>
+      <c r="N178" s="4" t="n"/>
+      <c r="O178" s="4" t="n"/>
+      <c r="P178" s="4" t="n"/>
+      <c r="Q178" s="4" t="n"/>
+      <c r="R178" s="4" t="n"/>
+      <c r="S178" s="4" t="n"/>
+      <c r="T178" s="4" t="n"/>
+      <c r="U178" s="4" t="n"/>
+      <c r="V178" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W178" s="4" t="inlineStr"/>
+      <c r="X178" s="4" t="n"/>
+      <c r="Y178" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z178" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA178" s="4" t="n"/>
+      <c r="AB178" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC178" s="4" t="n"/>
+      <c r="AD178" s="4" t="n"/>
+      <c r="AE178" s="4" t="n"/>
+      <c r="AF178" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-24
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF178"/>
+  <dimension ref="A1:AF215"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -14570,6 +14570,2918 @@
         <v>1</v>
       </c>
     </row>
+    <row r="179">
+      <c r="A179" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B179" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C179" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D179" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E179" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F179" s="4" t="n"/>
+      <c r="G179" s="4" t="n"/>
+      <c r="H179" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I179" s="4" t="inlineStr"/>
+      <c r="J179" s="4" t="inlineStr"/>
+      <c r="K179" s="4" t="inlineStr"/>
+      <c r="L179" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M179" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N179" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O179" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P179" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q179" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R179" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S179" s="4" t="n"/>
+      <c r="T179" s="4" t="n"/>
+      <c r="U179" s="4" t="n"/>
+      <c r="V179" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W179" s="4" t="inlineStr"/>
+      <c r="X179" s="4" t="n"/>
+      <c r="Y179" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z179" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA179" s="4" t="n"/>
+      <c r="AB179" s="4" t="n"/>
+      <c r="AC179" s="4" t="n"/>
+      <c r="AD179" s="4" t="n"/>
+      <c r="AE179" s="4" t="n"/>
+      <c r="AF179" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B180" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C180" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D180" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E180" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F180" s="6" t="n"/>
+      <c r="G180" s="6" t="n"/>
+      <c r="H180" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I180" s="6" t="inlineStr"/>
+      <c r="J180" s="6" t="inlineStr"/>
+      <c r="K180" s="6" t="inlineStr"/>
+      <c r="L180" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M180" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N180" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O180" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P180" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q180" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R180" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S180" s="6" t="n"/>
+      <c r="T180" s="6" t="n"/>
+      <c r="U180" s="6" t="n"/>
+      <c r="V180" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W180" s="6" t="inlineStr"/>
+      <c r="X180" s="6" t="n"/>
+      <c r="Y180" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z180" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA180" s="6" t="n"/>
+      <c r="AB180" s="6" t="n"/>
+      <c r="AC180" s="6" t="n"/>
+      <c r="AD180" s="6" t="n"/>
+      <c r="AE180" s="6" t="n"/>
+      <c r="AF180" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="A181" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B181" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C181" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D181" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E181" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="F181" s="4" t="n"/>
+      <c r="G181" s="4" t="n"/>
+      <c r="H181" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I181" s="4" t="inlineStr"/>
+      <c r="J181" s="4" t="inlineStr"/>
+      <c r="K181" s="4" t="inlineStr"/>
+      <c r="L181" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M181" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N181" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O181" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P181" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q181" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R181" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S181" s="4" t="n"/>
+      <c r="T181" s="4" t="n"/>
+      <c r="U181" s="4" t="n"/>
+      <c r="V181" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W181" s="4" t="inlineStr"/>
+      <c r="X181" s="4" t="n"/>
+      <c r="Y181" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z181" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA181" s="4" t="n"/>
+      <c r="AB181" s="4" t="n"/>
+      <c r="AC181" s="4" t="n"/>
+      <c r="AD181" s="4" t="n"/>
+      <c r="AE181" s="4" t="n"/>
+      <c r="AF181" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="A182" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B182" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C182" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D182" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E182" s="6" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="F182" s="6" t="n"/>
+      <c r="G182" s="6" t="n"/>
+      <c r="H182" s="6" t="n">
+        <v>35.82</v>
+      </c>
+      <c r="I182" s="6" t="inlineStr"/>
+      <c r="J182" s="6" t="inlineStr"/>
+      <c r="K182" s="6" t="inlineStr"/>
+      <c r="L182" s="6" t="n">
+        <v>49.75</v>
+      </c>
+      <c r="M182" s="6" t="n">
+        <v>1.492</v>
+      </c>
+      <c r="N182" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O182" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P182" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q182" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R182" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S182" s="6" t="n"/>
+      <c r="T182" s="6" t="n"/>
+      <c r="U182" s="6" t="n"/>
+      <c r="V182" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W182" s="6" t="inlineStr"/>
+      <c r="X182" s="6" t="n"/>
+      <c r="Y182" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z182" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA182" s="6" t="n"/>
+      <c r="AB182" s="6" t="n"/>
+      <c r="AC182" s="6" t="n"/>
+      <c r="AD182" s="6" t="n"/>
+      <c r="AE182" s="6" t="n"/>
+      <c r="AF182" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="A183" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B183" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C183" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D183" s="4" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E183" s="4" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="F183" s="4" t="n"/>
+      <c r="G183" s="4" t="n"/>
+      <c r="H183" s="4" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="I183" s="4" t="inlineStr"/>
+      <c r="J183" s="4" t="inlineStr"/>
+      <c r="K183" s="4" t="inlineStr"/>
+      <c r="L183" s="4" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="M183" s="4" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="N183" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O183" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P183" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q183" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R183" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S183" s="4" t="n"/>
+      <c r="T183" s="4" t="n"/>
+      <c r="U183" s="4" t="n"/>
+      <c r="V183" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W183" s="4" t="inlineStr"/>
+      <c r="X183" s="4" t="n"/>
+      <c r="Y183" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z183" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA183" s="4" t="n"/>
+      <c r="AB183" s="4" t="n"/>
+      <c r="AC183" s="4" t="n"/>
+      <c r="AD183" s="4" t="n"/>
+      <c r="AE183" s="4" t="n"/>
+      <c r="AF183" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="184">
+      <c r="A184" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B184" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C184" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D184" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E184" s="6" t="n">
+        <v>26.49</v>
+      </c>
+      <c r="F184" s="6" t="n"/>
+      <c r="G184" s="6" t="n"/>
+      <c r="H184" s="6" t="n">
+        <v>35.32</v>
+      </c>
+      <c r="I184" s="6" t="inlineStr"/>
+      <c r="J184" s="6" t="inlineStr"/>
+      <c r="K184" s="6" t="inlineStr"/>
+      <c r="L184" s="6" t="n">
+        <v>49.06</v>
+      </c>
+      <c r="M184" s="6" t="n">
+        <v>1.472</v>
+      </c>
+      <c r="N184" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O184" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P184" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q184" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R184" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S184" s="6" t="n"/>
+      <c r="T184" s="6" t="n"/>
+      <c r="U184" s="6" t="n"/>
+      <c r="V184" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W184" s="6" t="inlineStr"/>
+      <c r="X184" s="6" t="n"/>
+      <c r="Y184" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z184" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA184" s="6" t="n"/>
+      <c r="AB184" s="6" t="n"/>
+      <c r="AC184" s="6" t="n"/>
+      <c r="AD184" s="6" t="n"/>
+      <c r="AE184" s="6" t="n"/>
+      <c r="AF184" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="A185" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B185" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C185" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D185" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E185" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F185" s="4" t="n"/>
+      <c r="G185" s="4" t="n"/>
+      <c r="H185" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I185" s="4" t="inlineStr"/>
+      <c r="J185" s="4" t="inlineStr"/>
+      <c r="K185" s="4" t="inlineStr"/>
+      <c r="L185" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M185" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N185" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O185" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P185" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q185" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R185" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S185" s="4" t="n"/>
+      <c r="T185" s="4" t="n"/>
+      <c r="U185" s="4" t="n"/>
+      <c r="V185" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W185" s="4" t="inlineStr"/>
+      <c r="X185" s="4" t="n"/>
+      <c r="Y185" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z185" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA185" s="4" t="n"/>
+      <c r="AB185" s="4" t="n"/>
+      <c r="AC185" s="4" t="n"/>
+      <c r="AD185" s="4" t="n"/>
+      <c r="AE185" s="4" t="n"/>
+      <c r="AF185" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B186" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C186" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D186" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E186" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F186" s="6" t="n"/>
+      <c r="G186" s="6" t="n"/>
+      <c r="H186" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I186" s="6" t="inlineStr"/>
+      <c r="J186" s="6" t="inlineStr"/>
+      <c r="K186" s="6" t="inlineStr"/>
+      <c r="L186" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M186" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N186" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O186" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P186" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q186" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R186" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S186" s="6" t="n"/>
+      <c r="T186" s="6" t="n"/>
+      <c r="U186" s="6" t="n"/>
+      <c r="V186" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W186" s="6" t="inlineStr"/>
+      <c r="X186" s="6" t="n"/>
+      <c r="Y186" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z186" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA186" s="6" t="n"/>
+      <c r="AB186" s="6" t="n"/>
+      <c r="AC186" s="6" t="n"/>
+      <c r="AD186" s="6" t="n"/>
+      <c r="AE186" s="6" t="n"/>
+      <c r="AF186" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B187" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C187" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D187" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E187" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F187" s="4" t="n"/>
+      <c r="G187" s="4" t="n"/>
+      <c r="H187" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I187" s="4" t="inlineStr"/>
+      <c r="J187" s="4" t="inlineStr"/>
+      <c r="K187" s="4" t="inlineStr"/>
+      <c r="L187" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M187" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N187" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O187" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P187" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q187" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R187" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S187" s="4" t="n"/>
+      <c r="T187" s="4" t="n"/>
+      <c r="U187" s="4" t="n"/>
+      <c r="V187" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W187" s="4" t="inlineStr"/>
+      <c r="X187" s="4" t="n"/>
+      <c r="Y187" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z187" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA187" s="4" t="n"/>
+      <c r="AB187" s="4" t="n"/>
+      <c r="AC187" s="4" t="n"/>
+      <c r="AD187" s="4" t="n"/>
+      <c r="AE187" s="4" t="n"/>
+      <c r="AF187" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B188" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C188" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D188" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E188" s="6" t="n">
+        <v>73.98999999999999</v>
+      </c>
+      <c r="F188" s="6" t="n"/>
+      <c r="G188" s="6" t="n"/>
+      <c r="H188" s="6" t="n">
+        <v>35.74</v>
+      </c>
+      <c r="I188" s="6" t="inlineStr"/>
+      <c r="J188" s="6" t="inlineStr"/>
+      <c r="K188" s="6" t="inlineStr"/>
+      <c r="L188" s="6" t="n">
+        <v>49.64</v>
+      </c>
+      <c r="M188" s="6" t="n">
+        <v>1.489</v>
+      </c>
+      <c r="N188" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O188" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P188" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q188" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R188" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S188" s="6" t="n"/>
+      <c r="T188" s="6" t="n"/>
+      <c r="U188" s="6" t="n"/>
+      <c r="V188" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W188" s="6" t="inlineStr"/>
+      <c r="X188" s="6" t="n"/>
+      <c r="Y188" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z188" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA188" s="6" t="n"/>
+      <c r="AB188" s="6" t="n"/>
+      <c r="AC188" s="6" t="n"/>
+      <c r="AD188" s="6" t="n"/>
+      <c r="AE188" s="6" t="n"/>
+      <c r="AF188" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B189" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C189" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D189" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E189" s="4" t="n">
+        <v>118.99</v>
+      </c>
+      <c r="F189" s="4" t="n"/>
+      <c r="G189" s="4" t="n"/>
+      <c r="H189" s="4" t="n">
+        <v>33.05</v>
+      </c>
+      <c r="I189" s="4" t="inlineStr"/>
+      <c r="J189" s="4" t="inlineStr"/>
+      <c r="K189" s="4" t="inlineStr"/>
+      <c r="L189" s="4" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="M189" s="4" t="n">
+        <v>1.377</v>
+      </c>
+      <c r="N189" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O189" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P189" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q189" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R189" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S189" s="4" t="n"/>
+      <c r="T189" s="4" t="n"/>
+      <c r="U189" s="4" t="n"/>
+      <c r="V189" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W189" s="4" t="inlineStr"/>
+      <c r="X189" s="4" t="n"/>
+      <c r="Y189" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z189" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA189" s="4" t="n"/>
+      <c r="AB189" s="4" t="n"/>
+      <c r="AC189" s="4" t="n"/>
+      <c r="AD189" s="4" t="n"/>
+      <c r="AE189" s="4" t="n"/>
+      <c r="AF189" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B190" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C190" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D190" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E190" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F190" s="6" t="n"/>
+      <c r="G190" s="6" t="n"/>
+      <c r="H190" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I190" s="6" t="inlineStr"/>
+      <c r="J190" s="6" t="inlineStr"/>
+      <c r="K190" s="6" t="inlineStr"/>
+      <c r="L190" s="6" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M190" s="6" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N190" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O190" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P190" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q190" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R190" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S190" s="6" t="n"/>
+      <c r="T190" s="6" t="n"/>
+      <c r="U190" s="6" t="n"/>
+      <c r="V190" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W190" s="6" t="inlineStr"/>
+      <c r="X190" s="6" t="n"/>
+      <c r="Y190" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z190" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA190" s="6" t="n"/>
+      <c r="AB190" s="6" t="n"/>
+      <c r="AC190" s="6" t="n"/>
+      <c r="AD190" s="6" t="n"/>
+      <c r="AE190" s="6" t="n"/>
+      <c r="AF190" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B191" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C191" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D191" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E191" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F191" s="4" t="n"/>
+      <c r="G191" s="4" t="n"/>
+      <c r="H191" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I191" s="4" t="inlineStr"/>
+      <c r="J191" s="4" t="inlineStr"/>
+      <c r="K191" s="4" t="inlineStr"/>
+      <c r="L191" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M191" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N191" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O191" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P191" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q191" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R191" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S191" s="4" t="n"/>
+      <c r="T191" s="4" t="n"/>
+      <c r="U191" s="4" t="n"/>
+      <c r="V191" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W191" s="4" t="inlineStr"/>
+      <c r="X191" s="4" t="n"/>
+      <c r="Y191" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z191" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA191" s="4" t="n"/>
+      <c r="AB191" s="4" t="n"/>
+      <c r="AC191" s="4" t="n"/>
+      <c r="AD191" s="4" t="n"/>
+      <c r="AE191" s="4" t="n"/>
+      <c r="AF191" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B192" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C192" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D192" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E192" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F192" s="6" t="n"/>
+      <c r="G192" s="6" t="n"/>
+      <c r="H192" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I192" s="6" t="inlineStr"/>
+      <c r="J192" s="6" t="inlineStr"/>
+      <c r="K192" s="6" t="inlineStr"/>
+      <c r="L192" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M192" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N192" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O192" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P192" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q192" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R192" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S192" s="6" t="n"/>
+      <c r="T192" s="6" t="n"/>
+      <c r="U192" s="6" t="n"/>
+      <c r="V192" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W192" s="6" t="inlineStr"/>
+      <c r="X192" s="6" t="n"/>
+      <c r="Y192" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z192" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA192" s="6" t="n"/>
+      <c r="AB192" s="6" t="n"/>
+      <c r="AC192" s="6" t="n"/>
+      <c r="AD192" s="6" t="n"/>
+      <c r="AE192" s="6" t="n"/>
+      <c r="AF192" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B193" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C193" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D193" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E193" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F193" s="4" t="n"/>
+      <c r="G193" s="4" t="n"/>
+      <c r="H193" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I193" s="4" t="inlineStr"/>
+      <c r="J193" s="4" t="inlineStr"/>
+      <c r="K193" s="4" t="inlineStr"/>
+      <c r="L193" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M193" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N193" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O193" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P193" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q193" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R193" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S193" s="4" t="n"/>
+      <c r="T193" s="4" t="n"/>
+      <c r="U193" s="4" t="n"/>
+      <c r="V193" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W193" s="4" t="inlineStr"/>
+      <c r="X193" s="4" t="n"/>
+      <c r="Y193" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z193" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA193" s="4" t="n"/>
+      <c r="AB193" s="4" t="n"/>
+      <c r="AC193" s="4" t="n"/>
+      <c r="AD193" s="4" t="n"/>
+      <c r="AE193" s="4" t="n"/>
+      <c r="AF193" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B194" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C194" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D194" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E194" s="6" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F194" s="6" t="n"/>
+      <c r="G194" s="6" t="n"/>
+      <c r="H194" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I194" s="6" t="inlineStr"/>
+      <c r="J194" s="6" t="inlineStr"/>
+      <c r="K194" s="6" t="inlineStr"/>
+      <c r="L194" s="6" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M194" s="6" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N194" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O194" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P194" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q194" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R194" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S194" s="6" t="n"/>
+      <c r="T194" s="6" t="n"/>
+      <c r="U194" s="6" t="n"/>
+      <c r="V194" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W194" s="6" t="inlineStr"/>
+      <c r="X194" s="6" t="n"/>
+      <c r="Y194" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z194" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA194" s="6" t="n"/>
+      <c r="AB194" s="6" t="n"/>
+      <c r="AC194" s="6" t="n"/>
+      <c r="AD194" s="6" t="n"/>
+      <c r="AE194" s="6" t="n"/>
+      <c r="AF194" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B195" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C195" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D195" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E195" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F195" s="4" t="n"/>
+      <c r="G195" s="4" t="n"/>
+      <c r="H195" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I195" s="4" t="inlineStr"/>
+      <c r="J195" s="4" t="inlineStr"/>
+      <c r="K195" s="4" t="inlineStr"/>
+      <c r="L195" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M195" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N195" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O195" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P195" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q195" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R195" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S195" s="4" t="n"/>
+      <c r="T195" s="4" t="n"/>
+      <c r="U195" s="4" t="n"/>
+      <c r="V195" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W195" s="4" t="inlineStr"/>
+      <c r="X195" s="4" t="n"/>
+      <c r="Y195" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z195" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA195" s="4" t="n"/>
+      <c r="AB195" s="4" t="n"/>
+      <c r="AC195" s="4" t="n"/>
+      <c r="AD195" s="4" t="n"/>
+      <c r="AE195" s="4" t="n"/>
+      <c r="AF195" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B196" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C196" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D196" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E196" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F196" s="6" t="n"/>
+      <c r="G196" s="6" t="n"/>
+      <c r="H196" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I196" s="6" t="inlineStr"/>
+      <c r="J196" s="6" t="inlineStr"/>
+      <c r="K196" s="6" t="inlineStr"/>
+      <c r="L196" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M196" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N196" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O196" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P196" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q196" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R196" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S196" s="6" t="n"/>
+      <c r="T196" s="6" t="n"/>
+      <c r="U196" s="6" t="n"/>
+      <c r="V196" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W196" s="6" t="inlineStr"/>
+      <c r="X196" s="6" t="n"/>
+      <c r="Y196" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z196" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA196" s="6" t="n"/>
+      <c r="AB196" s="6" t="n"/>
+      <c r="AC196" s="6" t="n"/>
+      <c r="AD196" s="6" t="n"/>
+      <c r="AE196" s="6" t="n"/>
+      <c r="AF196" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B197" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C197" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D197" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E197" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F197" s="4" t="n"/>
+      <c r="G197" s="4" t="n"/>
+      <c r="H197" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I197" s="4" t="inlineStr"/>
+      <c r="J197" s="4" t="inlineStr"/>
+      <c r="K197" s="4" t="inlineStr"/>
+      <c r="L197" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M197" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N197" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O197" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P197" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q197" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R197" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S197" s="4" t="n"/>
+      <c r="T197" s="4" t="n"/>
+      <c r="U197" s="4" t="n"/>
+      <c r="V197" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W197" s="4" t="inlineStr"/>
+      <c r="X197" s="4" t="n"/>
+      <c r="Y197" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z197" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA197" s="4" t="n"/>
+      <c r="AB197" s="4" t="n"/>
+      <c r="AC197" s="4" t="n"/>
+      <c r="AD197" s="4" t="n"/>
+      <c r="AE197" s="4" t="n"/>
+      <c r="AF197" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B198" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C198" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D198" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E198" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F198" s="6" t="n"/>
+      <c r="G198" s="6" t="n"/>
+      <c r="H198" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I198" s="6" t="inlineStr"/>
+      <c r="J198" s="6" t="inlineStr"/>
+      <c r="K198" s="6" t="inlineStr"/>
+      <c r="L198" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M198" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N198" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O198" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P198" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q198" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R198" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S198" s="6" t="n"/>
+      <c r="T198" s="6" t="n"/>
+      <c r="U198" s="6" t="n"/>
+      <c r="V198" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W198" s="6" t="inlineStr"/>
+      <c r="X198" s="6" t="n"/>
+      <c r="Y198" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z198" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA198" s="6" t="n"/>
+      <c r="AB198" s="6" t="n"/>
+      <c r="AC198" s="6" t="n"/>
+      <c r="AD198" s="6" t="n"/>
+      <c r="AE198" s="6" t="n"/>
+      <c r="AF198" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B199" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C199" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D199" s="4" t="inlineStr">
+        <is>
+          <t>910g</t>
+        </is>
+      </c>
+      <c r="E199" s="4" t="n">
+        <v>49.99</v>
+      </c>
+      <c r="F199" s="4" t="n"/>
+      <c r="G199" s="4" t="n"/>
+      <c r="H199" s="4" t="n">
+        <v>54.93</v>
+      </c>
+      <c r="I199" s="4" t="inlineStr"/>
+      <c r="J199" s="4" t="inlineStr"/>
+      <c r="K199" s="4" t="inlineStr"/>
+      <c r="L199" s="4" t="n">
+        <v>69.53</v>
+      </c>
+      <c r="M199" s="4" t="n">
+        <v>2.086</v>
+      </c>
+      <c r="N199" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O199" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P199" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q199" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R199" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S199" s="4" t="n"/>
+      <c r="T199" s="4" t="n"/>
+      <c r="U199" s="4" t="n"/>
+      <c r="V199" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W199" s="4" t="inlineStr"/>
+      <c r="X199" s="4" t="n"/>
+      <c r="Y199" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z199" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA199" s="4" t="n"/>
+      <c r="AB199" s="4" t="n"/>
+      <c r="AC199" s="4" t="n"/>
+      <c r="AD199" s="4" t="n"/>
+      <c r="AE199" s="4" t="n"/>
+      <c r="AF199" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B200" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C200" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D200" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E200" s="6" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="F200" s="6" t="n"/>
+      <c r="G200" s="6" t="n"/>
+      <c r="H200" s="6" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="I200" s="6" t="inlineStr"/>
+      <c r="J200" s="6" t="inlineStr"/>
+      <c r="K200" s="6" t="inlineStr"/>
+      <c r="L200" s="6" t="n">
+        <v>63.91</v>
+      </c>
+      <c r="M200" s="6" t="n">
+        <v>1.917</v>
+      </c>
+      <c r="N200" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O200" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P200" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q200" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R200" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S200" s="6" t="n"/>
+      <c r="T200" s="6" t="n"/>
+      <c r="U200" s="6" t="n"/>
+      <c r="V200" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W200" s="6" t="inlineStr"/>
+      <c r="X200" s="6" t="n"/>
+      <c r="Y200" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z200" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA200" s="6" t="n"/>
+      <c r="AB200" s="6" t="n"/>
+      <c r="AC200" s="6" t="n"/>
+      <c r="AD200" s="6" t="n"/>
+      <c r="AE200" s="6" t="n"/>
+      <c r="AF200" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B201" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C201" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D201" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E201" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F201" s="4" t="n"/>
+      <c r="G201" s="4" t="n"/>
+      <c r="H201" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I201" s="4" t="inlineStr"/>
+      <c r="J201" s="4" t="inlineStr"/>
+      <c r="K201" s="4" t="inlineStr"/>
+      <c r="L201" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M201" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N201" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O201" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P201" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q201" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R201" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S201" s="4" t="n"/>
+      <c r="T201" s="4" t="n"/>
+      <c r="U201" s="4" t="n"/>
+      <c r="V201" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W201" s="4" t="inlineStr"/>
+      <c r="X201" s="4" t="n"/>
+      <c r="Y201" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z201" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA201" s="4" t="n"/>
+      <c r="AB201" s="4" t="n"/>
+      <c r="AC201" s="4" t="n"/>
+      <c r="AD201" s="4" t="n"/>
+      <c r="AE201" s="4" t="n"/>
+      <c r="AF201" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B202" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C202" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D202" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E202" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F202" s="6" t="n"/>
+      <c r="G202" s="6" t="n"/>
+      <c r="H202" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I202" s="6" t="inlineStr"/>
+      <c r="J202" s="6" t="inlineStr"/>
+      <c r="K202" s="6" t="inlineStr"/>
+      <c r="L202" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M202" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N202" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O202" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P202" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q202" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R202" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S202" s="6" t="n"/>
+      <c r="T202" s="6" t="n"/>
+      <c r="U202" s="6" t="n"/>
+      <c r="V202" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W202" s="6" t="inlineStr"/>
+      <c r="X202" s="6" t="n"/>
+      <c r="Y202" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z202" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA202" s="6" t="n"/>
+      <c r="AB202" s="6" t="n"/>
+      <c r="AC202" s="6" t="n"/>
+      <c r="AD202" s="6" t="n"/>
+      <c r="AE202" s="6" t="n"/>
+      <c r="AF202" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B203" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C203" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D203" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E203" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F203" s="4" t="n"/>
+      <c r="G203" s="4" t="n"/>
+      <c r="H203" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I203" s="4" t="inlineStr"/>
+      <c r="J203" s="4" t="inlineStr"/>
+      <c r="K203" s="4" t="inlineStr"/>
+      <c r="L203" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M203" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N203" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O203" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P203" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q203" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R203" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S203" s="4" t="n"/>
+      <c r="T203" s="4" t="n"/>
+      <c r="U203" s="4" t="n"/>
+      <c r="V203" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W203" s="4" t="inlineStr"/>
+      <c r="X203" s="4" t="n"/>
+      <c r="Y203" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z203" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA203" s="4" t="n"/>
+      <c r="AB203" s="4" t="n"/>
+      <c r="AC203" s="4" t="n"/>
+      <c r="AD203" s="4" t="n"/>
+      <c r="AE203" s="4" t="n"/>
+      <c r="AF203" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B204" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C204" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D204" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E204" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F204" s="6" t="n"/>
+      <c r="G204" s="6" t="n"/>
+      <c r="H204" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I204" s="6" t="inlineStr"/>
+      <c r="J204" s="6" t="inlineStr"/>
+      <c r="K204" s="6" t="inlineStr"/>
+      <c r="L204" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M204" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N204" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O204" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P204" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q204" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R204" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S204" s="6" t="n"/>
+      <c r="T204" s="6" t="n"/>
+      <c r="U204" s="6" t="n"/>
+      <c r="V204" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W204" s="6" t="inlineStr"/>
+      <c r="X204" s="6" t="n"/>
+      <c r="Y204" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z204" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA204" s="6" t="n"/>
+      <c r="AB204" s="6" t="n"/>
+      <c r="AC204" s="6" t="n"/>
+      <c r="AD204" s="6" t="n"/>
+      <c r="AE204" s="6" t="n"/>
+      <c r="AF204" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B205" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C205" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D205" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E205" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F205" s="4" t="n"/>
+      <c r="G205" s="4" t="n"/>
+      <c r="H205" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I205" s="4" t="inlineStr"/>
+      <c r="J205" s="4" t="inlineStr"/>
+      <c r="K205" s="4" t="inlineStr"/>
+      <c r="L205" s="4" t="n"/>
+      <c r="M205" s="4" t="n"/>
+      <c r="N205" s="4" t="n"/>
+      <c r="O205" s="4" t="n"/>
+      <c r="P205" s="4" t="n"/>
+      <c r="Q205" s="4" t="n"/>
+      <c r="R205" s="4" t="n"/>
+      <c r="S205" s="4" t="n"/>
+      <c r="T205" s="4" t="n"/>
+      <c r="U205" s="4" t="n"/>
+      <c r="V205" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W205" s="4" t="inlineStr"/>
+      <c r="X205" s="4" t="n"/>
+      <c r="Y205" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z205" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA205" s="4" t="n"/>
+      <c r="AB205" s="4" t="n"/>
+      <c r="AC205" s="4" t="n"/>
+      <c r="AD205" s="4" t="n"/>
+      <c r="AE205" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF205" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B206" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C206" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D206" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E206" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F206" s="6" t="n"/>
+      <c r="G206" s="6" t="n"/>
+      <c r="H206" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I206" s="6" t="inlineStr"/>
+      <c r="J206" s="6" t="inlineStr"/>
+      <c r="K206" s="6" t="inlineStr"/>
+      <c r="L206" s="6" t="n"/>
+      <c r="M206" s="6" t="n"/>
+      <c r="N206" s="6" t="n"/>
+      <c r="O206" s="6" t="n"/>
+      <c r="P206" s="6" t="n"/>
+      <c r="Q206" s="6" t="n"/>
+      <c r="R206" s="6" t="n"/>
+      <c r="S206" s="6" t="n"/>
+      <c r="T206" s="6" t="n"/>
+      <c r="U206" s="6" t="n"/>
+      <c r="V206" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W206" s="6" t="inlineStr"/>
+      <c r="X206" s="6" t="n"/>
+      <c r="Y206" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z206" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA206" s="6" t="n"/>
+      <c r="AB206" s="6" t="n"/>
+      <c r="AC206" s="6" t="n"/>
+      <c r="AD206" s="6" t="n"/>
+      <c r="AE206" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF206" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B207" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C207" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D207" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E207" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F207" s="4" t="n"/>
+      <c r="G207" s="4" t="n"/>
+      <c r="H207" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I207" s="4" t="inlineStr"/>
+      <c r="J207" s="4" t="inlineStr"/>
+      <c r="K207" s="4" t="inlineStr"/>
+      <c r="L207" s="4" t="n"/>
+      <c r="M207" s="4" t="n"/>
+      <c r="N207" s="4" t="n"/>
+      <c r="O207" s="4" t="n"/>
+      <c r="P207" s="4" t="n"/>
+      <c r="Q207" s="4" t="n"/>
+      <c r="R207" s="4" t="n"/>
+      <c r="S207" s="4" t="n"/>
+      <c r="T207" s="4" t="n"/>
+      <c r="U207" s="4" t="n"/>
+      <c r="V207" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W207" s="4" t="inlineStr"/>
+      <c r="X207" s="4" t="n"/>
+      <c r="Y207" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z207" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA207" s="4" t="n"/>
+      <c r="AB207" s="4" t="n"/>
+      <c r="AC207" s="4" t="n"/>
+      <c r="AD207" s="4" t="n"/>
+      <c r="AE207" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF207" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B208" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C208" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D208" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E208" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F208" s="6" t="n"/>
+      <c r="G208" s="6" t="n"/>
+      <c r="H208" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I208" s="6" t="inlineStr"/>
+      <c r="J208" s="6" t="inlineStr"/>
+      <c r="K208" s="6" t="inlineStr"/>
+      <c r="L208" s="6" t="n"/>
+      <c r="M208" s="6" t="n"/>
+      <c r="N208" s="6" t="n"/>
+      <c r="O208" s="6" t="n"/>
+      <c r="P208" s="6" t="n"/>
+      <c r="Q208" s="6" t="n"/>
+      <c r="R208" s="6" t="n"/>
+      <c r="S208" s="6" t="n"/>
+      <c r="T208" s="6" t="n"/>
+      <c r="U208" s="6" t="n"/>
+      <c r="V208" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W208" s="6" t="inlineStr"/>
+      <c r="X208" s="6" t="n"/>
+      <c r="Y208" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z208" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA208" s="6" t="n"/>
+      <c r="AB208" s="6" t="n"/>
+      <c r="AC208" s="6" t="n"/>
+      <c r="AD208" s="6" t="n"/>
+      <c r="AE208" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF208" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B209" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C209" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D209" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E209" s="4" t="n">
+        <v>15.99</v>
+      </c>
+      <c r="F209" s="4" t="n"/>
+      <c r="G209" s="4" t="n"/>
+      <c r="H209" s="4" t="n">
+        <v>63.96</v>
+      </c>
+      <c r="I209" s="4" t="inlineStr"/>
+      <c r="J209" s="4" t="inlineStr"/>
+      <c r="K209" s="4" t="inlineStr"/>
+      <c r="L209" s="4" t="n"/>
+      <c r="M209" s="4" t="n"/>
+      <c r="N209" s="4" t="n"/>
+      <c r="O209" s="4" t="n"/>
+      <c r="P209" s="4" t="n"/>
+      <c r="Q209" s="4" t="n"/>
+      <c r="R209" s="4" t="n"/>
+      <c r="S209" s="4" t="n"/>
+      <c r="T209" s="4" t="n"/>
+      <c r="U209" s="4" t="n"/>
+      <c r="V209" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W209" s="4" t="inlineStr"/>
+      <c r="X209" s="4" t="n"/>
+      <c r="Y209" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z209" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA209" s="4" t="n"/>
+      <c r="AB209" s="4" t="n"/>
+      <c r="AC209" s="4" t="n"/>
+      <c r="AD209" s="4" t="n"/>
+      <c r="AE209" s="4" t="n">
+        <v>63.96</v>
+      </c>
+      <c r="AF209" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B210" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C210" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D210" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E210" s="6" t="n">
+        <v>23.69</v>
+      </c>
+      <c r="F210" s="6" t="n"/>
+      <c r="G210" s="6" t="n"/>
+      <c r="H210" s="6" t="n">
+        <v>47.38</v>
+      </c>
+      <c r="I210" s="6" t="inlineStr"/>
+      <c r="J210" s="6" t="inlineStr"/>
+      <c r="K210" s="6" t="inlineStr"/>
+      <c r="L210" s="6" t="n"/>
+      <c r="M210" s="6" t="n"/>
+      <c r="N210" s="6" t="n"/>
+      <c r="O210" s="6" t="n"/>
+      <c r="P210" s="6" t="n"/>
+      <c r="Q210" s="6" t="n"/>
+      <c r="R210" s="6" t="n"/>
+      <c r="S210" s="6" t="n"/>
+      <c r="T210" s="6" t="n"/>
+      <c r="U210" s="6" t="n"/>
+      <c r="V210" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W210" s="6" t="inlineStr"/>
+      <c r="X210" s="6" t="n"/>
+      <c r="Y210" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z210" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA210" s="6" t="n"/>
+      <c r="AB210" s="6" t="n"/>
+      <c r="AC210" s="6" t="n"/>
+      <c r="AD210" s="6" t="n"/>
+      <c r="AE210" s="6" t="n">
+        <v>47.38</v>
+      </c>
+      <c r="AF210" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B211" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C211" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D211" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E211" s="4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="F211" s="4" t="n"/>
+      <c r="G211" s="4" t="n"/>
+      <c r="H211" s="4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="I211" s="4" t="inlineStr"/>
+      <c r="J211" s="4" t="inlineStr"/>
+      <c r="K211" s="4" t="inlineStr"/>
+      <c r="L211" s="4" t="n"/>
+      <c r="M211" s="4" t="n"/>
+      <c r="N211" s="4" t="n"/>
+      <c r="O211" s="4" t="n"/>
+      <c r="P211" s="4" t="n"/>
+      <c r="Q211" s="4" t="n"/>
+      <c r="R211" s="4" t="n"/>
+      <c r="S211" s="4" t="n"/>
+      <c r="T211" s="4" t="n"/>
+      <c r="U211" s="4" t="n"/>
+      <c r="V211" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W211" s="4" t="inlineStr"/>
+      <c r="X211" s="4" t="n"/>
+      <c r="Y211" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z211" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA211" s="4" t="n"/>
+      <c r="AB211" s="4" t="n"/>
+      <c r="AC211" s="4" t="n"/>
+      <c r="AD211" s="4" t="n"/>
+      <c r="AE211" s="4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="AF211" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B212" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C212" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D212" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E212" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F212" s="6" t="n"/>
+      <c r="G212" s="6" t="n"/>
+      <c r="H212" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I212" s="6" t="inlineStr"/>
+      <c r="J212" s="6" t="inlineStr"/>
+      <c r="K212" s="6" t="inlineStr"/>
+      <c r="L212" s="6" t="n"/>
+      <c r="M212" s="6" t="n"/>
+      <c r="N212" s="6" t="n"/>
+      <c r="O212" s="6" t="n"/>
+      <c r="P212" s="6" t="n"/>
+      <c r="Q212" s="6" t="n"/>
+      <c r="R212" s="6" t="n"/>
+      <c r="S212" s="6" t="n"/>
+      <c r="T212" s="6" t="n"/>
+      <c r="U212" s="6" t="n"/>
+      <c r="V212" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W212" s="6" t="inlineStr"/>
+      <c r="X212" s="6" t="n"/>
+      <c r="Y212" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z212" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA212" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB212" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC212" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD212" s="6" t="n"/>
+      <c r="AE212" s="6" t="n"/>
+      <c r="AF212" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B213" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C213" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D213" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E213" s="4" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="F213" s="4" t="n"/>
+      <c r="G213" s="4" t="n"/>
+      <c r="H213" s="4" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="I213" s="4" t="inlineStr"/>
+      <c r="J213" s="4" t="inlineStr"/>
+      <c r="K213" s="4" t="inlineStr"/>
+      <c r="L213" s="4" t="n"/>
+      <c r="M213" s="4" t="n"/>
+      <c r="N213" s="4" t="n"/>
+      <c r="O213" s="4" t="n"/>
+      <c r="P213" s="4" t="n"/>
+      <c r="Q213" s="4" t="n"/>
+      <c r="R213" s="4" t="n"/>
+      <c r="S213" s="4" t="n"/>
+      <c r="T213" s="4" t="n"/>
+      <c r="U213" s="4" t="n"/>
+      <c r="V213" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W213" s="4" t="inlineStr"/>
+      <c r="X213" s="4" t="n"/>
+      <c r="Y213" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z213" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA213" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB213" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC213" s="4" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AD213" s="4" t="n"/>
+      <c r="AE213" s="4" t="n"/>
+      <c r="AF213" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B214" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C214" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D214" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E214" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F214" s="6" t="n"/>
+      <c r="G214" s="6" t="n"/>
+      <c r="H214" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I214" s="6" t="inlineStr"/>
+      <c r="J214" s="6" t="inlineStr"/>
+      <c r="K214" s="6" t="inlineStr"/>
+      <c r="L214" s="6" t="n"/>
+      <c r="M214" s="6" t="n"/>
+      <c r="N214" s="6" t="n"/>
+      <c r="O214" s="6" t="n"/>
+      <c r="P214" s="6" t="n"/>
+      <c r="Q214" s="6" t="n"/>
+      <c r="R214" s="6" t="n"/>
+      <c r="S214" s="6" t="n"/>
+      <c r="T214" s="6" t="n"/>
+      <c r="U214" s="6" t="n"/>
+      <c r="V214" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W214" s="6" t="inlineStr"/>
+      <c r="X214" s="6" t="n"/>
+      <c r="Y214" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z214" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA214" s="6" t="n"/>
+      <c r="AB214" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC214" s="6" t="n"/>
+      <c r="AD214" s="6" t="n"/>
+      <c r="AE214" s="6" t="n"/>
+      <c r="AF214" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-24</t>
+        </is>
+      </c>
+      <c r="B215" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C215" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D215" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E215" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F215" s="4" t="n"/>
+      <c r="G215" s="4" t="n"/>
+      <c r="H215" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I215" s="4" t="inlineStr"/>
+      <c r="J215" s="4" t="inlineStr"/>
+      <c r="K215" s="4" t="inlineStr"/>
+      <c r="L215" s="4" t="n"/>
+      <c r="M215" s="4" t="n"/>
+      <c r="N215" s="4" t="n"/>
+      <c r="O215" s="4" t="n"/>
+      <c r="P215" s="4" t="n"/>
+      <c r="Q215" s="4" t="n"/>
+      <c r="R215" s="4" t="n"/>
+      <c r="S215" s="4" t="n"/>
+      <c r="T215" s="4" t="n"/>
+      <c r="U215" s="4" t="n"/>
+      <c r="V215" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W215" s="4" t="inlineStr"/>
+      <c r="X215" s="4" t="n"/>
+      <c r="Y215" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z215" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA215" s="4" t="n"/>
+      <c r="AB215" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC215" s="4" t="n"/>
+      <c r="AD215" s="4" t="n"/>
+      <c r="AE215" s="4" t="n"/>
+      <c r="AF215" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-25
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF215"/>
+  <dimension ref="A1:AF252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -17482,6 +17482,2918 @@
         <v>1</v>
       </c>
     </row>
+    <row r="216">
+      <c r="A216" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B216" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C216" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D216" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E216" s="4" t="n">
+        <v>10.44</v>
+      </c>
+      <c r="F216" s="4" t="n"/>
+      <c r="G216" s="4" t="n"/>
+      <c r="H216" s="4" t="n">
+        <v>41.76</v>
+      </c>
+      <c r="I216" s="4" t="inlineStr"/>
+      <c r="J216" s="4" t="inlineStr"/>
+      <c r="K216" s="4" t="inlineStr"/>
+      <c r="L216" s="4" t="n">
+        <v>58</v>
+      </c>
+      <c r="M216" s="4" t="n">
+        <v>1.74</v>
+      </c>
+      <c r="N216" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O216" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P216" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q216" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R216" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S216" s="4" t="n"/>
+      <c r="T216" s="4" t="n"/>
+      <c r="U216" s="4" t="n"/>
+      <c r="V216" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W216" s="4" t="inlineStr"/>
+      <c r="X216" s="4" t="n"/>
+      <c r="Y216" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z216" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA216" s="4" t="n"/>
+      <c r="AB216" s="4" t="n"/>
+      <c r="AC216" s="4" t="n"/>
+      <c r="AD216" s="4" t="n"/>
+      <c r="AE216" s="4" t="n"/>
+      <c r="AF216" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B217" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C217" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D217" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E217" s="6" t="n">
+        <v>14.84</v>
+      </c>
+      <c r="F217" s="6" t="n"/>
+      <c r="G217" s="6" t="n"/>
+      <c r="H217" s="6" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="I217" s="6" t="inlineStr"/>
+      <c r="J217" s="6" t="inlineStr"/>
+      <c r="K217" s="6" t="inlineStr"/>
+      <c r="L217" s="6" t="n">
+        <v>59.74</v>
+      </c>
+      <c r="M217" s="6" t="n">
+        <v>1.792</v>
+      </c>
+      <c r="N217" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O217" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P217" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q217" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R217" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S217" s="6" t="n"/>
+      <c r="T217" s="6" t="n"/>
+      <c r="U217" s="6" t="n"/>
+      <c r="V217" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W217" s="6" t="inlineStr"/>
+      <c r="X217" s="6" t="n"/>
+      <c r="Y217" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z217" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA217" s="6" t="n"/>
+      <c r="AB217" s="6" t="n"/>
+      <c r="AC217" s="6" t="n"/>
+      <c r="AD217" s="6" t="n"/>
+      <c r="AE217" s="6" t="n"/>
+      <c r="AF217" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B218" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C218" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D218" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E218" s="4" t="n">
+        <v>19.79</v>
+      </c>
+      <c r="F218" s="4" t="n"/>
+      <c r="G218" s="4" t="n"/>
+      <c r="H218" s="4" t="n">
+        <v>32.98</v>
+      </c>
+      <c r="I218" s="4" t="inlineStr"/>
+      <c r="J218" s="4" t="inlineStr"/>
+      <c r="K218" s="4" t="inlineStr"/>
+      <c r="L218" s="4" t="n">
+        <v>45.81</v>
+      </c>
+      <c r="M218" s="4" t="n">
+        <v>1.374</v>
+      </c>
+      <c r="N218" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O218" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P218" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q218" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R218" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S218" s="4" t="n"/>
+      <c r="T218" s="4" t="n"/>
+      <c r="U218" s="4" t="n"/>
+      <c r="V218" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W218" s="4" t="inlineStr"/>
+      <c r="X218" s="4" t="n"/>
+      <c r="Y218" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z218" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA218" s="4" t="n"/>
+      <c r="AB218" s="4" t="n"/>
+      <c r="AC218" s="4" t="n"/>
+      <c r="AD218" s="4" t="n"/>
+      <c r="AE218" s="4" t="n"/>
+      <c r="AF218" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B219" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C219" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D219" s="6" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E219" s="6" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="F219" s="6" t="n"/>
+      <c r="G219" s="6" t="n"/>
+      <c r="H219" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="I219" s="6" t="inlineStr"/>
+      <c r="J219" s="6" t="inlineStr"/>
+      <c r="K219" s="6" t="inlineStr"/>
+      <c r="L219" s="6" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="M219" s="6" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="N219" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O219" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P219" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q219" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R219" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S219" s="6" t="n"/>
+      <c r="T219" s="6" t="n"/>
+      <c r="U219" s="6" t="n"/>
+      <c r="V219" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W219" s="6" t="inlineStr"/>
+      <c r="X219" s="6" t="n"/>
+      <c r="Y219" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z219" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA219" s="6" t="n"/>
+      <c r="AB219" s="6" t="n"/>
+      <c r="AC219" s="6" t="n"/>
+      <c r="AD219" s="6" t="n"/>
+      <c r="AE219" s="6" t="n"/>
+      <c r="AF219" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B220" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C220" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D220" s="4" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E220" s="4" t="n">
+        <v>24.19</v>
+      </c>
+      <c r="F220" s="4" t="n"/>
+      <c r="G220" s="4" t="n"/>
+      <c r="H220" s="4" t="n">
+        <v>32.25</v>
+      </c>
+      <c r="I220" s="4" t="inlineStr"/>
+      <c r="J220" s="4" t="inlineStr"/>
+      <c r="K220" s="4" t="inlineStr"/>
+      <c r="L220" s="4" t="n">
+        <v>44.79</v>
+      </c>
+      <c r="M220" s="4" t="n">
+        <v>1.344</v>
+      </c>
+      <c r="N220" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O220" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P220" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q220" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R220" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S220" s="4" t="n"/>
+      <c r="T220" s="4" t="n"/>
+      <c r="U220" s="4" t="n"/>
+      <c r="V220" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W220" s="4" t="inlineStr"/>
+      <c r="X220" s="4" t="n"/>
+      <c r="Y220" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z220" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA220" s="4" t="n"/>
+      <c r="AB220" s="4" t="n"/>
+      <c r="AC220" s="4" t="n"/>
+      <c r="AD220" s="4" t="n"/>
+      <c r="AE220" s="4" t="n"/>
+      <c r="AF220" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B221" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C221" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D221" s="6" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E221" s="6" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="F221" s="6" t="n"/>
+      <c r="G221" s="6" t="n"/>
+      <c r="H221" s="6" t="n">
+        <v>29.78</v>
+      </c>
+      <c r="I221" s="6" t="inlineStr"/>
+      <c r="J221" s="6" t="inlineStr"/>
+      <c r="K221" s="6" t="inlineStr"/>
+      <c r="L221" s="6" t="n">
+        <v>41.36</v>
+      </c>
+      <c r="M221" s="6" t="n">
+        <v>1.241</v>
+      </c>
+      <c r="N221" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O221" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P221" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q221" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R221" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S221" s="6" t="n"/>
+      <c r="T221" s="6" t="n"/>
+      <c r="U221" s="6" t="n"/>
+      <c r="V221" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W221" s="6" t="inlineStr"/>
+      <c r="X221" s="6" t="n"/>
+      <c r="Y221" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z221" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA221" s="6" t="n"/>
+      <c r="AB221" s="6" t="n"/>
+      <c r="AC221" s="6" t="n"/>
+      <c r="AD221" s="6" t="n"/>
+      <c r="AE221" s="6" t="n"/>
+      <c r="AF221" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B222" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C222" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D222" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E222" s="4" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="F222" s="4" t="n"/>
+      <c r="G222" s="4" t="n"/>
+      <c r="H222" s="4" t="n">
+        <v>28.59</v>
+      </c>
+      <c r="I222" s="4" t="inlineStr"/>
+      <c r="J222" s="4" t="inlineStr"/>
+      <c r="K222" s="4" t="inlineStr"/>
+      <c r="L222" s="4" t="n">
+        <v>39.71</v>
+      </c>
+      <c r="M222" s="4" t="n">
+        <v>1.191</v>
+      </c>
+      <c r="N222" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O222" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P222" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q222" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R222" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S222" s="4" t="n"/>
+      <c r="T222" s="4" t="n"/>
+      <c r="U222" s="4" t="n"/>
+      <c r="V222" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W222" s="4" t="inlineStr"/>
+      <c r="X222" s="4" t="n"/>
+      <c r="Y222" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z222" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA222" s="4" t="n"/>
+      <c r="AB222" s="4" t="n"/>
+      <c r="AC222" s="4" t="n"/>
+      <c r="AD222" s="4" t="n"/>
+      <c r="AE222" s="4" t="n"/>
+      <c r="AF222" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B223" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C223" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D223" s="6" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E223" s="6" t="n">
+        <v>54.99</v>
+      </c>
+      <c r="F223" s="6" t="n"/>
+      <c r="G223" s="6" t="n"/>
+      <c r="H223" s="6" t="n">
+        <v>28.64</v>
+      </c>
+      <c r="I223" s="6" t="inlineStr"/>
+      <c r="J223" s="6" t="inlineStr"/>
+      <c r="K223" s="6" t="inlineStr"/>
+      <c r="L223" s="6" t="n">
+        <v>39.78</v>
+      </c>
+      <c r="M223" s="6" t="n">
+        <v>1.193</v>
+      </c>
+      <c r="N223" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O223" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P223" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q223" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R223" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S223" s="6" t="n"/>
+      <c r="T223" s="6" t="n"/>
+      <c r="U223" s="6" t="n"/>
+      <c r="V223" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W223" s="6" t="inlineStr"/>
+      <c r="X223" s="6" t="n"/>
+      <c r="Y223" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z223" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA223" s="6" t="n"/>
+      <c r="AB223" s="6" t="n"/>
+      <c r="AC223" s="6" t="n"/>
+      <c r="AD223" s="6" t="n"/>
+      <c r="AE223" s="6" t="n"/>
+      <c r="AF223" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B224" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C224" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D224" s="4" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E224" s="4" t="n">
+        <v>67.64</v>
+      </c>
+      <c r="F224" s="4" t="n"/>
+      <c r="G224" s="4" t="n"/>
+      <c r="H224" s="4" t="n">
+        <v>32.68</v>
+      </c>
+      <c r="I224" s="4" t="inlineStr"/>
+      <c r="J224" s="4" t="inlineStr"/>
+      <c r="K224" s="4" t="inlineStr"/>
+      <c r="L224" s="4" t="n">
+        <v>45.39</v>
+      </c>
+      <c r="M224" s="4" t="n">
+        <v>1.362</v>
+      </c>
+      <c r="N224" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O224" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P224" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q224" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R224" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S224" s="4" t="n"/>
+      <c r="T224" s="4" t="n"/>
+      <c r="U224" s="4" t="n"/>
+      <c r="V224" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W224" s="4" t="inlineStr"/>
+      <c r="X224" s="4" t="n"/>
+      <c r="Y224" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z224" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA224" s="4" t="n"/>
+      <c r="AB224" s="4" t="n"/>
+      <c r="AC224" s="4" t="n"/>
+      <c r="AD224" s="4" t="n"/>
+      <c r="AE224" s="4" t="n"/>
+      <c r="AF224" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B225" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C225" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D225" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E225" s="6" t="n">
+        <v>68.73999999999999</v>
+      </c>
+      <c r="F225" s="6" t="n"/>
+      <c r="G225" s="6" t="n"/>
+      <c r="H225" s="6" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="I225" s="6" t="inlineStr"/>
+      <c r="J225" s="6" t="inlineStr"/>
+      <c r="K225" s="6" t="inlineStr"/>
+      <c r="L225" s="6" t="n">
+        <v>38.19</v>
+      </c>
+      <c r="M225" s="6" t="n">
+        <v>1.146</v>
+      </c>
+      <c r="N225" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O225" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P225" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q225" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R225" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S225" s="6" t="n"/>
+      <c r="T225" s="6" t="n"/>
+      <c r="U225" s="6" t="n"/>
+      <c r="V225" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W225" s="6" t="inlineStr"/>
+      <c r="X225" s="6" t="n"/>
+      <c r="Y225" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z225" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA225" s="6" t="n"/>
+      <c r="AB225" s="6" t="n"/>
+      <c r="AC225" s="6" t="n"/>
+      <c r="AD225" s="6" t="n"/>
+      <c r="AE225" s="6" t="n"/>
+      <c r="AF225" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B226" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C226" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D226" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E226" s="4" t="n">
+        <v>108.34</v>
+      </c>
+      <c r="F226" s="4" t="n"/>
+      <c r="G226" s="4" t="n"/>
+      <c r="H226" s="4" t="n">
+        <v>30.09</v>
+      </c>
+      <c r="I226" s="4" t="inlineStr"/>
+      <c r="J226" s="4" t="inlineStr"/>
+      <c r="K226" s="4" t="inlineStr"/>
+      <c r="L226" s="4" t="n">
+        <v>41.79</v>
+      </c>
+      <c r="M226" s="4" t="n">
+        <v>1.254</v>
+      </c>
+      <c r="N226" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O226" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P226" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q226" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R226" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S226" s="4" t="n"/>
+      <c r="T226" s="4" t="n"/>
+      <c r="U226" s="4" t="n"/>
+      <c r="V226" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W226" s="4" t="inlineStr"/>
+      <c r="X226" s="4" t="n"/>
+      <c r="Y226" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z226" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA226" s="4" t="n"/>
+      <c r="AB226" s="4" t="n"/>
+      <c r="AC226" s="4" t="n"/>
+      <c r="AD226" s="4" t="n"/>
+      <c r="AE226" s="4" t="n"/>
+      <c r="AF226" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B227" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C227" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D227" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E227" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F227" s="6" t="n"/>
+      <c r="G227" s="6" t="n"/>
+      <c r="H227" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I227" s="6" t="inlineStr"/>
+      <c r="J227" s="6" t="inlineStr"/>
+      <c r="K227" s="6" t="inlineStr"/>
+      <c r="L227" s="6" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M227" s="6" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N227" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O227" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P227" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q227" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R227" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S227" s="6" t="n"/>
+      <c r="T227" s="6" t="n"/>
+      <c r="U227" s="6" t="n"/>
+      <c r="V227" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W227" s="6" t="inlineStr"/>
+      <c r="X227" s="6" t="n"/>
+      <c r="Y227" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z227" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA227" s="6" t="n"/>
+      <c r="AB227" s="6" t="n"/>
+      <c r="AC227" s="6" t="n"/>
+      <c r="AD227" s="6" t="n"/>
+      <c r="AE227" s="6" t="n"/>
+      <c r="AF227" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B228" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C228" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D228" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E228" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F228" s="4" t="n"/>
+      <c r="G228" s="4" t="n"/>
+      <c r="H228" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I228" s="4" t="inlineStr"/>
+      <c r="J228" s="4" t="inlineStr"/>
+      <c r="K228" s="4" t="inlineStr"/>
+      <c r="L228" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M228" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N228" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O228" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P228" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q228" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R228" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S228" s="4" t="n"/>
+      <c r="T228" s="4" t="n"/>
+      <c r="U228" s="4" t="n"/>
+      <c r="V228" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W228" s="4" t="inlineStr"/>
+      <c r="X228" s="4" t="n"/>
+      <c r="Y228" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z228" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA228" s="4" t="n"/>
+      <c r="AB228" s="4" t="n"/>
+      <c r="AC228" s="4" t="n"/>
+      <c r="AD228" s="4" t="n"/>
+      <c r="AE228" s="4" t="n"/>
+      <c r="AF228" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B229" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C229" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D229" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E229" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F229" s="6" t="n"/>
+      <c r="G229" s="6" t="n"/>
+      <c r="H229" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I229" s="6" t="inlineStr"/>
+      <c r="J229" s="6" t="inlineStr"/>
+      <c r="K229" s="6" t="inlineStr"/>
+      <c r="L229" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M229" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N229" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O229" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P229" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q229" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R229" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S229" s="6" t="n"/>
+      <c r="T229" s="6" t="n"/>
+      <c r="U229" s="6" t="n"/>
+      <c r="V229" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W229" s="6" t="inlineStr"/>
+      <c r="X229" s="6" t="n"/>
+      <c r="Y229" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z229" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA229" s="6" t="n"/>
+      <c r="AB229" s="6" t="n"/>
+      <c r="AC229" s="6" t="n"/>
+      <c r="AD229" s="6" t="n"/>
+      <c r="AE229" s="6" t="n"/>
+      <c r="AF229" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B230" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C230" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D230" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E230" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F230" s="4" t="n"/>
+      <c r="G230" s="4" t="n"/>
+      <c r="H230" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I230" s="4" t="inlineStr"/>
+      <c r="J230" s="4" t="inlineStr"/>
+      <c r="K230" s="4" t="inlineStr"/>
+      <c r="L230" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M230" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N230" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O230" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P230" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q230" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R230" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S230" s="4" t="n"/>
+      <c r="T230" s="4" t="n"/>
+      <c r="U230" s="4" t="n"/>
+      <c r="V230" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W230" s="4" t="inlineStr"/>
+      <c r="X230" s="4" t="n"/>
+      <c r="Y230" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z230" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA230" s="4" t="n"/>
+      <c r="AB230" s="4" t="n"/>
+      <c r="AC230" s="4" t="n"/>
+      <c r="AD230" s="4" t="n"/>
+      <c r="AE230" s="4" t="n"/>
+      <c r="AF230" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B231" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C231" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D231" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E231" s="6" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F231" s="6" t="n"/>
+      <c r="G231" s="6" t="n"/>
+      <c r="H231" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I231" s="6" t="inlineStr"/>
+      <c r="J231" s="6" t="inlineStr"/>
+      <c r="K231" s="6" t="inlineStr"/>
+      <c r="L231" s="6" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M231" s="6" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N231" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O231" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P231" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q231" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R231" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S231" s="6" t="n"/>
+      <c r="T231" s="6" t="n"/>
+      <c r="U231" s="6" t="n"/>
+      <c r="V231" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W231" s="6" t="inlineStr"/>
+      <c r="X231" s="6" t="n"/>
+      <c r="Y231" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z231" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA231" s="6" t="n"/>
+      <c r="AB231" s="6" t="n"/>
+      <c r="AC231" s="6" t="n"/>
+      <c r="AD231" s="6" t="n"/>
+      <c r="AE231" s="6" t="n"/>
+      <c r="AF231" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B232" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C232" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D232" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E232" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F232" s="4" t="n"/>
+      <c r="G232" s="4" t="n"/>
+      <c r="H232" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I232" s="4" t="inlineStr"/>
+      <c r="J232" s="4" t="inlineStr"/>
+      <c r="K232" s="4" t="inlineStr"/>
+      <c r="L232" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M232" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N232" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O232" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P232" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q232" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R232" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S232" s="4" t="n"/>
+      <c r="T232" s="4" t="n"/>
+      <c r="U232" s="4" t="n"/>
+      <c r="V232" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W232" s="4" t="inlineStr"/>
+      <c r="X232" s="4" t="n"/>
+      <c r="Y232" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z232" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA232" s="4" t="n"/>
+      <c r="AB232" s="4" t="n"/>
+      <c r="AC232" s="4" t="n"/>
+      <c r="AD232" s="4" t="n"/>
+      <c r="AE232" s="4" t="n"/>
+      <c r="AF232" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B233" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C233" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D233" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E233" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F233" s="6" t="n"/>
+      <c r="G233" s="6" t="n"/>
+      <c r="H233" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I233" s="6" t="inlineStr"/>
+      <c r="J233" s="6" t="inlineStr"/>
+      <c r="K233" s="6" t="inlineStr"/>
+      <c r="L233" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M233" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N233" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O233" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P233" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q233" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R233" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S233" s="6" t="n"/>
+      <c r="T233" s="6" t="n"/>
+      <c r="U233" s="6" t="n"/>
+      <c r="V233" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W233" s="6" t="inlineStr"/>
+      <c r="X233" s="6" t="n"/>
+      <c r="Y233" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z233" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA233" s="6" t="n"/>
+      <c r="AB233" s="6" t="n"/>
+      <c r="AC233" s="6" t="n"/>
+      <c r="AD233" s="6" t="n"/>
+      <c r="AE233" s="6" t="n"/>
+      <c r="AF233" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B234" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C234" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D234" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E234" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F234" s="4" t="n"/>
+      <c r="G234" s="4" t="n"/>
+      <c r="H234" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I234" s="4" t="inlineStr"/>
+      <c r="J234" s="4" t="inlineStr"/>
+      <c r="K234" s="4" t="inlineStr"/>
+      <c r="L234" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M234" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N234" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O234" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P234" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q234" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R234" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S234" s="4" t="n"/>
+      <c r="T234" s="4" t="n"/>
+      <c r="U234" s="4" t="n"/>
+      <c r="V234" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W234" s="4" t="inlineStr"/>
+      <c r="X234" s="4" t="n"/>
+      <c r="Y234" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z234" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA234" s="4" t="n"/>
+      <c r="AB234" s="4" t="n"/>
+      <c r="AC234" s="4" t="n"/>
+      <c r="AD234" s="4" t="n"/>
+      <c r="AE234" s="4" t="n"/>
+      <c r="AF234" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B235" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C235" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D235" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E235" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F235" s="6" t="n"/>
+      <c r="G235" s="6" t="n"/>
+      <c r="H235" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I235" s="6" t="inlineStr"/>
+      <c r="J235" s="6" t="inlineStr"/>
+      <c r="K235" s="6" t="inlineStr"/>
+      <c r="L235" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M235" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N235" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O235" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P235" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q235" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R235" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S235" s="6" t="n"/>
+      <c r="T235" s="6" t="n"/>
+      <c r="U235" s="6" t="n"/>
+      <c r="V235" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W235" s="6" t="inlineStr"/>
+      <c r="X235" s="6" t="n"/>
+      <c r="Y235" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z235" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA235" s="6" t="n"/>
+      <c r="AB235" s="6" t="n"/>
+      <c r="AC235" s="6" t="n"/>
+      <c r="AD235" s="6" t="n"/>
+      <c r="AE235" s="6" t="n"/>
+      <c r="AF235" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B236" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C236" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D236" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E236" s="4" t="n">
+        <v>51.09</v>
+      </c>
+      <c r="F236" s="4" t="n"/>
+      <c r="G236" s="4" t="n"/>
+      <c r="H236" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="I236" s="4" t="inlineStr"/>
+      <c r="J236" s="4" t="inlineStr"/>
+      <c r="K236" s="4" t="inlineStr"/>
+      <c r="L236" s="4" t="n">
+        <v>73.91</v>
+      </c>
+      <c r="M236" s="4" t="n">
+        <v>2.217</v>
+      </c>
+      <c r="N236" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O236" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P236" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q236" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R236" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S236" s="4" t="n"/>
+      <c r="T236" s="4" t="n"/>
+      <c r="U236" s="4" t="n"/>
+      <c r="V236" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W236" s="4" t="inlineStr"/>
+      <c r="X236" s="4" t="n"/>
+      <c r="Y236" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z236" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA236" s="4" t="n"/>
+      <c r="AB236" s="4" t="n"/>
+      <c r="AC236" s="4" t="n"/>
+      <c r="AD236" s="4" t="n"/>
+      <c r="AE236" s="4" t="n"/>
+      <c r="AF236" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B237" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C237" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D237" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E237" s="6" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="F237" s="6" t="n"/>
+      <c r="G237" s="6" t="n"/>
+      <c r="H237" s="6" t="n">
+        <v>50.49</v>
+      </c>
+      <c r="I237" s="6" t="inlineStr"/>
+      <c r="J237" s="6" t="inlineStr"/>
+      <c r="K237" s="6" t="inlineStr"/>
+      <c r="L237" s="6" t="n">
+        <v>63.91</v>
+      </c>
+      <c r="M237" s="6" t="n">
+        <v>1.917</v>
+      </c>
+      <c r="N237" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O237" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P237" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q237" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R237" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S237" s="6" t="n"/>
+      <c r="T237" s="6" t="n"/>
+      <c r="U237" s="6" t="n"/>
+      <c r="V237" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W237" s="6" t="inlineStr"/>
+      <c r="X237" s="6" t="n"/>
+      <c r="Y237" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z237" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA237" s="6" t="n"/>
+      <c r="AB237" s="6" t="n"/>
+      <c r="AC237" s="6" t="n"/>
+      <c r="AD237" s="6" t="n"/>
+      <c r="AE237" s="6" t="n"/>
+      <c r="AF237" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B238" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C238" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D238" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E238" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F238" s="4" t="n"/>
+      <c r="G238" s="4" t="n"/>
+      <c r="H238" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I238" s="4" t="inlineStr"/>
+      <c r="J238" s="4" t="inlineStr"/>
+      <c r="K238" s="4" t="inlineStr"/>
+      <c r="L238" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M238" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N238" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O238" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P238" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q238" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R238" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S238" s="4" t="n"/>
+      <c r="T238" s="4" t="n"/>
+      <c r="U238" s="4" t="n"/>
+      <c r="V238" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W238" s="4" t="inlineStr"/>
+      <c r="X238" s="4" t="n"/>
+      <c r="Y238" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z238" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA238" s="4" t="n"/>
+      <c r="AB238" s="4" t="n"/>
+      <c r="AC238" s="4" t="n"/>
+      <c r="AD238" s="4" t="n"/>
+      <c r="AE238" s="4" t="n"/>
+      <c r="AF238" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B239" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C239" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D239" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E239" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F239" s="6" t="n"/>
+      <c r="G239" s="6" t="n"/>
+      <c r="H239" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I239" s="6" t="inlineStr"/>
+      <c r="J239" s="6" t="inlineStr"/>
+      <c r="K239" s="6" t="inlineStr"/>
+      <c r="L239" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M239" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N239" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O239" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P239" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q239" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R239" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S239" s="6" t="n"/>
+      <c r="T239" s="6" t="n"/>
+      <c r="U239" s="6" t="n"/>
+      <c r="V239" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W239" s="6" t="inlineStr"/>
+      <c r="X239" s="6" t="n"/>
+      <c r="Y239" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z239" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA239" s="6" t="n"/>
+      <c r="AB239" s="6" t="n"/>
+      <c r="AC239" s="6" t="n"/>
+      <c r="AD239" s="6" t="n"/>
+      <c r="AE239" s="6" t="n"/>
+      <c r="AF239" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B240" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C240" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D240" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E240" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F240" s="4" t="n"/>
+      <c r="G240" s="4" t="n"/>
+      <c r="H240" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I240" s="4" t="inlineStr"/>
+      <c r="J240" s="4" t="inlineStr"/>
+      <c r="K240" s="4" t="inlineStr"/>
+      <c r="L240" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M240" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N240" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O240" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P240" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q240" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R240" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S240" s="4" t="n"/>
+      <c r="T240" s="4" t="n"/>
+      <c r="U240" s="4" t="n"/>
+      <c r="V240" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W240" s="4" t="inlineStr"/>
+      <c r="X240" s="4" t="n"/>
+      <c r="Y240" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z240" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA240" s="4" t="n"/>
+      <c r="AB240" s="4" t="n"/>
+      <c r="AC240" s="4" t="n"/>
+      <c r="AD240" s="4" t="n"/>
+      <c r="AE240" s="4" t="n"/>
+      <c r="AF240" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B241" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C241" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D241" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E241" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F241" s="6" t="n"/>
+      <c r="G241" s="6" t="n"/>
+      <c r="H241" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I241" s="6" t="inlineStr"/>
+      <c r="J241" s="6" t="inlineStr"/>
+      <c r="K241" s="6" t="inlineStr"/>
+      <c r="L241" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M241" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N241" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O241" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P241" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q241" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R241" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S241" s="6" t="n"/>
+      <c r="T241" s="6" t="n"/>
+      <c r="U241" s="6" t="n"/>
+      <c r="V241" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W241" s="6" t="inlineStr"/>
+      <c r="X241" s="6" t="n"/>
+      <c r="Y241" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z241" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA241" s="6" t="n"/>
+      <c r="AB241" s="6" t="n"/>
+      <c r="AC241" s="6" t="n"/>
+      <c r="AD241" s="6" t="n"/>
+      <c r="AE241" s="6" t="n"/>
+      <c r="AF241" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B242" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C242" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D242" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E242" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F242" s="4" t="n"/>
+      <c r="G242" s="4" t="n"/>
+      <c r="H242" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I242" s="4" t="inlineStr"/>
+      <c r="J242" s="4" t="inlineStr"/>
+      <c r="K242" s="4" t="inlineStr"/>
+      <c r="L242" s="4" t="n"/>
+      <c r="M242" s="4" t="n"/>
+      <c r="N242" s="4" t="n"/>
+      <c r="O242" s="4" t="n"/>
+      <c r="P242" s="4" t="n"/>
+      <c r="Q242" s="4" t="n"/>
+      <c r="R242" s="4" t="n"/>
+      <c r="S242" s="4" t="n"/>
+      <c r="T242" s="4" t="n"/>
+      <c r="U242" s="4" t="n"/>
+      <c r="V242" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W242" s="4" t="inlineStr"/>
+      <c r="X242" s="4" t="n"/>
+      <c r="Y242" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z242" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA242" s="4" t="n"/>
+      <c r="AB242" s="4" t="n"/>
+      <c r="AC242" s="4" t="n"/>
+      <c r="AD242" s="4" t="n"/>
+      <c r="AE242" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF242" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B243" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C243" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D243" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E243" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F243" s="6" t="n"/>
+      <c r="G243" s="6" t="n"/>
+      <c r="H243" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I243" s="6" t="inlineStr"/>
+      <c r="J243" s="6" t="inlineStr"/>
+      <c r="K243" s="6" t="inlineStr"/>
+      <c r="L243" s="6" t="n"/>
+      <c r="M243" s="6" t="n"/>
+      <c r="N243" s="6" t="n"/>
+      <c r="O243" s="6" t="n"/>
+      <c r="P243" s="6" t="n"/>
+      <c r="Q243" s="6" t="n"/>
+      <c r="R243" s="6" t="n"/>
+      <c r="S243" s="6" t="n"/>
+      <c r="T243" s="6" t="n"/>
+      <c r="U243" s="6" t="n"/>
+      <c r="V243" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W243" s="6" t="inlineStr"/>
+      <c r="X243" s="6" t="n"/>
+      <c r="Y243" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z243" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA243" s="6" t="n"/>
+      <c r="AB243" s="6" t="n"/>
+      <c r="AC243" s="6" t="n"/>
+      <c r="AD243" s="6" t="n"/>
+      <c r="AE243" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF243" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B244" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C244" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D244" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E244" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F244" s="4" t="n"/>
+      <c r="G244" s="4" t="n"/>
+      <c r="H244" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I244" s="4" t="inlineStr"/>
+      <c r="J244" s="4" t="inlineStr"/>
+      <c r="K244" s="4" t="inlineStr"/>
+      <c r="L244" s="4" t="n"/>
+      <c r="M244" s="4" t="n"/>
+      <c r="N244" s="4" t="n"/>
+      <c r="O244" s="4" t="n"/>
+      <c r="P244" s="4" t="n"/>
+      <c r="Q244" s="4" t="n"/>
+      <c r="R244" s="4" t="n"/>
+      <c r="S244" s="4" t="n"/>
+      <c r="T244" s="4" t="n"/>
+      <c r="U244" s="4" t="n"/>
+      <c r="V244" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W244" s="4" t="inlineStr"/>
+      <c r="X244" s="4" t="n"/>
+      <c r="Y244" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z244" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA244" s="4" t="n"/>
+      <c r="AB244" s="4" t="n"/>
+      <c r="AC244" s="4" t="n"/>
+      <c r="AD244" s="4" t="n"/>
+      <c r="AE244" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF244" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B245" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C245" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D245" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E245" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F245" s="6" t="n"/>
+      <c r="G245" s="6" t="n"/>
+      <c r="H245" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I245" s="6" t="inlineStr"/>
+      <c r="J245" s="6" t="inlineStr"/>
+      <c r="K245" s="6" t="inlineStr"/>
+      <c r="L245" s="6" t="n"/>
+      <c r="M245" s="6" t="n"/>
+      <c r="N245" s="6" t="n"/>
+      <c r="O245" s="6" t="n"/>
+      <c r="P245" s="6" t="n"/>
+      <c r="Q245" s="6" t="n"/>
+      <c r="R245" s="6" t="n"/>
+      <c r="S245" s="6" t="n"/>
+      <c r="T245" s="6" t="n"/>
+      <c r="U245" s="6" t="n"/>
+      <c r="V245" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W245" s="6" t="inlineStr"/>
+      <c r="X245" s="6" t="n"/>
+      <c r="Y245" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z245" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA245" s="6" t="n"/>
+      <c r="AB245" s="6" t="n"/>
+      <c r="AC245" s="6" t="n"/>
+      <c r="AD245" s="6" t="n"/>
+      <c r="AE245" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF245" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B246" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C246" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D246" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E246" s="4" t="n">
+        <v>15.99</v>
+      </c>
+      <c r="F246" s="4" t="n"/>
+      <c r="G246" s="4" t="n"/>
+      <c r="H246" s="4" t="n">
+        <v>63.96</v>
+      </c>
+      <c r="I246" s="4" t="inlineStr"/>
+      <c r="J246" s="4" t="inlineStr"/>
+      <c r="K246" s="4" t="inlineStr"/>
+      <c r="L246" s="4" t="n"/>
+      <c r="M246" s="4" t="n"/>
+      <c r="N246" s="4" t="n"/>
+      <c r="O246" s="4" t="n"/>
+      <c r="P246" s="4" t="n"/>
+      <c r="Q246" s="4" t="n"/>
+      <c r="R246" s="4" t="n"/>
+      <c r="S246" s="4" t="n"/>
+      <c r="T246" s="4" t="n"/>
+      <c r="U246" s="4" t="n"/>
+      <c r="V246" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W246" s="4" t="inlineStr"/>
+      <c r="X246" s="4" t="n"/>
+      <c r="Y246" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z246" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA246" s="4" t="n"/>
+      <c r="AB246" s="4" t="n"/>
+      <c r="AC246" s="4" t="n"/>
+      <c r="AD246" s="4" t="n"/>
+      <c r="AE246" s="4" t="n">
+        <v>63.96</v>
+      </c>
+      <c r="AF246" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B247" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C247" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D247" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E247" s="6" t="n">
+        <v>23.69</v>
+      </c>
+      <c r="F247" s="6" t="n"/>
+      <c r="G247" s="6" t="n"/>
+      <c r="H247" s="6" t="n">
+        <v>47.38</v>
+      </c>
+      <c r="I247" s="6" t="inlineStr"/>
+      <c r="J247" s="6" t="inlineStr"/>
+      <c r="K247" s="6" t="inlineStr"/>
+      <c r="L247" s="6" t="n"/>
+      <c r="M247" s="6" t="n"/>
+      <c r="N247" s="6" t="n"/>
+      <c r="O247" s="6" t="n"/>
+      <c r="P247" s="6" t="n"/>
+      <c r="Q247" s="6" t="n"/>
+      <c r="R247" s="6" t="n"/>
+      <c r="S247" s="6" t="n"/>
+      <c r="T247" s="6" t="n"/>
+      <c r="U247" s="6" t="n"/>
+      <c r="V247" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W247" s="6" t="inlineStr"/>
+      <c r="X247" s="6" t="n"/>
+      <c r="Y247" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z247" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA247" s="6" t="n"/>
+      <c r="AB247" s="6" t="n"/>
+      <c r="AC247" s="6" t="n"/>
+      <c r="AD247" s="6" t="n"/>
+      <c r="AE247" s="6" t="n">
+        <v>47.38</v>
+      </c>
+      <c r="AF247" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B248" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C248" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D248" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E248" s="4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="F248" s="4" t="n"/>
+      <c r="G248" s="4" t="n"/>
+      <c r="H248" s="4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="I248" s="4" t="inlineStr"/>
+      <c r="J248" s="4" t="inlineStr"/>
+      <c r="K248" s="4" t="inlineStr"/>
+      <c r="L248" s="4" t="n"/>
+      <c r="M248" s="4" t="n"/>
+      <c r="N248" s="4" t="n"/>
+      <c r="O248" s="4" t="n"/>
+      <c r="P248" s="4" t="n"/>
+      <c r="Q248" s="4" t="n"/>
+      <c r="R248" s="4" t="n"/>
+      <c r="S248" s="4" t="n"/>
+      <c r="T248" s="4" t="n"/>
+      <c r="U248" s="4" t="n"/>
+      <c r="V248" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W248" s="4" t="inlineStr"/>
+      <c r="X248" s="4" t="n"/>
+      <c r="Y248" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z248" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA248" s="4" t="n"/>
+      <c r="AB248" s="4" t="n"/>
+      <c r="AC248" s="4" t="n"/>
+      <c r="AD248" s="4" t="n"/>
+      <c r="AE248" s="4" t="n">
+        <v>46.49</v>
+      </c>
+      <c r="AF248" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B249" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C249" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D249" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E249" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F249" s="6" t="n"/>
+      <c r="G249" s="6" t="n"/>
+      <c r="H249" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I249" s="6" t="inlineStr"/>
+      <c r="J249" s="6" t="inlineStr"/>
+      <c r="K249" s="6" t="inlineStr"/>
+      <c r="L249" s="6" t="n"/>
+      <c r="M249" s="6" t="n"/>
+      <c r="N249" s="6" t="n"/>
+      <c r="O249" s="6" t="n"/>
+      <c r="P249" s="6" t="n"/>
+      <c r="Q249" s="6" t="n"/>
+      <c r="R249" s="6" t="n"/>
+      <c r="S249" s="6" t="n"/>
+      <c r="T249" s="6" t="n"/>
+      <c r="U249" s="6" t="n"/>
+      <c r="V249" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W249" s="6" t="inlineStr"/>
+      <c r="X249" s="6" t="n"/>
+      <c r="Y249" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z249" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA249" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB249" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC249" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD249" s="6" t="n"/>
+      <c r="AE249" s="6" t="n"/>
+      <c r="AF249" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B250" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C250" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D250" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E250" s="4" t="n">
+        <v>21.49</v>
+      </c>
+      <c r="F250" s="4" t="n"/>
+      <c r="G250" s="4" t="n"/>
+      <c r="H250" s="4" t="n">
+        <v>85.95999999999999</v>
+      </c>
+      <c r="I250" s="4" t="inlineStr"/>
+      <c r="J250" s="4" t="inlineStr"/>
+      <c r="K250" s="4" t="inlineStr"/>
+      <c r="L250" s="4" t="n"/>
+      <c r="M250" s="4" t="n"/>
+      <c r="N250" s="4" t="n"/>
+      <c r="O250" s="4" t="n"/>
+      <c r="P250" s="4" t="n"/>
+      <c r="Q250" s="4" t="n"/>
+      <c r="R250" s="4" t="n"/>
+      <c r="S250" s="4" t="n"/>
+      <c r="T250" s="4" t="n"/>
+      <c r="U250" s="4" t="n"/>
+      <c r="V250" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W250" s="4" t="inlineStr"/>
+      <c r="X250" s="4" t="n"/>
+      <c r="Y250" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z250" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA250" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB250" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC250" s="4" t="n">
+        <v>0.287</v>
+      </c>
+      <c r="AD250" s="4" t="n"/>
+      <c r="AE250" s="4" t="n"/>
+      <c r="AF250" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B251" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C251" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D251" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E251" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F251" s="6" t="n"/>
+      <c r="G251" s="6" t="n"/>
+      <c r="H251" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I251" s="6" t="inlineStr"/>
+      <c r="J251" s="6" t="inlineStr"/>
+      <c r="K251" s="6" t="inlineStr"/>
+      <c r="L251" s="6" t="n"/>
+      <c r="M251" s="6" t="n"/>
+      <c r="N251" s="6" t="n"/>
+      <c r="O251" s="6" t="n"/>
+      <c r="P251" s="6" t="n"/>
+      <c r="Q251" s="6" t="n"/>
+      <c r="R251" s="6" t="n"/>
+      <c r="S251" s="6" t="n"/>
+      <c r="T251" s="6" t="n"/>
+      <c r="U251" s="6" t="n"/>
+      <c r="V251" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W251" s="6" t="inlineStr"/>
+      <c r="X251" s="6" t="n"/>
+      <c r="Y251" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z251" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA251" s="6" t="n"/>
+      <c r="AB251" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC251" s="6" t="n"/>
+      <c r="AD251" s="6" t="n"/>
+      <c r="AE251" s="6" t="n"/>
+      <c r="AF251" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-25</t>
+        </is>
+      </c>
+      <c r="B252" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C252" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D252" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E252" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F252" s="4" t="n"/>
+      <c r="G252" s="4" t="n"/>
+      <c r="H252" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I252" s="4" t="inlineStr"/>
+      <c r="J252" s="4" t="inlineStr"/>
+      <c r="K252" s="4" t="inlineStr"/>
+      <c r="L252" s="4" t="n"/>
+      <c r="M252" s="4" t="n"/>
+      <c r="N252" s="4" t="n"/>
+      <c r="O252" s="4" t="n"/>
+      <c r="P252" s="4" t="n"/>
+      <c r="Q252" s="4" t="n"/>
+      <c r="R252" s="4" t="n"/>
+      <c r="S252" s="4" t="n"/>
+      <c r="T252" s="4" t="n"/>
+      <c r="U252" s="4" t="n"/>
+      <c r="V252" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W252" s="4" t="inlineStr"/>
+      <c r="X252" s="4" t="n"/>
+      <c r="Y252" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z252" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA252" s="4" t="n"/>
+      <c r="AB252" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC252" s="4" t="n"/>
+      <c r="AD252" s="4" t="n"/>
+      <c r="AE252" s="4" t="n"/>
+      <c r="AF252" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-26
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF252"/>
+  <dimension ref="A1:AF289"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -20394,6 +20394,2918 @@
         <v>1</v>
       </c>
     </row>
+    <row r="253">
+      <c r="A253" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B253" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C253" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D253" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E253" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F253" s="4" t="n"/>
+      <c r="G253" s="4" t="n"/>
+      <c r="H253" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I253" s="4" t="inlineStr"/>
+      <c r="J253" s="4" t="inlineStr"/>
+      <c r="K253" s="4" t="inlineStr"/>
+      <c r="L253" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M253" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N253" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O253" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P253" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q253" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R253" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S253" s="4" t="n"/>
+      <c r="T253" s="4" t="n"/>
+      <c r="U253" s="4" t="n"/>
+      <c r="V253" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W253" s="4" t="inlineStr"/>
+      <c r="X253" s="4" t="n"/>
+      <c r="Y253" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z253" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA253" s="4" t="n"/>
+      <c r="AB253" s="4" t="n"/>
+      <c r="AC253" s="4" t="n"/>
+      <c r="AD253" s="4" t="n"/>
+      <c r="AE253" s="4" t="n"/>
+      <c r="AF253" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B254" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C254" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D254" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E254" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F254" s="6" t="n"/>
+      <c r="G254" s="6" t="n"/>
+      <c r="H254" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I254" s="6" t="inlineStr"/>
+      <c r="J254" s="6" t="inlineStr"/>
+      <c r="K254" s="6" t="inlineStr"/>
+      <c r="L254" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M254" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N254" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O254" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P254" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q254" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R254" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S254" s="6" t="n"/>
+      <c r="T254" s="6" t="n"/>
+      <c r="U254" s="6" t="n"/>
+      <c r="V254" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W254" s="6" t="inlineStr"/>
+      <c r="X254" s="6" t="n"/>
+      <c r="Y254" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z254" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA254" s="6" t="n"/>
+      <c r="AB254" s="6" t="n"/>
+      <c r="AC254" s="6" t="n"/>
+      <c r="AD254" s="6" t="n"/>
+      <c r="AE254" s="6" t="n"/>
+      <c r="AF254" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B255" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C255" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D255" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E255" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F255" s="4" t="n"/>
+      <c r="G255" s="4" t="n"/>
+      <c r="H255" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I255" s="4" t="inlineStr"/>
+      <c r="J255" s="4" t="inlineStr"/>
+      <c r="K255" s="4" t="inlineStr"/>
+      <c r="L255" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M255" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N255" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O255" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P255" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q255" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R255" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S255" s="4" t="n"/>
+      <c r="T255" s="4" t="n"/>
+      <c r="U255" s="4" t="n"/>
+      <c r="V255" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W255" s="4" t="inlineStr"/>
+      <c r="X255" s="4" t="n"/>
+      <c r="Y255" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z255" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA255" s="4" t="n"/>
+      <c r="AB255" s="4" t="n"/>
+      <c r="AC255" s="4" t="n"/>
+      <c r="AD255" s="4" t="n"/>
+      <c r="AE255" s="4" t="n"/>
+      <c r="AF255" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B256" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C256" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D256" s="6" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E256" s="6" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="F256" s="6" t="n"/>
+      <c r="G256" s="6" t="n"/>
+      <c r="H256" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="I256" s="6" t="inlineStr"/>
+      <c r="J256" s="6" t="inlineStr"/>
+      <c r="K256" s="6" t="inlineStr"/>
+      <c r="L256" s="6" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="M256" s="6" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="N256" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O256" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P256" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q256" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R256" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S256" s="6" t="n"/>
+      <c r="T256" s="6" t="n"/>
+      <c r="U256" s="6" t="n"/>
+      <c r="V256" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W256" s="6" t="inlineStr"/>
+      <c r="X256" s="6" t="n"/>
+      <c r="Y256" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z256" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA256" s="6" t="n"/>
+      <c r="AB256" s="6" t="n"/>
+      <c r="AC256" s="6" t="n"/>
+      <c r="AD256" s="6" t="n"/>
+      <c r="AE256" s="6" t="n"/>
+      <c r="AF256" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B257" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C257" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D257" s="4" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E257" s="4" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F257" s="4" t="n"/>
+      <c r="G257" s="4" t="n"/>
+      <c r="H257" s="4" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I257" s="4" t="inlineStr"/>
+      <c r="J257" s="4" t="inlineStr"/>
+      <c r="K257" s="4" t="inlineStr"/>
+      <c r="L257" s="4" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M257" s="4" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N257" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O257" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P257" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q257" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R257" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S257" s="4" t="n"/>
+      <c r="T257" s="4" t="n"/>
+      <c r="U257" s="4" t="n"/>
+      <c r="V257" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W257" s="4" t="inlineStr"/>
+      <c r="X257" s="4" t="n"/>
+      <c r="Y257" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z257" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA257" s="4" t="n"/>
+      <c r="AB257" s="4" t="n"/>
+      <c r="AC257" s="4" t="n"/>
+      <c r="AD257" s="4" t="n"/>
+      <c r="AE257" s="4" t="n"/>
+      <c r="AF257" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B258" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C258" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D258" s="6" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E258" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F258" s="6" t="n"/>
+      <c r="G258" s="6" t="n"/>
+      <c r="H258" s="6" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I258" s="6" t="inlineStr"/>
+      <c r="J258" s="6" t="inlineStr"/>
+      <c r="K258" s="6" t="inlineStr"/>
+      <c r="L258" s="6" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M258" s="6" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N258" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O258" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P258" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q258" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R258" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S258" s="6" t="n"/>
+      <c r="T258" s="6" t="n"/>
+      <c r="U258" s="6" t="n"/>
+      <c r="V258" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W258" s="6" t="inlineStr"/>
+      <c r="X258" s="6" t="n"/>
+      <c r="Y258" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z258" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA258" s="6" t="n"/>
+      <c r="AB258" s="6" t="n"/>
+      <c r="AC258" s="6" t="n"/>
+      <c r="AD258" s="6" t="n"/>
+      <c r="AE258" s="6" t="n"/>
+      <c r="AF258" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B259" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C259" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D259" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E259" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F259" s="4" t="n"/>
+      <c r="G259" s="4" t="n"/>
+      <c r="H259" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I259" s="4" t="inlineStr"/>
+      <c r="J259" s="4" t="inlineStr"/>
+      <c r="K259" s="4" t="inlineStr"/>
+      <c r="L259" s="4" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M259" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N259" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O259" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P259" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q259" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R259" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S259" s="4" t="n"/>
+      <c r="T259" s="4" t="n"/>
+      <c r="U259" s="4" t="n"/>
+      <c r="V259" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W259" s="4" t="inlineStr"/>
+      <c r="X259" s="4" t="n"/>
+      <c r="Y259" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z259" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA259" s="4" t="n"/>
+      <c r="AB259" s="4" t="n"/>
+      <c r="AC259" s="4" t="n"/>
+      <c r="AD259" s="4" t="n"/>
+      <c r="AE259" s="4" t="n"/>
+      <c r="AF259" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B260" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C260" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D260" s="6" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E260" s="6" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F260" s="6" t="n"/>
+      <c r="G260" s="6" t="n"/>
+      <c r="H260" s="6" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I260" s="6" t="inlineStr"/>
+      <c r="J260" s="6" t="inlineStr"/>
+      <c r="K260" s="6" t="inlineStr"/>
+      <c r="L260" s="6" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M260" s="6" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N260" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O260" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P260" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q260" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R260" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S260" s="6" t="n"/>
+      <c r="T260" s="6" t="n"/>
+      <c r="U260" s="6" t="n"/>
+      <c r="V260" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W260" s="6" t="inlineStr"/>
+      <c r="X260" s="6" t="n"/>
+      <c r="Y260" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z260" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA260" s="6" t="n"/>
+      <c r="AB260" s="6" t="n"/>
+      <c r="AC260" s="6" t="n"/>
+      <c r="AD260" s="6" t="n"/>
+      <c r="AE260" s="6" t="n"/>
+      <c r="AF260" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B261" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C261" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D261" s="4" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E261" s="4" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F261" s="4" t="n"/>
+      <c r="G261" s="4" t="n"/>
+      <c r="H261" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I261" s="4" t="inlineStr"/>
+      <c r="J261" s="4" t="inlineStr"/>
+      <c r="K261" s="4" t="inlineStr"/>
+      <c r="L261" s="4" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M261" s="4" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N261" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O261" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P261" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q261" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R261" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S261" s="4" t="n"/>
+      <c r="T261" s="4" t="n"/>
+      <c r="U261" s="4" t="n"/>
+      <c r="V261" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W261" s="4" t="inlineStr"/>
+      <c r="X261" s="4" t="n"/>
+      <c r="Y261" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z261" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA261" s="4" t="n"/>
+      <c r="AB261" s="4" t="n"/>
+      <c r="AC261" s="4" t="n"/>
+      <c r="AD261" s="4" t="n"/>
+      <c r="AE261" s="4" t="n"/>
+      <c r="AF261" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B262" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C262" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D262" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E262" s="6" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F262" s="6" t="n"/>
+      <c r="G262" s="6" t="n"/>
+      <c r="H262" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I262" s="6" t="inlineStr"/>
+      <c r="J262" s="6" t="inlineStr"/>
+      <c r="K262" s="6" t="inlineStr"/>
+      <c r="L262" s="6" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M262" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N262" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O262" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P262" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q262" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R262" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S262" s="6" t="n"/>
+      <c r="T262" s="6" t="n"/>
+      <c r="U262" s="6" t="n"/>
+      <c r="V262" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W262" s="6" t="inlineStr"/>
+      <c r="X262" s="6" t="n"/>
+      <c r="Y262" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z262" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA262" s="6" t="n"/>
+      <c r="AB262" s="6" t="n"/>
+      <c r="AC262" s="6" t="n"/>
+      <c r="AD262" s="6" t="n"/>
+      <c r="AE262" s="6" t="n"/>
+      <c r="AF262" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B263" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C263" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D263" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E263" s="4" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F263" s="4" t="n"/>
+      <c r="G263" s="4" t="n"/>
+      <c r="H263" s="4" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I263" s="4" t="inlineStr"/>
+      <c r="J263" s="4" t="inlineStr"/>
+      <c r="K263" s="4" t="inlineStr"/>
+      <c r="L263" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M263" s="4" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N263" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O263" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P263" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q263" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R263" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S263" s="4" t="n"/>
+      <c r="T263" s="4" t="n"/>
+      <c r="U263" s="4" t="n"/>
+      <c r="V263" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W263" s="4" t="inlineStr"/>
+      <c r="X263" s="4" t="n"/>
+      <c r="Y263" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z263" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA263" s="4" t="n"/>
+      <c r="AB263" s="4" t="n"/>
+      <c r="AC263" s="4" t="n"/>
+      <c r="AD263" s="4" t="n"/>
+      <c r="AE263" s="4" t="n"/>
+      <c r="AF263" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B264" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C264" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D264" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E264" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F264" s="6" t="n"/>
+      <c r="G264" s="6" t="n"/>
+      <c r="H264" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I264" s="6" t="inlineStr"/>
+      <c r="J264" s="6" t="inlineStr"/>
+      <c r="K264" s="6" t="inlineStr"/>
+      <c r="L264" s="6" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M264" s="6" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N264" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O264" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P264" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q264" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R264" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S264" s="6" t="n"/>
+      <c r="T264" s="6" t="n"/>
+      <c r="U264" s="6" t="n"/>
+      <c r="V264" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W264" s="6" t="inlineStr"/>
+      <c r="X264" s="6" t="n"/>
+      <c r="Y264" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z264" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA264" s="6" t="n"/>
+      <c r="AB264" s="6" t="n"/>
+      <c r="AC264" s="6" t="n"/>
+      <c r="AD264" s="6" t="n"/>
+      <c r="AE264" s="6" t="n"/>
+      <c r="AF264" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B265" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C265" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D265" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E265" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F265" s="4" t="n"/>
+      <c r="G265" s="4" t="n"/>
+      <c r="H265" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I265" s="4" t="inlineStr"/>
+      <c r="J265" s="4" t="inlineStr"/>
+      <c r="K265" s="4" t="inlineStr"/>
+      <c r="L265" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M265" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N265" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O265" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P265" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q265" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R265" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S265" s="4" t="n"/>
+      <c r="T265" s="4" t="n"/>
+      <c r="U265" s="4" t="n"/>
+      <c r="V265" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W265" s="4" t="inlineStr"/>
+      <c r="X265" s="4" t="n"/>
+      <c r="Y265" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z265" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA265" s="4" t="n"/>
+      <c r="AB265" s="4" t="n"/>
+      <c r="AC265" s="4" t="n"/>
+      <c r="AD265" s="4" t="n"/>
+      <c r="AE265" s="4" t="n"/>
+      <c r="AF265" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B266" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C266" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D266" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E266" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F266" s="6" t="n"/>
+      <c r="G266" s="6" t="n"/>
+      <c r="H266" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I266" s="6" t="inlineStr"/>
+      <c r="J266" s="6" t="inlineStr"/>
+      <c r="K266" s="6" t="inlineStr"/>
+      <c r="L266" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M266" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N266" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O266" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P266" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q266" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R266" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S266" s="6" t="n"/>
+      <c r="T266" s="6" t="n"/>
+      <c r="U266" s="6" t="n"/>
+      <c r="V266" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W266" s="6" t="inlineStr"/>
+      <c r="X266" s="6" t="n"/>
+      <c r="Y266" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z266" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA266" s="6" t="n"/>
+      <c r="AB266" s="6" t="n"/>
+      <c r="AC266" s="6" t="n"/>
+      <c r="AD266" s="6" t="n"/>
+      <c r="AE266" s="6" t="n"/>
+      <c r="AF266" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B267" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C267" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D267" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E267" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F267" s="4" t="n"/>
+      <c r="G267" s="4" t="n"/>
+      <c r="H267" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I267" s="4" t="inlineStr"/>
+      <c r="J267" s="4" t="inlineStr"/>
+      <c r="K267" s="4" t="inlineStr"/>
+      <c r="L267" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M267" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N267" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O267" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P267" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q267" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R267" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S267" s="4" t="n"/>
+      <c r="T267" s="4" t="n"/>
+      <c r="U267" s="4" t="n"/>
+      <c r="V267" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W267" s="4" t="inlineStr"/>
+      <c r="X267" s="4" t="n"/>
+      <c r="Y267" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z267" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA267" s="4" t="n"/>
+      <c r="AB267" s="4" t="n"/>
+      <c r="AC267" s="4" t="n"/>
+      <c r="AD267" s="4" t="n"/>
+      <c r="AE267" s="4" t="n"/>
+      <c r="AF267" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B268" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C268" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D268" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E268" s="6" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F268" s="6" t="n"/>
+      <c r="G268" s="6" t="n"/>
+      <c r="H268" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I268" s="6" t="inlineStr"/>
+      <c r="J268" s="6" t="inlineStr"/>
+      <c r="K268" s="6" t="inlineStr"/>
+      <c r="L268" s="6" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M268" s="6" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N268" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O268" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P268" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q268" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R268" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S268" s="6" t="n"/>
+      <c r="T268" s="6" t="n"/>
+      <c r="U268" s="6" t="n"/>
+      <c r="V268" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W268" s="6" t="inlineStr"/>
+      <c r="X268" s="6" t="n"/>
+      <c r="Y268" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z268" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA268" s="6" t="n"/>
+      <c r="AB268" s="6" t="n"/>
+      <c r="AC268" s="6" t="n"/>
+      <c r="AD268" s="6" t="n"/>
+      <c r="AE268" s="6" t="n"/>
+      <c r="AF268" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B269" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C269" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D269" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E269" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F269" s="4" t="n"/>
+      <c r="G269" s="4" t="n"/>
+      <c r="H269" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I269" s="4" t="inlineStr"/>
+      <c r="J269" s="4" t="inlineStr"/>
+      <c r="K269" s="4" t="inlineStr"/>
+      <c r="L269" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M269" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N269" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O269" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P269" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q269" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R269" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S269" s="4" t="n"/>
+      <c r="T269" s="4" t="n"/>
+      <c r="U269" s="4" t="n"/>
+      <c r="V269" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W269" s="4" t="inlineStr"/>
+      <c r="X269" s="4" t="n"/>
+      <c r="Y269" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z269" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA269" s="4" t="n"/>
+      <c r="AB269" s="4" t="n"/>
+      <c r="AC269" s="4" t="n"/>
+      <c r="AD269" s="4" t="n"/>
+      <c r="AE269" s="4" t="n"/>
+      <c r="AF269" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B270" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C270" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D270" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E270" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F270" s="6" t="n"/>
+      <c r="G270" s="6" t="n"/>
+      <c r="H270" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I270" s="6" t="inlineStr"/>
+      <c r="J270" s="6" t="inlineStr"/>
+      <c r="K270" s="6" t="inlineStr"/>
+      <c r="L270" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M270" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N270" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O270" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P270" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q270" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R270" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S270" s="6" t="n"/>
+      <c r="T270" s="6" t="n"/>
+      <c r="U270" s="6" t="n"/>
+      <c r="V270" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W270" s="6" t="inlineStr"/>
+      <c r="X270" s="6" t="n"/>
+      <c r="Y270" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z270" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA270" s="6" t="n"/>
+      <c r="AB270" s="6" t="n"/>
+      <c r="AC270" s="6" t="n"/>
+      <c r="AD270" s="6" t="n"/>
+      <c r="AE270" s="6" t="n"/>
+      <c r="AF270" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B271" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C271" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D271" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E271" s="4" t="n">
+        <v>20.89</v>
+      </c>
+      <c r="F271" s="4" t="n"/>
+      <c r="G271" s="4" t="n"/>
+      <c r="H271" s="4" t="n">
+        <v>53.56</v>
+      </c>
+      <c r="I271" s="4" t="inlineStr"/>
+      <c r="J271" s="4" t="inlineStr"/>
+      <c r="K271" s="4" t="inlineStr"/>
+      <c r="L271" s="4" t="n">
+        <v>67.8</v>
+      </c>
+      <c r="M271" s="4" t="n">
+        <v>2.034</v>
+      </c>
+      <c r="N271" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O271" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P271" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q271" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R271" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S271" s="4" t="n"/>
+      <c r="T271" s="4" t="n"/>
+      <c r="U271" s="4" t="n"/>
+      <c r="V271" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W271" s="4" t="inlineStr"/>
+      <c r="X271" s="4" t="n"/>
+      <c r="Y271" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z271" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA271" s="4" t="n"/>
+      <c r="AB271" s="4" t="n"/>
+      <c r="AC271" s="4" t="n"/>
+      <c r="AD271" s="4" t="n"/>
+      <c r="AE271" s="4" t="n"/>
+      <c r="AF271" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B272" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C272" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D272" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E272" s="6" t="n">
+        <v>25.84</v>
+      </c>
+      <c r="F272" s="6" t="n"/>
+      <c r="G272" s="6" t="n"/>
+      <c r="H272" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="I272" s="6" t="inlineStr"/>
+      <c r="J272" s="6" t="inlineStr"/>
+      <c r="K272" s="6" t="inlineStr"/>
+      <c r="L272" s="6" t="n">
+        <v>65.42</v>
+      </c>
+      <c r="M272" s="6" t="n">
+        <v>1.963</v>
+      </c>
+      <c r="N272" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O272" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P272" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q272" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R272" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S272" s="6" t="n"/>
+      <c r="T272" s="6" t="n"/>
+      <c r="U272" s="6" t="n"/>
+      <c r="V272" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W272" s="6" t="inlineStr"/>
+      <c r="X272" s="6" t="n"/>
+      <c r="Y272" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z272" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA272" s="6" t="n"/>
+      <c r="AB272" s="6" t="n"/>
+      <c r="AC272" s="6" t="n"/>
+      <c r="AD272" s="6" t="n"/>
+      <c r="AE272" s="6" t="n"/>
+      <c r="AF272" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B273" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C273" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D273" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E273" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F273" s="4" t="n"/>
+      <c r="G273" s="4" t="n"/>
+      <c r="H273" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I273" s="4" t="inlineStr"/>
+      <c r="J273" s="4" t="inlineStr"/>
+      <c r="K273" s="4" t="inlineStr"/>
+      <c r="L273" s="4" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="M273" s="4" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="N273" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O273" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P273" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q273" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R273" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S273" s="4" t="n"/>
+      <c r="T273" s="4" t="n"/>
+      <c r="U273" s="4" t="n"/>
+      <c r="V273" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W273" s="4" t="inlineStr"/>
+      <c r="X273" s="4" t="n"/>
+      <c r="Y273" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z273" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA273" s="4" t="n"/>
+      <c r="AB273" s="4" t="n"/>
+      <c r="AC273" s="4" t="n"/>
+      <c r="AD273" s="4" t="n"/>
+      <c r="AE273" s="4" t="n"/>
+      <c r="AF273" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B274" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C274" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D274" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E274" s="6" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="F274" s="6" t="n"/>
+      <c r="G274" s="6" t="n"/>
+      <c r="H274" s="6" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="I274" s="6" t="inlineStr"/>
+      <c r="J274" s="6" t="inlineStr"/>
+      <c r="K274" s="6" t="inlineStr"/>
+      <c r="L274" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M274" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N274" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O274" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P274" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q274" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R274" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S274" s="6" t="n"/>
+      <c r="T274" s="6" t="n"/>
+      <c r="U274" s="6" t="n"/>
+      <c r="V274" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W274" s="6" t="inlineStr"/>
+      <c r="X274" s="6" t="n"/>
+      <c r="Y274" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z274" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA274" s="6" t="n"/>
+      <c r="AB274" s="6" t="n"/>
+      <c r="AC274" s="6" t="n"/>
+      <c r="AD274" s="6" t="n"/>
+      <c r="AE274" s="6" t="n"/>
+      <c r="AF274" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B275" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C275" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D275" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E275" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F275" s="4" t="n"/>
+      <c r="G275" s="4" t="n"/>
+      <c r="H275" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I275" s="4" t="inlineStr"/>
+      <c r="J275" s="4" t="inlineStr"/>
+      <c r="K275" s="4" t="inlineStr"/>
+      <c r="L275" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M275" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N275" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O275" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P275" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q275" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R275" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S275" s="4" t="n"/>
+      <c r="T275" s="4" t="n"/>
+      <c r="U275" s="4" t="n"/>
+      <c r="V275" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W275" s="4" t="inlineStr"/>
+      <c r="X275" s="4" t="n"/>
+      <c r="Y275" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z275" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA275" s="4" t="n"/>
+      <c r="AB275" s="4" t="n"/>
+      <c r="AC275" s="4" t="n"/>
+      <c r="AD275" s="4" t="n"/>
+      <c r="AE275" s="4" t="n"/>
+      <c r="AF275" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B276" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C276" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D276" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E276" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F276" s="6" t="n"/>
+      <c r="G276" s="6" t="n"/>
+      <c r="H276" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I276" s="6" t="inlineStr"/>
+      <c r="J276" s="6" t="inlineStr"/>
+      <c r="K276" s="6" t="inlineStr"/>
+      <c r="L276" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M276" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N276" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O276" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P276" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q276" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R276" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S276" s="6" t="n"/>
+      <c r="T276" s="6" t="n"/>
+      <c r="U276" s="6" t="n"/>
+      <c r="V276" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W276" s="6" t="inlineStr"/>
+      <c r="X276" s="6" t="n"/>
+      <c r="Y276" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z276" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA276" s="6" t="n"/>
+      <c r="AB276" s="6" t="n"/>
+      <c r="AC276" s="6" t="n"/>
+      <c r="AD276" s="6" t="n"/>
+      <c r="AE276" s="6" t="n"/>
+      <c r="AF276" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B277" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C277" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D277" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E277" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F277" s="4" t="n"/>
+      <c r="G277" s="4" t="n"/>
+      <c r="H277" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I277" s="4" t="inlineStr"/>
+      <c r="J277" s="4" t="inlineStr"/>
+      <c r="K277" s="4" t="inlineStr"/>
+      <c r="L277" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M277" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N277" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O277" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P277" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q277" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R277" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S277" s="4" t="n"/>
+      <c r="T277" s="4" t="n"/>
+      <c r="U277" s="4" t="n"/>
+      <c r="V277" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W277" s="4" t="inlineStr"/>
+      <c r="X277" s="4" t="n"/>
+      <c r="Y277" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z277" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA277" s="4" t="n"/>
+      <c r="AB277" s="4" t="n"/>
+      <c r="AC277" s="4" t="n"/>
+      <c r="AD277" s="4" t="n"/>
+      <c r="AE277" s="4" t="n"/>
+      <c r="AF277" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B278" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C278" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D278" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E278" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F278" s="6" t="n"/>
+      <c r="G278" s="6" t="n"/>
+      <c r="H278" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I278" s="6" t="inlineStr"/>
+      <c r="J278" s="6" t="inlineStr"/>
+      <c r="K278" s="6" t="inlineStr"/>
+      <c r="L278" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M278" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N278" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O278" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P278" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q278" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R278" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S278" s="6" t="n"/>
+      <c r="T278" s="6" t="n"/>
+      <c r="U278" s="6" t="n"/>
+      <c r="V278" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W278" s="6" t="inlineStr"/>
+      <c r="X278" s="6" t="n"/>
+      <c r="Y278" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z278" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA278" s="6" t="n"/>
+      <c r="AB278" s="6" t="n"/>
+      <c r="AC278" s="6" t="n"/>
+      <c r="AD278" s="6" t="n"/>
+      <c r="AE278" s="6" t="n"/>
+      <c r="AF278" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B279" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C279" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D279" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E279" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F279" s="4" t="n"/>
+      <c r="G279" s="4" t="n"/>
+      <c r="H279" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I279" s="4" t="inlineStr"/>
+      <c r="J279" s="4" t="inlineStr"/>
+      <c r="K279" s="4" t="inlineStr"/>
+      <c r="L279" s="4" t="n"/>
+      <c r="M279" s="4" t="n"/>
+      <c r="N279" s="4" t="n"/>
+      <c r="O279" s="4" t="n"/>
+      <c r="P279" s="4" t="n"/>
+      <c r="Q279" s="4" t="n"/>
+      <c r="R279" s="4" t="n"/>
+      <c r="S279" s="4" t="n"/>
+      <c r="T279" s="4" t="n"/>
+      <c r="U279" s="4" t="n"/>
+      <c r="V279" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W279" s="4" t="inlineStr"/>
+      <c r="X279" s="4" t="n"/>
+      <c r="Y279" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z279" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA279" s="4" t="n"/>
+      <c r="AB279" s="4" t="n"/>
+      <c r="AC279" s="4" t="n"/>
+      <c r="AD279" s="4" t="n"/>
+      <c r="AE279" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF279" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B280" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C280" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D280" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E280" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F280" s="6" t="n"/>
+      <c r="G280" s="6" t="n"/>
+      <c r="H280" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I280" s="6" t="inlineStr"/>
+      <c r="J280" s="6" t="inlineStr"/>
+      <c r="K280" s="6" t="inlineStr"/>
+      <c r="L280" s="6" t="n"/>
+      <c r="M280" s="6" t="n"/>
+      <c r="N280" s="6" t="n"/>
+      <c r="O280" s="6" t="n"/>
+      <c r="P280" s="6" t="n"/>
+      <c r="Q280" s="6" t="n"/>
+      <c r="R280" s="6" t="n"/>
+      <c r="S280" s="6" t="n"/>
+      <c r="T280" s="6" t="n"/>
+      <c r="U280" s="6" t="n"/>
+      <c r="V280" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W280" s="6" t="inlineStr"/>
+      <c r="X280" s="6" t="n"/>
+      <c r="Y280" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z280" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA280" s="6" t="n"/>
+      <c r="AB280" s="6" t="n"/>
+      <c r="AC280" s="6" t="n"/>
+      <c r="AD280" s="6" t="n"/>
+      <c r="AE280" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF280" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B281" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C281" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D281" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E281" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F281" s="4" t="n"/>
+      <c r="G281" s="4" t="n"/>
+      <c r="H281" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I281" s="4" t="inlineStr"/>
+      <c r="J281" s="4" t="inlineStr"/>
+      <c r="K281" s="4" t="inlineStr"/>
+      <c r="L281" s="4" t="n"/>
+      <c r="M281" s="4" t="n"/>
+      <c r="N281" s="4" t="n"/>
+      <c r="O281" s="4" t="n"/>
+      <c r="P281" s="4" t="n"/>
+      <c r="Q281" s="4" t="n"/>
+      <c r="R281" s="4" t="n"/>
+      <c r="S281" s="4" t="n"/>
+      <c r="T281" s="4" t="n"/>
+      <c r="U281" s="4" t="n"/>
+      <c r="V281" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W281" s="4" t="inlineStr"/>
+      <c r="X281" s="4" t="n"/>
+      <c r="Y281" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z281" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA281" s="4" t="n"/>
+      <c r="AB281" s="4" t="n"/>
+      <c r="AC281" s="4" t="n"/>
+      <c r="AD281" s="4" t="n"/>
+      <c r="AE281" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF281" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B282" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C282" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D282" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E282" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F282" s="6" t="n"/>
+      <c r="G282" s="6" t="n"/>
+      <c r="H282" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I282" s="6" t="inlineStr"/>
+      <c r="J282" s="6" t="inlineStr"/>
+      <c r="K282" s="6" t="inlineStr"/>
+      <c r="L282" s="6" t="n"/>
+      <c r="M282" s="6" t="n"/>
+      <c r="N282" s="6" t="n"/>
+      <c r="O282" s="6" t="n"/>
+      <c r="P282" s="6" t="n"/>
+      <c r="Q282" s="6" t="n"/>
+      <c r="R282" s="6" t="n"/>
+      <c r="S282" s="6" t="n"/>
+      <c r="T282" s="6" t="n"/>
+      <c r="U282" s="6" t="n"/>
+      <c r="V282" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W282" s="6" t="inlineStr"/>
+      <c r="X282" s="6" t="n"/>
+      <c r="Y282" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z282" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA282" s="6" t="n"/>
+      <c r="AB282" s="6" t="n"/>
+      <c r="AC282" s="6" t="n"/>
+      <c r="AD282" s="6" t="n"/>
+      <c r="AE282" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF282" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B283" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C283" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D283" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E283" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F283" s="4" t="n"/>
+      <c r="G283" s="4" t="n"/>
+      <c r="H283" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I283" s="4" t="inlineStr"/>
+      <c r="J283" s="4" t="inlineStr"/>
+      <c r="K283" s="4" t="inlineStr"/>
+      <c r="L283" s="4" t="n"/>
+      <c r="M283" s="4" t="n"/>
+      <c r="N283" s="4" t="n"/>
+      <c r="O283" s="4" t="n"/>
+      <c r="P283" s="4" t="n"/>
+      <c r="Q283" s="4" t="n"/>
+      <c r="R283" s="4" t="n"/>
+      <c r="S283" s="4" t="n"/>
+      <c r="T283" s="4" t="n"/>
+      <c r="U283" s="4" t="n"/>
+      <c r="V283" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W283" s="4" t="inlineStr"/>
+      <c r="X283" s="4" t="n"/>
+      <c r="Y283" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z283" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA283" s="4" t="n"/>
+      <c r="AB283" s="4" t="n"/>
+      <c r="AC283" s="4" t="n"/>
+      <c r="AD283" s="4" t="n"/>
+      <c r="AE283" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF283" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B284" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C284" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D284" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E284" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F284" s="6" t="n"/>
+      <c r="G284" s="6" t="n"/>
+      <c r="H284" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I284" s="6" t="inlineStr"/>
+      <c r="J284" s="6" t="inlineStr"/>
+      <c r="K284" s="6" t="inlineStr"/>
+      <c r="L284" s="6" t="n"/>
+      <c r="M284" s="6" t="n"/>
+      <c r="N284" s="6" t="n"/>
+      <c r="O284" s="6" t="n"/>
+      <c r="P284" s="6" t="n"/>
+      <c r="Q284" s="6" t="n"/>
+      <c r="R284" s="6" t="n"/>
+      <c r="S284" s="6" t="n"/>
+      <c r="T284" s="6" t="n"/>
+      <c r="U284" s="6" t="n"/>
+      <c r="V284" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W284" s="6" t="inlineStr"/>
+      <c r="X284" s="6" t="n"/>
+      <c r="Y284" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z284" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA284" s="6" t="n"/>
+      <c r="AB284" s="6" t="n"/>
+      <c r="AC284" s="6" t="n"/>
+      <c r="AD284" s="6" t="n"/>
+      <c r="AE284" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF284" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B285" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C285" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D285" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E285" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F285" s="4" t="n"/>
+      <c r="G285" s="4" t="n"/>
+      <c r="H285" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I285" s="4" t="inlineStr"/>
+      <c r="J285" s="4" t="inlineStr"/>
+      <c r="K285" s="4" t="inlineStr"/>
+      <c r="L285" s="4" t="n"/>
+      <c r="M285" s="4" t="n"/>
+      <c r="N285" s="4" t="n"/>
+      <c r="O285" s="4" t="n"/>
+      <c r="P285" s="4" t="n"/>
+      <c r="Q285" s="4" t="n"/>
+      <c r="R285" s="4" t="n"/>
+      <c r="S285" s="4" t="n"/>
+      <c r="T285" s="4" t="n"/>
+      <c r="U285" s="4" t="n"/>
+      <c r="V285" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W285" s="4" t="inlineStr"/>
+      <c r="X285" s="4" t="n"/>
+      <c r="Y285" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z285" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA285" s="4" t="n"/>
+      <c r="AB285" s="4" t="n"/>
+      <c r="AC285" s="4" t="n"/>
+      <c r="AD285" s="4" t="n"/>
+      <c r="AE285" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF285" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B286" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C286" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D286" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E286" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F286" s="6" t="n"/>
+      <c r="G286" s="6" t="n"/>
+      <c r="H286" s="6" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="I286" s="6" t="inlineStr"/>
+      <c r="J286" s="6" t="inlineStr"/>
+      <c r="K286" s="6" t="inlineStr"/>
+      <c r="L286" s="6" t="n"/>
+      <c r="M286" s="6" t="n"/>
+      <c r="N286" s="6" t="n"/>
+      <c r="O286" s="6" t="n"/>
+      <c r="P286" s="6" t="n"/>
+      <c r="Q286" s="6" t="n"/>
+      <c r="R286" s="6" t="n"/>
+      <c r="S286" s="6" t="n"/>
+      <c r="T286" s="6" t="n"/>
+      <c r="U286" s="6" t="n"/>
+      <c r="V286" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W286" s="6" t="inlineStr"/>
+      <c r="X286" s="6" t="n"/>
+      <c r="Y286" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z286" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA286" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB286" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC286" s="6" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="AD286" s="6" t="n"/>
+      <c r="AE286" s="6" t="n"/>
+      <c r="AF286" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B287" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C287" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D287" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E287" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F287" s="4" t="n"/>
+      <c r="G287" s="4" t="n"/>
+      <c r="H287" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="I287" s="4" t="inlineStr"/>
+      <c r="J287" s="4" t="inlineStr"/>
+      <c r="K287" s="4" t="inlineStr"/>
+      <c r="L287" s="4" t="n"/>
+      <c r="M287" s="4" t="n"/>
+      <c r="N287" s="4" t="n"/>
+      <c r="O287" s="4" t="n"/>
+      <c r="P287" s="4" t="n"/>
+      <c r="Q287" s="4" t="n"/>
+      <c r="R287" s="4" t="n"/>
+      <c r="S287" s="4" t="n"/>
+      <c r="T287" s="4" t="n"/>
+      <c r="U287" s="4" t="n"/>
+      <c r="V287" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W287" s="4" t="inlineStr"/>
+      <c r="X287" s="4" t="n"/>
+      <c r="Y287" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z287" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA287" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB287" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC287" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AD287" s="4" t="n"/>
+      <c r="AE287" s="4" t="n"/>
+      <c r="AF287" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B288" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C288" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D288" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E288" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F288" s="6" t="n"/>
+      <c r="G288" s="6" t="n"/>
+      <c r="H288" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I288" s="6" t="inlineStr"/>
+      <c r="J288" s="6" t="inlineStr"/>
+      <c r="K288" s="6" t="inlineStr"/>
+      <c r="L288" s="6" t="n"/>
+      <c r="M288" s="6" t="n"/>
+      <c r="N288" s="6" t="n"/>
+      <c r="O288" s="6" t="n"/>
+      <c r="P288" s="6" t="n"/>
+      <c r="Q288" s="6" t="n"/>
+      <c r="R288" s="6" t="n"/>
+      <c r="S288" s="6" t="n"/>
+      <c r="T288" s="6" t="n"/>
+      <c r="U288" s="6" t="n"/>
+      <c r="V288" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W288" s="6" t="inlineStr"/>
+      <c r="X288" s="6" t="n"/>
+      <c r="Y288" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z288" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA288" s="6" t="n"/>
+      <c r="AB288" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC288" s="6" t="n"/>
+      <c r="AD288" s="6" t="n"/>
+      <c r="AE288" s="6" t="n"/>
+      <c r="AF288" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="B289" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C289" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D289" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E289" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F289" s="4" t="n"/>
+      <c r="G289" s="4" t="n"/>
+      <c r="H289" s="4" t="n">
+        <v>194.44</v>
+      </c>
+      <c r="I289" s="4" t="inlineStr"/>
+      <c r="J289" s="4" t="inlineStr"/>
+      <c r="K289" s="4" t="inlineStr"/>
+      <c r="L289" s="4" t="n"/>
+      <c r="M289" s="4" t="n"/>
+      <c r="N289" s="4" t="n"/>
+      <c r="O289" s="4" t="n"/>
+      <c r="P289" s="4" t="n"/>
+      <c r="Q289" s="4" t="n"/>
+      <c r="R289" s="4" t="n"/>
+      <c r="S289" s="4" t="n"/>
+      <c r="T289" s="4" t="n"/>
+      <c r="U289" s="4" t="n"/>
+      <c r="V289" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W289" s="4" t="inlineStr"/>
+      <c r="X289" s="4" t="n"/>
+      <c r="Y289" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z289" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA289" s="4" t="n"/>
+      <c r="AB289" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC289" s="4" t="n"/>
+      <c r="AD289" s="4" t="n"/>
+      <c r="AE289" s="4" t="n"/>
+      <c r="AF289" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-27
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF289"/>
+  <dimension ref="A1:AF326"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -23306,6 +23306,2918 @@
         <v>1</v>
       </c>
     </row>
+    <row r="290">
+      <c r="A290" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B290" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C290" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D290" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E290" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F290" s="4" t="n"/>
+      <c r="G290" s="4" t="n"/>
+      <c r="H290" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I290" s="4" t="inlineStr"/>
+      <c r="J290" s="4" t="inlineStr"/>
+      <c r="K290" s="4" t="inlineStr"/>
+      <c r="L290" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M290" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N290" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O290" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P290" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q290" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R290" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S290" s="4" t="n"/>
+      <c r="T290" s="4" t="n"/>
+      <c r="U290" s="4" t="n"/>
+      <c r="V290" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W290" s="4" t="inlineStr"/>
+      <c r="X290" s="4" t="n"/>
+      <c r="Y290" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z290" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA290" s="4" t="n"/>
+      <c r="AB290" s="4" t="n"/>
+      <c r="AC290" s="4" t="n"/>
+      <c r="AD290" s="4" t="n"/>
+      <c r="AE290" s="4" t="n"/>
+      <c r="AF290" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B291" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C291" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D291" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E291" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F291" s="6" t="n"/>
+      <c r="G291" s="6" t="n"/>
+      <c r="H291" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I291" s="6" t="inlineStr"/>
+      <c r="J291" s="6" t="inlineStr"/>
+      <c r="K291" s="6" t="inlineStr"/>
+      <c r="L291" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M291" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N291" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O291" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P291" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q291" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R291" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S291" s="6" t="n"/>
+      <c r="T291" s="6" t="n"/>
+      <c r="U291" s="6" t="n"/>
+      <c r="V291" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W291" s="6" t="inlineStr"/>
+      <c r="X291" s="6" t="n"/>
+      <c r="Y291" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z291" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA291" s="6" t="n"/>
+      <c r="AB291" s="6" t="n"/>
+      <c r="AC291" s="6" t="n"/>
+      <c r="AD291" s="6" t="n"/>
+      <c r="AE291" s="6" t="n"/>
+      <c r="AF291" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B292" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C292" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D292" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E292" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F292" s="4" t="n"/>
+      <c r="G292" s="4" t="n"/>
+      <c r="H292" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I292" s="4" t="inlineStr"/>
+      <c r="J292" s="4" t="inlineStr"/>
+      <c r="K292" s="4" t="inlineStr"/>
+      <c r="L292" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M292" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N292" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O292" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P292" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q292" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R292" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S292" s="4" t="n"/>
+      <c r="T292" s="4" t="n"/>
+      <c r="U292" s="4" t="n"/>
+      <c r="V292" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W292" s="4" t="inlineStr"/>
+      <c r="X292" s="4" t="n"/>
+      <c r="Y292" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z292" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA292" s="4" t="n"/>
+      <c r="AB292" s="4" t="n"/>
+      <c r="AC292" s="4" t="n"/>
+      <c r="AD292" s="4" t="n"/>
+      <c r="AE292" s="4" t="n"/>
+      <c r="AF292" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B293" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C293" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D293" s="6" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E293" s="6" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="F293" s="6" t="n"/>
+      <c r="G293" s="6" t="n"/>
+      <c r="H293" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="I293" s="6" t="inlineStr"/>
+      <c r="J293" s="6" t="inlineStr"/>
+      <c r="K293" s="6" t="inlineStr"/>
+      <c r="L293" s="6" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="M293" s="6" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="N293" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O293" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P293" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q293" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R293" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S293" s="6" t="n"/>
+      <c r="T293" s="6" t="n"/>
+      <c r="U293" s="6" t="n"/>
+      <c r="V293" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W293" s="6" t="inlineStr"/>
+      <c r="X293" s="6" t="n"/>
+      <c r="Y293" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z293" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA293" s="6" t="n"/>
+      <c r="AB293" s="6" t="n"/>
+      <c r="AC293" s="6" t="n"/>
+      <c r="AD293" s="6" t="n"/>
+      <c r="AE293" s="6" t="n"/>
+      <c r="AF293" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B294" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C294" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D294" s="4" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E294" s="4" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F294" s="4" t="n"/>
+      <c r="G294" s="4" t="n"/>
+      <c r="H294" s="4" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I294" s="4" t="inlineStr"/>
+      <c r="J294" s="4" t="inlineStr"/>
+      <c r="K294" s="4" t="inlineStr"/>
+      <c r="L294" s="4" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M294" s="4" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N294" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O294" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P294" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q294" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R294" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S294" s="4" t="n"/>
+      <c r="T294" s="4" t="n"/>
+      <c r="U294" s="4" t="n"/>
+      <c r="V294" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W294" s="4" t="inlineStr"/>
+      <c r="X294" s="4" t="n"/>
+      <c r="Y294" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z294" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA294" s="4" t="n"/>
+      <c r="AB294" s="4" t="n"/>
+      <c r="AC294" s="4" t="n"/>
+      <c r="AD294" s="4" t="n"/>
+      <c r="AE294" s="4" t="n"/>
+      <c r="AF294" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B295" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C295" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D295" s="6" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E295" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F295" s="6" t="n"/>
+      <c r="G295" s="6" t="n"/>
+      <c r="H295" s="6" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I295" s="6" t="inlineStr"/>
+      <c r="J295" s="6" t="inlineStr"/>
+      <c r="K295" s="6" t="inlineStr"/>
+      <c r="L295" s="6" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M295" s="6" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N295" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O295" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P295" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q295" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R295" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S295" s="6" t="n"/>
+      <c r="T295" s="6" t="n"/>
+      <c r="U295" s="6" t="n"/>
+      <c r="V295" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W295" s="6" t="inlineStr"/>
+      <c r="X295" s="6" t="n"/>
+      <c r="Y295" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z295" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA295" s="6" t="n"/>
+      <c r="AB295" s="6" t="n"/>
+      <c r="AC295" s="6" t="n"/>
+      <c r="AD295" s="6" t="n"/>
+      <c r="AE295" s="6" t="n"/>
+      <c r="AF295" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B296" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C296" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D296" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E296" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F296" s="4" t="n"/>
+      <c r="G296" s="4" t="n"/>
+      <c r="H296" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I296" s="4" t="inlineStr"/>
+      <c r="J296" s="4" t="inlineStr"/>
+      <c r="K296" s="4" t="inlineStr"/>
+      <c r="L296" s="4" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M296" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N296" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O296" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P296" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q296" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R296" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S296" s="4" t="n"/>
+      <c r="T296" s="4" t="n"/>
+      <c r="U296" s="4" t="n"/>
+      <c r="V296" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W296" s="4" t="inlineStr"/>
+      <c r="X296" s="4" t="n"/>
+      <c r="Y296" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z296" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA296" s="4" t="n"/>
+      <c r="AB296" s="4" t="n"/>
+      <c r="AC296" s="4" t="n"/>
+      <c r="AD296" s="4" t="n"/>
+      <c r="AE296" s="4" t="n"/>
+      <c r="AF296" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B297" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C297" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D297" s="6" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E297" s="6" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F297" s="6" t="n"/>
+      <c r="G297" s="6" t="n"/>
+      <c r="H297" s="6" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I297" s="6" t="inlineStr"/>
+      <c r="J297" s="6" t="inlineStr"/>
+      <c r="K297" s="6" t="inlineStr"/>
+      <c r="L297" s="6" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M297" s="6" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N297" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O297" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P297" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q297" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R297" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S297" s="6" t="n"/>
+      <c r="T297" s="6" t="n"/>
+      <c r="U297" s="6" t="n"/>
+      <c r="V297" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W297" s="6" t="inlineStr"/>
+      <c r="X297" s="6" t="n"/>
+      <c r="Y297" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z297" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA297" s="6" t="n"/>
+      <c r="AB297" s="6" t="n"/>
+      <c r="AC297" s="6" t="n"/>
+      <c r="AD297" s="6" t="n"/>
+      <c r="AE297" s="6" t="n"/>
+      <c r="AF297" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B298" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C298" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D298" s="4" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E298" s="4" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F298" s="4" t="n"/>
+      <c r="G298" s="4" t="n"/>
+      <c r="H298" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I298" s="4" t="inlineStr"/>
+      <c r="J298" s="4" t="inlineStr"/>
+      <c r="K298" s="4" t="inlineStr"/>
+      <c r="L298" s="4" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M298" s="4" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N298" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O298" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P298" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q298" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R298" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S298" s="4" t="n"/>
+      <c r="T298" s="4" t="n"/>
+      <c r="U298" s="4" t="n"/>
+      <c r="V298" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W298" s="4" t="inlineStr"/>
+      <c r="X298" s="4" t="n"/>
+      <c r="Y298" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z298" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA298" s="4" t="n"/>
+      <c r="AB298" s="4" t="n"/>
+      <c r="AC298" s="4" t="n"/>
+      <c r="AD298" s="4" t="n"/>
+      <c r="AE298" s="4" t="n"/>
+      <c r="AF298" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B299" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C299" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D299" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E299" s="6" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F299" s="6" t="n"/>
+      <c r="G299" s="6" t="n"/>
+      <c r="H299" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I299" s="6" t="inlineStr"/>
+      <c r="J299" s="6" t="inlineStr"/>
+      <c r="K299" s="6" t="inlineStr"/>
+      <c r="L299" s="6" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M299" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N299" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O299" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P299" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q299" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R299" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S299" s="6" t="n"/>
+      <c r="T299" s="6" t="n"/>
+      <c r="U299" s="6" t="n"/>
+      <c r="V299" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W299" s="6" t="inlineStr"/>
+      <c r="X299" s="6" t="n"/>
+      <c r="Y299" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z299" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA299" s="6" t="n"/>
+      <c r="AB299" s="6" t="n"/>
+      <c r="AC299" s="6" t="n"/>
+      <c r="AD299" s="6" t="n"/>
+      <c r="AE299" s="6" t="n"/>
+      <c r="AF299" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B300" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C300" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D300" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E300" s="4" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F300" s="4" t="n"/>
+      <c r="G300" s="4" t="n"/>
+      <c r="H300" s="4" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I300" s="4" t="inlineStr"/>
+      <c r="J300" s="4" t="inlineStr"/>
+      <c r="K300" s="4" t="inlineStr"/>
+      <c r="L300" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M300" s="4" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N300" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O300" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P300" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q300" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R300" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S300" s="4" t="n"/>
+      <c r="T300" s="4" t="n"/>
+      <c r="U300" s="4" t="n"/>
+      <c r="V300" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W300" s="4" t="inlineStr"/>
+      <c r="X300" s="4" t="n"/>
+      <c r="Y300" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z300" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA300" s="4" t="n"/>
+      <c r="AB300" s="4" t="n"/>
+      <c r="AC300" s="4" t="n"/>
+      <c r="AD300" s="4" t="n"/>
+      <c r="AE300" s="4" t="n"/>
+      <c r="AF300" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B301" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C301" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D301" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E301" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F301" s="6" t="n"/>
+      <c r="G301" s="6" t="n"/>
+      <c r="H301" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I301" s="6" t="inlineStr"/>
+      <c r="J301" s="6" t="inlineStr"/>
+      <c r="K301" s="6" t="inlineStr"/>
+      <c r="L301" s="6" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M301" s="6" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N301" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O301" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P301" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q301" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R301" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S301" s="6" t="n"/>
+      <c r="T301" s="6" t="n"/>
+      <c r="U301" s="6" t="n"/>
+      <c r="V301" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W301" s="6" t="inlineStr"/>
+      <c r="X301" s="6" t="n"/>
+      <c r="Y301" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z301" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA301" s="6" t="n"/>
+      <c r="AB301" s="6" t="n"/>
+      <c r="AC301" s="6" t="n"/>
+      <c r="AD301" s="6" t="n"/>
+      <c r="AE301" s="6" t="n"/>
+      <c r="AF301" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B302" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C302" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D302" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E302" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F302" s="4" t="n"/>
+      <c r="G302" s="4" t="n"/>
+      <c r="H302" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I302" s="4" t="inlineStr"/>
+      <c r="J302" s="4" t="inlineStr"/>
+      <c r="K302" s="4" t="inlineStr"/>
+      <c r="L302" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M302" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N302" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O302" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P302" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q302" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R302" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S302" s="4" t="n"/>
+      <c r="T302" s="4" t="n"/>
+      <c r="U302" s="4" t="n"/>
+      <c r="V302" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W302" s="4" t="inlineStr"/>
+      <c r="X302" s="4" t="n"/>
+      <c r="Y302" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z302" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA302" s="4" t="n"/>
+      <c r="AB302" s="4" t="n"/>
+      <c r="AC302" s="4" t="n"/>
+      <c r="AD302" s="4" t="n"/>
+      <c r="AE302" s="4" t="n"/>
+      <c r="AF302" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B303" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C303" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D303" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E303" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F303" s="6" t="n"/>
+      <c r="G303" s="6" t="n"/>
+      <c r="H303" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I303" s="6" t="inlineStr"/>
+      <c r="J303" s="6" t="inlineStr"/>
+      <c r="K303" s="6" t="inlineStr"/>
+      <c r="L303" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M303" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N303" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O303" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P303" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q303" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R303" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S303" s="6" t="n"/>
+      <c r="T303" s="6" t="n"/>
+      <c r="U303" s="6" t="n"/>
+      <c r="V303" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W303" s="6" t="inlineStr"/>
+      <c r="X303" s="6" t="n"/>
+      <c r="Y303" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z303" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA303" s="6" t="n"/>
+      <c r="AB303" s="6" t="n"/>
+      <c r="AC303" s="6" t="n"/>
+      <c r="AD303" s="6" t="n"/>
+      <c r="AE303" s="6" t="n"/>
+      <c r="AF303" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B304" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C304" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D304" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E304" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F304" s="4" t="n"/>
+      <c r="G304" s="4" t="n"/>
+      <c r="H304" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I304" s="4" t="inlineStr"/>
+      <c r="J304" s="4" t="inlineStr"/>
+      <c r="K304" s="4" t="inlineStr"/>
+      <c r="L304" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M304" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N304" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O304" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P304" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q304" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R304" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S304" s="4" t="n"/>
+      <c r="T304" s="4" t="n"/>
+      <c r="U304" s="4" t="n"/>
+      <c r="V304" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W304" s="4" t="inlineStr"/>
+      <c r="X304" s="4" t="n"/>
+      <c r="Y304" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z304" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA304" s="4" t="n"/>
+      <c r="AB304" s="4" t="n"/>
+      <c r="AC304" s="4" t="n"/>
+      <c r="AD304" s="4" t="n"/>
+      <c r="AE304" s="4" t="n"/>
+      <c r="AF304" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B305" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C305" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D305" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E305" s="6" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F305" s="6" t="n"/>
+      <c r="G305" s="6" t="n"/>
+      <c r="H305" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I305" s="6" t="inlineStr"/>
+      <c r="J305" s="6" t="inlineStr"/>
+      <c r="K305" s="6" t="inlineStr"/>
+      <c r="L305" s="6" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M305" s="6" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N305" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O305" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P305" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q305" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R305" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S305" s="6" t="n"/>
+      <c r="T305" s="6" t="n"/>
+      <c r="U305" s="6" t="n"/>
+      <c r="V305" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W305" s="6" t="inlineStr"/>
+      <c r="X305" s="6" t="n"/>
+      <c r="Y305" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z305" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA305" s="6" t="n"/>
+      <c r="AB305" s="6" t="n"/>
+      <c r="AC305" s="6" t="n"/>
+      <c r="AD305" s="6" t="n"/>
+      <c r="AE305" s="6" t="n"/>
+      <c r="AF305" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B306" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C306" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D306" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E306" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F306" s="4" t="n"/>
+      <c r="G306" s="4" t="n"/>
+      <c r="H306" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I306" s="4" t="inlineStr"/>
+      <c r="J306" s="4" t="inlineStr"/>
+      <c r="K306" s="4" t="inlineStr"/>
+      <c r="L306" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M306" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N306" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O306" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P306" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q306" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R306" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S306" s="4" t="n"/>
+      <c r="T306" s="4" t="n"/>
+      <c r="U306" s="4" t="n"/>
+      <c r="V306" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W306" s="4" t="inlineStr"/>
+      <c r="X306" s="4" t="n"/>
+      <c r="Y306" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z306" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA306" s="4" t="n"/>
+      <c r="AB306" s="4" t="n"/>
+      <c r="AC306" s="4" t="n"/>
+      <c r="AD306" s="4" t="n"/>
+      <c r="AE306" s="4" t="n"/>
+      <c r="AF306" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B307" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C307" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D307" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E307" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F307" s="6" t="n"/>
+      <c r="G307" s="6" t="n"/>
+      <c r="H307" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I307" s="6" t="inlineStr"/>
+      <c r="J307" s="6" t="inlineStr"/>
+      <c r="K307" s="6" t="inlineStr"/>
+      <c r="L307" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M307" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N307" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O307" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P307" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q307" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R307" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S307" s="6" t="n"/>
+      <c r="T307" s="6" t="n"/>
+      <c r="U307" s="6" t="n"/>
+      <c r="V307" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W307" s="6" t="inlineStr"/>
+      <c r="X307" s="6" t="n"/>
+      <c r="Y307" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z307" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA307" s="6" t="n"/>
+      <c r="AB307" s="6" t="n"/>
+      <c r="AC307" s="6" t="n"/>
+      <c r="AD307" s="6" t="n"/>
+      <c r="AE307" s="6" t="n"/>
+      <c r="AF307" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B308" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C308" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D308" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E308" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F308" s="4" t="n"/>
+      <c r="G308" s="4" t="n"/>
+      <c r="H308" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I308" s="4" t="inlineStr"/>
+      <c r="J308" s="4" t="inlineStr"/>
+      <c r="K308" s="4" t="inlineStr"/>
+      <c r="L308" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M308" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N308" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O308" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P308" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q308" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R308" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S308" s="4" t="n"/>
+      <c r="T308" s="4" t="n"/>
+      <c r="U308" s="4" t="n"/>
+      <c r="V308" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W308" s="4" t="inlineStr"/>
+      <c r="X308" s="4" t="n"/>
+      <c r="Y308" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z308" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA308" s="4" t="n"/>
+      <c r="AB308" s="4" t="n"/>
+      <c r="AC308" s="4" t="n"/>
+      <c r="AD308" s="4" t="n"/>
+      <c r="AE308" s="4" t="n"/>
+      <c r="AF308" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B309" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C309" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D309" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E309" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F309" s="6" t="n"/>
+      <c r="G309" s="6" t="n"/>
+      <c r="H309" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I309" s="6" t="inlineStr"/>
+      <c r="J309" s="6" t="inlineStr"/>
+      <c r="K309" s="6" t="inlineStr"/>
+      <c r="L309" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M309" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N309" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O309" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P309" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q309" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R309" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S309" s="6" t="n"/>
+      <c r="T309" s="6" t="n"/>
+      <c r="U309" s="6" t="n"/>
+      <c r="V309" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W309" s="6" t="inlineStr"/>
+      <c r="X309" s="6" t="n"/>
+      <c r="Y309" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z309" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA309" s="6" t="n"/>
+      <c r="AB309" s="6" t="n"/>
+      <c r="AC309" s="6" t="n"/>
+      <c r="AD309" s="6" t="n"/>
+      <c r="AE309" s="6" t="n"/>
+      <c r="AF309" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B310" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C310" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D310" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E310" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F310" s="4" t="n"/>
+      <c r="G310" s="4" t="n"/>
+      <c r="H310" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I310" s="4" t="inlineStr"/>
+      <c r="J310" s="4" t="inlineStr"/>
+      <c r="K310" s="4" t="inlineStr"/>
+      <c r="L310" s="4" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="M310" s="4" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="N310" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O310" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P310" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q310" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R310" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S310" s="4" t="n"/>
+      <c r="T310" s="4" t="n"/>
+      <c r="U310" s="4" t="n"/>
+      <c r="V310" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W310" s="4" t="inlineStr"/>
+      <c r="X310" s="4" t="n"/>
+      <c r="Y310" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z310" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA310" s="4" t="n"/>
+      <c r="AB310" s="4" t="n"/>
+      <c r="AC310" s="4" t="n"/>
+      <c r="AD310" s="4" t="n"/>
+      <c r="AE310" s="4" t="n"/>
+      <c r="AF310" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B311" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C311" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D311" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E311" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F311" s="6" t="n"/>
+      <c r="G311" s="6" t="n"/>
+      <c r="H311" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I311" s="6" t="inlineStr"/>
+      <c r="J311" s="6" t="inlineStr"/>
+      <c r="K311" s="6" t="inlineStr"/>
+      <c r="L311" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M311" s="6" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N311" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O311" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P311" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q311" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R311" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S311" s="6" t="n"/>
+      <c r="T311" s="6" t="n"/>
+      <c r="U311" s="6" t="n"/>
+      <c r="V311" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W311" s="6" t="inlineStr"/>
+      <c r="X311" s="6" t="n"/>
+      <c r="Y311" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z311" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA311" s="6" t="n"/>
+      <c r="AB311" s="6" t="n"/>
+      <c r="AC311" s="6" t="n"/>
+      <c r="AD311" s="6" t="n"/>
+      <c r="AE311" s="6" t="n"/>
+      <c r="AF311" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B312" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C312" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D312" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E312" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F312" s="4" t="n"/>
+      <c r="G312" s="4" t="n"/>
+      <c r="H312" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I312" s="4" t="inlineStr"/>
+      <c r="J312" s="4" t="inlineStr"/>
+      <c r="K312" s="4" t="inlineStr"/>
+      <c r="L312" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M312" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N312" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O312" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P312" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q312" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R312" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S312" s="4" t="n"/>
+      <c r="T312" s="4" t="n"/>
+      <c r="U312" s="4" t="n"/>
+      <c r="V312" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W312" s="4" t="inlineStr"/>
+      <c r="X312" s="4" t="n"/>
+      <c r="Y312" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z312" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA312" s="4" t="n"/>
+      <c r="AB312" s="4" t="n"/>
+      <c r="AC312" s="4" t="n"/>
+      <c r="AD312" s="4" t="n"/>
+      <c r="AE312" s="4" t="n"/>
+      <c r="AF312" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B313" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C313" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D313" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E313" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F313" s="6" t="n"/>
+      <c r="G313" s="6" t="n"/>
+      <c r="H313" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I313" s="6" t="inlineStr"/>
+      <c r="J313" s="6" t="inlineStr"/>
+      <c r="K313" s="6" t="inlineStr"/>
+      <c r="L313" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M313" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N313" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O313" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P313" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q313" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R313" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S313" s="6" t="n"/>
+      <c r="T313" s="6" t="n"/>
+      <c r="U313" s="6" t="n"/>
+      <c r="V313" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W313" s="6" t="inlineStr"/>
+      <c r="X313" s="6" t="n"/>
+      <c r="Y313" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z313" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA313" s="6" t="n"/>
+      <c r="AB313" s="6" t="n"/>
+      <c r="AC313" s="6" t="n"/>
+      <c r="AD313" s="6" t="n"/>
+      <c r="AE313" s="6" t="n"/>
+      <c r="AF313" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B314" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C314" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D314" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E314" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F314" s="4" t="n"/>
+      <c r="G314" s="4" t="n"/>
+      <c r="H314" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I314" s="4" t="inlineStr"/>
+      <c r="J314" s="4" t="inlineStr"/>
+      <c r="K314" s="4" t="inlineStr"/>
+      <c r="L314" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M314" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N314" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O314" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P314" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q314" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R314" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S314" s="4" t="n"/>
+      <c r="T314" s="4" t="n"/>
+      <c r="U314" s="4" t="n"/>
+      <c r="V314" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W314" s="4" t="inlineStr"/>
+      <c r="X314" s="4" t="n"/>
+      <c r="Y314" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z314" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA314" s="4" t="n"/>
+      <c r="AB314" s="4" t="n"/>
+      <c r="AC314" s="4" t="n"/>
+      <c r="AD314" s="4" t="n"/>
+      <c r="AE314" s="4" t="n"/>
+      <c r="AF314" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B315" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C315" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D315" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E315" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F315" s="6" t="n"/>
+      <c r="G315" s="6" t="n"/>
+      <c r="H315" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I315" s="6" t="inlineStr"/>
+      <c r="J315" s="6" t="inlineStr"/>
+      <c r="K315" s="6" t="inlineStr"/>
+      <c r="L315" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M315" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N315" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O315" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P315" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q315" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R315" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S315" s="6" t="n"/>
+      <c r="T315" s="6" t="n"/>
+      <c r="U315" s="6" t="n"/>
+      <c r="V315" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W315" s="6" t="inlineStr"/>
+      <c r="X315" s="6" t="n"/>
+      <c r="Y315" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z315" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA315" s="6" t="n"/>
+      <c r="AB315" s="6" t="n"/>
+      <c r="AC315" s="6" t="n"/>
+      <c r="AD315" s="6" t="n"/>
+      <c r="AE315" s="6" t="n"/>
+      <c r="AF315" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B316" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C316" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D316" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E316" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F316" s="4" t="n"/>
+      <c r="G316" s="4" t="n"/>
+      <c r="H316" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I316" s="4" t="inlineStr"/>
+      <c r="J316" s="4" t="inlineStr"/>
+      <c r="K316" s="4" t="inlineStr"/>
+      <c r="L316" s="4" t="n"/>
+      <c r="M316" s="4" t="n"/>
+      <c r="N316" s="4" t="n"/>
+      <c r="O316" s="4" t="n"/>
+      <c r="P316" s="4" t="n"/>
+      <c r="Q316" s="4" t="n"/>
+      <c r="R316" s="4" t="n"/>
+      <c r="S316" s="4" t="n"/>
+      <c r="T316" s="4" t="n"/>
+      <c r="U316" s="4" t="n"/>
+      <c r="V316" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W316" s="4" t="inlineStr"/>
+      <c r="X316" s="4" t="n"/>
+      <c r="Y316" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z316" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA316" s="4" t="n"/>
+      <c r="AB316" s="4" t="n"/>
+      <c r="AC316" s="4" t="n"/>
+      <c r="AD316" s="4" t="n"/>
+      <c r="AE316" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF316" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B317" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C317" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D317" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E317" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F317" s="6" t="n"/>
+      <c r="G317" s="6" t="n"/>
+      <c r="H317" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I317" s="6" t="inlineStr"/>
+      <c r="J317" s="6" t="inlineStr"/>
+      <c r="K317" s="6" t="inlineStr"/>
+      <c r="L317" s="6" t="n"/>
+      <c r="M317" s="6" t="n"/>
+      <c r="N317" s="6" t="n"/>
+      <c r="O317" s="6" t="n"/>
+      <c r="P317" s="6" t="n"/>
+      <c r="Q317" s="6" t="n"/>
+      <c r="R317" s="6" t="n"/>
+      <c r="S317" s="6" t="n"/>
+      <c r="T317" s="6" t="n"/>
+      <c r="U317" s="6" t="n"/>
+      <c r="V317" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W317" s="6" t="inlineStr"/>
+      <c r="X317" s="6" t="n"/>
+      <c r="Y317" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z317" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA317" s="6" t="n"/>
+      <c r="AB317" s="6" t="n"/>
+      <c r="AC317" s="6" t="n"/>
+      <c r="AD317" s="6" t="n"/>
+      <c r="AE317" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF317" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B318" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C318" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D318" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E318" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F318" s="4" t="n"/>
+      <c r="G318" s="4" t="n"/>
+      <c r="H318" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I318" s="4" t="inlineStr"/>
+      <c r="J318" s="4" t="inlineStr"/>
+      <c r="K318" s="4" t="inlineStr"/>
+      <c r="L318" s="4" t="n"/>
+      <c r="M318" s="4" t="n"/>
+      <c r="N318" s="4" t="n"/>
+      <c r="O318" s="4" t="n"/>
+      <c r="P318" s="4" t="n"/>
+      <c r="Q318" s="4" t="n"/>
+      <c r="R318" s="4" t="n"/>
+      <c r="S318" s="4" t="n"/>
+      <c r="T318" s="4" t="n"/>
+      <c r="U318" s="4" t="n"/>
+      <c r="V318" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W318" s="4" t="inlineStr"/>
+      <c r="X318" s="4" t="n"/>
+      <c r="Y318" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z318" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA318" s="4" t="n"/>
+      <c r="AB318" s="4" t="n"/>
+      <c r="AC318" s="4" t="n"/>
+      <c r="AD318" s="4" t="n"/>
+      <c r="AE318" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF318" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B319" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C319" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D319" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E319" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F319" s="6" t="n"/>
+      <c r="G319" s="6" t="n"/>
+      <c r="H319" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I319" s="6" t="inlineStr"/>
+      <c r="J319" s="6" t="inlineStr"/>
+      <c r="K319" s="6" t="inlineStr"/>
+      <c r="L319" s="6" t="n"/>
+      <c r="M319" s="6" t="n"/>
+      <c r="N319" s="6" t="n"/>
+      <c r="O319" s="6" t="n"/>
+      <c r="P319" s="6" t="n"/>
+      <c r="Q319" s="6" t="n"/>
+      <c r="R319" s="6" t="n"/>
+      <c r="S319" s="6" t="n"/>
+      <c r="T319" s="6" t="n"/>
+      <c r="U319" s="6" t="n"/>
+      <c r="V319" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W319" s="6" t="inlineStr"/>
+      <c r="X319" s="6" t="n"/>
+      <c r="Y319" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z319" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA319" s="6" t="n"/>
+      <c r="AB319" s="6" t="n"/>
+      <c r="AC319" s="6" t="n"/>
+      <c r="AD319" s="6" t="n"/>
+      <c r="AE319" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF319" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B320" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C320" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D320" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E320" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F320" s="4" t="n"/>
+      <c r="G320" s="4" t="n"/>
+      <c r="H320" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I320" s="4" t="inlineStr"/>
+      <c r="J320" s="4" t="inlineStr"/>
+      <c r="K320" s="4" t="inlineStr"/>
+      <c r="L320" s="4" t="n"/>
+      <c r="M320" s="4" t="n"/>
+      <c r="N320" s="4" t="n"/>
+      <c r="O320" s="4" t="n"/>
+      <c r="P320" s="4" t="n"/>
+      <c r="Q320" s="4" t="n"/>
+      <c r="R320" s="4" t="n"/>
+      <c r="S320" s="4" t="n"/>
+      <c r="T320" s="4" t="n"/>
+      <c r="U320" s="4" t="n"/>
+      <c r="V320" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W320" s="4" t="inlineStr"/>
+      <c r="X320" s="4" t="n"/>
+      <c r="Y320" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z320" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA320" s="4" t="n"/>
+      <c r="AB320" s="4" t="n"/>
+      <c r="AC320" s="4" t="n"/>
+      <c r="AD320" s="4" t="n"/>
+      <c r="AE320" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF320" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B321" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C321" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D321" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E321" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F321" s="6" t="n"/>
+      <c r="G321" s="6" t="n"/>
+      <c r="H321" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I321" s="6" t="inlineStr"/>
+      <c r="J321" s="6" t="inlineStr"/>
+      <c r="K321" s="6" t="inlineStr"/>
+      <c r="L321" s="6" t="n"/>
+      <c r="M321" s="6" t="n"/>
+      <c r="N321" s="6" t="n"/>
+      <c r="O321" s="6" t="n"/>
+      <c r="P321" s="6" t="n"/>
+      <c r="Q321" s="6" t="n"/>
+      <c r="R321" s="6" t="n"/>
+      <c r="S321" s="6" t="n"/>
+      <c r="T321" s="6" t="n"/>
+      <c r="U321" s="6" t="n"/>
+      <c r="V321" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W321" s="6" t="inlineStr"/>
+      <c r="X321" s="6" t="n"/>
+      <c r="Y321" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z321" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA321" s="6" t="n"/>
+      <c r="AB321" s="6" t="n"/>
+      <c r="AC321" s="6" t="n"/>
+      <c r="AD321" s="6" t="n"/>
+      <c r="AE321" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF321" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B322" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C322" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D322" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E322" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F322" s="4" t="n"/>
+      <c r="G322" s="4" t="n"/>
+      <c r="H322" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I322" s="4" t="inlineStr"/>
+      <c r="J322" s="4" t="inlineStr"/>
+      <c r="K322" s="4" t="inlineStr"/>
+      <c r="L322" s="4" t="n"/>
+      <c r="M322" s="4" t="n"/>
+      <c r="N322" s="4" t="n"/>
+      <c r="O322" s="4" t="n"/>
+      <c r="P322" s="4" t="n"/>
+      <c r="Q322" s="4" t="n"/>
+      <c r="R322" s="4" t="n"/>
+      <c r="S322" s="4" t="n"/>
+      <c r="T322" s="4" t="n"/>
+      <c r="U322" s="4" t="n"/>
+      <c r="V322" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W322" s="4" t="inlineStr"/>
+      <c r="X322" s="4" t="n"/>
+      <c r="Y322" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z322" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA322" s="4" t="n"/>
+      <c r="AB322" s="4" t="n"/>
+      <c r="AC322" s="4" t="n"/>
+      <c r="AD322" s="4" t="n"/>
+      <c r="AE322" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF322" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B323" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C323" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D323" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E323" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F323" s="6" t="n"/>
+      <c r="G323" s="6" t="n"/>
+      <c r="H323" s="6" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="I323" s="6" t="inlineStr"/>
+      <c r="J323" s="6" t="inlineStr"/>
+      <c r="K323" s="6" t="inlineStr"/>
+      <c r="L323" s="6" t="n"/>
+      <c r="M323" s="6" t="n"/>
+      <c r="N323" s="6" t="n"/>
+      <c r="O323" s="6" t="n"/>
+      <c r="P323" s="6" t="n"/>
+      <c r="Q323" s="6" t="n"/>
+      <c r="R323" s="6" t="n"/>
+      <c r="S323" s="6" t="n"/>
+      <c r="T323" s="6" t="n"/>
+      <c r="U323" s="6" t="n"/>
+      <c r="V323" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W323" s="6" t="inlineStr"/>
+      <c r="X323" s="6" t="n"/>
+      <c r="Y323" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z323" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA323" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB323" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC323" s="6" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="AD323" s="6" t="n"/>
+      <c r="AE323" s="6" t="n"/>
+      <c r="AF323" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B324" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C324" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D324" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E324" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F324" s="4" t="n"/>
+      <c r="G324" s="4" t="n"/>
+      <c r="H324" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="I324" s="4" t="inlineStr"/>
+      <c r="J324" s="4" t="inlineStr"/>
+      <c r="K324" s="4" t="inlineStr"/>
+      <c r="L324" s="4" t="n"/>
+      <c r="M324" s="4" t="n"/>
+      <c r="N324" s="4" t="n"/>
+      <c r="O324" s="4" t="n"/>
+      <c r="P324" s="4" t="n"/>
+      <c r="Q324" s="4" t="n"/>
+      <c r="R324" s="4" t="n"/>
+      <c r="S324" s="4" t="n"/>
+      <c r="T324" s="4" t="n"/>
+      <c r="U324" s="4" t="n"/>
+      <c r="V324" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W324" s="4" t="inlineStr"/>
+      <c r="X324" s="4" t="n"/>
+      <c r="Y324" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z324" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA324" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB324" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC324" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AD324" s="4" t="n"/>
+      <c r="AE324" s="4" t="n"/>
+      <c r="AF324" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B325" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C325" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D325" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E325" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F325" s="6" t="n"/>
+      <c r="G325" s="6" t="n"/>
+      <c r="H325" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I325" s="6" t="inlineStr"/>
+      <c r="J325" s="6" t="inlineStr"/>
+      <c r="K325" s="6" t="inlineStr"/>
+      <c r="L325" s="6" t="n"/>
+      <c r="M325" s="6" t="n"/>
+      <c r="N325" s="6" t="n"/>
+      <c r="O325" s="6" t="n"/>
+      <c r="P325" s="6" t="n"/>
+      <c r="Q325" s="6" t="n"/>
+      <c r="R325" s="6" t="n"/>
+      <c r="S325" s="6" t="n"/>
+      <c r="T325" s="6" t="n"/>
+      <c r="U325" s="6" t="n"/>
+      <c r="V325" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W325" s="6" t="inlineStr"/>
+      <c r="X325" s="6" t="n"/>
+      <c r="Y325" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z325" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA325" s="6" t="n"/>
+      <c r="AB325" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC325" s="6" t="n"/>
+      <c r="AD325" s="6" t="n"/>
+      <c r="AE325" s="6" t="n"/>
+      <c r="AF325" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="B326" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C326" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D326" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E326" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F326" s="4" t="n"/>
+      <c r="G326" s="4" t="n"/>
+      <c r="H326" s="4" t="n">
+        <v>194.44</v>
+      </c>
+      <c r="I326" s="4" t="inlineStr"/>
+      <c r="J326" s="4" t="inlineStr"/>
+      <c r="K326" s="4" t="inlineStr"/>
+      <c r="L326" s="4" t="n"/>
+      <c r="M326" s="4" t="n"/>
+      <c r="N326" s="4" t="n"/>
+      <c r="O326" s="4" t="n"/>
+      <c r="P326" s="4" t="n"/>
+      <c r="Q326" s="4" t="n"/>
+      <c r="R326" s="4" t="n"/>
+      <c r="S326" s="4" t="n"/>
+      <c r="T326" s="4" t="n"/>
+      <c r="U326" s="4" t="n"/>
+      <c r="V326" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W326" s="4" t="inlineStr"/>
+      <c r="X326" s="4" t="n"/>
+      <c r="Y326" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z326" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA326" s="4" t="n"/>
+      <c r="AB326" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC326" s="4" t="n"/>
+      <c r="AD326" s="4" t="n"/>
+      <c r="AE326" s="4" t="n"/>
+      <c r="AF326" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-28
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF326"/>
+  <dimension ref="A1:AF363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -26218,6 +26218,2918 @@
         <v>1</v>
       </c>
     </row>
+    <row r="327">
+      <c r="A327" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B327" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C327" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D327" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E327" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F327" s="4" t="n"/>
+      <c r="G327" s="4" t="n"/>
+      <c r="H327" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I327" s="4" t="inlineStr"/>
+      <c r="J327" s="4" t="inlineStr"/>
+      <c r="K327" s="4" t="inlineStr"/>
+      <c r="L327" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M327" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N327" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O327" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P327" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q327" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R327" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S327" s="4" t="n"/>
+      <c r="T327" s="4" t="n"/>
+      <c r="U327" s="4" t="n"/>
+      <c r="V327" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W327" s="4" t="inlineStr"/>
+      <c r="X327" s="4" t="n"/>
+      <c r="Y327" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z327" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA327" s="4" t="n"/>
+      <c r="AB327" s="4" t="n"/>
+      <c r="AC327" s="4" t="n"/>
+      <c r="AD327" s="4" t="n"/>
+      <c r="AE327" s="4" t="n"/>
+      <c r="AF327" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B328" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C328" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D328" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E328" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F328" s="6" t="n"/>
+      <c r="G328" s="6" t="n"/>
+      <c r="H328" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I328" s="6" t="inlineStr"/>
+      <c r="J328" s="6" t="inlineStr"/>
+      <c r="K328" s="6" t="inlineStr"/>
+      <c r="L328" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M328" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N328" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O328" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P328" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q328" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R328" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S328" s="6" t="n"/>
+      <c r="T328" s="6" t="n"/>
+      <c r="U328" s="6" t="n"/>
+      <c r="V328" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W328" s="6" t="inlineStr"/>
+      <c r="X328" s="6" t="n"/>
+      <c r="Y328" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z328" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA328" s="6" t="n"/>
+      <c r="AB328" s="6" t="n"/>
+      <c r="AC328" s="6" t="n"/>
+      <c r="AD328" s="6" t="n"/>
+      <c r="AE328" s="6" t="n"/>
+      <c r="AF328" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B329" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C329" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D329" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E329" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F329" s="4" t="n"/>
+      <c r="G329" s="4" t="n"/>
+      <c r="H329" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I329" s="4" t="inlineStr"/>
+      <c r="J329" s="4" t="inlineStr"/>
+      <c r="K329" s="4" t="inlineStr"/>
+      <c r="L329" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M329" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N329" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O329" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P329" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q329" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R329" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S329" s="4" t="n"/>
+      <c r="T329" s="4" t="n"/>
+      <c r="U329" s="4" t="n"/>
+      <c r="V329" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W329" s="4" t="inlineStr"/>
+      <c r="X329" s="4" t="n"/>
+      <c r="Y329" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z329" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA329" s="4" t="n"/>
+      <c r="AB329" s="4" t="n"/>
+      <c r="AC329" s="4" t="n"/>
+      <c r="AD329" s="4" t="n"/>
+      <c r="AE329" s="4" t="n"/>
+      <c r="AF329" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B330" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C330" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D330" s="6" t="inlineStr">
+        <is>
+          <t>625g</t>
+        </is>
+      </c>
+      <c r="E330" s="6" t="n">
+        <v>22.19</v>
+      </c>
+      <c r="F330" s="6" t="n"/>
+      <c r="G330" s="6" t="n"/>
+      <c r="H330" s="6" t="n">
+        <v>35.5</v>
+      </c>
+      <c r="I330" s="6" t="inlineStr"/>
+      <c r="J330" s="6" t="inlineStr"/>
+      <c r="K330" s="6" t="inlineStr"/>
+      <c r="L330" s="6" t="n">
+        <v>49.31</v>
+      </c>
+      <c r="M330" s="6" t="n">
+        <v>1.479</v>
+      </c>
+      <c r="N330" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O330" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P330" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q330" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R330" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S330" s="6" t="n"/>
+      <c r="T330" s="6" t="n"/>
+      <c r="U330" s="6" t="n"/>
+      <c r="V330" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W330" s="6" t="inlineStr"/>
+      <c r="X330" s="6" t="n"/>
+      <c r="Y330" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z330" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA330" s="6" t="n"/>
+      <c r="AB330" s="6" t="n"/>
+      <c r="AC330" s="6" t="n"/>
+      <c r="AD330" s="6" t="n"/>
+      <c r="AE330" s="6" t="n"/>
+      <c r="AF330" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B331" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C331" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D331" s="4" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E331" s="4" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F331" s="4" t="n"/>
+      <c r="G331" s="4" t="n"/>
+      <c r="H331" s="4" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I331" s="4" t="inlineStr"/>
+      <c r="J331" s="4" t="inlineStr"/>
+      <c r="K331" s="4" t="inlineStr"/>
+      <c r="L331" s="4" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M331" s="4" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N331" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O331" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P331" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q331" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R331" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S331" s="4" t="n"/>
+      <c r="T331" s="4" t="n"/>
+      <c r="U331" s="4" t="n"/>
+      <c r="V331" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W331" s="4" t="inlineStr"/>
+      <c r="X331" s="4" t="n"/>
+      <c r="Y331" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z331" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA331" s="4" t="n"/>
+      <c r="AB331" s="4" t="n"/>
+      <c r="AC331" s="4" t="n"/>
+      <c r="AD331" s="4" t="n"/>
+      <c r="AE331" s="4" t="n"/>
+      <c r="AF331" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B332" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C332" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D332" s="6" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E332" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F332" s="6" t="n"/>
+      <c r="G332" s="6" t="n"/>
+      <c r="H332" s="6" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I332" s="6" t="inlineStr"/>
+      <c r="J332" s="6" t="inlineStr"/>
+      <c r="K332" s="6" t="inlineStr"/>
+      <c r="L332" s="6" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M332" s="6" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N332" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O332" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P332" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q332" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R332" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S332" s="6" t="n"/>
+      <c r="T332" s="6" t="n"/>
+      <c r="U332" s="6" t="n"/>
+      <c r="V332" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W332" s="6" t="inlineStr"/>
+      <c r="X332" s="6" t="n"/>
+      <c r="Y332" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z332" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA332" s="6" t="n"/>
+      <c r="AB332" s="6" t="n"/>
+      <c r="AC332" s="6" t="n"/>
+      <c r="AD332" s="6" t="n"/>
+      <c r="AE332" s="6" t="n"/>
+      <c r="AF332" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B333" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C333" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D333" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E333" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F333" s="4" t="n"/>
+      <c r="G333" s="4" t="n"/>
+      <c r="H333" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I333" s="4" t="inlineStr"/>
+      <c r="J333" s="4" t="inlineStr"/>
+      <c r="K333" s="4" t="inlineStr"/>
+      <c r="L333" s="4" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M333" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N333" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O333" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P333" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q333" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R333" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S333" s="4" t="n"/>
+      <c r="T333" s="4" t="n"/>
+      <c r="U333" s="4" t="n"/>
+      <c r="V333" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W333" s="4" t="inlineStr"/>
+      <c r="X333" s="4" t="n"/>
+      <c r="Y333" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z333" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA333" s="4" t="n"/>
+      <c r="AB333" s="4" t="n"/>
+      <c r="AC333" s="4" t="n"/>
+      <c r="AD333" s="4" t="n"/>
+      <c r="AE333" s="4" t="n"/>
+      <c r="AF333" s="4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B334" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C334" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D334" s="6" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E334" s="6" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F334" s="6" t="n"/>
+      <c r="G334" s="6" t="n"/>
+      <c r="H334" s="6" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I334" s="6" t="inlineStr"/>
+      <c r="J334" s="6" t="inlineStr"/>
+      <c r="K334" s="6" t="inlineStr"/>
+      <c r="L334" s="6" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M334" s="6" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N334" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O334" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P334" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q334" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R334" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S334" s="6" t="n"/>
+      <c r="T334" s="6" t="n"/>
+      <c r="U334" s="6" t="n"/>
+      <c r="V334" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W334" s="6" t="inlineStr"/>
+      <c r="X334" s="6" t="n"/>
+      <c r="Y334" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z334" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA334" s="6" t="n"/>
+      <c r="AB334" s="6" t="n"/>
+      <c r="AC334" s="6" t="n"/>
+      <c r="AD334" s="6" t="n"/>
+      <c r="AE334" s="6" t="n"/>
+      <c r="AF334" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B335" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C335" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D335" s="4" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E335" s="4" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F335" s="4" t="n"/>
+      <c r="G335" s="4" t="n"/>
+      <c r="H335" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I335" s="4" t="inlineStr"/>
+      <c r="J335" s="4" t="inlineStr"/>
+      <c r="K335" s="4" t="inlineStr"/>
+      <c r="L335" s="4" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M335" s="4" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N335" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O335" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P335" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q335" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R335" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S335" s="4" t="n"/>
+      <c r="T335" s="4" t="n"/>
+      <c r="U335" s="4" t="n"/>
+      <c r="V335" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W335" s="4" t="inlineStr"/>
+      <c r="X335" s="4" t="n"/>
+      <c r="Y335" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z335" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA335" s="4" t="n"/>
+      <c r="AB335" s="4" t="n"/>
+      <c r="AC335" s="4" t="n"/>
+      <c r="AD335" s="4" t="n"/>
+      <c r="AE335" s="4" t="n"/>
+      <c r="AF335" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B336" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C336" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D336" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E336" s="6" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F336" s="6" t="n"/>
+      <c r="G336" s="6" t="n"/>
+      <c r="H336" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I336" s="6" t="inlineStr"/>
+      <c r="J336" s="6" t="inlineStr"/>
+      <c r="K336" s="6" t="inlineStr"/>
+      <c r="L336" s="6" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M336" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N336" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O336" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P336" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q336" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R336" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S336" s="6" t="n"/>
+      <c r="T336" s="6" t="n"/>
+      <c r="U336" s="6" t="n"/>
+      <c r="V336" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W336" s="6" t="inlineStr"/>
+      <c r="X336" s="6" t="n"/>
+      <c r="Y336" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z336" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA336" s="6" t="n"/>
+      <c r="AB336" s="6" t="n"/>
+      <c r="AC336" s="6" t="n"/>
+      <c r="AD336" s="6" t="n"/>
+      <c r="AE336" s="6" t="n"/>
+      <c r="AF336" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B337" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C337" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D337" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E337" s="4" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F337" s="4" t="n"/>
+      <c r="G337" s="4" t="n"/>
+      <c r="H337" s="4" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I337" s="4" t="inlineStr"/>
+      <c r="J337" s="4" t="inlineStr"/>
+      <c r="K337" s="4" t="inlineStr"/>
+      <c r="L337" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M337" s="4" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N337" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O337" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P337" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q337" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R337" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S337" s="4" t="n"/>
+      <c r="T337" s="4" t="n"/>
+      <c r="U337" s="4" t="n"/>
+      <c r="V337" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W337" s="4" t="inlineStr"/>
+      <c r="X337" s="4" t="n"/>
+      <c r="Y337" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z337" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA337" s="4" t="n"/>
+      <c r="AB337" s="4" t="n"/>
+      <c r="AC337" s="4" t="n"/>
+      <c r="AD337" s="4" t="n"/>
+      <c r="AE337" s="4" t="n"/>
+      <c r="AF337" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B338" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C338" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D338" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E338" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F338" s="6" t="n"/>
+      <c r="G338" s="6" t="n"/>
+      <c r="H338" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I338" s="6" t="inlineStr"/>
+      <c r="J338" s="6" t="inlineStr"/>
+      <c r="K338" s="6" t="inlineStr"/>
+      <c r="L338" s="6" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M338" s="6" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N338" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O338" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P338" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q338" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R338" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S338" s="6" t="n"/>
+      <c r="T338" s="6" t="n"/>
+      <c r="U338" s="6" t="n"/>
+      <c r="V338" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W338" s="6" t="inlineStr"/>
+      <c r="X338" s="6" t="n"/>
+      <c r="Y338" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z338" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA338" s="6" t="n"/>
+      <c r="AB338" s="6" t="n"/>
+      <c r="AC338" s="6" t="n"/>
+      <c r="AD338" s="6" t="n"/>
+      <c r="AE338" s="6" t="n"/>
+      <c r="AF338" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B339" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C339" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D339" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E339" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F339" s="4" t="n"/>
+      <c r="G339" s="4" t="n"/>
+      <c r="H339" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I339" s="4" t="inlineStr"/>
+      <c r="J339" s="4" t="inlineStr"/>
+      <c r="K339" s="4" t="inlineStr"/>
+      <c r="L339" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M339" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N339" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O339" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P339" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q339" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R339" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S339" s="4" t="n"/>
+      <c r="T339" s="4" t="n"/>
+      <c r="U339" s="4" t="n"/>
+      <c r="V339" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W339" s="4" t="inlineStr"/>
+      <c r="X339" s="4" t="n"/>
+      <c r="Y339" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z339" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA339" s="4" t="n"/>
+      <c r="AB339" s="4" t="n"/>
+      <c r="AC339" s="4" t="n"/>
+      <c r="AD339" s="4" t="n"/>
+      <c r="AE339" s="4" t="n"/>
+      <c r="AF339" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B340" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C340" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D340" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E340" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F340" s="6" t="n"/>
+      <c r="G340" s="6" t="n"/>
+      <c r="H340" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I340" s="6" t="inlineStr"/>
+      <c r="J340" s="6" t="inlineStr"/>
+      <c r="K340" s="6" t="inlineStr"/>
+      <c r="L340" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M340" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N340" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O340" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P340" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q340" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R340" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S340" s="6" t="n"/>
+      <c r="T340" s="6" t="n"/>
+      <c r="U340" s="6" t="n"/>
+      <c r="V340" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W340" s="6" t="inlineStr"/>
+      <c r="X340" s="6" t="n"/>
+      <c r="Y340" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z340" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA340" s="6" t="n"/>
+      <c r="AB340" s="6" t="n"/>
+      <c r="AC340" s="6" t="n"/>
+      <c r="AD340" s="6" t="n"/>
+      <c r="AE340" s="6" t="n"/>
+      <c r="AF340" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B341" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C341" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D341" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E341" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F341" s="4" t="n"/>
+      <c r="G341" s="4" t="n"/>
+      <c r="H341" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I341" s="4" t="inlineStr"/>
+      <c r="J341" s="4" t="inlineStr"/>
+      <c r="K341" s="4" t="inlineStr"/>
+      <c r="L341" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M341" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N341" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O341" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P341" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q341" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R341" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S341" s="4" t="n"/>
+      <c r="T341" s="4" t="n"/>
+      <c r="U341" s="4" t="n"/>
+      <c r="V341" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W341" s="4" t="inlineStr"/>
+      <c r="X341" s="4" t="n"/>
+      <c r="Y341" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z341" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA341" s="4" t="n"/>
+      <c r="AB341" s="4" t="n"/>
+      <c r="AC341" s="4" t="n"/>
+      <c r="AD341" s="4" t="n"/>
+      <c r="AE341" s="4" t="n"/>
+      <c r="AF341" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B342" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C342" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D342" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E342" s="6" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F342" s="6" t="n"/>
+      <c r="G342" s="6" t="n"/>
+      <c r="H342" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I342" s="6" t="inlineStr"/>
+      <c r="J342" s="6" t="inlineStr"/>
+      <c r="K342" s="6" t="inlineStr"/>
+      <c r="L342" s="6" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M342" s="6" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N342" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O342" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P342" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q342" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R342" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S342" s="6" t="n"/>
+      <c r="T342" s="6" t="n"/>
+      <c r="U342" s="6" t="n"/>
+      <c r="V342" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W342" s="6" t="inlineStr"/>
+      <c r="X342" s="6" t="n"/>
+      <c r="Y342" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z342" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA342" s="6" t="n"/>
+      <c r="AB342" s="6" t="n"/>
+      <c r="AC342" s="6" t="n"/>
+      <c r="AD342" s="6" t="n"/>
+      <c r="AE342" s="6" t="n"/>
+      <c r="AF342" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B343" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C343" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D343" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E343" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F343" s="4" t="n"/>
+      <c r="G343" s="4" t="n"/>
+      <c r="H343" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I343" s="4" t="inlineStr"/>
+      <c r="J343" s="4" t="inlineStr"/>
+      <c r="K343" s="4" t="inlineStr"/>
+      <c r="L343" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M343" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N343" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O343" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P343" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q343" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R343" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S343" s="4" t="n"/>
+      <c r="T343" s="4" t="n"/>
+      <c r="U343" s="4" t="n"/>
+      <c r="V343" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W343" s="4" t="inlineStr"/>
+      <c r="X343" s="4" t="n"/>
+      <c r="Y343" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z343" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA343" s="4" t="n"/>
+      <c r="AB343" s="4" t="n"/>
+      <c r="AC343" s="4" t="n"/>
+      <c r="AD343" s="4" t="n"/>
+      <c r="AE343" s="4" t="n"/>
+      <c r="AF343" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B344" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C344" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D344" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E344" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F344" s="6" t="n"/>
+      <c r="G344" s="6" t="n"/>
+      <c r="H344" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I344" s="6" t="inlineStr"/>
+      <c r="J344" s="6" t="inlineStr"/>
+      <c r="K344" s="6" t="inlineStr"/>
+      <c r="L344" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M344" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N344" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O344" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P344" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q344" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R344" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S344" s="6" t="n"/>
+      <c r="T344" s="6" t="n"/>
+      <c r="U344" s="6" t="n"/>
+      <c r="V344" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W344" s="6" t="inlineStr"/>
+      <c r="X344" s="6" t="n"/>
+      <c r="Y344" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z344" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA344" s="6" t="n"/>
+      <c r="AB344" s="6" t="n"/>
+      <c r="AC344" s="6" t="n"/>
+      <c r="AD344" s="6" t="n"/>
+      <c r="AE344" s="6" t="n"/>
+      <c r="AF344" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B345" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C345" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D345" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E345" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F345" s="4" t="n"/>
+      <c r="G345" s="4" t="n"/>
+      <c r="H345" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I345" s="4" t="inlineStr"/>
+      <c r="J345" s="4" t="inlineStr"/>
+      <c r="K345" s="4" t="inlineStr"/>
+      <c r="L345" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M345" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N345" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O345" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P345" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q345" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R345" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S345" s="4" t="n"/>
+      <c r="T345" s="4" t="n"/>
+      <c r="U345" s="4" t="n"/>
+      <c r="V345" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W345" s="4" t="inlineStr"/>
+      <c r="X345" s="4" t="n"/>
+      <c r="Y345" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z345" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA345" s="4" t="n"/>
+      <c r="AB345" s="4" t="n"/>
+      <c r="AC345" s="4" t="n"/>
+      <c r="AD345" s="4" t="n"/>
+      <c r="AE345" s="4" t="n"/>
+      <c r="AF345" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B346" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C346" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D346" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E346" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F346" s="6" t="n"/>
+      <c r="G346" s="6" t="n"/>
+      <c r="H346" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I346" s="6" t="inlineStr"/>
+      <c r="J346" s="6" t="inlineStr"/>
+      <c r="K346" s="6" t="inlineStr"/>
+      <c r="L346" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M346" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N346" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O346" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P346" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q346" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R346" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S346" s="6" t="n"/>
+      <c r="T346" s="6" t="n"/>
+      <c r="U346" s="6" t="n"/>
+      <c r="V346" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W346" s="6" t="inlineStr"/>
+      <c r="X346" s="6" t="n"/>
+      <c r="Y346" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z346" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA346" s="6" t="n"/>
+      <c r="AB346" s="6" t="n"/>
+      <c r="AC346" s="6" t="n"/>
+      <c r="AD346" s="6" t="n"/>
+      <c r="AE346" s="6" t="n"/>
+      <c r="AF346" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B347" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C347" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D347" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E347" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F347" s="4" t="n"/>
+      <c r="G347" s="4" t="n"/>
+      <c r="H347" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I347" s="4" t="inlineStr"/>
+      <c r="J347" s="4" t="inlineStr"/>
+      <c r="K347" s="4" t="inlineStr"/>
+      <c r="L347" s="4" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="M347" s="4" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="N347" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O347" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P347" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q347" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R347" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S347" s="4" t="n"/>
+      <c r="T347" s="4" t="n"/>
+      <c r="U347" s="4" t="n"/>
+      <c r="V347" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W347" s="4" t="inlineStr"/>
+      <c r="X347" s="4" t="n"/>
+      <c r="Y347" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z347" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA347" s="4" t="n"/>
+      <c r="AB347" s="4" t="n"/>
+      <c r="AC347" s="4" t="n"/>
+      <c r="AD347" s="4" t="n"/>
+      <c r="AE347" s="4" t="n"/>
+      <c r="AF347" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B348" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C348" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D348" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E348" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F348" s="6" t="n"/>
+      <c r="G348" s="6" t="n"/>
+      <c r="H348" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I348" s="6" t="inlineStr"/>
+      <c r="J348" s="6" t="inlineStr"/>
+      <c r="K348" s="6" t="inlineStr"/>
+      <c r="L348" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M348" s="6" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N348" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O348" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P348" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q348" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R348" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S348" s="6" t="n"/>
+      <c r="T348" s="6" t="n"/>
+      <c r="U348" s="6" t="n"/>
+      <c r="V348" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W348" s="6" t="inlineStr"/>
+      <c r="X348" s="6" t="n"/>
+      <c r="Y348" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z348" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA348" s="6" t="n"/>
+      <c r="AB348" s="6" t="n"/>
+      <c r="AC348" s="6" t="n"/>
+      <c r="AD348" s="6" t="n"/>
+      <c r="AE348" s="6" t="n"/>
+      <c r="AF348" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B349" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C349" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D349" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E349" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F349" s="4" t="n"/>
+      <c r="G349" s="4" t="n"/>
+      <c r="H349" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I349" s="4" t="inlineStr"/>
+      <c r="J349" s="4" t="inlineStr"/>
+      <c r="K349" s="4" t="inlineStr"/>
+      <c r="L349" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M349" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N349" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O349" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P349" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q349" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R349" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S349" s="4" t="n"/>
+      <c r="T349" s="4" t="n"/>
+      <c r="U349" s="4" t="n"/>
+      <c r="V349" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W349" s="4" t="inlineStr"/>
+      <c r="X349" s="4" t="n"/>
+      <c r="Y349" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z349" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA349" s="4" t="n"/>
+      <c r="AB349" s="4" t="n"/>
+      <c r="AC349" s="4" t="n"/>
+      <c r="AD349" s="4" t="n"/>
+      <c r="AE349" s="4" t="n"/>
+      <c r="AF349" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B350" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C350" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D350" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E350" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F350" s="6" t="n"/>
+      <c r="G350" s="6" t="n"/>
+      <c r="H350" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I350" s="6" t="inlineStr"/>
+      <c r="J350" s="6" t="inlineStr"/>
+      <c r="K350" s="6" t="inlineStr"/>
+      <c r="L350" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M350" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N350" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O350" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P350" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q350" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R350" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S350" s="6" t="n"/>
+      <c r="T350" s="6" t="n"/>
+      <c r="U350" s="6" t="n"/>
+      <c r="V350" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W350" s="6" t="inlineStr"/>
+      <c r="X350" s="6" t="n"/>
+      <c r="Y350" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z350" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA350" s="6" t="n"/>
+      <c r="AB350" s="6" t="n"/>
+      <c r="AC350" s="6" t="n"/>
+      <c r="AD350" s="6" t="n"/>
+      <c r="AE350" s="6" t="n"/>
+      <c r="AF350" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B351" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C351" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D351" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E351" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F351" s="4" t="n"/>
+      <c r="G351" s="4" t="n"/>
+      <c r="H351" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I351" s="4" t="inlineStr"/>
+      <c r="J351" s="4" t="inlineStr"/>
+      <c r="K351" s="4" t="inlineStr"/>
+      <c r="L351" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M351" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N351" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O351" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P351" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q351" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R351" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S351" s="4" t="n"/>
+      <c r="T351" s="4" t="n"/>
+      <c r="U351" s="4" t="n"/>
+      <c r="V351" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W351" s="4" t="inlineStr"/>
+      <c r="X351" s="4" t="n"/>
+      <c r="Y351" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z351" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA351" s="4" t="n"/>
+      <c r="AB351" s="4" t="n"/>
+      <c r="AC351" s="4" t="n"/>
+      <c r="AD351" s="4" t="n"/>
+      <c r="AE351" s="4" t="n"/>
+      <c r="AF351" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B352" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C352" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D352" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E352" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F352" s="6" t="n"/>
+      <c r="G352" s="6" t="n"/>
+      <c r="H352" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I352" s="6" t="inlineStr"/>
+      <c r="J352" s="6" t="inlineStr"/>
+      <c r="K352" s="6" t="inlineStr"/>
+      <c r="L352" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M352" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N352" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O352" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P352" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q352" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R352" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S352" s="6" t="n"/>
+      <c r="T352" s="6" t="n"/>
+      <c r="U352" s="6" t="n"/>
+      <c r="V352" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W352" s="6" t="inlineStr"/>
+      <c r="X352" s="6" t="n"/>
+      <c r="Y352" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z352" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA352" s="6" t="n"/>
+      <c r="AB352" s="6" t="n"/>
+      <c r="AC352" s="6" t="n"/>
+      <c r="AD352" s="6" t="n"/>
+      <c r="AE352" s="6" t="n"/>
+      <c r="AF352" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B353" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C353" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D353" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E353" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F353" s="4" t="n"/>
+      <c r="G353" s="4" t="n"/>
+      <c r="H353" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I353" s="4" t="inlineStr"/>
+      <c r="J353" s="4" t="inlineStr"/>
+      <c r="K353" s="4" t="inlineStr"/>
+      <c r="L353" s="4" t="n"/>
+      <c r="M353" s="4" t="n"/>
+      <c r="N353" s="4" t="n"/>
+      <c r="O353" s="4" t="n"/>
+      <c r="P353" s="4" t="n"/>
+      <c r="Q353" s="4" t="n"/>
+      <c r="R353" s="4" t="n"/>
+      <c r="S353" s="4" t="n"/>
+      <c r="T353" s="4" t="n"/>
+      <c r="U353" s="4" t="n"/>
+      <c r="V353" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W353" s="4" t="inlineStr"/>
+      <c r="X353" s="4" t="n"/>
+      <c r="Y353" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z353" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA353" s="4" t="n"/>
+      <c r="AB353" s="4" t="n"/>
+      <c r="AC353" s="4" t="n"/>
+      <c r="AD353" s="4" t="n"/>
+      <c r="AE353" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF353" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B354" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C354" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D354" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E354" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F354" s="6" t="n"/>
+      <c r="G354" s="6" t="n"/>
+      <c r="H354" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I354" s="6" t="inlineStr"/>
+      <c r="J354" s="6" t="inlineStr"/>
+      <c r="K354" s="6" t="inlineStr"/>
+      <c r="L354" s="6" t="n"/>
+      <c r="M354" s="6" t="n"/>
+      <c r="N354" s="6" t="n"/>
+      <c r="O354" s="6" t="n"/>
+      <c r="P354" s="6" t="n"/>
+      <c r="Q354" s="6" t="n"/>
+      <c r="R354" s="6" t="n"/>
+      <c r="S354" s="6" t="n"/>
+      <c r="T354" s="6" t="n"/>
+      <c r="U354" s="6" t="n"/>
+      <c r="V354" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W354" s="6" t="inlineStr"/>
+      <c r="X354" s="6" t="n"/>
+      <c r="Y354" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z354" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA354" s="6" t="n"/>
+      <c r="AB354" s="6" t="n"/>
+      <c r="AC354" s="6" t="n"/>
+      <c r="AD354" s="6" t="n"/>
+      <c r="AE354" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF354" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B355" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C355" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D355" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E355" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F355" s="4" t="n"/>
+      <c r="G355" s="4" t="n"/>
+      <c r="H355" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I355" s="4" t="inlineStr"/>
+      <c r="J355" s="4" t="inlineStr"/>
+      <c r="K355" s="4" t="inlineStr"/>
+      <c r="L355" s="4" t="n"/>
+      <c r="M355" s="4" t="n"/>
+      <c r="N355" s="4" t="n"/>
+      <c r="O355" s="4" t="n"/>
+      <c r="P355" s="4" t="n"/>
+      <c r="Q355" s="4" t="n"/>
+      <c r="R355" s="4" t="n"/>
+      <c r="S355" s="4" t="n"/>
+      <c r="T355" s="4" t="n"/>
+      <c r="U355" s="4" t="n"/>
+      <c r="V355" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W355" s="4" t="inlineStr"/>
+      <c r="X355" s="4" t="n"/>
+      <c r="Y355" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z355" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA355" s="4" t="n"/>
+      <c r="AB355" s="4" t="n"/>
+      <c r="AC355" s="4" t="n"/>
+      <c r="AD355" s="4" t="n"/>
+      <c r="AE355" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF355" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B356" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C356" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D356" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E356" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F356" s="6" t="n"/>
+      <c r="G356" s="6" t="n"/>
+      <c r="H356" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I356" s="6" t="inlineStr"/>
+      <c r="J356" s="6" t="inlineStr"/>
+      <c r="K356" s="6" t="inlineStr"/>
+      <c r="L356" s="6" t="n"/>
+      <c r="M356" s="6" t="n"/>
+      <c r="N356" s="6" t="n"/>
+      <c r="O356" s="6" t="n"/>
+      <c r="P356" s="6" t="n"/>
+      <c r="Q356" s="6" t="n"/>
+      <c r="R356" s="6" t="n"/>
+      <c r="S356" s="6" t="n"/>
+      <c r="T356" s="6" t="n"/>
+      <c r="U356" s="6" t="n"/>
+      <c r="V356" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W356" s="6" t="inlineStr"/>
+      <c r="X356" s="6" t="n"/>
+      <c r="Y356" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z356" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA356" s="6" t="n"/>
+      <c r="AB356" s="6" t="n"/>
+      <c r="AC356" s="6" t="n"/>
+      <c r="AD356" s="6" t="n"/>
+      <c r="AE356" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF356" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B357" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C357" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D357" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E357" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F357" s="4" t="n"/>
+      <c r="G357" s="4" t="n"/>
+      <c r="H357" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I357" s="4" t="inlineStr"/>
+      <c r="J357" s="4" t="inlineStr"/>
+      <c r="K357" s="4" t="inlineStr"/>
+      <c r="L357" s="4" t="n"/>
+      <c r="M357" s="4" t="n"/>
+      <c r="N357" s="4" t="n"/>
+      <c r="O357" s="4" t="n"/>
+      <c r="P357" s="4" t="n"/>
+      <c r="Q357" s="4" t="n"/>
+      <c r="R357" s="4" t="n"/>
+      <c r="S357" s="4" t="n"/>
+      <c r="T357" s="4" t="n"/>
+      <c r="U357" s="4" t="n"/>
+      <c r="V357" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W357" s="4" t="inlineStr"/>
+      <c r="X357" s="4" t="n"/>
+      <c r="Y357" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z357" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA357" s="4" t="n"/>
+      <c r="AB357" s="4" t="n"/>
+      <c r="AC357" s="4" t="n"/>
+      <c r="AD357" s="4" t="n"/>
+      <c r="AE357" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF357" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B358" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C358" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D358" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E358" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F358" s="6" t="n"/>
+      <c r="G358" s="6" t="n"/>
+      <c r="H358" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I358" s="6" t="inlineStr"/>
+      <c r="J358" s="6" t="inlineStr"/>
+      <c r="K358" s="6" t="inlineStr"/>
+      <c r="L358" s="6" t="n"/>
+      <c r="M358" s="6" t="n"/>
+      <c r="N358" s="6" t="n"/>
+      <c r="O358" s="6" t="n"/>
+      <c r="P358" s="6" t="n"/>
+      <c r="Q358" s="6" t="n"/>
+      <c r="R358" s="6" t="n"/>
+      <c r="S358" s="6" t="n"/>
+      <c r="T358" s="6" t="n"/>
+      <c r="U358" s="6" t="n"/>
+      <c r="V358" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W358" s="6" t="inlineStr"/>
+      <c r="X358" s="6" t="n"/>
+      <c r="Y358" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z358" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA358" s="6" t="n"/>
+      <c r="AB358" s="6" t="n"/>
+      <c r="AC358" s="6" t="n"/>
+      <c r="AD358" s="6" t="n"/>
+      <c r="AE358" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF358" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B359" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C359" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D359" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E359" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F359" s="4" t="n"/>
+      <c r="G359" s="4" t="n"/>
+      <c r="H359" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I359" s="4" t="inlineStr"/>
+      <c r="J359" s="4" t="inlineStr"/>
+      <c r="K359" s="4" t="inlineStr"/>
+      <c r="L359" s="4" t="n"/>
+      <c r="M359" s="4" t="n"/>
+      <c r="N359" s="4" t="n"/>
+      <c r="O359" s="4" t="n"/>
+      <c r="P359" s="4" t="n"/>
+      <c r="Q359" s="4" t="n"/>
+      <c r="R359" s="4" t="n"/>
+      <c r="S359" s="4" t="n"/>
+      <c r="T359" s="4" t="n"/>
+      <c r="U359" s="4" t="n"/>
+      <c r="V359" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W359" s="4" t="inlineStr"/>
+      <c r="X359" s="4" t="n"/>
+      <c r="Y359" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z359" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA359" s="4" t="n"/>
+      <c r="AB359" s="4" t="n"/>
+      <c r="AC359" s="4" t="n"/>
+      <c r="AD359" s="4" t="n"/>
+      <c r="AE359" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF359" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B360" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C360" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D360" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E360" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F360" s="6" t="n"/>
+      <c r="G360" s="6" t="n"/>
+      <c r="H360" s="6" t="n">
+        <v>83.33</v>
+      </c>
+      <c r="I360" s="6" t="inlineStr"/>
+      <c r="J360" s="6" t="inlineStr"/>
+      <c r="K360" s="6" t="inlineStr"/>
+      <c r="L360" s="6" t="n"/>
+      <c r="M360" s="6" t="n"/>
+      <c r="N360" s="6" t="n"/>
+      <c r="O360" s="6" t="n"/>
+      <c r="P360" s="6" t="n"/>
+      <c r="Q360" s="6" t="n"/>
+      <c r="R360" s="6" t="n"/>
+      <c r="S360" s="6" t="n"/>
+      <c r="T360" s="6" t="n"/>
+      <c r="U360" s="6" t="n"/>
+      <c r="V360" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W360" s="6" t="inlineStr"/>
+      <c r="X360" s="6" t="n"/>
+      <c r="Y360" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z360" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA360" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB360" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC360" s="6" t="n">
+        <v>0.278</v>
+      </c>
+      <c r="AD360" s="6" t="n"/>
+      <c r="AE360" s="6" t="n"/>
+      <c r="AF360" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B361" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C361" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D361" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E361" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="F361" s="4" t="n"/>
+      <c r="G361" s="4" t="n"/>
+      <c r="H361" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="I361" s="4" t="inlineStr"/>
+      <c r="J361" s="4" t="inlineStr"/>
+      <c r="K361" s="4" t="inlineStr"/>
+      <c r="L361" s="4" t="n"/>
+      <c r="M361" s="4" t="n"/>
+      <c r="N361" s="4" t="n"/>
+      <c r="O361" s="4" t="n"/>
+      <c r="P361" s="4" t="n"/>
+      <c r="Q361" s="4" t="n"/>
+      <c r="R361" s="4" t="n"/>
+      <c r="S361" s="4" t="n"/>
+      <c r="T361" s="4" t="n"/>
+      <c r="U361" s="4" t="n"/>
+      <c r="V361" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W361" s="4" t="inlineStr"/>
+      <c r="X361" s="4" t="n"/>
+      <c r="Y361" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z361" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA361" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB361" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC361" s="4" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AD361" s="4" t="n"/>
+      <c r="AE361" s="4" t="n"/>
+      <c r="AF361" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B362" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C362" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D362" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E362" s="6" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F362" s="6" t="n"/>
+      <c r="G362" s="6" t="n"/>
+      <c r="H362" s="6" t="n">
+        <v>250</v>
+      </c>
+      <c r="I362" s="6" t="inlineStr"/>
+      <c r="J362" s="6" t="inlineStr"/>
+      <c r="K362" s="6" t="inlineStr"/>
+      <c r="L362" s="6" t="n"/>
+      <c r="M362" s="6" t="n"/>
+      <c r="N362" s="6" t="n"/>
+      <c r="O362" s="6" t="n"/>
+      <c r="P362" s="6" t="n"/>
+      <c r="Q362" s="6" t="n"/>
+      <c r="R362" s="6" t="n"/>
+      <c r="S362" s="6" t="n"/>
+      <c r="T362" s="6" t="n"/>
+      <c r="U362" s="6" t="n"/>
+      <c r="V362" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W362" s="6" t="inlineStr"/>
+      <c r="X362" s="6" t="n"/>
+      <c r="Y362" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z362" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA362" s="6" t="n"/>
+      <c r="AB362" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC362" s="6" t="n"/>
+      <c r="AD362" s="6" t="n"/>
+      <c r="AE362" s="6" t="n"/>
+      <c r="AF362" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B363" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C363" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D363" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E363" s="4" t="n">
+        <v>17.5</v>
+      </c>
+      <c r="F363" s="4" t="n"/>
+      <c r="G363" s="4" t="n"/>
+      <c r="H363" s="4" t="n">
+        <v>194.44</v>
+      </c>
+      <c r="I363" s="4" t="inlineStr"/>
+      <c r="J363" s="4" t="inlineStr"/>
+      <c r="K363" s="4" t="inlineStr"/>
+      <c r="L363" s="4" t="n"/>
+      <c r="M363" s="4" t="n"/>
+      <c r="N363" s="4" t="n"/>
+      <c r="O363" s="4" t="n"/>
+      <c r="P363" s="4" t="n"/>
+      <c r="Q363" s="4" t="n"/>
+      <c r="R363" s="4" t="n"/>
+      <c r="S363" s="4" t="n"/>
+      <c r="T363" s="4" t="n"/>
+      <c r="U363" s="4" t="n"/>
+      <c r="V363" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W363" s="4" t="inlineStr"/>
+      <c r="X363" s="4" t="n"/>
+      <c r="Y363" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z363" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA363" s="4" t="n"/>
+      <c r="AB363" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC363" s="4" t="n"/>
+      <c r="AD363" s="4" t="n"/>
+      <c r="AE363" s="4" t="n"/>
+      <c r="AF363" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-29
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF363"/>
+  <dimension ref="A1:AF399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -29130,6 +29130,2836 @@
         <v>1</v>
       </c>
     </row>
+    <row r="364">
+      <c r="A364" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B364" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C364" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D364" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E364" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F364" s="4" t="n"/>
+      <c r="G364" s="4" t="n"/>
+      <c r="H364" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I364" s="4" t="inlineStr"/>
+      <c r="J364" s="4" t="inlineStr"/>
+      <c r="K364" s="4" t="inlineStr"/>
+      <c r="L364" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M364" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N364" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O364" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P364" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q364" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R364" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S364" s="4" t="n"/>
+      <c r="T364" s="4" t="n"/>
+      <c r="U364" s="4" t="n"/>
+      <c r="V364" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W364" s="4" t="inlineStr"/>
+      <c r="X364" s="4" t="n"/>
+      <c r="Y364" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z364" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA364" s="4" t="n"/>
+      <c r="AB364" s="4" t="n"/>
+      <c r="AC364" s="4" t="n"/>
+      <c r="AD364" s="4" t="n"/>
+      <c r="AE364" s="4" t="n"/>
+      <c r="AF364" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B365" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C365" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D365" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E365" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F365" s="6" t="n"/>
+      <c r="G365" s="6" t="n"/>
+      <c r="H365" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I365" s="6" t="inlineStr"/>
+      <c r="J365" s="6" t="inlineStr"/>
+      <c r="K365" s="6" t="inlineStr"/>
+      <c r="L365" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M365" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N365" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O365" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P365" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q365" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R365" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S365" s="6" t="n"/>
+      <c r="T365" s="6" t="n"/>
+      <c r="U365" s="6" t="n"/>
+      <c r="V365" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W365" s="6" t="inlineStr"/>
+      <c r="X365" s="6" t="n"/>
+      <c r="Y365" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z365" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA365" s="6" t="n"/>
+      <c r="AB365" s="6" t="n"/>
+      <c r="AC365" s="6" t="n"/>
+      <c r="AD365" s="6" t="n"/>
+      <c r="AE365" s="6" t="n"/>
+      <c r="AF365" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B366" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C366" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D366" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E366" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F366" s="4" t="n"/>
+      <c r="G366" s="4" t="n"/>
+      <c r="H366" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I366" s="4" t="inlineStr"/>
+      <c r="J366" s="4" t="inlineStr"/>
+      <c r="K366" s="4" t="inlineStr"/>
+      <c r="L366" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M366" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N366" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O366" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P366" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q366" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R366" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S366" s="4" t="n"/>
+      <c r="T366" s="4" t="n"/>
+      <c r="U366" s="4" t="n"/>
+      <c r="V366" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W366" s="4" t="inlineStr"/>
+      <c r="X366" s="4" t="n"/>
+      <c r="Y366" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z366" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA366" s="4" t="n"/>
+      <c r="AB366" s="4" t="n"/>
+      <c r="AC366" s="4" t="n"/>
+      <c r="AD366" s="4" t="n"/>
+      <c r="AE366" s="4" t="n"/>
+      <c r="AF366" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B367" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C367" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D367" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E367" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F367" s="6" t="n"/>
+      <c r="G367" s="6" t="n"/>
+      <c r="H367" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I367" s="6" t="inlineStr"/>
+      <c r="J367" s="6" t="inlineStr"/>
+      <c r="K367" s="6" t="inlineStr"/>
+      <c r="L367" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M367" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N367" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O367" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P367" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q367" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R367" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S367" s="6" t="n"/>
+      <c r="T367" s="6" t="n"/>
+      <c r="U367" s="6" t="n"/>
+      <c r="V367" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W367" s="6" t="inlineStr"/>
+      <c r="X367" s="6" t="n"/>
+      <c r="Y367" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z367" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA367" s="6" t="n"/>
+      <c r="AB367" s="6" t="n"/>
+      <c r="AC367" s="6" t="n"/>
+      <c r="AD367" s="6" t="n"/>
+      <c r="AE367" s="6" t="n"/>
+      <c r="AF367" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B368" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C368" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D368" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E368" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F368" s="4" t="n"/>
+      <c r="G368" s="4" t="n"/>
+      <c r="H368" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I368" s="4" t="inlineStr"/>
+      <c r="J368" s="4" t="inlineStr"/>
+      <c r="K368" s="4" t="inlineStr"/>
+      <c r="L368" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M368" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N368" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O368" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P368" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q368" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R368" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S368" s="4" t="n"/>
+      <c r="T368" s="4" t="n"/>
+      <c r="U368" s="4" t="n"/>
+      <c r="V368" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W368" s="4" t="inlineStr"/>
+      <c r="X368" s="4" t="n"/>
+      <c r="Y368" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z368" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA368" s="4" t="n"/>
+      <c r="AB368" s="4" t="n"/>
+      <c r="AC368" s="4" t="n"/>
+      <c r="AD368" s="4" t="n"/>
+      <c r="AE368" s="4" t="n"/>
+      <c r="AF368" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B369" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C369" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D369" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E369" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F369" s="6" t="n"/>
+      <c r="G369" s="6" t="n"/>
+      <c r="H369" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I369" s="6" t="inlineStr"/>
+      <c r="J369" s="6" t="inlineStr"/>
+      <c r="K369" s="6" t="inlineStr"/>
+      <c r="L369" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M369" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N369" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O369" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P369" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q369" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R369" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S369" s="6" t="n"/>
+      <c r="T369" s="6" t="n"/>
+      <c r="U369" s="6" t="n"/>
+      <c r="V369" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W369" s="6" t="inlineStr"/>
+      <c r="X369" s="6" t="n"/>
+      <c r="Y369" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z369" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA369" s="6" t="n"/>
+      <c r="AB369" s="6" t="n"/>
+      <c r="AC369" s="6" t="n"/>
+      <c r="AD369" s="6" t="n"/>
+      <c r="AE369" s="6" t="n"/>
+      <c r="AF369" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B370" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C370" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D370" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E370" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F370" s="4" t="n"/>
+      <c r="G370" s="4" t="n"/>
+      <c r="H370" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I370" s="4" t="inlineStr"/>
+      <c r="J370" s="4" t="inlineStr"/>
+      <c r="K370" s="4" t="inlineStr"/>
+      <c r="L370" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M370" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N370" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O370" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P370" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q370" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R370" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S370" s="4" t="n"/>
+      <c r="T370" s="4" t="n"/>
+      <c r="U370" s="4" t="n"/>
+      <c r="V370" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W370" s="4" t="inlineStr"/>
+      <c r="X370" s="4" t="n"/>
+      <c r="Y370" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z370" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA370" s="4" t="n"/>
+      <c r="AB370" s="4" t="n"/>
+      <c r="AC370" s="4" t="n"/>
+      <c r="AD370" s="4" t="n"/>
+      <c r="AE370" s="4" t="n"/>
+      <c r="AF370" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B371" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C371" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D371" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E371" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F371" s="6" t="n"/>
+      <c r="G371" s="6" t="n"/>
+      <c r="H371" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I371" s="6" t="inlineStr"/>
+      <c r="J371" s="6" t="inlineStr"/>
+      <c r="K371" s="6" t="inlineStr"/>
+      <c r="L371" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M371" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N371" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O371" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P371" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q371" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R371" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S371" s="6" t="n"/>
+      <c r="T371" s="6" t="n"/>
+      <c r="U371" s="6" t="n"/>
+      <c r="V371" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W371" s="6" t="inlineStr"/>
+      <c r="X371" s="6" t="n"/>
+      <c r="Y371" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z371" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA371" s="6" t="n"/>
+      <c r="AB371" s="6" t="n"/>
+      <c r="AC371" s="6" t="n"/>
+      <c r="AD371" s="6" t="n"/>
+      <c r="AE371" s="6" t="n"/>
+      <c r="AF371" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B372" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C372" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D372" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E372" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F372" s="4" t="n"/>
+      <c r="G372" s="4" t="n"/>
+      <c r="H372" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I372" s="4" t="inlineStr"/>
+      <c r="J372" s="4" t="inlineStr"/>
+      <c r="K372" s="4" t="inlineStr"/>
+      <c r="L372" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M372" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N372" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O372" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P372" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q372" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R372" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S372" s="4" t="n"/>
+      <c r="T372" s="4" t="n"/>
+      <c r="U372" s="4" t="n"/>
+      <c r="V372" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W372" s="4" t="inlineStr"/>
+      <c r="X372" s="4" t="n"/>
+      <c r="Y372" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z372" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA372" s="4" t="n"/>
+      <c r="AB372" s="4" t="n"/>
+      <c r="AC372" s="4" t="n"/>
+      <c r="AD372" s="4" t="n"/>
+      <c r="AE372" s="4" t="n"/>
+      <c r="AF372" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B373" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C373" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D373" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E373" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F373" s="6" t="n"/>
+      <c r="G373" s="6" t="n"/>
+      <c r="H373" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I373" s="6" t="inlineStr"/>
+      <c r="J373" s="6" t="inlineStr"/>
+      <c r="K373" s="6" t="inlineStr"/>
+      <c r="L373" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M373" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N373" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O373" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P373" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q373" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R373" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S373" s="6" t="n"/>
+      <c r="T373" s="6" t="n"/>
+      <c r="U373" s="6" t="n"/>
+      <c r="V373" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W373" s="6" t="inlineStr"/>
+      <c r="X373" s="6" t="n"/>
+      <c r="Y373" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z373" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA373" s="6" t="n"/>
+      <c r="AB373" s="6" t="n"/>
+      <c r="AC373" s="6" t="n"/>
+      <c r="AD373" s="6" t="n"/>
+      <c r="AE373" s="6" t="n"/>
+      <c r="AF373" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B374" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C374" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D374" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E374" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F374" s="4" t="n"/>
+      <c r="G374" s="4" t="n"/>
+      <c r="H374" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I374" s="4" t="inlineStr"/>
+      <c r="J374" s="4" t="inlineStr"/>
+      <c r="K374" s="4" t="inlineStr"/>
+      <c r="L374" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M374" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N374" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O374" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P374" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q374" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R374" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S374" s="4" t="n"/>
+      <c r="T374" s="4" t="n"/>
+      <c r="U374" s="4" t="n"/>
+      <c r="V374" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W374" s="4" t="inlineStr"/>
+      <c r="X374" s="4" t="n"/>
+      <c r="Y374" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z374" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA374" s="4" t="n"/>
+      <c r="AB374" s="4" t="n"/>
+      <c r="AC374" s="4" t="n"/>
+      <c r="AD374" s="4" t="n"/>
+      <c r="AE374" s="4" t="n"/>
+      <c r="AF374" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B375" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C375" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D375" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E375" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F375" s="6" t="n"/>
+      <c r="G375" s="6" t="n"/>
+      <c r="H375" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I375" s="6" t="inlineStr"/>
+      <c r="J375" s="6" t="inlineStr"/>
+      <c r="K375" s="6" t="inlineStr"/>
+      <c r="L375" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M375" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N375" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O375" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P375" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q375" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R375" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S375" s="6" t="n"/>
+      <c r="T375" s="6" t="n"/>
+      <c r="U375" s="6" t="n"/>
+      <c r="V375" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W375" s="6" t="inlineStr"/>
+      <c r="X375" s="6" t="n"/>
+      <c r="Y375" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z375" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA375" s="6" t="n"/>
+      <c r="AB375" s="6" t="n"/>
+      <c r="AC375" s="6" t="n"/>
+      <c r="AD375" s="6" t="n"/>
+      <c r="AE375" s="6" t="n"/>
+      <c r="AF375" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B376" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C376" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D376" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E376" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F376" s="4" t="n"/>
+      <c r="G376" s="4" t="n"/>
+      <c r="H376" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I376" s="4" t="inlineStr"/>
+      <c r="J376" s="4" t="inlineStr"/>
+      <c r="K376" s="4" t="inlineStr"/>
+      <c r="L376" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M376" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N376" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O376" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P376" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q376" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R376" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S376" s="4" t="n"/>
+      <c r="T376" s="4" t="n"/>
+      <c r="U376" s="4" t="n"/>
+      <c r="V376" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W376" s="4" t="inlineStr"/>
+      <c r="X376" s="4" t="n"/>
+      <c r="Y376" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z376" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA376" s="4" t="n"/>
+      <c r="AB376" s="4" t="n"/>
+      <c r="AC376" s="4" t="n"/>
+      <c r="AD376" s="4" t="n"/>
+      <c r="AE376" s="4" t="n"/>
+      <c r="AF376" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B377" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C377" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D377" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E377" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F377" s="6" t="n"/>
+      <c r="G377" s="6" t="n"/>
+      <c r="H377" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I377" s="6" t="inlineStr"/>
+      <c r="J377" s="6" t="inlineStr"/>
+      <c r="K377" s="6" t="inlineStr"/>
+      <c r="L377" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M377" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N377" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O377" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P377" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q377" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R377" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S377" s="6" t="n"/>
+      <c r="T377" s="6" t="n"/>
+      <c r="U377" s="6" t="n"/>
+      <c r="V377" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W377" s="6" t="inlineStr"/>
+      <c r="X377" s="6" t="n"/>
+      <c r="Y377" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z377" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA377" s="6" t="n"/>
+      <c r="AB377" s="6" t="n"/>
+      <c r="AC377" s="6" t="n"/>
+      <c r="AD377" s="6" t="n"/>
+      <c r="AE377" s="6" t="n"/>
+      <c r="AF377" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B378" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C378" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D378" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E378" s="4" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F378" s="4" t="n"/>
+      <c r="G378" s="4" t="n"/>
+      <c r="H378" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I378" s="4" t="inlineStr"/>
+      <c r="J378" s="4" t="inlineStr"/>
+      <c r="K378" s="4" t="inlineStr"/>
+      <c r="L378" s="4" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M378" s="4" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N378" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O378" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P378" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q378" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R378" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S378" s="4" t="n"/>
+      <c r="T378" s="4" t="n"/>
+      <c r="U378" s="4" t="n"/>
+      <c r="V378" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W378" s="4" t="inlineStr"/>
+      <c r="X378" s="4" t="n"/>
+      <c r="Y378" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z378" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA378" s="4" t="n"/>
+      <c r="AB378" s="4" t="n"/>
+      <c r="AC378" s="4" t="n"/>
+      <c r="AD378" s="4" t="n"/>
+      <c r="AE378" s="4" t="n"/>
+      <c r="AF378" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B379" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C379" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D379" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E379" s="6" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F379" s="6" t="n"/>
+      <c r="G379" s="6" t="n"/>
+      <c r="H379" s="6" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I379" s="6" t="inlineStr"/>
+      <c r="J379" s="6" t="inlineStr"/>
+      <c r="K379" s="6" t="inlineStr"/>
+      <c r="L379" s="6" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M379" s="6" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N379" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O379" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P379" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q379" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R379" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S379" s="6" t="n"/>
+      <c r="T379" s="6" t="n"/>
+      <c r="U379" s="6" t="n"/>
+      <c r="V379" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W379" s="6" t="inlineStr"/>
+      <c r="X379" s="6" t="n"/>
+      <c r="Y379" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z379" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA379" s="6" t="n"/>
+      <c r="AB379" s="6" t="n"/>
+      <c r="AC379" s="6" t="n"/>
+      <c r="AD379" s="6" t="n"/>
+      <c r="AE379" s="6" t="n"/>
+      <c r="AF379" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B380" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C380" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D380" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E380" s="4" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F380" s="4" t="n"/>
+      <c r="G380" s="4" t="n"/>
+      <c r="H380" s="4" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I380" s="4" t="inlineStr"/>
+      <c r="J380" s="4" t="inlineStr"/>
+      <c r="K380" s="4" t="inlineStr"/>
+      <c r="L380" s="4" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M380" s="4" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N380" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O380" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P380" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q380" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R380" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S380" s="4" t="n"/>
+      <c r="T380" s="4" t="n"/>
+      <c r="U380" s="4" t="n"/>
+      <c r="V380" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W380" s="4" t="inlineStr"/>
+      <c r="X380" s="4" t="n"/>
+      <c r="Y380" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z380" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA380" s="4" t="n"/>
+      <c r="AB380" s="4" t="n"/>
+      <c r="AC380" s="4" t="n"/>
+      <c r="AD380" s="4" t="n"/>
+      <c r="AE380" s="4" t="n"/>
+      <c r="AF380" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B381" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C381" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D381" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E381" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F381" s="6" t="n"/>
+      <c r="G381" s="6" t="n"/>
+      <c r="H381" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I381" s="6" t="inlineStr"/>
+      <c r="J381" s="6" t="inlineStr"/>
+      <c r="K381" s="6" t="inlineStr"/>
+      <c r="L381" s="6" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M381" s="6" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N381" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O381" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P381" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q381" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R381" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S381" s="6" t="n"/>
+      <c r="T381" s="6" t="n"/>
+      <c r="U381" s="6" t="n"/>
+      <c r="V381" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W381" s="6" t="inlineStr"/>
+      <c r="X381" s="6" t="n"/>
+      <c r="Y381" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z381" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA381" s="6" t="n"/>
+      <c r="AB381" s="6" t="n"/>
+      <c r="AC381" s="6" t="n"/>
+      <c r="AD381" s="6" t="n"/>
+      <c r="AE381" s="6" t="n"/>
+      <c r="AF381" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B382" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C382" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D382" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E382" s="4" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F382" s="4" t="n"/>
+      <c r="G382" s="4" t="n"/>
+      <c r="H382" s="4" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I382" s="4" t="inlineStr"/>
+      <c r="J382" s="4" t="inlineStr"/>
+      <c r="K382" s="4" t="inlineStr"/>
+      <c r="L382" s="4" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M382" s="4" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N382" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O382" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P382" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q382" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R382" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S382" s="4" t="n"/>
+      <c r="T382" s="4" t="n"/>
+      <c r="U382" s="4" t="n"/>
+      <c r="V382" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W382" s="4" t="inlineStr"/>
+      <c r="X382" s="4" t="n"/>
+      <c r="Y382" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z382" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA382" s="4" t="n"/>
+      <c r="AB382" s="4" t="n"/>
+      <c r="AC382" s="4" t="n"/>
+      <c r="AD382" s="4" t="n"/>
+      <c r="AE382" s="4" t="n"/>
+      <c r="AF382" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B383" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C383" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D383" s="6" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E383" s="6" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F383" s="6" t="n"/>
+      <c r="G383" s="6" t="n"/>
+      <c r="H383" s="6" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I383" s="6" t="inlineStr"/>
+      <c r="J383" s="6" t="inlineStr"/>
+      <c r="K383" s="6" t="inlineStr"/>
+      <c r="L383" s="6" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="M383" s="6" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="N383" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O383" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P383" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q383" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R383" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S383" s="6" t="n"/>
+      <c r="T383" s="6" t="n"/>
+      <c r="U383" s="6" t="n"/>
+      <c r="V383" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W383" s="6" t="inlineStr"/>
+      <c r="X383" s="6" t="n"/>
+      <c r="Y383" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z383" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA383" s="6" t="n"/>
+      <c r="AB383" s="6" t="n"/>
+      <c r="AC383" s="6" t="n"/>
+      <c r="AD383" s="6" t="n"/>
+      <c r="AE383" s="6" t="n"/>
+      <c r="AF383" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B384" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C384" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D384" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E384" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F384" s="4" t="n"/>
+      <c r="G384" s="4" t="n"/>
+      <c r="H384" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I384" s="4" t="inlineStr"/>
+      <c r="J384" s="4" t="inlineStr"/>
+      <c r="K384" s="4" t="inlineStr"/>
+      <c r="L384" s="4" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M384" s="4" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N384" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O384" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P384" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q384" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R384" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S384" s="4" t="n"/>
+      <c r="T384" s="4" t="n"/>
+      <c r="U384" s="4" t="n"/>
+      <c r="V384" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W384" s="4" t="inlineStr"/>
+      <c r="X384" s="4" t="n"/>
+      <c r="Y384" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z384" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA384" s="4" t="n"/>
+      <c r="AB384" s="4" t="n"/>
+      <c r="AC384" s="4" t="n"/>
+      <c r="AD384" s="4" t="n"/>
+      <c r="AE384" s="4" t="n"/>
+      <c r="AF384" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B385" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C385" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D385" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E385" s="6" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F385" s="6" t="n"/>
+      <c r="G385" s="6" t="n"/>
+      <c r="H385" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I385" s="6" t="inlineStr"/>
+      <c r="J385" s="6" t="inlineStr"/>
+      <c r="K385" s="6" t="inlineStr"/>
+      <c r="L385" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M385" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N385" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O385" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P385" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q385" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R385" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S385" s="6" t="n"/>
+      <c r="T385" s="6" t="n"/>
+      <c r="U385" s="6" t="n"/>
+      <c r="V385" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W385" s="6" t="inlineStr"/>
+      <c r="X385" s="6" t="n"/>
+      <c r="Y385" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z385" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA385" s="6" t="n"/>
+      <c r="AB385" s="6" t="n"/>
+      <c r="AC385" s="6" t="n"/>
+      <c r="AD385" s="6" t="n"/>
+      <c r="AE385" s="6" t="n"/>
+      <c r="AF385" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B386" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C386" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D386" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E386" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F386" s="4" t="n"/>
+      <c r="G386" s="4" t="n"/>
+      <c r="H386" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I386" s="4" t="inlineStr"/>
+      <c r="J386" s="4" t="inlineStr"/>
+      <c r="K386" s="4" t="inlineStr"/>
+      <c r="L386" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M386" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N386" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O386" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P386" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q386" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R386" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S386" s="4" t="n"/>
+      <c r="T386" s="4" t="n"/>
+      <c r="U386" s="4" t="n"/>
+      <c r="V386" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W386" s="4" t="inlineStr"/>
+      <c r="X386" s="4" t="n"/>
+      <c r="Y386" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z386" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA386" s="4" t="n"/>
+      <c r="AB386" s="4" t="n"/>
+      <c r="AC386" s="4" t="n"/>
+      <c r="AD386" s="4" t="n"/>
+      <c r="AE386" s="4" t="n"/>
+      <c r="AF386" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B387" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C387" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D387" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E387" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F387" s="6" t="n"/>
+      <c r="G387" s="6" t="n"/>
+      <c r="H387" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I387" s="6" t="inlineStr"/>
+      <c r="J387" s="6" t="inlineStr"/>
+      <c r="K387" s="6" t="inlineStr"/>
+      <c r="L387" s="6" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M387" s="6" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N387" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O387" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P387" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q387" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R387" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S387" s="6" t="n"/>
+      <c r="T387" s="6" t="n"/>
+      <c r="U387" s="6" t="n"/>
+      <c r="V387" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W387" s="6" t="inlineStr"/>
+      <c r="X387" s="6" t="n"/>
+      <c r="Y387" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z387" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA387" s="6" t="n"/>
+      <c r="AB387" s="6" t="n"/>
+      <c r="AC387" s="6" t="n"/>
+      <c r="AD387" s="6" t="n"/>
+      <c r="AE387" s="6" t="n"/>
+      <c r="AF387" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B388" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C388" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D388" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E388" s="4" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F388" s="4" t="n"/>
+      <c r="G388" s="4" t="n"/>
+      <c r="H388" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I388" s="4" t="inlineStr"/>
+      <c r="J388" s="4" t="inlineStr"/>
+      <c r="K388" s="4" t="inlineStr"/>
+      <c r="L388" s="4" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M388" s="4" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N388" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O388" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P388" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q388" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R388" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S388" s="4" t="n"/>
+      <c r="T388" s="4" t="n"/>
+      <c r="U388" s="4" t="n"/>
+      <c r="V388" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W388" s="4" t="inlineStr"/>
+      <c r="X388" s="4" t="n"/>
+      <c r="Y388" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z388" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA388" s="4" t="n"/>
+      <c r="AB388" s="4" t="n"/>
+      <c r="AC388" s="4" t="n"/>
+      <c r="AD388" s="4" t="n"/>
+      <c r="AE388" s="4" t="n"/>
+      <c r="AF388" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B389" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C389" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D389" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E389" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F389" s="6" t="n"/>
+      <c r="G389" s="6" t="n"/>
+      <c r="H389" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="I389" s="6" t="inlineStr"/>
+      <c r="J389" s="6" t="inlineStr"/>
+      <c r="K389" s="6" t="inlineStr"/>
+      <c r="L389" s="6" t="n"/>
+      <c r="M389" s="6" t="n"/>
+      <c r="N389" s="6" t="n"/>
+      <c r="O389" s="6" t="n"/>
+      <c r="P389" s="6" t="n"/>
+      <c r="Q389" s="6" t="n"/>
+      <c r="R389" s="6" t="n"/>
+      <c r="S389" s="6" t="n"/>
+      <c r="T389" s="6" t="n"/>
+      <c r="U389" s="6" t="n"/>
+      <c r="V389" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W389" s="6" t="inlineStr"/>
+      <c r="X389" s="6" t="n"/>
+      <c r="Y389" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z389" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA389" s="6" t="n"/>
+      <c r="AB389" s="6" t="n"/>
+      <c r="AC389" s="6" t="n"/>
+      <c r="AD389" s="6" t="n"/>
+      <c r="AE389" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="AF389" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B390" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C390" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D390" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E390" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F390" s="4" t="n"/>
+      <c r="G390" s="4" t="n"/>
+      <c r="H390" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I390" s="4" t="inlineStr"/>
+      <c r="J390" s="4" t="inlineStr"/>
+      <c r="K390" s="4" t="inlineStr"/>
+      <c r="L390" s="4" t="n"/>
+      <c r="M390" s="4" t="n"/>
+      <c r="N390" s="4" t="n"/>
+      <c r="O390" s="4" t="n"/>
+      <c r="P390" s="4" t="n"/>
+      <c r="Q390" s="4" t="n"/>
+      <c r="R390" s="4" t="n"/>
+      <c r="S390" s="4" t="n"/>
+      <c r="T390" s="4" t="n"/>
+      <c r="U390" s="4" t="n"/>
+      <c r="V390" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W390" s="4" t="inlineStr"/>
+      <c r="X390" s="4" t="n"/>
+      <c r="Y390" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z390" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA390" s="4" t="n"/>
+      <c r="AB390" s="4" t="n"/>
+      <c r="AC390" s="4" t="n"/>
+      <c r="AD390" s="4" t="n"/>
+      <c r="AE390" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF390" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B391" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C391" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D391" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E391" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F391" s="6" t="n"/>
+      <c r="G391" s="6" t="n"/>
+      <c r="H391" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I391" s="6" t="inlineStr"/>
+      <c r="J391" s="6" t="inlineStr"/>
+      <c r="K391" s="6" t="inlineStr"/>
+      <c r="L391" s="6" t="n"/>
+      <c r="M391" s="6" t="n"/>
+      <c r="N391" s="6" t="n"/>
+      <c r="O391" s="6" t="n"/>
+      <c r="P391" s="6" t="n"/>
+      <c r="Q391" s="6" t="n"/>
+      <c r="R391" s="6" t="n"/>
+      <c r="S391" s="6" t="n"/>
+      <c r="T391" s="6" t="n"/>
+      <c r="U391" s="6" t="n"/>
+      <c r="V391" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W391" s="6" t="inlineStr"/>
+      <c r="X391" s="6" t="n"/>
+      <c r="Y391" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z391" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA391" s="6" t="n"/>
+      <c r="AB391" s="6" t="n"/>
+      <c r="AC391" s="6" t="n"/>
+      <c r="AD391" s="6" t="n"/>
+      <c r="AE391" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="AF391" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B392" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C392" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D392" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E392" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F392" s="4" t="n"/>
+      <c r="G392" s="4" t="n"/>
+      <c r="H392" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="I392" s="4" t="inlineStr"/>
+      <c r="J392" s="4" t="inlineStr"/>
+      <c r="K392" s="4" t="inlineStr"/>
+      <c r="L392" s="4" t="n"/>
+      <c r="M392" s="4" t="n"/>
+      <c r="N392" s="4" t="n"/>
+      <c r="O392" s="4" t="n"/>
+      <c r="P392" s="4" t="n"/>
+      <c r="Q392" s="4" t="n"/>
+      <c r="R392" s="4" t="n"/>
+      <c r="S392" s="4" t="n"/>
+      <c r="T392" s="4" t="n"/>
+      <c r="U392" s="4" t="n"/>
+      <c r="V392" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W392" s="4" t="inlineStr"/>
+      <c r="X392" s="4" t="n"/>
+      <c r="Y392" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z392" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA392" s="4" t="n"/>
+      <c r="AB392" s="4" t="n"/>
+      <c r="AC392" s="4" t="n"/>
+      <c r="AD392" s="4" t="n"/>
+      <c r="AE392" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="AF392" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B393" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C393" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D393" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E393" s="6" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F393" s="6" t="n"/>
+      <c r="G393" s="6" t="n"/>
+      <c r="H393" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I393" s="6" t="inlineStr"/>
+      <c r="J393" s="6" t="inlineStr"/>
+      <c r="K393" s="6" t="inlineStr"/>
+      <c r="L393" s="6" t="n"/>
+      <c r="M393" s="6" t="n"/>
+      <c r="N393" s="6" t="n"/>
+      <c r="O393" s="6" t="n"/>
+      <c r="P393" s="6" t="n"/>
+      <c r="Q393" s="6" t="n"/>
+      <c r="R393" s="6" t="n"/>
+      <c r="S393" s="6" t="n"/>
+      <c r="T393" s="6" t="n"/>
+      <c r="U393" s="6" t="n"/>
+      <c r="V393" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W393" s="6" t="inlineStr"/>
+      <c r="X393" s="6" t="n"/>
+      <c r="Y393" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z393" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA393" s="6" t="n"/>
+      <c r="AB393" s="6" t="n"/>
+      <c r="AC393" s="6" t="n"/>
+      <c r="AD393" s="6" t="n"/>
+      <c r="AE393" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF393" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B394" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C394" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D394" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E394" s="4" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F394" s="4" t="n"/>
+      <c r="G394" s="4" t="n"/>
+      <c r="H394" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I394" s="4" t="inlineStr"/>
+      <c r="J394" s="4" t="inlineStr"/>
+      <c r="K394" s="4" t="inlineStr"/>
+      <c r="L394" s="4" t="n"/>
+      <c r="M394" s="4" t="n"/>
+      <c r="N394" s="4" t="n"/>
+      <c r="O394" s="4" t="n"/>
+      <c r="P394" s="4" t="n"/>
+      <c r="Q394" s="4" t="n"/>
+      <c r="R394" s="4" t="n"/>
+      <c r="S394" s="4" t="n"/>
+      <c r="T394" s="4" t="n"/>
+      <c r="U394" s="4" t="n"/>
+      <c r="V394" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W394" s="4" t="inlineStr"/>
+      <c r="X394" s="4" t="n"/>
+      <c r="Y394" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z394" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA394" s="4" t="n"/>
+      <c r="AB394" s="4" t="n"/>
+      <c r="AC394" s="4" t="n"/>
+      <c r="AD394" s="4" t="n"/>
+      <c r="AE394" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF394" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B395" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C395" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D395" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E395" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F395" s="6" t="n"/>
+      <c r="G395" s="6" t="n"/>
+      <c r="H395" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I395" s="6" t="inlineStr"/>
+      <c r="J395" s="6" t="inlineStr"/>
+      <c r="K395" s="6" t="inlineStr"/>
+      <c r="L395" s="6" t="n"/>
+      <c r="M395" s="6" t="n"/>
+      <c r="N395" s="6" t="n"/>
+      <c r="O395" s="6" t="n"/>
+      <c r="P395" s="6" t="n"/>
+      <c r="Q395" s="6" t="n"/>
+      <c r="R395" s="6" t="n"/>
+      <c r="S395" s="6" t="n"/>
+      <c r="T395" s="6" t="n"/>
+      <c r="U395" s="6" t="n"/>
+      <c r="V395" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W395" s="6" t="inlineStr"/>
+      <c r="X395" s="6" t="n"/>
+      <c r="Y395" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z395" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA395" s="6" t="n"/>
+      <c r="AB395" s="6" t="n"/>
+      <c r="AC395" s="6" t="n"/>
+      <c r="AD395" s="6" t="n"/>
+      <c r="AE395" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF395" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B396" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C396" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D396" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E396" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F396" s="4" t="n"/>
+      <c r="G396" s="4" t="n"/>
+      <c r="H396" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I396" s="4" t="inlineStr"/>
+      <c r="J396" s="4" t="inlineStr"/>
+      <c r="K396" s="4" t="inlineStr"/>
+      <c r="L396" s="4" t="n"/>
+      <c r="M396" s="4" t="n"/>
+      <c r="N396" s="4" t="n"/>
+      <c r="O396" s="4" t="n"/>
+      <c r="P396" s="4" t="n"/>
+      <c r="Q396" s="4" t="n"/>
+      <c r="R396" s="4" t="n"/>
+      <c r="S396" s="4" t="n"/>
+      <c r="T396" s="4" t="n"/>
+      <c r="U396" s="4" t="n"/>
+      <c r="V396" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W396" s="4" t="inlineStr"/>
+      <c r="X396" s="4" t="n"/>
+      <c r="Y396" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z396" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA396" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB396" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC396" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD396" s="4" t="n"/>
+      <c r="AE396" s="4" t="n"/>
+      <c r="AF396" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B397" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C397" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D397" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E397" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F397" s="6" t="n"/>
+      <c r="G397" s="6" t="n"/>
+      <c r="H397" s="6" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I397" s="6" t="inlineStr"/>
+      <c r="J397" s="6" t="inlineStr"/>
+      <c r="K397" s="6" t="inlineStr"/>
+      <c r="L397" s="6" t="n"/>
+      <c r="M397" s="6" t="n"/>
+      <c r="N397" s="6" t="n"/>
+      <c r="O397" s="6" t="n"/>
+      <c r="P397" s="6" t="n"/>
+      <c r="Q397" s="6" t="n"/>
+      <c r="R397" s="6" t="n"/>
+      <c r="S397" s="6" t="n"/>
+      <c r="T397" s="6" t="n"/>
+      <c r="U397" s="6" t="n"/>
+      <c r="V397" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W397" s="6" t="inlineStr"/>
+      <c r="X397" s="6" t="n"/>
+      <c r="Y397" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z397" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA397" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB397" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC397" s="6" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD397" s="6" t="n"/>
+      <c r="AE397" s="6" t="n"/>
+      <c r="AF397" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B398" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C398" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D398" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E398" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F398" s="4" t="n"/>
+      <c r="G398" s="4" t="n"/>
+      <c r="H398" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I398" s="4" t="inlineStr"/>
+      <c r="J398" s="4" t="inlineStr"/>
+      <c r="K398" s="4" t="inlineStr"/>
+      <c r="L398" s="4" t="n"/>
+      <c r="M398" s="4" t="n"/>
+      <c r="N398" s="4" t="n"/>
+      <c r="O398" s="4" t="n"/>
+      <c r="P398" s="4" t="n"/>
+      <c r="Q398" s="4" t="n"/>
+      <c r="R398" s="4" t="n"/>
+      <c r="S398" s="4" t="n"/>
+      <c r="T398" s="4" t="n"/>
+      <c r="U398" s="4" t="n"/>
+      <c r="V398" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W398" s="4" t="inlineStr"/>
+      <c r="X398" s="4" t="n"/>
+      <c r="Y398" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z398" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA398" s="4" t="n"/>
+      <c r="AB398" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC398" s="4" t="n"/>
+      <c r="AD398" s="4" t="n"/>
+      <c r="AE398" s="4" t="n"/>
+      <c r="AF398" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="B399" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C399" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D399" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E399" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F399" s="6" t="n"/>
+      <c r="G399" s="6" t="n"/>
+      <c r="H399" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I399" s="6" t="inlineStr"/>
+      <c r="J399" s="6" t="inlineStr"/>
+      <c r="K399" s="6" t="inlineStr"/>
+      <c r="L399" s="6" t="n"/>
+      <c r="M399" s="6" t="n"/>
+      <c r="N399" s="6" t="n"/>
+      <c r="O399" s="6" t="n"/>
+      <c r="P399" s="6" t="n"/>
+      <c r="Q399" s="6" t="n"/>
+      <c r="R399" s="6" t="n"/>
+      <c r="S399" s="6" t="n"/>
+      <c r="T399" s="6" t="n"/>
+      <c r="U399" s="6" t="n"/>
+      <c r="V399" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W399" s="6" t="inlineStr"/>
+      <c r="X399" s="6" t="n"/>
+      <c r="Y399" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z399" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA399" s="6" t="n"/>
+      <c r="AB399" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC399" s="6" t="n"/>
+      <c r="AD399" s="6" t="n"/>
+      <c r="AE399" s="6" t="n"/>
+      <c r="AF399" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-06-30
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF399"/>
+  <dimension ref="A1:AF435"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -31960,6 +31960,2836 @@
         <v>1</v>
       </c>
     </row>
+    <row r="400">
+      <c r="A400" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B400" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C400" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D400" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E400" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F400" s="4" t="n"/>
+      <c r="G400" s="4" t="n"/>
+      <c r="H400" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I400" s="4" t="inlineStr"/>
+      <c r="J400" s="4" t="inlineStr"/>
+      <c r="K400" s="4" t="inlineStr"/>
+      <c r="L400" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M400" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N400" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O400" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P400" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q400" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R400" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S400" s="4" t="n"/>
+      <c r="T400" s="4" t="n"/>
+      <c r="U400" s="4" t="n"/>
+      <c r="V400" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W400" s="4" t="inlineStr"/>
+      <c r="X400" s="4" t="n"/>
+      <c r="Y400" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z400" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA400" s="4" t="n"/>
+      <c r="AB400" s="4" t="n"/>
+      <c r="AC400" s="4" t="n"/>
+      <c r="AD400" s="4" t="n"/>
+      <c r="AE400" s="4" t="n"/>
+      <c r="AF400" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B401" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C401" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D401" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E401" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F401" s="6" t="n"/>
+      <c r="G401" s="6" t="n"/>
+      <c r="H401" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I401" s="6" t="inlineStr"/>
+      <c r="J401" s="6" t="inlineStr"/>
+      <c r="K401" s="6" t="inlineStr"/>
+      <c r="L401" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M401" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N401" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O401" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P401" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q401" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R401" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S401" s="6" t="n"/>
+      <c r="T401" s="6" t="n"/>
+      <c r="U401" s="6" t="n"/>
+      <c r="V401" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W401" s="6" t="inlineStr"/>
+      <c r="X401" s="6" t="n"/>
+      <c r="Y401" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z401" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA401" s="6" t="n"/>
+      <c r="AB401" s="6" t="n"/>
+      <c r="AC401" s="6" t="n"/>
+      <c r="AD401" s="6" t="n"/>
+      <c r="AE401" s="6" t="n"/>
+      <c r="AF401" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B402" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C402" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D402" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E402" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F402" s="4" t="n"/>
+      <c r="G402" s="4" t="n"/>
+      <c r="H402" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I402" s="4" t="inlineStr"/>
+      <c r="J402" s="4" t="inlineStr"/>
+      <c r="K402" s="4" t="inlineStr"/>
+      <c r="L402" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M402" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N402" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O402" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P402" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q402" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R402" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S402" s="4" t="n"/>
+      <c r="T402" s="4" t="n"/>
+      <c r="U402" s="4" t="n"/>
+      <c r="V402" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W402" s="4" t="inlineStr"/>
+      <c r="X402" s="4" t="n"/>
+      <c r="Y402" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z402" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA402" s="4" t="n"/>
+      <c r="AB402" s="4" t="n"/>
+      <c r="AC402" s="4" t="n"/>
+      <c r="AD402" s="4" t="n"/>
+      <c r="AE402" s="4" t="n"/>
+      <c r="AF402" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B403" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C403" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D403" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E403" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F403" s="6" t="n"/>
+      <c r="G403" s="6" t="n"/>
+      <c r="H403" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I403" s="6" t="inlineStr"/>
+      <c r="J403" s="6" t="inlineStr"/>
+      <c r="K403" s="6" t="inlineStr"/>
+      <c r="L403" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M403" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N403" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O403" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P403" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q403" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R403" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S403" s="6" t="n"/>
+      <c r="T403" s="6" t="n"/>
+      <c r="U403" s="6" t="n"/>
+      <c r="V403" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W403" s="6" t="inlineStr"/>
+      <c r="X403" s="6" t="n"/>
+      <c r="Y403" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z403" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA403" s="6" t="n"/>
+      <c r="AB403" s="6" t="n"/>
+      <c r="AC403" s="6" t="n"/>
+      <c r="AD403" s="6" t="n"/>
+      <c r="AE403" s="6" t="n"/>
+      <c r="AF403" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B404" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C404" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D404" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E404" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F404" s="4" t="n"/>
+      <c r="G404" s="4" t="n"/>
+      <c r="H404" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I404" s="4" t="inlineStr"/>
+      <c r="J404" s="4" t="inlineStr"/>
+      <c r="K404" s="4" t="inlineStr"/>
+      <c r="L404" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M404" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N404" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O404" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P404" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q404" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R404" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S404" s="4" t="n"/>
+      <c r="T404" s="4" t="n"/>
+      <c r="U404" s="4" t="n"/>
+      <c r="V404" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W404" s="4" t="inlineStr"/>
+      <c r="X404" s="4" t="n"/>
+      <c r="Y404" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z404" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA404" s="4" t="n"/>
+      <c r="AB404" s="4" t="n"/>
+      <c r="AC404" s="4" t="n"/>
+      <c r="AD404" s="4" t="n"/>
+      <c r="AE404" s="4" t="n"/>
+      <c r="AF404" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B405" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C405" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D405" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E405" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F405" s="6" t="n"/>
+      <c r="G405" s="6" t="n"/>
+      <c r="H405" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I405" s="6" t="inlineStr"/>
+      <c r="J405" s="6" t="inlineStr"/>
+      <c r="K405" s="6" t="inlineStr"/>
+      <c r="L405" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M405" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N405" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O405" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P405" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q405" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R405" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S405" s="6" t="n"/>
+      <c r="T405" s="6" t="n"/>
+      <c r="U405" s="6" t="n"/>
+      <c r="V405" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W405" s="6" t="inlineStr"/>
+      <c r="X405" s="6" t="n"/>
+      <c r="Y405" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z405" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA405" s="6" t="n"/>
+      <c r="AB405" s="6" t="n"/>
+      <c r="AC405" s="6" t="n"/>
+      <c r="AD405" s="6" t="n"/>
+      <c r="AE405" s="6" t="n"/>
+      <c r="AF405" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B406" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C406" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D406" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E406" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F406" s="4" t="n"/>
+      <c r="G406" s="4" t="n"/>
+      <c r="H406" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I406" s="4" t="inlineStr"/>
+      <c r="J406" s="4" t="inlineStr"/>
+      <c r="K406" s="4" t="inlineStr"/>
+      <c r="L406" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M406" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N406" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O406" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P406" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q406" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R406" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S406" s="4" t="n"/>
+      <c r="T406" s="4" t="n"/>
+      <c r="U406" s="4" t="n"/>
+      <c r="V406" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W406" s="4" t="inlineStr"/>
+      <c r="X406" s="4" t="n"/>
+      <c r="Y406" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z406" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA406" s="4" t="n"/>
+      <c r="AB406" s="4" t="n"/>
+      <c r="AC406" s="4" t="n"/>
+      <c r="AD406" s="4" t="n"/>
+      <c r="AE406" s="4" t="n"/>
+      <c r="AF406" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B407" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C407" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D407" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E407" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F407" s="6" t="n"/>
+      <c r="G407" s="6" t="n"/>
+      <c r="H407" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I407" s="6" t="inlineStr"/>
+      <c r="J407" s="6" t="inlineStr"/>
+      <c r="K407" s="6" t="inlineStr"/>
+      <c r="L407" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M407" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N407" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O407" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P407" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q407" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R407" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S407" s="6" t="n"/>
+      <c r="T407" s="6" t="n"/>
+      <c r="U407" s="6" t="n"/>
+      <c r="V407" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W407" s="6" t="inlineStr"/>
+      <c r="X407" s="6" t="n"/>
+      <c r="Y407" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z407" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA407" s="6" t="n"/>
+      <c r="AB407" s="6" t="n"/>
+      <c r="AC407" s="6" t="n"/>
+      <c r="AD407" s="6" t="n"/>
+      <c r="AE407" s="6" t="n"/>
+      <c r="AF407" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B408" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C408" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D408" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E408" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F408" s="4" t="n"/>
+      <c r="G408" s="4" t="n"/>
+      <c r="H408" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I408" s="4" t="inlineStr"/>
+      <c r="J408" s="4" t="inlineStr"/>
+      <c r="K408" s="4" t="inlineStr"/>
+      <c r="L408" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M408" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N408" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O408" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P408" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q408" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R408" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S408" s="4" t="n"/>
+      <c r="T408" s="4" t="n"/>
+      <c r="U408" s="4" t="n"/>
+      <c r="V408" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W408" s="4" t="inlineStr"/>
+      <c r="X408" s="4" t="n"/>
+      <c r="Y408" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z408" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA408" s="4" t="n"/>
+      <c r="AB408" s="4" t="n"/>
+      <c r="AC408" s="4" t="n"/>
+      <c r="AD408" s="4" t="n"/>
+      <c r="AE408" s="4" t="n"/>
+      <c r="AF408" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B409" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C409" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D409" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E409" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F409" s="6" t="n"/>
+      <c r="G409" s="6" t="n"/>
+      <c r="H409" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I409" s="6" t="inlineStr"/>
+      <c r="J409" s="6" t="inlineStr"/>
+      <c r="K409" s="6" t="inlineStr"/>
+      <c r="L409" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M409" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N409" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O409" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P409" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q409" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R409" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S409" s="6" t="n"/>
+      <c r="T409" s="6" t="n"/>
+      <c r="U409" s="6" t="n"/>
+      <c r="V409" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W409" s="6" t="inlineStr"/>
+      <c r="X409" s="6" t="n"/>
+      <c r="Y409" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z409" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA409" s="6" t="n"/>
+      <c r="AB409" s="6" t="n"/>
+      <c r="AC409" s="6" t="n"/>
+      <c r="AD409" s="6" t="n"/>
+      <c r="AE409" s="6" t="n"/>
+      <c r="AF409" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B410" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C410" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D410" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E410" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F410" s="4" t="n"/>
+      <c r="G410" s="4" t="n"/>
+      <c r="H410" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I410" s="4" t="inlineStr"/>
+      <c r="J410" s="4" t="inlineStr"/>
+      <c r="K410" s="4" t="inlineStr"/>
+      <c r="L410" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M410" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N410" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O410" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P410" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q410" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R410" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S410" s="4" t="n"/>
+      <c r="T410" s="4" t="n"/>
+      <c r="U410" s="4" t="n"/>
+      <c r="V410" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W410" s="4" t="inlineStr"/>
+      <c r="X410" s="4" t="n"/>
+      <c r="Y410" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z410" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA410" s="4" t="n"/>
+      <c r="AB410" s="4" t="n"/>
+      <c r="AC410" s="4" t="n"/>
+      <c r="AD410" s="4" t="n"/>
+      <c r="AE410" s="4" t="n"/>
+      <c r="AF410" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B411" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C411" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D411" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E411" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F411" s="6" t="n"/>
+      <c r="G411" s="6" t="n"/>
+      <c r="H411" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I411" s="6" t="inlineStr"/>
+      <c r="J411" s="6" t="inlineStr"/>
+      <c r="K411" s="6" t="inlineStr"/>
+      <c r="L411" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M411" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N411" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O411" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P411" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q411" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R411" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S411" s="6" t="n"/>
+      <c r="T411" s="6" t="n"/>
+      <c r="U411" s="6" t="n"/>
+      <c r="V411" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W411" s="6" t="inlineStr"/>
+      <c r="X411" s="6" t="n"/>
+      <c r="Y411" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z411" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA411" s="6" t="n"/>
+      <c r="AB411" s="6" t="n"/>
+      <c r="AC411" s="6" t="n"/>
+      <c r="AD411" s="6" t="n"/>
+      <c r="AE411" s="6" t="n"/>
+      <c r="AF411" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B412" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C412" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D412" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E412" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F412" s="4" t="n"/>
+      <c r="G412" s="4" t="n"/>
+      <c r="H412" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I412" s="4" t="inlineStr"/>
+      <c r="J412" s="4" t="inlineStr"/>
+      <c r="K412" s="4" t="inlineStr"/>
+      <c r="L412" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M412" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N412" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O412" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P412" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q412" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R412" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S412" s="4" t="n"/>
+      <c r="T412" s="4" t="n"/>
+      <c r="U412" s="4" t="n"/>
+      <c r="V412" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W412" s="4" t="inlineStr"/>
+      <c r="X412" s="4" t="n"/>
+      <c r="Y412" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z412" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA412" s="4" t="n"/>
+      <c r="AB412" s="4" t="n"/>
+      <c r="AC412" s="4" t="n"/>
+      <c r="AD412" s="4" t="n"/>
+      <c r="AE412" s="4" t="n"/>
+      <c r="AF412" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B413" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C413" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D413" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E413" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F413" s="6" t="n"/>
+      <c r="G413" s="6" t="n"/>
+      <c r="H413" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I413" s="6" t="inlineStr"/>
+      <c r="J413" s="6" t="inlineStr"/>
+      <c r="K413" s="6" t="inlineStr"/>
+      <c r="L413" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M413" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N413" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O413" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P413" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q413" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R413" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S413" s="6" t="n"/>
+      <c r="T413" s="6" t="n"/>
+      <c r="U413" s="6" t="n"/>
+      <c r="V413" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W413" s="6" t="inlineStr"/>
+      <c r="X413" s="6" t="n"/>
+      <c r="Y413" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z413" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA413" s="6" t="n"/>
+      <c r="AB413" s="6" t="n"/>
+      <c r="AC413" s="6" t="n"/>
+      <c r="AD413" s="6" t="n"/>
+      <c r="AE413" s="6" t="n"/>
+      <c r="AF413" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B414" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C414" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D414" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E414" s="4" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F414" s="4" t="n"/>
+      <c r="G414" s="4" t="n"/>
+      <c r="H414" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I414" s="4" t="inlineStr"/>
+      <c r="J414" s="4" t="inlineStr"/>
+      <c r="K414" s="4" t="inlineStr"/>
+      <c r="L414" s="4" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M414" s="4" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N414" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O414" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P414" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q414" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R414" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S414" s="4" t="n"/>
+      <c r="T414" s="4" t="n"/>
+      <c r="U414" s="4" t="n"/>
+      <c r="V414" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W414" s="4" t="inlineStr"/>
+      <c r="X414" s="4" t="n"/>
+      <c r="Y414" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z414" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA414" s="4" t="n"/>
+      <c r="AB414" s="4" t="n"/>
+      <c r="AC414" s="4" t="n"/>
+      <c r="AD414" s="4" t="n"/>
+      <c r="AE414" s="4" t="n"/>
+      <c r="AF414" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B415" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C415" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D415" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E415" s="6" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F415" s="6" t="n"/>
+      <c r="G415" s="6" t="n"/>
+      <c r="H415" s="6" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I415" s="6" t="inlineStr"/>
+      <c r="J415" s="6" t="inlineStr"/>
+      <c r="K415" s="6" t="inlineStr"/>
+      <c r="L415" s="6" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M415" s="6" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N415" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O415" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P415" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q415" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R415" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S415" s="6" t="n"/>
+      <c r="T415" s="6" t="n"/>
+      <c r="U415" s="6" t="n"/>
+      <c r="V415" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W415" s="6" t="inlineStr"/>
+      <c r="X415" s="6" t="n"/>
+      <c r="Y415" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z415" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA415" s="6" t="n"/>
+      <c r="AB415" s="6" t="n"/>
+      <c r="AC415" s="6" t="n"/>
+      <c r="AD415" s="6" t="n"/>
+      <c r="AE415" s="6" t="n"/>
+      <c r="AF415" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B416" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C416" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D416" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E416" s="4" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F416" s="4" t="n"/>
+      <c r="G416" s="4" t="n"/>
+      <c r="H416" s="4" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I416" s="4" t="inlineStr"/>
+      <c r="J416" s="4" t="inlineStr"/>
+      <c r="K416" s="4" t="inlineStr"/>
+      <c r="L416" s="4" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M416" s="4" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N416" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O416" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P416" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q416" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R416" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S416" s="4" t="n"/>
+      <c r="T416" s="4" t="n"/>
+      <c r="U416" s="4" t="n"/>
+      <c r="V416" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W416" s="4" t="inlineStr"/>
+      <c r="X416" s="4" t="n"/>
+      <c r="Y416" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z416" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA416" s="4" t="n"/>
+      <c r="AB416" s="4" t="n"/>
+      <c r="AC416" s="4" t="n"/>
+      <c r="AD416" s="4" t="n"/>
+      <c r="AE416" s="4" t="n"/>
+      <c r="AF416" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B417" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C417" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D417" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E417" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F417" s="6" t="n"/>
+      <c r="G417" s="6" t="n"/>
+      <c r="H417" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I417" s="6" t="inlineStr"/>
+      <c r="J417" s="6" t="inlineStr"/>
+      <c r="K417" s="6" t="inlineStr"/>
+      <c r="L417" s="6" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M417" s="6" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N417" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O417" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P417" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q417" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R417" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S417" s="6" t="n"/>
+      <c r="T417" s="6" t="n"/>
+      <c r="U417" s="6" t="n"/>
+      <c r="V417" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W417" s="6" t="inlineStr"/>
+      <c r="X417" s="6" t="n"/>
+      <c r="Y417" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z417" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA417" s="6" t="n"/>
+      <c r="AB417" s="6" t="n"/>
+      <c r="AC417" s="6" t="n"/>
+      <c r="AD417" s="6" t="n"/>
+      <c r="AE417" s="6" t="n"/>
+      <c r="AF417" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B418" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C418" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D418" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E418" s="4" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F418" s="4" t="n"/>
+      <c r="G418" s="4" t="n"/>
+      <c r="H418" s="4" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I418" s="4" t="inlineStr"/>
+      <c r="J418" s="4" t="inlineStr"/>
+      <c r="K418" s="4" t="inlineStr"/>
+      <c r="L418" s="4" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M418" s="4" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N418" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O418" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P418" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q418" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R418" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S418" s="4" t="n"/>
+      <c r="T418" s="4" t="n"/>
+      <c r="U418" s="4" t="n"/>
+      <c r="V418" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W418" s="4" t="inlineStr"/>
+      <c r="X418" s="4" t="n"/>
+      <c r="Y418" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z418" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA418" s="4" t="n"/>
+      <c r="AB418" s="4" t="n"/>
+      <c r="AC418" s="4" t="n"/>
+      <c r="AD418" s="4" t="n"/>
+      <c r="AE418" s="4" t="n"/>
+      <c r="AF418" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B419" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C419" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D419" s="6" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E419" s="6" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F419" s="6" t="n"/>
+      <c r="G419" s="6" t="n"/>
+      <c r="H419" s="6" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I419" s="6" t="inlineStr"/>
+      <c r="J419" s="6" t="inlineStr"/>
+      <c r="K419" s="6" t="inlineStr"/>
+      <c r="L419" s="6" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="M419" s="6" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="N419" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O419" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P419" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q419" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R419" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S419" s="6" t="n"/>
+      <c r="T419" s="6" t="n"/>
+      <c r="U419" s="6" t="n"/>
+      <c r="V419" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W419" s="6" t="inlineStr"/>
+      <c r="X419" s="6" t="n"/>
+      <c r="Y419" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z419" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA419" s="6" t="n"/>
+      <c r="AB419" s="6" t="n"/>
+      <c r="AC419" s="6" t="n"/>
+      <c r="AD419" s="6" t="n"/>
+      <c r="AE419" s="6" t="n"/>
+      <c r="AF419" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B420" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C420" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D420" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E420" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F420" s="4" t="n"/>
+      <c r="G420" s="4" t="n"/>
+      <c r="H420" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I420" s="4" t="inlineStr"/>
+      <c r="J420" s="4" t="inlineStr"/>
+      <c r="K420" s="4" t="inlineStr"/>
+      <c r="L420" s="4" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M420" s="4" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N420" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O420" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P420" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q420" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R420" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S420" s="4" t="n"/>
+      <c r="T420" s="4" t="n"/>
+      <c r="U420" s="4" t="n"/>
+      <c r="V420" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W420" s="4" t="inlineStr"/>
+      <c r="X420" s="4" t="n"/>
+      <c r="Y420" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z420" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA420" s="4" t="n"/>
+      <c r="AB420" s="4" t="n"/>
+      <c r="AC420" s="4" t="n"/>
+      <c r="AD420" s="4" t="n"/>
+      <c r="AE420" s="4" t="n"/>
+      <c r="AF420" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B421" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C421" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D421" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E421" s="6" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F421" s="6" t="n"/>
+      <c r="G421" s="6" t="n"/>
+      <c r="H421" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I421" s="6" t="inlineStr"/>
+      <c r="J421" s="6" t="inlineStr"/>
+      <c r="K421" s="6" t="inlineStr"/>
+      <c r="L421" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M421" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N421" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O421" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P421" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q421" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R421" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S421" s="6" t="n"/>
+      <c r="T421" s="6" t="n"/>
+      <c r="U421" s="6" t="n"/>
+      <c r="V421" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W421" s="6" t="inlineStr"/>
+      <c r="X421" s="6" t="n"/>
+      <c r="Y421" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z421" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA421" s="6" t="n"/>
+      <c r="AB421" s="6" t="n"/>
+      <c r="AC421" s="6" t="n"/>
+      <c r="AD421" s="6" t="n"/>
+      <c r="AE421" s="6" t="n"/>
+      <c r="AF421" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B422" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C422" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D422" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E422" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F422" s="4" t="n"/>
+      <c r="G422" s="4" t="n"/>
+      <c r="H422" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I422" s="4" t="inlineStr"/>
+      <c r="J422" s="4" t="inlineStr"/>
+      <c r="K422" s="4" t="inlineStr"/>
+      <c r="L422" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M422" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N422" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O422" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P422" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q422" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R422" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S422" s="4" t="n"/>
+      <c r="T422" s="4" t="n"/>
+      <c r="U422" s="4" t="n"/>
+      <c r="V422" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W422" s="4" t="inlineStr"/>
+      <c r="X422" s="4" t="n"/>
+      <c r="Y422" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z422" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA422" s="4" t="n"/>
+      <c r="AB422" s="4" t="n"/>
+      <c r="AC422" s="4" t="n"/>
+      <c r="AD422" s="4" t="n"/>
+      <c r="AE422" s="4" t="n"/>
+      <c r="AF422" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B423" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C423" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D423" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E423" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F423" s="6" t="n"/>
+      <c r="G423" s="6" t="n"/>
+      <c r="H423" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I423" s="6" t="inlineStr"/>
+      <c r="J423" s="6" t="inlineStr"/>
+      <c r="K423" s="6" t="inlineStr"/>
+      <c r="L423" s="6" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M423" s="6" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N423" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O423" s="6" t="n">
+        <v>357</v>
+      </c>
+      <c r="P423" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q423" s="6" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R423" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S423" s="6" t="n"/>
+      <c r="T423" s="6" t="n"/>
+      <c r="U423" s="6" t="n"/>
+      <c r="V423" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W423" s="6" t="inlineStr"/>
+      <c r="X423" s="6" t="n"/>
+      <c r="Y423" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z423" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA423" s="6" t="n"/>
+      <c r="AB423" s="6" t="n"/>
+      <c r="AC423" s="6" t="n"/>
+      <c r="AD423" s="6" t="n"/>
+      <c r="AE423" s="6" t="n"/>
+      <c r="AF423" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B424" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C424" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D424" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E424" s="4" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F424" s="4" t="n"/>
+      <c r="G424" s="4" t="n"/>
+      <c r="H424" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I424" s="4" t="inlineStr"/>
+      <c r="J424" s="4" t="inlineStr"/>
+      <c r="K424" s="4" t="inlineStr"/>
+      <c r="L424" s="4" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M424" s="4" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N424" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O424" s="4" t="n">
+        <v>357</v>
+      </c>
+      <c r="P424" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="Q424" s="4" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="R424" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S424" s="4" t="n"/>
+      <c r="T424" s="4" t="n"/>
+      <c r="U424" s="4" t="n"/>
+      <c r="V424" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (74 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (7 %), Poudre de cacao maigre,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (à base d'huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Arôme, Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme® (0,1 %) (Alpha-amylase, Protéase, Lactase, Cellulase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W424" s="4" t="inlineStr"/>
+      <c r="X424" s="4" t="n"/>
+      <c r="Y424" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z424" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA424" s="4" t="n"/>
+      <c r="AB424" s="4" t="n"/>
+      <c r="AC424" s="4" t="n"/>
+      <c r="AD424" s="4" t="n"/>
+      <c r="AE424" s="4" t="n"/>
+      <c r="AF424" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B425" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C425" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D425" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E425" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="F425" s="6" t="n"/>
+      <c r="G425" s="6" t="n"/>
+      <c r="H425" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="I425" s="6" t="inlineStr"/>
+      <c r="J425" s="6" t="inlineStr"/>
+      <c r="K425" s="6" t="inlineStr"/>
+      <c r="L425" s="6" t="n"/>
+      <c r="M425" s="6" t="n"/>
+      <c r="N425" s="6" t="n"/>
+      <c r="O425" s="6" t="n"/>
+      <c r="P425" s="6" t="n"/>
+      <c r="Q425" s="6" t="n"/>
+      <c r="R425" s="6" t="n"/>
+      <c r="S425" s="6" t="n"/>
+      <c r="T425" s="6" t="n"/>
+      <c r="U425" s="6" t="n"/>
+      <c r="V425" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W425" s="6" t="inlineStr"/>
+      <c r="X425" s="6" t="n"/>
+      <c r="Y425" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z425" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA425" s="6" t="n"/>
+      <c r="AB425" s="6" t="n"/>
+      <c r="AC425" s="6" t="n"/>
+      <c r="AD425" s="6" t="n"/>
+      <c r="AE425" s="6" t="n">
+        <v>40</v>
+      </c>
+      <c r="AF425" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B426" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C426" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D426" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E426" s="4" t="n">
+        <v>7.5</v>
+      </c>
+      <c r="F426" s="4" t="n"/>
+      <c r="G426" s="4" t="n"/>
+      <c r="H426" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I426" s="4" t="inlineStr"/>
+      <c r="J426" s="4" t="inlineStr"/>
+      <c r="K426" s="4" t="inlineStr"/>
+      <c r="L426" s="4" t="n"/>
+      <c r="M426" s="4" t="n"/>
+      <c r="N426" s="4" t="n"/>
+      <c r="O426" s="4" t="n"/>
+      <c r="P426" s="4" t="n"/>
+      <c r="Q426" s="4" t="n"/>
+      <c r="R426" s="4" t="n"/>
+      <c r="S426" s="4" t="n"/>
+      <c r="T426" s="4" t="n"/>
+      <c r="U426" s="4" t="n"/>
+      <c r="V426" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W426" s="4" t="inlineStr"/>
+      <c r="X426" s="4" t="n"/>
+      <c r="Y426" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z426" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA426" s="4" t="n"/>
+      <c r="AB426" s="4" t="n"/>
+      <c r="AC426" s="4" t="n"/>
+      <c r="AD426" s="4" t="n"/>
+      <c r="AE426" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="AF426" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B427" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C427" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D427" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E427" s="6" t="n">
+        <v>12.5</v>
+      </c>
+      <c r="F427" s="6" t="n"/>
+      <c r="G427" s="6" t="n"/>
+      <c r="H427" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="I427" s="6" t="inlineStr"/>
+      <c r="J427" s="6" t="inlineStr"/>
+      <c r="K427" s="6" t="inlineStr"/>
+      <c r="L427" s="6" t="n"/>
+      <c r="M427" s="6" t="n"/>
+      <c r="N427" s="6" t="n"/>
+      <c r="O427" s="6" t="n"/>
+      <c r="P427" s="6" t="n"/>
+      <c r="Q427" s="6" t="n"/>
+      <c r="R427" s="6" t="n"/>
+      <c r="S427" s="6" t="n"/>
+      <c r="T427" s="6" t="n"/>
+      <c r="U427" s="6" t="n"/>
+      <c r="V427" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W427" s="6" t="inlineStr"/>
+      <c r="X427" s="6" t="n"/>
+      <c r="Y427" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z427" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA427" s="6" t="n"/>
+      <c r="AB427" s="6" t="n"/>
+      <c r="AC427" s="6" t="n"/>
+      <c r="AD427" s="6" t="n"/>
+      <c r="AE427" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="AF427" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B428" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C428" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D428" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E428" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F428" s="4" t="n"/>
+      <c r="G428" s="4" t="n"/>
+      <c r="H428" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="I428" s="4" t="inlineStr"/>
+      <c r="J428" s="4" t="inlineStr"/>
+      <c r="K428" s="4" t="inlineStr"/>
+      <c r="L428" s="4" t="n"/>
+      <c r="M428" s="4" t="n"/>
+      <c r="N428" s="4" t="n"/>
+      <c r="O428" s="4" t="n"/>
+      <c r="P428" s="4" t="n"/>
+      <c r="Q428" s="4" t="n"/>
+      <c r="R428" s="4" t="n"/>
+      <c r="S428" s="4" t="n"/>
+      <c r="T428" s="4" t="n"/>
+      <c r="U428" s="4" t="n"/>
+      <c r="V428" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W428" s="4" t="inlineStr"/>
+      <c r="X428" s="4" t="n"/>
+      <c r="Y428" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z428" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA428" s="4" t="n"/>
+      <c r="AB428" s="4" t="n"/>
+      <c r="AC428" s="4" t="n"/>
+      <c r="AD428" s="4" t="n"/>
+      <c r="AE428" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="AF428" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B429" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C429" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D429" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E429" s="6" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F429" s="6" t="n"/>
+      <c r="G429" s="6" t="n"/>
+      <c r="H429" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I429" s="6" t="inlineStr"/>
+      <c r="J429" s="6" t="inlineStr"/>
+      <c r="K429" s="6" t="inlineStr"/>
+      <c r="L429" s="6" t="n"/>
+      <c r="M429" s="6" t="n"/>
+      <c r="N429" s="6" t="n"/>
+      <c r="O429" s="6" t="n"/>
+      <c r="P429" s="6" t="n"/>
+      <c r="Q429" s="6" t="n"/>
+      <c r="R429" s="6" t="n"/>
+      <c r="S429" s="6" t="n"/>
+      <c r="T429" s="6" t="n"/>
+      <c r="U429" s="6" t="n"/>
+      <c r="V429" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W429" s="6" t="inlineStr"/>
+      <c r="X429" s="6" t="n"/>
+      <c r="Y429" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z429" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA429" s="6" t="n"/>
+      <c r="AB429" s="6" t="n"/>
+      <c r="AC429" s="6" t="n"/>
+      <c r="AD429" s="6" t="n"/>
+      <c r="AE429" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF429" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B430" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C430" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D430" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E430" s="4" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F430" s="4" t="n"/>
+      <c r="G430" s="4" t="n"/>
+      <c r="H430" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I430" s="4" t="inlineStr"/>
+      <c r="J430" s="4" t="inlineStr"/>
+      <c r="K430" s="4" t="inlineStr"/>
+      <c r="L430" s="4" t="n"/>
+      <c r="M430" s="4" t="n"/>
+      <c r="N430" s="4" t="n"/>
+      <c r="O430" s="4" t="n"/>
+      <c r="P430" s="4" t="n"/>
+      <c r="Q430" s="4" t="n"/>
+      <c r="R430" s="4" t="n"/>
+      <c r="S430" s="4" t="n"/>
+      <c r="T430" s="4" t="n"/>
+      <c r="U430" s="4" t="n"/>
+      <c r="V430" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W430" s="4" t="inlineStr"/>
+      <c r="X430" s="4" t="n"/>
+      <c r="Y430" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z430" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA430" s="4" t="n"/>
+      <c r="AB430" s="4" t="n"/>
+      <c r="AC430" s="4" t="n"/>
+      <c r="AD430" s="4" t="n"/>
+      <c r="AE430" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF430" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B431" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C431" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D431" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E431" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F431" s="6" t="n"/>
+      <c r="G431" s="6" t="n"/>
+      <c r="H431" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I431" s="6" t="inlineStr"/>
+      <c r="J431" s="6" t="inlineStr"/>
+      <c r="K431" s="6" t="inlineStr"/>
+      <c r="L431" s="6" t="n"/>
+      <c r="M431" s="6" t="n"/>
+      <c r="N431" s="6" t="n"/>
+      <c r="O431" s="6" t="n"/>
+      <c r="P431" s="6" t="n"/>
+      <c r="Q431" s="6" t="n"/>
+      <c r="R431" s="6" t="n"/>
+      <c r="S431" s="6" t="n"/>
+      <c r="T431" s="6" t="n"/>
+      <c r="U431" s="6" t="n"/>
+      <c r="V431" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W431" s="6" t="inlineStr"/>
+      <c r="X431" s="6" t="n"/>
+      <c r="Y431" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z431" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA431" s="6" t="n"/>
+      <c r="AB431" s="6" t="n"/>
+      <c r="AC431" s="6" t="n"/>
+      <c r="AD431" s="6" t="n"/>
+      <c r="AE431" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF431" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B432" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C432" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D432" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E432" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F432" s="4" t="n"/>
+      <c r="G432" s="4" t="n"/>
+      <c r="H432" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I432" s="4" t="inlineStr"/>
+      <c r="J432" s="4" t="inlineStr"/>
+      <c r="K432" s="4" t="inlineStr"/>
+      <c r="L432" s="4" t="n"/>
+      <c r="M432" s="4" t="n"/>
+      <c r="N432" s="4" t="n"/>
+      <c r="O432" s="4" t="n"/>
+      <c r="P432" s="4" t="n"/>
+      <c r="Q432" s="4" t="n"/>
+      <c r="R432" s="4" t="n"/>
+      <c r="S432" s="4" t="n"/>
+      <c r="T432" s="4" t="n"/>
+      <c r="U432" s="4" t="n"/>
+      <c r="V432" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W432" s="4" t="inlineStr"/>
+      <c r="X432" s="4" t="n"/>
+      <c r="Y432" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z432" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA432" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB432" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC432" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD432" s="4" t="n"/>
+      <c r="AE432" s="4" t="n"/>
+      <c r="AF432" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B433" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C433" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D433" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E433" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F433" s="6" t="n"/>
+      <c r="G433" s="6" t="n"/>
+      <c r="H433" s="6" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I433" s="6" t="inlineStr"/>
+      <c r="J433" s="6" t="inlineStr"/>
+      <c r="K433" s="6" t="inlineStr"/>
+      <c r="L433" s="6" t="n"/>
+      <c r="M433" s="6" t="n"/>
+      <c r="N433" s="6" t="n"/>
+      <c r="O433" s="6" t="n"/>
+      <c r="P433" s="6" t="n"/>
+      <c r="Q433" s="6" t="n"/>
+      <c r="R433" s="6" t="n"/>
+      <c r="S433" s="6" t="n"/>
+      <c r="T433" s="6" t="n"/>
+      <c r="U433" s="6" t="n"/>
+      <c r="V433" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W433" s="6" t="inlineStr"/>
+      <c r="X433" s="6" t="n"/>
+      <c r="Y433" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z433" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA433" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB433" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC433" s="6" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD433" s="6" t="n"/>
+      <c r="AE433" s="6" t="n"/>
+      <c r="AF433" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B434" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C434" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D434" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E434" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F434" s="4" t="n"/>
+      <c r="G434" s="4" t="n"/>
+      <c r="H434" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I434" s="4" t="inlineStr"/>
+      <c r="J434" s="4" t="inlineStr"/>
+      <c r="K434" s="4" t="inlineStr"/>
+      <c r="L434" s="4" t="n"/>
+      <c r="M434" s="4" t="n"/>
+      <c r="N434" s="4" t="n"/>
+      <c r="O434" s="4" t="n"/>
+      <c r="P434" s="4" t="n"/>
+      <c r="Q434" s="4" t="n"/>
+      <c r="R434" s="4" t="n"/>
+      <c r="S434" s="4" t="n"/>
+      <c r="T434" s="4" t="n"/>
+      <c r="U434" s="4" t="n"/>
+      <c r="V434" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W434" s="4" t="inlineStr"/>
+      <c r="X434" s="4" t="n"/>
+      <c r="Y434" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z434" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA434" s="4" t="n"/>
+      <c r="AB434" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC434" s="4" t="n"/>
+      <c r="AD434" s="4" t="n"/>
+      <c r="AE434" s="4" t="n"/>
+      <c r="AF434" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" s="2" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B435" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C435" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D435" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E435" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F435" s="6" t="n"/>
+      <c r="G435" s="6" t="n"/>
+      <c r="H435" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I435" s="6" t="inlineStr"/>
+      <c r="J435" s="6" t="inlineStr"/>
+      <c r="K435" s="6" t="inlineStr"/>
+      <c r="L435" s="6" t="n"/>
+      <c r="M435" s="6" t="n"/>
+      <c r="N435" s="6" t="n"/>
+      <c r="O435" s="6" t="n"/>
+      <c r="P435" s="6" t="n"/>
+      <c r="Q435" s="6" t="n"/>
+      <c r="R435" s="6" t="n"/>
+      <c r="S435" s="6" t="n"/>
+      <c r="T435" s="6" t="n"/>
+      <c r="U435" s="6" t="n"/>
+      <c r="V435" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W435" s="6" t="inlineStr"/>
+      <c r="X435" s="6" t="n"/>
+      <c r="Y435" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z435" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA435" s="6" t="n"/>
+      <c r="AB435" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC435" s="6" t="n"/>
+      <c r="AD435" s="6" t="n"/>
+      <c r="AE435" s="6" t="n"/>
+      <c r="AF435" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-01
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF435"/>
+  <dimension ref="A1:AF471"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -34790,6 +34790,2840 @@
         <v>1</v>
       </c>
     </row>
+    <row r="436">
+      <c r="A436" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B436" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C436" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D436" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E436" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F436" s="4" t="n"/>
+      <c r="G436" s="4" t="n"/>
+      <c r="H436" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I436" s="4" t="inlineStr"/>
+      <c r="J436" s="4" t="inlineStr"/>
+      <c r="K436" s="4" t="inlineStr"/>
+      <c r="L436" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M436" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N436" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O436" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P436" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q436" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R436" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S436" s="4" t="n"/>
+      <c r="T436" s="4" t="n"/>
+      <c r="U436" s="4" t="n"/>
+      <c r="V436" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W436" s="4" t="inlineStr"/>
+      <c r="X436" s="4" t="n"/>
+      <c r="Y436" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z436" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA436" s="4" t="n"/>
+      <c r="AB436" s="4" t="n"/>
+      <c r="AC436" s="4" t="n"/>
+      <c r="AD436" s="4" t="n"/>
+      <c r="AE436" s="4" t="n"/>
+      <c r="AF436" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B437" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C437" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D437" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E437" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F437" s="6" t="n"/>
+      <c r="G437" s="6" t="n"/>
+      <c r="H437" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I437" s="6" t="inlineStr"/>
+      <c r="J437" s="6" t="inlineStr"/>
+      <c r="K437" s="6" t="inlineStr"/>
+      <c r="L437" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M437" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N437" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O437" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P437" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q437" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R437" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S437" s="6" t="n"/>
+      <c r="T437" s="6" t="n"/>
+      <c r="U437" s="6" t="n"/>
+      <c r="V437" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W437" s="6" t="inlineStr"/>
+      <c r="X437" s="6" t="n"/>
+      <c r="Y437" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z437" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA437" s="6" t="n"/>
+      <c r="AB437" s="6" t="n"/>
+      <c r="AC437" s="6" t="n"/>
+      <c r="AD437" s="6" t="n"/>
+      <c r="AE437" s="6" t="n"/>
+      <c r="AF437" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B438" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C438" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D438" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E438" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F438" s="4" t="n"/>
+      <c r="G438" s="4" t="n"/>
+      <c r="H438" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I438" s="4" t="inlineStr"/>
+      <c r="J438" s="4" t="inlineStr"/>
+      <c r="K438" s="4" t="inlineStr"/>
+      <c r="L438" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M438" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N438" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O438" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P438" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q438" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R438" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S438" s="4" t="n"/>
+      <c r="T438" s="4" t="n"/>
+      <c r="U438" s="4" t="n"/>
+      <c r="V438" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W438" s="4" t="inlineStr"/>
+      <c r="X438" s="4" t="n"/>
+      <c r="Y438" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z438" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA438" s="4" t="n"/>
+      <c r="AB438" s="4" t="n"/>
+      <c r="AC438" s="4" t="n"/>
+      <c r="AD438" s="4" t="n"/>
+      <c r="AE438" s="4" t="n"/>
+      <c r="AF438" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B439" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C439" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D439" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E439" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F439" s="6" t="n"/>
+      <c r="G439" s="6" t="n"/>
+      <c r="H439" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I439" s="6" t="inlineStr"/>
+      <c r="J439" s="6" t="inlineStr"/>
+      <c r="K439" s="6" t="inlineStr"/>
+      <c r="L439" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M439" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N439" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O439" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P439" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q439" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R439" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S439" s="6" t="n"/>
+      <c r="T439" s="6" t="n"/>
+      <c r="U439" s="6" t="n"/>
+      <c r="V439" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W439" s="6" t="inlineStr"/>
+      <c r="X439" s="6" t="n"/>
+      <c r="Y439" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z439" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA439" s="6" t="n"/>
+      <c r="AB439" s="6" t="n"/>
+      <c r="AC439" s="6" t="n"/>
+      <c r="AD439" s="6" t="n"/>
+      <c r="AE439" s="6" t="n"/>
+      <c r="AF439" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B440" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C440" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D440" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E440" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F440" s="4" t="n"/>
+      <c r="G440" s="4" t="n"/>
+      <c r="H440" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I440" s="4" t="inlineStr"/>
+      <c r="J440" s="4" t="inlineStr"/>
+      <c r="K440" s="4" t="inlineStr"/>
+      <c r="L440" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M440" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N440" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O440" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P440" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q440" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R440" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S440" s="4" t="n"/>
+      <c r="T440" s="4" t="n"/>
+      <c r="U440" s="4" t="n"/>
+      <c r="V440" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W440" s="4" t="inlineStr"/>
+      <c r="X440" s="4" t="n"/>
+      <c r="Y440" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z440" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA440" s="4" t="n"/>
+      <c r="AB440" s="4" t="n"/>
+      <c r="AC440" s="4" t="n"/>
+      <c r="AD440" s="4" t="n"/>
+      <c r="AE440" s="4" t="n"/>
+      <c r="AF440" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B441" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C441" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D441" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E441" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F441" s="6" t="n"/>
+      <c r="G441" s="6" t="n"/>
+      <c r="H441" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I441" s="6" t="inlineStr"/>
+      <c r="J441" s="6" t="inlineStr"/>
+      <c r="K441" s="6" t="inlineStr"/>
+      <c r="L441" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M441" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N441" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O441" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P441" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q441" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R441" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S441" s="6" t="n"/>
+      <c r="T441" s="6" t="n"/>
+      <c r="U441" s="6" t="n"/>
+      <c r="V441" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W441" s="6" t="inlineStr"/>
+      <c r="X441" s="6" t="n"/>
+      <c r="Y441" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z441" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA441" s="6" t="n"/>
+      <c r="AB441" s="6" t="n"/>
+      <c r="AC441" s="6" t="n"/>
+      <c r="AD441" s="6" t="n"/>
+      <c r="AE441" s="6" t="n"/>
+      <c r="AF441" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B442" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C442" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D442" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E442" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F442" s="4" t="n"/>
+      <c r="G442" s="4" t="n"/>
+      <c r="H442" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I442" s="4" t="inlineStr"/>
+      <c r="J442" s="4" t="inlineStr"/>
+      <c r="K442" s="4" t="inlineStr"/>
+      <c r="L442" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M442" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N442" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O442" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P442" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q442" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R442" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S442" s="4" t="n"/>
+      <c r="T442" s="4" t="n"/>
+      <c r="U442" s="4" t="n"/>
+      <c r="V442" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W442" s="4" t="inlineStr"/>
+      <c r="X442" s="4" t="n"/>
+      <c r="Y442" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z442" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA442" s="4" t="n"/>
+      <c r="AB442" s="4" t="n"/>
+      <c r="AC442" s="4" t="n"/>
+      <c r="AD442" s="4" t="n"/>
+      <c r="AE442" s="4" t="n"/>
+      <c r="AF442" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B443" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C443" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D443" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E443" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F443" s="6" t="n"/>
+      <c r="G443" s="6" t="n"/>
+      <c r="H443" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I443" s="6" t="inlineStr"/>
+      <c r="J443" s="6" t="inlineStr"/>
+      <c r="K443" s="6" t="inlineStr"/>
+      <c r="L443" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M443" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N443" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O443" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P443" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q443" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R443" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S443" s="6" t="n"/>
+      <c r="T443" s="6" t="n"/>
+      <c r="U443" s="6" t="n"/>
+      <c r="V443" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W443" s="6" t="inlineStr"/>
+      <c r="X443" s="6" t="n"/>
+      <c r="Y443" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z443" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA443" s="6" t="n"/>
+      <c r="AB443" s="6" t="n"/>
+      <c r="AC443" s="6" t="n"/>
+      <c r="AD443" s="6" t="n"/>
+      <c r="AE443" s="6" t="n"/>
+      <c r="AF443" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B444" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C444" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D444" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E444" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F444" s="4" t="n"/>
+      <c r="G444" s="4" t="n"/>
+      <c r="H444" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I444" s="4" t="inlineStr"/>
+      <c r="J444" s="4" t="inlineStr"/>
+      <c r="K444" s="4" t="inlineStr"/>
+      <c r="L444" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M444" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N444" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O444" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P444" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q444" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R444" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S444" s="4" t="n"/>
+      <c r="T444" s="4" t="n"/>
+      <c r="U444" s="4" t="n"/>
+      <c r="V444" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W444" s="4" t="inlineStr"/>
+      <c r="X444" s="4" t="n"/>
+      <c r="Y444" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z444" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA444" s="4" t="n"/>
+      <c r="AB444" s="4" t="n"/>
+      <c r="AC444" s="4" t="n"/>
+      <c r="AD444" s="4" t="n"/>
+      <c r="AE444" s="4" t="n"/>
+      <c r="AF444" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B445" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C445" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D445" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E445" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F445" s="6" t="n"/>
+      <c r="G445" s="6" t="n"/>
+      <c r="H445" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I445" s="6" t="inlineStr"/>
+      <c r="J445" s="6" t="inlineStr"/>
+      <c r="K445" s="6" t="inlineStr"/>
+      <c r="L445" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M445" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N445" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O445" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P445" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q445" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R445" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S445" s="6" t="n"/>
+      <c r="T445" s="6" t="n"/>
+      <c r="U445" s="6" t="n"/>
+      <c r="V445" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W445" s="6" t="inlineStr"/>
+      <c r="X445" s="6" t="n"/>
+      <c r="Y445" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z445" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA445" s="6" t="n"/>
+      <c r="AB445" s="6" t="n"/>
+      <c r="AC445" s="6" t="n"/>
+      <c r="AD445" s="6" t="n"/>
+      <c r="AE445" s="6" t="n"/>
+      <c r="AF445" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B446" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C446" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D446" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E446" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F446" s="4" t="n"/>
+      <c r="G446" s="4" t="n"/>
+      <c r="H446" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I446" s="4" t="inlineStr"/>
+      <c r="J446" s="4" t="inlineStr"/>
+      <c r="K446" s="4" t="inlineStr"/>
+      <c r="L446" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M446" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N446" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O446" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P446" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q446" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R446" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S446" s="4" t="n"/>
+      <c r="T446" s="4" t="n"/>
+      <c r="U446" s="4" t="n"/>
+      <c r="V446" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W446" s="4" t="inlineStr"/>
+      <c r="X446" s="4" t="n"/>
+      <c r="Y446" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z446" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA446" s="4" t="n"/>
+      <c r="AB446" s="4" t="n"/>
+      <c r="AC446" s="4" t="n"/>
+      <c r="AD446" s="4" t="n"/>
+      <c r="AE446" s="4" t="n"/>
+      <c r="AF446" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B447" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C447" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D447" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E447" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F447" s="6" t="n"/>
+      <c r="G447" s="6" t="n"/>
+      <c r="H447" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I447" s="6" t="inlineStr"/>
+      <c r="J447" s="6" t="inlineStr"/>
+      <c r="K447" s="6" t="inlineStr"/>
+      <c r="L447" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M447" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N447" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O447" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P447" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q447" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R447" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S447" s="6" t="n"/>
+      <c r="T447" s="6" t="n"/>
+      <c r="U447" s="6" t="n"/>
+      <c r="V447" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W447" s="6" t="inlineStr"/>
+      <c r="X447" s="6" t="n"/>
+      <c r="Y447" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z447" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA447" s="6" t="n"/>
+      <c r="AB447" s="6" t="n"/>
+      <c r="AC447" s="6" t="n"/>
+      <c r="AD447" s="6" t="n"/>
+      <c r="AE447" s="6" t="n"/>
+      <c r="AF447" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B448" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C448" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D448" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E448" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F448" s="4" t="n"/>
+      <c r="G448" s="4" t="n"/>
+      <c r="H448" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I448" s="4" t="inlineStr"/>
+      <c r="J448" s="4" t="inlineStr"/>
+      <c r="K448" s="4" t="inlineStr"/>
+      <c r="L448" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M448" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N448" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O448" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P448" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q448" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R448" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S448" s="4" t="n"/>
+      <c r="T448" s="4" t="n"/>
+      <c r="U448" s="4" t="n"/>
+      <c r="V448" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W448" s="4" t="inlineStr"/>
+      <c r="X448" s="4" t="n"/>
+      <c r="Y448" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z448" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA448" s="4" t="n"/>
+      <c r="AB448" s="4" t="n"/>
+      <c r="AC448" s="4" t="n"/>
+      <c r="AD448" s="4" t="n"/>
+      <c r="AE448" s="4" t="n"/>
+      <c r="AF448" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B449" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C449" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D449" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E449" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F449" s="6" t="n"/>
+      <c r="G449" s="6" t="n"/>
+      <c r="H449" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I449" s="6" t="inlineStr"/>
+      <c r="J449" s="6" t="inlineStr"/>
+      <c r="K449" s="6" t="inlineStr"/>
+      <c r="L449" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M449" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N449" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O449" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P449" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q449" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R449" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S449" s="6" t="n"/>
+      <c r="T449" s="6" t="n"/>
+      <c r="U449" s="6" t="n"/>
+      <c r="V449" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W449" s="6" t="inlineStr"/>
+      <c r="X449" s="6" t="n"/>
+      <c r="Y449" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z449" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA449" s="6" t="n"/>
+      <c r="AB449" s="6" t="n"/>
+      <c r="AC449" s="6" t="n"/>
+      <c r="AD449" s="6" t="n"/>
+      <c r="AE449" s="6" t="n"/>
+      <c r="AF449" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C450" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D450" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E450" s="4" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F450" s="4" t="n"/>
+      <c r="G450" s="4" t="n"/>
+      <c r="H450" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I450" s="4" t="inlineStr"/>
+      <c r="J450" s="4" t="inlineStr"/>
+      <c r="K450" s="4" t="inlineStr"/>
+      <c r="L450" s="4" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M450" s="4" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N450" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O450" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P450" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q450" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R450" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S450" s="4" t="n"/>
+      <c r="T450" s="4" t="n"/>
+      <c r="U450" s="4" t="n"/>
+      <c r="V450" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W450" s="4" t="inlineStr"/>
+      <c r="X450" s="4" t="n"/>
+      <c r="Y450" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z450" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA450" s="4" t="n"/>
+      <c r="AB450" s="4" t="n"/>
+      <c r="AC450" s="4" t="n"/>
+      <c r="AD450" s="4" t="n"/>
+      <c r="AE450" s="4" t="n"/>
+      <c r="AF450" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B451" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C451" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D451" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E451" s="6" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F451" s="6" t="n"/>
+      <c r="G451" s="6" t="n"/>
+      <c r="H451" s="6" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I451" s="6" t="inlineStr"/>
+      <c r="J451" s="6" t="inlineStr"/>
+      <c r="K451" s="6" t="inlineStr"/>
+      <c r="L451" s="6" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M451" s="6" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N451" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O451" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P451" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q451" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R451" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S451" s="6" t="n"/>
+      <c r="T451" s="6" t="n"/>
+      <c r="U451" s="6" t="n"/>
+      <c r="V451" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W451" s="6" t="inlineStr"/>
+      <c r="X451" s="6" t="n"/>
+      <c r="Y451" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z451" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA451" s="6" t="n"/>
+      <c r="AB451" s="6" t="n"/>
+      <c r="AC451" s="6" t="n"/>
+      <c r="AD451" s="6" t="n"/>
+      <c r="AE451" s="6" t="n"/>
+      <c r="AF451" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B452" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C452" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D452" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E452" s="4" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F452" s="4" t="n"/>
+      <c r="G452" s="4" t="n"/>
+      <c r="H452" s="4" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I452" s="4" t="inlineStr"/>
+      <c r="J452" s="4" t="inlineStr"/>
+      <c r="K452" s="4" t="inlineStr"/>
+      <c r="L452" s="4" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M452" s="4" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N452" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O452" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P452" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q452" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R452" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S452" s="4" t="n"/>
+      <c r="T452" s="4" t="n"/>
+      <c r="U452" s="4" t="n"/>
+      <c r="V452" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W452" s="4" t="inlineStr"/>
+      <c r="X452" s="4" t="n"/>
+      <c r="Y452" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z452" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA452" s="4" t="n"/>
+      <c r="AB452" s="4" t="n"/>
+      <c r="AC452" s="4" t="n"/>
+      <c r="AD452" s="4" t="n"/>
+      <c r="AE452" s="4" t="n"/>
+      <c r="AF452" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B453" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C453" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D453" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E453" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F453" s="6" t="n"/>
+      <c r="G453" s="6" t="n"/>
+      <c r="H453" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I453" s="6" t="inlineStr"/>
+      <c r="J453" s="6" t="inlineStr"/>
+      <c r="K453" s="6" t="inlineStr"/>
+      <c r="L453" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="M453" s="6" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N453" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O453" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P453" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q453" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R453" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S453" s="6" t="n"/>
+      <c r="T453" s="6" t="n"/>
+      <c r="U453" s="6" t="n"/>
+      <c r="V453" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W453" s="6" t="inlineStr"/>
+      <c r="X453" s="6" t="n"/>
+      <c r="Y453" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z453" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA453" s="6" t="n"/>
+      <c r="AB453" s="6" t="n"/>
+      <c r="AC453" s="6" t="n"/>
+      <c r="AD453" s="6" t="n"/>
+      <c r="AE453" s="6" t="n"/>
+      <c r="AF453" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B454" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C454" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D454" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E454" s="4" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F454" s="4" t="n"/>
+      <c r="G454" s="4" t="n"/>
+      <c r="H454" s="4" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I454" s="4" t="inlineStr"/>
+      <c r="J454" s="4" t="inlineStr"/>
+      <c r="K454" s="4" t="inlineStr"/>
+      <c r="L454" s="4" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M454" s="4" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N454" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O454" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P454" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q454" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R454" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S454" s="4" t="n"/>
+      <c r="T454" s="4" t="n"/>
+      <c r="U454" s="4" t="n"/>
+      <c r="V454" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W454" s="4" t="inlineStr"/>
+      <c r="X454" s="4" t="n"/>
+      <c r="Y454" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z454" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA454" s="4" t="n"/>
+      <c r="AB454" s="4" t="n"/>
+      <c r="AC454" s="4" t="n"/>
+      <c r="AD454" s="4" t="n"/>
+      <c r="AE454" s="4" t="n"/>
+      <c r="AF454" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B455" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C455" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D455" s="6" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E455" s="6" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F455" s="6" t="n"/>
+      <c r="G455" s="6" t="n"/>
+      <c r="H455" s="6" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I455" s="6" t="inlineStr"/>
+      <c r="J455" s="6" t="inlineStr"/>
+      <c r="K455" s="6" t="inlineStr"/>
+      <c r="L455" s="6" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M455" s="6" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N455" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O455" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P455" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q455" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R455" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S455" s="6" t="n"/>
+      <c r="T455" s="6" t="n"/>
+      <c r="U455" s="6" t="n"/>
+      <c r="V455" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W455" s="6" t="inlineStr"/>
+      <c r="X455" s="6" t="n"/>
+      <c r="Y455" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z455" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA455" s="6" t="n"/>
+      <c r="AB455" s="6" t="n"/>
+      <c r="AC455" s="6" t="n"/>
+      <c r="AD455" s="6" t="n"/>
+      <c r="AE455" s="6" t="n"/>
+      <c r="AF455" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B456" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C456" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D456" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E456" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F456" s="4" t="n"/>
+      <c r="G456" s="4" t="n"/>
+      <c r="H456" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I456" s="4" t="inlineStr"/>
+      <c r="J456" s="4" t="inlineStr"/>
+      <c r="K456" s="4" t="inlineStr"/>
+      <c r="L456" s="4" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M456" s="4" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N456" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O456" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P456" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q456" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R456" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S456" s="4" t="n"/>
+      <c r="T456" s="4" t="n"/>
+      <c r="U456" s="4" t="n"/>
+      <c r="V456" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W456" s="4" t="inlineStr"/>
+      <c r="X456" s="4" t="n"/>
+      <c r="Y456" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z456" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA456" s="4" t="n"/>
+      <c r="AB456" s="4" t="n"/>
+      <c r="AC456" s="4" t="n"/>
+      <c r="AD456" s="4" t="n"/>
+      <c r="AE456" s="4" t="n"/>
+      <c r="AF456" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B457" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C457" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D457" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E457" s="6" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F457" s="6" t="n"/>
+      <c r="G457" s="6" t="n"/>
+      <c r="H457" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I457" s="6" t="inlineStr"/>
+      <c r="J457" s="6" t="inlineStr"/>
+      <c r="K457" s="6" t="inlineStr"/>
+      <c r="L457" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M457" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N457" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O457" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P457" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q457" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R457" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S457" s="6" t="n"/>
+      <c r="T457" s="6" t="n"/>
+      <c r="U457" s="6" t="n"/>
+      <c r="V457" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W457" s="6" t="inlineStr"/>
+      <c r="X457" s="6" t="n"/>
+      <c r="Y457" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z457" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA457" s="6" t="n"/>
+      <c r="AB457" s="6" t="n"/>
+      <c r="AC457" s="6" t="n"/>
+      <c r="AD457" s="6" t="n"/>
+      <c r="AE457" s="6" t="n"/>
+      <c r="AF457" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B458" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C458" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D458" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E458" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F458" s="4" t="n"/>
+      <c r="G458" s="4" t="n"/>
+      <c r="H458" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I458" s="4" t="inlineStr"/>
+      <c r="J458" s="4" t="inlineStr"/>
+      <c r="K458" s="4" t="inlineStr"/>
+      <c r="L458" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M458" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N458" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O458" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P458" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q458" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R458" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S458" s="4" t="n"/>
+      <c r="T458" s="4" t="n"/>
+      <c r="U458" s="4" t="n"/>
+      <c r="V458" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W458" s="4" t="inlineStr"/>
+      <c r="X458" s="4" t="n"/>
+      <c r="Y458" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z458" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA458" s="4" t="n"/>
+      <c r="AB458" s="4" t="n"/>
+      <c r="AC458" s="4" t="n"/>
+      <c r="AD458" s="4" t="n"/>
+      <c r="AE458" s="4" t="n"/>
+      <c r="AF458" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B459" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C459" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D459" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E459" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F459" s="6" t="n"/>
+      <c r="G459" s="6" t="n"/>
+      <c r="H459" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I459" s="6" t="inlineStr"/>
+      <c r="J459" s="6" t="inlineStr"/>
+      <c r="K459" s="6" t="inlineStr"/>
+      <c r="L459" s="6" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M459" s="6" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N459" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O459" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P459" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q459" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R459" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S459" s="6" t="n"/>
+      <c r="T459" s="6" t="n"/>
+      <c r="U459" s="6" t="n"/>
+      <c r="V459" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W459" s="6" t="inlineStr"/>
+      <c r="X459" s="6" t="n"/>
+      <c r="Y459" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z459" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA459" s="6" t="n"/>
+      <c r="AB459" s="6" t="n"/>
+      <c r="AC459" s="6" t="n"/>
+      <c r="AD459" s="6" t="n"/>
+      <c r="AE459" s="6" t="n"/>
+      <c r="AF459" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B460" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C460" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D460" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E460" s="4" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F460" s="4" t="n"/>
+      <c r="G460" s="4" t="n"/>
+      <c r="H460" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I460" s="4" t="inlineStr"/>
+      <c r="J460" s="4" t="inlineStr"/>
+      <c r="K460" s="4" t="inlineStr"/>
+      <c r="L460" s="4" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M460" s="4" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N460" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O460" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P460" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q460" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R460" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S460" s="4" t="n"/>
+      <c r="T460" s="4" t="n"/>
+      <c r="U460" s="4" t="n"/>
+      <c r="V460" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W460" s="4" t="inlineStr"/>
+      <c r="X460" s="4" t="n"/>
+      <c r="Y460" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z460" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA460" s="4" t="n"/>
+      <c r="AB460" s="4" t="n"/>
+      <c r="AC460" s="4" t="n"/>
+      <c r="AD460" s="4" t="n"/>
+      <c r="AE460" s="4" t="n"/>
+      <c r="AF460" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B461" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C461" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D461" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E461" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F461" s="6" t="n"/>
+      <c r="G461" s="6" t="n"/>
+      <c r="H461" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I461" s="6" t="inlineStr"/>
+      <c r="J461" s="6" t="inlineStr"/>
+      <c r="K461" s="6" t="inlineStr"/>
+      <c r="L461" s="6" t="n"/>
+      <c r="M461" s="6" t="n"/>
+      <c r="N461" s="6" t="n"/>
+      <c r="O461" s="6" t="n"/>
+      <c r="P461" s="6" t="n"/>
+      <c r="Q461" s="6" t="n"/>
+      <c r="R461" s="6" t="n"/>
+      <c r="S461" s="6" t="n"/>
+      <c r="T461" s="6" t="n"/>
+      <c r="U461" s="6" t="n"/>
+      <c r="V461" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W461" s="6" t="inlineStr"/>
+      <c r="X461" s="6" t="n"/>
+      <c r="Y461" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z461" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA461" s="6" t="n"/>
+      <c r="AB461" s="6" t="n"/>
+      <c r="AC461" s="6" t="n"/>
+      <c r="AD461" s="6" t="n"/>
+      <c r="AE461" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF461" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B462" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C462" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D462" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E462" s="4" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F462" s="4" t="n"/>
+      <c r="G462" s="4" t="n"/>
+      <c r="H462" s="4" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I462" s="4" t="inlineStr"/>
+      <c r="J462" s="4" t="inlineStr"/>
+      <c r="K462" s="4" t="inlineStr"/>
+      <c r="L462" s="4" t="n"/>
+      <c r="M462" s="4" t="n"/>
+      <c r="N462" s="4" t="n"/>
+      <c r="O462" s="4" t="n"/>
+      <c r="P462" s="4" t="n"/>
+      <c r="Q462" s="4" t="n"/>
+      <c r="R462" s="4" t="n"/>
+      <c r="S462" s="4" t="n"/>
+      <c r="T462" s="4" t="n"/>
+      <c r="U462" s="4" t="n"/>
+      <c r="V462" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W462" s="4" t="inlineStr"/>
+      <c r="X462" s="4" t="n"/>
+      <c r="Y462" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z462" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA462" s="4" t="n"/>
+      <c r="AB462" s="4" t="n"/>
+      <c r="AC462" s="4" t="n"/>
+      <c r="AD462" s="4" t="n"/>
+      <c r="AE462" s="4" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF462" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B463" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C463" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D463" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E463" s="6" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F463" s="6" t="n"/>
+      <c r="G463" s="6" t="n"/>
+      <c r="H463" s="6" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I463" s="6" t="inlineStr"/>
+      <c r="J463" s="6" t="inlineStr"/>
+      <c r="K463" s="6" t="inlineStr"/>
+      <c r="L463" s="6" t="n"/>
+      <c r="M463" s="6" t="n"/>
+      <c r="N463" s="6" t="n"/>
+      <c r="O463" s="6" t="n"/>
+      <c r="P463" s="6" t="n"/>
+      <c r="Q463" s="6" t="n"/>
+      <c r="R463" s="6" t="n"/>
+      <c r="S463" s="6" t="n"/>
+      <c r="T463" s="6" t="n"/>
+      <c r="U463" s="6" t="n"/>
+      <c r="V463" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W463" s="6" t="inlineStr"/>
+      <c r="X463" s="6" t="n"/>
+      <c r="Y463" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z463" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA463" s="6" t="n"/>
+      <c r="AB463" s="6" t="n"/>
+      <c r="AC463" s="6" t="n"/>
+      <c r="AD463" s="6" t="n"/>
+      <c r="AE463" s="6" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF463" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B464" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C464" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D464" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E464" s="4" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F464" s="4" t="n"/>
+      <c r="G464" s="4" t="n"/>
+      <c r="H464" s="4" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I464" s="4" t="inlineStr"/>
+      <c r="J464" s="4" t="inlineStr"/>
+      <c r="K464" s="4" t="inlineStr"/>
+      <c r="L464" s="4" t="n"/>
+      <c r="M464" s="4" t="n"/>
+      <c r="N464" s="4" t="n"/>
+      <c r="O464" s="4" t="n"/>
+      <c r="P464" s="4" t="n"/>
+      <c r="Q464" s="4" t="n"/>
+      <c r="R464" s="4" t="n"/>
+      <c r="S464" s="4" t="n"/>
+      <c r="T464" s="4" t="n"/>
+      <c r="U464" s="4" t="n"/>
+      <c r="V464" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W464" s="4" t="inlineStr"/>
+      <c r="X464" s="4" t="n"/>
+      <c r="Y464" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z464" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA464" s="4" t="n"/>
+      <c r="AB464" s="4" t="n"/>
+      <c r="AC464" s="4" t="n"/>
+      <c r="AD464" s="4" t="n"/>
+      <c r="AE464" s="4" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF464" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B465" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C465" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D465" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E465" s="6" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F465" s="6" t="n"/>
+      <c r="G465" s="6" t="n"/>
+      <c r="H465" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I465" s="6" t="inlineStr"/>
+      <c r="J465" s="6" t="inlineStr"/>
+      <c r="K465" s="6" t="inlineStr"/>
+      <c r="L465" s="6" t="n"/>
+      <c r="M465" s="6" t="n"/>
+      <c r="N465" s="6" t="n"/>
+      <c r="O465" s="6" t="n"/>
+      <c r="P465" s="6" t="n"/>
+      <c r="Q465" s="6" t="n"/>
+      <c r="R465" s="6" t="n"/>
+      <c r="S465" s="6" t="n"/>
+      <c r="T465" s="6" t="n"/>
+      <c r="U465" s="6" t="n"/>
+      <c r="V465" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W465" s="6" t="inlineStr"/>
+      <c r="X465" s="6" t="n"/>
+      <c r="Y465" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z465" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA465" s="6" t="n"/>
+      <c r="AB465" s="6" t="n"/>
+      <c r="AC465" s="6" t="n"/>
+      <c r="AD465" s="6" t="n"/>
+      <c r="AE465" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF465" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B466" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C466" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D466" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E466" s="4" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F466" s="4" t="n"/>
+      <c r="G466" s="4" t="n"/>
+      <c r="H466" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I466" s="4" t="inlineStr"/>
+      <c r="J466" s="4" t="inlineStr"/>
+      <c r="K466" s="4" t="inlineStr"/>
+      <c r="L466" s="4" t="n"/>
+      <c r="M466" s="4" t="n"/>
+      <c r="N466" s="4" t="n"/>
+      <c r="O466" s="4" t="n"/>
+      <c r="P466" s="4" t="n"/>
+      <c r="Q466" s="4" t="n"/>
+      <c r="R466" s="4" t="n"/>
+      <c r="S466" s="4" t="n"/>
+      <c r="T466" s="4" t="n"/>
+      <c r="U466" s="4" t="n"/>
+      <c r="V466" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W466" s="4" t="inlineStr"/>
+      <c r="X466" s="4" t="n"/>
+      <c r="Y466" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z466" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA466" s="4" t="n"/>
+      <c r="AB466" s="4" t="n"/>
+      <c r="AC466" s="4" t="n"/>
+      <c r="AD466" s="4" t="n"/>
+      <c r="AE466" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF466" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B467" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C467" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D467" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E467" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F467" s="6" t="n"/>
+      <c r="G467" s="6" t="n"/>
+      <c r="H467" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I467" s="6" t="inlineStr"/>
+      <c r="J467" s="6" t="inlineStr"/>
+      <c r="K467" s="6" t="inlineStr"/>
+      <c r="L467" s="6" t="n"/>
+      <c r="M467" s="6" t="n"/>
+      <c r="N467" s="6" t="n"/>
+      <c r="O467" s="6" t="n"/>
+      <c r="P467" s="6" t="n"/>
+      <c r="Q467" s="6" t="n"/>
+      <c r="R467" s="6" t="n"/>
+      <c r="S467" s="6" t="n"/>
+      <c r="T467" s="6" t="n"/>
+      <c r="U467" s="6" t="n"/>
+      <c r="V467" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W467" s="6" t="inlineStr"/>
+      <c r="X467" s="6" t="n"/>
+      <c r="Y467" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z467" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA467" s="6" t="n"/>
+      <c r="AB467" s="6" t="n"/>
+      <c r="AC467" s="6" t="n"/>
+      <c r="AD467" s="6" t="n"/>
+      <c r="AE467" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF467" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B468" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C468" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D468" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E468" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F468" s="4" t="n"/>
+      <c r="G468" s="4" t="n"/>
+      <c r="H468" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I468" s="4" t="inlineStr"/>
+      <c r="J468" s="4" t="inlineStr"/>
+      <c r="K468" s="4" t="inlineStr"/>
+      <c r="L468" s="4" t="n"/>
+      <c r="M468" s="4" t="n"/>
+      <c r="N468" s="4" t="n"/>
+      <c r="O468" s="4" t="n"/>
+      <c r="P468" s="4" t="n"/>
+      <c r="Q468" s="4" t="n"/>
+      <c r="R468" s="4" t="n"/>
+      <c r="S468" s="4" t="n"/>
+      <c r="T468" s="4" t="n"/>
+      <c r="U468" s="4" t="n"/>
+      <c r="V468" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W468" s="4" t="inlineStr"/>
+      <c r="X468" s="4" t="n"/>
+      <c r="Y468" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z468" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA468" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB468" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC468" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD468" s="4" t="n"/>
+      <c r="AE468" s="4" t="n"/>
+      <c r="AF468" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B469" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C469" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D469" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E469" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F469" s="6" t="n"/>
+      <c r="G469" s="6" t="n"/>
+      <c r="H469" s="6" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I469" s="6" t="inlineStr"/>
+      <c r="J469" s="6" t="inlineStr"/>
+      <c r="K469" s="6" t="inlineStr"/>
+      <c r="L469" s="6" t="n"/>
+      <c r="M469" s="6" t="n"/>
+      <c r="N469" s="6" t="n"/>
+      <c r="O469" s="6" t="n"/>
+      <c r="P469" s="6" t="n"/>
+      <c r="Q469" s="6" t="n"/>
+      <c r="R469" s="6" t="n"/>
+      <c r="S469" s="6" t="n"/>
+      <c r="T469" s="6" t="n"/>
+      <c r="U469" s="6" t="n"/>
+      <c r="V469" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W469" s="6" t="inlineStr"/>
+      <c r="X469" s="6" t="n"/>
+      <c r="Y469" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z469" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA469" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB469" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC469" s="6" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD469" s="6" t="n"/>
+      <c r="AE469" s="6" t="n"/>
+      <c r="AF469" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B470" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C470" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D470" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E470" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F470" s="4" t="n"/>
+      <c r="G470" s="4" t="n"/>
+      <c r="H470" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I470" s="4" t="inlineStr"/>
+      <c r="J470" s="4" t="inlineStr"/>
+      <c r="K470" s="4" t="inlineStr"/>
+      <c r="L470" s="4" t="n"/>
+      <c r="M470" s="4" t="n"/>
+      <c r="N470" s="4" t="n"/>
+      <c r="O470" s="4" t="n"/>
+      <c r="P470" s="4" t="n"/>
+      <c r="Q470" s="4" t="n"/>
+      <c r="R470" s="4" t="n"/>
+      <c r="S470" s="4" t="n"/>
+      <c r="T470" s="4" t="n"/>
+      <c r="U470" s="4" t="n"/>
+      <c r="V470" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W470" s="4" t="inlineStr"/>
+      <c r="X470" s="4" t="n"/>
+      <c r="Y470" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z470" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA470" s="4" t="n"/>
+      <c r="AB470" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC470" s="4" t="n"/>
+      <c r="AD470" s="4" t="n"/>
+      <c r="AE470" s="4" t="n"/>
+      <c r="AF470" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-01</t>
+        </is>
+      </c>
+      <c r="B471" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C471" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D471" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E471" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F471" s="6" t="n"/>
+      <c r="G471" s="6" t="n"/>
+      <c r="H471" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I471" s="6" t="inlineStr"/>
+      <c r="J471" s="6" t="inlineStr"/>
+      <c r="K471" s="6" t="inlineStr"/>
+      <c r="L471" s="6" t="n"/>
+      <c r="M471" s="6" t="n"/>
+      <c r="N471" s="6" t="n"/>
+      <c r="O471" s="6" t="n"/>
+      <c r="P471" s="6" t="n"/>
+      <c r="Q471" s="6" t="n"/>
+      <c r="R471" s="6" t="n"/>
+      <c r="S471" s="6" t="n"/>
+      <c r="T471" s="6" t="n"/>
+      <c r="U471" s="6" t="n"/>
+      <c r="V471" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W471" s="6" t="inlineStr"/>
+      <c r="X471" s="6" t="n"/>
+      <c r="Y471" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z471" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA471" s="6" t="n"/>
+      <c r="AB471" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC471" s="6" t="n"/>
+      <c r="AD471" s="6" t="n"/>
+      <c r="AE471" s="6" t="n"/>
+      <c r="AF471" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-02
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF471"/>
+  <dimension ref="A1:AF507"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -37624,6 +37624,2840 @@
         <v>1</v>
       </c>
     </row>
+    <row r="472">
+      <c r="A472" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B472" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C472" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D472" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E472" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F472" s="4" t="n"/>
+      <c r="G472" s="4" t="n"/>
+      <c r="H472" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I472" s="4" t="inlineStr"/>
+      <c r="J472" s="4" t="inlineStr"/>
+      <c r="K472" s="4" t="inlineStr"/>
+      <c r="L472" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M472" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N472" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O472" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P472" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q472" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R472" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S472" s="4" t="n"/>
+      <c r="T472" s="4" t="n"/>
+      <c r="U472" s="4" t="n"/>
+      <c r="V472" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W472" s="4" t="inlineStr"/>
+      <c r="X472" s="4" t="n"/>
+      <c r="Y472" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z472" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA472" s="4" t="n"/>
+      <c r="AB472" s="4" t="n"/>
+      <c r="AC472" s="4" t="n"/>
+      <c r="AD472" s="4" t="n"/>
+      <c r="AE472" s="4" t="n"/>
+      <c r="AF472" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B473" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C473" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D473" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E473" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F473" s="6" t="n"/>
+      <c r="G473" s="6" t="n"/>
+      <c r="H473" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I473" s="6" t="inlineStr"/>
+      <c r="J473" s="6" t="inlineStr"/>
+      <c r="K473" s="6" t="inlineStr"/>
+      <c r="L473" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M473" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N473" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O473" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P473" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q473" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R473" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S473" s="6" t="n"/>
+      <c r="T473" s="6" t="n"/>
+      <c r="U473" s="6" t="n"/>
+      <c r="V473" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W473" s="6" t="inlineStr"/>
+      <c r="X473" s="6" t="n"/>
+      <c r="Y473" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z473" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA473" s="6" t="n"/>
+      <c r="AB473" s="6" t="n"/>
+      <c r="AC473" s="6" t="n"/>
+      <c r="AD473" s="6" t="n"/>
+      <c r="AE473" s="6" t="n"/>
+      <c r="AF473" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D474" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E474" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F474" s="4" t="n"/>
+      <c r="G474" s="4" t="n"/>
+      <c r="H474" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I474" s="4" t="inlineStr"/>
+      <c r="J474" s="4" t="inlineStr"/>
+      <c r="K474" s="4" t="inlineStr"/>
+      <c r="L474" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M474" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N474" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O474" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P474" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q474" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R474" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S474" s="4" t="n"/>
+      <c r="T474" s="4" t="n"/>
+      <c r="U474" s="4" t="n"/>
+      <c r="V474" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W474" s="4" t="inlineStr"/>
+      <c r="X474" s="4" t="n"/>
+      <c r="Y474" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z474" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA474" s="4" t="n"/>
+      <c r="AB474" s="4" t="n"/>
+      <c r="AC474" s="4" t="n"/>
+      <c r="AD474" s="4" t="n"/>
+      <c r="AE474" s="4" t="n"/>
+      <c r="AF474" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B475" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C475" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D475" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E475" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F475" s="6" t="n"/>
+      <c r="G475" s="6" t="n"/>
+      <c r="H475" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I475" s="6" t="inlineStr"/>
+      <c r="J475" s="6" t="inlineStr"/>
+      <c r="K475" s="6" t="inlineStr"/>
+      <c r="L475" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M475" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N475" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O475" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P475" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q475" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R475" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S475" s="6" t="n"/>
+      <c r="T475" s="6" t="n"/>
+      <c r="U475" s="6" t="n"/>
+      <c r="V475" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W475" s="6" t="inlineStr"/>
+      <c r="X475" s="6" t="n"/>
+      <c r="Y475" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z475" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA475" s="6" t="n"/>
+      <c r="AB475" s="6" t="n"/>
+      <c r="AC475" s="6" t="n"/>
+      <c r="AD475" s="6" t="n"/>
+      <c r="AE475" s="6" t="n"/>
+      <c r="AF475" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B476" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C476" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D476" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E476" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F476" s="4" t="n"/>
+      <c r="G476" s="4" t="n"/>
+      <c r="H476" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I476" s="4" t="inlineStr"/>
+      <c r="J476" s="4" t="inlineStr"/>
+      <c r="K476" s="4" t="inlineStr"/>
+      <c r="L476" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M476" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N476" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O476" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P476" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q476" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R476" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S476" s="4" t="n"/>
+      <c r="T476" s="4" t="n"/>
+      <c r="U476" s="4" t="n"/>
+      <c r="V476" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W476" s="4" t="inlineStr"/>
+      <c r="X476" s="4" t="n"/>
+      <c r="Y476" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z476" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA476" s="4" t="n"/>
+      <c r="AB476" s="4" t="n"/>
+      <c r="AC476" s="4" t="n"/>
+      <c r="AD476" s="4" t="n"/>
+      <c r="AE476" s="4" t="n"/>
+      <c r="AF476" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B477" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C477" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D477" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E477" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F477" s="6" t="n"/>
+      <c r="G477" s="6" t="n"/>
+      <c r="H477" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I477" s="6" t="inlineStr"/>
+      <c r="J477" s="6" t="inlineStr"/>
+      <c r="K477" s="6" t="inlineStr"/>
+      <c r="L477" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M477" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N477" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O477" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P477" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q477" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R477" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S477" s="6" t="n"/>
+      <c r="T477" s="6" t="n"/>
+      <c r="U477" s="6" t="n"/>
+      <c r="V477" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W477" s="6" t="inlineStr"/>
+      <c r="X477" s="6" t="n"/>
+      <c r="Y477" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z477" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA477" s="6" t="n"/>
+      <c r="AB477" s="6" t="n"/>
+      <c r="AC477" s="6" t="n"/>
+      <c r="AD477" s="6" t="n"/>
+      <c r="AE477" s="6" t="n"/>
+      <c r="AF477" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B478" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C478" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D478" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E478" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F478" s="4" t="n"/>
+      <c r="G478" s="4" t="n"/>
+      <c r="H478" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I478" s="4" t="inlineStr"/>
+      <c r="J478" s="4" t="inlineStr"/>
+      <c r="K478" s="4" t="inlineStr"/>
+      <c r="L478" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M478" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N478" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O478" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P478" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q478" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R478" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S478" s="4" t="n"/>
+      <c r="T478" s="4" t="n"/>
+      <c r="U478" s="4" t="n"/>
+      <c r="V478" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W478" s="4" t="inlineStr"/>
+      <c r="X478" s="4" t="n"/>
+      <c r="Y478" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z478" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA478" s="4" t="n"/>
+      <c r="AB478" s="4" t="n"/>
+      <c r="AC478" s="4" t="n"/>
+      <c r="AD478" s="4" t="n"/>
+      <c r="AE478" s="4" t="n"/>
+      <c r="AF478" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B479" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C479" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D479" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E479" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F479" s="6" t="n"/>
+      <c r="G479" s="6" t="n"/>
+      <c r="H479" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I479" s="6" t="inlineStr"/>
+      <c r="J479" s="6" t="inlineStr"/>
+      <c r="K479" s="6" t="inlineStr"/>
+      <c r="L479" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M479" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N479" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O479" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P479" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q479" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R479" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S479" s="6" t="n"/>
+      <c r="T479" s="6" t="n"/>
+      <c r="U479" s="6" t="n"/>
+      <c r="V479" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W479" s="6" t="inlineStr"/>
+      <c r="X479" s="6" t="n"/>
+      <c r="Y479" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z479" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA479" s="6" t="n"/>
+      <c r="AB479" s="6" t="n"/>
+      <c r="AC479" s="6" t="n"/>
+      <c r="AD479" s="6" t="n"/>
+      <c r="AE479" s="6" t="n"/>
+      <c r="AF479" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C480" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D480" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E480" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F480" s="4" t="n"/>
+      <c r="G480" s="4" t="n"/>
+      <c r="H480" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I480" s="4" t="inlineStr"/>
+      <c r="J480" s="4" t="inlineStr"/>
+      <c r="K480" s="4" t="inlineStr"/>
+      <c r="L480" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M480" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N480" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O480" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P480" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q480" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R480" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S480" s="4" t="n"/>
+      <c r="T480" s="4" t="n"/>
+      <c r="U480" s="4" t="n"/>
+      <c r="V480" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W480" s="4" t="inlineStr"/>
+      <c r="X480" s="4" t="n"/>
+      <c r="Y480" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z480" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA480" s="4" t="n"/>
+      <c r="AB480" s="4" t="n"/>
+      <c r="AC480" s="4" t="n"/>
+      <c r="AD480" s="4" t="n"/>
+      <c r="AE480" s="4" t="n"/>
+      <c r="AF480" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B481" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C481" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D481" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E481" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F481" s="6" t="n"/>
+      <c r="G481" s="6" t="n"/>
+      <c r="H481" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I481" s="6" t="inlineStr"/>
+      <c r="J481" s="6" t="inlineStr"/>
+      <c r="K481" s="6" t="inlineStr"/>
+      <c r="L481" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M481" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N481" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O481" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P481" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q481" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R481" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S481" s="6" t="n"/>
+      <c r="T481" s="6" t="n"/>
+      <c r="U481" s="6" t="n"/>
+      <c r="V481" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W481" s="6" t="inlineStr"/>
+      <c r="X481" s="6" t="n"/>
+      <c r="Y481" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z481" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA481" s="6" t="n"/>
+      <c r="AB481" s="6" t="n"/>
+      <c r="AC481" s="6" t="n"/>
+      <c r="AD481" s="6" t="n"/>
+      <c r="AE481" s="6" t="n"/>
+      <c r="AF481" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C482" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D482" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E482" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F482" s="4" t="n"/>
+      <c r="G482" s="4" t="n"/>
+      <c r="H482" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I482" s="4" t="inlineStr"/>
+      <c r="J482" s="4" t="inlineStr"/>
+      <c r="K482" s="4" t="inlineStr"/>
+      <c r="L482" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M482" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N482" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O482" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P482" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q482" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R482" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S482" s="4" t="n"/>
+      <c r="T482" s="4" t="n"/>
+      <c r="U482" s="4" t="n"/>
+      <c r="V482" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W482" s="4" t="inlineStr"/>
+      <c r="X482" s="4" t="n"/>
+      <c r="Y482" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z482" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA482" s="4" t="n"/>
+      <c r="AB482" s="4" t="n"/>
+      <c r="AC482" s="4" t="n"/>
+      <c r="AD482" s="4" t="n"/>
+      <c r="AE482" s="4" t="n"/>
+      <c r="AF482" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B483" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C483" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D483" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E483" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F483" s="6" t="n"/>
+      <c r="G483" s="6" t="n"/>
+      <c r="H483" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I483" s="6" t="inlineStr"/>
+      <c r="J483" s="6" t="inlineStr"/>
+      <c r="K483" s="6" t="inlineStr"/>
+      <c r="L483" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M483" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N483" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O483" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P483" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q483" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R483" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S483" s="6" t="n"/>
+      <c r="T483" s="6" t="n"/>
+      <c r="U483" s="6" t="n"/>
+      <c r="V483" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W483" s="6" t="inlineStr"/>
+      <c r="X483" s="6" t="n"/>
+      <c r="Y483" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z483" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA483" s="6" t="n"/>
+      <c r="AB483" s="6" t="n"/>
+      <c r="AC483" s="6" t="n"/>
+      <c r="AD483" s="6" t="n"/>
+      <c r="AE483" s="6" t="n"/>
+      <c r="AF483" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C484" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D484" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E484" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F484" s="4" t="n"/>
+      <c r="G484" s="4" t="n"/>
+      <c r="H484" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I484" s="4" t="inlineStr"/>
+      <c r="J484" s="4" t="inlineStr"/>
+      <c r="K484" s="4" t="inlineStr"/>
+      <c r="L484" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M484" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N484" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O484" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P484" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q484" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R484" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S484" s="4" t="n"/>
+      <c r="T484" s="4" t="n"/>
+      <c r="U484" s="4" t="n"/>
+      <c r="V484" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W484" s="4" t="inlineStr"/>
+      <c r="X484" s="4" t="n"/>
+      <c r="Y484" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z484" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA484" s="4" t="n"/>
+      <c r="AB484" s="4" t="n"/>
+      <c r="AC484" s="4" t="n"/>
+      <c r="AD484" s="4" t="n"/>
+      <c r="AE484" s="4" t="n"/>
+      <c r="AF484" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B485" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C485" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D485" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E485" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F485" s="6" t="n"/>
+      <c r="G485" s="6" t="n"/>
+      <c r="H485" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I485" s="6" t="inlineStr"/>
+      <c r="J485" s="6" t="inlineStr"/>
+      <c r="K485" s="6" t="inlineStr"/>
+      <c r="L485" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M485" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N485" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O485" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P485" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q485" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R485" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S485" s="6" t="n"/>
+      <c r="T485" s="6" t="n"/>
+      <c r="U485" s="6" t="n"/>
+      <c r="V485" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W485" s="6" t="inlineStr"/>
+      <c r="X485" s="6" t="n"/>
+      <c r="Y485" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z485" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA485" s="6" t="n"/>
+      <c r="AB485" s="6" t="n"/>
+      <c r="AC485" s="6" t="n"/>
+      <c r="AD485" s="6" t="n"/>
+      <c r="AE485" s="6" t="n"/>
+      <c r="AF485" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C486" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D486" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E486" s="4" t="n">
+        <v>113.99</v>
+      </c>
+      <c r="F486" s="4" t="n"/>
+      <c r="G486" s="4" t="n"/>
+      <c r="H486" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="I486" s="4" t="inlineStr"/>
+      <c r="J486" s="4" t="inlineStr"/>
+      <c r="K486" s="4" t="inlineStr"/>
+      <c r="L486" s="4" t="n">
+        <v>55.61</v>
+      </c>
+      <c r="M486" s="4" t="n">
+        <v>1.668</v>
+      </c>
+      <c r="N486" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O486" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P486" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q486" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R486" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S486" s="4" t="n"/>
+      <c r="T486" s="4" t="n"/>
+      <c r="U486" s="4" t="n"/>
+      <c r="V486" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W486" s="4" t="inlineStr"/>
+      <c r="X486" s="4" t="n"/>
+      <c r="Y486" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z486" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA486" s="4" t="n"/>
+      <c r="AB486" s="4" t="n"/>
+      <c r="AC486" s="4" t="n"/>
+      <c r="AD486" s="4" t="n"/>
+      <c r="AE486" s="4" t="n"/>
+      <c r="AF486" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B487" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C487" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D487" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E487" s="6" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F487" s="6" t="n"/>
+      <c r="G487" s="6" t="n"/>
+      <c r="H487" s="6" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I487" s="6" t="inlineStr"/>
+      <c r="J487" s="6" t="inlineStr"/>
+      <c r="K487" s="6" t="inlineStr"/>
+      <c r="L487" s="6" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M487" s="6" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N487" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O487" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P487" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q487" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R487" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S487" s="6" t="n"/>
+      <c r="T487" s="6" t="n"/>
+      <c r="U487" s="6" t="n"/>
+      <c r="V487" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W487" s="6" t="inlineStr"/>
+      <c r="X487" s="6" t="n"/>
+      <c r="Y487" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z487" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA487" s="6" t="n"/>
+      <c r="AB487" s="6" t="n"/>
+      <c r="AC487" s="6" t="n"/>
+      <c r="AD487" s="6" t="n"/>
+      <c r="AE487" s="6" t="n"/>
+      <c r="AF487" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C488" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D488" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E488" s="4" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F488" s="4" t="n"/>
+      <c r="G488" s="4" t="n"/>
+      <c r="H488" s="4" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I488" s="4" t="inlineStr"/>
+      <c r="J488" s="4" t="inlineStr"/>
+      <c r="K488" s="4" t="inlineStr"/>
+      <c r="L488" s="4" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M488" s="4" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N488" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O488" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P488" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q488" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R488" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S488" s="4" t="n"/>
+      <c r="T488" s="4" t="n"/>
+      <c r="U488" s="4" t="n"/>
+      <c r="V488" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W488" s="4" t="inlineStr"/>
+      <c r="X488" s="4" t="n"/>
+      <c r="Y488" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z488" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA488" s="4" t="n"/>
+      <c r="AB488" s="4" t="n"/>
+      <c r="AC488" s="4" t="n"/>
+      <c r="AD488" s="4" t="n"/>
+      <c r="AE488" s="4" t="n"/>
+      <c r="AF488" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B489" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C489" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D489" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E489" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F489" s="6" t="n"/>
+      <c r="G489" s="6" t="n"/>
+      <c r="H489" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I489" s="6" t="inlineStr"/>
+      <c r="J489" s="6" t="inlineStr"/>
+      <c r="K489" s="6" t="inlineStr"/>
+      <c r="L489" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="M489" s="6" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N489" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O489" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P489" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q489" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R489" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S489" s="6" t="n"/>
+      <c r="T489" s="6" t="n"/>
+      <c r="U489" s="6" t="n"/>
+      <c r="V489" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W489" s="6" t="inlineStr"/>
+      <c r="X489" s="6" t="n"/>
+      <c r="Y489" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z489" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA489" s="6" t="n"/>
+      <c r="AB489" s="6" t="n"/>
+      <c r="AC489" s="6" t="n"/>
+      <c r="AD489" s="6" t="n"/>
+      <c r="AE489" s="6" t="n"/>
+      <c r="AF489" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D490" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E490" s="4" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F490" s="4" t="n"/>
+      <c r="G490" s="4" t="n"/>
+      <c r="H490" s="4" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I490" s="4" t="inlineStr"/>
+      <c r="J490" s="4" t="inlineStr"/>
+      <c r="K490" s="4" t="inlineStr"/>
+      <c r="L490" s="4" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M490" s="4" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N490" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O490" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P490" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q490" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R490" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S490" s="4" t="n"/>
+      <c r="T490" s="4" t="n"/>
+      <c r="U490" s="4" t="n"/>
+      <c r="V490" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W490" s="4" t="inlineStr"/>
+      <c r="X490" s="4" t="n"/>
+      <c r="Y490" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z490" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA490" s="4" t="n"/>
+      <c r="AB490" s="4" t="n"/>
+      <c r="AC490" s="4" t="n"/>
+      <c r="AD490" s="4" t="n"/>
+      <c r="AE490" s="4" t="n"/>
+      <c r="AF490" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B491" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C491" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D491" s="6" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E491" s="6" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F491" s="6" t="n"/>
+      <c r="G491" s="6" t="n"/>
+      <c r="H491" s="6" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I491" s="6" t="inlineStr"/>
+      <c r="J491" s="6" t="inlineStr"/>
+      <c r="K491" s="6" t="inlineStr"/>
+      <c r="L491" s="6" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M491" s="6" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N491" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O491" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P491" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q491" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R491" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S491" s="6" t="n"/>
+      <c r="T491" s="6" t="n"/>
+      <c r="U491" s="6" t="n"/>
+      <c r="V491" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W491" s="6" t="inlineStr"/>
+      <c r="X491" s="6" t="n"/>
+      <c r="Y491" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z491" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA491" s="6" t="n"/>
+      <c r="AB491" s="6" t="n"/>
+      <c r="AC491" s="6" t="n"/>
+      <c r="AD491" s="6" t="n"/>
+      <c r="AE491" s="6" t="n"/>
+      <c r="AF491" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C492" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D492" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E492" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F492" s="4" t="n"/>
+      <c r="G492" s="4" t="n"/>
+      <c r="H492" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I492" s="4" t="inlineStr"/>
+      <c r="J492" s="4" t="inlineStr"/>
+      <c r="K492" s="4" t="inlineStr"/>
+      <c r="L492" s="4" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M492" s="4" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N492" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O492" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P492" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q492" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R492" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S492" s="4" t="n"/>
+      <c r="T492" s="4" t="n"/>
+      <c r="U492" s="4" t="n"/>
+      <c r="V492" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W492" s="4" t="inlineStr"/>
+      <c r="X492" s="4" t="n"/>
+      <c r="Y492" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z492" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA492" s="4" t="n"/>
+      <c r="AB492" s="4" t="n"/>
+      <c r="AC492" s="4" t="n"/>
+      <c r="AD492" s="4" t="n"/>
+      <c r="AE492" s="4" t="n"/>
+      <c r="AF492" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B493" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C493" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D493" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E493" s="6" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F493" s="6" t="n"/>
+      <c r="G493" s="6" t="n"/>
+      <c r="H493" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I493" s="6" t="inlineStr"/>
+      <c r="J493" s="6" t="inlineStr"/>
+      <c r="K493" s="6" t="inlineStr"/>
+      <c r="L493" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M493" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N493" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O493" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P493" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q493" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R493" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S493" s="6" t="n"/>
+      <c r="T493" s="6" t="n"/>
+      <c r="U493" s="6" t="n"/>
+      <c r="V493" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W493" s="6" t="inlineStr"/>
+      <c r="X493" s="6" t="n"/>
+      <c r="Y493" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z493" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA493" s="6" t="n"/>
+      <c r="AB493" s="6" t="n"/>
+      <c r="AC493" s="6" t="n"/>
+      <c r="AD493" s="6" t="n"/>
+      <c r="AE493" s="6" t="n"/>
+      <c r="AF493" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C494" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D494" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E494" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F494" s="4" t="n"/>
+      <c r="G494" s="4" t="n"/>
+      <c r="H494" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I494" s="4" t="inlineStr"/>
+      <c r="J494" s="4" t="inlineStr"/>
+      <c r="K494" s="4" t="inlineStr"/>
+      <c r="L494" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M494" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N494" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O494" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P494" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q494" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R494" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S494" s="4" t="n"/>
+      <c r="T494" s="4" t="n"/>
+      <c r="U494" s="4" t="n"/>
+      <c r="V494" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W494" s="4" t="inlineStr"/>
+      <c r="X494" s="4" t="n"/>
+      <c r="Y494" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z494" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA494" s="4" t="n"/>
+      <c r="AB494" s="4" t="n"/>
+      <c r="AC494" s="4" t="n"/>
+      <c r="AD494" s="4" t="n"/>
+      <c r="AE494" s="4" t="n"/>
+      <c r="AF494" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B495" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C495" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D495" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E495" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F495" s="6" t="n"/>
+      <c r="G495" s="6" t="n"/>
+      <c r="H495" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I495" s="6" t="inlineStr"/>
+      <c r="J495" s="6" t="inlineStr"/>
+      <c r="K495" s="6" t="inlineStr"/>
+      <c r="L495" s="6" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M495" s="6" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N495" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O495" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P495" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q495" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R495" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S495" s="6" t="n"/>
+      <c r="T495" s="6" t="n"/>
+      <c r="U495" s="6" t="n"/>
+      <c r="V495" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W495" s="6" t="inlineStr"/>
+      <c r="X495" s="6" t="n"/>
+      <c r="Y495" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z495" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA495" s="6" t="n"/>
+      <c r="AB495" s="6" t="n"/>
+      <c r="AC495" s="6" t="n"/>
+      <c r="AD495" s="6" t="n"/>
+      <c r="AE495" s="6" t="n"/>
+      <c r="AF495" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C496" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D496" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E496" s="4" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F496" s="4" t="n"/>
+      <c r="G496" s="4" t="n"/>
+      <c r="H496" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I496" s="4" t="inlineStr"/>
+      <c r="J496" s="4" t="inlineStr"/>
+      <c r="K496" s="4" t="inlineStr"/>
+      <c r="L496" s="4" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M496" s="4" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N496" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O496" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P496" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q496" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R496" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S496" s="4" t="n"/>
+      <c r="T496" s="4" t="n"/>
+      <c r="U496" s="4" t="n"/>
+      <c r="V496" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W496" s="4" t="inlineStr"/>
+      <c r="X496" s="4" t="n"/>
+      <c r="Y496" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z496" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA496" s="4" t="n"/>
+      <c r="AB496" s="4" t="n"/>
+      <c r="AC496" s="4" t="n"/>
+      <c r="AD496" s="4" t="n"/>
+      <c r="AE496" s="4" t="n"/>
+      <c r="AF496" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B497" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C497" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D497" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E497" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F497" s="6" t="n"/>
+      <c r="G497" s="6" t="n"/>
+      <c r="H497" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I497" s="6" t="inlineStr"/>
+      <c r="J497" s="6" t="inlineStr"/>
+      <c r="K497" s="6" t="inlineStr"/>
+      <c r="L497" s="6" t="n"/>
+      <c r="M497" s="6" t="n"/>
+      <c r="N497" s="6" t="n"/>
+      <c r="O497" s="6" t="n"/>
+      <c r="P497" s="6" t="n"/>
+      <c r="Q497" s="6" t="n"/>
+      <c r="R497" s="6" t="n"/>
+      <c r="S497" s="6" t="n"/>
+      <c r="T497" s="6" t="n"/>
+      <c r="U497" s="6" t="n"/>
+      <c r="V497" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W497" s="6" t="inlineStr"/>
+      <c r="X497" s="6" t="n"/>
+      <c r="Y497" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z497" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA497" s="6" t="n"/>
+      <c r="AB497" s="6" t="n"/>
+      <c r="AC497" s="6" t="n"/>
+      <c r="AD497" s="6" t="n"/>
+      <c r="AE497" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF497" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B498" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C498" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D498" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E498" s="4" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F498" s="4" t="n"/>
+      <c r="G498" s="4" t="n"/>
+      <c r="H498" s="4" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I498" s="4" t="inlineStr"/>
+      <c r="J498" s="4" t="inlineStr"/>
+      <c r="K498" s="4" t="inlineStr"/>
+      <c r="L498" s="4" t="n"/>
+      <c r="M498" s="4" t="n"/>
+      <c r="N498" s="4" t="n"/>
+      <c r="O498" s="4" t="n"/>
+      <c r="P498" s="4" t="n"/>
+      <c r="Q498" s="4" t="n"/>
+      <c r="R498" s="4" t="n"/>
+      <c r="S498" s="4" t="n"/>
+      <c r="T498" s="4" t="n"/>
+      <c r="U498" s="4" t="n"/>
+      <c r="V498" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W498" s="4" t="inlineStr"/>
+      <c r="X498" s="4" t="n"/>
+      <c r="Y498" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z498" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA498" s="4" t="n"/>
+      <c r="AB498" s="4" t="n"/>
+      <c r="AC498" s="4" t="n"/>
+      <c r="AD498" s="4" t="n"/>
+      <c r="AE498" s="4" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF498" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B499" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C499" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D499" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E499" s="6" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F499" s="6" t="n"/>
+      <c r="G499" s="6" t="n"/>
+      <c r="H499" s="6" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I499" s="6" t="inlineStr"/>
+      <c r="J499" s="6" t="inlineStr"/>
+      <c r="K499" s="6" t="inlineStr"/>
+      <c r="L499" s="6" t="n"/>
+      <c r="M499" s="6" t="n"/>
+      <c r="N499" s="6" t="n"/>
+      <c r="O499" s="6" t="n"/>
+      <c r="P499" s="6" t="n"/>
+      <c r="Q499" s="6" t="n"/>
+      <c r="R499" s="6" t="n"/>
+      <c r="S499" s="6" t="n"/>
+      <c r="T499" s="6" t="n"/>
+      <c r="U499" s="6" t="n"/>
+      <c r="V499" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W499" s="6" t="inlineStr"/>
+      <c r="X499" s="6" t="n"/>
+      <c r="Y499" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z499" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA499" s="6" t="n"/>
+      <c r="AB499" s="6" t="n"/>
+      <c r="AC499" s="6" t="n"/>
+      <c r="AD499" s="6" t="n"/>
+      <c r="AE499" s="6" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF499" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C500" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D500" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E500" s="4" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F500" s="4" t="n"/>
+      <c r="G500" s="4" t="n"/>
+      <c r="H500" s="4" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I500" s="4" t="inlineStr"/>
+      <c r="J500" s="4" t="inlineStr"/>
+      <c r="K500" s="4" t="inlineStr"/>
+      <c r="L500" s="4" t="n"/>
+      <c r="M500" s="4" t="n"/>
+      <c r="N500" s="4" t="n"/>
+      <c r="O500" s="4" t="n"/>
+      <c r="P500" s="4" t="n"/>
+      <c r="Q500" s="4" t="n"/>
+      <c r="R500" s="4" t="n"/>
+      <c r="S500" s="4" t="n"/>
+      <c r="T500" s="4" t="n"/>
+      <c r="U500" s="4" t="n"/>
+      <c r="V500" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W500" s="4" t="inlineStr"/>
+      <c r="X500" s="4" t="n"/>
+      <c r="Y500" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z500" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA500" s="4" t="n"/>
+      <c r="AB500" s="4" t="n"/>
+      <c r="AC500" s="4" t="n"/>
+      <c r="AD500" s="4" t="n"/>
+      <c r="AE500" s="4" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF500" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B501" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C501" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D501" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E501" s="6" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F501" s="6" t="n"/>
+      <c r="G501" s="6" t="n"/>
+      <c r="H501" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I501" s="6" t="inlineStr"/>
+      <c r="J501" s="6" t="inlineStr"/>
+      <c r="K501" s="6" t="inlineStr"/>
+      <c r="L501" s="6" t="n"/>
+      <c r="M501" s="6" t="n"/>
+      <c r="N501" s="6" t="n"/>
+      <c r="O501" s="6" t="n"/>
+      <c r="P501" s="6" t="n"/>
+      <c r="Q501" s="6" t="n"/>
+      <c r="R501" s="6" t="n"/>
+      <c r="S501" s="6" t="n"/>
+      <c r="T501" s="6" t="n"/>
+      <c r="U501" s="6" t="n"/>
+      <c r="V501" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W501" s="6" t="inlineStr"/>
+      <c r="X501" s="6" t="n"/>
+      <c r="Y501" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z501" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA501" s="6" t="n"/>
+      <c r="AB501" s="6" t="n"/>
+      <c r="AC501" s="6" t="n"/>
+      <c r="AD501" s="6" t="n"/>
+      <c r="AE501" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF501" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B502" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C502" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D502" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E502" s="4" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F502" s="4" t="n"/>
+      <c r="G502" s="4" t="n"/>
+      <c r="H502" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I502" s="4" t="inlineStr"/>
+      <c r="J502" s="4" t="inlineStr"/>
+      <c r="K502" s="4" t="inlineStr"/>
+      <c r="L502" s="4" t="n"/>
+      <c r="M502" s="4" t="n"/>
+      <c r="N502" s="4" t="n"/>
+      <c r="O502" s="4" t="n"/>
+      <c r="P502" s="4" t="n"/>
+      <c r="Q502" s="4" t="n"/>
+      <c r="R502" s="4" t="n"/>
+      <c r="S502" s="4" t="n"/>
+      <c r="T502" s="4" t="n"/>
+      <c r="U502" s="4" t="n"/>
+      <c r="V502" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W502" s="4" t="inlineStr"/>
+      <c r="X502" s="4" t="n"/>
+      <c r="Y502" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z502" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA502" s="4" t="n"/>
+      <c r="AB502" s="4" t="n"/>
+      <c r="AC502" s="4" t="n"/>
+      <c r="AD502" s="4" t="n"/>
+      <c r="AE502" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF502" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B503" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C503" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D503" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E503" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F503" s="6" t="n"/>
+      <c r="G503" s="6" t="n"/>
+      <c r="H503" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I503" s="6" t="inlineStr"/>
+      <c r="J503" s="6" t="inlineStr"/>
+      <c r="K503" s="6" t="inlineStr"/>
+      <c r="L503" s="6" t="n"/>
+      <c r="M503" s="6" t="n"/>
+      <c r="N503" s="6" t="n"/>
+      <c r="O503" s="6" t="n"/>
+      <c r="P503" s="6" t="n"/>
+      <c r="Q503" s="6" t="n"/>
+      <c r="R503" s="6" t="n"/>
+      <c r="S503" s="6" t="n"/>
+      <c r="T503" s="6" t="n"/>
+      <c r="U503" s="6" t="n"/>
+      <c r="V503" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W503" s="6" t="inlineStr"/>
+      <c r="X503" s="6" t="n"/>
+      <c r="Y503" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z503" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA503" s="6" t="n"/>
+      <c r="AB503" s="6" t="n"/>
+      <c r="AC503" s="6" t="n"/>
+      <c r="AD503" s="6" t="n"/>
+      <c r="AE503" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF503" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B504" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C504" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D504" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E504" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F504" s="4" t="n"/>
+      <c r="G504" s="4" t="n"/>
+      <c r="H504" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I504" s="4" t="inlineStr"/>
+      <c r="J504" s="4" t="inlineStr"/>
+      <c r="K504" s="4" t="inlineStr"/>
+      <c r="L504" s="4" t="n"/>
+      <c r="M504" s="4" t="n"/>
+      <c r="N504" s="4" t="n"/>
+      <c r="O504" s="4" t="n"/>
+      <c r="P504" s="4" t="n"/>
+      <c r="Q504" s="4" t="n"/>
+      <c r="R504" s="4" t="n"/>
+      <c r="S504" s="4" t="n"/>
+      <c r="T504" s="4" t="n"/>
+      <c r="U504" s="4" t="n"/>
+      <c r="V504" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W504" s="4" t="inlineStr"/>
+      <c r="X504" s="4" t="n"/>
+      <c r="Y504" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z504" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA504" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB504" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC504" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD504" s="4" t="n"/>
+      <c r="AE504" s="4" t="n"/>
+      <c r="AF504" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B505" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C505" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D505" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E505" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F505" s="6" t="n"/>
+      <c r="G505" s="6" t="n"/>
+      <c r="H505" s="6" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I505" s="6" t="inlineStr"/>
+      <c r="J505" s="6" t="inlineStr"/>
+      <c r="K505" s="6" t="inlineStr"/>
+      <c r="L505" s="6" t="n"/>
+      <c r="M505" s="6" t="n"/>
+      <c r="N505" s="6" t="n"/>
+      <c r="O505" s="6" t="n"/>
+      <c r="P505" s="6" t="n"/>
+      <c r="Q505" s="6" t="n"/>
+      <c r="R505" s="6" t="n"/>
+      <c r="S505" s="6" t="n"/>
+      <c r="T505" s="6" t="n"/>
+      <c r="U505" s="6" t="n"/>
+      <c r="V505" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W505" s="6" t="inlineStr"/>
+      <c r="X505" s="6" t="n"/>
+      <c r="Y505" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z505" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA505" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB505" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC505" s="6" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD505" s="6" t="n"/>
+      <c r="AE505" s="6" t="n"/>
+      <c r="AF505" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B506" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C506" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D506" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E506" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F506" s="4" t="n"/>
+      <c r="G506" s="4" t="n"/>
+      <c r="H506" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I506" s="4" t="inlineStr"/>
+      <c r="J506" s="4" t="inlineStr"/>
+      <c r="K506" s="4" t="inlineStr"/>
+      <c r="L506" s="4" t="n"/>
+      <c r="M506" s="4" t="n"/>
+      <c r="N506" s="4" t="n"/>
+      <c r="O506" s="4" t="n"/>
+      <c r="P506" s="4" t="n"/>
+      <c r="Q506" s="4" t="n"/>
+      <c r="R506" s="4" t="n"/>
+      <c r="S506" s="4" t="n"/>
+      <c r="T506" s="4" t="n"/>
+      <c r="U506" s="4" t="n"/>
+      <c r="V506" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W506" s="4" t="inlineStr"/>
+      <c r="X506" s="4" t="n"/>
+      <c r="Y506" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z506" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA506" s="4" t="n"/>
+      <c r="AB506" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC506" s="4" t="n"/>
+      <c r="AD506" s="4" t="n"/>
+      <c r="AE506" s="4" t="n"/>
+      <c r="AF506" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-02</t>
+        </is>
+      </c>
+      <c r="B507" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C507" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D507" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E507" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F507" s="6" t="n"/>
+      <c r="G507" s="6" t="n"/>
+      <c r="H507" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I507" s="6" t="inlineStr"/>
+      <c r="J507" s="6" t="inlineStr"/>
+      <c r="K507" s="6" t="inlineStr"/>
+      <c r="L507" s="6" t="n"/>
+      <c r="M507" s="6" t="n"/>
+      <c r="N507" s="6" t="n"/>
+      <c r="O507" s="6" t="n"/>
+      <c r="P507" s="6" t="n"/>
+      <c r="Q507" s="6" t="n"/>
+      <c r="R507" s="6" t="n"/>
+      <c r="S507" s="6" t="n"/>
+      <c r="T507" s="6" t="n"/>
+      <c r="U507" s="6" t="n"/>
+      <c r="V507" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W507" s="6" t="inlineStr"/>
+      <c r="X507" s="6" t="n"/>
+      <c r="Y507" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z507" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA507" s="6" t="n"/>
+      <c r="AB507" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC507" s="6" t="n"/>
+      <c r="AD507" s="6" t="n"/>
+      <c r="AE507" s="6" t="n"/>
+      <c r="AF507" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-03
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF507"/>
+  <dimension ref="A1:AF542"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -40458,6 +40458,2758 @@
         <v>1</v>
       </c>
     </row>
+    <row r="508">
+      <c r="A508" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B508" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C508" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D508" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E508" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F508" s="4" t="n"/>
+      <c r="G508" s="4" t="n"/>
+      <c r="H508" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I508" s="4" t="inlineStr"/>
+      <c r="J508" s="4" t="inlineStr"/>
+      <c r="K508" s="4" t="inlineStr"/>
+      <c r="L508" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M508" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N508" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O508" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P508" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q508" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R508" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S508" s="4" t="n"/>
+      <c r="T508" s="4" t="n"/>
+      <c r="U508" s="4" t="n"/>
+      <c r="V508" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W508" s="4" t="inlineStr"/>
+      <c r="X508" s="4" t="n"/>
+      <c r="Y508" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z508" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA508" s="4" t="n"/>
+      <c r="AB508" s="4" t="n"/>
+      <c r="AC508" s="4" t="n"/>
+      <c r="AD508" s="4" t="n"/>
+      <c r="AE508" s="4" t="n"/>
+      <c r="AF508" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B509" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C509" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D509" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E509" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F509" s="6" t="n"/>
+      <c r="G509" s="6" t="n"/>
+      <c r="H509" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I509" s="6" t="inlineStr"/>
+      <c r="J509" s="6" t="inlineStr"/>
+      <c r="K509" s="6" t="inlineStr"/>
+      <c r="L509" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M509" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N509" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O509" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P509" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q509" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R509" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S509" s="6" t="n"/>
+      <c r="T509" s="6" t="n"/>
+      <c r="U509" s="6" t="n"/>
+      <c r="V509" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W509" s="6" t="inlineStr"/>
+      <c r="X509" s="6" t="n"/>
+      <c r="Y509" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z509" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA509" s="6" t="n"/>
+      <c r="AB509" s="6" t="n"/>
+      <c r="AC509" s="6" t="n"/>
+      <c r="AD509" s="6" t="n"/>
+      <c r="AE509" s="6" t="n"/>
+      <c r="AF509" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B510" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C510" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D510" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E510" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F510" s="4" t="n"/>
+      <c r="G510" s="4" t="n"/>
+      <c r="H510" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I510" s="4" t="inlineStr"/>
+      <c r="J510" s="4" t="inlineStr"/>
+      <c r="K510" s="4" t="inlineStr"/>
+      <c r="L510" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M510" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N510" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O510" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P510" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q510" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R510" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S510" s="4" t="n"/>
+      <c r="T510" s="4" t="n"/>
+      <c r="U510" s="4" t="n"/>
+      <c r="V510" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W510" s="4" t="inlineStr"/>
+      <c r="X510" s="4" t="n"/>
+      <c r="Y510" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z510" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA510" s="4" t="n"/>
+      <c r="AB510" s="4" t="n"/>
+      <c r="AC510" s="4" t="n"/>
+      <c r="AD510" s="4" t="n"/>
+      <c r="AE510" s="4" t="n"/>
+      <c r="AF510" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B511" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C511" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D511" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E511" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F511" s="6" t="n"/>
+      <c r="G511" s="6" t="n"/>
+      <c r="H511" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I511" s="6" t="inlineStr"/>
+      <c r="J511" s="6" t="inlineStr"/>
+      <c r="K511" s="6" t="inlineStr"/>
+      <c r="L511" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M511" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N511" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O511" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P511" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q511" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R511" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S511" s="6" t="n"/>
+      <c r="T511" s="6" t="n"/>
+      <c r="U511" s="6" t="n"/>
+      <c r="V511" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W511" s="6" t="inlineStr"/>
+      <c r="X511" s="6" t="n"/>
+      <c r="Y511" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z511" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA511" s="6" t="n"/>
+      <c r="AB511" s="6" t="n"/>
+      <c r="AC511" s="6" t="n"/>
+      <c r="AD511" s="6" t="n"/>
+      <c r="AE511" s="6" t="n"/>
+      <c r="AF511" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B512" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C512" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D512" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E512" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F512" s="4" t="n"/>
+      <c r="G512" s="4" t="n"/>
+      <c r="H512" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I512" s="4" t="inlineStr"/>
+      <c r="J512" s="4" t="inlineStr"/>
+      <c r="K512" s="4" t="inlineStr"/>
+      <c r="L512" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M512" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N512" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O512" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P512" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q512" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R512" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S512" s="4" t="n"/>
+      <c r="T512" s="4" t="n"/>
+      <c r="U512" s="4" t="n"/>
+      <c r="V512" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W512" s="4" t="inlineStr"/>
+      <c r="X512" s="4" t="n"/>
+      <c r="Y512" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z512" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA512" s="4" t="n"/>
+      <c r="AB512" s="4" t="n"/>
+      <c r="AC512" s="4" t="n"/>
+      <c r="AD512" s="4" t="n"/>
+      <c r="AE512" s="4" t="n"/>
+      <c r="AF512" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B513" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C513" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D513" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E513" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F513" s="6" t="n"/>
+      <c r="G513" s="6" t="n"/>
+      <c r="H513" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I513" s="6" t="inlineStr"/>
+      <c r="J513" s="6" t="inlineStr"/>
+      <c r="K513" s="6" t="inlineStr"/>
+      <c r="L513" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M513" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N513" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O513" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P513" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q513" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R513" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S513" s="6" t="n"/>
+      <c r="T513" s="6" t="n"/>
+      <c r="U513" s="6" t="n"/>
+      <c r="V513" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W513" s="6" t="inlineStr"/>
+      <c r="X513" s="6" t="n"/>
+      <c r="Y513" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z513" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA513" s="6" t="n"/>
+      <c r="AB513" s="6" t="n"/>
+      <c r="AC513" s="6" t="n"/>
+      <c r="AD513" s="6" t="n"/>
+      <c r="AE513" s="6" t="n"/>
+      <c r="AF513" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B514" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C514" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D514" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E514" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F514" s="4" t="n"/>
+      <c r="G514" s="4" t="n"/>
+      <c r="H514" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I514" s="4" t="inlineStr"/>
+      <c r="J514" s="4" t="inlineStr"/>
+      <c r="K514" s="4" t="inlineStr"/>
+      <c r="L514" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M514" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N514" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O514" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P514" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q514" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R514" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S514" s="4" t="n"/>
+      <c r="T514" s="4" t="n"/>
+      <c r="U514" s="4" t="n"/>
+      <c r="V514" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W514" s="4" t="inlineStr"/>
+      <c r="X514" s="4" t="n"/>
+      <c r="Y514" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z514" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA514" s="4" t="n"/>
+      <c r="AB514" s="4" t="n"/>
+      <c r="AC514" s="4" t="n"/>
+      <c r="AD514" s="4" t="n"/>
+      <c r="AE514" s="4" t="n"/>
+      <c r="AF514" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B515" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C515" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D515" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E515" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F515" s="6" t="n"/>
+      <c r="G515" s="6" t="n"/>
+      <c r="H515" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I515" s="6" t="inlineStr"/>
+      <c r="J515" s="6" t="inlineStr"/>
+      <c r="K515" s="6" t="inlineStr"/>
+      <c r="L515" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M515" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N515" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O515" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P515" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q515" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R515" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S515" s="6" t="n"/>
+      <c r="T515" s="6" t="n"/>
+      <c r="U515" s="6" t="n"/>
+      <c r="V515" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W515" s="6" t="inlineStr"/>
+      <c r="X515" s="6" t="n"/>
+      <c r="Y515" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z515" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA515" s="6" t="n"/>
+      <c r="AB515" s="6" t="n"/>
+      <c r="AC515" s="6" t="n"/>
+      <c r="AD515" s="6" t="n"/>
+      <c r="AE515" s="6" t="n"/>
+      <c r="AF515" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B516" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C516" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D516" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E516" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F516" s="4" t="n"/>
+      <c r="G516" s="4" t="n"/>
+      <c r="H516" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I516" s="4" t="inlineStr"/>
+      <c r="J516" s="4" t="inlineStr"/>
+      <c r="K516" s="4" t="inlineStr"/>
+      <c r="L516" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M516" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N516" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O516" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P516" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q516" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R516" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S516" s="4" t="n"/>
+      <c r="T516" s="4" t="n"/>
+      <c r="U516" s="4" t="n"/>
+      <c r="V516" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W516" s="4" t="inlineStr"/>
+      <c r="X516" s="4" t="n"/>
+      <c r="Y516" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z516" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA516" s="4" t="n"/>
+      <c r="AB516" s="4" t="n"/>
+      <c r="AC516" s="4" t="n"/>
+      <c r="AD516" s="4" t="n"/>
+      <c r="AE516" s="4" t="n"/>
+      <c r="AF516" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B517" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C517" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D517" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E517" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F517" s="6" t="n"/>
+      <c r="G517" s="6" t="n"/>
+      <c r="H517" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I517" s="6" t="inlineStr"/>
+      <c r="J517" s="6" t="inlineStr"/>
+      <c r="K517" s="6" t="inlineStr"/>
+      <c r="L517" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M517" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N517" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O517" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P517" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q517" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R517" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S517" s="6" t="n"/>
+      <c r="T517" s="6" t="n"/>
+      <c r="U517" s="6" t="n"/>
+      <c r="V517" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W517" s="6" t="inlineStr"/>
+      <c r="X517" s="6" t="n"/>
+      <c r="Y517" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z517" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA517" s="6" t="n"/>
+      <c r="AB517" s="6" t="n"/>
+      <c r="AC517" s="6" t="n"/>
+      <c r="AD517" s="6" t="n"/>
+      <c r="AE517" s="6" t="n"/>
+      <c r="AF517" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B518" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C518" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D518" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E518" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F518" s="4" t="n"/>
+      <c r="G518" s="4" t="n"/>
+      <c r="H518" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I518" s="4" t="inlineStr"/>
+      <c r="J518" s="4" t="inlineStr"/>
+      <c r="K518" s="4" t="inlineStr"/>
+      <c r="L518" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M518" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N518" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O518" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P518" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q518" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R518" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S518" s="4" t="n"/>
+      <c r="T518" s="4" t="n"/>
+      <c r="U518" s="4" t="n"/>
+      <c r="V518" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W518" s="4" t="inlineStr"/>
+      <c r="X518" s="4" t="n"/>
+      <c r="Y518" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z518" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA518" s="4" t="n"/>
+      <c r="AB518" s="4" t="n"/>
+      <c r="AC518" s="4" t="n"/>
+      <c r="AD518" s="4" t="n"/>
+      <c r="AE518" s="4" t="n"/>
+      <c r="AF518" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B519" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C519" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D519" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E519" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F519" s="6" t="n"/>
+      <c r="G519" s="6" t="n"/>
+      <c r="H519" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I519" s="6" t="inlineStr"/>
+      <c r="J519" s="6" t="inlineStr"/>
+      <c r="K519" s="6" t="inlineStr"/>
+      <c r="L519" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M519" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N519" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O519" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P519" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q519" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R519" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S519" s="6" t="n"/>
+      <c r="T519" s="6" t="n"/>
+      <c r="U519" s="6" t="n"/>
+      <c r="V519" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W519" s="6" t="inlineStr"/>
+      <c r="X519" s="6" t="n"/>
+      <c r="Y519" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z519" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA519" s="6" t="n"/>
+      <c r="AB519" s="6" t="n"/>
+      <c r="AC519" s="6" t="n"/>
+      <c r="AD519" s="6" t="n"/>
+      <c r="AE519" s="6" t="n"/>
+      <c r="AF519" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B520" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C520" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D520" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E520" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F520" s="4" t="n"/>
+      <c r="G520" s="4" t="n"/>
+      <c r="H520" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I520" s="4" t="inlineStr"/>
+      <c r="J520" s="4" t="inlineStr"/>
+      <c r="K520" s="4" t="inlineStr"/>
+      <c r="L520" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M520" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N520" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O520" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P520" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q520" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R520" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S520" s="4" t="n"/>
+      <c r="T520" s="4" t="n"/>
+      <c r="U520" s="4" t="n"/>
+      <c r="V520" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W520" s="4" t="inlineStr"/>
+      <c r="X520" s="4" t="n"/>
+      <c r="Y520" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z520" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA520" s="4" t="n"/>
+      <c r="AB520" s="4" t="n"/>
+      <c r="AC520" s="4" t="n"/>
+      <c r="AD520" s="4" t="n"/>
+      <c r="AE520" s="4" t="n"/>
+      <c r="AF520" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B521" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C521" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D521" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E521" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F521" s="6" t="n"/>
+      <c r="G521" s="6" t="n"/>
+      <c r="H521" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I521" s="6" t="inlineStr"/>
+      <c r="J521" s="6" t="inlineStr"/>
+      <c r="K521" s="6" t="inlineStr"/>
+      <c r="L521" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M521" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N521" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O521" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P521" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q521" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R521" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S521" s="6" t="n"/>
+      <c r="T521" s="6" t="n"/>
+      <c r="U521" s="6" t="n"/>
+      <c r="V521" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W521" s="6" t="inlineStr"/>
+      <c r="X521" s="6" t="n"/>
+      <c r="Y521" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z521" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA521" s="6" t="n"/>
+      <c r="AB521" s="6" t="n"/>
+      <c r="AC521" s="6" t="n"/>
+      <c r="AD521" s="6" t="n"/>
+      <c r="AE521" s="6" t="n"/>
+      <c r="AF521" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B522" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C522" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D522" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E522" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F522" s="4" t="n"/>
+      <c r="G522" s="4" t="n"/>
+      <c r="H522" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I522" s="4" t="inlineStr"/>
+      <c r="J522" s="4" t="inlineStr"/>
+      <c r="K522" s="4" t="inlineStr"/>
+      <c r="L522" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M522" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N522" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O522" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P522" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q522" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R522" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S522" s="4" t="n"/>
+      <c r="T522" s="4" t="n"/>
+      <c r="U522" s="4" t="n"/>
+      <c r="V522" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W522" s="4" t="inlineStr"/>
+      <c r="X522" s="4" t="n"/>
+      <c r="Y522" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z522" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA522" s="4" t="n"/>
+      <c r="AB522" s="4" t="n"/>
+      <c r="AC522" s="4" t="n"/>
+      <c r="AD522" s="4" t="n"/>
+      <c r="AE522" s="4" t="n"/>
+      <c r="AF522" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B523" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C523" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D523" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E523" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F523" s="6" t="n"/>
+      <c r="G523" s="6" t="n"/>
+      <c r="H523" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I523" s="6" t="inlineStr"/>
+      <c r="J523" s="6" t="inlineStr"/>
+      <c r="K523" s="6" t="inlineStr"/>
+      <c r="L523" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M523" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N523" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O523" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P523" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q523" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R523" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S523" s="6" t="n"/>
+      <c r="T523" s="6" t="n"/>
+      <c r="U523" s="6" t="n"/>
+      <c r="V523" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W523" s="6" t="inlineStr"/>
+      <c r="X523" s="6" t="n"/>
+      <c r="Y523" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z523" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA523" s="6" t="n"/>
+      <c r="AB523" s="6" t="n"/>
+      <c r="AC523" s="6" t="n"/>
+      <c r="AD523" s="6" t="n"/>
+      <c r="AE523" s="6" t="n"/>
+      <c r="AF523" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B524" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C524" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D524" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E524" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F524" s="4" t="n"/>
+      <c r="G524" s="4" t="n"/>
+      <c r="H524" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I524" s="4" t="inlineStr"/>
+      <c r="J524" s="4" t="inlineStr"/>
+      <c r="K524" s="4" t="inlineStr"/>
+      <c r="L524" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="M524" s="4" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N524" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O524" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P524" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q524" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R524" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S524" s="4" t="n"/>
+      <c r="T524" s="4" t="n"/>
+      <c r="U524" s="4" t="n"/>
+      <c r="V524" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W524" s="4" t="inlineStr"/>
+      <c r="X524" s="4" t="n"/>
+      <c r="Y524" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z524" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA524" s="4" t="n"/>
+      <c r="AB524" s="4" t="n"/>
+      <c r="AC524" s="4" t="n"/>
+      <c r="AD524" s="4" t="n"/>
+      <c r="AE524" s="4" t="n"/>
+      <c r="AF524" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B525" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C525" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D525" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E525" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F525" s="6" t="n"/>
+      <c r="G525" s="6" t="n"/>
+      <c r="H525" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I525" s="6" t="inlineStr"/>
+      <c r="J525" s="6" t="inlineStr"/>
+      <c r="K525" s="6" t="inlineStr"/>
+      <c r="L525" s="6" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M525" s="6" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N525" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O525" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P525" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q525" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R525" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S525" s="6" t="n"/>
+      <c r="T525" s="6" t="n"/>
+      <c r="U525" s="6" t="n"/>
+      <c r="V525" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W525" s="6" t="inlineStr"/>
+      <c r="X525" s="6" t="n"/>
+      <c r="Y525" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z525" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA525" s="6" t="n"/>
+      <c r="AB525" s="6" t="n"/>
+      <c r="AC525" s="6" t="n"/>
+      <c r="AD525" s="6" t="n"/>
+      <c r="AE525" s="6" t="n"/>
+      <c r="AF525" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B526" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C526" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D526" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E526" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F526" s="4" t="n"/>
+      <c r="G526" s="4" t="n"/>
+      <c r="H526" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I526" s="4" t="inlineStr"/>
+      <c r="J526" s="4" t="inlineStr"/>
+      <c r="K526" s="4" t="inlineStr"/>
+      <c r="L526" s="4" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M526" s="4" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N526" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O526" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P526" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q526" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R526" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S526" s="4" t="n"/>
+      <c r="T526" s="4" t="n"/>
+      <c r="U526" s="4" t="n"/>
+      <c r="V526" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W526" s="4" t="inlineStr"/>
+      <c r="X526" s="4" t="n"/>
+      <c r="Y526" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z526" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA526" s="4" t="n"/>
+      <c r="AB526" s="4" t="n"/>
+      <c r="AC526" s="4" t="n"/>
+      <c r="AD526" s="4" t="n"/>
+      <c r="AE526" s="4" t="n"/>
+      <c r="AF526" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B527" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C527" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D527" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E527" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F527" s="6" t="n"/>
+      <c r="G527" s="6" t="n"/>
+      <c r="H527" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I527" s="6" t="inlineStr"/>
+      <c r="J527" s="6" t="inlineStr"/>
+      <c r="K527" s="6" t="inlineStr"/>
+      <c r="L527" s="6" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M527" s="6" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N527" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O527" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P527" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q527" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R527" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S527" s="6" t="n"/>
+      <c r="T527" s="6" t="n"/>
+      <c r="U527" s="6" t="n"/>
+      <c r="V527" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W527" s="6" t="inlineStr"/>
+      <c r="X527" s="6" t="n"/>
+      <c r="Y527" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z527" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA527" s="6" t="n"/>
+      <c r="AB527" s="6" t="n"/>
+      <c r="AC527" s="6" t="n"/>
+      <c r="AD527" s="6" t="n"/>
+      <c r="AE527" s="6" t="n"/>
+      <c r="AF527" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B528" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C528" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D528" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E528" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F528" s="4" t="n"/>
+      <c r="G528" s="4" t="n"/>
+      <c r="H528" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I528" s="4" t="inlineStr"/>
+      <c r="J528" s="4" t="inlineStr"/>
+      <c r="K528" s="4" t="inlineStr"/>
+      <c r="L528" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M528" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N528" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O528" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P528" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q528" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R528" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S528" s="4" t="n"/>
+      <c r="T528" s="4" t="n"/>
+      <c r="U528" s="4" t="n"/>
+      <c r="V528" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W528" s="4" t="inlineStr"/>
+      <c r="X528" s="4" t="n"/>
+      <c r="Y528" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z528" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA528" s="4" t="n"/>
+      <c r="AB528" s="4" t="n"/>
+      <c r="AC528" s="4" t="n"/>
+      <c r="AD528" s="4" t="n"/>
+      <c r="AE528" s="4" t="n"/>
+      <c r="AF528" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B529" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C529" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D529" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E529" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F529" s="6" t="n"/>
+      <c r="G529" s="6" t="n"/>
+      <c r="H529" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I529" s="6" t="inlineStr"/>
+      <c r="J529" s="6" t="inlineStr"/>
+      <c r="K529" s="6" t="inlineStr"/>
+      <c r="L529" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M529" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N529" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O529" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P529" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q529" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R529" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S529" s="6" t="n"/>
+      <c r="T529" s="6" t="n"/>
+      <c r="U529" s="6" t="n"/>
+      <c r="V529" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W529" s="6" t="inlineStr"/>
+      <c r="X529" s="6" t="n"/>
+      <c r="Y529" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z529" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA529" s="6" t="n"/>
+      <c r="AB529" s="6" t="n"/>
+      <c r="AC529" s="6" t="n"/>
+      <c r="AD529" s="6" t="n"/>
+      <c r="AE529" s="6" t="n"/>
+      <c r="AF529" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B530" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C530" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D530" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E530" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F530" s="4" t="n"/>
+      <c r="G530" s="4" t="n"/>
+      <c r="H530" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I530" s="4" t="inlineStr"/>
+      <c r="J530" s="4" t="inlineStr"/>
+      <c r="K530" s="4" t="inlineStr"/>
+      <c r="L530" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M530" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N530" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O530" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P530" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q530" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R530" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S530" s="4" t="n"/>
+      <c r="T530" s="4" t="n"/>
+      <c r="U530" s="4" t="n"/>
+      <c r="V530" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W530" s="4" t="inlineStr"/>
+      <c r="X530" s="4" t="n"/>
+      <c r="Y530" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z530" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA530" s="4" t="n"/>
+      <c r="AB530" s="4" t="n"/>
+      <c r="AC530" s="4" t="n"/>
+      <c r="AD530" s="4" t="n"/>
+      <c r="AE530" s="4" t="n"/>
+      <c r="AF530" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B531" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C531" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D531" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E531" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F531" s="6" t="n"/>
+      <c r="G531" s="6" t="n"/>
+      <c r="H531" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I531" s="6" t="inlineStr"/>
+      <c r="J531" s="6" t="inlineStr"/>
+      <c r="K531" s="6" t="inlineStr"/>
+      <c r="L531" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M531" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N531" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O531" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P531" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q531" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R531" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S531" s="6" t="n"/>
+      <c r="T531" s="6" t="n"/>
+      <c r="U531" s="6" t="n"/>
+      <c r="V531" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W531" s="6" t="inlineStr"/>
+      <c r="X531" s="6" t="n"/>
+      <c r="Y531" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z531" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA531" s="6" t="n"/>
+      <c r="AB531" s="6" t="n"/>
+      <c r="AC531" s="6" t="n"/>
+      <c r="AD531" s="6" t="n"/>
+      <c r="AE531" s="6" t="n"/>
+      <c r="AF531" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B532" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C532" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D532" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E532" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F532" s="4" t="n"/>
+      <c r="G532" s="4" t="n"/>
+      <c r="H532" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I532" s="4" t="inlineStr"/>
+      <c r="J532" s="4" t="inlineStr"/>
+      <c r="K532" s="4" t="inlineStr"/>
+      <c r="L532" s="4" t="n"/>
+      <c r="M532" s="4" t="n"/>
+      <c r="N532" s="4" t="n"/>
+      <c r="O532" s="4" t="n"/>
+      <c r="P532" s="4" t="n"/>
+      <c r="Q532" s="4" t="n"/>
+      <c r="R532" s="4" t="n"/>
+      <c r="S532" s="4" t="n"/>
+      <c r="T532" s="4" t="n"/>
+      <c r="U532" s="4" t="n"/>
+      <c r="V532" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W532" s="4" t="inlineStr"/>
+      <c r="X532" s="4" t="n"/>
+      <c r="Y532" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z532" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA532" s="4" t="n"/>
+      <c r="AB532" s="4" t="n"/>
+      <c r="AC532" s="4" t="n"/>
+      <c r="AD532" s="4" t="n"/>
+      <c r="AE532" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF532" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B533" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C533" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D533" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E533" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F533" s="6" t="n"/>
+      <c r="G533" s="6" t="n"/>
+      <c r="H533" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I533" s="6" t="inlineStr"/>
+      <c r="J533" s="6" t="inlineStr"/>
+      <c r="K533" s="6" t="inlineStr"/>
+      <c r="L533" s="6" t="n"/>
+      <c r="M533" s="6" t="n"/>
+      <c r="N533" s="6" t="n"/>
+      <c r="O533" s="6" t="n"/>
+      <c r="P533" s="6" t="n"/>
+      <c r="Q533" s="6" t="n"/>
+      <c r="R533" s="6" t="n"/>
+      <c r="S533" s="6" t="n"/>
+      <c r="T533" s="6" t="n"/>
+      <c r="U533" s="6" t="n"/>
+      <c r="V533" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W533" s="6" t="inlineStr"/>
+      <c r="X533" s="6" t="n"/>
+      <c r="Y533" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z533" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA533" s="6" t="n"/>
+      <c r="AB533" s="6" t="n"/>
+      <c r="AC533" s="6" t="n"/>
+      <c r="AD533" s="6" t="n"/>
+      <c r="AE533" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF533" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B534" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C534" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D534" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E534" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F534" s="4" t="n"/>
+      <c r="G534" s="4" t="n"/>
+      <c r="H534" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I534" s="4" t="inlineStr"/>
+      <c r="J534" s="4" t="inlineStr"/>
+      <c r="K534" s="4" t="inlineStr"/>
+      <c r="L534" s="4" t="n"/>
+      <c r="M534" s="4" t="n"/>
+      <c r="N534" s="4" t="n"/>
+      <c r="O534" s="4" t="n"/>
+      <c r="P534" s="4" t="n"/>
+      <c r="Q534" s="4" t="n"/>
+      <c r="R534" s="4" t="n"/>
+      <c r="S534" s="4" t="n"/>
+      <c r="T534" s="4" t="n"/>
+      <c r="U534" s="4" t="n"/>
+      <c r="V534" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W534" s="4" t="inlineStr"/>
+      <c r="X534" s="4" t="n"/>
+      <c r="Y534" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z534" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA534" s="4" t="n"/>
+      <c r="AB534" s="4" t="n"/>
+      <c r="AC534" s="4" t="n"/>
+      <c r="AD534" s="4" t="n"/>
+      <c r="AE534" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF534" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B535" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C535" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D535" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E535" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F535" s="6" t="n"/>
+      <c r="G535" s="6" t="n"/>
+      <c r="H535" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I535" s="6" t="inlineStr"/>
+      <c r="J535" s="6" t="inlineStr"/>
+      <c r="K535" s="6" t="inlineStr"/>
+      <c r="L535" s="6" t="n"/>
+      <c r="M535" s="6" t="n"/>
+      <c r="N535" s="6" t="n"/>
+      <c r="O535" s="6" t="n"/>
+      <c r="P535" s="6" t="n"/>
+      <c r="Q535" s="6" t="n"/>
+      <c r="R535" s="6" t="n"/>
+      <c r="S535" s="6" t="n"/>
+      <c r="T535" s="6" t="n"/>
+      <c r="U535" s="6" t="n"/>
+      <c r="V535" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W535" s="6" t="inlineStr"/>
+      <c r="X535" s="6" t="n"/>
+      <c r="Y535" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z535" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA535" s="6" t="n"/>
+      <c r="AB535" s="6" t="n"/>
+      <c r="AC535" s="6" t="n"/>
+      <c r="AD535" s="6" t="n"/>
+      <c r="AE535" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF535" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B536" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C536" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D536" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E536" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F536" s="4" t="n"/>
+      <c r="G536" s="4" t="n"/>
+      <c r="H536" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I536" s="4" t="inlineStr"/>
+      <c r="J536" s="4" t="inlineStr"/>
+      <c r="K536" s="4" t="inlineStr"/>
+      <c r="L536" s="4" t="n"/>
+      <c r="M536" s="4" t="n"/>
+      <c r="N536" s="4" t="n"/>
+      <c r="O536" s="4" t="n"/>
+      <c r="P536" s="4" t="n"/>
+      <c r="Q536" s="4" t="n"/>
+      <c r="R536" s="4" t="n"/>
+      <c r="S536" s="4" t="n"/>
+      <c r="T536" s="4" t="n"/>
+      <c r="U536" s="4" t="n"/>
+      <c r="V536" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W536" s="4" t="inlineStr"/>
+      <c r="X536" s="4" t="n"/>
+      <c r="Y536" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z536" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA536" s="4" t="n"/>
+      <c r="AB536" s="4" t="n"/>
+      <c r="AC536" s="4" t="n"/>
+      <c r="AD536" s="4" t="n"/>
+      <c r="AE536" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF536" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B537" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C537" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D537" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E537" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F537" s="6" t="n"/>
+      <c r="G537" s="6" t="n"/>
+      <c r="H537" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I537" s="6" t="inlineStr"/>
+      <c r="J537" s="6" t="inlineStr"/>
+      <c r="K537" s="6" t="inlineStr"/>
+      <c r="L537" s="6" t="n"/>
+      <c r="M537" s="6" t="n"/>
+      <c r="N537" s="6" t="n"/>
+      <c r="O537" s="6" t="n"/>
+      <c r="P537" s="6" t="n"/>
+      <c r="Q537" s="6" t="n"/>
+      <c r="R537" s="6" t="n"/>
+      <c r="S537" s="6" t="n"/>
+      <c r="T537" s="6" t="n"/>
+      <c r="U537" s="6" t="n"/>
+      <c r="V537" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W537" s="6" t="inlineStr"/>
+      <c r="X537" s="6" t="n"/>
+      <c r="Y537" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z537" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA537" s="6" t="n"/>
+      <c r="AB537" s="6" t="n"/>
+      <c r="AC537" s="6" t="n"/>
+      <c r="AD537" s="6" t="n"/>
+      <c r="AE537" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF537" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B538" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C538" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D538" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E538" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F538" s="4" t="n"/>
+      <c r="G538" s="4" t="n"/>
+      <c r="H538" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I538" s="4" t="inlineStr"/>
+      <c r="J538" s="4" t="inlineStr"/>
+      <c r="K538" s="4" t="inlineStr"/>
+      <c r="L538" s="4" t="n"/>
+      <c r="M538" s="4" t="n"/>
+      <c r="N538" s="4" t="n"/>
+      <c r="O538" s="4" t="n"/>
+      <c r="P538" s="4" t="n"/>
+      <c r="Q538" s="4" t="n"/>
+      <c r="R538" s="4" t="n"/>
+      <c r="S538" s="4" t="n"/>
+      <c r="T538" s="4" t="n"/>
+      <c r="U538" s="4" t="n"/>
+      <c r="V538" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W538" s="4" t="inlineStr"/>
+      <c r="X538" s="4" t="n"/>
+      <c r="Y538" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z538" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA538" s="4" t="n"/>
+      <c r="AB538" s="4" t="n"/>
+      <c r="AC538" s="4" t="n"/>
+      <c r="AD538" s="4" t="n"/>
+      <c r="AE538" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF538" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B539" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C539" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D539" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E539" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F539" s="6" t="n"/>
+      <c r="G539" s="6" t="n"/>
+      <c r="H539" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I539" s="6" t="inlineStr"/>
+      <c r="J539" s="6" t="inlineStr"/>
+      <c r="K539" s="6" t="inlineStr"/>
+      <c r="L539" s="6" t="n"/>
+      <c r="M539" s="6" t="n"/>
+      <c r="N539" s="6" t="n"/>
+      <c r="O539" s="6" t="n"/>
+      <c r="P539" s="6" t="n"/>
+      <c r="Q539" s="6" t="n"/>
+      <c r="R539" s="6" t="n"/>
+      <c r="S539" s="6" t="n"/>
+      <c r="T539" s="6" t="n"/>
+      <c r="U539" s="6" t="n"/>
+      <c r="V539" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W539" s="6" t="inlineStr"/>
+      <c r="X539" s="6" t="n"/>
+      <c r="Y539" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z539" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA539" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB539" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC539" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD539" s="6" t="n"/>
+      <c r="AE539" s="6" t="n"/>
+      <c r="AF539" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B540" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C540" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D540" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E540" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F540" s="4" t="n"/>
+      <c r="G540" s="4" t="n"/>
+      <c r="H540" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I540" s="4" t="inlineStr"/>
+      <c r="J540" s="4" t="inlineStr"/>
+      <c r="K540" s="4" t="inlineStr"/>
+      <c r="L540" s="4" t="n"/>
+      <c r="M540" s="4" t="n"/>
+      <c r="N540" s="4" t="n"/>
+      <c r="O540" s="4" t="n"/>
+      <c r="P540" s="4" t="n"/>
+      <c r="Q540" s="4" t="n"/>
+      <c r="R540" s="4" t="n"/>
+      <c r="S540" s="4" t="n"/>
+      <c r="T540" s="4" t="n"/>
+      <c r="U540" s="4" t="n"/>
+      <c r="V540" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W540" s="4" t="inlineStr"/>
+      <c r="X540" s="4" t="n"/>
+      <c r="Y540" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z540" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA540" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB540" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC540" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD540" s="4" t="n"/>
+      <c r="AE540" s="4" t="n"/>
+      <c r="AF540" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B541" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C541" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D541" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E541" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F541" s="6" t="n"/>
+      <c r="G541" s="6" t="n"/>
+      <c r="H541" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I541" s="6" t="inlineStr"/>
+      <c r="J541" s="6" t="inlineStr"/>
+      <c r="K541" s="6" t="inlineStr"/>
+      <c r="L541" s="6" t="n"/>
+      <c r="M541" s="6" t="n"/>
+      <c r="N541" s="6" t="n"/>
+      <c r="O541" s="6" t="n"/>
+      <c r="P541" s="6" t="n"/>
+      <c r="Q541" s="6" t="n"/>
+      <c r="R541" s="6" t="n"/>
+      <c r="S541" s="6" t="n"/>
+      <c r="T541" s="6" t="n"/>
+      <c r="U541" s="6" t="n"/>
+      <c r="V541" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W541" s="6" t="inlineStr"/>
+      <c r="X541" s="6" t="n"/>
+      <c r="Y541" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z541" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA541" s="6" t="n"/>
+      <c r="AB541" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC541" s="6" t="n"/>
+      <c r="AD541" s="6" t="n"/>
+      <c r="AE541" s="6" t="n"/>
+      <c r="AF541" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-03</t>
+        </is>
+      </c>
+      <c r="B542" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C542" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D542" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E542" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F542" s="4" t="n"/>
+      <c r="G542" s="4" t="n"/>
+      <c r="H542" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I542" s="4" t="inlineStr"/>
+      <c r="J542" s="4" t="inlineStr"/>
+      <c r="K542" s="4" t="inlineStr"/>
+      <c r="L542" s="4" t="n"/>
+      <c r="M542" s="4" t="n"/>
+      <c r="N542" s="4" t="n"/>
+      <c r="O542" s="4" t="n"/>
+      <c r="P542" s="4" t="n"/>
+      <c r="Q542" s="4" t="n"/>
+      <c r="R542" s="4" t="n"/>
+      <c r="S542" s="4" t="n"/>
+      <c r="T542" s="4" t="n"/>
+      <c r="U542" s="4" t="n"/>
+      <c r="V542" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W542" s="4" t="inlineStr"/>
+      <c r="X542" s="4" t="n"/>
+      <c r="Y542" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z542" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA542" s="4" t="n"/>
+      <c r="AB542" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC542" s="4" t="n"/>
+      <c r="AD542" s="4" t="n"/>
+      <c r="AE542" s="4" t="n"/>
+      <c r="AF542" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-04
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF542"/>
+  <dimension ref="A1:AF577"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -43210,6 +43210,2758 @@
         <v>1</v>
       </c>
     </row>
+    <row r="543">
+      <c r="A543" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B543" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C543" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D543" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E543" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F543" s="4" t="n"/>
+      <c r="G543" s="4" t="n"/>
+      <c r="H543" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I543" s="4" t="inlineStr"/>
+      <c r="J543" s="4" t="inlineStr"/>
+      <c r="K543" s="4" t="inlineStr"/>
+      <c r="L543" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M543" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N543" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O543" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P543" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q543" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R543" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S543" s="4" t="n"/>
+      <c r="T543" s="4" t="n"/>
+      <c r="U543" s="4" t="n"/>
+      <c r="V543" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W543" s="4" t="inlineStr"/>
+      <c r="X543" s="4" t="n"/>
+      <c r="Y543" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z543" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA543" s="4" t="n"/>
+      <c r="AB543" s="4" t="n"/>
+      <c r="AC543" s="4" t="n"/>
+      <c r="AD543" s="4" t="n"/>
+      <c r="AE543" s="4" t="n"/>
+      <c r="AF543" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B544" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C544" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D544" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E544" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F544" s="6" t="n"/>
+      <c r="G544" s="6" t="n"/>
+      <c r="H544" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I544" s="6" t="inlineStr"/>
+      <c r="J544" s="6" t="inlineStr"/>
+      <c r="K544" s="6" t="inlineStr"/>
+      <c r="L544" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M544" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N544" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O544" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P544" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q544" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R544" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S544" s="6" t="n"/>
+      <c r="T544" s="6" t="n"/>
+      <c r="U544" s="6" t="n"/>
+      <c r="V544" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W544" s="6" t="inlineStr"/>
+      <c r="X544" s="6" t="n"/>
+      <c r="Y544" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z544" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA544" s="6" t="n"/>
+      <c r="AB544" s="6" t="n"/>
+      <c r="AC544" s="6" t="n"/>
+      <c r="AD544" s="6" t="n"/>
+      <c r="AE544" s="6" t="n"/>
+      <c r="AF544" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B545" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C545" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D545" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E545" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F545" s="4" t="n"/>
+      <c r="G545" s="4" t="n"/>
+      <c r="H545" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I545" s="4" t="inlineStr"/>
+      <c r="J545" s="4" t="inlineStr"/>
+      <c r="K545" s="4" t="inlineStr"/>
+      <c r="L545" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M545" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N545" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O545" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P545" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q545" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R545" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S545" s="4" t="n"/>
+      <c r="T545" s="4" t="n"/>
+      <c r="U545" s="4" t="n"/>
+      <c r="V545" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W545" s="4" t="inlineStr"/>
+      <c r="X545" s="4" t="n"/>
+      <c r="Y545" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z545" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA545" s="4" t="n"/>
+      <c r="AB545" s="4" t="n"/>
+      <c r="AC545" s="4" t="n"/>
+      <c r="AD545" s="4" t="n"/>
+      <c r="AE545" s="4" t="n"/>
+      <c r="AF545" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B546" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C546" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D546" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E546" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F546" s="6" t="n"/>
+      <c r="G546" s="6" t="n"/>
+      <c r="H546" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I546" s="6" t="inlineStr"/>
+      <c r="J546" s="6" t="inlineStr"/>
+      <c r="K546" s="6" t="inlineStr"/>
+      <c r="L546" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M546" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N546" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O546" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P546" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q546" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R546" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S546" s="6" t="n"/>
+      <c r="T546" s="6" t="n"/>
+      <c r="U546" s="6" t="n"/>
+      <c r="V546" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W546" s="6" t="inlineStr"/>
+      <c r="X546" s="6" t="n"/>
+      <c r="Y546" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z546" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA546" s="6" t="n"/>
+      <c r="AB546" s="6" t="n"/>
+      <c r="AC546" s="6" t="n"/>
+      <c r="AD546" s="6" t="n"/>
+      <c r="AE546" s="6" t="n"/>
+      <c r="AF546" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B547" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C547" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D547" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E547" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F547" s="4" t="n"/>
+      <c r="G547" s="4" t="n"/>
+      <c r="H547" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I547" s="4" t="inlineStr"/>
+      <c r="J547" s="4" t="inlineStr"/>
+      <c r="K547" s="4" t="inlineStr"/>
+      <c r="L547" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M547" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N547" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O547" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P547" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q547" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R547" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S547" s="4" t="n"/>
+      <c r="T547" s="4" t="n"/>
+      <c r="U547" s="4" t="n"/>
+      <c r="V547" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W547" s="4" t="inlineStr"/>
+      <c r="X547" s="4" t="n"/>
+      <c r="Y547" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z547" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA547" s="4" t="n"/>
+      <c r="AB547" s="4" t="n"/>
+      <c r="AC547" s="4" t="n"/>
+      <c r="AD547" s="4" t="n"/>
+      <c r="AE547" s="4" t="n"/>
+      <c r="AF547" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B548" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C548" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D548" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E548" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F548" s="6" t="n"/>
+      <c r="G548" s="6" t="n"/>
+      <c r="H548" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I548" s="6" t="inlineStr"/>
+      <c r="J548" s="6" t="inlineStr"/>
+      <c r="K548" s="6" t="inlineStr"/>
+      <c r="L548" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M548" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N548" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O548" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P548" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q548" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R548" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S548" s="6" t="n"/>
+      <c r="T548" s="6" t="n"/>
+      <c r="U548" s="6" t="n"/>
+      <c r="V548" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W548" s="6" t="inlineStr"/>
+      <c r="X548" s="6" t="n"/>
+      <c r="Y548" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z548" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA548" s="6" t="n"/>
+      <c r="AB548" s="6" t="n"/>
+      <c r="AC548" s="6" t="n"/>
+      <c r="AD548" s="6" t="n"/>
+      <c r="AE548" s="6" t="n"/>
+      <c r="AF548" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B549" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C549" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D549" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E549" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F549" s="4" t="n"/>
+      <c r="G549" s="4" t="n"/>
+      <c r="H549" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I549" s="4" t="inlineStr"/>
+      <c r="J549" s="4" t="inlineStr"/>
+      <c r="K549" s="4" t="inlineStr"/>
+      <c r="L549" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M549" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N549" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O549" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P549" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q549" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R549" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S549" s="4" t="n"/>
+      <c r="T549" s="4" t="n"/>
+      <c r="U549" s="4" t="n"/>
+      <c r="V549" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W549" s="4" t="inlineStr"/>
+      <c r="X549" s="4" t="n"/>
+      <c r="Y549" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z549" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA549" s="4" t="n"/>
+      <c r="AB549" s="4" t="n"/>
+      <c r="AC549" s="4" t="n"/>
+      <c r="AD549" s="4" t="n"/>
+      <c r="AE549" s="4" t="n"/>
+      <c r="AF549" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B550" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C550" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D550" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E550" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F550" s="6" t="n"/>
+      <c r="G550" s="6" t="n"/>
+      <c r="H550" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I550" s="6" t="inlineStr"/>
+      <c r="J550" s="6" t="inlineStr"/>
+      <c r="K550" s="6" t="inlineStr"/>
+      <c r="L550" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M550" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N550" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O550" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P550" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q550" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R550" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S550" s="6" t="n"/>
+      <c r="T550" s="6" t="n"/>
+      <c r="U550" s="6" t="n"/>
+      <c r="V550" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W550" s="6" t="inlineStr"/>
+      <c r="X550" s="6" t="n"/>
+      <c r="Y550" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z550" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA550" s="6" t="n"/>
+      <c r="AB550" s="6" t="n"/>
+      <c r="AC550" s="6" t="n"/>
+      <c r="AD550" s="6" t="n"/>
+      <c r="AE550" s="6" t="n"/>
+      <c r="AF550" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B551" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C551" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D551" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E551" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F551" s="4" t="n"/>
+      <c r="G551" s="4" t="n"/>
+      <c r="H551" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I551" s="4" t="inlineStr"/>
+      <c r="J551" s="4" t="inlineStr"/>
+      <c r="K551" s="4" t="inlineStr"/>
+      <c r="L551" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M551" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N551" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O551" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P551" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q551" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R551" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S551" s="4" t="n"/>
+      <c r="T551" s="4" t="n"/>
+      <c r="U551" s="4" t="n"/>
+      <c r="V551" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W551" s="4" t="inlineStr"/>
+      <c r="X551" s="4" t="n"/>
+      <c r="Y551" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z551" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA551" s="4" t="n"/>
+      <c r="AB551" s="4" t="n"/>
+      <c r="AC551" s="4" t="n"/>
+      <c r="AD551" s="4" t="n"/>
+      <c r="AE551" s="4" t="n"/>
+      <c r="AF551" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B552" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C552" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D552" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E552" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F552" s="6" t="n"/>
+      <c r="G552" s="6" t="n"/>
+      <c r="H552" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I552" s="6" t="inlineStr"/>
+      <c r="J552" s="6" t="inlineStr"/>
+      <c r="K552" s="6" t="inlineStr"/>
+      <c r="L552" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M552" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N552" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O552" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P552" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q552" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R552" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S552" s="6" t="n"/>
+      <c r="T552" s="6" t="n"/>
+      <c r="U552" s="6" t="n"/>
+      <c r="V552" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W552" s="6" t="inlineStr"/>
+      <c r="X552" s="6" t="n"/>
+      <c r="Y552" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z552" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA552" s="6" t="n"/>
+      <c r="AB552" s="6" t="n"/>
+      <c r="AC552" s="6" t="n"/>
+      <c r="AD552" s="6" t="n"/>
+      <c r="AE552" s="6" t="n"/>
+      <c r="AF552" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B553" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C553" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D553" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E553" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F553" s="4" t="n"/>
+      <c r="G553" s="4" t="n"/>
+      <c r="H553" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I553" s="4" t="inlineStr"/>
+      <c r="J553" s="4" t="inlineStr"/>
+      <c r="K553" s="4" t="inlineStr"/>
+      <c r="L553" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M553" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N553" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O553" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P553" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q553" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R553" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S553" s="4" t="n"/>
+      <c r="T553" s="4" t="n"/>
+      <c r="U553" s="4" t="n"/>
+      <c r="V553" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W553" s="4" t="inlineStr"/>
+      <c r="X553" s="4" t="n"/>
+      <c r="Y553" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z553" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA553" s="4" t="n"/>
+      <c r="AB553" s="4" t="n"/>
+      <c r="AC553" s="4" t="n"/>
+      <c r="AD553" s="4" t="n"/>
+      <c r="AE553" s="4" t="n"/>
+      <c r="AF553" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B554" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C554" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D554" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E554" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F554" s="6" t="n"/>
+      <c r="G554" s="6" t="n"/>
+      <c r="H554" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I554" s="6" t="inlineStr"/>
+      <c r="J554" s="6" t="inlineStr"/>
+      <c r="K554" s="6" t="inlineStr"/>
+      <c r="L554" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M554" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N554" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O554" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P554" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q554" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R554" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S554" s="6" t="n"/>
+      <c r="T554" s="6" t="n"/>
+      <c r="U554" s="6" t="n"/>
+      <c r="V554" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W554" s="6" t="inlineStr"/>
+      <c r="X554" s="6" t="n"/>
+      <c r="Y554" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z554" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA554" s="6" t="n"/>
+      <c r="AB554" s="6" t="n"/>
+      <c r="AC554" s="6" t="n"/>
+      <c r="AD554" s="6" t="n"/>
+      <c r="AE554" s="6" t="n"/>
+      <c r="AF554" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B555" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C555" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D555" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E555" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F555" s="4" t="n"/>
+      <c r="G555" s="4" t="n"/>
+      <c r="H555" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I555" s="4" t="inlineStr"/>
+      <c r="J555" s="4" t="inlineStr"/>
+      <c r="K555" s="4" t="inlineStr"/>
+      <c r="L555" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M555" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N555" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O555" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P555" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q555" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R555" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S555" s="4" t="n"/>
+      <c r="T555" s="4" t="n"/>
+      <c r="U555" s="4" t="n"/>
+      <c r="V555" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W555" s="4" t="inlineStr"/>
+      <c r="X555" s="4" t="n"/>
+      <c r="Y555" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z555" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA555" s="4" t="n"/>
+      <c r="AB555" s="4" t="n"/>
+      <c r="AC555" s="4" t="n"/>
+      <c r="AD555" s="4" t="n"/>
+      <c r="AE555" s="4" t="n"/>
+      <c r="AF555" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B556" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C556" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D556" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E556" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F556" s="6" t="n"/>
+      <c r="G556" s="6" t="n"/>
+      <c r="H556" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I556" s="6" t="inlineStr"/>
+      <c r="J556" s="6" t="inlineStr"/>
+      <c r="K556" s="6" t="inlineStr"/>
+      <c r="L556" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M556" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N556" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O556" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P556" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q556" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R556" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S556" s="6" t="n"/>
+      <c r="T556" s="6" t="n"/>
+      <c r="U556" s="6" t="n"/>
+      <c r="V556" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W556" s="6" t="inlineStr"/>
+      <c r="X556" s="6" t="n"/>
+      <c r="Y556" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z556" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA556" s="6" t="n"/>
+      <c r="AB556" s="6" t="n"/>
+      <c r="AC556" s="6" t="n"/>
+      <c r="AD556" s="6" t="n"/>
+      <c r="AE556" s="6" t="n"/>
+      <c r="AF556" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B557" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C557" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D557" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E557" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F557" s="4" t="n"/>
+      <c r="G557" s="4" t="n"/>
+      <c r="H557" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I557" s="4" t="inlineStr"/>
+      <c r="J557" s="4" t="inlineStr"/>
+      <c r="K557" s="4" t="inlineStr"/>
+      <c r="L557" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M557" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N557" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O557" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P557" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q557" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R557" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S557" s="4" t="n"/>
+      <c r="T557" s="4" t="n"/>
+      <c r="U557" s="4" t="n"/>
+      <c r="V557" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W557" s="4" t="inlineStr"/>
+      <c r="X557" s="4" t="n"/>
+      <c r="Y557" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z557" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA557" s="4" t="n"/>
+      <c r="AB557" s="4" t="n"/>
+      <c r="AC557" s="4" t="n"/>
+      <c r="AD557" s="4" t="n"/>
+      <c r="AE557" s="4" t="n"/>
+      <c r="AF557" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B558" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C558" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D558" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E558" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F558" s="6" t="n"/>
+      <c r="G558" s="6" t="n"/>
+      <c r="H558" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I558" s="6" t="inlineStr"/>
+      <c r="J558" s="6" t="inlineStr"/>
+      <c r="K558" s="6" t="inlineStr"/>
+      <c r="L558" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M558" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N558" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O558" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P558" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q558" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R558" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S558" s="6" t="n"/>
+      <c r="T558" s="6" t="n"/>
+      <c r="U558" s="6" t="n"/>
+      <c r="V558" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W558" s="6" t="inlineStr"/>
+      <c r="X558" s="6" t="n"/>
+      <c r="Y558" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z558" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA558" s="6" t="n"/>
+      <c r="AB558" s="6" t="n"/>
+      <c r="AC558" s="6" t="n"/>
+      <c r="AD558" s="6" t="n"/>
+      <c r="AE558" s="6" t="n"/>
+      <c r="AF558" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B559" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C559" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D559" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E559" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F559" s="4" t="n"/>
+      <c r="G559" s="4" t="n"/>
+      <c r="H559" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I559" s="4" t="inlineStr"/>
+      <c r="J559" s="4" t="inlineStr"/>
+      <c r="K559" s="4" t="inlineStr"/>
+      <c r="L559" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="M559" s="4" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N559" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O559" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P559" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q559" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R559" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S559" s="4" t="n"/>
+      <c r="T559" s="4" t="n"/>
+      <c r="U559" s="4" t="n"/>
+      <c r="V559" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W559" s="4" t="inlineStr"/>
+      <c r="X559" s="4" t="n"/>
+      <c r="Y559" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z559" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA559" s="4" t="n"/>
+      <c r="AB559" s="4" t="n"/>
+      <c r="AC559" s="4" t="n"/>
+      <c r="AD559" s="4" t="n"/>
+      <c r="AE559" s="4" t="n"/>
+      <c r="AF559" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B560" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C560" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D560" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E560" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F560" s="6" t="n"/>
+      <c r="G560" s="6" t="n"/>
+      <c r="H560" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I560" s="6" t="inlineStr"/>
+      <c r="J560" s="6" t="inlineStr"/>
+      <c r="K560" s="6" t="inlineStr"/>
+      <c r="L560" s="6" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M560" s="6" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N560" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O560" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P560" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q560" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R560" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S560" s="6" t="n"/>
+      <c r="T560" s="6" t="n"/>
+      <c r="U560" s="6" t="n"/>
+      <c r="V560" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W560" s="6" t="inlineStr"/>
+      <c r="X560" s="6" t="n"/>
+      <c r="Y560" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z560" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA560" s="6" t="n"/>
+      <c r="AB560" s="6" t="n"/>
+      <c r="AC560" s="6" t="n"/>
+      <c r="AD560" s="6" t="n"/>
+      <c r="AE560" s="6" t="n"/>
+      <c r="AF560" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B561" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C561" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D561" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E561" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F561" s="4" t="n"/>
+      <c r="G561" s="4" t="n"/>
+      <c r="H561" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I561" s="4" t="inlineStr"/>
+      <c r="J561" s="4" t="inlineStr"/>
+      <c r="K561" s="4" t="inlineStr"/>
+      <c r="L561" s="4" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M561" s="4" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N561" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O561" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P561" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q561" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R561" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S561" s="4" t="n"/>
+      <c r="T561" s="4" t="n"/>
+      <c r="U561" s="4" t="n"/>
+      <c r="V561" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W561" s="4" t="inlineStr"/>
+      <c r="X561" s="4" t="n"/>
+      <c r="Y561" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z561" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA561" s="4" t="n"/>
+      <c r="AB561" s="4" t="n"/>
+      <c r="AC561" s="4" t="n"/>
+      <c r="AD561" s="4" t="n"/>
+      <c r="AE561" s="4" t="n"/>
+      <c r="AF561" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B562" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C562" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D562" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E562" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F562" s="6" t="n"/>
+      <c r="G562" s="6" t="n"/>
+      <c r="H562" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I562" s="6" t="inlineStr"/>
+      <c r="J562" s="6" t="inlineStr"/>
+      <c r="K562" s="6" t="inlineStr"/>
+      <c r="L562" s="6" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M562" s="6" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N562" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O562" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P562" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q562" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R562" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S562" s="6" t="n"/>
+      <c r="T562" s="6" t="n"/>
+      <c r="U562" s="6" t="n"/>
+      <c r="V562" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W562" s="6" t="inlineStr"/>
+      <c r="X562" s="6" t="n"/>
+      <c r="Y562" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z562" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA562" s="6" t="n"/>
+      <c r="AB562" s="6" t="n"/>
+      <c r="AC562" s="6" t="n"/>
+      <c r="AD562" s="6" t="n"/>
+      <c r="AE562" s="6" t="n"/>
+      <c r="AF562" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B563" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C563" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D563" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E563" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F563" s="4" t="n"/>
+      <c r="G563" s="4" t="n"/>
+      <c r="H563" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I563" s="4" t="inlineStr"/>
+      <c r="J563" s="4" t="inlineStr"/>
+      <c r="K563" s="4" t="inlineStr"/>
+      <c r="L563" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M563" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N563" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O563" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P563" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q563" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R563" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S563" s="4" t="n"/>
+      <c r="T563" s="4" t="n"/>
+      <c r="U563" s="4" t="n"/>
+      <c r="V563" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W563" s="4" t="inlineStr"/>
+      <c r="X563" s="4" t="n"/>
+      <c r="Y563" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z563" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA563" s="4" t="n"/>
+      <c r="AB563" s="4" t="n"/>
+      <c r="AC563" s="4" t="n"/>
+      <c r="AD563" s="4" t="n"/>
+      <c r="AE563" s="4" t="n"/>
+      <c r="AF563" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B564" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C564" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D564" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E564" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F564" s="6" t="n"/>
+      <c r="G564" s="6" t="n"/>
+      <c r="H564" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I564" s="6" t="inlineStr"/>
+      <c r="J564" s="6" t="inlineStr"/>
+      <c r="K564" s="6" t="inlineStr"/>
+      <c r="L564" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M564" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N564" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O564" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P564" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q564" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R564" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S564" s="6" t="n"/>
+      <c r="T564" s="6" t="n"/>
+      <c r="U564" s="6" t="n"/>
+      <c r="V564" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W564" s="6" t="inlineStr"/>
+      <c r="X564" s="6" t="n"/>
+      <c r="Y564" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z564" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA564" s="6" t="n"/>
+      <c r="AB564" s="6" t="n"/>
+      <c r="AC564" s="6" t="n"/>
+      <c r="AD564" s="6" t="n"/>
+      <c r="AE564" s="6" t="n"/>
+      <c r="AF564" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B565" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C565" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D565" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E565" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F565" s="4" t="n"/>
+      <c r="G565" s="4" t="n"/>
+      <c r="H565" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I565" s="4" t="inlineStr"/>
+      <c r="J565" s="4" t="inlineStr"/>
+      <c r="K565" s="4" t="inlineStr"/>
+      <c r="L565" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M565" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N565" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O565" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P565" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q565" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R565" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S565" s="4" t="n"/>
+      <c r="T565" s="4" t="n"/>
+      <c r="U565" s="4" t="n"/>
+      <c r="V565" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W565" s="4" t="inlineStr"/>
+      <c r="X565" s="4" t="n"/>
+      <c r="Y565" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z565" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA565" s="4" t="n"/>
+      <c r="AB565" s="4" t="n"/>
+      <c r="AC565" s="4" t="n"/>
+      <c r="AD565" s="4" t="n"/>
+      <c r="AE565" s="4" t="n"/>
+      <c r="AF565" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B566" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C566" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D566" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E566" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F566" s="6" t="n"/>
+      <c r="G566" s="6" t="n"/>
+      <c r="H566" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I566" s="6" t="inlineStr"/>
+      <c r="J566" s="6" t="inlineStr"/>
+      <c r="K566" s="6" t="inlineStr"/>
+      <c r="L566" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M566" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N566" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O566" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P566" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q566" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R566" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S566" s="6" t="n"/>
+      <c r="T566" s="6" t="n"/>
+      <c r="U566" s="6" t="n"/>
+      <c r="V566" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W566" s="6" t="inlineStr"/>
+      <c r="X566" s="6" t="n"/>
+      <c r="Y566" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z566" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA566" s="6" t="n"/>
+      <c r="AB566" s="6" t="n"/>
+      <c r="AC566" s="6" t="n"/>
+      <c r="AD566" s="6" t="n"/>
+      <c r="AE566" s="6" t="n"/>
+      <c r="AF566" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B567" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C567" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D567" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E567" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F567" s="4" t="n"/>
+      <c r="G567" s="4" t="n"/>
+      <c r="H567" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I567" s="4" t="inlineStr"/>
+      <c r="J567" s="4" t="inlineStr"/>
+      <c r="K567" s="4" t="inlineStr"/>
+      <c r="L567" s="4" t="n"/>
+      <c r="M567" s="4" t="n"/>
+      <c r="N567" s="4" t="n"/>
+      <c r="O567" s="4" t="n"/>
+      <c r="P567" s="4" t="n"/>
+      <c r="Q567" s="4" t="n"/>
+      <c r="R567" s="4" t="n"/>
+      <c r="S567" s="4" t="n"/>
+      <c r="T567" s="4" t="n"/>
+      <c r="U567" s="4" t="n"/>
+      <c r="V567" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W567" s="4" t="inlineStr"/>
+      <c r="X567" s="4" t="n"/>
+      <c r="Y567" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z567" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA567" s="4" t="n"/>
+      <c r="AB567" s="4" t="n"/>
+      <c r="AC567" s="4" t="n"/>
+      <c r="AD567" s="4" t="n"/>
+      <c r="AE567" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF567" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B568" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C568" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D568" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E568" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F568" s="6" t="n"/>
+      <c r="G568" s="6" t="n"/>
+      <c r="H568" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I568" s="6" t="inlineStr"/>
+      <c r="J568" s="6" t="inlineStr"/>
+      <c r="K568" s="6" t="inlineStr"/>
+      <c r="L568" s="6" t="n"/>
+      <c r="M568" s="6" t="n"/>
+      <c r="N568" s="6" t="n"/>
+      <c r="O568" s="6" t="n"/>
+      <c r="P568" s="6" t="n"/>
+      <c r="Q568" s="6" t="n"/>
+      <c r="R568" s="6" t="n"/>
+      <c r="S568" s="6" t="n"/>
+      <c r="T568" s="6" t="n"/>
+      <c r="U568" s="6" t="n"/>
+      <c r="V568" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W568" s="6" t="inlineStr"/>
+      <c r="X568" s="6" t="n"/>
+      <c r="Y568" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z568" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA568" s="6" t="n"/>
+      <c r="AB568" s="6" t="n"/>
+      <c r="AC568" s="6" t="n"/>
+      <c r="AD568" s="6" t="n"/>
+      <c r="AE568" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF568" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B569" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C569" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D569" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E569" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F569" s="4" t="n"/>
+      <c r="G569" s="4" t="n"/>
+      <c r="H569" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I569" s="4" t="inlineStr"/>
+      <c r="J569" s="4" t="inlineStr"/>
+      <c r="K569" s="4" t="inlineStr"/>
+      <c r="L569" s="4" t="n"/>
+      <c r="M569" s="4" t="n"/>
+      <c r="N569" s="4" t="n"/>
+      <c r="O569" s="4" t="n"/>
+      <c r="P569" s="4" t="n"/>
+      <c r="Q569" s="4" t="n"/>
+      <c r="R569" s="4" t="n"/>
+      <c r="S569" s="4" t="n"/>
+      <c r="T569" s="4" t="n"/>
+      <c r="U569" s="4" t="n"/>
+      <c r="V569" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W569" s="4" t="inlineStr"/>
+      <c r="X569" s="4" t="n"/>
+      <c r="Y569" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z569" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA569" s="4" t="n"/>
+      <c r="AB569" s="4" t="n"/>
+      <c r="AC569" s="4" t="n"/>
+      <c r="AD569" s="4" t="n"/>
+      <c r="AE569" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF569" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B570" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C570" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D570" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E570" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F570" s="6" t="n"/>
+      <c r="G570" s="6" t="n"/>
+      <c r="H570" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I570" s="6" t="inlineStr"/>
+      <c r="J570" s="6" t="inlineStr"/>
+      <c r="K570" s="6" t="inlineStr"/>
+      <c r="L570" s="6" t="n"/>
+      <c r="M570" s="6" t="n"/>
+      <c r="N570" s="6" t="n"/>
+      <c r="O570" s="6" t="n"/>
+      <c r="P570" s="6" t="n"/>
+      <c r="Q570" s="6" t="n"/>
+      <c r="R570" s="6" t="n"/>
+      <c r="S570" s="6" t="n"/>
+      <c r="T570" s="6" t="n"/>
+      <c r="U570" s="6" t="n"/>
+      <c r="V570" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W570" s="6" t="inlineStr"/>
+      <c r="X570" s="6" t="n"/>
+      <c r="Y570" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z570" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA570" s="6" t="n"/>
+      <c r="AB570" s="6" t="n"/>
+      <c r="AC570" s="6" t="n"/>
+      <c r="AD570" s="6" t="n"/>
+      <c r="AE570" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF570" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B571" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C571" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D571" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E571" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F571" s="4" t="n"/>
+      <c r="G571" s="4" t="n"/>
+      <c r="H571" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I571" s="4" t="inlineStr"/>
+      <c r="J571" s="4" t="inlineStr"/>
+      <c r="K571" s="4" t="inlineStr"/>
+      <c r="L571" s="4" t="n"/>
+      <c r="M571" s="4" t="n"/>
+      <c r="N571" s="4" t="n"/>
+      <c r="O571" s="4" t="n"/>
+      <c r="P571" s="4" t="n"/>
+      <c r="Q571" s="4" t="n"/>
+      <c r="R571" s="4" t="n"/>
+      <c r="S571" s="4" t="n"/>
+      <c r="T571" s="4" t="n"/>
+      <c r="U571" s="4" t="n"/>
+      <c r="V571" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W571" s="4" t="inlineStr"/>
+      <c r="X571" s="4" t="n"/>
+      <c r="Y571" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z571" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA571" s="4" t="n"/>
+      <c r="AB571" s="4" t="n"/>
+      <c r="AC571" s="4" t="n"/>
+      <c r="AD571" s="4" t="n"/>
+      <c r="AE571" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF571" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B572" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C572" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D572" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E572" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F572" s="6" t="n"/>
+      <c r="G572" s="6" t="n"/>
+      <c r="H572" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I572" s="6" t="inlineStr"/>
+      <c r="J572" s="6" t="inlineStr"/>
+      <c r="K572" s="6" t="inlineStr"/>
+      <c r="L572" s="6" t="n"/>
+      <c r="M572" s="6" t="n"/>
+      <c r="N572" s="6" t="n"/>
+      <c r="O572" s="6" t="n"/>
+      <c r="P572" s="6" t="n"/>
+      <c r="Q572" s="6" t="n"/>
+      <c r="R572" s="6" t="n"/>
+      <c r="S572" s="6" t="n"/>
+      <c r="T572" s="6" t="n"/>
+      <c r="U572" s="6" t="n"/>
+      <c r="V572" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W572" s="6" t="inlineStr"/>
+      <c r="X572" s="6" t="n"/>
+      <c r="Y572" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z572" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA572" s="6" t="n"/>
+      <c r="AB572" s="6" t="n"/>
+      <c r="AC572" s="6" t="n"/>
+      <c r="AD572" s="6" t="n"/>
+      <c r="AE572" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF572" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B573" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C573" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D573" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E573" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F573" s="4" t="n"/>
+      <c r="G573" s="4" t="n"/>
+      <c r="H573" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I573" s="4" t="inlineStr"/>
+      <c r="J573" s="4" t="inlineStr"/>
+      <c r="K573" s="4" t="inlineStr"/>
+      <c r="L573" s="4" t="n"/>
+      <c r="M573" s="4" t="n"/>
+      <c r="N573" s="4" t="n"/>
+      <c r="O573" s="4" t="n"/>
+      <c r="P573" s="4" t="n"/>
+      <c r="Q573" s="4" t="n"/>
+      <c r="R573" s="4" t="n"/>
+      <c r="S573" s="4" t="n"/>
+      <c r="T573" s="4" t="n"/>
+      <c r="U573" s="4" t="n"/>
+      <c r="V573" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W573" s="4" t="inlineStr"/>
+      <c r="X573" s="4" t="n"/>
+      <c r="Y573" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z573" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA573" s="4" t="n"/>
+      <c r="AB573" s="4" t="n"/>
+      <c r="AC573" s="4" t="n"/>
+      <c r="AD573" s="4" t="n"/>
+      <c r="AE573" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF573" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B574" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C574" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D574" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E574" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F574" s="6" t="n"/>
+      <c r="G574" s="6" t="n"/>
+      <c r="H574" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I574" s="6" t="inlineStr"/>
+      <c r="J574" s="6" t="inlineStr"/>
+      <c r="K574" s="6" t="inlineStr"/>
+      <c r="L574" s="6" t="n"/>
+      <c r="M574" s="6" t="n"/>
+      <c r="N574" s="6" t="n"/>
+      <c r="O574" s="6" t="n"/>
+      <c r="P574" s="6" t="n"/>
+      <c r="Q574" s="6" t="n"/>
+      <c r="R574" s="6" t="n"/>
+      <c r="S574" s="6" t="n"/>
+      <c r="T574" s="6" t="n"/>
+      <c r="U574" s="6" t="n"/>
+      <c r="V574" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W574" s="6" t="inlineStr"/>
+      <c r="X574" s="6" t="n"/>
+      <c r="Y574" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z574" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA574" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB574" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC574" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD574" s="6" t="n"/>
+      <c r="AE574" s="6" t="n"/>
+      <c r="AF574" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B575" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C575" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D575" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E575" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F575" s="4" t="n"/>
+      <c r="G575" s="4" t="n"/>
+      <c r="H575" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I575" s="4" t="inlineStr"/>
+      <c r="J575" s="4" t="inlineStr"/>
+      <c r="K575" s="4" t="inlineStr"/>
+      <c r="L575" s="4" t="n"/>
+      <c r="M575" s="4" t="n"/>
+      <c r="N575" s="4" t="n"/>
+      <c r="O575" s="4" t="n"/>
+      <c r="P575" s="4" t="n"/>
+      <c r="Q575" s="4" t="n"/>
+      <c r="R575" s="4" t="n"/>
+      <c r="S575" s="4" t="n"/>
+      <c r="T575" s="4" t="n"/>
+      <c r="U575" s="4" t="n"/>
+      <c r="V575" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W575" s="4" t="inlineStr"/>
+      <c r="X575" s="4" t="n"/>
+      <c r="Y575" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z575" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA575" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB575" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC575" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD575" s="4" t="n"/>
+      <c r="AE575" s="4" t="n"/>
+      <c r="AF575" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B576" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C576" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D576" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E576" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F576" s="6" t="n"/>
+      <c r="G576" s="6" t="n"/>
+      <c r="H576" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I576" s="6" t="inlineStr"/>
+      <c r="J576" s="6" t="inlineStr"/>
+      <c r="K576" s="6" t="inlineStr"/>
+      <c r="L576" s="6" t="n"/>
+      <c r="M576" s="6" t="n"/>
+      <c r="N576" s="6" t="n"/>
+      <c r="O576" s="6" t="n"/>
+      <c r="P576" s="6" t="n"/>
+      <c r="Q576" s="6" t="n"/>
+      <c r="R576" s="6" t="n"/>
+      <c r="S576" s="6" t="n"/>
+      <c r="T576" s="6" t="n"/>
+      <c r="U576" s="6" t="n"/>
+      <c r="V576" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W576" s="6" t="inlineStr"/>
+      <c r="X576" s="6" t="n"/>
+      <c r="Y576" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z576" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA576" s="6" t="n"/>
+      <c r="AB576" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC576" s="6" t="n"/>
+      <c r="AD576" s="6" t="n"/>
+      <c r="AE576" s="6" t="n"/>
+      <c r="AF576" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-04</t>
+        </is>
+      </c>
+      <c r="B577" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C577" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D577" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E577" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F577" s="4" t="n"/>
+      <c r="G577" s="4" t="n"/>
+      <c r="H577" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I577" s="4" t="inlineStr"/>
+      <c r="J577" s="4" t="inlineStr"/>
+      <c r="K577" s="4" t="inlineStr"/>
+      <c r="L577" s="4" t="n"/>
+      <c r="M577" s="4" t="n"/>
+      <c r="N577" s="4" t="n"/>
+      <c r="O577" s="4" t="n"/>
+      <c r="P577" s="4" t="n"/>
+      <c r="Q577" s="4" t="n"/>
+      <c r="R577" s="4" t="n"/>
+      <c r="S577" s="4" t="n"/>
+      <c r="T577" s="4" t="n"/>
+      <c r="U577" s="4" t="n"/>
+      <c r="V577" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W577" s="4" t="inlineStr"/>
+      <c r="X577" s="4" t="n"/>
+      <c r="Y577" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z577" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA577" s="4" t="n"/>
+      <c r="AB577" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC577" s="4" t="n"/>
+      <c r="AD577" s="4" t="n"/>
+      <c r="AE577" s="4" t="n"/>
+      <c r="AF577" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-05
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF577"/>
+  <dimension ref="A1:AF612"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -45962,6 +45962,2758 @@
         <v>1</v>
       </c>
     </row>
+    <row r="578">
+      <c r="A578" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B578" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C578" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D578" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E578" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F578" s="4" t="n"/>
+      <c r="G578" s="4" t="n"/>
+      <c r="H578" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I578" s="4" t="inlineStr"/>
+      <c r="J578" s="4" t="inlineStr"/>
+      <c r="K578" s="4" t="inlineStr"/>
+      <c r="L578" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M578" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N578" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O578" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P578" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q578" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R578" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S578" s="4" t="n"/>
+      <c r="T578" s="4" t="n"/>
+      <c r="U578" s="4" t="n"/>
+      <c r="V578" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W578" s="4" t="inlineStr"/>
+      <c r="X578" s="4" t="n"/>
+      <c r="Y578" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z578" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA578" s="4" t="n"/>
+      <c r="AB578" s="4" t="n"/>
+      <c r="AC578" s="4" t="n"/>
+      <c r="AD578" s="4" t="n"/>
+      <c r="AE578" s="4" t="n"/>
+      <c r="AF578" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="579">
+      <c r="A579" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B579" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C579" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D579" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E579" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F579" s="6" t="n"/>
+      <c r="G579" s="6" t="n"/>
+      <c r="H579" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I579" s="6" t="inlineStr"/>
+      <c r="J579" s="6" t="inlineStr"/>
+      <c r="K579" s="6" t="inlineStr"/>
+      <c r="L579" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M579" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N579" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O579" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P579" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q579" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R579" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S579" s="6" t="n"/>
+      <c r="T579" s="6" t="n"/>
+      <c r="U579" s="6" t="n"/>
+      <c r="V579" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W579" s="6" t="inlineStr"/>
+      <c r="X579" s="6" t="n"/>
+      <c r="Y579" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z579" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA579" s="6" t="n"/>
+      <c r="AB579" s="6" t="n"/>
+      <c r="AC579" s="6" t="n"/>
+      <c r="AD579" s="6" t="n"/>
+      <c r="AE579" s="6" t="n"/>
+      <c r="AF579" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="580">
+      <c r="A580" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B580" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C580" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D580" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E580" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F580" s="4" t="n"/>
+      <c r="G580" s="4" t="n"/>
+      <c r="H580" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I580" s="4" t="inlineStr"/>
+      <c r="J580" s="4" t="inlineStr"/>
+      <c r="K580" s="4" t="inlineStr"/>
+      <c r="L580" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M580" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N580" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O580" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P580" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q580" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R580" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S580" s="4" t="n"/>
+      <c r="T580" s="4" t="n"/>
+      <c r="U580" s="4" t="n"/>
+      <c r="V580" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W580" s="4" t="inlineStr"/>
+      <c r="X580" s="4" t="n"/>
+      <c r="Y580" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z580" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA580" s="4" t="n"/>
+      <c r="AB580" s="4" t="n"/>
+      <c r="AC580" s="4" t="n"/>
+      <c r="AD580" s="4" t="n"/>
+      <c r="AE580" s="4" t="n"/>
+      <c r="AF580" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="581">
+      <c r="A581" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B581" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C581" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D581" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E581" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F581" s="6" t="n"/>
+      <c r="G581" s="6" t="n"/>
+      <c r="H581" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I581" s="6" t="inlineStr"/>
+      <c r="J581" s="6" t="inlineStr"/>
+      <c r="K581" s="6" t="inlineStr"/>
+      <c r="L581" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M581" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N581" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O581" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P581" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q581" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R581" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S581" s="6" t="n"/>
+      <c r="T581" s="6" t="n"/>
+      <c r="U581" s="6" t="n"/>
+      <c r="V581" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W581" s="6" t="inlineStr"/>
+      <c r="X581" s="6" t="n"/>
+      <c r="Y581" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z581" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA581" s="6" t="n"/>
+      <c r="AB581" s="6" t="n"/>
+      <c r="AC581" s="6" t="n"/>
+      <c r="AD581" s="6" t="n"/>
+      <c r="AE581" s="6" t="n"/>
+      <c r="AF581" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="582">
+      <c r="A582" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B582" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C582" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D582" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E582" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F582" s="4" t="n"/>
+      <c r="G582" s="4" t="n"/>
+      <c r="H582" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I582" s="4" t="inlineStr"/>
+      <c r="J582" s="4" t="inlineStr"/>
+      <c r="K582" s="4" t="inlineStr"/>
+      <c r="L582" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M582" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N582" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O582" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P582" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q582" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R582" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S582" s="4" t="n"/>
+      <c r="T582" s="4" t="n"/>
+      <c r="U582" s="4" t="n"/>
+      <c r="V582" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W582" s="4" t="inlineStr"/>
+      <c r="X582" s="4" t="n"/>
+      <c r="Y582" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z582" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA582" s="4" t="n"/>
+      <c r="AB582" s="4" t="n"/>
+      <c r="AC582" s="4" t="n"/>
+      <c r="AD582" s="4" t="n"/>
+      <c r="AE582" s="4" t="n"/>
+      <c r="AF582" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="583">
+      <c r="A583" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B583" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C583" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D583" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E583" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F583" s="6" t="n"/>
+      <c r="G583" s="6" t="n"/>
+      <c r="H583" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I583" s="6" t="inlineStr"/>
+      <c r="J583" s="6" t="inlineStr"/>
+      <c r="K583" s="6" t="inlineStr"/>
+      <c r="L583" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M583" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N583" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O583" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P583" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q583" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R583" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S583" s="6" t="n"/>
+      <c r="T583" s="6" t="n"/>
+      <c r="U583" s="6" t="n"/>
+      <c r="V583" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W583" s="6" t="inlineStr"/>
+      <c r="X583" s="6" t="n"/>
+      <c r="Y583" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z583" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA583" s="6" t="n"/>
+      <c r="AB583" s="6" t="n"/>
+      <c r="AC583" s="6" t="n"/>
+      <c r="AD583" s="6" t="n"/>
+      <c r="AE583" s="6" t="n"/>
+      <c r="AF583" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="584">
+      <c r="A584" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B584" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C584" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D584" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E584" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F584" s="4" t="n"/>
+      <c r="G584" s="4" t="n"/>
+      <c r="H584" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I584" s="4" t="inlineStr"/>
+      <c r="J584" s="4" t="inlineStr"/>
+      <c r="K584" s="4" t="inlineStr"/>
+      <c r="L584" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M584" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N584" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O584" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P584" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q584" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R584" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S584" s="4" t="n"/>
+      <c r="T584" s="4" t="n"/>
+      <c r="U584" s="4" t="n"/>
+      <c r="V584" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W584" s="4" t="inlineStr"/>
+      <c r="X584" s="4" t="n"/>
+      <c r="Y584" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z584" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA584" s="4" t="n"/>
+      <c r="AB584" s="4" t="n"/>
+      <c r="AC584" s="4" t="n"/>
+      <c r="AD584" s="4" t="n"/>
+      <c r="AE584" s="4" t="n"/>
+      <c r="AF584" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="585">
+      <c r="A585" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B585" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C585" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D585" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E585" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F585" s="6" t="n"/>
+      <c r="G585" s="6" t="n"/>
+      <c r="H585" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I585" s="6" t="inlineStr"/>
+      <c r="J585" s="6" t="inlineStr"/>
+      <c r="K585" s="6" t="inlineStr"/>
+      <c r="L585" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M585" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N585" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O585" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P585" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q585" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R585" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S585" s="6" t="n"/>
+      <c r="T585" s="6" t="n"/>
+      <c r="U585" s="6" t="n"/>
+      <c r="V585" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W585" s="6" t="inlineStr"/>
+      <c r="X585" s="6" t="n"/>
+      <c r="Y585" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z585" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA585" s="6" t="n"/>
+      <c r="AB585" s="6" t="n"/>
+      <c r="AC585" s="6" t="n"/>
+      <c r="AD585" s="6" t="n"/>
+      <c r="AE585" s="6" t="n"/>
+      <c r="AF585" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="586">
+      <c r="A586" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B586" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C586" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D586" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E586" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F586" s="4" t="n"/>
+      <c r="G586" s="4" t="n"/>
+      <c r="H586" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I586" s="4" t="inlineStr"/>
+      <c r="J586" s="4" t="inlineStr"/>
+      <c r="K586" s="4" t="inlineStr"/>
+      <c r="L586" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M586" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N586" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O586" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P586" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q586" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R586" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S586" s="4" t="n"/>
+      <c r="T586" s="4" t="n"/>
+      <c r="U586" s="4" t="n"/>
+      <c r="V586" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W586" s="4" t="inlineStr"/>
+      <c r="X586" s="4" t="n"/>
+      <c r="Y586" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z586" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA586" s="4" t="n"/>
+      <c r="AB586" s="4" t="n"/>
+      <c r="AC586" s="4" t="n"/>
+      <c r="AD586" s="4" t="n"/>
+      <c r="AE586" s="4" t="n"/>
+      <c r="AF586" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="587">
+      <c r="A587" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B587" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C587" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D587" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E587" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F587" s="6" t="n"/>
+      <c r="G587" s="6" t="n"/>
+      <c r="H587" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I587" s="6" t="inlineStr"/>
+      <c r="J587" s="6" t="inlineStr"/>
+      <c r="K587" s="6" t="inlineStr"/>
+      <c r="L587" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M587" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N587" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O587" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P587" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q587" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R587" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S587" s="6" t="n"/>
+      <c r="T587" s="6" t="n"/>
+      <c r="U587" s="6" t="n"/>
+      <c r="V587" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W587" s="6" t="inlineStr"/>
+      <c r="X587" s="6" t="n"/>
+      <c r="Y587" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z587" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA587" s="6" t="n"/>
+      <c r="AB587" s="6" t="n"/>
+      <c r="AC587" s="6" t="n"/>
+      <c r="AD587" s="6" t="n"/>
+      <c r="AE587" s="6" t="n"/>
+      <c r="AF587" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="588">
+      <c r="A588" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B588" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C588" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D588" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E588" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F588" s="4" t="n"/>
+      <c r="G588" s="4" t="n"/>
+      <c r="H588" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I588" s="4" t="inlineStr"/>
+      <c r="J588" s="4" t="inlineStr"/>
+      <c r="K588" s="4" t="inlineStr"/>
+      <c r="L588" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M588" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N588" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O588" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P588" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q588" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R588" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S588" s="4" t="n"/>
+      <c r="T588" s="4" t="n"/>
+      <c r="U588" s="4" t="n"/>
+      <c r="V588" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W588" s="4" t="inlineStr"/>
+      <c r="X588" s="4" t="n"/>
+      <c r="Y588" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z588" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA588" s="4" t="n"/>
+      <c r="AB588" s="4" t="n"/>
+      <c r="AC588" s="4" t="n"/>
+      <c r="AD588" s="4" t="n"/>
+      <c r="AE588" s="4" t="n"/>
+      <c r="AF588" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="589">
+      <c r="A589" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B589" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C589" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D589" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E589" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F589" s="6" t="n"/>
+      <c r="G589" s="6" t="n"/>
+      <c r="H589" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I589" s="6" t="inlineStr"/>
+      <c r="J589" s="6" t="inlineStr"/>
+      <c r="K589" s="6" t="inlineStr"/>
+      <c r="L589" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M589" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N589" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O589" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P589" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q589" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R589" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S589" s="6" t="n"/>
+      <c r="T589" s="6" t="n"/>
+      <c r="U589" s="6" t="n"/>
+      <c r="V589" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W589" s="6" t="inlineStr"/>
+      <c r="X589" s="6" t="n"/>
+      <c r="Y589" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z589" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA589" s="6" t="n"/>
+      <c r="AB589" s="6" t="n"/>
+      <c r="AC589" s="6" t="n"/>
+      <c r="AD589" s="6" t="n"/>
+      <c r="AE589" s="6" t="n"/>
+      <c r="AF589" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="590">
+      <c r="A590" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B590" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C590" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D590" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E590" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F590" s="4" t="n"/>
+      <c r="G590" s="4" t="n"/>
+      <c r="H590" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I590" s="4" t="inlineStr"/>
+      <c r="J590" s="4" t="inlineStr"/>
+      <c r="K590" s="4" t="inlineStr"/>
+      <c r="L590" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M590" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N590" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O590" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P590" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q590" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R590" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S590" s="4" t="n"/>
+      <c r="T590" s="4" t="n"/>
+      <c r="U590" s="4" t="n"/>
+      <c r="V590" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W590" s="4" t="inlineStr"/>
+      <c r="X590" s="4" t="n"/>
+      <c r="Y590" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z590" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA590" s="4" t="n"/>
+      <c r="AB590" s="4" t="n"/>
+      <c r="AC590" s="4" t="n"/>
+      <c r="AD590" s="4" t="n"/>
+      <c r="AE590" s="4" t="n"/>
+      <c r="AF590" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B591" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C591" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D591" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E591" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F591" s="6" t="n"/>
+      <c r="G591" s="6" t="n"/>
+      <c r="H591" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I591" s="6" t="inlineStr"/>
+      <c r="J591" s="6" t="inlineStr"/>
+      <c r="K591" s="6" t="inlineStr"/>
+      <c r="L591" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M591" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N591" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O591" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P591" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q591" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R591" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S591" s="6" t="n"/>
+      <c r="T591" s="6" t="n"/>
+      <c r="U591" s="6" t="n"/>
+      <c r="V591" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W591" s="6" t="inlineStr"/>
+      <c r="X591" s="6" t="n"/>
+      <c r="Y591" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z591" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA591" s="6" t="n"/>
+      <c r="AB591" s="6" t="n"/>
+      <c r="AC591" s="6" t="n"/>
+      <c r="AD591" s="6" t="n"/>
+      <c r="AE591" s="6" t="n"/>
+      <c r="AF591" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B592" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C592" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D592" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E592" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F592" s="4" t="n"/>
+      <c r="G592" s="4" t="n"/>
+      <c r="H592" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I592" s="4" t="inlineStr"/>
+      <c r="J592" s="4" t="inlineStr"/>
+      <c r="K592" s="4" t="inlineStr"/>
+      <c r="L592" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M592" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N592" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O592" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P592" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q592" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R592" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S592" s="4" t="n"/>
+      <c r="T592" s="4" t="n"/>
+      <c r="U592" s="4" t="n"/>
+      <c r="V592" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W592" s="4" t="inlineStr"/>
+      <c r="X592" s="4" t="n"/>
+      <c r="Y592" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z592" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA592" s="4" t="n"/>
+      <c r="AB592" s="4" t="n"/>
+      <c r="AC592" s="4" t="n"/>
+      <c r="AD592" s="4" t="n"/>
+      <c r="AE592" s="4" t="n"/>
+      <c r="AF592" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B593" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C593" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D593" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E593" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F593" s="6" t="n"/>
+      <c r="G593" s="6" t="n"/>
+      <c r="H593" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I593" s="6" t="inlineStr"/>
+      <c r="J593" s="6" t="inlineStr"/>
+      <c r="K593" s="6" t="inlineStr"/>
+      <c r="L593" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M593" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N593" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O593" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P593" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q593" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R593" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S593" s="6" t="n"/>
+      <c r="T593" s="6" t="n"/>
+      <c r="U593" s="6" t="n"/>
+      <c r="V593" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W593" s="6" t="inlineStr"/>
+      <c r="X593" s="6" t="n"/>
+      <c r="Y593" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z593" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA593" s="6" t="n"/>
+      <c r="AB593" s="6" t="n"/>
+      <c r="AC593" s="6" t="n"/>
+      <c r="AD593" s="6" t="n"/>
+      <c r="AE593" s="6" t="n"/>
+      <c r="AF593" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B594" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C594" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D594" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E594" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F594" s="4" t="n"/>
+      <c r="G594" s="4" t="n"/>
+      <c r="H594" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I594" s="4" t="inlineStr"/>
+      <c r="J594" s="4" t="inlineStr"/>
+      <c r="K594" s="4" t="inlineStr"/>
+      <c r="L594" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="M594" s="4" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N594" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O594" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P594" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q594" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R594" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S594" s="4" t="n"/>
+      <c r="T594" s="4" t="n"/>
+      <c r="U594" s="4" t="n"/>
+      <c r="V594" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W594" s="4" t="inlineStr"/>
+      <c r="X594" s="4" t="n"/>
+      <c r="Y594" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z594" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA594" s="4" t="n"/>
+      <c r="AB594" s="4" t="n"/>
+      <c r="AC594" s="4" t="n"/>
+      <c r="AD594" s="4" t="n"/>
+      <c r="AE594" s="4" t="n"/>
+      <c r="AF594" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B595" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C595" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D595" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E595" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F595" s="6" t="n"/>
+      <c r="G595" s="6" t="n"/>
+      <c r="H595" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I595" s="6" t="inlineStr"/>
+      <c r="J595" s="6" t="inlineStr"/>
+      <c r="K595" s="6" t="inlineStr"/>
+      <c r="L595" s="6" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M595" s="6" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N595" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O595" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P595" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q595" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R595" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S595" s="6" t="n"/>
+      <c r="T595" s="6" t="n"/>
+      <c r="U595" s="6" t="n"/>
+      <c r="V595" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W595" s="6" t="inlineStr"/>
+      <c r="X595" s="6" t="n"/>
+      <c r="Y595" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z595" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA595" s="6" t="n"/>
+      <c r="AB595" s="6" t="n"/>
+      <c r="AC595" s="6" t="n"/>
+      <c r="AD595" s="6" t="n"/>
+      <c r="AE595" s="6" t="n"/>
+      <c r="AF595" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B596" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C596" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D596" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E596" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F596" s="4" t="n"/>
+      <c r="G596" s="4" t="n"/>
+      <c r="H596" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I596" s="4" t="inlineStr"/>
+      <c r="J596" s="4" t="inlineStr"/>
+      <c r="K596" s="4" t="inlineStr"/>
+      <c r="L596" s="4" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M596" s="4" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N596" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O596" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P596" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q596" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R596" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S596" s="4" t="n"/>
+      <c r="T596" s="4" t="n"/>
+      <c r="U596" s="4" t="n"/>
+      <c r="V596" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W596" s="4" t="inlineStr"/>
+      <c r="X596" s="4" t="n"/>
+      <c r="Y596" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z596" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA596" s="4" t="n"/>
+      <c r="AB596" s="4" t="n"/>
+      <c r="AC596" s="4" t="n"/>
+      <c r="AD596" s="4" t="n"/>
+      <c r="AE596" s="4" t="n"/>
+      <c r="AF596" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B597" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C597" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D597" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E597" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F597" s="6" t="n"/>
+      <c r="G597" s="6" t="n"/>
+      <c r="H597" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I597" s="6" t="inlineStr"/>
+      <c r="J597" s="6" t="inlineStr"/>
+      <c r="K597" s="6" t="inlineStr"/>
+      <c r="L597" s="6" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M597" s="6" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N597" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O597" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P597" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q597" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R597" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S597" s="6" t="n"/>
+      <c r="T597" s="6" t="n"/>
+      <c r="U597" s="6" t="n"/>
+      <c r="V597" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W597" s="6" t="inlineStr"/>
+      <c r="X597" s="6" t="n"/>
+      <c r="Y597" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z597" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA597" s="6" t="n"/>
+      <c r="AB597" s="6" t="n"/>
+      <c r="AC597" s="6" t="n"/>
+      <c r="AD597" s="6" t="n"/>
+      <c r="AE597" s="6" t="n"/>
+      <c r="AF597" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B598" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C598" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D598" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E598" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F598" s="4" t="n"/>
+      <c r="G598" s="4" t="n"/>
+      <c r="H598" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I598" s="4" t="inlineStr"/>
+      <c r="J598" s="4" t="inlineStr"/>
+      <c r="K598" s="4" t="inlineStr"/>
+      <c r="L598" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M598" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N598" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O598" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P598" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q598" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R598" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S598" s="4" t="n"/>
+      <c r="T598" s="4" t="n"/>
+      <c r="U598" s="4" t="n"/>
+      <c r="V598" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W598" s="4" t="inlineStr"/>
+      <c r="X598" s="4" t="n"/>
+      <c r="Y598" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z598" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA598" s="4" t="n"/>
+      <c r="AB598" s="4" t="n"/>
+      <c r="AC598" s="4" t="n"/>
+      <c r="AD598" s="4" t="n"/>
+      <c r="AE598" s="4" t="n"/>
+      <c r="AF598" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B599" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C599" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D599" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E599" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F599" s="6" t="n"/>
+      <c r="G599" s="6" t="n"/>
+      <c r="H599" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I599" s="6" t="inlineStr"/>
+      <c r="J599" s="6" t="inlineStr"/>
+      <c r="K599" s="6" t="inlineStr"/>
+      <c r="L599" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M599" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N599" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O599" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P599" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q599" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R599" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S599" s="6" t="n"/>
+      <c r="T599" s="6" t="n"/>
+      <c r="U599" s="6" t="n"/>
+      <c r="V599" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W599" s="6" t="inlineStr"/>
+      <c r="X599" s="6" t="n"/>
+      <c r="Y599" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z599" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA599" s="6" t="n"/>
+      <c r="AB599" s="6" t="n"/>
+      <c r="AC599" s="6" t="n"/>
+      <c r="AD599" s="6" t="n"/>
+      <c r="AE599" s="6" t="n"/>
+      <c r="AF599" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B600" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C600" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D600" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E600" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F600" s="4" t="n"/>
+      <c r="G600" s="4" t="n"/>
+      <c r="H600" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I600" s="4" t="inlineStr"/>
+      <c r="J600" s="4" t="inlineStr"/>
+      <c r="K600" s="4" t="inlineStr"/>
+      <c r="L600" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M600" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N600" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O600" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P600" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q600" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R600" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S600" s="4" t="n"/>
+      <c r="T600" s="4" t="n"/>
+      <c r="U600" s="4" t="n"/>
+      <c r="V600" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W600" s="4" t="inlineStr"/>
+      <c r="X600" s="4" t="n"/>
+      <c r="Y600" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z600" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA600" s="4" t="n"/>
+      <c r="AB600" s="4" t="n"/>
+      <c r="AC600" s="4" t="n"/>
+      <c r="AD600" s="4" t="n"/>
+      <c r="AE600" s="4" t="n"/>
+      <c r="AF600" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B601" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C601" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D601" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E601" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F601" s="6" t="n"/>
+      <c r="G601" s="6" t="n"/>
+      <c r="H601" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I601" s="6" t="inlineStr"/>
+      <c r="J601" s="6" t="inlineStr"/>
+      <c r="K601" s="6" t="inlineStr"/>
+      <c r="L601" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M601" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N601" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O601" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P601" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q601" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R601" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S601" s="6" t="n"/>
+      <c r="T601" s="6" t="n"/>
+      <c r="U601" s="6" t="n"/>
+      <c r="V601" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W601" s="6" t="inlineStr"/>
+      <c r="X601" s="6" t="n"/>
+      <c r="Y601" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z601" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA601" s="6" t="n"/>
+      <c r="AB601" s="6" t="n"/>
+      <c r="AC601" s="6" t="n"/>
+      <c r="AD601" s="6" t="n"/>
+      <c r="AE601" s="6" t="n"/>
+      <c r="AF601" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B602" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C602" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D602" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E602" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F602" s="4" t="n"/>
+      <c r="G602" s="4" t="n"/>
+      <c r="H602" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I602" s="4" t="inlineStr"/>
+      <c r="J602" s="4" t="inlineStr"/>
+      <c r="K602" s="4" t="inlineStr"/>
+      <c r="L602" s="4" t="n"/>
+      <c r="M602" s="4" t="n"/>
+      <c r="N602" s="4" t="n"/>
+      <c r="O602" s="4" t="n"/>
+      <c r="P602" s="4" t="n"/>
+      <c r="Q602" s="4" t="n"/>
+      <c r="R602" s="4" t="n"/>
+      <c r="S602" s="4" t="n"/>
+      <c r="T602" s="4" t="n"/>
+      <c r="U602" s="4" t="n"/>
+      <c r="V602" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W602" s="4" t="inlineStr"/>
+      <c r="X602" s="4" t="n"/>
+      <c r="Y602" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z602" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA602" s="4" t="n"/>
+      <c r="AB602" s="4" t="n"/>
+      <c r="AC602" s="4" t="n"/>
+      <c r="AD602" s="4" t="n"/>
+      <c r="AE602" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF602" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B603" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C603" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D603" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E603" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F603" s="6" t="n"/>
+      <c r="G603" s="6" t="n"/>
+      <c r="H603" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I603" s="6" t="inlineStr"/>
+      <c r="J603" s="6" t="inlineStr"/>
+      <c r="K603" s="6" t="inlineStr"/>
+      <c r="L603" s="6" t="n"/>
+      <c r="M603" s="6" t="n"/>
+      <c r="N603" s="6" t="n"/>
+      <c r="O603" s="6" t="n"/>
+      <c r="P603" s="6" t="n"/>
+      <c r="Q603" s="6" t="n"/>
+      <c r="R603" s="6" t="n"/>
+      <c r="S603" s="6" t="n"/>
+      <c r="T603" s="6" t="n"/>
+      <c r="U603" s="6" t="n"/>
+      <c r="V603" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W603" s="6" t="inlineStr"/>
+      <c r="X603" s="6" t="n"/>
+      <c r="Y603" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z603" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA603" s="6" t="n"/>
+      <c r="AB603" s="6" t="n"/>
+      <c r="AC603" s="6" t="n"/>
+      <c r="AD603" s="6" t="n"/>
+      <c r="AE603" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF603" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B604" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C604" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D604" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E604" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F604" s="4" t="n"/>
+      <c r="G604" s="4" t="n"/>
+      <c r="H604" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I604" s="4" t="inlineStr"/>
+      <c r="J604" s="4" t="inlineStr"/>
+      <c r="K604" s="4" t="inlineStr"/>
+      <c r="L604" s="4" t="n"/>
+      <c r="M604" s="4" t="n"/>
+      <c r="N604" s="4" t="n"/>
+      <c r="O604" s="4" t="n"/>
+      <c r="P604" s="4" t="n"/>
+      <c r="Q604" s="4" t="n"/>
+      <c r="R604" s="4" t="n"/>
+      <c r="S604" s="4" t="n"/>
+      <c r="T604" s="4" t="n"/>
+      <c r="U604" s="4" t="n"/>
+      <c r="V604" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W604" s="4" t="inlineStr"/>
+      <c r="X604" s="4" t="n"/>
+      <c r="Y604" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z604" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA604" s="4" t="n"/>
+      <c r="AB604" s="4" t="n"/>
+      <c r="AC604" s="4" t="n"/>
+      <c r="AD604" s="4" t="n"/>
+      <c r="AE604" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF604" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B605" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C605" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D605" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E605" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F605" s="6" t="n"/>
+      <c r="G605" s="6" t="n"/>
+      <c r="H605" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I605" s="6" t="inlineStr"/>
+      <c r="J605" s="6" t="inlineStr"/>
+      <c r="K605" s="6" t="inlineStr"/>
+      <c r="L605" s="6" t="n"/>
+      <c r="M605" s="6" t="n"/>
+      <c r="N605" s="6" t="n"/>
+      <c r="O605" s="6" t="n"/>
+      <c r="P605" s="6" t="n"/>
+      <c r="Q605" s="6" t="n"/>
+      <c r="R605" s="6" t="n"/>
+      <c r="S605" s="6" t="n"/>
+      <c r="T605" s="6" t="n"/>
+      <c r="U605" s="6" t="n"/>
+      <c r="V605" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W605" s="6" t="inlineStr"/>
+      <c r="X605" s="6" t="n"/>
+      <c r="Y605" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z605" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA605" s="6" t="n"/>
+      <c r="AB605" s="6" t="n"/>
+      <c r="AC605" s="6" t="n"/>
+      <c r="AD605" s="6" t="n"/>
+      <c r="AE605" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF605" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B606" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C606" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D606" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E606" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F606" s="4" t="n"/>
+      <c r="G606" s="4" t="n"/>
+      <c r="H606" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I606" s="4" t="inlineStr"/>
+      <c r="J606" s="4" t="inlineStr"/>
+      <c r="K606" s="4" t="inlineStr"/>
+      <c r="L606" s="4" t="n"/>
+      <c r="M606" s="4" t="n"/>
+      <c r="N606" s="4" t="n"/>
+      <c r="O606" s="4" t="n"/>
+      <c r="P606" s="4" t="n"/>
+      <c r="Q606" s="4" t="n"/>
+      <c r="R606" s="4" t="n"/>
+      <c r="S606" s="4" t="n"/>
+      <c r="T606" s="4" t="n"/>
+      <c r="U606" s="4" t="n"/>
+      <c r="V606" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W606" s="4" t="inlineStr"/>
+      <c r="X606" s="4" t="n"/>
+      <c r="Y606" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z606" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA606" s="4" t="n"/>
+      <c r="AB606" s="4" t="n"/>
+      <c r="AC606" s="4" t="n"/>
+      <c r="AD606" s="4" t="n"/>
+      <c r="AE606" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF606" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B607" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C607" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D607" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E607" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F607" s="6" t="n"/>
+      <c r="G607" s="6" t="n"/>
+      <c r="H607" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I607" s="6" t="inlineStr"/>
+      <c r="J607" s="6" t="inlineStr"/>
+      <c r="K607" s="6" t="inlineStr"/>
+      <c r="L607" s="6" t="n"/>
+      <c r="M607" s="6" t="n"/>
+      <c r="N607" s="6" t="n"/>
+      <c r="O607" s="6" t="n"/>
+      <c r="P607" s="6" t="n"/>
+      <c r="Q607" s="6" t="n"/>
+      <c r="R607" s="6" t="n"/>
+      <c r="S607" s="6" t="n"/>
+      <c r="T607" s="6" t="n"/>
+      <c r="U607" s="6" t="n"/>
+      <c r="V607" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W607" s="6" t="inlineStr"/>
+      <c r="X607" s="6" t="n"/>
+      <c r="Y607" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z607" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA607" s="6" t="n"/>
+      <c r="AB607" s="6" t="n"/>
+      <c r="AC607" s="6" t="n"/>
+      <c r="AD607" s="6" t="n"/>
+      <c r="AE607" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF607" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B608" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C608" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D608" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E608" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F608" s="4" t="n"/>
+      <c r="G608" s="4" t="n"/>
+      <c r="H608" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I608" s="4" t="inlineStr"/>
+      <c r="J608" s="4" t="inlineStr"/>
+      <c r="K608" s="4" t="inlineStr"/>
+      <c r="L608" s="4" t="n"/>
+      <c r="M608" s="4" t="n"/>
+      <c r="N608" s="4" t="n"/>
+      <c r="O608" s="4" t="n"/>
+      <c r="P608" s="4" t="n"/>
+      <c r="Q608" s="4" t="n"/>
+      <c r="R608" s="4" t="n"/>
+      <c r="S608" s="4" t="n"/>
+      <c r="T608" s="4" t="n"/>
+      <c r="U608" s="4" t="n"/>
+      <c r="V608" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W608" s="4" t="inlineStr"/>
+      <c r="X608" s="4" t="n"/>
+      <c r="Y608" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z608" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA608" s="4" t="n"/>
+      <c r="AB608" s="4" t="n"/>
+      <c r="AC608" s="4" t="n"/>
+      <c r="AD608" s="4" t="n"/>
+      <c r="AE608" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF608" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B609" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C609" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D609" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E609" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F609" s="6" t="n"/>
+      <c r="G609" s="6" t="n"/>
+      <c r="H609" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I609" s="6" t="inlineStr"/>
+      <c r="J609" s="6" t="inlineStr"/>
+      <c r="K609" s="6" t="inlineStr"/>
+      <c r="L609" s="6" t="n"/>
+      <c r="M609" s="6" t="n"/>
+      <c r="N609" s="6" t="n"/>
+      <c r="O609" s="6" t="n"/>
+      <c r="P609" s="6" t="n"/>
+      <c r="Q609" s="6" t="n"/>
+      <c r="R609" s="6" t="n"/>
+      <c r="S609" s="6" t="n"/>
+      <c r="T609" s="6" t="n"/>
+      <c r="U609" s="6" t="n"/>
+      <c r="V609" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W609" s="6" t="inlineStr"/>
+      <c r="X609" s="6" t="n"/>
+      <c r="Y609" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z609" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA609" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB609" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC609" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD609" s="6" t="n"/>
+      <c r="AE609" s="6" t="n"/>
+      <c r="AF609" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B610" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C610" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D610" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E610" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F610" s="4" t="n"/>
+      <c r="G610" s="4" t="n"/>
+      <c r="H610" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I610" s="4" t="inlineStr"/>
+      <c r="J610" s="4" t="inlineStr"/>
+      <c r="K610" s="4" t="inlineStr"/>
+      <c r="L610" s="4" t="n"/>
+      <c r="M610" s="4" t="n"/>
+      <c r="N610" s="4" t="n"/>
+      <c r="O610" s="4" t="n"/>
+      <c r="P610" s="4" t="n"/>
+      <c r="Q610" s="4" t="n"/>
+      <c r="R610" s="4" t="n"/>
+      <c r="S610" s="4" t="n"/>
+      <c r="T610" s="4" t="n"/>
+      <c r="U610" s="4" t="n"/>
+      <c r="V610" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W610" s="4" t="inlineStr"/>
+      <c r="X610" s="4" t="n"/>
+      <c r="Y610" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z610" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA610" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB610" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC610" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD610" s="4" t="n"/>
+      <c r="AE610" s="4" t="n"/>
+      <c r="AF610" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B611" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C611" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D611" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E611" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F611" s="6" t="n"/>
+      <c r="G611" s="6" t="n"/>
+      <c r="H611" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I611" s="6" t="inlineStr"/>
+      <c r="J611" s="6" t="inlineStr"/>
+      <c r="K611" s="6" t="inlineStr"/>
+      <c r="L611" s="6" t="n"/>
+      <c r="M611" s="6" t="n"/>
+      <c r="N611" s="6" t="n"/>
+      <c r="O611" s="6" t="n"/>
+      <c r="P611" s="6" t="n"/>
+      <c r="Q611" s="6" t="n"/>
+      <c r="R611" s="6" t="n"/>
+      <c r="S611" s="6" t="n"/>
+      <c r="T611" s="6" t="n"/>
+      <c r="U611" s="6" t="n"/>
+      <c r="V611" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W611" s="6" t="inlineStr"/>
+      <c r="X611" s="6" t="n"/>
+      <c r="Y611" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z611" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA611" s="6" t="n"/>
+      <c r="AB611" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC611" s="6" t="n"/>
+      <c r="AD611" s="6" t="n"/>
+      <c r="AE611" s="6" t="n"/>
+      <c r="AF611" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="B612" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C612" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D612" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E612" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F612" s="4" t="n"/>
+      <c r="G612" s="4" t="n"/>
+      <c r="H612" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I612" s="4" t="inlineStr"/>
+      <c r="J612" s="4" t="inlineStr"/>
+      <c r="K612" s="4" t="inlineStr"/>
+      <c r="L612" s="4" t="n"/>
+      <c r="M612" s="4" t="n"/>
+      <c r="N612" s="4" t="n"/>
+      <c r="O612" s="4" t="n"/>
+      <c r="P612" s="4" t="n"/>
+      <c r="Q612" s="4" t="n"/>
+      <c r="R612" s="4" t="n"/>
+      <c r="S612" s="4" t="n"/>
+      <c r="T612" s="4" t="n"/>
+      <c r="U612" s="4" t="n"/>
+      <c r="V612" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W612" s="4" t="inlineStr"/>
+      <c r="X612" s="4" t="n"/>
+      <c r="Y612" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z612" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA612" s="4" t="n"/>
+      <c r="AB612" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC612" s="4" t="n"/>
+      <c r="AD612" s="4" t="n"/>
+      <c r="AE612" s="4" t="n"/>
+      <c r="AF612" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-06
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF612"/>
+  <dimension ref="A1:AF647"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -48714,6 +48714,2758 @@
         <v>1</v>
       </c>
     </row>
+    <row r="613">
+      <c r="A613" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B613" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C613" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D613" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E613" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F613" s="4" t="n"/>
+      <c r="G613" s="4" t="n"/>
+      <c r="H613" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I613" s="4" t="inlineStr"/>
+      <c r="J613" s="4" t="inlineStr"/>
+      <c r="K613" s="4" t="inlineStr"/>
+      <c r="L613" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M613" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N613" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O613" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P613" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q613" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R613" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S613" s="4" t="n"/>
+      <c r="T613" s="4" t="n"/>
+      <c r="U613" s="4" t="n"/>
+      <c r="V613" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W613" s="4" t="inlineStr"/>
+      <c r="X613" s="4" t="n"/>
+      <c r="Y613" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z613" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA613" s="4" t="n"/>
+      <c r="AB613" s="4" t="n"/>
+      <c r="AC613" s="4" t="n"/>
+      <c r="AD613" s="4" t="n"/>
+      <c r="AE613" s="4" t="n"/>
+      <c r="AF613" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B614" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C614" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D614" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E614" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F614" s="6" t="n"/>
+      <c r="G614" s="6" t="n"/>
+      <c r="H614" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I614" s="6" t="inlineStr"/>
+      <c r="J614" s="6" t="inlineStr"/>
+      <c r="K614" s="6" t="inlineStr"/>
+      <c r="L614" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M614" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N614" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O614" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P614" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q614" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R614" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S614" s="6" t="n"/>
+      <c r="T614" s="6" t="n"/>
+      <c r="U614" s="6" t="n"/>
+      <c r="V614" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W614" s="6" t="inlineStr"/>
+      <c r="X614" s="6" t="n"/>
+      <c r="Y614" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z614" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA614" s="6" t="n"/>
+      <c r="AB614" s="6" t="n"/>
+      <c r="AC614" s="6" t="n"/>
+      <c r="AD614" s="6" t="n"/>
+      <c r="AE614" s="6" t="n"/>
+      <c r="AF614" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B615" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C615" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D615" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E615" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F615" s="4" t="n"/>
+      <c r="G615" s="4" t="n"/>
+      <c r="H615" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I615" s="4" t="inlineStr"/>
+      <c r="J615" s="4" t="inlineStr"/>
+      <c r="K615" s="4" t="inlineStr"/>
+      <c r="L615" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M615" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N615" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O615" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P615" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q615" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R615" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S615" s="4" t="n"/>
+      <c r="T615" s="4" t="n"/>
+      <c r="U615" s="4" t="n"/>
+      <c r="V615" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W615" s="4" t="inlineStr"/>
+      <c r="X615" s="4" t="n"/>
+      <c r="Y615" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z615" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA615" s="4" t="n"/>
+      <c r="AB615" s="4" t="n"/>
+      <c r="AC615" s="4" t="n"/>
+      <c r="AD615" s="4" t="n"/>
+      <c r="AE615" s="4" t="n"/>
+      <c r="AF615" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B616" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C616" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D616" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E616" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F616" s="6" t="n"/>
+      <c r="G616" s="6" t="n"/>
+      <c r="H616" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I616" s="6" t="inlineStr"/>
+      <c r="J616" s="6" t="inlineStr"/>
+      <c r="K616" s="6" t="inlineStr"/>
+      <c r="L616" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M616" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N616" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O616" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P616" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q616" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R616" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S616" s="6" t="n"/>
+      <c r="T616" s="6" t="n"/>
+      <c r="U616" s="6" t="n"/>
+      <c r="V616" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W616" s="6" t="inlineStr"/>
+      <c r="X616" s="6" t="n"/>
+      <c r="Y616" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z616" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA616" s="6" t="n"/>
+      <c r="AB616" s="6" t="n"/>
+      <c r="AC616" s="6" t="n"/>
+      <c r="AD616" s="6" t="n"/>
+      <c r="AE616" s="6" t="n"/>
+      <c r="AF616" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B617" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C617" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D617" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E617" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F617" s="4" t="n"/>
+      <c r="G617" s="4" t="n"/>
+      <c r="H617" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I617" s="4" t="inlineStr"/>
+      <c r="J617" s="4" t="inlineStr"/>
+      <c r="K617" s="4" t="inlineStr"/>
+      <c r="L617" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M617" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N617" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O617" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P617" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q617" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R617" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S617" s="4" t="n"/>
+      <c r="T617" s="4" t="n"/>
+      <c r="U617" s="4" t="n"/>
+      <c r="V617" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W617" s="4" t="inlineStr"/>
+      <c r="X617" s="4" t="n"/>
+      <c r="Y617" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z617" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA617" s="4" t="n"/>
+      <c r="AB617" s="4" t="n"/>
+      <c r="AC617" s="4" t="n"/>
+      <c r="AD617" s="4" t="n"/>
+      <c r="AE617" s="4" t="n"/>
+      <c r="AF617" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B618" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C618" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D618" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E618" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F618" s="6" t="n"/>
+      <c r="G618" s="6" t="n"/>
+      <c r="H618" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I618" s="6" t="inlineStr"/>
+      <c r="J618" s="6" t="inlineStr"/>
+      <c r="K618" s="6" t="inlineStr"/>
+      <c r="L618" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M618" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N618" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O618" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P618" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q618" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R618" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S618" s="6" t="n"/>
+      <c r="T618" s="6" t="n"/>
+      <c r="U618" s="6" t="n"/>
+      <c r="V618" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W618" s="6" t="inlineStr"/>
+      <c r="X618" s="6" t="n"/>
+      <c r="Y618" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z618" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA618" s="6" t="n"/>
+      <c r="AB618" s="6" t="n"/>
+      <c r="AC618" s="6" t="n"/>
+      <c r="AD618" s="6" t="n"/>
+      <c r="AE618" s="6" t="n"/>
+      <c r="AF618" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B619" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C619" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D619" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E619" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F619" s="4" t="n"/>
+      <c r="G619" s="4" t="n"/>
+      <c r="H619" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I619" s="4" t="inlineStr"/>
+      <c r="J619" s="4" t="inlineStr"/>
+      <c r="K619" s="4" t="inlineStr"/>
+      <c r="L619" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M619" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N619" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O619" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P619" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q619" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R619" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S619" s="4" t="n"/>
+      <c r="T619" s="4" t="n"/>
+      <c r="U619" s="4" t="n"/>
+      <c r="V619" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W619" s="4" t="inlineStr"/>
+      <c r="X619" s="4" t="n"/>
+      <c r="Y619" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z619" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA619" s="4" t="n"/>
+      <c r="AB619" s="4" t="n"/>
+      <c r="AC619" s="4" t="n"/>
+      <c r="AD619" s="4" t="n"/>
+      <c r="AE619" s="4" t="n"/>
+      <c r="AF619" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B620" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C620" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D620" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E620" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F620" s="6" t="n"/>
+      <c r="G620" s="6" t="n"/>
+      <c r="H620" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I620" s="6" t="inlineStr"/>
+      <c r="J620" s="6" t="inlineStr"/>
+      <c r="K620" s="6" t="inlineStr"/>
+      <c r="L620" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M620" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N620" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O620" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P620" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q620" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R620" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S620" s="6" t="n"/>
+      <c r="T620" s="6" t="n"/>
+      <c r="U620" s="6" t="n"/>
+      <c r="V620" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W620" s="6" t="inlineStr"/>
+      <c r="X620" s="6" t="n"/>
+      <c r="Y620" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z620" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA620" s="6" t="n"/>
+      <c r="AB620" s="6" t="n"/>
+      <c r="AC620" s="6" t="n"/>
+      <c r="AD620" s="6" t="n"/>
+      <c r="AE620" s="6" t="n"/>
+      <c r="AF620" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B621" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C621" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D621" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E621" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F621" s="4" t="n"/>
+      <c r="G621" s="4" t="n"/>
+      <c r="H621" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I621" s="4" t="inlineStr"/>
+      <c r="J621" s="4" t="inlineStr"/>
+      <c r="K621" s="4" t="inlineStr"/>
+      <c r="L621" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M621" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N621" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O621" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P621" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q621" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R621" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S621" s="4" t="n"/>
+      <c r="T621" s="4" t="n"/>
+      <c r="U621" s="4" t="n"/>
+      <c r="V621" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W621" s="4" t="inlineStr"/>
+      <c r="X621" s="4" t="n"/>
+      <c r="Y621" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z621" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA621" s="4" t="n"/>
+      <c r="AB621" s="4" t="n"/>
+      <c r="AC621" s="4" t="n"/>
+      <c r="AD621" s="4" t="n"/>
+      <c r="AE621" s="4" t="n"/>
+      <c r="AF621" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B622" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C622" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D622" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E622" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F622" s="6" t="n"/>
+      <c r="G622" s="6" t="n"/>
+      <c r="H622" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I622" s="6" t="inlineStr"/>
+      <c r="J622" s="6" t="inlineStr"/>
+      <c r="K622" s="6" t="inlineStr"/>
+      <c r="L622" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M622" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N622" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O622" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P622" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q622" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R622" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S622" s="6" t="n"/>
+      <c r="T622" s="6" t="n"/>
+      <c r="U622" s="6" t="n"/>
+      <c r="V622" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W622" s="6" t="inlineStr"/>
+      <c r="X622" s="6" t="n"/>
+      <c r="Y622" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z622" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA622" s="6" t="n"/>
+      <c r="AB622" s="6" t="n"/>
+      <c r="AC622" s="6" t="n"/>
+      <c r="AD622" s="6" t="n"/>
+      <c r="AE622" s="6" t="n"/>
+      <c r="AF622" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B623" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C623" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D623" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E623" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F623" s="4" t="n"/>
+      <c r="G623" s="4" t="n"/>
+      <c r="H623" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I623" s="4" t="inlineStr"/>
+      <c r="J623" s="4" t="inlineStr"/>
+      <c r="K623" s="4" t="inlineStr"/>
+      <c r="L623" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M623" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N623" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O623" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P623" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q623" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R623" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S623" s="4" t="n"/>
+      <c r="T623" s="4" t="n"/>
+      <c r="U623" s="4" t="n"/>
+      <c r="V623" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W623" s="4" t="inlineStr"/>
+      <c r="X623" s="4" t="n"/>
+      <c r="Y623" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z623" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA623" s="4" t="n"/>
+      <c r="AB623" s="4" t="n"/>
+      <c r="AC623" s="4" t="n"/>
+      <c r="AD623" s="4" t="n"/>
+      <c r="AE623" s="4" t="n"/>
+      <c r="AF623" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="624">
+      <c r="A624" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B624" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C624" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D624" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E624" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F624" s="6" t="n"/>
+      <c r="G624" s="6" t="n"/>
+      <c r="H624" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I624" s="6" t="inlineStr"/>
+      <c r="J624" s="6" t="inlineStr"/>
+      <c r="K624" s="6" t="inlineStr"/>
+      <c r="L624" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M624" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N624" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O624" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P624" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q624" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R624" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S624" s="6" t="n"/>
+      <c r="T624" s="6" t="n"/>
+      <c r="U624" s="6" t="n"/>
+      <c r="V624" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W624" s="6" t="inlineStr"/>
+      <c r="X624" s="6" t="n"/>
+      <c r="Y624" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z624" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA624" s="6" t="n"/>
+      <c r="AB624" s="6" t="n"/>
+      <c r="AC624" s="6" t="n"/>
+      <c r="AD624" s="6" t="n"/>
+      <c r="AE624" s="6" t="n"/>
+      <c r="AF624" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="625">
+      <c r="A625" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B625" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C625" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D625" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E625" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F625" s="4" t="n"/>
+      <c r="G625" s="4" t="n"/>
+      <c r="H625" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I625" s="4" t="inlineStr"/>
+      <c r="J625" s="4" t="inlineStr"/>
+      <c r="K625" s="4" t="inlineStr"/>
+      <c r="L625" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M625" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N625" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O625" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P625" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q625" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R625" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S625" s="4" t="n"/>
+      <c r="T625" s="4" t="n"/>
+      <c r="U625" s="4" t="n"/>
+      <c r="V625" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W625" s="4" t="inlineStr"/>
+      <c r="X625" s="4" t="n"/>
+      <c r="Y625" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z625" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA625" s="4" t="n"/>
+      <c r="AB625" s="4" t="n"/>
+      <c r="AC625" s="4" t="n"/>
+      <c r="AD625" s="4" t="n"/>
+      <c r="AE625" s="4" t="n"/>
+      <c r="AF625" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="626">
+      <c r="A626" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B626" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C626" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D626" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E626" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F626" s="6" t="n"/>
+      <c r="G626" s="6" t="n"/>
+      <c r="H626" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I626" s="6" t="inlineStr"/>
+      <c r="J626" s="6" t="inlineStr"/>
+      <c r="K626" s="6" t="inlineStr"/>
+      <c r="L626" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M626" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N626" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O626" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P626" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q626" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R626" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S626" s="6" t="n"/>
+      <c r="T626" s="6" t="n"/>
+      <c r="U626" s="6" t="n"/>
+      <c r="V626" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W626" s="6" t="inlineStr"/>
+      <c r="X626" s="6" t="n"/>
+      <c r="Y626" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z626" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA626" s="6" t="n"/>
+      <c r="AB626" s="6" t="n"/>
+      <c r="AC626" s="6" t="n"/>
+      <c r="AD626" s="6" t="n"/>
+      <c r="AE626" s="6" t="n"/>
+      <c r="AF626" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="627">
+      <c r="A627" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B627" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C627" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D627" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E627" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F627" s="4" t="n"/>
+      <c r="G627" s="4" t="n"/>
+      <c r="H627" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I627" s="4" t="inlineStr"/>
+      <c r="J627" s="4" t="inlineStr"/>
+      <c r="K627" s="4" t="inlineStr"/>
+      <c r="L627" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M627" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N627" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O627" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P627" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q627" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R627" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S627" s="4" t="n"/>
+      <c r="T627" s="4" t="n"/>
+      <c r="U627" s="4" t="n"/>
+      <c r="V627" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W627" s="4" t="inlineStr"/>
+      <c r="X627" s="4" t="n"/>
+      <c r="Y627" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z627" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA627" s="4" t="n"/>
+      <c r="AB627" s="4" t="n"/>
+      <c r="AC627" s="4" t="n"/>
+      <c r="AD627" s="4" t="n"/>
+      <c r="AE627" s="4" t="n"/>
+      <c r="AF627" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="628">
+      <c r="A628" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B628" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C628" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D628" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E628" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F628" s="6" t="n"/>
+      <c r="G628" s="6" t="n"/>
+      <c r="H628" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I628" s="6" t="inlineStr"/>
+      <c r="J628" s="6" t="inlineStr"/>
+      <c r="K628" s="6" t="inlineStr"/>
+      <c r="L628" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M628" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N628" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O628" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P628" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q628" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R628" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S628" s="6" t="n"/>
+      <c r="T628" s="6" t="n"/>
+      <c r="U628" s="6" t="n"/>
+      <c r="V628" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W628" s="6" t="inlineStr"/>
+      <c r="X628" s="6" t="n"/>
+      <c r="Y628" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z628" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA628" s="6" t="n"/>
+      <c r="AB628" s="6" t="n"/>
+      <c r="AC628" s="6" t="n"/>
+      <c r="AD628" s="6" t="n"/>
+      <c r="AE628" s="6" t="n"/>
+      <c r="AF628" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="629">
+      <c r="A629" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B629" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C629" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D629" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E629" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F629" s="4" t="n"/>
+      <c r="G629" s="4" t="n"/>
+      <c r="H629" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I629" s="4" t="inlineStr"/>
+      <c r="J629" s="4" t="inlineStr"/>
+      <c r="K629" s="4" t="inlineStr"/>
+      <c r="L629" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="M629" s="4" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N629" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O629" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P629" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q629" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R629" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S629" s="4" t="n"/>
+      <c r="T629" s="4" t="n"/>
+      <c r="U629" s="4" t="n"/>
+      <c r="V629" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W629" s="4" t="inlineStr"/>
+      <c r="X629" s="4" t="n"/>
+      <c r="Y629" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z629" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA629" s="4" t="n"/>
+      <c r="AB629" s="4" t="n"/>
+      <c r="AC629" s="4" t="n"/>
+      <c r="AD629" s="4" t="n"/>
+      <c r="AE629" s="4" t="n"/>
+      <c r="AF629" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="630">
+      <c r="A630" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B630" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C630" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D630" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E630" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F630" s="6" t="n"/>
+      <c r="G630" s="6" t="n"/>
+      <c r="H630" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I630" s="6" t="inlineStr"/>
+      <c r="J630" s="6" t="inlineStr"/>
+      <c r="K630" s="6" t="inlineStr"/>
+      <c r="L630" s="6" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M630" s="6" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N630" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O630" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P630" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q630" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R630" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S630" s="6" t="n"/>
+      <c r="T630" s="6" t="n"/>
+      <c r="U630" s="6" t="n"/>
+      <c r="V630" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W630" s="6" t="inlineStr"/>
+      <c r="X630" s="6" t="n"/>
+      <c r="Y630" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z630" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA630" s="6" t="n"/>
+      <c r="AB630" s="6" t="n"/>
+      <c r="AC630" s="6" t="n"/>
+      <c r="AD630" s="6" t="n"/>
+      <c r="AE630" s="6" t="n"/>
+      <c r="AF630" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="631">
+      <c r="A631" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B631" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C631" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D631" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E631" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F631" s="4" t="n"/>
+      <c r="G631" s="4" t="n"/>
+      <c r="H631" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I631" s="4" t="inlineStr"/>
+      <c r="J631" s="4" t="inlineStr"/>
+      <c r="K631" s="4" t="inlineStr"/>
+      <c r="L631" s="4" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M631" s="4" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N631" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O631" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P631" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q631" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R631" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S631" s="4" t="n"/>
+      <c r="T631" s="4" t="n"/>
+      <c r="U631" s="4" t="n"/>
+      <c r="V631" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W631" s="4" t="inlineStr"/>
+      <c r="X631" s="4" t="n"/>
+      <c r="Y631" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z631" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA631" s="4" t="n"/>
+      <c r="AB631" s="4" t="n"/>
+      <c r="AC631" s="4" t="n"/>
+      <c r="AD631" s="4" t="n"/>
+      <c r="AE631" s="4" t="n"/>
+      <c r="AF631" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="632">
+      <c r="A632" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B632" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C632" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D632" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E632" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F632" s="6" t="n"/>
+      <c r="G632" s="6" t="n"/>
+      <c r="H632" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I632" s="6" t="inlineStr"/>
+      <c r="J632" s="6" t="inlineStr"/>
+      <c r="K632" s="6" t="inlineStr"/>
+      <c r="L632" s="6" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M632" s="6" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N632" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O632" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P632" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q632" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R632" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S632" s="6" t="n"/>
+      <c r="T632" s="6" t="n"/>
+      <c r="U632" s="6" t="n"/>
+      <c r="V632" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W632" s="6" t="inlineStr"/>
+      <c r="X632" s="6" t="n"/>
+      <c r="Y632" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z632" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA632" s="6" t="n"/>
+      <c r="AB632" s="6" t="n"/>
+      <c r="AC632" s="6" t="n"/>
+      <c r="AD632" s="6" t="n"/>
+      <c r="AE632" s="6" t="n"/>
+      <c r="AF632" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="633">
+      <c r="A633" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B633" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C633" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D633" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E633" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F633" s="4" t="n"/>
+      <c r="G633" s="4" t="n"/>
+      <c r="H633" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I633" s="4" t="inlineStr"/>
+      <c r="J633" s="4" t="inlineStr"/>
+      <c r="K633" s="4" t="inlineStr"/>
+      <c r="L633" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M633" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N633" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O633" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P633" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q633" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R633" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S633" s="4" t="n"/>
+      <c r="T633" s="4" t="n"/>
+      <c r="U633" s="4" t="n"/>
+      <c r="V633" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W633" s="4" t="inlineStr"/>
+      <c r="X633" s="4" t="n"/>
+      <c r="Y633" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z633" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA633" s="4" t="n"/>
+      <c r="AB633" s="4" t="n"/>
+      <c r="AC633" s="4" t="n"/>
+      <c r="AD633" s="4" t="n"/>
+      <c r="AE633" s="4" t="n"/>
+      <c r="AF633" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="634">
+      <c r="A634" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B634" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C634" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D634" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E634" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F634" s="6" t="n"/>
+      <c r="G634" s="6" t="n"/>
+      <c r="H634" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I634" s="6" t="inlineStr"/>
+      <c r="J634" s="6" t="inlineStr"/>
+      <c r="K634" s="6" t="inlineStr"/>
+      <c r="L634" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M634" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N634" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O634" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P634" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q634" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R634" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S634" s="6" t="n"/>
+      <c r="T634" s="6" t="n"/>
+      <c r="U634" s="6" t="n"/>
+      <c r="V634" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W634" s="6" t="inlineStr"/>
+      <c r="X634" s="6" t="n"/>
+      <c r="Y634" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z634" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA634" s="6" t="n"/>
+      <c r="AB634" s="6" t="n"/>
+      <c r="AC634" s="6" t="n"/>
+      <c r="AD634" s="6" t="n"/>
+      <c r="AE634" s="6" t="n"/>
+      <c r="AF634" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="635">
+      <c r="A635" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B635" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C635" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D635" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E635" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F635" s="4" t="n"/>
+      <c r="G635" s="4" t="n"/>
+      <c r="H635" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I635" s="4" t="inlineStr"/>
+      <c r="J635" s="4" t="inlineStr"/>
+      <c r="K635" s="4" t="inlineStr"/>
+      <c r="L635" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M635" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N635" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O635" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P635" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q635" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R635" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S635" s="4" t="n"/>
+      <c r="T635" s="4" t="n"/>
+      <c r="U635" s="4" t="n"/>
+      <c r="V635" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W635" s="4" t="inlineStr"/>
+      <c r="X635" s="4" t="n"/>
+      <c r="Y635" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z635" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA635" s="4" t="n"/>
+      <c r="AB635" s="4" t="n"/>
+      <c r="AC635" s="4" t="n"/>
+      <c r="AD635" s="4" t="n"/>
+      <c r="AE635" s="4" t="n"/>
+      <c r="AF635" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="636">
+      <c r="A636" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B636" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C636" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D636" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E636" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F636" s="6" t="n"/>
+      <c r="G636" s="6" t="n"/>
+      <c r="H636" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I636" s="6" t="inlineStr"/>
+      <c r="J636" s="6" t="inlineStr"/>
+      <c r="K636" s="6" t="inlineStr"/>
+      <c r="L636" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M636" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N636" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O636" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P636" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q636" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R636" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S636" s="6" t="n"/>
+      <c r="T636" s="6" t="n"/>
+      <c r="U636" s="6" t="n"/>
+      <c r="V636" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W636" s="6" t="inlineStr"/>
+      <c r="X636" s="6" t="n"/>
+      <c r="Y636" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z636" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA636" s="6" t="n"/>
+      <c r="AB636" s="6" t="n"/>
+      <c r="AC636" s="6" t="n"/>
+      <c r="AD636" s="6" t="n"/>
+      <c r="AE636" s="6" t="n"/>
+      <c r="AF636" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="637">
+      <c r="A637" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B637" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C637" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D637" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E637" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F637" s="4" t="n"/>
+      <c r="G637" s="4" t="n"/>
+      <c r="H637" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I637" s="4" t="inlineStr"/>
+      <c r="J637" s="4" t="inlineStr"/>
+      <c r="K637" s="4" t="inlineStr"/>
+      <c r="L637" s="4" t="n"/>
+      <c r="M637" s="4" t="n"/>
+      <c r="N637" s="4" t="n"/>
+      <c r="O637" s="4" t="n"/>
+      <c r="P637" s="4" t="n"/>
+      <c r="Q637" s="4" t="n"/>
+      <c r="R637" s="4" t="n"/>
+      <c r="S637" s="4" t="n"/>
+      <c r="T637" s="4" t="n"/>
+      <c r="U637" s="4" t="n"/>
+      <c r="V637" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W637" s="4" t="inlineStr"/>
+      <c r="X637" s="4" t="n"/>
+      <c r="Y637" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z637" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA637" s="4" t="n"/>
+      <c r="AB637" s="4" t="n"/>
+      <c r="AC637" s="4" t="n"/>
+      <c r="AD637" s="4" t="n"/>
+      <c r="AE637" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF637" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="638">
+      <c r="A638" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B638" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C638" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D638" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E638" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F638" s="6" t="n"/>
+      <c r="G638" s="6" t="n"/>
+      <c r="H638" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I638" s="6" t="inlineStr"/>
+      <c r="J638" s="6" t="inlineStr"/>
+      <c r="K638" s="6" t="inlineStr"/>
+      <c r="L638" s="6" t="n"/>
+      <c r="M638" s="6" t="n"/>
+      <c r="N638" s="6" t="n"/>
+      <c r="O638" s="6" t="n"/>
+      <c r="P638" s="6" t="n"/>
+      <c r="Q638" s="6" t="n"/>
+      <c r="R638" s="6" t="n"/>
+      <c r="S638" s="6" t="n"/>
+      <c r="T638" s="6" t="n"/>
+      <c r="U638" s="6" t="n"/>
+      <c r="V638" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W638" s="6" t="inlineStr"/>
+      <c r="X638" s="6" t="n"/>
+      <c r="Y638" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z638" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA638" s="6" t="n"/>
+      <c r="AB638" s="6" t="n"/>
+      <c r="AC638" s="6" t="n"/>
+      <c r="AD638" s="6" t="n"/>
+      <c r="AE638" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF638" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="639">
+      <c r="A639" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B639" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C639" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D639" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E639" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F639" s="4" t="n"/>
+      <c r="G639" s="4" t="n"/>
+      <c r="H639" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I639" s="4" t="inlineStr"/>
+      <c r="J639" s="4" t="inlineStr"/>
+      <c r="K639" s="4" t="inlineStr"/>
+      <c r="L639" s="4" t="n"/>
+      <c r="M639" s="4" t="n"/>
+      <c r="N639" s="4" t="n"/>
+      <c r="O639" s="4" t="n"/>
+      <c r="P639" s="4" t="n"/>
+      <c r="Q639" s="4" t="n"/>
+      <c r="R639" s="4" t="n"/>
+      <c r="S639" s="4" t="n"/>
+      <c r="T639" s="4" t="n"/>
+      <c r="U639" s="4" t="n"/>
+      <c r="V639" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W639" s="4" t="inlineStr"/>
+      <c r="X639" s="4" t="n"/>
+      <c r="Y639" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z639" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA639" s="4" t="n"/>
+      <c r="AB639" s="4" t="n"/>
+      <c r="AC639" s="4" t="n"/>
+      <c r="AD639" s="4" t="n"/>
+      <c r="AE639" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF639" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="640">
+      <c r="A640" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B640" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C640" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D640" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E640" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F640" s="6" t="n"/>
+      <c r="G640" s="6" t="n"/>
+      <c r="H640" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I640" s="6" t="inlineStr"/>
+      <c r="J640" s="6" t="inlineStr"/>
+      <c r="K640" s="6" t="inlineStr"/>
+      <c r="L640" s="6" t="n"/>
+      <c r="M640" s="6" t="n"/>
+      <c r="N640" s="6" t="n"/>
+      <c r="O640" s="6" t="n"/>
+      <c r="P640" s="6" t="n"/>
+      <c r="Q640" s="6" t="n"/>
+      <c r="R640" s="6" t="n"/>
+      <c r="S640" s="6" t="n"/>
+      <c r="T640" s="6" t="n"/>
+      <c r="U640" s="6" t="n"/>
+      <c r="V640" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W640" s="6" t="inlineStr"/>
+      <c r="X640" s="6" t="n"/>
+      <c r="Y640" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z640" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA640" s="6" t="n"/>
+      <c r="AB640" s="6" t="n"/>
+      <c r="AC640" s="6" t="n"/>
+      <c r="AD640" s="6" t="n"/>
+      <c r="AE640" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF640" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="641">
+      <c r="A641" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B641" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C641" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D641" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E641" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F641" s="4" t="n"/>
+      <c r="G641" s="4" t="n"/>
+      <c r="H641" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I641" s="4" t="inlineStr"/>
+      <c r="J641" s="4" t="inlineStr"/>
+      <c r="K641" s="4" t="inlineStr"/>
+      <c r="L641" s="4" t="n"/>
+      <c r="M641" s="4" t="n"/>
+      <c r="N641" s="4" t="n"/>
+      <c r="O641" s="4" t="n"/>
+      <c r="P641" s="4" t="n"/>
+      <c r="Q641" s="4" t="n"/>
+      <c r="R641" s="4" t="n"/>
+      <c r="S641" s="4" t="n"/>
+      <c r="T641" s="4" t="n"/>
+      <c r="U641" s="4" t="n"/>
+      <c r="V641" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W641" s="4" t="inlineStr"/>
+      <c r="X641" s="4" t="n"/>
+      <c r="Y641" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z641" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA641" s="4" t="n"/>
+      <c r="AB641" s="4" t="n"/>
+      <c r="AC641" s="4" t="n"/>
+      <c r="AD641" s="4" t="n"/>
+      <c r="AE641" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF641" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="642">
+      <c r="A642" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B642" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C642" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D642" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E642" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F642" s="6" t="n"/>
+      <c r="G642" s="6" t="n"/>
+      <c r="H642" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I642" s="6" t="inlineStr"/>
+      <c r="J642" s="6" t="inlineStr"/>
+      <c r="K642" s="6" t="inlineStr"/>
+      <c r="L642" s="6" t="n"/>
+      <c r="M642" s="6" t="n"/>
+      <c r="N642" s="6" t="n"/>
+      <c r="O642" s="6" t="n"/>
+      <c r="P642" s="6" t="n"/>
+      <c r="Q642" s="6" t="n"/>
+      <c r="R642" s="6" t="n"/>
+      <c r="S642" s="6" t="n"/>
+      <c r="T642" s="6" t="n"/>
+      <c r="U642" s="6" t="n"/>
+      <c r="V642" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W642" s="6" t="inlineStr"/>
+      <c r="X642" s="6" t="n"/>
+      <c r="Y642" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z642" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA642" s="6" t="n"/>
+      <c r="AB642" s="6" t="n"/>
+      <c r="AC642" s="6" t="n"/>
+      <c r="AD642" s="6" t="n"/>
+      <c r="AE642" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF642" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="643">
+      <c r="A643" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B643" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C643" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D643" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E643" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F643" s="4" t="n"/>
+      <c r="G643" s="4" t="n"/>
+      <c r="H643" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I643" s="4" t="inlineStr"/>
+      <c r="J643" s="4" t="inlineStr"/>
+      <c r="K643" s="4" t="inlineStr"/>
+      <c r="L643" s="4" t="n"/>
+      <c r="M643" s="4" t="n"/>
+      <c r="N643" s="4" t="n"/>
+      <c r="O643" s="4" t="n"/>
+      <c r="P643" s="4" t="n"/>
+      <c r="Q643" s="4" t="n"/>
+      <c r="R643" s="4" t="n"/>
+      <c r="S643" s="4" t="n"/>
+      <c r="T643" s="4" t="n"/>
+      <c r="U643" s="4" t="n"/>
+      <c r="V643" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W643" s="4" t="inlineStr"/>
+      <c r="X643" s="4" t="n"/>
+      <c r="Y643" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z643" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA643" s="4" t="n"/>
+      <c r="AB643" s="4" t="n"/>
+      <c r="AC643" s="4" t="n"/>
+      <c r="AD643" s="4" t="n"/>
+      <c r="AE643" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF643" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="644">
+      <c r="A644" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B644" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C644" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D644" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E644" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F644" s="6" t="n"/>
+      <c r="G644" s="6" t="n"/>
+      <c r="H644" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I644" s="6" t="inlineStr"/>
+      <c r="J644" s="6" t="inlineStr"/>
+      <c r="K644" s="6" t="inlineStr"/>
+      <c r="L644" s="6" t="n"/>
+      <c r="M644" s="6" t="n"/>
+      <c r="N644" s="6" t="n"/>
+      <c r="O644" s="6" t="n"/>
+      <c r="P644" s="6" t="n"/>
+      <c r="Q644" s="6" t="n"/>
+      <c r="R644" s="6" t="n"/>
+      <c r="S644" s="6" t="n"/>
+      <c r="T644" s="6" t="n"/>
+      <c r="U644" s="6" t="n"/>
+      <c r="V644" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W644" s="6" t="inlineStr"/>
+      <c r="X644" s="6" t="n"/>
+      <c r="Y644" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z644" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA644" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB644" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC644" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD644" s="6" t="n"/>
+      <c r="AE644" s="6" t="n"/>
+      <c r="AF644" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="645">
+      <c r="A645" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B645" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C645" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D645" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E645" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F645" s="4" t="n"/>
+      <c r="G645" s="4" t="n"/>
+      <c r="H645" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I645" s="4" t="inlineStr"/>
+      <c r="J645" s="4" t="inlineStr"/>
+      <c r="K645" s="4" t="inlineStr"/>
+      <c r="L645" s="4" t="n"/>
+      <c r="M645" s="4" t="n"/>
+      <c r="N645" s="4" t="n"/>
+      <c r="O645" s="4" t="n"/>
+      <c r="P645" s="4" t="n"/>
+      <c r="Q645" s="4" t="n"/>
+      <c r="R645" s="4" t="n"/>
+      <c r="S645" s="4" t="n"/>
+      <c r="T645" s="4" t="n"/>
+      <c r="U645" s="4" t="n"/>
+      <c r="V645" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W645" s="4" t="inlineStr"/>
+      <c r="X645" s="4" t="n"/>
+      <c r="Y645" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z645" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA645" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB645" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC645" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD645" s="4" t="n"/>
+      <c r="AE645" s="4" t="n"/>
+      <c r="AF645" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="646">
+      <c r="A646" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B646" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C646" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D646" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E646" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F646" s="6" t="n"/>
+      <c r="G646" s="6" t="n"/>
+      <c r="H646" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I646" s="6" t="inlineStr"/>
+      <c r="J646" s="6" t="inlineStr"/>
+      <c r="K646" s="6" t="inlineStr"/>
+      <c r="L646" s="6" t="n"/>
+      <c r="M646" s="6" t="n"/>
+      <c r="N646" s="6" t="n"/>
+      <c r="O646" s="6" t="n"/>
+      <c r="P646" s="6" t="n"/>
+      <c r="Q646" s="6" t="n"/>
+      <c r="R646" s="6" t="n"/>
+      <c r="S646" s="6" t="n"/>
+      <c r="T646" s="6" t="n"/>
+      <c r="U646" s="6" t="n"/>
+      <c r="V646" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W646" s="6" t="inlineStr"/>
+      <c r="X646" s="6" t="n"/>
+      <c r="Y646" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z646" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA646" s="6" t="n"/>
+      <c r="AB646" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC646" s="6" t="n"/>
+      <c r="AD646" s="6" t="n"/>
+      <c r="AE646" s="6" t="n"/>
+      <c r="AF646" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="647">
+      <c r="A647" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-06</t>
+        </is>
+      </c>
+      <c r="B647" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C647" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D647" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E647" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F647" s="4" t="n"/>
+      <c r="G647" s="4" t="n"/>
+      <c r="H647" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I647" s="4" t="inlineStr"/>
+      <c r="J647" s="4" t="inlineStr"/>
+      <c r="K647" s="4" t="inlineStr"/>
+      <c r="L647" s="4" t="n"/>
+      <c r="M647" s="4" t="n"/>
+      <c r="N647" s="4" t="n"/>
+      <c r="O647" s="4" t="n"/>
+      <c r="P647" s="4" t="n"/>
+      <c r="Q647" s="4" t="n"/>
+      <c r="R647" s="4" t="n"/>
+      <c r="S647" s="4" t="n"/>
+      <c r="T647" s="4" t="n"/>
+      <c r="U647" s="4" t="n"/>
+      <c r="V647" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W647" s="4" t="inlineStr"/>
+      <c r="X647" s="4" t="n"/>
+      <c r="Y647" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z647" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA647" s="4" t="n"/>
+      <c r="AB647" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC647" s="4" t="n"/>
+      <c r="AD647" s="4" t="n"/>
+      <c r="AE647" s="4" t="n"/>
+      <c r="AF647" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-07
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF647"/>
+  <dimension ref="A1:AF682"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -51466,6 +51466,2758 @@
         <v>1</v>
       </c>
     </row>
+    <row r="648">
+      <c r="A648" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B648" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C648" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D648" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E648" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F648" s="4" t="n"/>
+      <c r="G648" s="4" t="n"/>
+      <c r="H648" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I648" s="4" t="inlineStr"/>
+      <c r="J648" s="4" t="inlineStr"/>
+      <c r="K648" s="4" t="inlineStr"/>
+      <c r="L648" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M648" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N648" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O648" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P648" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q648" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R648" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S648" s="4" t="n"/>
+      <c r="T648" s="4" t="n"/>
+      <c r="U648" s="4" t="n"/>
+      <c r="V648" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W648" s="4" t="inlineStr"/>
+      <c r="X648" s="4" t="n"/>
+      <c r="Y648" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z648" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA648" s="4" t="n"/>
+      <c r="AB648" s="4" t="n"/>
+      <c r="AC648" s="4" t="n"/>
+      <c r="AD648" s="4" t="n"/>
+      <c r="AE648" s="4" t="n"/>
+      <c r="AF648" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="649">
+      <c r="A649" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B649" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C649" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D649" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E649" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F649" s="6" t="n"/>
+      <c r="G649" s="6" t="n"/>
+      <c r="H649" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I649" s="6" t="inlineStr"/>
+      <c r="J649" s="6" t="inlineStr"/>
+      <c r="K649" s="6" t="inlineStr"/>
+      <c r="L649" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M649" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N649" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O649" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P649" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q649" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R649" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S649" s="6" t="n"/>
+      <c r="T649" s="6" t="n"/>
+      <c r="U649" s="6" t="n"/>
+      <c r="V649" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W649" s="6" t="inlineStr"/>
+      <c r="X649" s="6" t="n"/>
+      <c r="Y649" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z649" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA649" s="6" t="n"/>
+      <c r="AB649" s="6" t="n"/>
+      <c r="AC649" s="6" t="n"/>
+      <c r="AD649" s="6" t="n"/>
+      <c r="AE649" s="6" t="n"/>
+      <c r="AF649" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="650">
+      <c r="A650" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B650" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C650" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D650" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E650" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F650" s="4" t="n"/>
+      <c r="G650" s="4" t="n"/>
+      <c r="H650" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I650" s="4" t="inlineStr"/>
+      <c r="J650" s="4" t="inlineStr"/>
+      <c r="K650" s="4" t="inlineStr"/>
+      <c r="L650" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M650" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N650" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O650" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P650" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q650" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R650" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S650" s="4" t="n"/>
+      <c r="T650" s="4" t="n"/>
+      <c r="U650" s="4" t="n"/>
+      <c r="V650" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W650" s="4" t="inlineStr"/>
+      <c r="X650" s="4" t="n"/>
+      <c r="Y650" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z650" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA650" s="4" t="n"/>
+      <c r="AB650" s="4" t="n"/>
+      <c r="AC650" s="4" t="n"/>
+      <c r="AD650" s="4" t="n"/>
+      <c r="AE650" s="4" t="n"/>
+      <c r="AF650" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="651">
+      <c r="A651" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B651" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C651" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D651" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E651" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F651" s="6" t="n"/>
+      <c r="G651" s="6" t="n"/>
+      <c r="H651" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I651" s="6" t="inlineStr"/>
+      <c r="J651" s="6" t="inlineStr"/>
+      <c r="K651" s="6" t="inlineStr"/>
+      <c r="L651" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M651" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N651" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O651" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P651" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q651" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R651" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S651" s="6" t="n"/>
+      <c r="T651" s="6" t="n"/>
+      <c r="U651" s="6" t="n"/>
+      <c r="V651" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W651" s="6" t="inlineStr"/>
+      <c r="X651" s="6" t="n"/>
+      <c r="Y651" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z651" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA651" s="6" t="n"/>
+      <c r="AB651" s="6" t="n"/>
+      <c r="AC651" s="6" t="n"/>
+      <c r="AD651" s="6" t="n"/>
+      <c r="AE651" s="6" t="n"/>
+      <c r="AF651" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="652">
+      <c r="A652" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B652" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C652" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D652" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E652" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F652" s="4" t="n"/>
+      <c r="G652" s="4" t="n"/>
+      <c r="H652" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I652" s="4" t="inlineStr"/>
+      <c r="J652" s="4" t="inlineStr"/>
+      <c r="K652" s="4" t="inlineStr"/>
+      <c r="L652" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M652" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N652" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O652" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P652" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q652" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R652" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S652" s="4" t="n"/>
+      <c r="T652" s="4" t="n"/>
+      <c r="U652" s="4" t="n"/>
+      <c r="V652" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W652" s="4" t="inlineStr"/>
+      <c r="X652" s="4" t="n"/>
+      <c r="Y652" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z652" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA652" s="4" t="n"/>
+      <c r="AB652" s="4" t="n"/>
+      <c r="AC652" s="4" t="n"/>
+      <c r="AD652" s="4" t="n"/>
+      <c r="AE652" s="4" t="n"/>
+      <c r="AF652" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="653">
+      <c r="A653" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B653" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C653" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D653" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E653" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F653" s="6" t="n"/>
+      <c r="G653" s="6" t="n"/>
+      <c r="H653" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I653" s="6" t="inlineStr"/>
+      <c r="J653" s="6" t="inlineStr"/>
+      <c r="K653" s="6" t="inlineStr"/>
+      <c r="L653" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M653" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N653" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O653" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P653" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q653" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R653" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S653" s="6" t="n"/>
+      <c r="T653" s="6" t="n"/>
+      <c r="U653" s="6" t="n"/>
+      <c r="V653" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W653" s="6" t="inlineStr"/>
+      <c r="X653" s="6" t="n"/>
+      <c r="Y653" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z653" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA653" s="6" t="n"/>
+      <c r="AB653" s="6" t="n"/>
+      <c r="AC653" s="6" t="n"/>
+      <c r="AD653" s="6" t="n"/>
+      <c r="AE653" s="6" t="n"/>
+      <c r="AF653" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="654">
+      <c r="A654" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B654" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C654" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D654" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E654" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F654" s="4" t="n"/>
+      <c r="G654" s="4" t="n"/>
+      <c r="H654" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I654" s="4" t="inlineStr"/>
+      <c r="J654" s="4" t="inlineStr"/>
+      <c r="K654" s="4" t="inlineStr"/>
+      <c r="L654" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M654" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N654" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O654" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P654" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q654" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R654" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S654" s="4" t="n"/>
+      <c r="T654" s="4" t="n"/>
+      <c r="U654" s="4" t="n"/>
+      <c r="V654" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W654" s="4" t="inlineStr"/>
+      <c r="X654" s="4" t="n"/>
+      <c r="Y654" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z654" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA654" s="4" t="n"/>
+      <c r="AB654" s="4" t="n"/>
+      <c r="AC654" s="4" t="n"/>
+      <c r="AD654" s="4" t="n"/>
+      <c r="AE654" s="4" t="n"/>
+      <c r="AF654" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="655">
+      <c r="A655" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B655" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C655" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D655" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E655" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F655" s="6" t="n"/>
+      <c r="G655" s="6" t="n"/>
+      <c r="H655" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I655" s="6" t="inlineStr"/>
+      <c r="J655" s="6" t="inlineStr"/>
+      <c r="K655" s="6" t="inlineStr"/>
+      <c r="L655" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M655" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N655" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O655" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P655" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q655" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R655" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S655" s="6" t="n"/>
+      <c r="T655" s="6" t="n"/>
+      <c r="U655" s="6" t="n"/>
+      <c r="V655" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W655" s="6" t="inlineStr"/>
+      <c r="X655" s="6" t="n"/>
+      <c r="Y655" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z655" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA655" s="6" t="n"/>
+      <c r="AB655" s="6" t="n"/>
+      <c r="AC655" s="6" t="n"/>
+      <c r="AD655" s="6" t="n"/>
+      <c r="AE655" s="6" t="n"/>
+      <c r="AF655" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="656">
+      <c r="A656" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B656" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C656" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D656" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E656" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F656" s="4" t="n"/>
+      <c r="G656" s="4" t="n"/>
+      <c r="H656" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I656" s="4" t="inlineStr"/>
+      <c r="J656" s="4" t="inlineStr"/>
+      <c r="K656" s="4" t="inlineStr"/>
+      <c r="L656" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M656" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N656" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O656" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P656" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q656" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R656" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S656" s="4" t="n"/>
+      <c r="T656" s="4" t="n"/>
+      <c r="U656" s="4" t="n"/>
+      <c r="V656" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W656" s="4" t="inlineStr"/>
+      <c r="X656" s="4" t="n"/>
+      <c r="Y656" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z656" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA656" s="4" t="n"/>
+      <c r="AB656" s="4" t="n"/>
+      <c r="AC656" s="4" t="n"/>
+      <c r="AD656" s="4" t="n"/>
+      <c r="AE656" s="4" t="n"/>
+      <c r="AF656" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="657">
+      <c r="A657" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B657" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C657" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D657" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E657" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F657" s="6" t="n"/>
+      <c r="G657" s="6" t="n"/>
+      <c r="H657" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I657" s="6" t="inlineStr"/>
+      <c r="J657" s="6" t="inlineStr"/>
+      <c r="K657" s="6" t="inlineStr"/>
+      <c r="L657" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M657" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N657" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O657" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P657" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q657" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R657" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S657" s="6" t="n"/>
+      <c r="T657" s="6" t="n"/>
+      <c r="U657" s="6" t="n"/>
+      <c r="V657" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W657" s="6" t="inlineStr"/>
+      <c r="X657" s="6" t="n"/>
+      <c r="Y657" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z657" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA657" s="6" t="n"/>
+      <c r="AB657" s="6" t="n"/>
+      <c r="AC657" s="6" t="n"/>
+      <c r="AD657" s="6" t="n"/>
+      <c r="AE657" s="6" t="n"/>
+      <c r="AF657" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="658">
+      <c r="A658" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B658" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C658" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D658" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E658" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F658" s="4" t="n"/>
+      <c r="G658" s="4" t="n"/>
+      <c r="H658" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I658" s="4" t="inlineStr"/>
+      <c r="J658" s="4" t="inlineStr"/>
+      <c r="K658" s="4" t="inlineStr"/>
+      <c r="L658" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M658" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N658" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O658" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P658" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q658" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R658" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S658" s="4" t="n"/>
+      <c r="T658" s="4" t="n"/>
+      <c r="U658" s="4" t="n"/>
+      <c r="V658" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W658" s="4" t="inlineStr"/>
+      <c r="X658" s="4" t="n"/>
+      <c r="Y658" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z658" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA658" s="4" t="n"/>
+      <c r="AB658" s="4" t="n"/>
+      <c r="AC658" s="4" t="n"/>
+      <c r="AD658" s="4" t="n"/>
+      <c r="AE658" s="4" t="n"/>
+      <c r="AF658" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="659">
+      <c r="A659" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B659" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C659" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D659" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E659" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F659" s="6" t="n"/>
+      <c r="G659" s="6" t="n"/>
+      <c r="H659" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I659" s="6" t="inlineStr"/>
+      <c r="J659" s="6" t="inlineStr"/>
+      <c r="K659" s="6" t="inlineStr"/>
+      <c r="L659" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M659" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N659" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O659" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P659" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q659" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R659" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S659" s="6" t="n"/>
+      <c r="T659" s="6" t="n"/>
+      <c r="U659" s="6" t="n"/>
+      <c r="V659" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W659" s="6" t="inlineStr"/>
+      <c r="X659" s="6" t="n"/>
+      <c r="Y659" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z659" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA659" s="6" t="n"/>
+      <c r="AB659" s="6" t="n"/>
+      <c r="AC659" s="6" t="n"/>
+      <c r="AD659" s="6" t="n"/>
+      <c r="AE659" s="6" t="n"/>
+      <c r="AF659" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="660">
+      <c r="A660" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B660" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C660" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D660" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E660" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F660" s="4" t="n"/>
+      <c r="G660" s="4" t="n"/>
+      <c r="H660" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I660" s="4" t="inlineStr"/>
+      <c r="J660" s="4" t="inlineStr"/>
+      <c r="K660" s="4" t="inlineStr"/>
+      <c r="L660" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M660" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N660" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O660" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P660" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q660" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R660" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S660" s="4" t="n"/>
+      <c r="T660" s="4" t="n"/>
+      <c r="U660" s="4" t="n"/>
+      <c r="V660" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W660" s="4" t="inlineStr"/>
+      <c r="X660" s="4" t="n"/>
+      <c r="Y660" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z660" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA660" s="4" t="n"/>
+      <c r="AB660" s="4" t="n"/>
+      <c r="AC660" s="4" t="n"/>
+      <c r="AD660" s="4" t="n"/>
+      <c r="AE660" s="4" t="n"/>
+      <c r="AF660" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="661">
+      <c r="A661" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B661" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C661" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D661" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E661" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F661" s="6" t="n"/>
+      <c r="G661" s="6" t="n"/>
+      <c r="H661" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I661" s="6" t="inlineStr"/>
+      <c r="J661" s="6" t="inlineStr"/>
+      <c r="K661" s="6" t="inlineStr"/>
+      <c r="L661" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M661" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N661" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O661" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P661" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q661" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R661" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S661" s="6" t="n"/>
+      <c r="T661" s="6" t="n"/>
+      <c r="U661" s="6" t="n"/>
+      <c r="V661" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W661" s="6" t="inlineStr"/>
+      <c r="X661" s="6" t="n"/>
+      <c r="Y661" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z661" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA661" s="6" t="n"/>
+      <c r="AB661" s="6" t="n"/>
+      <c r="AC661" s="6" t="n"/>
+      <c r="AD661" s="6" t="n"/>
+      <c r="AE661" s="6" t="n"/>
+      <c r="AF661" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="662">
+      <c r="A662" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B662" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C662" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D662" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E662" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F662" s="4" t="n"/>
+      <c r="G662" s="4" t="n"/>
+      <c r="H662" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I662" s="4" t="inlineStr"/>
+      <c r="J662" s="4" t="inlineStr"/>
+      <c r="K662" s="4" t="inlineStr"/>
+      <c r="L662" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M662" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N662" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O662" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P662" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q662" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R662" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S662" s="4" t="n"/>
+      <c r="T662" s="4" t="n"/>
+      <c r="U662" s="4" t="n"/>
+      <c r="V662" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W662" s="4" t="inlineStr"/>
+      <c r="X662" s="4" t="n"/>
+      <c r="Y662" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z662" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA662" s="4" t="n"/>
+      <c r="AB662" s="4" t="n"/>
+      <c r="AC662" s="4" t="n"/>
+      <c r="AD662" s="4" t="n"/>
+      <c r="AE662" s="4" t="n"/>
+      <c r="AF662" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="663">
+      <c r="A663" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B663" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C663" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D663" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E663" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F663" s="6" t="n"/>
+      <c r="G663" s="6" t="n"/>
+      <c r="H663" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I663" s="6" t="inlineStr"/>
+      <c r="J663" s="6" t="inlineStr"/>
+      <c r="K663" s="6" t="inlineStr"/>
+      <c r="L663" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M663" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N663" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O663" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P663" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q663" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R663" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S663" s="6" t="n"/>
+      <c r="T663" s="6" t="n"/>
+      <c r="U663" s="6" t="n"/>
+      <c r="V663" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W663" s="6" t="inlineStr"/>
+      <c r="X663" s="6" t="n"/>
+      <c r="Y663" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z663" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA663" s="6" t="n"/>
+      <c r="AB663" s="6" t="n"/>
+      <c r="AC663" s="6" t="n"/>
+      <c r="AD663" s="6" t="n"/>
+      <c r="AE663" s="6" t="n"/>
+      <c r="AF663" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="664">
+      <c r="A664" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B664" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C664" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D664" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E664" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F664" s="4" t="n"/>
+      <c r="G664" s="4" t="n"/>
+      <c r="H664" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I664" s="4" t="inlineStr"/>
+      <c r="J664" s="4" t="inlineStr"/>
+      <c r="K664" s="4" t="inlineStr"/>
+      <c r="L664" s="4" t="n">
+        <v>84</v>
+      </c>
+      <c r="M664" s="4" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N664" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O664" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P664" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q664" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R664" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S664" s="4" t="n"/>
+      <c r="T664" s="4" t="n"/>
+      <c r="U664" s="4" t="n"/>
+      <c r="V664" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W664" s="4" t="inlineStr"/>
+      <c r="X664" s="4" t="n"/>
+      <c r="Y664" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z664" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA664" s="4" t="n"/>
+      <c r="AB664" s="4" t="n"/>
+      <c r="AC664" s="4" t="n"/>
+      <c r="AD664" s="4" t="n"/>
+      <c r="AE664" s="4" t="n"/>
+      <c r="AF664" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B665" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C665" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D665" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E665" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F665" s="6" t="n"/>
+      <c r="G665" s="6" t="n"/>
+      <c r="H665" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I665" s="6" t="inlineStr"/>
+      <c r="J665" s="6" t="inlineStr"/>
+      <c r="K665" s="6" t="inlineStr"/>
+      <c r="L665" s="6" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M665" s="6" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N665" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O665" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P665" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q665" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R665" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S665" s="6" t="n"/>
+      <c r="T665" s="6" t="n"/>
+      <c r="U665" s="6" t="n"/>
+      <c r="V665" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W665" s="6" t="inlineStr"/>
+      <c r="X665" s="6" t="n"/>
+      <c r="Y665" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z665" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA665" s="6" t="n"/>
+      <c r="AB665" s="6" t="n"/>
+      <c r="AC665" s="6" t="n"/>
+      <c r="AD665" s="6" t="n"/>
+      <c r="AE665" s="6" t="n"/>
+      <c r="AF665" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B666" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C666" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D666" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E666" s="4" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F666" s="4" t="n"/>
+      <c r="G666" s="4" t="n"/>
+      <c r="H666" s="4" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I666" s="4" t="inlineStr"/>
+      <c r="J666" s="4" t="inlineStr"/>
+      <c r="K666" s="4" t="inlineStr"/>
+      <c r="L666" s="4" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M666" s="4" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N666" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O666" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P666" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q666" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R666" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S666" s="4" t="n"/>
+      <c r="T666" s="4" t="n"/>
+      <c r="U666" s="4" t="n"/>
+      <c r="V666" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W666" s="4" t="inlineStr"/>
+      <c r="X666" s="4" t="n"/>
+      <c r="Y666" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z666" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA666" s="4" t="n"/>
+      <c r="AB666" s="4" t="n"/>
+      <c r="AC666" s="4" t="n"/>
+      <c r="AD666" s="4" t="n"/>
+      <c r="AE666" s="4" t="n"/>
+      <c r="AF666" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="667">
+      <c r="A667" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B667" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C667" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D667" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E667" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F667" s="6" t="n"/>
+      <c r="G667" s="6" t="n"/>
+      <c r="H667" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I667" s="6" t="inlineStr"/>
+      <c r="J667" s="6" t="inlineStr"/>
+      <c r="K667" s="6" t="inlineStr"/>
+      <c r="L667" s="6" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M667" s="6" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N667" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O667" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P667" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q667" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R667" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S667" s="6" t="n"/>
+      <c r="T667" s="6" t="n"/>
+      <c r="U667" s="6" t="n"/>
+      <c r="V667" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W667" s="6" t="inlineStr"/>
+      <c r="X667" s="6" t="n"/>
+      <c r="Y667" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z667" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA667" s="6" t="n"/>
+      <c r="AB667" s="6" t="n"/>
+      <c r="AC667" s="6" t="n"/>
+      <c r="AD667" s="6" t="n"/>
+      <c r="AE667" s="6" t="n"/>
+      <c r="AF667" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="668">
+      <c r="A668" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B668" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C668" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D668" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E668" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F668" s="4" t="n"/>
+      <c r="G668" s="4" t="n"/>
+      <c r="H668" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I668" s="4" t="inlineStr"/>
+      <c r="J668" s="4" t="inlineStr"/>
+      <c r="K668" s="4" t="inlineStr"/>
+      <c r="L668" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M668" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N668" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O668" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P668" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q668" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R668" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S668" s="4" t="n"/>
+      <c r="T668" s="4" t="n"/>
+      <c r="U668" s="4" t="n"/>
+      <c r="V668" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W668" s="4" t="inlineStr"/>
+      <c r="X668" s="4" t="n"/>
+      <c r="Y668" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z668" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA668" s="4" t="n"/>
+      <c r="AB668" s="4" t="n"/>
+      <c r="AC668" s="4" t="n"/>
+      <c r="AD668" s="4" t="n"/>
+      <c r="AE668" s="4" t="n"/>
+      <c r="AF668" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="669">
+      <c r="A669" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B669" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C669" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D669" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E669" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F669" s="6" t="n"/>
+      <c r="G669" s="6" t="n"/>
+      <c r="H669" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I669" s="6" t="inlineStr"/>
+      <c r="J669" s="6" t="inlineStr"/>
+      <c r="K669" s="6" t="inlineStr"/>
+      <c r="L669" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M669" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N669" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O669" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P669" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q669" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R669" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S669" s="6" t="n"/>
+      <c r="T669" s="6" t="n"/>
+      <c r="U669" s="6" t="n"/>
+      <c r="V669" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W669" s="6" t="inlineStr"/>
+      <c r="X669" s="6" t="n"/>
+      <c r="Y669" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z669" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA669" s="6" t="n"/>
+      <c r="AB669" s="6" t="n"/>
+      <c r="AC669" s="6" t="n"/>
+      <c r="AD669" s="6" t="n"/>
+      <c r="AE669" s="6" t="n"/>
+      <c r="AF669" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="670">
+      <c r="A670" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B670" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C670" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D670" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E670" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F670" s="4" t="n"/>
+      <c r="G670" s="4" t="n"/>
+      <c r="H670" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I670" s="4" t="inlineStr"/>
+      <c r="J670" s="4" t="inlineStr"/>
+      <c r="K670" s="4" t="inlineStr"/>
+      <c r="L670" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M670" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N670" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O670" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P670" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q670" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R670" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S670" s="4" t="n"/>
+      <c r="T670" s="4" t="n"/>
+      <c r="U670" s="4" t="n"/>
+      <c r="V670" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W670" s="4" t="inlineStr"/>
+      <c r="X670" s="4" t="n"/>
+      <c r="Y670" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z670" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA670" s="4" t="n"/>
+      <c r="AB670" s="4" t="n"/>
+      <c r="AC670" s="4" t="n"/>
+      <c r="AD670" s="4" t="n"/>
+      <c r="AE670" s="4" t="n"/>
+      <c r="AF670" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="671">
+      <c r="A671" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B671" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C671" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D671" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E671" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F671" s="6" t="n"/>
+      <c r="G671" s="6" t="n"/>
+      <c r="H671" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I671" s="6" t="inlineStr"/>
+      <c r="J671" s="6" t="inlineStr"/>
+      <c r="K671" s="6" t="inlineStr"/>
+      <c r="L671" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M671" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N671" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O671" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P671" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q671" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R671" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S671" s="6" t="n"/>
+      <c r="T671" s="6" t="n"/>
+      <c r="U671" s="6" t="n"/>
+      <c r="V671" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W671" s="6" t="inlineStr"/>
+      <c r="X671" s="6" t="n"/>
+      <c r="Y671" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z671" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA671" s="6" t="n"/>
+      <c r="AB671" s="6" t="n"/>
+      <c r="AC671" s="6" t="n"/>
+      <c r="AD671" s="6" t="n"/>
+      <c r="AE671" s="6" t="n"/>
+      <c r="AF671" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="672">
+      <c r="A672" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B672" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C672" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D672" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E672" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F672" s="4" t="n"/>
+      <c r="G672" s="4" t="n"/>
+      <c r="H672" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I672" s="4" t="inlineStr"/>
+      <c r="J672" s="4" t="inlineStr"/>
+      <c r="K672" s="4" t="inlineStr"/>
+      <c r="L672" s="4" t="n"/>
+      <c r="M672" s="4" t="n"/>
+      <c r="N672" s="4" t="n"/>
+      <c r="O672" s="4" t="n"/>
+      <c r="P672" s="4" t="n"/>
+      <c r="Q672" s="4" t="n"/>
+      <c r="R672" s="4" t="n"/>
+      <c r="S672" s="4" t="n"/>
+      <c r="T672" s="4" t="n"/>
+      <c r="U672" s="4" t="n"/>
+      <c r="V672" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W672" s="4" t="inlineStr"/>
+      <c r="X672" s="4" t="n"/>
+      <c r="Y672" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z672" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA672" s="4" t="n"/>
+      <c r="AB672" s="4" t="n"/>
+      <c r="AC672" s="4" t="n"/>
+      <c r="AD672" s="4" t="n"/>
+      <c r="AE672" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF672" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="673">
+      <c r="A673" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B673" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C673" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D673" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E673" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F673" s="6" t="n"/>
+      <c r="G673" s="6" t="n"/>
+      <c r="H673" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I673" s="6" t="inlineStr"/>
+      <c r="J673" s="6" t="inlineStr"/>
+      <c r="K673" s="6" t="inlineStr"/>
+      <c r="L673" s="6" t="n"/>
+      <c r="M673" s="6" t="n"/>
+      <c r="N673" s="6" t="n"/>
+      <c r="O673" s="6" t="n"/>
+      <c r="P673" s="6" t="n"/>
+      <c r="Q673" s="6" t="n"/>
+      <c r="R673" s="6" t="n"/>
+      <c r="S673" s="6" t="n"/>
+      <c r="T673" s="6" t="n"/>
+      <c r="U673" s="6" t="n"/>
+      <c r="V673" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W673" s="6" t="inlineStr"/>
+      <c r="X673" s="6" t="n"/>
+      <c r="Y673" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z673" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA673" s="6" t="n"/>
+      <c r="AB673" s="6" t="n"/>
+      <c r="AC673" s="6" t="n"/>
+      <c r="AD673" s="6" t="n"/>
+      <c r="AE673" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF673" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="674">
+      <c r="A674" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B674" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C674" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D674" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E674" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F674" s="4" t="n"/>
+      <c r="G674" s="4" t="n"/>
+      <c r="H674" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I674" s="4" t="inlineStr"/>
+      <c r="J674" s="4" t="inlineStr"/>
+      <c r="K674" s="4" t="inlineStr"/>
+      <c r="L674" s="4" t="n"/>
+      <c r="M674" s="4" t="n"/>
+      <c r="N674" s="4" t="n"/>
+      <c r="O674" s="4" t="n"/>
+      <c r="P674" s="4" t="n"/>
+      <c r="Q674" s="4" t="n"/>
+      <c r="R674" s="4" t="n"/>
+      <c r="S674" s="4" t="n"/>
+      <c r="T674" s="4" t="n"/>
+      <c r="U674" s="4" t="n"/>
+      <c r="V674" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W674" s="4" t="inlineStr"/>
+      <c r="X674" s="4" t="n"/>
+      <c r="Y674" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z674" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA674" s="4" t="n"/>
+      <c r="AB674" s="4" t="n"/>
+      <c r="AC674" s="4" t="n"/>
+      <c r="AD674" s="4" t="n"/>
+      <c r="AE674" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF674" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="675">
+      <c r="A675" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B675" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C675" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D675" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E675" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F675" s="6" t="n"/>
+      <c r="G675" s="6" t="n"/>
+      <c r="H675" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I675" s="6" t="inlineStr"/>
+      <c r="J675" s="6" t="inlineStr"/>
+      <c r="K675" s="6" t="inlineStr"/>
+      <c r="L675" s="6" t="n"/>
+      <c r="M675" s="6" t="n"/>
+      <c r="N675" s="6" t="n"/>
+      <c r="O675" s="6" t="n"/>
+      <c r="P675" s="6" t="n"/>
+      <c r="Q675" s="6" t="n"/>
+      <c r="R675" s="6" t="n"/>
+      <c r="S675" s="6" t="n"/>
+      <c r="T675" s="6" t="n"/>
+      <c r="U675" s="6" t="n"/>
+      <c r="V675" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W675" s="6" t="inlineStr"/>
+      <c r="X675" s="6" t="n"/>
+      <c r="Y675" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z675" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA675" s="6" t="n"/>
+      <c r="AB675" s="6" t="n"/>
+      <c r="AC675" s="6" t="n"/>
+      <c r="AD675" s="6" t="n"/>
+      <c r="AE675" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF675" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="676">
+      <c r="A676" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B676" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C676" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D676" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E676" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F676" s="4" t="n"/>
+      <c r="G676" s="4" t="n"/>
+      <c r="H676" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I676" s="4" t="inlineStr"/>
+      <c r="J676" s="4" t="inlineStr"/>
+      <c r="K676" s="4" t="inlineStr"/>
+      <c r="L676" s="4" t="n"/>
+      <c r="M676" s="4" t="n"/>
+      <c r="N676" s="4" t="n"/>
+      <c r="O676" s="4" t="n"/>
+      <c r="P676" s="4" t="n"/>
+      <c r="Q676" s="4" t="n"/>
+      <c r="R676" s="4" t="n"/>
+      <c r="S676" s="4" t="n"/>
+      <c r="T676" s="4" t="n"/>
+      <c r="U676" s="4" t="n"/>
+      <c r="V676" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W676" s="4" t="inlineStr"/>
+      <c r="X676" s="4" t="n"/>
+      <c r="Y676" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z676" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA676" s="4" t="n"/>
+      <c r="AB676" s="4" t="n"/>
+      <c r="AC676" s="4" t="n"/>
+      <c r="AD676" s="4" t="n"/>
+      <c r="AE676" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF676" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="677">
+      <c r="A677" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B677" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C677" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D677" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E677" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F677" s="6" t="n"/>
+      <c r="G677" s="6" t="n"/>
+      <c r="H677" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I677" s="6" t="inlineStr"/>
+      <c r="J677" s="6" t="inlineStr"/>
+      <c r="K677" s="6" t="inlineStr"/>
+      <c r="L677" s="6" t="n"/>
+      <c r="M677" s="6" t="n"/>
+      <c r="N677" s="6" t="n"/>
+      <c r="O677" s="6" t="n"/>
+      <c r="P677" s="6" t="n"/>
+      <c r="Q677" s="6" t="n"/>
+      <c r="R677" s="6" t="n"/>
+      <c r="S677" s="6" t="n"/>
+      <c r="T677" s="6" t="n"/>
+      <c r="U677" s="6" t="n"/>
+      <c r="V677" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W677" s="6" t="inlineStr"/>
+      <c r="X677" s="6" t="n"/>
+      <c r="Y677" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z677" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA677" s="6" t="n"/>
+      <c r="AB677" s="6" t="n"/>
+      <c r="AC677" s="6" t="n"/>
+      <c r="AD677" s="6" t="n"/>
+      <c r="AE677" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF677" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="678">
+      <c r="A678" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B678" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C678" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D678" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E678" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F678" s="4" t="n"/>
+      <c r="G678" s="4" t="n"/>
+      <c r="H678" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I678" s="4" t="inlineStr"/>
+      <c r="J678" s="4" t="inlineStr"/>
+      <c r="K678" s="4" t="inlineStr"/>
+      <c r="L678" s="4" t="n"/>
+      <c r="M678" s="4" t="n"/>
+      <c r="N678" s="4" t="n"/>
+      <c r="O678" s="4" t="n"/>
+      <c r="P678" s="4" t="n"/>
+      <c r="Q678" s="4" t="n"/>
+      <c r="R678" s="4" t="n"/>
+      <c r="S678" s="4" t="n"/>
+      <c r="T678" s="4" t="n"/>
+      <c r="U678" s="4" t="n"/>
+      <c r="V678" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W678" s="4" t="inlineStr"/>
+      <c r="X678" s="4" t="n"/>
+      <c r="Y678" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z678" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA678" s="4" t="n"/>
+      <c r="AB678" s="4" t="n"/>
+      <c r="AC678" s="4" t="n"/>
+      <c r="AD678" s="4" t="n"/>
+      <c r="AE678" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF678" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="679">
+      <c r="A679" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B679" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C679" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D679" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E679" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F679" s="6" t="n"/>
+      <c r="G679" s="6" t="n"/>
+      <c r="H679" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I679" s="6" t="inlineStr"/>
+      <c r="J679" s="6" t="inlineStr"/>
+      <c r="K679" s="6" t="inlineStr"/>
+      <c r="L679" s="6" t="n"/>
+      <c r="M679" s="6" t="n"/>
+      <c r="N679" s="6" t="n"/>
+      <c r="O679" s="6" t="n"/>
+      <c r="P679" s="6" t="n"/>
+      <c r="Q679" s="6" t="n"/>
+      <c r="R679" s="6" t="n"/>
+      <c r="S679" s="6" t="n"/>
+      <c r="T679" s="6" t="n"/>
+      <c r="U679" s="6" t="n"/>
+      <c r="V679" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W679" s="6" t="inlineStr"/>
+      <c r="X679" s="6" t="n"/>
+      <c r="Y679" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z679" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA679" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB679" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC679" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD679" s="6" t="n"/>
+      <c r="AE679" s="6" t="n"/>
+      <c r="AF679" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="680">
+      <c r="A680" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B680" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C680" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D680" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E680" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F680" s="4" t="n"/>
+      <c r="G680" s="4" t="n"/>
+      <c r="H680" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I680" s="4" t="inlineStr"/>
+      <c r="J680" s="4" t="inlineStr"/>
+      <c r="K680" s="4" t="inlineStr"/>
+      <c r="L680" s="4" t="n"/>
+      <c r="M680" s="4" t="n"/>
+      <c r="N680" s="4" t="n"/>
+      <c r="O680" s="4" t="n"/>
+      <c r="P680" s="4" t="n"/>
+      <c r="Q680" s="4" t="n"/>
+      <c r="R680" s="4" t="n"/>
+      <c r="S680" s="4" t="n"/>
+      <c r="T680" s="4" t="n"/>
+      <c r="U680" s="4" t="n"/>
+      <c r="V680" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W680" s="4" t="inlineStr"/>
+      <c r="X680" s="4" t="n"/>
+      <c r="Y680" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z680" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA680" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB680" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC680" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD680" s="4" t="n"/>
+      <c r="AE680" s="4" t="n"/>
+      <c r="AF680" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="681">
+      <c r="A681" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B681" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C681" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D681" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E681" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F681" s="6" t="n"/>
+      <c r="G681" s="6" t="n"/>
+      <c r="H681" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I681" s="6" t="inlineStr"/>
+      <c r="J681" s="6" t="inlineStr"/>
+      <c r="K681" s="6" t="inlineStr"/>
+      <c r="L681" s="6" t="n"/>
+      <c r="M681" s="6" t="n"/>
+      <c r="N681" s="6" t="n"/>
+      <c r="O681" s="6" t="n"/>
+      <c r="P681" s="6" t="n"/>
+      <c r="Q681" s="6" t="n"/>
+      <c r="R681" s="6" t="n"/>
+      <c r="S681" s="6" t="n"/>
+      <c r="T681" s="6" t="n"/>
+      <c r="U681" s="6" t="n"/>
+      <c r="V681" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W681" s="6" t="inlineStr"/>
+      <c r="X681" s="6" t="n"/>
+      <c r="Y681" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z681" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA681" s="6" t="n"/>
+      <c r="AB681" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC681" s="6" t="n"/>
+      <c r="AD681" s="6" t="n"/>
+      <c r="AE681" s="6" t="n"/>
+      <c r="AF681" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="682">
+      <c r="A682" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-07</t>
+        </is>
+      </c>
+      <c r="B682" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C682" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D682" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E682" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F682" s="4" t="n"/>
+      <c r="G682" s="4" t="n"/>
+      <c r="H682" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I682" s="4" t="inlineStr"/>
+      <c r="J682" s="4" t="inlineStr"/>
+      <c r="K682" s="4" t="inlineStr"/>
+      <c r="L682" s="4" t="n"/>
+      <c r="M682" s="4" t="n"/>
+      <c r="N682" s="4" t="n"/>
+      <c r="O682" s="4" t="n"/>
+      <c r="P682" s="4" t="n"/>
+      <c r="Q682" s="4" t="n"/>
+      <c r="R682" s="4" t="n"/>
+      <c r="S682" s="4" t="n"/>
+      <c r="T682" s="4" t="n"/>
+      <c r="U682" s="4" t="n"/>
+      <c r="V682" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W682" s="4" t="inlineStr"/>
+      <c r="X682" s="4" t="n"/>
+      <c r="Y682" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z682" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA682" s="4" t="n"/>
+      <c r="AB682" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC682" s="4" t="n"/>
+      <c r="AD682" s="4" t="n"/>
+      <c r="AE682" s="4" t="n"/>
+      <c r="AF682" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-08
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF682"/>
+  <dimension ref="A1:AF718"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -54218,6 +54218,2840 @@
         <v>1</v>
       </c>
     </row>
+    <row r="683">
+      <c r="A683" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B683" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C683" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D683" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E683" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F683" s="4" t="n"/>
+      <c r="G683" s="4" t="n"/>
+      <c r="H683" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I683" s="4" t="inlineStr"/>
+      <c r="J683" s="4" t="inlineStr"/>
+      <c r="K683" s="4" t="inlineStr"/>
+      <c r="L683" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M683" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N683" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O683" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P683" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q683" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R683" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S683" s="4" t="n"/>
+      <c r="T683" s="4" t="n"/>
+      <c r="U683" s="4" t="n"/>
+      <c r="V683" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W683" s="4" t="inlineStr"/>
+      <c r="X683" s="4" t="n"/>
+      <c r="Y683" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z683" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA683" s="4" t="n"/>
+      <c r="AB683" s="4" t="n"/>
+      <c r="AC683" s="4" t="n"/>
+      <c r="AD683" s="4" t="n"/>
+      <c r="AE683" s="4" t="n"/>
+      <c r="AF683" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="684">
+      <c r="A684" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B684" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C684" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D684" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E684" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F684" s="6" t="n"/>
+      <c r="G684" s="6" t="n"/>
+      <c r="H684" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I684" s="6" t="inlineStr"/>
+      <c r="J684" s="6" t="inlineStr"/>
+      <c r="K684" s="6" t="inlineStr"/>
+      <c r="L684" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M684" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N684" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O684" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P684" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q684" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R684" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S684" s="6" t="n"/>
+      <c r="T684" s="6" t="n"/>
+      <c r="U684" s="6" t="n"/>
+      <c r="V684" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W684" s="6" t="inlineStr"/>
+      <c r="X684" s="6" t="n"/>
+      <c r="Y684" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z684" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA684" s="6" t="n"/>
+      <c r="AB684" s="6" t="n"/>
+      <c r="AC684" s="6" t="n"/>
+      <c r="AD684" s="6" t="n"/>
+      <c r="AE684" s="6" t="n"/>
+      <c r="AF684" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="685">
+      <c r="A685" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B685" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C685" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D685" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E685" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F685" s="4" t="n"/>
+      <c r="G685" s="4" t="n"/>
+      <c r="H685" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I685" s="4" t="inlineStr"/>
+      <c r="J685" s="4" t="inlineStr"/>
+      <c r="K685" s="4" t="inlineStr"/>
+      <c r="L685" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M685" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N685" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O685" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P685" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q685" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R685" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S685" s="4" t="n"/>
+      <c r="T685" s="4" t="n"/>
+      <c r="U685" s="4" t="n"/>
+      <c r="V685" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W685" s="4" t="inlineStr"/>
+      <c r="X685" s="4" t="n"/>
+      <c r="Y685" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z685" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA685" s="4" t="n"/>
+      <c r="AB685" s="4" t="n"/>
+      <c r="AC685" s="4" t="n"/>
+      <c r="AD685" s="4" t="n"/>
+      <c r="AE685" s="4" t="n"/>
+      <c r="AF685" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="686">
+      <c r="A686" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B686" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C686" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D686" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E686" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F686" s="6" t="n"/>
+      <c r="G686" s="6" t="n"/>
+      <c r="H686" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I686" s="6" t="inlineStr"/>
+      <c r="J686" s="6" t="inlineStr"/>
+      <c r="K686" s="6" t="inlineStr"/>
+      <c r="L686" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M686" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N686" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O686" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P686" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q686" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R686" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S686" s="6" t="n"/>
+      <c r="T686" s="6" t="n"/>
+      <c r="U686" s="6" t="n"/>
+      <c r="V686" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W686" s="6" t="inlineStr"/>
+      <c r="X686" s="6" t="n"/>
+      <c r="Y686" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z686" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA686" s="6" t="n"/>
+      <c r="AB686" s="6" t="n"/>
+      <c r="AC686" s="6" t="n"/>
+      <c r="AD686" s="6" t="n"/>
+      <c r="AE686" s="6" t="n"/>
+      <c r="AF686" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="687">
+      <c r="A687" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B687" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C687" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D687" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E687" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F687" s="4" t="n"/>
+      <c r="G687" s="4" t="n"/>
+      <c r="H687" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I687" s="4" t="inlineStr"/>
+      <c r="J687" s="4" t="inlineStr"/>
+      <c r="K687" s="4" t="inlineStr"/>
+      <c r="L687" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M687" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N687" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O687" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P687" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q687" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R687" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S687" s="4" t="n"/>
+      <c r="T687" s="4" t="n"/>
+      <c r="U687" s="4" t="n"/>
+      <c r="V687" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W687" s="4" t="inlineStr"/>
+      <c r="X687" s="4" t="n"/>
+      <c r="Y687" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z687" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA687" s="4" t="n"/>
+      <c r="AB687" s="4" t="n"/>
+      <c r="AC687" s="4" t="n"/>
+      <c r="AD687" s="4" t="n"/>
+      <c r="AE687" s="4" t="n"/>
+      <c r="AF687" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="688">
+      <c r="A688" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B688" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C688" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D688" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E688" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F688" s="6" t="n"/>
+      <c r="G688" s="6" t="n"/>
+      <c r="H688" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I688" s="6" t="inlineStr"/>
+      <c r="J688" s="6" t="inlineStr"/>
+      <c r="K688" s="6" t="inlineStr"/>
+      <c r="L688" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M688" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N688" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O688" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P688" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q688" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R688" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S688" s="6" t="n"/>
+      <c r="T688" s="6" t="n"/>
+      <c r="U688" s="6" t="n"/>
+      <c r="V688" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W688" s="6" t="inlineStr"/>
+      <c r="X688" s="6" t="n"/>
+      <c r="Y688" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z688" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA688" s="6" t="n"/>
+      <c r="AB688" s="6" t="n"/>
+      <c r="AC688" s="6" t="n"/>
+      <c r="AD688" s="6" t="n"/>
+      <c r="AE688" s="6" t="n"/>
+      <c r="AF688" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="689">
+      <c r="A689" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B689" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C689" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D689" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E689" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F689" s="4" t="n"/>
+      <c r="G689" s="4" t="n"/>
+      <c r="H689" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I689" s="4" t="inlineStr"/>
+      <c r="J689" s="4" t="inlineStr"/>
+      <c r="K689" s="4" t="inlineStr"/>
+      <c r="L689" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M689" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N689" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O689" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P689" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q689" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R689" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S689" s="4" t="n"/>
+      <c r="T689" s="4" t="n"/>
+      <c r="U689" s="4" t="n"/>
+      <c r="V689" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W689" s="4" t="inlineStr"/>
+      <c r="X689" s="4" t="n"/>
+      <c r="Y689" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z689" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA689" s="4" t="n"/>
+      <c r="AB689" s="4" t="n"/>
+      <c r="AC689" s="4" t="n"/>
+      <c r="AD689" s="4" t="n"/>
+      <c r="AE689" s="4" t="n"/>
+      <c r="AF689" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="690">
+      <c r="A690" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B690" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C690" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D690" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E690" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F690" s="6" t="n"/>
+      <c r="G690" s="6" t="n"/>
+      <c r="H690" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I690" s="6" t="inlineStr"/>
+      <c r="J690" s="6" t="inlineStr"/>
+      <c r="K690" s="6" t="inlineStr"/>
+      <c r="L690" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M690" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N690" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O690" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P690" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q690" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R690" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S690" s="6" t="n"/>
+      <c r="T690" s="6" t="n"/>
+      <c r="U690" s="6" t="n"/>
+      <c r="V690" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W690" s="6" t="inlineStr"/>
+      <c r="X690" s="6" t="n"/>
+      <c r="Y690" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z690" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA690" s="6" t="n"/>
+      <c r="AB690" s="6" t="n"/>
+      <c r="AC690" s="6" t="n"/>
+      <c r="AD690" s="6" t="n"/>
+      <c r="AE690" s="6" t="n"/>
+      <c r="AF690" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="691">
+      <c r="A691" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B691" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C691" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D691" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E691" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F691" s="4" t="n"/>
+      <c r="G691" s="4" t="n"/>
+      <c r="H691" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I691" s="4" t="inlineStr"/>
+      <c r="J691" s="4" t="inlineStr"/>
+      <c r="K691" s="4" t="inlineStr"/>
+      <c r="L691" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M691" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N691" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O691" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P691" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q691" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R691" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S691" s="4" t="n"/>
+      <c r="T691" s="4" t="n"/>
+      <c r="U691" s="4" t="n"/>
+      <c r="V691" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W691" s="4" t="inlineStr"/>
+      <c r="X691" s="4" t="n"/>
+      <c r="Y691" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z691" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA691" s="4" t="n"/>
+      <c r="AB691" s="4" t="n"/>
+      <c r="AC691" s="4" t="n"/>
+      <c r="AD691" s="4" t="n"/>
+      <c r="AE691" s="4" t="n"/>
+      <c r="AF691" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="692">
+      <c r="A692" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B692" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C692" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D692" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E692" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F692" s="6" t="n"/>
+      <c r="G692" s="6" t="n"/>
+      <c r="H692" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I692" s="6" t="inlineStr"/>
+      <c r="J692" s="6" t="inlineStr"/>
+      <c r="K692" s="6" t="inlineStr"/>
+      <c r="L692" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M692" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N692" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O692" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P692" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q692" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R692" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S692" s="6" t="n"/>
+      <c r="T692" s="6" t="n"/>
+      <c r="U692" s="6" t="n"/>
+      <c r="V692" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W692" s="6" t="inlineStr"/>
+      <c r="X692" s="6" t="n"/>
+      <c r="Y692" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z692" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA692" s="6" t="n"/>
+      <c r="AB692" s="6" t="n"/>
+      <c r="AC692" s="6" t="n"/>
+      <c r="AD692" s="6" t="n"/>
+      <c r="AE692" s="6" t="n"/>
+      <c r="AF692" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="693">
+      <c r="A693" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B693" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C693" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D693" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E693" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F693" s="4" t="n"/>
+      <c r="G693" s="4" t="n"/>
+      <c r="H693" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I693" s="4" t="inlineStr"/>
+      <c r="J693" s="4" t="inlineStr"/>
+      <c r="K693" s="4" t="inlineStr"/>
+      <c r="L693" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M693" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N693" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O693" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P693" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q693" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R693" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S693" s="4" t="n"/>
+      <c r="T693" s="4" t="n"/>
+      <c r="U693" s="4" t="n"/>
+      <c r="V693" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W693" s="4" t="inlineStr"/>
+      <c r="X693" s="4" t="n"/>
+      <c r="Y693" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z693" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA693" s="4" t="n"/>
+      <c r="AB693" s="4" t="n"/>
+      <c r="AC693" s="4" t="n"/>
+      <c r="AD693" s="4" t="n"/>
+      <c r="AE693" s="4" t="n"/>
+      <c r="AF693" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="694">
+      <c r="A694" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B694" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C694" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D694" s="6" t="inlineStr">
+        <is>
+          <t>480g</t>
+        </is>
+      </c>
+      <c r="E694" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F694" s="6" t="n"/>
+      <c r="G694" s="6" t="n"/>
+      <c r="H694" s="6" t="n">
+        <v>62.48</v>
+      </c>
+      <c r="I694" s="6" t="inlineStr"/>
+      <c r="J694" s="6" t="inlineStr"/>
+      <c r="K694" s="6" t="inlineStr"/>
+      <c r="L694" s="6" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="M694" s="6" t="n">
+        <v>2.286</v>
+      </c>
+      <c r="N694" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O694" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P694" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q694" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R694" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S694" s="6" t="n"/>
+      <c r="T694" s="6" t="n"/>
+      <c r="U694" s="6" t="n"/>
+      <c r="V694" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W694" s="6" t="inlineStr"/>
+      <c r="X694" s="6" t="n"/>
+      <c r="Y694" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z694" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA694" s="6" t="n"/>
+      <c r="AB694" s="6" t="n"/>
+      <c r="AC694" s="6" t="n"/>
+      <c r="AD694" s="6" t="n"/>
+      <c r="AE694" s="6" t="n"/>
+      <c r="AF694" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="695">
+      <c r="A695" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B695" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C695" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D695" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E695" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F695" s="4" t="n"/>
+      <c r="G695" s="4" t="n"/>
+      <c r="H695" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I695" s="4" t="inlineStr"/>
+      <c r="J695" s="4" t="inlineStr"/>
+      <c r="K695" s="4" t="inlineStr"/>
+      <c r="L695" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M695" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N695" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O695" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P695" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q695" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R695" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S695" s="4" t="n"/>
+      <c r="T695" s="4" t="n"/>
+      <c r="U695" s="4" t="n"/>
+      <c r="V695" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W695" s="4" t="inlineStr"/>
+      <c r="X695" s="4" t="n"/>
+      <c r="Y695" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z695" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA695" s="4" t="n"/>
+      <c r="AB695" s="4" t="n"/>
+      <c r="AC695" s="4" t="n"/>
+      <c r="AD695" s="4" t="n"/>
+      <c r="AE695" s="4" t="n"/>
+      <c r="AF695" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="696">
+      <c r="A696" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B696" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C696" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D696" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E696" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F696" s="6" t="n"/>
+      <c r="G696" s="6" t="n"/>
+      <c r="H696" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I696" s="6" t="inlineStr"/>
+      <c r="J696" s="6" t="inlineStr"/>
+      <c r="K696" s="6" t="inlineStr"/>
+      <c r="L696" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M696" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N696" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O696" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P696" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q696" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R696" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S696" s="6" t="n"/>
+      <c r="T696" s="6" t="n"/>
+      <c r="U696" s="6" t="n"/>
+      <c r="V696" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W696" s="6" t="inlineStr"/>
+      <c r="X696" s="6" t="n"/>
+      <c r="Y696" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z696" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA696" s="6" t="n"/>
+      <c r="AB696" s="6" t="n"/>
+      <c r="AC696" s="6" t="n"/>
+      <c r="AD696" s="6" t="n"/>
+      <c r="AE696" s="6" t="n"/>
+      <c r="AF696" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="697">
+      <c r="A697" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B697" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C697" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D697" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E697" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F697" s="4" t="n"/>
+      <c r="G697" s="4" t="n"/>
+      <c r="H697" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I697" s="4" t="inlineStr"/>
+      <c r="J697" s="4" t="inlineStr"/>
+      <c r="K697" s="4" t="inlineStr"/>
+      <c r="L697" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M697" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N697" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O697" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P697" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q697" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R697" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S697" s="4" t="n"/>
+      <c r="T697" s="4" t="n"/>
+      <c r="U697" s="4" t="n"/>
+      <c r="V697" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W697" s="4" t="inlineStr"/>
+      <c r="X697" s="4" t="n"/>
+      <c r="Y697" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z697" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA697" s="4" t="n"/>
+      <c r="AB697" s="4" t="n"/>
+      <c r="AC697" s="4" t="n"/>
+      <c r="AD697" s="4" t="n"/>
+      <c r="AE697" s="4" t="n"/>
+      <c r="AF697" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="698">
+      <c r="A698" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B698" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C698" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D698" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E698" s="6" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F698" s="6" t="n"/>
+      <c r="G698" s="6" t="n"/>
+      <c r="H698" s="6" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I698" s="6" t="inlineStr"/>
+      <c r="J698" s="6" t="inlineStr"/>
+      <c r="K698" s="6" t="inlineStr"/>
+      <c r="L698" s="6" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M698" s="6" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N698" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O698" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P698" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q698" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R698" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S698" s="6" t="n"/>
+      <c r="T698" s="6" t="n"/>
+      <c r="U698" s="6" t="n"/>
+      <c r="V698" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W698" s="6" t="inlineStr"/>
+      <c r="X698" s="6" t="n"/>
+      <c r="Y698" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z698" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA698" s="6" t="n"/>
+      <c r="AB698" s="6" t="n"/>
+      <c r="AC698" s="6" t="n"/>
+      <c r="AD698" s="6" t="n"/>
+      <c r="AE698" s="6" t="n"/>
+      <c r="AF698" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="699">
+      <c r="A699" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B699" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C699" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D699" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E699" s="4" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F699" s="4" t="n"/>
+      <c r="G699" s="4" t="n"/>
+      <c r="H699" s="4" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I699" s="4" t="inlineStr"/>
+      <c r="J699" s="4" t="inlineStr"/>
+      <c r="K699" s="4" t="inlineStr"/>
+      <c r="L699" s="4" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M699" s="4" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N699" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O699" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P699" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q699" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R699" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S699" s="4" t="n"/>
+      <c r="T699" s="4" t="n"/>
+      <c r="U699" s="4" t="n"/>
+      <c r="V699" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W699" s="4" t="inlineStr"/>
+      <c r="X699" s="4" t="n"/>
+      <c r="Y699" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z699" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA699" s="4" t="n"/>
+      <c r="AB699" s="4" t="n"/>
+      <c r="AC699" s="4" t="n"/>
+      <c r="AD699" s="4" t="n"/>
+      <c r="AE699" s="4" t="n"/>
+      <c r="AF699" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="700">
+      <c r="A700" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B700" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C700" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D700" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E700" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F700" s="6" t="n"/>
+      <c r="G700" s="6" t="n"/>
+      <c r="H700" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I700" s="6" t="inlineStr"/>
+      <c r="J700" s="6" t="inlineStr"/>
+      <c r="K700" s="6" t="inlineStr"/>
+      <c r="L700" s="6" t="n">
+        <v>84</v>
+      </c>
+      <c r="M700" s="6" t="n">
+        <v>2.52</v>
+      </c>
+      <c r="N700" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O700" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P700" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q700" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R700" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S700" s="6" t="n"/>
+      <c r="T700" s="6" t="n"/>
+      <c r="U700" s="6" t="n"/>
+      <c r="V700" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W700" s="6" t="inlineStr"/>
+      <c r="X700" s="6" t="n"/>
+      <c r="Y700" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z700" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA700" s="6" t="n"/>
+      <c r="AB700" s="6" t="n"/>
+      <c r="AC700" s="6" t="n"/>
+      <c r="AD700" s="6" t="n"/>
+      <c r="AE700" s="6" t="n"/>
+      <c r="AF700" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="701">
+      <c r="A701" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B701" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C701" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D701" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E701" s="4" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F701" s="4" t="n"/>
+      <c r="G701" s="4" t="n"/>
+      <c r="H701" s="4" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I701" s="4" t="inlineStr"/>
+      <c r="J701" s="4" t="inlineStr"/>
+      <c r="K701" s="4" t="inlineStr"/>
+      <c r="L701" s="4" t="n">
+        <v>66.33</v>
+      </c>
+      <c r="M701" s="4" t="n">
+        <v>1.99</v>
+      </c>
+      <c r="N701" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O701" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P701" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q701" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R701" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S701" s="4" t="n"/>
+      <c r="T701" s="4" t="n"/>
+      <c r="U701" s="4" t="n"/>
+      <c r="V701" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W701" s="4" t="inlineStr"/>
+      <c r="X701" s="4" t="n"/>
+      <c r="Y701" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z701" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA701" s="4" t="n"/>
+      <c r="AB701" s="4" t="n"/>
+      <c r="AC701" s="4" t="n"/>
+      <c r="AD701" s="4" t="n"/>
+      <c r="AE701" s="4" t="n"/>
+      <c r="AF701" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="702">
+      <c r="A702" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B702" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C702" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D702" s="6" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E702" s="6" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F702" s="6" t="n"/>
+      <c r="G702" s="6" t="n"/>
+      <c r="H702" s="6" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I702" s="6" t="inlineStr"/>
+      <c r="J702" s="6" t="inlineStr"/>
+      <c r="K702" s="6" t="inlineStr"/>
+      <c r="L702" s="6" t="n">
+        <v>78.51000000000001</v>
+      </c>
+      <c r="M702" s="6" t="n">
+        <v>2.355</v>
+      </c>
+      <c r="N702" s="6" t="n">
+        <v>85</v>
+      </c>
+      <c r="O702" s="6" t="n">
+        <v>355</v>
+      </c>
+      <c r="P702" s="6" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q702" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R702" s="6" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S702" s="6" t="n"/>
+      <c r="T702" s="6" t="n"/>
+      <c r="U702" s="6" t="n"/>
+      <c r="V702" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W702" s="6" t="inlineStr"/>
+      <c r="X702" s="6" t="n"/>
+      <c r="Y702" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z702" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA702" s="6" t="n"/>
+      <c r="AB702" s="6" t="n"/>
+      <c r="AC702" s="6" t="n"/>
+      <c r="AD702" s="6" t="n"/>
+      <c r="AE702" s="6" t="n"/>
+      <c r="AF702" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="703">
+      <c r="A703" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B703" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C703" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D703" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E703" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F703" s="4" t="n"/>
+      <c r="G703" s="4" t="n"/>
+      <c r="H703" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I703" s="4" t="inlineStr"/>
+      <c r="J703" s="4" t="inlineStr"/>
+      <c r="K703" s="4" t="inlineStr"/>
+      <c r="L703" s="4" t="n">
+        <v>59.28</v>
+      </c>
+      <c r="M703" s="4" t="n">
+        <v>1.778</v>
+      </c>
+      <c r="N703" s="4" t="n">
+        <v>85</v>
+      </c>
+      <c r="O703" s="4" t="n">
+        <v>355</v>
+      </c>
+      <c r="P703" s="4" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="Q703" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R703" s="4" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="S703" s="4" t="n"/>
+      <c r="T703" s="4" t="n"/>
+      <c r="U703" s="4" t="n"/>
+      <c r="V703" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          INGRÉDIENTS: Mélange de protéines (92%) (isolat de protéines de lactosérum hydrolysées [lait] (contient agent antimoussant [dioxyde de silicium], huile de colza), peptides de collagène hydrolysés d’origine bovine), arômes naturels, édulcorant (sucralose), concentré de betterave, agents antimoussants (dioxyde de silicium, diméthylpolysiloxane), vitamine C.
+INFORMATIONS RELATIVES AUX ALLERGÈNES: Les allergènes apparaissent en gras dans la liste des ingrédients.</t>
+        </is>
+      </c>
+      <c r="W703" s="4" t="inlineStr"/>
+      <c r="X703" s="4" t="n"/>
+      <c r="Y703" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z703" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA703" s="4" t="n"/>
+      <c r="AB703" s="4" t="n"/>
+      <c r="AC703" s="4" t="n"/>
+      <c r="AD703" s="4" t="n"/>
+      <c r="AE703" s="4" t="n"/>
+      <c r="AF703" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="704">
+      <c r="A704" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B704" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C704" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D704" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E704" s="6" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F704" s="6" t="n"/>
+      <c r="G704" s="6" t="n"/>
+      <c r="H704" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I704" s="6" t="inlineStr"/>
+      <c r="J704" s="6" t="inlineStr"/>
+      <c r="K704" s="6" t="inlineStr"/>
+      <c r="L704" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M704" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N704" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O704" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P704" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q704" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R704" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S704" s="6" t="n"/>
+      <c r="T704" s="6" t="n"/>
+      <c r="U704" s="6" t="n"/>
+      <c r="V704" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W704" s="6" t="inlineStr"/>
+      <c r="X704" s="6" t="n"/>
+      <c r="Y704" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z704" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA704" s="6" t="n"/>
+      <c r="AB704" s="6" t="n"/>
+      <c r="AC704" s="6" t="n"/>
+      <c r="AD704" s="6" t="n"/>
+      <c r="AE704" s="6" t="n"/>
+      <c r="AF704" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="705">
+      <c r="A705" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B705" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C705" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D705" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E705" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F705" s="4" t="n"/>
+      <c r="G705" s="4" t="n"/>
+      <c r="H705" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I705" s="4" t="inlineStr"/>
+      <c r="J705" s="4" t="inlineStr"/>
+      <c r="K705" s="4" t="inlineStr"/>
+      <c r="L705" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M705" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N705" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O705" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P705" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q705" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R705" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S705" s="4" t="n"/>
+      <c r="T705" s="4" t="n"/>
+      <c r="U705" s="4" t="n"/>
+      <c r="V705" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W705" s="4" t="inlineStr"/>
+      <c r="X705" s="4" t="n"/>
+      <c r="Y705" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z705" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA705" s="4" t="n"/>
+      <c r="AB705" s="4" t="n"/>
+      <c r="AC705" s="4" t="n"/>
+      <c r="AD705" s="4" t="n"/>
+      <c r="AE705" s="4" t="n"/>
+      <c r="AF705" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="706">
+      <c r="A706" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B706" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C706" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D706" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E706" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F706" s="6" t="n"/>
+      <c r="G706" s="6" t="n"/>
+      <c r="H706" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I706" s="6" t="inlineStr"/>
+      <c r="J706" s="6" t="inlineStr"/>
+      <c r="K706" s="6" t="inlineStr"/>
+      <c r="L706" s="6" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M706" s="6" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N706" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O706" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P706" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q706" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R706" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S706" s="6" t="n"/>
+      <c r="T706" s="6" t="n"/>
+      <c r="U706" s="6" t="n"/>
+      <c r="V706" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W706" s="6" t="inlineStr"/>
+      <c r="X706" s="6" t="n"/>
+      <c r="Y706" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z706" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA706" s="6" t="n"/>
+      <c r="AB706" s="6" t="n"/>
+      <c r="AC706" s="6" t="n"/>
+      <c r="AD706" s="6" t="n"/>
+      <c r="AE706" s="6" t="n"/>
+      <c r="AF706" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="707">
+      <c r="A707" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B707" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C707" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D707" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E707" s="4" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F707" s="4" t="n"/>
+      <c r="G707" s="4" t="n"/>
+      <c r="H707" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I707" s="4" t="inlineStr"/>
+      <c r="J707" s="4" t="inlineStr"/>
+      <c r="K707" s="4" t="inlineStr"/>
+      <c r="L707" s="4" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M707" s="4" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N707" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O707" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P707" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q707" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R707" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S707" s="4" t="n"/>
+      <c r="T707" s="4" t="n"/>
+      <c r="U707" s="4" t="n"/>
+      <c r="V707" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W707" s="4" t="inlineStr"/>
+      <c r="X707" s="4" t="n"/>
+      <c r="Y707" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z707" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA707" s="4" t="n"/>
+      <c r="AB707" s="4" t="n"/>
+      <c r="AC707" s="4" t="n"/>
+      <c r="AD707" s="4" t="n"/>
+      <c r="AE707" s="4" t="n"/>
+      <c r="AF707" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="708">
+      <c r="A708" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B708" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C708" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D708" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E708" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F708" s="6" t="n"/>
+      <c r="G708" s="6" t="n"/>
+      <c r="H708" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I708" s="6" t="inlineStr"/>
+      <c r="J708" s="6" t="inlineStr"/>
+      <c r="K708" s="6" t="inlineStr"/>
+      <c r="L708" s="6" t="n"/>
+      <c r="M708" s="6" t="n"/>
+      <c r="N708" s="6" t="n"/>
+      <c r="O708" s="6" t="n"/>
+      <c r="P708" s="6" t="n"/>
+      <c r="Q708" s="6" t="n"/>
+      <c r="R708" s="6" t="n"/>
+      <c r="S708" s="6" t="n"/>
+      <c r="T708" s="6" t="n"/>
+      <c r="U708" s="6" t="n"/>
+      <c r="V708" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W708" s="6" t="inlineStr"/>
+      <c r="X708" s="6" t="n"/>
+      <c r="Y708" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z708" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA708" s="6" t="n"/>
+      <c r="AB708" s="6" t="n"/>
+      <c r="AC708" s="6" t="n"/>
+      <c r="AD708" s="6" t="n"/>
+      <c r="AE708" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF708" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="709">
+      <c r="A709" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B709" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C709" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D709" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E709" s="4" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F709" s="4" t="n"/>
+      <c r="G709" s="4" t="n"/>
+      <c r="H709" s="4" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I709" s="4" t="inlineStr"/>
+      <c r="J709" s="4" t="inlineStr"/>
+      <c r="K709" s="4" t="inlineStr"/>
+      <c r="L709" s="4" t="n"/>
+      <c r="M709" s="4" t="n"/>
+      <c r="N709" s="4" t="n"/>
+      <c r="O709" s="4" t="n"/>
+      <c r="P709" s="4" t="n"/>
+      <c r="Q709" s="4" t="n"/>
+      <c r="R709" s="4" t="n"/>
+      <c r="S709" s="4" t="n"/>
+      <c r="T709" s="4" t="n"/>
+      <c r="U709" s="4" t="n"/>
+      <c r="V709" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W709" s="4" t="inlineStr"/>
+      <c r="X709" s="4" t="n"/>
+      <c r="Y709" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z709" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA709" s="4" t="n"/>
+      <c r="AB709" s="4" t="n"/>
+      <c r="AC709" s="4" t="n"/>
+      <c r="AD709" s="4" t="n"/>
+      <c r="AE709" s="4" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF709" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="710">
+      <c r="A710" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B710" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C710" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D710" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E710" s="6" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F710" s="6" t="n"/>
+      <c r="G710" s="6" t="n"/>
+      <c r="H710" s="6" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I710" s="6" t="inlineStr"/>
+      <c r="J710" s="6" t="inlineStr"/>
+      <c r="K710" s="6" t="inlineStr"/>
+      <c r="L710" s="6" t="n"/>
+      <c r="M710" s="6" t="n"/>
+      <c r="N710" s="6" t="n"/>
+      <c r="O710" s="6" t="n"/>
+      <c r="P710" s="6" t="n"/>
+      <c r="Q710" s="6" t="n"/>
+      <c r="R710" s="6" t="n"/>
+      <c r="S710" s="6" t="n"/>
+      <c r="T710" s="6" t="n"/>
+      <c r="U710" s="6" t="n"/>
+      <c r="V710" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W710" s="6" t="inlineStr"/>
+      <c r="X710" s="6" t="n"/>
+      <c r="Y710" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z710" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA710" s="6" t="n"/>
+      <c r="AB710" s="6" t="n"/>
+      <c r="AC710" s="6" t="n"/>
+      <c r="AD710" s="6" t="n"/>
+      <c r="AE710" s="6" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF710" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="711">
+      <c r="A711" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B711" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C711" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D711" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E711" s="4" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F711" s="4" t="n"/>
+      <c r="G711" s="4" t="n"/>
+      <c r="H711" s="4" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I711" s="4" t="inlineStr"/>
+      <c r="J711" s="4" t="inlineStr"/>
+      <c r="K711" s="4" t="inlineStr"/>
+      <c r="L711" s="4" t="n"/>
+      <c r="M711" s="4" t="n"/>
+      <c r="N711" s="4" t="n"/>
+      <c r="O711" s="4" t="n"/>
+      <c r="P711" s="4" t="n"/>
+      <c r="Q711" s="4" t="n"/>
+      <c r="R711" s="4" t="n"/>
+      <c r="S711" s="4" t="n"/>
+      <c r="T711" s="4" t="n"/>
+      <c r="U711" s="4" t="n"/>
+      <c r="V711" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W711" s="4" t="inlineStr"/>
+      <c r="X711" s="4" t="n"/>
+      <c r="Y711" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z711" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA711" s="4" t="n"/>
+      <c r="AB711" s="4" t="n"/>
+      <c r="AC711" s="4" t="n"/>
+      <c r="AD711" s="4" t="n"/>
+      <c r="AE711" s="4" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF711" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="712">
+      <c r="A712" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B712" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C712" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D712" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E712" s="6" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F712" s="6" t="n"/>
+      <c r="G712" s="6" t="n"/>
+      <c r="H712" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I712" s="6" t="inlineStr"/>
+      <c r="J712" s="6" t="inlineStr"/>
+      <c r="K712" s="6" t="inlineStr"/>
+      <c r="L712" s="6" t="n"/>
+      <c r="M712" s="6" t="n"/>
+      <c r="N712" s="6" t="n"/>
+      <c r="O712" s="6" t="n"/>
+      <c r="P712" s="6" t="n"/>
+      <c r="Q712" s="6" t="n"/>
+      <c r="R712" s="6" t="n"/>
+      <c r="S712" s="6" t="n"/>
+      <c r="T712" s="6" t="n"/>
+      <c r="U712" s="6" t="n"/>
+      <c r="V712" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W712" s="6" t="inlineStr"/>
+      <c r="X712" s="6" t="n"/>
+      <c r="Y712" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z712" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA712" s="6" t="n"/>
+      <c r="AB712" s="6" t="n"/>
+      <c r="AC712" s="6" t="n"/>
+      <c r="AD712" s="6" t="n"/>
+      <c r="AE712" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF712" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="713">
+      <c r="A713" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B713" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C713" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D713" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E713" s="4" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F713" s="4" t="n"/>
+      <c r="G713" s="4" t="n"/>
+      <c r="H713" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I713" s="4" t="inlineStr"/>
+      <c r="J713" s="4" t="inlineStr"/>
+      <c r="K713" s="4" t="inlineStr"/>
+      <c r="L713" s="4" t="n"/>
+      <c r="M713" s="4" t="n"/>
+      <c r="N713" s="4" t="n"/>
+      <c r="O713" s="4" t="n"/>
+      <c r="P713" s="4" t="n"/>
+      <c r="Q713" s="4" t="n"/>
+      <c r="R713" s="4" t="n"/>
+      <c r="S713" s="4" t="n"/>
+      <c r="T713" s="4" t="n"/>
+      <c r="U713" s="4" t="n"/>
+      <c r="V713" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W713" s="4" t="inlineStr"/>
+      <c r="X713" s="4" t="n"/>
+      <c r="Y713" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z713" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA713" s="4" t="n"/>
+      <c r="AB713" s="4" t="n"/>
+      <c r="AC713" s="4" t="n"/>
+      <c r="AD713" s="4" t="n"/>
+      <c r="AE713" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF713" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="714">
+      <c r="A714" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B714" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C714" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D714" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E714" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F714" s="6" t="n"/>
+      <c r="G714" s="6" t="n"/>
+      <c r="H714" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I714" s="6" t="inlineStr"/>
+      <c r="J714" s="6" t="inlineStr"/>
+      <c r="K714" s="6" t="inlineStr"/>
+      <c r="L714" s="6" t="n"/>
+      <c r="M714" s="6" t="n"/>
+      <c r="N714" s="6" t="n"/>
+      <c r="O714" s="6" t="n"/>
+      <c r="P714" s="6" t="n"/>
+      <c r="Q714" s="6" t="n"/>
+      <c r="R714" s="6" t="n"/>
+      <c r="S714" s="6" t="n"/>
+      <c r="T714" s="6" t="n"/>
+      <c r="U714" s="6" t="n"/>
+      <c r="V714" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W714" s="6" t="inlineStr"/>
+      <c r="X714" s="6" t="n"/>
+      <c r="Y714" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z714" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA714" s="6" t="n"/>
+      <c r="AB714" s="6" t="n"/>
+      <c r="AC714" s="6" t="n"/>
+      <c r="AD714" s="6" t="n"/>
+      <c r="AE714" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF714" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="715">
+      <c r="A715" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B715" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C715" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D715" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E715" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F715" s="4" t="n"/>
+      <c r="G715" s="4" t="n"/>
+      <c r="H715" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I715" s="4" t="inlineStr"/>
+      <c r="J715" s="4" t="inlineStr"/>
+      <c r="K715" s="4" t="inlineStr"/>
+      <c r="L715" s="4" t="n"/>
+      <c r="M715" s="4" t="n"/>
+      <c r="N715" s="4" t="n"/>
+      <c r="O715" s="4" t="n"/>
+      <c r="P715" s="4" t="n"/>
+      <c r="Q715" s="4" t="n"/>
+      <c r="R715" s="4" t="n"/>
+      <c r="S715" s="4" t="n"/>
+      <c r="T715" s="4" t="n"/>
+      <c r="U715" s="4" t="n"/>
+      <c r="V715" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W715" s="4" t="inlineStr"/>
+      <c r="X715" s="4" t="n"/>
+      <c r="Y715" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z715" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA715" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB715" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC715" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD715" s="4" t="n"/>
+      <c r="AE715" s="4" t="n"/>
+      <c r="AF715" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="716">
+      <c r="A716" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B716" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C716" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D716" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E716" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F716" s="6" t="n"/>
+      <c r="G716" s="6" t="n"/>
+      <c r="H716" s="6" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I716" s="6" t="inlineStr"/>
+      <c r="J716" s="6" t="inlineStr"/>
+      <c r="K716" s="6" t="inlineStr"/>
+      <c r="L716" s="6" t="n"/>
+      <c r="M716" s="6" t="n"/>
+      <c r="N716" s="6" t="n"/>
+      <c r="O716" s="6" t="n"/>
+      <c r="P716" s="6" t="n"/>
+      <c r="Q716" s="6" t="n"/>
+      <c r="R716" s="6" t="n"/>
+      <c r="S716" s="6" t="n"/>
+      <c r="T716" s="6" t="n"/>
+      <c r="U716" s="6" t="n"/>
+      <c r="V716" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W716" s="6" t="inlineStr"/>
+      <c r="X716" s="6" t="n"/>
+      <c r="Y716" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z716" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA716" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB716" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC716" s="6" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD716" s="6" t="n"/>
+      <c r="AE716" s="6" t="n"/>
+      <c r="AF716" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="717">
+      <c r="A717" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B717" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C717" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D717" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E717" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F717" s="4" t="n"/>
+      <c r="G717" s="4" t="n"/>
+      <c r="H717" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I717" s="4" t="inlineStr"/>
+      <c r="J717" s="4" t="inlineStr"/>
+      <c r="K717" s="4" t="inlineStr"/>
+      <c r="L717" s="4" t="n"/>
+      <c r="M717" s="4" t="n"/>
+      <c r="N717" s="4" t="n"/>
+      <c r="O717" s="4" t="n"/>
+      <c r="P717" s="4" t="n"/>
+      <c r="Q717" s="4" t="n"/>
+      <c r="R717" s="4" t="n"/>
+      <c r="S717" s="4" t="n"/>
+      <c r="T717" s="4" t="n"/>
+      <c r="U717" s="4" t="n"/>
+      <c r="V717" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W717" s="4" t="inlineStr"/>
+      <c r="X717" s="4" t="n"/>
+      <c r="Y717" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z717" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA717" s="4" t="n"/>
+      <c r="AB717" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC717" s="4" t="n"/>
+      <c r="AD717" s="4" t="n"/>
+      <c r="AE717" s="4" t="n"/>
+      <c r="AF717" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="718">
+      <c r="A718" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-08</t>
+        </is>
+      </c>
+      <c r="B718" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C718" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D718" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E718" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F718" s="6" t="n"/>
+      <c r="G718" s="6" t="n"/>
+      <c r="H718" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I718" s="6" t="inlineStr"/>
+      <c r="J718" s="6" t="inlineStr"/>
+      <c r="K718" s="6" t="inlineStr"/>
+      <c r="L718" s="6" t="n"/>
+      <c r="M718" s="6" t="n"/>
+      <c r="N718" s="6" t="n"/>
+      <c r="O718" s="6" t="n"/>
+      <c r="P718" s="6" t="n"/>
+      <c r="Q718" s="6" t="n"/>
+      <c r="R718" s="6" t="n"/>
+      <c r="S718" s="6" t="n"/>
+      <c r="T718" s="6" t="n"/>
+      <c r="U718" s="6" t="n"/>
+      <c r="V718" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W718" s="6" t="inlineStr"/>
+      <c r="X718" s="6" t="n"/>
+      <c r="Y718" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z718" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA718" s="6" t="n"/>
+      <c r="AB718" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC718" s="6" t="n"/>
+      <c r="AD718" s="6" t="n"/>
+      <c r="AE718" s="6" t="n"/>
+      <c r="AF718" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-09
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF718"/>
+  <dimension ref="A1:AF754"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -57052,6 +57052,2836 @@
         <v>1</v>
       </c>
     </row>
+    <row r="719">
+      <c r="A719" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B719" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C719" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D719" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E719" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F719" s="4" t="n"/>
+      <c r="G719" s="4" t="n"/>
+      <c r="H719" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I719" s="4" t="inlineStr"/>
+      <c r="J719" s="4" t="inlineStr"/>
+      <c r="K719" s="4" t="inlineStr"/>
+      <c r="L719" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M719" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N719" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O719" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P719" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q719" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R719" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S719" s="4" t="n"/>
+      <c r="T719" s="4" t="n"/>
+      <c r="U719" s="4" t="n"/>
+      <c r="V719" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W719" s="4" t="inlineStr"/>
+      <c r="X719" s="4" t="n"/>
+      <c r="Y719" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z719" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA719" s="4" t="n"/>
+      <c r="AB719" s="4" t="n"/>
+      <c r="AC719" s="4" t="n"/>
+      <c r="AD719" s="4" t="n"/>
+      <c r="AE719" s="4" t="n"/>
+      <c r="AF719" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="720">
+      <c r="A720" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B720" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C720" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D720" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E720" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F720" s="6" t="n"/>
+      <c r="G720" s="6" t="n"/>
+      <c r="H720" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I720" s="6" t="inlineStr"/>
+      <c r="J720" s="6" t="inlineStr"/>
+      <c r="K720" s="6" t="inlineStr"/>
+      <c r="L720" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M720" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N720" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O720" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P720" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q720" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R720" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S720" s="6" t="n"/>
+      <c r="T720" s="6" t="n"/>
+      <c r="U720" s="6" t="n"/>
+      <c r="V720" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W720" s="6" t="inlineStr"/>
+      <c r="X720" s="6" t="n"/>
+      <c r="Y720" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z720" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA720" s="6" t="n"/>
+      <c r="AB720" s="6" t="n"/>
+      <c r="AC720" s="6" t="n"/>
+      <c r="AD720" s="6" t="n"/>
+      <c r="AE720" s="6" t="n"/>
+      <c r="AF720" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="721">
+      <c r="A721" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B721" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C721" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D721" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E721" s="4" t="n">
+        <v>17.99</v>
+      </c>
+      <c r="F721" s="4" t="n"/>
+      <c r="G721" s="4" t="n"/>
+      <c r="H721" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I721" s="4" t="inlineStr"/>
+      <c r="J721" s="4" t="inlineStr"/>
+      <c r="K721" s="4" t="inlineStr"/>
+      <c r="L721" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M721" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N721" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O721" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P721" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q721" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R721" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S721" s="4" t="n"/>
+      <c r="T721" s="4" t="n"/>
+      <c r="U721" s="4" t="n"/>
+      <c r="V721" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W721" s="4" t="inlineStr"/>
+      <c r="X721" s="4" t="n"/>
+      <c r="Y721" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z721" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA721" s="4" t="n"/>
+      <c r="AB721" s="4" t="n"/>
+      <c r="AC721" s="4" t="n"/>
+      <c r="AD721" s="4" t="n"/>
+      <c r="AE721" s="4" t="n"/>
+      <c r="AF721" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="722">
+      <c r="A722" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B722" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C722" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D722" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E722" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F722" s="6" t="n"/>
+      <c r="G722" s="6" t="n"/>
+      <c r="H722" s="6" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I722" s="6" t="inlineStr"/>
+      <c r="J722" s="6" t="inlineStr"/>
+      <c r="K722" s="6" t="inlineStr"/>
+      <c r="L722" s="6" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M722" s="6" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N722" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O722" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P722" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q722" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R722" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S722" s="6" t="n"/>
+      <c r="T722" s="6" t="n"/>
+      <c r="U722" s="6" t="n"/>
+      <c r="V722" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W722" s="6" t="inlineStr"/>
+      <c r="X722" s="6" t="n"/>
+      <c r="Y722" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z722" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA722" s="6" t="n"/>
+      <c r="AB722" s="6" t="n"/>
+      <c r="AC722" s="6" t="n"/>
+      <c r="AD722" s="6" t="n"/>
+      <c r="AE722" s="6" t="n"/>
+      <c r="AF722" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="723">
+      <c r="A723" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B723" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C723" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D723" s="4" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E723" s="4" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F723" s="4" t="n"/>
+      <c r="G723" s="4" t="n"/>
+      <c r="H723" s="4" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I723" s="4" t="inlineStr"/>
+      <c r="J723" s="4" t="inlineStr"/>
+      <c r="K723" s="4" t="inlineStr"/>
+      <c r="L723" s="4" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M723" s="4" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N723" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O723" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P723" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q723" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R723" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S723" s="4" t="n"/>
+      <c r="T723" s="4" t="n"/>
+      <c r="U723" s="4" t="n"/>
+      <c r="V723" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W723" s="4" t="inlineStr"/>
+      <c r="X723" s="4" t="n"/>
+      <c r="Y723" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z723" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA723" s="4" t="n"/>
+      <c r="AB723" s="4" t="n"/>
+      <c r="AC723" s="4" t="n"/>
+      <c r="AD723" s="4" t="n"/>
+      <c r="AE723" s="4" t="n"/>
+      <c r="AF723" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="724">
+      <c r="A724" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B724" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C724" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D724" s="6" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E724" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F724" s="6" t="n"/>
+      <c r="G724" s="6" t="n"/>
+      <c r="H724" s="6" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I724" s="6" t="inlineStr"/>
+      <c r="J724" s="6" t="inlineStr"/>
+      <c r="K724" s="6" t="inlineStr"/>
+      <c r="L724" s="6" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M724" s="6" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N724" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O724" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P724" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q724" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R724" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S724" s="6" t="n"/>
+      <c r="T724" s="6" t="n"/>
+      <c r="U724" s="6" t="n"/>
+      <c r="V724" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W724" s="6" t="inlineStr"/>
+      <c r="X724" s="6" t="n"/>
+      <c r="Y724" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z724" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA724" s="6" t="n"/>
+      <c r="AB724" s="6" t="n"/>
+      <c r="AC724" s="6" t="n"/>
+      <c r="AD724" s="6" t="n"/>
+      <c r="AE724" s="6" t="n"/>
+      <c r="AF724" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="725">
+      <c r="A725" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B725" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C725" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D725" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E725" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F725" s="4" t="n"/>
+      <c r="G725" s="4" t="n"/>
+      <c r="H725" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I725" s="4" t="inlineStr"/>
+      <c r="J725" s="4" t="inlineStr"/>
+      <c r="K725" s="4" t="inlineStr"/>
+      <c r="L725" s="4" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M725" s="4" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N725" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O725" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P725" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q725" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R725" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S725" s="4" t="n"/>
+      <c r="T725" s="4" t="n"/>
+      <c r="U725" s="4" t="n"/>
+      <c r="V725" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W725" s="4" t="inlineStr"/>
+      <c r="X725" s="4" t="n"/>
+      <c r="Y725" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z725" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA725" s="4" t="n"/>
+      <c r="AB725" s="4" t="n"/>
+      <c r="AC725" s="4" t="n"/>
+      <c r="AD725" s="4" t="n"/>
+      <c r="AE725" s="4" t="n"/>
+      <c r="AF725" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="726">
+      <c r="A726" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B726" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C726" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D726" s="6" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E726" s="6" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F726" s="6" t="n"/>
+      <c r="G726" s="6" t="n"/>
+      <c r="H726" s="6" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I726" s="6" t="inlineStr"/>
+      <c r="J726" s="6" t="inlineStr"/>
+      <c r="K726" s="6" t="inlineStr"/>
+      <c r="L726" s="6" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M726" s="6" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N726" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O726" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P726" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q726" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R726" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S726" s="6" t="n"/>
+      <c r="T726" s="6" t="n"/>
+      <c r="U726" s="6" t="n"/>
+      <c r="V726" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W726" s="6" t="inlineStr"/>
+      <c r="X726" s="6" t="n"/>
+      <c r="Y726" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z726" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA726" s="6" t="n"/>
+      <c r="AB726" s="6" t="n"/>
+      <c r="AC726" s="6" t="n"/>
+      <c r="AD726" s="6" t="n"/>
+      <c r="AE726" s="6" t="n"/>
+      <c r="AF726" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="727">
+      <c r="A727" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B727" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C727" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D727" s="4" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E727" s="4" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F727" s="4" t="n"/>
+      <c r="G727" s="4" t="n"/>
+      <c r="H727" s="4" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I727" s="4" t="inlineStr"/>
+      <c r="J727" s="4" t="inlineStr"/>
+      <c r="K727" s="4" t="inlineStr"/>
+      <c r="L727" s="4" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M727" s="4" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N727" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O727" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P727" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q727" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R727" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S727" s="4" t="n"/>
+      <c r="T727" s="4" t="n"/>
+      <c r="U727" s="4" t="n"/>
+      <c r="V727" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W727" s="4" t="inlineStr"/>
+      <c r="X727" s="4" t="n"/>
+      <c r="Y727" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z727" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA727" s="4" t="n"/>
+      <c r="AB727" s="4" t="n"/>
+      <c r="AC727" s="4" t="n"/>
+      <c r="AD727" s="4" t="n"/>
+      <c r="AE727" s="4" t="n"/>
+      <c r="AF727" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="728">
+      <c r="A728" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B728" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C728" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D728" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E728" s="6" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F728" s="6" t="n"/>
+      <c r="G728" s="6" t="n"/>
+      <c r="H728" s="6" t="n">
+        <v>30</v>
+      </c>
+      <c r="I728" s="6" t="inlineStr"/>
+      <c r="J728" s="6" t="inlineStr"/>
+      <c r="K728" s="6" t="inlineStr"/>
+      <c r="L728" s="6" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M728" s="6" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N728" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O728" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P728" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q728" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R728" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S728" s="6" t="n"/>
+      <c r="T728" s="6" t="n"/>
+      <c r="U728" s="6" t="n"/>
+      <c r="V728" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W728" s="6" t="inlineStr"/>
+      <c r="X728" s="6" t="n"/>
+      <c r="Y728" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z728" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA728" s="6" t="n"/>
+      <c r="AB728" s="6" t="n"/>
+      <c r="AC728" s="6" t="n"/>
+      <c r="AD728" s="6" t="n"/>
+      <c r="AE728" s="6" t="n"/>
+      <c r="AF728" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="729">
+      <c r="A729" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B729" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C729" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D729" s="4" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E729" s="4" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F729" s="4" t="n"/>
+      <c r="G729" s="4" t="n"/>
+      <c r="H729" s="4" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I729" s="4" t="inlineStr"/>
+      <c r="J729" s="4" t="inlineStr"/>
+      <c r="K729" s="4" t="inlineStr"/>
+      <c r="L729" s="4" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M729" s="4" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N729" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O729" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P729" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q729" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R729" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S729" s="4" t="n"/>
+      <c r="T729" s="4" t="n"/>
+      <c r="U729" s="4" t="n"/>
+      <c r="V729" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W729" s="4" t="inlineStr"/>
+      <c r="X729" s="4" t="n"/>
+      <c r="Y729" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z729" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA729" s="4" t="n"/>
+      <c r="AB729" s="4" t="n"/>
+      <c r="AC729" s="4" t="n"/>
+      <c r="AD729" s="4" t="n"/>
+      <c r="AE729" s="4" t="n"/>
+      <c r="AF729" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="730">
+      <c r="A730" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B730" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C730" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D730" s="6" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E730" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F730" s="6" t="n"/>
+      <c r="G730" s="6" t="n"/>
+      <c r="H730" s="6" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I730" s="6" t="inlineStr"/>
+      <c r="J730" s="6" t="inlineStr"/>
+      <c r="K730" s="6" t="inlineStr"/>
+      <c r="L730" s="6" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M730" s="6" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N730" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O730" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P730" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q730" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R730" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S730" s="6" t="n"/>
+      <c r="T730" s="6" t="n"/>
+      <c r="U730" s="6" t="n"/>
+      <c r="V730" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W730" s="6" t="inlineStr"/>
+      <c r="X730" s="6" t="n"/>
+      <c r="Y730" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z730" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA730" s="6" t="n"/>
+      <c r="AB730" s="6" t="n"/>
+      <c r="AC730" s="6" t="n"/>
+      <c r="AD730" s="6" t="n"/>
+      <c r="AE730" s="6" t="n"/>
+      <c r="AF730" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="731">
+      <c r="A731" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B731" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C731" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D731" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E731" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F731" s="4" t="n"/>
+      <c r="G731" s="4" t="n"/>
+      <c r="H731" s="4" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I731" s="4" t="inlineStr"/>
+      <c r="J731" s="4" t="inlineStr"/>
+      <c r="K731" s="4" t="inlineStr"/>
+      <c r="L731" s="4" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M731" s="4" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N731" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O731" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P731" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q731" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R731" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S731" s="4" t="n"/>
+      <c r="T731" s="4" t="n"/>
+      <c r="U731" s="4" t="n"/>
+      <c r="V731" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W731" s="4" t="inlineStr"/>
+      <c r="X731" s="4" t="n"/>
+      <c r="Y731" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z731" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA731" s="4" t="n"/>
+      <c r="AB731" s="4" t="n"/>
+      <c r="AC731" s="4" t="n"/>
+      <c r="AD731" s="4" t="n"/>
+      <c r="AE731" s="4" t="n"/>
+      <c r="AF731" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="732">
+      <c r="A732" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B732" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C732" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D732" s="6" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E732" s="6" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F732" s="6" t="n"/>
+      <c r="G732" s="6" t="n"/>
+      <c r="H732" s="6" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I732" s="6" t="inlineStr"/>
+      <c r="J732" s="6" t="inlineStr"/>
+      <c r="K732" s="6" t="inlineStr"/>
+      <c r="L732" s="6" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M732" s="6" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N732" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O732" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P732" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q732" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R732" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S732" s="6" t="n"/>
+      <c r="T732" s="6" t="n"/>
+      <c r="U732" s="6" t="n"/>
+      <c r="V732" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W732" s="6" t="inlineStr"/>
+      <c r="X732" s="6" t="n"/>
+      <c r="Y732" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z732" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA732" s="6" t="n"/>
+      <c r="AB732" s="6" t="n"/>
+      <c r="AC732" s="6" t="n"/>
+      <c r="AD732" s="6" t="n"/>
+      <c r="AE732" s="6" t="n"/>
+      <c r="AF732" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="733">
+      <c r="A733" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B733" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C733" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D733" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E733" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F733" s="4" t="n"/>
+      <c r="G733" s="4" t="n"/>
+      <c r="H733" s="4" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I733" s="4" t="inlineStr"/>
+      <c r="J733" s="4" t="inlineStr"/>
+      <c r="K733" s="4" t="inlineStr"/>
+      <c r="L733" s="4" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M733" s="4" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N733" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O733" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P733" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q733" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R733" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S733" s="4" t="n"/>
+      <c r="T733" s="4" t="n"/>
+      <c r="U733" s="4" t="n"/>
+      <c r="V733" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W733" s="4" t="inlineStr"/>
+      <c r="X733" s="4" t="n"/>
+      <c r="Y733" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z733" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA733" s="4" t="n"/>
+      <c r="AB733" s="4" t="n"/>
+      <c r="AC733" s="4" t="n"/>
+      <c r="AD733" s="4" t="n"/>
+      <c r="AE733" s="4" t="n"/>
+      <c r="AF733" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="734">
+      <c r="A734" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B734" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C734" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D734" s="6" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E734" s="6" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F734" s="6" t="n"/>
+      <c r="G734" s="6" t="n"/>
+      <c r="H734" s="6" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I734" s="6" t="inlineStr"/>
+      <c r="J734" s="6" t="inlineStr"/>
+      <c r="K734" s="6" t="inlineStr"/>
+      <c r="L734" s="6" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M734" s="6" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N734" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O734" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P734" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q734" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R734" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S734" s="6" t="n"/>
+      <c r="T734" s="6" t="n"/>
+      <c r="U734" s="6" t="n"/>
+      <c r="V734" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W734" s="6" t="inlineStr"/>
+      <c r="X734" s="6" t="n"/>
+      <c r="Y734" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z734" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA734" s="6" t="n"/>
+      <c r="AB734" s="6" t="n"/>
+      <c r="AC734" s="6" t="n"/>
+      <c r="AD734" s="6" t="n"/>
+      <c r="AE734" s="6" t="n"/>
+      <c r="AF734" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="735">
+      <c r="A735" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B735" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C735" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D735" s="4" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E735" s="4" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F735" s="4" t="n"/>
+      <c r="G735" s="4" t="n"/>
+      <c r="H735" s="4" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I735" s="4" t="inlineStr"/>
+      <c r="J735" s="4" t="inlineStr"/>
+      <c r="K735" s="4" t="inlineStr"/>
+      <c r="L735" s="4" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M735" s="4" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N735" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O735" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P735" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q735" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R735" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S735" s="4" t="n"/>
+      <c r="T735" s="4" t="n"/>
+      <c r="U735" s="4" t="n"/>
+      <c r="V735" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W735" s="4" t="inlineStr"/>
+      <c r="X735" s="4" t="n"/>
+      <c r="Y735" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z735" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA735" s="4" t="n"/>
+      <c r="AB735" s="4" t="n"/>
+      <c r="AC735" s="4" t="n"/>
+      <c r="AD735" s="4" t="n"/>
+      <c r="AE735" s="4" t="n"/>
+      <c r="AF735" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="736">
+      <c r="A736" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B736" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C736" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D736" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E736" s="6" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F736" s="6" t="n"/>
+      <c r="G736" s="6" t="n"/>
+      <c r="H736" s="6" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I736" s="6" t="inlineStr"/>
+      <c r="J736" s="6" t="inlineStr"/>
+      <c r="K736" s="6" t="inlineStr"/>
+      <c r="L736" s="6" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M736" s="6" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N736" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O736" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P736" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q736" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R736" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S736" s="6" t="n"/>
+      <c r="T736" s="6" t="n"/>
+      <c r="U736" s="6" t="n"/>
+      <c r="V736" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W736" s="6" t="inlineStr"/>
+      <c r="X736" s="6" t="n"/>
+      <c r="Y736" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z736" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA736" s="6" t="n"/>
+      <c r="AB736" s="6" t="n"/>
+      <c r="AC736" s="6" t="n"/>
+      <c r="AD736" s="6" t="n"/>
+      <c r="AE736" s="6" t="n"/>
+      <c r="AF736" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="737">
+      <c r="A737" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B737" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C737" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D737" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E737" s="4" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F737" s="4" t="n"/>
+      <c r="G737" s="4" t="n"/>
+      <c r="H737" s="4" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I737" s="4" t="inlineStr"/>
+      <c r="J737" s="4" t="inlineStr"/>
+      <c r="K737" s="4" t="inlineStr"/>
+      <c r="L737" s="4" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M737" s="4" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N737" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O737" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P737" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q737" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R737" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S737" s="4" t="n"/>
+      <c r="T737" s="4" t="n"/>
+      <c r="U737" s="4" t="n"/>
+      <c r="V737" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W737" s="4" t="inlineStr"/>
+      <c r="X737" s="4" t="n"/>
+      <c r="Y737" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z737" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA737" s="4" t="n"/>
+      <c r="AB737" s="4" t="n"/>
+      <c r="AC737" s="4" t="n"/>
+      <c r="AD737" s="4" t="n"/>
+      <c r="AE737" s="4" t="n"/>
+      <c r="AF737" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="738">
+      <c r="A738" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B738" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C738" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D738" s="6" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E738" s="6" t="n">
+        <v>58.39</v>
+      </c>
+      <c r="F738" s="6" t="n"/>
+      <c r="G738" s="6" t="n"/>
+      <c r="H738" s="6" t="n">
+        <v>66.73</v>
+      </c>
+      <c r="I738" s="6" t="inlineStr"/>
+      <c r="J738" s="6" t="inlineStr"/>
+      <c r="K738" s="6" t="inlineStr"/>
+      <c r="L738" s="6" t="n">
+        <v>84.47</v>
+      </c>
+      <c r="M738" s="6" t="n">
+        <v>2.534</v>
+      </c>
+      <c r="N738" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O738" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P738" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q738" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R738" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S738" s="6" t="n"/>
+      <c r="T738" s="6" t="n"/>
+      <c r="U738" s="6" t="n"/>
+      <c r="V738" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W738" s="6" t="inlineStr"/>
+      <c r="X738" s="6" t="n"/>
+      <c r="Y738" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z738" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA738" s="6" t="n"/>
+      <c r="AB738" s="6" t="n"/>
+      <c r="AC738" s="6" t="n"/>
+      <c r="AD738" s="6" t="n"/>
+      <c r="AE738" s="6" t="n"/>
+      <c r="AF738" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="739">
+      <c r="A739" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B739" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C739" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D739" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E739" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F739" s="4" t="n"/>
+      <c r="G739" s="4" t="n"/>
+      <c r="H739" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I739" s="4" t="inlineStr"/>
+      <c r="J739" s="4" t="inlineStr"/>
+      <c r="K739" s="4" t="inlineStr"/>
+      <c r="L739" s="4" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M739" s="4" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N739" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O739" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P739" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q739" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R739" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S739" s="4" t="n"/>
+      <c r="T739" s="4" t="n"/>
+      <c r="U739" s="4" t="n"/>
+      <c r="V739" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W739" s="4" t="inlineStr"/>
+      <c r="X739" s="4" t="n"/>
+      <c r="Y739" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z739" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA739" s="4" t="n"/>
+      <c r="AB739" s="4" t="n"/>
+      <c r="AC739" s="4" t="n"/>
+      <c r="AD739" s="4" t="n"/>
+      <c r="AE739" s="4" t="n"/>
+      <c r="AF739" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="740">
+      <c r="A740" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B740" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C740" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D740" s="6" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E740" s="6" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F740" s="6" t="n"/>
+      <c r="G740" s="6" t="n"/>
+      <c r="H740" s="6" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I740" s="6" t="inlineStr"/>
+      <c r="J740" s="6" t="inlineStr"/>
+      <c r="K740" s="6" t="inlineStr"/>
+      <c r="L740" s="6" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M740" s="6" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N740" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O740" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P740" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q740" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R740" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S740" s="6" t="n"/>
+      <c r="T740" s="6" t="n"/>
+      <c r="U740" s="6" t="n"/>
+      <c r="V740" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W740" s="6" t="inlineStr"/>
+      <c r="X740" s="6" t="n"/>
+      <c r="Y740" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z740" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA740" s="6" t="n"/>
+      <c r="AB740" s="6" t="n"/>
+      <c r="AC740" s="6" t="n"/>
+      <c r="AD740" s="6" t="n"/>
+      <c r="AE740" s="6" t="n"/>
+      <c r="AF740" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="741">
+      <c r="A741" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B741" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C741" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D741" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E741" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F741" s="4" t="n"/>
+      <c r="G741" s="4" t="n"/>
+      <c r="H741" s="4" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I741" s="4" t="inlineStr"/>
+      <c r="J741" s="4" t="inlineStr"/>
+      <c r="K741" s="4" t="inlineStr"/>
+      <c r="L741" s="4" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M741" s="4" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N741" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O741" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P741" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q741" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R741" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S741" s="4" t="n"/>
+      <c r="T741" s="4" t="n"/>
+      <c r="U741" s="4" t="n"/>
+      <c r="V741" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W741" s="4" t="inlineStr"/>
+      <c r="X741" s="4" t="n"/>
+      <c r="Y741" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z741" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA741" s="4" t="n"/>
+      <c r="AB741" s="4" t="n"/>
+      <c r="AC741" s="4" t="n"/>
+      <c r="AD741" s="4" t="n"/>
+      <c r="AE741" s="4" t="n"/>
+      <c r="AF741" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="742">
+      <c r="A742" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B742" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C742" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D742" s="6" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E742" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F742" s="6" t="n"/>
+      <c r="G742" s="6" t="n"/>
+      <c r="H742" s="6" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I742" s="6" t="inlineStr"/>
+      <c r="J742" s="6" t="inlineStr"/>
+      <c r="K742" s="6" t="inlineStr"/>
+      <c r="L742" s="6" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M742" s="6" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N742" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O742" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P742" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q742" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R742" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S742" s="6" t="n"/>
+      <c r="T742" s="6" t="n"/>
+      <c r="U742" s="6" t="n"/>
+      <c r="V742" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W742" s="6" t="inlineStr"/>
+      <c r="X742" s="6" t="n"/>
+      <c r="Y742" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z742" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA742" s="6" t="n"/>
+      <c r="AB742" s="6" t="n"/>
+      <c r="AC742" s="6" t="n"/>
+      <c r="AD742" s="6" t="n"/>
+      <c r="AE742" s="6" t="n"/>
+      <c r="AF742" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="743">
+      <c r="A743" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B743" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C743" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D743" s="4" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E743" s="4" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F743" s="4" t="n"/>
+      <c r="G743" s="4" t="n"/>
+      <c r="H743" s="4" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I743" s="4" t="inlineStr"/>
+      <c r="J743" s="4" t="inlineStr"/>
+      <c r="K743" s="4" t="inlineStr"/>
+      <c r="L743" s="4" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M743" s="4" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N743" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O743" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P743" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q743" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R743" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S743" s="4" t="n"/>
+      <c r="T743" s="4" t="n"/>
+      <c r="U743" s="4" t="n"/>
+      <c r="V743" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W743" s="4" t="inlineStr"/>
+      <c r="X743" s="4" t="n"/>
+      <c r="Y743" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z743" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA743" s="4" t="n"/>
+      <c r="AB743" s="4" t="n"/>
+      <c r="AC743" s="4" t="n"/>
+      <c r="AD743" s="4" t="n"/>
+      <c r="AE743" s="4" t="n"/>
+      <c r="AF743" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="744">
+      <c r="A744" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B744" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C744" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D744" s="6" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E744" s="6" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F744" s="6" t="n"/>
+      <c r="G744" s="6" t="n"/>
+      <c r="H744" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I744" s="6" t="inlineStr"/>
+      <c r="J744" s="6" t="inlineStr"/>
+      <c r="K744" s="6" t="inlineStr"/>
+      <c r="L744" s="6" t="n"/>
+      <c r="M744" s="6" t="n"/>
+      <c r="N744" s="6" t="n"/>
+      <c r="O744" s="6" t="n"/>
+      <c r="P744" s="6" t="n"/>
+      <c r="Q744" s="6" t="n"/>
+      <c r="R744" s="6" t="n"/>
+      <c r="S744" s="6" t="n"/>
+      <c r="T744" s="6" t="n"/>
+      <c r="U744" s="6" t="n"/>
+      <c r="V744" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W744" s="6" t="inlineStr"/>
+      <c r="X744" s="6" t="n"/>
+      <c r="Y744" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z744" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA744" s="6" t="n"/>
+      <c r="AB744" s="6" t="n"/>
+      <c r="AC744" s="6" t="n"/>
+      <c r="AD744" s="6" t="n"/>
+      <c r="AE744" s="6" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF744" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="745">
+      <c r="A745" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B745" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C745" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D745" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E745" s="4" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F745" s="4" t="n"/>
+      <c r="G745" s="4" t="n"/>
+      <c r="H745" s="4" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I745" s="4" t="inlineStr"/>
+      <c r="J745" s="4" t="inlineStr"/>
+      <c r="K745" s="4" t="inlineStr"/>
+      <c r="L745" s="4" t="n"/>
+      <c r="M745" s="4" t="n"/>
+      <c r="N745" s="4" t="n"/>
+      <c r="O745" s="4" t="n"/>
+      <c r="P745" s="4" t="n"/>
+      <c r="Q745" s="4" t="n"/>
+      <c r="R745" s="4" t="n"/>
+      <c r="S745" s="4" t="n"/>
+      <c r="T745" s="4" t="n"/>
+      <c r="U745" s="4" t="n"/>
+      <c r="V745" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W745" s="4" t="inlineStr"/>
+      <c r="X745" s="4" t="n"/>
+      <c r="Y745" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z745" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA745" s="4" t="n"/>
+      <c r="AB745" s="4" t="n"/>
+      <c r="AC745" s="4" t="n"/>
+      <c r="AD745" s="4" t="n"/>
+      <c r="AE745" s="4" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF745" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="746">
+      <c r="A746" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B746" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C746" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D746" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E746" s="6" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F746" s="6" t="n"/>
+      <c r="G746" s="6" t="n"/>
+      <c r="H746" s="6" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I746" s="6" t="inlineStr"/>
+      <c r="J746" s="6" t="inlineStr"/>
+      <c r="K746" s="6" t="inlineStr"/>
+      <c r="L746" s="6" t="n"/>
+      <c r="M746" s="6" t="n"/>
+      <c r="N746" s="6" t="n"/>
+      <c r="O746" s="6" t="n"/>
+      <c r="P746" s="6" t="n"/>
+      <c r="Q746" s="6" t="n"/>
+      <c r="R746" s="6" t="n"/>
+      <c r="S746" s="6" t="n"/>
+      <c r="T746" s="6" t="n"/>
+      <c r="U746" s="6" t="n"/>
+      <c r="V746" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W746" s="6" t="inlineStr"/>
+      <c r="X746" s="6" t="n"/>
+      <c r="Y746" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z746" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA746" s="6" t="n"/>
+      <c r="AB746" s="6" t="n"/>
+      <c r="AC746" s="6" t="n"/>
+      <c r="AD746" s="6" t="n"/>
+      <c r="AE746" s="6" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF746" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="747">
+      <c r="A747" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B747" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C747" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D747" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E747" s="4" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F747" s="4" t="n"/>
+      <c r="G747" s="4" t="n"/>
+      <c r="H747" s="4" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I747" s="4" t="inlineStr"/>
+      <c r="J747" s="4" t="inlineStr"/>
+      <c r="K747" s="4" t="inlineStr"/>
+      <c r="L747" s="4" t="n"/>
+      <c r="M747" s="4" t="n"/>
+      <c r="N747" s="4" t="n"/>
+      <c r="O747" s="4" t="n"/>
+      <c r="P747" s="4" t="n"/>
+      <c r="Q747" s="4" t="n"/>
+      <c r="R747" s="4" t="n"/>
+      <c r="S747" s="4" t="n"/>
+      <c r="T747" s="4" t="n"/>
+      <c r="U747" s="4" t="n"/>
+      <c r="V747" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W747" s="4" t="inlineStr"/>
+      <c r="X747" s="4" t="n"/>
+      <c r="Y747" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z747" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA747" s="4" t="n"/>
+      <c r="AB747" s="4" t="n"/>
+      <c r="AC747" s="4" t="n"/>
+      <c r="AD747" s="4" t="n"/>
+      <c r="AE747" s="4" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF747" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="748">
+      <c r="A748" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B748" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C748" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D748" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E748" s="6" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F748" s="6" t="n"/>
+      <c r="G748" s="6" t="n"/>
+      <c r="H748" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I748" s="6" t="inlineStr"/>
+      <c r="J748" s="6" t="inlineStr"/>
+      <c r="K748" s="6" t="inlineStr"/>
+      <c r="L748" s="6" t="n"/>
+      <c r="M748" s="6" t="n"/>
+      <c r="N748" s="6" t="n"/>
+      <c r="O748" s="6" t="n"/>
+      <c r="P748" s="6" t="n"/>
+      <c r="Q748" s="6" t="n"/>
+      <c r="R748" s="6" t="n"/>
+      <c r="S748" s="6" t="n"/>
+      <c r="T748" s="6" t="n"/>
+      <c r="U748" s="6" t="n"/>
+      <c r="V748" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W748" s="6" t="inlineStr"/>
+      <c r="X748" s="6" t="n"/>
+      <c r="Y748" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z748" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA748" s="6" t="n"/>
+      <c r="AB748" s="6" t="n"/>
+      <c r="AC748" s="6" t="n"/>
+      <c r="AD748" s="6" t="n"/>
+      <c r="AE748" s="6" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF748" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="749">
+      <c r="A749" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B749" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C749" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D749" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E749" s="4" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F749" s="4" t="n"/>
+      <c r="G749" s="4" t="n"/>
+      <c r="H749" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I749" s="4" t="inlineStr"/>
+      <c r="J749" s="4" t="inlineStr"/>
+      <c r="K749" s="4" t="inlineStr"/>
+      <c r="L749" s="4" t="n"/>
+      <c r="M749" s="4" t="n"/>
+      <c r="N749" s="4" t="n"/>
+      <c r="O749" s="4" t="n"/>
+      <c r="P749" s="4" t="n"/>
+      <c r="Q749" s="4" t="n"/>
+      <c r="R749" s="4" t="n"/>
+      <c r="S749" s="4" t="n"/>
+      <c r="T749" s="4" t="n"/>
+      <c r="U749" s="4" t="n"/>
+      <c r="V749" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W749" s="4" t="inlineStr"/>
+      <c r="X749" s="4" t="n"/>
+      <c r="Y749" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z749" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA749" s="4" t="n"/>
+      <c r="AB749" s="4" t="n"/>
+      <c r="AC749" s="4" t="n"/>
+      <c r="AD749" s="4" t="n"/>
+      <c r="AE749" s="4" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF749" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="750">
+      <c r="A750" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B750" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C750" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D750" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E750" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F750" s="6" t="n"/>
+      <c r="G750" s="6" t="n"/>
+      <c r="H750" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I750" s="6" t="inlineStr"/>
+      <c r="J750" s="6" t="inlineStr"/>
+      <c r="K750" s="6" t="inlineStr"/>
+      <c r="L750" s="6" t="n"/>
+      <c r="M750" s="6" t="n"/>
+      <c r="N750" s="6" t="n"/>
+      <c r="O750" s="6" t="n"/>
+      <c r="P750" s="6" t="n"/>
+      <c r="Q750" s="6" t="n"/>
+      <c r="R750" s="6" t="n"/>
+      <c r="S750" s="6" t="n"/>
+      <c r="T750" s="6" t="n"/>
+      <c r="U750" s="6" t="n"/>
+      <c r="V750" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W750" s="6" t="inlineStr"/>
+      <c r="X750" s="6" t="n"/>
+      <c r="Y750" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z750" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA750" s="6" t="n"/>
+      <c r="AB750" s="6" t="n"/>
+      <c r="AC750" s="6" t="n"/>
+      <c r="AD750" s="6" t="n"/>
+      <c r="AE750" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF750" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="751">
+      <c r="A751" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B751" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C751" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D751" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E751" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F751" s="4" t="n"/>
+      <c r="G751" s="4" t="n"/>
+      <c r="H751" s="4" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I751" s="4" t="inlineStr"/>
+      <c r="J751" s="4" t="inlineStr"/>
+      <c r="K751" s="4" t="inlineStr"/>
+      <c r="L751" s="4" t="n"/>
+      <c r="M751" s="4" t="n"/>
+      <c r="N751" s="4" t="n"/>
+      <c r="O751" s="4" t="n"/>
+      <c r="P751" s="4" t="n"/>
+      <c r="Q751" s="4" t="n"/>
+      <c r="R751" s="4" t="n"/>
+      <c r="S751" s="4" t="n"/>
+      <c r="T751" s="4" t="n"/>
+      <c r="U751" s="4" t="n"/>
+      <c r="V751" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W751" s="4" t="inlineStr"/>
+      <c r="X751" s="4" t="n"/>
+      <c r="Y751" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z751" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA751" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB751" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC751" s="4" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD751" s="4" t="n"/>
+      <c r="AE751" s="4" t="n"/>
+      <c r="AF751" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="752">
+      <c r="A752" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B752" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C752" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D752" s="6" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E752" s="6" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F752" s="6" t="n"/>
+      <c r="G752" s="6" t="n"/>
+      <c r="H752" s="6" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I752" s="6" t="inlineStr"/>
+      <c r="J752" s="6" t="inlineStr"/>
+      <c r="K752" s="6" t="inlineStr"/>
+      <c r="L752" s="6" t="n"/>
+      <c r="M752" s="6" t="n"/>
+      <c r="N752" s="6" t="n"/>
+      <c r="O752" s="6" t="n"/>
+      <c r="P752" s="6" t="n"/>
+      <c r="Q752" s="6" t="n"/>
+      <c r="R752" s="6" t="n"/>
+      <c r="S752" s="6" t="n"/>
+      <c r="T752" s="6" t="n"/>
+      <c r="U752" s="6" t="n"/>
+      <c r="V752" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W752" s="6" t="inlineStr"/>
+      <c r="X752" s="6" t="n"/>
+      <c r="Y752" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z752" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA752" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB752" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC752" s="6" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD752" s="6" t="n"/>
+      <c r="AE752" s="6" t="n"/>
+      <c r="AF752" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="753">
+      <c r="A753" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B753" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C753" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D753" s="4" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E753" s="4" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F753" s="4" t="n"/>
+      <c r="G753" s="4" t="n"/>
+      <c r="H753" s="4" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I753" s="4" t="inlineStr"/>
+      <c r="J753" s="4" t="inlineStr"/>
+      <c r="K753" s="4" t="inlineStr"/>
+      <c r="L753" s="4" t="n"/>
+      <c r="M753" s="4" t="n"/>
+      <c r="N753" s="4" t="n"/>
+      <c r="O753" s="4" t="n"/>
+      <c r="P753" s="4" t="n"/>
+      <c r="Q753" s="4" t="n"/>
+      <c r="R753" s="4" t="n"/>
+      <c r="S753" s="4" t="n"/>
+      <c r="T753" s="4" t="n"/>
+      <c r="U753" s="4" t="n"/>
+      <c r="V753" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W753" s="4" t="inlineStr"/>
+      <c r="X753" s="4" t="n"/>
+      <c r="Y753" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z753" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA753" s="4" t="n"/>
+      <c r="AB753" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC753" s="4" t="n"/>
+      <c r="AD753" s="4" t="n"/>
+      <c r="AE753" s="4" t="n"/>
+      <c r="AF753" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="754">
+      <c r="A754" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B754" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C754" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D754" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E754" s="6" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F754" s="6" t="n"/>
+      <c r="G754" s="6" t="n"/>
+      <c r="H754" s="6" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I754" s="6" t="inlineStr"/>
+      <c r="J754" s="6" t="inlineStr"/>
+      <c r="K754" s="6" t="inlineStr"/>
+      <c r="L754" s="6" t="n"/>
+      <c r="M754" s="6" t="n"/>
+      <c r="N754" s="6" t="n"/>
+      <c r="O754" s="6" t="n"/>
+      <c r="P754" s="6" t="n"/>
+      <c r="Q754" s="6" t="n"/>
+      <c r="R754" s="6" t="n"/>
+      <c r="S754" s="6" t="n"/>
+      <c r="T754" s="6" t="n"/>
+      <c r="U754" s="6" t="n"/>
+      <c r="V754" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W754" s="6" t="inlineStr"/>
+      <c r="X754" s="6" t="n"/>
+      <c r="Y754" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z754" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA754" s="6" t="n"/>
+      <c r="AB754" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC754" s="6" t="n"/>
+      <c r="AD754" s="6" t="n"/>
+      <c r="AE754" s="6" t="n"/>
+      <c r="AF754" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-10
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF754"/>
+  <dimension ref="A1:AF789"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -59882,6 +59882,2754 @@
         <v>1</v>
       </c>
     </row>
+    <row r="755">
+      <c r="A755" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B755" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C755" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D755" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E755" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F755" s="4" t="n"/>
+      <c r="G755" s="4" t="n"/>
+      <c r="H755" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I755" s="4" t="inlineStr"/>
+      <c r="J755" s="4" t="inlineStr"/>
+      <c r="K755" s="4" t="inlineStr"/>
+      <c r="L755" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M755" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N755" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O755" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P755" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q755" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R755" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S755" s="4" t="n"/>
+      <c r="T755" s="4" t="n"/>
+      <c r="U755" s="4" t="n"/>
+      <c r="V755" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W755" s="4" t="inlineStr"/>
+      <c r="X755" s="4" t="n"/>
+      <c r="Y755" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z755" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA755" s="4" t="n"/>
+      <c r="AB755" s="4" t="n"/>
+      <c r="AC755" s="4" t="n"/>
+      <c r="AD755" s="4" t="n"/>
+      <c r="AE755" s="4" t="n"/>
+      <c r="AF755" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="756">
+      <c r="A756" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B756" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C756" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D756" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E756" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F756" s="6" t="n"/>
+      <c r="G756" s="6" t="n"/>
+      <c r="H756" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I756" s="6" t="inlineStr"/>
+      <c r="J756" s="6" t="inlineStr"/>
+      <c r="K756" s="6" t="inlineStr"/>
+      <c r="L756" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M756" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N756" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O756" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P756" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q756" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R756" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S756" s="6" t="n"/>
+      <c r="T756" s="6" t="n"/>
+      <c r="U756" s="6" t="n"/>
+      <c r="V756" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W756" s="6" t="inlineStr"/>
+      <c r="X756" s="6" t="n"/>
+      <c r="Y756" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z756" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA756" s="6" t="n"/>
+      <c r="AB756" s="6" t="n"/>
+      <c r="AC756" s="6" t="n"/>
+      <c r="AD756" s="6" t="n"/>
+      <c r="AE756" s="6" t="n"/>
+      <c r="AF756" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="757">
+      <c r="A757" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B757" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C757" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D757" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E757" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F757" s="4" t="n"/>
+      <c r="G757" s="4" t="n"/>
+      <c r="H757" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I757" s="4" t="inlineStr"/>
+      <c r="J757" s="4" t="inlineStr"/>
+      <c r="K757" s="4" t="inlineStr"/>
+      <c r="L757" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M757" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N757" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O757" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P757" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q757" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R757" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S757" s="4" t="n"/>
+      <c r="T757" s="4" t="n"/>
+      <c r="U757" s="4" t="n"/>
+      <c r="V757" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W757" s="4" t="inlineStr"/>
+      <c r="X757" s="4" t="n"/>
+      <c r="Y757" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z757" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA757" s="4" t="n"/>
+      <c r="AB757" s="4" t="n"/>
+      <c r="AC757" s="4" t="n"/>
+      <c r="AD757" s="4" t="n"/>
+      <c r="AE757" s="4" t="n"/>
+      <c r="AF757" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="758">
+      <c r="A758" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B758" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C758" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D758" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E758" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F758" s="6" t="n"/>
+      <c r="G758" s="6" t="n"/>
+      <c r="H758" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I758" s="6" t="inlineStr"/>
+      <c r="J758" s="6" t="inlineStr"/>
+      <c r="K758" s="6" t="inlineStr"/>
+      <c r="L758" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M758" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N758" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O758" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P758" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q758" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R758" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S758" s="6" t="n"/>
+      <c r="T758" s="6" t="n"/>
+      <c r="U758" s="6" t="n"/>
+      <c r="V758" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W758" s="6" t="inlineStr"/>
+      <c r="X758" s="6" t="n"/>
+      <c r="Y758" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z758" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA758" s="6" t="n"/>
+      <c r="AB758" s="6" t="n"/>
+      <c r="AC758" s="6" t="n"/>
+      <c r="AD758" s="6" t="n"/>
+      <c r="AE758" s="6" t="n"/>
+      <c r="AF758" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="759">
+      <c r="A759" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B759" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C759" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D759" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E759" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F759" s="4" t="n"/>
+      <c r="G759" s="4" t="n"/>
+      <c r="H759" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I759" s="4" t="inlineStr"/>
+      <c r="J759" s="4" t="inlineStr"/>
+      <c r="K759" s="4" t="inlineStr"/>
+      <c r="L759" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M759" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N759" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O759" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P759" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q759" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R759" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S759" s="4" t="n"/>
+      <c r="T759" s="4" t="n"/>
+      <c r="U759" s="4" t="n"/>
+      <c r="V759" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W759" s="4" t="inlineStr"/>
+      <c r="X759" s="4" t="n"/>
+      <c r="Y759" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z759" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA759" s="4" t="n"/>
+      <c r="AB759" s="4" t="n"/>
+      <c r="AC759" s="4" t="n"/>
+      <c r="AD759" s="4" t="n"/>
+      <c r="AE759" s="4" t="n"/>
+      <c r="AF759" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="760">
+      <c r="A760" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B760" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C760" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D760" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E760" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F760" s="6" t="n"/>
+      <c r="G760" s="6" t="n"/>
+      <c r="H760" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I760" s="6" t="inlineStr"/>
+      <c r="J760" s="6" t="inlineStr"/>
+      <c r="K760" s="6" t="inlineStr"/>
+      <c r="L760" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M760" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N760" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O760" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P760" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q760" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R760" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S760" s="6" t="n"/>
+      <c r="T760" s="6" t="n"/>
+      <c r="U760" s="6" t="n"/>
+      <c r="V760" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W760" s="6" t="inlineStr"/>
+      <c r="X760" s="6" t="n"/>
+      <c r="Y760" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z760" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA760" s="6" t="n"/>
+      <c r="AB760" s="6" t="n"/>
+      <c r="AC760" s="6" t="n"/>
+      <c r="AD760" s="6" t="n"/>
+      <c r="AE760" s="6" t="n"/>
+      <c r="AF760" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="761">
+      <c r="A761" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B761" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C761" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D761" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E761" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F761" s="4" t="n"/>
+      <c r="G761" s="4" t="n"/>
+      <c r="H761" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I761" s="4" t="inlineStr"/>
+      <c r="J761" s="4" t="inlineStr"/>
+      <c r="K761" s="4" t="inlineStr"/>
+      <c r="L761" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M761" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N761" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O761" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P761" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q761" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R761" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S761" s="4" t="n"/>
+      <c r="T761" s="4" t="n"/>
+      <c r="U761" s="4" t="n"/>
+      <c r="V761" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W761" s="4" t="inlineStr"/>
+      <c r="X761" s="4" t="n"/>
+      <c r="Y761" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z761" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA761" s="4" t="n"/>
+      <c r="AB761" s="4" t="n"/>
+      <c r="AC761" s="4" t="n"/>
+      <c r="AD761" s="4" t="n"/>
+      <c r="AE761" s="4" t="n"/>
+      <c r="AF761" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="762">
+      <c r="A762" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B762" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C762" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D762" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E762" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F762" s="6" t="n"/>
+      <c r="G762" s="6" t="n"/>
+      <c r="H762" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I762" s="6" t="inlineStr"/>
+      <c r="J762" s="6" t="inlineStr"/>
+      <c r="K762" s="6" t="inlineStr"/>
+      <c r="L762" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M762" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N762" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O762" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P762" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q762" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R762" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S762" s="6" t="n"/>
+      <c r="T762" s="6" t="n"/>
+      <c r="U762" s="6" t="n"/>
+      <c r="V762" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W762" s="6" t="inlineStr"/>
+      <c r="X762" s="6" t="n"/>
+      <c r="Y762" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z762" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA762" s="6" t="n"/>
+      <c r="AB762" s="6" t="n"/>
+      <c r="AC762" s="6" t="n"/>
+      <c r="AD762" s="6" t="n"/>
+      <c r="AE762" s="6" t="n"/>
+      <c r="AF762" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="763">
+      <c r="A763" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B763" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C763" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D763" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E763" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F763" s="4" t="n"/>
+      <c r="G763" s="4" t="n"/>
+      <c r="H763" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I763" s="4" t="inlineStr"/>
+      <c r="J763" s="4" t="inlineStr"/>
+      <c r="K763" s="4" t="inlineStr"/>
+      <c r="L763" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M763" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N763" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O763" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P763" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q763" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R763" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S763" s="4" t="n"/>
+      <c r="T763" s="4" t="n"/>
+      <c r="U763" s="4" t="n"/>
+      <c r="V763" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W763" s="4" t="inlineStr"/>
+      <c r="X763" s="4" t="n"/>
+      <c r="Y763" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z763" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA763" s="4" t="n"/>
+      <c r="AB763" s="4" t="n"/>
+      <c r="AC763" s="4" t="n"/>
+      <c r="AD763" s="4" t="n"/>
+      <c r="AE763" s="4" t="n"/>
+      <c r="AF763" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="764">
+      <c r="A764" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B764" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C764" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D764" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E764" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F764" s="6" t="n"/>
+      <c r="G764" s="6" t="n"/>
+      <c r="H764" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I764" s="6" t="inlineStr"/>
+      <c r="J764" s="6" t="inlineStr"/>
+      <c r="K764" s="6" t="inlineStr"/>
+      <c r="L764" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M764" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N764" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O764" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P764" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q764" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R764" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S764" s="6" t="n"/>
+      <c r="T764" s="6" t="n"/>
+      <c r="U764" s="6" t="n"/>
+      <c r="V764" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W764" s="6" t="inlineStr"/>
+      <c r="X764" s="6" t="n"/>
+      <c r="Y764" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z764" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA764" s="6" t="n"/>
+      <c r="AB764" s="6" t="n"/>
+      <c r="AC764" s="6" t="n"/>
+      <c r="AD764" s="6" t="n"/>
+      <c r="AE764" s="6" t="n"/>
+      <c r="AF764" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="765">
+      <c r="A765" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B765" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C765" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D765" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E765" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F765" s="4" t="n"/>
+      <c r="G765" s="4" t="n"/>
+      <c r="H765" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I765" s="4" t="inlineStr"/>
+      <c r="J765" s="4" t="inlineStr"/>
+      <c r="K765" s="4" t="inlineStr"/>
+      <c r="L765" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M765" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N765" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O765" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P765" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q765" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R765" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S765" s="4" t="n"/>
+      <c r="T765" s="4" t="n"/>
+      <c r="U765" s="4" t="n"/>
+      <c r="V765" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W765" s="4" t="inlineStr"/>
+      <c r="X765" s="4" t="n"/>
+      <c r="Y765" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z765" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA765" s="4" t="n"/>
+      <c r="AB765" s="4" t="n"/>
+      <c r="AC765" s="4" t="n"/>
+      <c r="AD765" s="4" t="n"/>
+      <c r="AE765" s="4" t="n"/>
+      <c r="AF765" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="766">
+      <c r="A766" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B766" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C766" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D766" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E766" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F766" s="6" t="n"/>
+      <c r="G766" s="6" t="n"/>
+      <c r="H766" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I766" s="6" t="inlineStr"/>
+      <c r="J766" s="6" t="inlineStr"/>
+      <c r="K766" s="6" t="inlineStr"/>
+      <c r="L766" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M766" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N766" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O766" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P766" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q766" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R766" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S766" s="6" t="n"/>
+      <c r="T766" s="6" t="n"/>
+      <c r="U766" s="6" t="n"/>
+      <c r="V766" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W766" s="6" t="inlineStr"/>
+      <c r="X766" s="6" t="n"/>
+      <c r="Y766" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z766" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA766" s="6" t="n"/>
+      <c r="AB766" s="6" t="n"/>
+      <c r="AC766" s="6" t="n"/>
+      <c r="AD766" s="6" t="n"/>
+      <c r="AE766" s="6" t="n"/>
+      <c r="AF766" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="767">
+      <c r="A767" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B767" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C767" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D767" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E767" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F767" s="4" t="n"/>
+      <c r="G767" s="4" t="n"/>
+      <c r="H767" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I767" s="4" t="inlineStr"/>
+      <c r="J767" s="4" t="inlineStr"/>
+      <c r="K767" s="4" t="inlineStr"/>
+      <c r="L767" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M767" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N767" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O767" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P767" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q767" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R767" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S767" s="4" t="n"/>
+      <c r="T767" s="4" t="n"/>
+      <c r="U767" s="4" t="n"/>
+      <c r="V767" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W767" s="4" t="inlineStr"/>
+      <c r="X767" s="4" t="n"/>
+      <c r="Y767" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z767" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA767" s="4" t="n"/>
+      <c r="AB767" s="4" t="n"/>
+      <c r="AC767" s="4" t="n"/>
+      <c r="AD767" s="4" t="n"/>
+      <c r="AE767" s="4" t="n"/>
+      <c r="AF767" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="768">
+      <c r="A768" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B768" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C768" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D768" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E768" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F768" s="6" t="n"/>
+      <c r="G768" s="6" t="n"/>
+      <c r="H768" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I768" s="6" t="inlineStr"/>
+      <c r="J768" s="6" t="inlineStr"/>
+      <c r="K768" s="6" t="inlineStr"/>
+      <c r="L768" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M768" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N768" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O768" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P768" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q768" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R768" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S768" s="6" t="n"/>
+      <c r="T768" s="6" t="n"/>
+      <c r="U768" s="6" t="n"/>
+      <c r="V768" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W768" s="6" t="inlineStr"/>
+      <c r="X768" s="6" t="n"/>
+      <c r="Y768" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z768" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA768" s="6" t="n"/>
+      <c r="AB768" s="6" t="n"/>
+      <c r="AC768" s="6" t="n"/>
+      <c r="AD768" s="6" t="n"/>
+      <c r="AE768" s="6" t="n"/>
+      <c r="AF768" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="769">
+      <c r="A769" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B769" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C769" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D769" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E769" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F769" s="4" t="n"/>
+      <c r="G769" s="4" t="n"/>
+      <c r="H769" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I769" s="4" t="inlineStr"/>
+      <c r="J769" s="4" t="inlineStr"/>
+      <c r="K769" s="4" t="inlineStr"/>
+      <c r="L769" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M769" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N769" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O769" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P769" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q769" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R769" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S769" s="4" t="n"/>
+      <c r="T769" s="4" t="n"/>
+      <c r="U769" s="4" t="n"/>
+      <c r="V769" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W769" s="4" t="inlineStr"/>
+      <c r="X769" s="4" t="n"/>
+      <c r="Y769" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z769" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA769" s="4" t="n"/>
+      <c r="AB769" s="4" t="n"/>
+      <c r="AC769" s="4" t="n"/>
+      <c r="AD769" s="4" t="n"/>
+      <c r="AE769" s="4" t="n"/>
+      <c r="AF769" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="770">
+      <c r="A770" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B770" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C770" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D770" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E770" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F770" s="6" t="n"/>
+      <c r="G770" s="6" t="n"/>
+      <c r="H770" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I770" s="6" t="inlineStr"/>
+      <c r="J770" s="6" t="inlineStr"/>
+      <c r="K770" s="6" t="inlineStr"/>
+      <c r="L770" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M770" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N770" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O770" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P770" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q770" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R770" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S770" s="6" t="n"/>
+      <c r="T770" s="6" t="n"/>
+      <c r="U770" s="6" t="n"/>
+      <c r="V770" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W770" s="6" t="inlineStr"/>
+      <c r="X770" s="6" t="n"/>
+      <c r="Y770" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z770" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA770" s="6" t="n"/>
+      <c r="AB770" s="6" t="n"/>
+      <c r="AC770" s="6" t="n"/>
+      <c r="AD770" s="6" t="n"/>
+      <c r="AE770" s="6" t="n"/>
+      <c r="AF770" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="771">
+      <c r="A771" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B771" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C771" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D771" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E771" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F771" s="4" t="n"/>
+      <c r="G771" s="4" t="n"/>
+      <c r="H771" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I771" s="4" t="inlineStr"/>
+      <c r="J771" s="4" t="inlineStr"/>
+      <c r="K771" s="4" t="inlineStr"/>
+      <c r="L771" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M771" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N771" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O771" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P771" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q771" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R771" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S771" s="4" t="n"/>
+      <c r="T771" s="4" t="n"/>
+      <c r="U771" s="4" t="n"/>
+      <c r="V771" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W771" s="4" t="inlineStr"/>
+      <c r="X771" s="4" t="n"/>
+      <c r="Y771" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z771" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA771" s="4" t="n"/>
+      <c r="AB771" s="4" t="n"/>
+      <c r="AC771" s="4" t="n"/>
+      <c r="AD771" s="4" t="n"/>
+      <c r="AE771" s="4" t="n"/>
+      <c r="AF771" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="772">
+      <c r="A772" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B772" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C772" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D772" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E772" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F772" s="6" t="n"/>
+      <c r="G772" s="6" t="n"/>
+      <c r="H772" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I772" s="6" t="inlineStr"/>
+      <c r="J772" s="6" t="inlineStr"/>
+      <c r="K772" s="6" t="inlineStr"/>
+      <c r="L772" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M772" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N772" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O772" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P772" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q772" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R772" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S772" s="6" t="n"/>
+      <c r="T772" s="6" t="n"/>
+      <c r="U772" s="6" t="n"/>
+      <c r="V772" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W772" s="6" t="inlineStr"/>
+      <c r="X772" s="6" t="n"/>
+      <c r="Y772" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z772" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA772" s="6" t="n"/>
+      <c r="AB772" s="6" t="n"/>
+      <c r="AC772" s="6" t="n"/>
+      <c r="AD772" s="6" t="n"/>
+      <c r="AE772" s="6" t="n"/>
+      <c r="AF772" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="773">
+      <c r="A773" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B773" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C773" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D773" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E773" s="4" t="n">
+        <v>54.99</v>
+      </c>
+      <c r="F773" s="4" t="n"/>
+      <c r="G773" s="4" t="n"/>
+      <c r="H773" s="4" t="n">
+        <v>62.85</v>
+      </c>
+      <c r="I773" s="4" t="inlineStr"/>
+      <c r="J773" s="4" t="inlineStr"/>
+      <c r="K773" s="4" t="inlineStr"/>
+      <c r="L773" s="4" t="n">
+        <v>79.56</v>
+      </c>
+      <c r="M773" s="4" t="n">
+        <v>2.387</v>
+      </c>
+      <c r="N773" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O773" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P773" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q773" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R773" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S773" s="4" t="n"/>
+      <c r="T773" s="4" t="n"/>
+      <c r="U773" s="4" t="n"/>
+      <c r="V773" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W773" s="4" t="inlineStr"/>
+      <c r="X773" s="4" t="n"/>
+      <c r="Y773" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z773" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA773" s="4" t="n"/>
+      <c r="AB773" s="4" t="n"/>
+      <c r="AC773" s="4" t="n"/>
+      <c r="AD773" s="4" t="n"/>
+      <c r="AE773" s="4" t="n"/>
+      <c r="AF773" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="774">
+      <c r="A774" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B774" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C774" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D774" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E774" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F774" s="6" t="n"/>
+      <c r="G774" s="6" t="n"/>
+      <c r="H774" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I774" s="6" t="inlineStr"/>
+      <c r="J774" s="6" t="inlineStr"/>
+      <c r="K774" s="6" t="inlineStr"/>
+      <c r="L774" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M774" s="6" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N774" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O774" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P774" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q774" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R774" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S774" s="6" t="n"/>
+      <c r="T774" s="6" t="n"/>
+      <c r="U774" s="6" t="n"/>
+      <c r="V774" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W774" s="6" t="inlineStr"/>
+      <c r="X774" s="6" t="n"/>
+      <c r="Y774" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z774" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA774" s="6" t="n"/>
+      <c r="AB774" s="6" t="n"/>
+      <c r="AC774" s="6" t="n"/>
+      <c r="AD774" s="6" t="n"/>
+      <c r="AE774" s="6" t="n"/>
+      <c r="AF774" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="775">
+      <c r="A775" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B775" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C775" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D775" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E775" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F775" s="4" t="n"/>
+      <c r="G775" s="4" t="n"/>
+      <c r="H775" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I775" s="4" t="inlineStr"/>
+      <c r="J775" s="4" t="inlineStr"/>
+      <c r="K775" s="4" t="inlineStr"/>
+      <c r="L775" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M775" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N775" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O775" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P775" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q775" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R775" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S775" s="4" t="n"/>
+      <c r="T775" s="4" t="n"/>
+      <c r="U775" s="4" t="n"/>
+      <c r="V775" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W775" s="4" t="inlineStr"/>
+      <c r="X775" s="4" t="n"/>
+      <c r="Y775" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z775" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA775" s="4" t="n"/>
+      <c r="AB775" s="4" t="n"/>
+      <c r="AC775" s="4" t="n"/>
+      <c r="AD775" s="4" t="n"/>
+      <c r="AE775" s="4" t="n"/>
+      <c r="AF775" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="776">
+      <c r="A776" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B776" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C776" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D776" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E776" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F776" s="6" t="n"/>
+      <c r="G776" s="6" t="n"/>
+      <c r="H776" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I776" s="6" t="inlineStr"/>
+      <c r="J776" s="6" t="inlineStr"/>
+      <c r="K776" s="6" t="inlineStr"/>
+      <c r="L776" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M776" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N776" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O776" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P776" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q776" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R776" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S776" s="6" t="n"/>
+      <c r="T776" s="6" t="n"/>
+      <c r="U776" s="6" t="n"/>
+      <c r="V776" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W776" s="6" t="inlineStr"/>
+      <c r="X776" s="6" t="n"/>
+      <c r="Y776" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z776" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA776" s="6" t="n"/>
+      <c r="AB776" s="6" t="n"/>
+      <c r="AC776" s="6" t="n"/>
+      <c r="AD776" s="6" t="n"/>
+      <c r="AE776" s="6" t="n"/>
+      <c r="AF776" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="777">
+      <c r="A777" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B777" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C777" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D777" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E777" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F777" s="4" t="n"/>
+      <c r="G777" s="4" t="n"/>
+      <c r="H777" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I777" s="4" t="inlineStr"/>
+      <c r="J777" s="4" t="inlineStr"/>
+      <c r="K777" s="4" t="inlineStr"/>
+      <c r="L777" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M777" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N777" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O777" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P777" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q777" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R777" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S777" s="4" t="n"/>
+      <c r="T777" s="4" t="n"/>
+      <c r="U777" s="4" t="n"/>
+      <c r="V777" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W777" s="4" t="inlineStr"/>
+      <c r="X777" s="4" t="n"/>
+      <c r="Y777" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z777" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA777" s="4" t="n"/>
+      <c r="AB777" s="4" t="n"/>
+      <c r="AC777" s="4" t="n"/>
+      <c r="AD777" s="4" t="n"/>
+      <c r="AE777" s="4" t="n"/>
+      <c r="AF777" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="778">
+      <c r="A778" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B778" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C778" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D778" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E778" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F778" s="6" t="n"/>
+      <c r="G778" s="6" t="n"/>
+      <c r="H778" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I778" s="6" t="inlineStr"/>
+      <c r="J778" s="6" t="inlineStr"/>
+      <c r="K778" s="6" t="inlineStr"/>
+      <c r="L778" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M778" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N778" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O778" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P778" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q778" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R778" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S778" s="6" t="n"/>
+      <c r="T778" s="6" t="n"/>
+      <c r="U778" s="6" t="n"/>
+      <c r="V778" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W778" s="6" t="inlineStr"/>
+      <c r="X778" s="6" t="n"/>
+      <c r="Y778" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z778" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA778" s="6" t="n"/>
+      <c r="AB778" s="6" t="n"/>
+      <c r="AC778" s="6" t="n"/>
+      <c r="AD778" s="6" t="n"/>
+      <c r="AE778" s="6" t="n"/>
+      <c r="AF778" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="779">
+      <c r="A779" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B779" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C779" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D779" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E779" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F779" s="4" t="n"/>
+      <c r="G779" s="4" t="n"/>
+      <c r="H779" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I779" s="4" t="inlineStr"/>
+      <c r="J779" s="4" t="inlineStr"/>
+      <c r="K779" s="4" t="inlineStr"/>
+      <c r="L779" s="4" t="n"/>
+      <c r="M779" s="4" t="n"/>
+      <c r="N779" s="4" t="n"/>
+      <c r="O779" s="4" t="n"/>
+      <c r="P779" s="4" t="n"/>
+      <c r="Q779" s="4" t="n"/>
+      <c r="R779" s="4" t="n"/>
+      <c r="S779" s="4" t="n"/>
+      <c r="T779" s="4" t="n"/>
+      <c r="U779" s="4" t="n"/>
+      <c r="V779" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W779" s="4" t="inlineStr"/>
+      <c r="X779" s="4" t="n"/>
+      <c r="Y779" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z779" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA779" s="4" t="n"/>
+      <c r="AB779" s="4" t="n"/>
+      <c r="AC779" s="4" t="n"/>
+      <c r="AD779" s="4" t="n"/>
+      <c r="AE779" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF779" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="780">
+      <c r="A780" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B780" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C780" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D780" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E780" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F780" s="6" t="n"/>
+      <c r="G780" s="6" t="n"/>
+      <c r="H780" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I780" s="6" t="inlineStr"/>
+      <c r="J780" s="6" t="inlineStr"/>
+      <c r="K780" s="6" t="inlineStr"/>
+      <c r="L780" s="6" t="n"/>
+      <c r="M780" s="6" t="n"/>
+      <c r="N780" s="6" t="n"/>
+      <c r="O780" s="6" t="n"/>
+      <c r="P780" s="6" t="n"/>
+      <c r="Q780" s="6" t="n"/>
+      <c r="R780" s="6" t="n"/>
+      <c r="S780" s="6" t="n"/>
+      <c r="T780" s="6" t="n"/>
+      <c r="U780" s="6" t="n"/>
+      <c r="V780" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W780" s="6" t="inlineStr"/>
+      <c r="X780" s="6" t="n"/>
+      <c r="Y780" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z780" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA780" s="6" t="n"/>
+      <c r="AB780" s="6" t="n"/>
+      <c r="AC780" s="6" t="n"/>
+      <c r="AD780" s="6" t="n"/>
+      <c r="AE780" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF780" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="781">
+      <c r="A781" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B781" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C781" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D781" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E781" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F781" s="4" t="n"/>
+      <c r="G781" s="4" t="n"/>
+      <c r="H781" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I781" s="4" t="inlineStr"/>
+      <c r="J781" s="4" t="inlineStr"/>
+      <c r="K781" s="4" t="inlineStr"/>
+      <c r="L781" s="4" t="n"/>
+      <c r="M781" s="4" t="n"/>
+      <c r="N781" s="4" t="n"/>
+      <c r="O781" s="4" t="n"/>
+      <c r="P781" s="4" t="n"/>
+      <c r="Q781" s="4" t="n"/>
+      <c r="R781" s="4" t="n"/>
+      <c r="S781" s="4" t="n"/>
+      <c r="T781" s="4" t="n"/>
+      <c r="U781" s="4" t="n"/>
+      <c r="V781" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W781" s="4" t="inlineStr"/>
+      <c r="X781" s="4" t="n"/>
+      <c r="Y781" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z781" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA781" s="4" t="n"/>
+      <c r="AB781" s="4" t="n"/>
+      <c r="AC781" s="4" t="n"/>
+      <c r="AD781" s="4" t="n"/>
+      <c r="AE781" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF781" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="782">
+      <c r="A782" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B782" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C782" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D782" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E782" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F782" s="6" t="n"/>
+      <c r="G782" s="6" t="n"/>
+      <c r="H782" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I782" s="6" t="inlineStr"/>
+      <c r="J782" s="6" t="inlineStr"/>
+      <c r="K782" s="6" t="inlineStr"/>
+      <c r="L782" s="6" t="n"/>
+      <c r="M782" s="6" t="n"/>
+      <c r="N782" s="6" t="n"/>
+      <c r="O782" s="6" t="n"/>
+      <c r="P782" s="6" t="n"/>
+      <c r="Q782" s="6" t="n"/>
+      <c r="R782" s="6" t="n"/>
+      <c r="S782" s="6" t="n"/>
+      <c r="T782" s="6" t="n"/>
+      <c r="U782" s="6" t="n"/>
+      <c r="V782" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W782" s="6" t="inlineStr"/>
+      <c r="X782" s="6" t="n"/>
+      <c r="Y782" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z782" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA782" s="6" t="n"/>
+      <c r="AB782" s="6" t="n"/>
+      <c r="AC782" s="6" t="n"/>
+      <c r="AD782" s="6" t="n"/>
+      <c r="AE782" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF782" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="783">
+      <c r="A783" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B783" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C783" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D783" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E783" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F783" s="4" t="n"/>
+      <c r="G783" s="4" t="n"/>
+      <c r="H783" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I783" s="4" t="inlineStr"/>
+      <c r="J783" s="4" t="inlineStr"/>
+      <c r="K783" s="4" t="inlineStr"/>
+      <c r="L783" s="4" t="n"/>
+      <c r="M783" s="4" t="n"/>
+      <c r="N783" s="4" t="n"/>
+      <c r="O783" s="4" t="n"/>
+      <c r="P783" s="4" t="n"/>
+      <c r="Q783" s="4" t="n"/>
+      <c r="R783" s="4" t="n"/>
+      <c r="S783" s="4" t="n"/>
+      <c r="T783" s="4" t="n"/>
+      <c r="U783" s="4" t="n"/>
+      <c r="V783" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W783" s="4" t="inlineStr"/>
+      <c r="X783" s="4" t="n"/>
+      <c r="Y783" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z783" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA783" s="4" t="n"/>
+      <c r="AB783" s="4" t="n"/>
+      <c r="AC783" s="4" t="n"/>
+      <c r="AD783" s="4" t="n"/>
+      <c r="AE783" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF783" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="784">
+      <c r="A784" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B784" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C784" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D784" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E784" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F784" s="6" t="n"/>
+      <c r="G784" s="6" t="n"/>
+      <c r="H784" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I784" s="6" t="inlineStr"/>
+      <c r="J784" s="6" t="inlineStr"/>
+      <c r="K784" s="6" t="inlineStr"/>
+      <c r="L784" s="6" t="n"/>
+      <c r="M784" s="6" t="n"/>
+      <c r="N784" s="6" t="n"/>
+      <c r="O784" s="6" t="n"/>
+      <c r="P784" s="6" t="n"/>
+      <c r="Q784" s="6" t="n"/>
+      <c r="R784" s="6" t="n"/>
+      <c r="S784" s="6" t="n"/>
+      <c r="T784" s="6" t="n"/>
+      <c r="U784" s="6" t="n"/>
+      <c r="V784" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W784" s="6" t="inlineStr"/>
+      <c r="X784" s="6" t="n"/>
+      <c r="Y784" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z784" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA784" s="6" t="n"/>
+      <c r="AB784" s="6" t="n"/>
+      <c r="AC784" s="6" t="n"/>
+      <c r="AD784" s="6" t="n"/>
+      <c r="AE784" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF784" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="785">
+      <c r="A785" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B785" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C785" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D785" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E785" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F785" s="4" t="n"/>
+      <c r="G785" s="4" t="n"/>
+      <c r="H785" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I785" s="4" t="inlineStr"/>
+      <c r="J785" s="4" t="inlineStr"/>
+      <c r="K785" s="4" t="inlineStr"/>
+      <c r="L785" s="4" t="n"/>
+      <c r="M785" s="4" t="n"/>
+      <c r="N785" s="4" t="n"/>
+      <c r="O785" s="4" t="n"/>
+      <c r="P785" s="4" t="n"/>
+      <c r="Q785" s="4" t="n"/>
+      <c r="R785" s="4" t="n"/>
+      <c r="S785" s="4" t="n"/>
+      <c r="T785" s="4" t="n"/>
+      <c r="U785" s="4" t="n"/>
+      <c r="V785" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W785" s="4" t="inlineStr"/>
+      <c r="X785" s="4" t="n"/>
+      <c r="Y785" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z785" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA785" s="4" t="n"/>
+      <c r="AB785" s="4" t="n"/>
+      <c r="AC785" s="4" t="n"/>
+      <c r="AD785" s="4" t="n"/>
+      <c r="AE785" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF785" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="786">
+      <c r="A786" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B786" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C786" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D786" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E786" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F786" s="6" t="n"/>
+      <c r="G786" s="6" t="n"/>
+      <c r="H786" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I786" s="6" t="inlineStr"/>
+      <c r="J786" s="6" t="inlineStr"/>
+      <c r="K786" s="6" t="inlineStr"/>
+      <c r="L786" s="6" t="n"/>
+      <c r="M786" s="6" t="n"/>
+      <c r="N786" s="6" t="n"/>
+      <c r="O786" s="6" t="n"/>
+      <c r="P786" s="6" t="n"/>
+      <c r="Q786" s="6" t="n"/>
+      <c r="R786" s="6" t="n"/>
+      <c r="S786" s="6" t="n"/>
+      <c r="T786" s="6" t="n"/>
+      <c r="U786" s="6" t="n"/>
+      <c r="V786" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W786" s="6" t="inlineStr"/>
+      <c r="X786" s="6" t="n"/>
+      <c r="Y786" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z786" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA786" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB786" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC786" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD786" s="6" t="n"/>
+      <c r="AE786" s="6" t="n"/>
+      <c r="AF786" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="787">
+      <c r="A787" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B787" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C787" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D787" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E787" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F787" s="4" t="n"/>
+      <c r="G787" s="4" t="n"/>
+      <c r="H787" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I787" s="4" t="inlineStr"/>
+      <c r="J787" s="4" t="inlineStr"/>
+      <c r="K787" s="4" t="inlineStr"/>
+      <c r="L787" s="4" t="n"/>
+      <c r="M787" s="4" t="n"/>
+      <c r="N787" s="4" t="n"/>
+      <c r="O787" s="4" t="n"/>
+      <c r="P787" s="4" t="n"/>
+      <c r="Q787" s="4" t="n"/>
+      <c r="R787" s="4" t="n"/>
+      <c r="S787" s="4" t="n"/>
+      <c r="T787" s="4" t="n"/>
+      <c r="U787" s="4" t="n"/>
+      <c r="V787" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W787" s="4" t="inlineStr"/>
+      <c r="X787" s="4" t="n"/>
+      <c r="Y787" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z787" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA787" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB787" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC787" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD787" s="4" t="n"/>
+      <c r="AE787" s="4" t="n"/>
+      <c r="AF787" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="788">
+      <c r="A788" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B788" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C788" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D788" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E788" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F788" s="6" t="n"/>
+      <c r="G788" s="6" t="n"/>
+      <c r="H788" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I788" s="6" t="inlineStr"/>
+      <c r="J788" s="6" t="inlineStr"/>
+      <c r="K788" s="6" t="inlineStr"/>
+      <c r="L788" s="6" t="n"/>
+      <c r="M788" s="6" t="n"/>
+      <c r="N788" s="6" t="n"/>
+      <c r="O788" s="6" t="n"/>
+      <c r="P788" s="6" t="n"/>
+      <c r="Q788" s="6" t="n"/>
+      <c r="R788" s="6" t="n"/>
+      <c r="S788" s="6" t="n"/>
+      <c r="T788" s="6" t="n"/>
+      <c r="U788" s="6" t="n"/>
+      <c r="V788" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W788" s="6" t="inlineStr"/>
+      <c r="X788" s="6" t="n"/>
+      <c r="Y788" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z788" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA788" s="6" t="n"/>
+      <c r="AB788" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC788" s="6" t="n"/>
+      <c r="AD788" s="6" t="n"/>
+      <c r="AE788" s="6" t="n"/>
+      <c r="AF788" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="789">
+      <c r="A789" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-10</t>
+        </is>
+      </c>
+      <c r="B789" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C789" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D789" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E789" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F789" s="4" t="n"/>
+      <c r="G789" s="4" t="n"/>
+      <c r="H789" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I789" s="4" t="inlineStr"/>
+      <c r="J789" s="4" t="inlineStr"/>
+      <c r="K789" s="4" t="inlineStr"/>
+      <c r="L789" s="4" t="n"/>
+      <c r="M789" s="4" t="n"/>
+      <c r="N789" s="4" t="n"/>
+      <c r="O789" s="4" t="n"/>
+      <c r="P789" s="4" t="n"/>
+      <c r="Q789" s="4" t="n"/>
+      <c r="R789" s="4" t="n"/>
+      <c r="S789" s="4" t="n"/>
+      <c r="T789" s="4" t="n"/>
+      <c r="U789" s="4" t="n"/>
+      <c r="V789" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W789" s="4" t="inlineStr"/>
+      <c r="X789" s="4" t="n"/>
+      <c r="Y789" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z789" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA789" s="4" t="n"/>
+      <c r="AB789" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC789" s="4" t="n"/>
+      <c r="AD789" s="4" t="n"/>
+      <c r="AE789" s="4" t="n"/>
+      <c r="AF789" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-11
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF789"/>
+  <dimension ref="A1:AF824"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -62630,6 +62630,2754 @@
         <v>1</v>
       </c>
     </row>
+    <row r="790">
+      <c r="A790" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B790" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C790" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D790" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E790" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F790" s="4" t="n"/>
+      <c r="G790" s="4" t="n"/>
+      <c r="H790" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I790" s="4" t="inlineStr"/>
+      <c r="J790" s="4" t="inlineStr"/>
+      <c r="K790" s="4" t="inlineStr"/>
+      <c r="L790" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M790" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N790" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O790" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P790" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q790" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R790" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S790" s="4" t="n"/>
+      <c r="T790" s="4" t="n"/>
+      <c r="U790" s="4" t="n"/>
+      <c r="V790" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W790" s="4" t="inlineStr"/>
+      <c r="X790" s="4" t="n"/>
+      <c r="Y790" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z790" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA790" s="4" t="n"/>
+      <c r="AB790" s="4" t="n"/>
+      <c r="AC790" s="4" t="n"/>
+      <c r="AD790" s="4" t="n"/>
+      <c r="AE790" s="4" t="n"/>
+      <c r="AF790" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="791">
+      <c r="A791" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B791" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C791" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D791" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E791" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F791" s="6" t="n"/>
+      <c r="G791" s="6" t="n"/>
+      <c r="H791" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I791" s="6" t="inlineStr"/>
+      <c r="J791" s="6" t="inlineStr"/>
+      <c r="K791" s="6" t="inlineStr"/>
+      <c r="L791" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M791" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N791" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O791" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P791" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q791" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R791" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S791" s="6" t="n"/>
+      <c r="T791" s="6" t="n"/>
+      <c r="U791" s="6" t="n"/>
+      <c r="V791" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W791" s="6" t="inlineStr"/>
+      <c r="X791" s="6" t="n"/>
+      <c r="Y791" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z791" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA791" s="6" t="n"/>
+      <c r="AB791" s="6" t="n"/>
+      <c r="AC791" s="6" t="n"/>
+      <c r="AD791" s="6" t="n"/>
+      <c r="AE791" s="6" t="n"/>
+      <c r="AF791" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="792">
+      <c r="A792" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B792" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C792" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D792" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E792" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F792" s="4" t="n"/>
+      <c r="G792" s="4" t="n"/>
+      <c r="H792" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I792" s="4" t="inlineStr"/>
+      <c r="J792" s="4" t="inlineStr"/>
+      <c r="K792" s="4" t="inlineStr"/>
+      <c r="L792" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M792" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N792" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O792" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P792" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q792" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R792" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S792" s="4" t="n"/>
+      <c r="T792" s="4" t="n"/>
+      <c r="U792" s="4" t="n"/>
+      <c r="V792" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W792" s="4" t="inlineStr"/>
+      <c r="X792" s="4" t="n"/>
+      <c r="Y792" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z792" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA792" s="4" t="n"/>
+      <c r="AB792" s="4" t="n"/>
+      <c r="AC792" s="4" t="n"/>
+      <c r="AD792" s="4" t="n"/>
+      <c r="AE792" s="4" t="n"/>
+      <c r="AF792" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="793">
+      <c r="A793" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B793" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C793" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D793" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E793" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F793" s="6" t="n"/>
+      <c r="G793" s="6" t="n"/>
+      <c r="H793" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I793" s="6" t="inlineStr"/>
+      <c r="J793" s="6" t="inlineStr"/>
+      <c r="K793" s="6" t="inlineStr"/>
+      <c r="L793" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M793" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N793" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O793" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P793" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q793" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R793" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S793" s="6" t="n"/>
+      <c r="T793" s="6" t="n"/>
+      <c r="U793" s="6" t="n"/>
+      <c r="V793" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W793" s="6" t="inlineStr"/>
+      <c r="X793" s="6" t="n"/>
+      <c r="Y793" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z793" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA793" s="6" t="n"/>
+      <c r="AB793" s="6" t="n"/>
+      <c r="AC793" s="6" t="n"/>
+      <c r="AD793" s="6" t="n"/>
+      <c r="AE793" s="6" t="n"/>
+      <c r="AF793" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="794">
+      <c r="A794" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B794" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C794" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D794" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E794" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F794" s="4" t="n"/>
+      <c r="G794" s="4" t="n"/>
+      <c r="H794" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I794" s="4" t="inlineStr"/>
+      <c r="J794" s="4" t="inlineStr"/>
+      <c r="K794" s="4" t="inlineStr"/>
+      <c r="L794" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M794" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N794" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O794" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P794" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q794" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R794" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S794" s="4" t="n"/>
+      <c r="T794" s="4" t="n"/>
+      <c r="U794" s="4" t="n"/>
+      <c r="V794" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W794" s="4" t="inlineStr"/>
+      <c r="X794" s="4" t="n"/>
+      <c r="Y794" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z794" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA794" s="4" t="n"/>
+      <c r="AB794" s="4" t="n"/>
+      <c r="AC794" s="4" t="n"/>
+      <c r="AD794" s="4" t="n"/>
+      <c r="AE794" s="4" t="n"/>
+      <c r="AF794" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="795">
+      <c r="A795" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B795" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C795" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D795" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E795" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F795" s="6" t="n"/>
+      <c r="G795" s="6" t="n"/>
+      <c r="H795" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I795" s="6" t="inlineStr"/>
+      <c r="J795" s="6" t="inlineStr"/>
+      <c r="K795" s="6" t="inlineStr"/>
+      <c r="L795" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M795" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N795" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O795" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P795" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q795" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R795" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S795" s="6" t="n"/>
+      <c r="T795" s="6" t="n"/>
+      <c r="U795" s="6" t="n"/>
+      <c r="V795" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W795" s="6" t="inlineStr"/>
+      <c r="X795" s="6" t="n"/>
+      <c r="Y795" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z795" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA795" s="6" t="n"/>
+      <c r="AB795" s="6" t="n"/>
+      <c r="AC795" s="6" t="n"/>
+      <c r="AD795" s="6" t="n"/>
+      <c r="AE795" s="6" t="n"/>
+      <c r="AF795" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="796">
+      <c r="A796" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B796" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C796" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D796" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E796" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F796" s="4" t="n"/>
+      <c r="G796" s="4" t="n"/>
+      <c r="H796" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I796" s="4" t="inlineStr"/>
+      <c r="J796" s="4" t="inlineStr"/>
+      <c r="K796" s="4" t="inlineStr"/>
+      <c r="L796" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M796" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N796" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O796" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P796" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q796" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R796" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S796" s="4" t="n"/>
+      <c r="T796" s="4" t="n"/>
+      <c r="U796" s="4" t="n"/>
+      <c r="V796" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W796" s="4" t="inlineStr"/>
+      <c r="X796" s="4" t="n"/>
+      <c r="Y796" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z796" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA796" s="4" t="n"/>
+      <c r="AB796" s="4" t="n"/>
+      <c r="AC796" s="4" t="n"/>
+      <c r="AD796" s="4" t="n"/>
+      <c r="AE796" s="4" t="n"/>
+      <c r="AF796" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="797">
+      <c r="A797" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B797" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C797" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D797" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E797" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F797" s="6" t="n"/>
+      <c r="G797" s="6" t="n"/>
+      <c r="H797" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I797" s="6" t="inlineStr"/>
+      <c r="J797" s="6" t="inlineStr"/>
+      <c r="K797" s="6" t="inlineStr"/>
+      <c r="L797" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M797" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N797" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O797" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P797" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q797" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R797" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S797" s="6" t="n"/>
+      <c r="T797" s="6" t="n"/>
+      <c r="U797" s="6" t="n"/>
+      <c r="V797" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W797" s="6" t="inlineStr"/>
+      <c r="X797" s="6" t="n"/>
+      <c r="Y797" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z797" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA797" s="6" t="n"/>
+      <c r="AB797" s="6" t="n"/>
+      <c r="AC797" s="6" t="n"/>
+      <c r="AD797" s="6" t="n"/>
+      <c r="AE797" s="6" t="n"/>
+      <c r="AF797" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="798">
+      <c r="A798" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B798" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C798" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D798" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E798" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F798" s="4" t="n"/>
+      <c r="G798" s="4" t="n"/>
+      <c r="H798" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I798" s="4" t="inlineStr"/>
+      <c r="J798" s="4" t="inlineStr"/>
+      <c r="K798" s="4" t="inlineStr"/>
+      <c r="L798" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M798" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N798" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O798" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P798" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q798" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R798" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S798" s="4" t="n"/>
+      <c r="T798" s="4" t="n"/>
+      <c r="U798" s="4" t="n"/>
+      <c r="V798" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W798" s="4" t="inlineStr"/>
+      <c r="X798" s="4" t="n"/>
+      <c r="Y798" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z798" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA798" s="4" t="n"/>
+      <c r="AB798" s="4" t="n"/>
+      <c r="AC798" s="4" t="n"/>
+      <c r="AD798" s="4" t="n"/>
+      <c r="AE798" s="4" t="n"/>
+      <c r="AF798" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="799">
+      <c r="A799" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B799" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C799" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D799" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E799" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F799" s="6" t="n"/>
+      <c r="G799" s="6" t="n"/>
+      <c r="H799" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I799" s="6" t="inlineStr"/>
+      <c r="J799" s="6" t="inlineStr"/>
+      <c r="K799" s="6" t="inlineStr"/>
+      <c r="L799" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M799" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N799" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O799" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P799" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q799" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R799" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S799" s="6" t="n"/>
+      <c r="T799" s="6" t="n"/>
+      <c r="U799" s="6" t="n"/>
+      <c r="V799" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W799" s="6" t="inlineStr"/>
+      <c r="X799" s="6" t="n"/>
+      <c r="Y799" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z799" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA799" s="6" t="n"/>
+      <c r="AB799" s="6" t="n"/>
+      <c r="AC799" s="6" t="n"/>
+      <c r="AD799" s="6" t="n"/>
+      <c r="AE799" s="6" t="n"/>
+      <c r="AF799" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="800">
+      <c r="A800" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B800" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C800" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D800" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E800" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F800" s="4" t="n"/>
+      <c r="G800" s="4" t="n"/>
+      <c r="H800" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I800" s="4" t="inlineStr"/>
+      <c r="J800" s="4" t="inlineStr"/>
+      <c r="K800" s="4" t="inlineStr"/>
+      <c r="L800" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M800" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N800" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O800" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P800" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q800" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R800" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S800" s="4" t="n"/>
+      <c r="T800" s="4" t="n"/>
+      <c r="U800" s="4" t="n"/>
+      <c r="V800" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W800" s="4" t="inlineStr"/>
+      <c r="X800" s="4" t="n"/>
+      <c r="Y800" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z800" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA800" s="4" t="n"/>
+      <c r="AB800" s="4" t="n"/>
+      <c r="AC800" s="4" t="n"/>
+      <c r="AD800" s="4" t="n"/>
+      <c r="AE800" s="4" t="n"/>
+      <c r="AF800" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="801">
+      <c r="A801" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B801" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C801" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D801" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E801" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F801" s="6" t="n"/>
+      <c r="G801" s="6" t="n"/>
+      <c r="H801" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I801" s="6" t="inlineStr"/>
+      <c r="J801" s="6" t="inlineStr"/>
+      <c r="K801" s="6" t="inlineStr"/>
+      <c r="L801" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M801" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N801" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O801" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P801" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q801" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R801" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S801" s="6" t="n"/>
+      <c r="T801" s="6" t="n"/>
+      <c r="U801" s="6" t="n"/>
+      <c r="V801" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W801" s="6" t="inlineStr"/>
+      <c r="X801" s="6" t="n"/>
+      <c r="Y801" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z801" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA801" s="6" t="n"/>
+      <c r="AB801" s="6" t="n"/>
+      <c r="AC801" s="6" t="n"/>
+      <c r="AD801" s="6" t="n"/>
+      <c r="AE801" s="6" t="n"/>
+      <c r="AF801" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="802">
+      <c r="A802" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B802" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C802" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D802" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E802" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F802" s="4" t="n"/>
+      <c r="G802" s="4" t="n"/>
+      <c r="H802" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I802" s="4" t="inlineStr"/>
+      <c r="J802" s="4" t="inlineStr"/>
+      <c r="K802" s="4" t="inlineStr"/>
+      <c r="L802" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M802" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N802" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O802" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P802" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q802" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R802" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S802" s="4" t="n"/>
+      <c r="T802" s="4" t="n"/>
+      <c r="U802" s="4" t="n"/>
+      <c r="V802" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W802" s="4" t="inlineStr"/>
+      <c r="X802" s="4" t="n"/>
+      <c r="Y802" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z802" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA802" s="4" t="n"/>
+      <c r="AB802" s="4" t="n"/>
+      <c r="AC802" s="4" t="n"/>
+      <c r="AD802" s="4" t="n"/>
+      <c r="AE802" s="4" t="n"/>
+      <c r="AF802" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="803">
+      <c r="A803" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B803" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C803" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D803" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E803" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F803" s="6" t="n"/>
+      <c r="G803" s="6" t="n"/>
+      <c r="H803" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I803" s="6" t="inlineStr"/>
+      <c r="J803" s="6" t="inlineStr"/>
+      <c r="K803" s="6" t="inlineStr"/>
+      <c r="L803" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M803" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N803" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O803" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P803" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q803" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R803" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S803" s="6" t="n"/>
+      <c r="T803" s="6" t="n"/>
+      <c r="U803" s="6" t="n"/>
+      <c r="V803" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W803" s="6" t="inlineStr"/>
+      <c r="X803" s="6" t="n"/>
+      <c r="Y803" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z803" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA803" s="6" t="n"/>
+      <c r="AB803" s="6" t="n"/>
+      <c r="AC803" s="6" t="n"/>
+      <c r="AD803" s="6" t="n"/>
+      <c r="AE803" s="6" t="n"/>
+      <c r="AF803" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="804">
+      <c r="A804" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B804" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C804" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D804" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E804" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F804" s="4" t="n"/>
+      <c r="G804" s="4" t="n"/>
+      <c r="H804" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I804" s="4" t="inlineStr"/>
+      <c r="J804" s="4" t="inlineStr"/>
+      <c r="K804" s="4" t="inlineStr"/>
+      <c r="L804" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M804" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N804" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O804" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P804" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q804" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R804" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S804" s="4" t="n"/>
+      <c r="T804" s="4" t="n"/>
+      <c r="U804" s="4" t="n"/>
+      <c r="V804" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W804" s="4" t="inlineStr"/>
+      <c r="X804" s="4" t="n"/>
+      <c r="Y804" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z804" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA804" s="4" t="n"/>
+      <c r="AB804" s="4" t="n"/>
+      <c r="AC804" s="4" t="n"/>
+      <c r="AD804" s="4" t="n"/>
+      <c r="AE804" s="4" t="n"/>
+      <c r="AF804" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="805">
+      <c r="A805" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B805" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C805" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D805" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E805" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F805" s="6" t="n"/>
+      <c r="G805" s="6" t="n"/>
+      <c r="H805" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I805" s="6" t="inlineStr"/>
+      <c r="J805" s="6" t="inlineStr"/>
+      <c r="K805" s="6" t="inlineStr"/>
+      <c r="L805" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M805" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N805" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O805" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P805" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q805" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R805" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S805" s="6" t="n"/>
+      <c r="T805" s="6" t="n"/>
+      <c r="U805" s="6" t="n"/>
+      <c r="V805" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W805" s="6" t="inlineStr"/>
+      <c r="X805" s="6" t="n"/>
+      <c r="Y805" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z805" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA805" s="6" t="n"/>
+      <c r="AB805" s="6" t="n"/>
+      <c r="AC805" s="6" t="n"/>
+      <c r="AD805" s="6" t="n"/>
+      <c r="AE805" s="6" t="n"/>
+      <c r="AF805" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="806">
+      <c r="A806" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B806" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C806" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D806" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E806" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F806" s="4" t="n"/>
+      <c r="G806" s="4" t="n"/>
+      <c r="H806" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I806" s="4" t="inlineStr"/>
+      <c r="J806" s="4" t="inlineStr"/>
+      <c r="K806" s="4" t="inlineStr"/>
+      <c r="L806" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M806" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N806" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O806" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P806" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q806" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R806" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S806" s="4" t="n"/>
+      <c r="T806" s="4" t="n"/>
+      <c r="U806" s="4" t="n"/>
+      <c r="V806" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W806" s="4" t="inlineStr"/>
+      <c r="X806" s="4" t="n"/>
+      <c r="Y806" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z806" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA806" s="4" t="n"/>
+      <c r="AB806" s="4" t="n"/>
+      <c r="AC806" s="4" t="n"/>
+      <c r="AD806" s="4" t="n"/>
+      <c r="AE806" s="4" t="n"/>
+      <c r="AF806" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="807">
+      <c r="A807" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B807" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C807" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D807" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E807" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F807" s="6" t="n"/>
+      <c r="G807" s="6" t="n"/>
+      <c r="H807" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I807" s="6" t="inlineStr"/>
+      <c r="J807" s="6" t="inlineStr"/>
+      <c r="K807" s="6" t="inlineStr"/>
+      <c r="L807" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M807" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N807" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O807" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P807" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q807" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R807" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S807" s="6" t="n"/>
+      <c r="T807" s="6" t="n"/>
+      <c r="U807" s="6" t="n"/>
+      <c r="V807" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W807" s="6" t="inlineStr"/>
+      <c r="X807" s="6" t="n"/>
+      <c r="Y807" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z807" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA807" s="6" t="n"/>
+      <c r="AB807" s="6" t="n"/>
+      <c r="AC807" s="6" t="n"/>
+      <c r="AD807" s="6" t="n"/>
+      <c r="AE807" s="6" t="n"/>
+      <c r="AF807" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="808">
+      <c r="A808" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B808" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C808" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D808" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E808" s="4" t="n">
+        <v>54.99</v>
+      </c>
+      <c r="F808" s="4" t="n"/>
+      <c r="G808" s="4" t="n"/>
+      <c r="H808" s="4" t="n">
+        <v>62.85</v>
+      </c>
+      <c r="I808" s="4" t="inlineStr"/>
+      <c r="J808" s="4" t="inlineStr"/>
+      <c r="K808" s="4" t="inlineStr"/>
+      <c r="L808" s="4" t="n">
+        <v>79.56</v>
+      </c>
+      <c r="M808" s="4" t="n">
+        <v>2.387</v>
+      </c>
+      <c r="N808" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O808" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P808" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q808" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R808" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S808" s="4" t="n"/>
+      <c r="T808" s="4" t="n"/>
+      <c r="U808" s="4" t="n"/>
+      <c r="V808" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W808" s="4" t="inlineStr"/>
+      <c r="X808" s="4" t="n"/>
+      <c r="Y808" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z808" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA808" s="4" t="n"/>
+      <c r="AB808" s="4" t="n"/>
+      <c r="AC808" s="4" t="n"/>
+      <c r="AD808" s="4" t="n"/>
+      <c r="AE808" s="4" t="n"/>
+      <c r="AF808" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="809">
+      <c r="A809" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B809" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C809" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D809" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E809" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F809" s="6" t="n"/>
+      <c r="G809" s="6" t="n"/>
+      <c r="H809" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I809" s="6" t="inlineStr"/>
+      <c r="J809" s="6" t="inlineStr"/>
+      <c r="K809" s="6" t="inlineStr"/>
+      <c r="L809" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M809" s="6" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N809" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O809" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P809" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q809" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R809" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S809" s="6" t="n"/>
+      <c r="T809" s="6" t="n"/>
+      <c r="U809" s="6" t="n"/>
+      <c r="V809" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W809" s="6" t="inlineStr"/>
+      <c r="X809" s="6" t="n"/>
+      <c r="Y809" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z809" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA809" s="6" t="n"/>
+      <c r="AB809" s="6" t="n"/>
+      <c r="AC809" s="6" t="n"/>
+      <c r="AD809" s="6" t="n"/>
+      <c r="AE809" s="6" t="n"/>
+      <c r="AF809" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="810">
+      <c r="A810" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B810" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C810" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D810" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E810" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F810" s="4" t="n"/>
+      <c r="G810" s="4" t="n"/>
+      <c r="H810" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I810" s="4" t="inlineStr"/>
+      <c r="J810" s="4" t="inlineStr"/>
+      <c r="K810" s="4" t="inlineStr"/>
+      <c r="L810" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M810" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N810" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O810" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P810" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q810" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R810" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S810" s="4" t="n"/>
+      <c r="T810" s="4" t="n"/>
+      <c r="U810" s="4" t="n"/>
+      <c r="V810" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W810" s="4" t="inlineStr"/>
+      <c r="X810" s="4" t="n"/>
+      <c r="Y810" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z810" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA810" s="4" t="n"/>
+      <c r="AB810" s="4" t="n"/>
+      <c r="AC810" s="4" t="n"/>
+      <c r="AD810" s="4" t="n"/>
+      <c r="AE810" s="4" t="n"/>
+      <c r="AF810" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="811">
+      <c r="A811" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B811" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C811" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D811" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E811" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F811" s="6" t="n"/>
+      <c r="G811" s="6" t="n"/>
+      <c r="H811" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I811" s="6" t="inlineStr"/>
+      <c r="J811" s="6" t="inlineStr"/>
+      <c r="K811" s="6" t="inlineStr"/>
+      <c r="L811" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M811" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N811" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O811" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P811" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q811" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R811" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S811" s="6" t="n"/>
+      <c r="T811" s="6" t="n"/>
+      <c r="U811" s="6" t="n"/>
+      <c r="V811" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W811" s="6" t="inlineStr"/>
+      <c r="X811" s="6" t="n"/>
+      <c r="Y811" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z811" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA811" s="6" t="n"/>
+      <c r="AB811" s="6" t="n"/>
+      <c r="AC811" s="6" t="n"/>
+      <c r="AD811" s="6" t="n"/>
+      <c r="AE811" s="6" t="n"/>
+      <c r="AF811" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="812">
+      <c r="A812" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B812" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C812" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D812" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E812" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F812" s="4" t="n"/>
+      <c r="G812" s="4" t="n"/>
+      <c r="H812" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I812" s="4" t="inlineStr"/>
+      <c r="J812" s="4" t="inlineStr"/>
+      <c r="K812" s="4" t="inlineStr"/>
+      <c r="L812" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M812" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N812" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O812" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P812" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q812" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R812" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S812" s="4" t="n"/>
+      <c r="T812" s="4" t="n"/>
+      <c r="U812" s="4" t="n"/>
+      <c r="V812" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W812" s="4" t="inlineStr"/>
+      <c r="X812" s="4" t="n"/>
+      <c r="Y812" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z812" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA812" s="4" t="n"/>
+      <c r="AB812" s="4" t="n"/>
+      <c r="AC812" s="4" t="n"/>
+      <c r="AD812" s="4" t="n"/>
+      <c r="AE812" s="4" t="n"/>
+      <c r="AF812" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="813">
+      <c r="A813" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B813" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C813" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D813" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E813" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F813" s="6" t="n"/>
+      <c r="G813" s="6" t="n"/>
+      <c r="H813" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I813" s="6" t="inlineStr"/>
+      <c r="J813" s="6" t="inlineStr"/>
+      <c r="K813" s="6" t="inlineStr"/>
+      <c r="L813" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M813" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N813" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O813" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P813" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q813" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R813" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S813" s="6" t="n"/>
+      <c r="T813" s="6" t="n"/>
+      <c r="U813" s="6" t="n"/>
+      <c r="V813" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W813" s="6" t="inlineStr"/>
+      <c r="X813" s="6" t="n"/>
+      <c r="Y813" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z813" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA813" s="6" t="n"/>
+      <c r="AB813" s="6" t="n"/>
+      <c r="AC813" s="6" t="n"/>
+      <c r="AD813" s="6" t="n"/>
+      <c r="AE813" s="6" t="n"/>
+      <c r="AF813" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="814">
+      <c r="A814" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B814" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C814" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D814" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E814" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F814" s="4" t="n"/>
+      <c r="G814" s="4" t="n"/>
+      <c r="H814" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I814" s="4" t="inlineStr"/>
+      <c r="J814" s="4" t="inlineStr"/>
+      <c r="K814" s="4" t="inlineStr"/>
+      <c r="L814" s="4" t="n"/>
+      <c r="M814" s="4" t="n"/>
+      <c r="N814" s="4" t="n"/>
+      <c r="O814" s="4" t="n"/>
+      <c r="P814" s="4" t="n"/>
+      <c r="Q814" s="4" t="n"/>
+      <c r="R814" s="4" t="n"/>
+      <c r="S814" s="4" t="n"/>
+      <c r="T814" s="4" t="n"/>
+      <c r="U814" s="4" t="n"/>
+      <c r="V814" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W814" s="4" t="inlineStr"/>
+      <c r="X814" s="4" t="n"/>
+      <c r="Y814" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z814" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA814" s="4" t="n"/>
+      <c r="AB814" s="4" t="n"/>
+      <c r="AC814" s="4" t="n"/>
+      <c r="AD814" s="4" t="n"/>
+      <c r="AE814" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF814" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="815">
+      <c r="A815" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B815" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C815" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D815" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E815" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F815" s="6" t="n"/>
+      <c r="G815" s="6" t="n"/>
+      <c r="H815" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I815" s="6" t="inlineStr"/>
+      <c r="J815" s="6" t="inlineStr"/>
+      <c r="K815" s="6" t="inlineStr"/>
+      <c r="L815" s="6" t="n"/>
+      <c r="M815" s="6" t="n"/>
+      <c r="N815" s="6" t="n"/>
+      <c r="O815" s="6" t="n"/>
+      <c r="P815" s="6" t="n"/>
+      <c r="Q815" s="6" t="n"/>
+      <c r="R815" s="6" t="n"/>
+      <c r="S815" s="6" t="n"/>
+      <c r="T815" s="6" t="n"/>
+      <c r="U815" s="6" t="n"/>
+      <c r="V815" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W815" s="6" t="inlineStr"/>
+      <c r="X815" s="6" t="n"/>
+      <c r="Y815" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z815" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA815" s="6" t="n"/>
+      <c r="AB815" s="6" t="n"/>
+      <c r="AC815" s="6" t="n"/>
+      <c r="AD815" s="6" t="n"/>
+      <c r="AE815" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF815" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="816">
+      <c r="A816" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B816" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C816" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D816" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E816" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F816" s="4" t="n"/>
+      <c r="G816" s="4" t="n"/>
+      <c r="H816" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I816" s="4" t="inlineStr"/>
+      <c r="J816" s="4" t="inlineStr"/>
+      <c r="K816" s="4" t="inlineStr"/>
+      <c r="L816" s="4" t="n"/>
+      <c r="M816" s="4" t="n"/>
+      <c r="N816" s="4" t="n"/>
+      <c r="O816" s="4" t="n"/>
+      <c r="P816" s="4" t="n"/>
+      <c r="Q816" s="4" t="n"/>
+      <c r="R816" s="4" t="n"/>
+      <c r="S816" s="4" t="n"/>
+      <c r="T816" s="4" t="n"/>
+      <c r="U816" s="4" t="n"/>
+      <c r="V816" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W816" s="4" t="inlineStr"/>
+      <c r="X816" s="4" t="n"/>
+      <c r="Y816" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z816" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA816" s="4" t="n"/>
+      <c r="AB816" s="4" t="n"/>
+      <c r="AC816" s="4" t="n"/>
+      <c r="AD816" s="4" t="n"/>
+      <c r="AE816" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF816" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="817">
+      <c r="A817" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B817" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C817" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D817" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E817" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F817" s="6" t="n"/>
+      <c r="G817" s="6" t="n"/>
+      <c r="H817" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I817" s="6" t="inlineStr"/>
+      <c r="J817" s="6" t="inlineStr"/>
+      <c r="K817" s="6" t="inlineStr"/>
+      <c r="L817" s="6" t="n"/>
+      <c r="M817" s="6" t="n"/>
+      <c r="N817" s="6" t="n"/>
+      <c r="O817" s="6" t="n"/>
+      <c r="P817" s="6" t="n"/>
+      <c r="Q817" s="6" t="n"/>
+      <c r="R817" s="6" t="n"/>
+      <c r="S817" s="6" t="n"/>
+      <c r="T817" s="6" t="n"/>
+      <c r="U817" s="6" t="n"/>
+      <c r="V817" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W817" s="6" t="inlineStr"/>
+      <c r="X817" s="6" t="n"/>
+      <c r="Y817" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z817" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA817" s="6" t="n"/>
+      <c r="AB817" s="6" t="n"/>
+      <c r="AC817" s="6" t="n"/>
+      <c r="AD817" s="6" t="n"/>
+      <c r="AE817" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF817" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="818">
+      <c r="A818" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B818" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C818" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D818" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E818" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F818" s="4" t="n"/>
+      <c r="G818" s="4" t="n"/>
+      <c r="H818" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I818" s="4" t="inlineStr"/>
+      <c r="J818" s="4" t="inlineStr"/>
+      <c r="K818" s="4" t="inlineStr"/>
+      <c r="L818" s="4" t="n"/>
+      <c r="M818" s="4" t="n"/>
+      <c r="N818" s="4" t="n"/>
+      <c r="O818" s="4" t="n"/>
+      <c r="P818" s="4" t="n"/>
+      <c r="Q818" s="4" t="n"/>
+      <c r="R818" s="4" t="n"/>
+      <c r="S818" s="4" t="n"/>
+      <c r="T818" s="4" t="n"/>
+      <c r="U818" s="4" t="n"/>
+      <c r="V818" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W818" s="4" t="inlineStr"/>
+      <c r="X818" s="4" t="n"/>
+      <c r="Y818" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z818" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA818" s="4" t="n"/>
+      <c r="AB818" s="4" t="n"/>
+      <c r="AC818" s="4" t="n"/>
+      <c r="AD818" s="4" t="n"/>
+      <c r="AE818" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF818" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="819">
+      <c r="A819" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B819" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C819" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D819" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E819" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F819" s="6" t="n"/>
+      <c r="G819" s="6" t="n"/>
+      <c r="H819" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I819" s="6" t="inlineStr"/>
+      <c r="J819" s="6" t="inlineStr"/>
+      <c r="K819" s="6" t="inlineStr"/>
+      <c r="L819" s="6" t="n"/>
+      <c r="M819" s="6" t="n"/>
+      <c r="N819" s="6" t="n"/>
+      <c r="O819" s="6" t="n"/>
+      <c r="P819" s="6" t="n"/>
+      <c r="Q819" s="6" t="n"/>
+      <c r="R819" s="6" t="n"/>
+      <c r="S819" s="6" t="n"/>
+      <c r="T819" s="6" t="n"/>
+      <c r="U819" s="6" t="n"/>
+      <c r="V819" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W819" s="6" t="inlineStr"/>
+      <c r="X819" s="6" t="n"/>
+      <c r="Y819" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z819" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA819" s="6" t="n"/>
+      <c r="AB819" s="6" t="n"/>
+      <c r="AC819" s="6" t="n"/>
+      <c r="AD819" s="6" t="n"/>
+      <c r="AE819" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF819" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="820">
+      <c r="A820" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B820" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C820" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D820" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E820" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F820" s="4" t="n"/>
+      <c r="G820" s="4" t="n"/>
+      <c r="H820" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I820" s="4" t="inlineStr"/>
+      <c r="J820" s="4" t="inlineStr"/>
+      <c r="K820" s="4" t="inlineStr"/>
+      <c r="L820" s="4" t="n"/>
+      <c r="M820" s="4" t="n"/>
+      <c r="N820" s="4" t="n"/>
+      <c r="O820" s="4" t="n"/>
+      <c r="P820" s="4" t="n"/>
+      <c r="Q820" s="4" t="n"/>
+      <c r="R820" s="4" t="n"/>
+      <c r="S820" s="4" t="n"/>
+      <c r="T820" s="4" t="n"/>
+      <c r="U820" s="4" t="n"/>
+      <c r="V820" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W820" s="4" t="inlineStr"/>
+      <c r="X820" s="4" t="n"/>
+      <c r="Y820" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z820" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA820" s="4" t="n"/>
+      <c r="AB820" s="4" t="n"/>
+      <c r="AC820" s="4" t="n"/>
+      <c r="AD820" s="4" t="n"/>
+      <c r="AE820" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF820" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="821">
+      <c r="A821" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B821" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C821" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D821" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E821" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F821" s="6" t="n"/>
+      <c r="G821" s="6" t="n"/>
+      <c r="H821" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I821" s="6" t="inlineStr"/>
+      <c r="J821" s="6" t="inlineStr"/>
+      <c r="K821" s="6" t="inlineStr"/>
+      <c r="L821" s="6" t="n"/>
+      <c r="M821" s="6" t="n"/>
+      <c r="N821" s="6" t="n"/>
+      <c r="O821" s="6" t="n"/>
+      <c r="P821" s="6" t="n"/>
+      <c r="Q821" s="6" t="n"/>
+      <c r="R821" s="6" t="n"/>
+      <c r="S821" s="6" t="n"/>
+      <c r="T821" s="6" t="n"/>
+      <c r="U821" s="6" t="n"/>
+      <c r="V821" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W821" s="6" t="inlineStr"/>
+      <c r="X821" s="6" t="n"/>
+      <c r="Y821" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z821" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA821" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB821" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC821" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD821" s="6" t="n"/>
+      <c r="AE821" s="6" t="n"/>
+      <c r="AF821" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="822">
+      <c r="A822" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B822" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C822" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D822" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E822" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F822" s="4" t="n"/>
+      <c r="G822" s="4" t="n"/>
+      <c r="H822" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I822" s="4" t="inlineStr"/>
+      <c r="J822" s="4" t="inlineStr"/>
+      <c r="K822" s="4" t="inlineStr"/>
+      <c r="L822" s="4" t="n"/>
+      <c r="M822" s="4" t="n"/>
+      <c r="N822" s="4" t="n"/>
+      <c r="O822" s="4" t="n"/>
+      <c r="P822" s="4" t="n"/>
+      <c r="Q822" s="4" t="n"/>
+      <c r="R822" s="4" t="n"/>
+      <c r="S822" s="4" t="n"/>
+      <c r="T822" s="4" t="n"/>
+      <c r="U822" s="4" t="n"/>
+      <c r="V822" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W822" s="4" t="inlineStr"/>
+      <c r="X822" s="4" t="n"/>
+      <c r="Y822" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z822" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA822" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB822" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC822" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD822" s="4" t="n"/>
+      <c r="AE822" s="4" t="n"/>
+      <c r="AF822" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="823">
+      <c r="A823" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B823" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C823" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D823" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E823" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F823" s="6" t="n"/>
+      <c r="G823" s="6" t="n"/>
+      <c r="H823" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I823" s="6" t="inlineStr"/>
+      <c r="J823" s="6" t="inlineStr"/>
+      <c r="K823" s="6" t="inlineStr"/>
+      <c r="L823" s="6" t="n"/>
+      <c r="M823" s="6" t="n"/>
+      <c r="N823" s="6" t="n"/>
+      <c r="O823" s="6" t="n"/>
+      <c r="P823" s="6" t="n"/>
+      <c r="Q823" s="6" t="n"/>
+      <c r="R823" s="6" t="n"/>
+      <c r="S823" s="6" t="n"/>
+      <c r="T823" s="6" t="n"/>
+      <c r="U823" s="6" t="n"/>
+      <c r="V823" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W823" s="6" t="inlineStr"/>
+      <c r="X823" s="6" t="n"/>
+      <c r="Y823" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z823" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA823" s="6" t="n"/>
+      <c r="AB823" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC823" s="6" t="n"/>
+      <c r="AD823" s="6" t="n"/>
+      <c r="AE823" s="6" t="n"/>
+      <c r="AF823" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="824">
+      <c r="A824" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-11</t>
+        </is>
+      </c>
+      <c r="B824" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C824" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D824" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E824" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F824" s="4" t="n"/>
+      <c r="G824" s="4" t="n"/>
+      <c r="H824" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I824" s="4" t="inlineStr"/>
+      <c r="J824" s="4" t="inlineStr"/>
+      <c r="K824" s="4" t="inlineStr"/>
+      <c r="L824" s="4" t="n"/>
+      <c r="M824" s="4" t="n"/>
+      <c r="N824" s="4" t="n"/>
+      <c r="O824" s="4" t="n"/>
+      <c r="P824" s="4" t="n"/>
+      <c r="Q824" s="4" t="n"/>
+      <c r="R824" s="4" t="n"/>
+      <c r="S824" s="4" t="n"/>
+      <c r="T824" s="4" t="n"/>
+      <c r="U824" s="4" t="n"/>
+      <c r="V824" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W824" s="4" t="inlineStr"/>
+      <c r="X824" s="4" t="n"/>
+      <c r="Y824" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z824" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA824" s="4" t="n"/>
+      <c r="AB824" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC824" s="4" t="n"/>
+      <c r="AD824" s="4" t="n"/>
+      <c r="AE824" s="4" t="n"/>
+      <c r="AF824" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-12
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF824"/>
+  <dimension ref="A1:AF859"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -65378,6 +65378,2754 @@
         <v>1</v>
       </c>
     </row>
+    <row r="825">
+      <c r="A825" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B825" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C825" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D825" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E825" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F825" s="4" t="n"/>
+      <c r="G825" s="4" t="n"/>
+      <c r="H825" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I825" s="4" t="inlineStr"/>
+      <c r="J825" s="4" t="inlineStr"/>
+      <c r="K825" s="4" t="inlineStr"/>
+      <c r="L825" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M825" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N825" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O825" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P825" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q825" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R825" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S825" s="4" t="n"/>
+      <c r="T825" s="4" t="n"/>
+      <c r="U825" s="4" t="n"/>
+      <c r="V825" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W825" s="4" t="inlineStr"/>
+      <c r="X825" s="4" t="n"/>
+      <c r="Y825" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z825" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA825" s="4" t="n"/>
+      <c r="AB825" s="4" t="n"/>
+      <c r="AC825" s="4" t="n"/>
+      <c r="AD825" s="4" t="n"/>
+      <c r="AE825" s="4" t="n"/>
+      <c r="AF825" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="826">
+      <c r="A826" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B826" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C826" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D826" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E826" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F826" s="6" t="n"/>
+      <c r="G826" s="6" t="n"/>
+      <c r="H826" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I826" s="6" t="inlineStr"/>
+      <c r="J826" s="6" t="inlineStr"/>
+      <c r="K826" s="6" t="inlineStr"/>
+      <c r="L826" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M826" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N826" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O826" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P826" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q826" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R826" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S826" s="6" t="n"/>
+      <c r="T826" s="6" t="n"/>
+      <c r="U826" s="6" t="n"/>
+      <c r="V826" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W826" s="6" t="inlineStr"/>
+      <c r="X826" s="6" t="n"/>
+      <c r="Y826" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z826" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA826" s="6" t="n"/>
+      <c r="AB826" s="6" t="n"/>
+      <c r="AC826" s="6" t="n"/>
+      <c r="AD826" s="6" t="n"/>
+      <c r="AE826" s="6" t="n"/>
+      <c r="AF826" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="827">
+      <c r="A827" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B827" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C827" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D827" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E827" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F827" s="4" t="n"/>
+      <c r="G827" s="4" t="n"/>
+      <c r="H827" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I827" s="4" t="inlineStr"/>
+      <c r="J827" s="4" t="inlineStr"/>
+      <c r="K827" s="4" t="inlineStr"/>
+      <c r="L827" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M827" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N827" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O827" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P827" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q827" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R827" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S827" s="4" t="n"/>
+      <c r="T827" s="4" t="n"/>
+      <c r="U827" s="4" t="n"/>
+      <c r="V827" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W827" s="4" t="inlineStr"/>
+      <c r="X827" s="4" t="n"/>
+      <c r="Y827" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z827" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA827" s="4" t="n"/>
+      <c r="AB827" s="4" t="n"/>
+      <c r="AC827" s="4" t="n"/>
+      <c r="AD827" s="4" t="n"/>
+      <c r="AE827" s="4" t="n"/>
+      <c r="AF827" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="828">
+      <c r="A828" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B828" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C828" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D828" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E828" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F828" s="6" t="n"/>
+      <c r="G828" s="6" t="n"/>
+      <c r="H828" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I828" s="6" t="inlineStr"/>
+      <c r="J828" s="6" t="inlineStr"/>
+      <c r="K828" s="6" t="inlineStr"/>
+      <c r="L828" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M828" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N828" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O828" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P828" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q828" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R828" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S828" s="6" t="n"/>
+      <c r="T828" s="6" t="n"/>
+      <c r="U828" s="6" t="n"/>
+      <c r="V828" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W828" s="6" t="inlineStr"/>
+      <c r="X828" s="6" t="n"/>
+      <c r="Y828" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z828" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA828" s="6" t="n"/>
+      <c r="AB828" s="6" t="n"/>
+      <c r="AC828" s="6" t="n"/>
+      <c r="AD828" s="6" t="n"/>
+      <c r="AE828" s="6" t="n"/>
+      <c r="AF828" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="829">
+      <c r="A829" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B829" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C829" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D829" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E829" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F829" s="4" t="n"/>
+      <c r="G829" s="4" t="n"/>
+      <c r="H829" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I829" s="4" t="inlineStr"/>
+      <c r="J829" s="4" t="inlineStr"/>
+      <c r="K829" s="4" t="inlineStr"/>
+      <c r="L829" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M829" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N829" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O829" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P829" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q829" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R829" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S829" s="4" t="n"/>
+      <c r="T829" s="4" t="n"/>
+      <c r="U829" s="4" t="n"/>
+      <c r="V829" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W829" s="4" t="inlineStr"/>
+      <c r="X829" s="4" t="n"/>
+      <c r="Y829" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z829" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA829" s="4" t="n"/>
+      <c r="AB829" s="4" t="n"/>
+      <c r="AC829" s="4" t="n"/>
+      <c r="AD829" s="4" t="n"/>
+      <c r="AE829" s="4" t="n"/>
+      <c r="AF829" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="830">
+      <c r="A830" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B830" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C830" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D830" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E830" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F830" s="6" t="n"/>
+      <c r="G830" s="6" t="n"/>
+      <c r="H830" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I830" s="6" t="inlineStr"/>
+      <c r="J830" s="6" t="inlineStr"/>
+      <c r="K830" s="6" t="inlineStr"/>
+      <c r="L830" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M830" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N830" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O830" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P830" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q830" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R830" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S830" s="6" t="n"/>
+      <c r="T830" s="6" t="n"/>
+      <c r="U830" s="6" t="n"/>
+      <c r="V830" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W830" s="6" t="inlineStr"/>
+      <c r="X830" s="6" t="n"/>
+      <c r="Y830" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z830" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA830" s="6" t="n"/>
+      <c r="AB830" s="6" t="n"/>
+      <c r="AC830" s="6" t="n"/>
+      <c r="AD830" s="6" t="n"/>
+      <c r="AE830" s="6" t="n"/>
+      <c r="AF830" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="831">
+      <c r="A831" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B831" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C831" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D831" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E831" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F831" s="4" t="n"/>
+      <c r="G831" s="4" t="n"/>
+      <c r="H831" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I831" s="4" t="inlineStr"/>
+      <c r="J831" s="4" t="inlineStr"/>
+      <c r="K831" s="4" t="inlineStr"/>
+      <c r="L831" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M831" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N831" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O831" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P831" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q831" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R831" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S831" s="4" t="n"/>
+      <c r="T831" s="4" t="n"/>
+      <c r="U831" s="4" t="n"/>
+      <c r="V831" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W831" s="4" t="inlineStr"/>
+      <c r="X831" s="4" t="n"/>
+      <c r="Y831" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z831" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA831" s="4" t="n"/>
+      <c r="AB831" s="4" t="n"/>
+      <c r="AC831" s="4" t="n"/>
+      <c r="AD831" s="4" t="n"/>
+      <c r="AE831" s="4" t="n"/>
+      <c r="AF831" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="832">
+      <c r="A832" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B832" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C832" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D832" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E832" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F832" s="6" t="n"/>
+      <c r="G832" s="6" t="n"/>
+      <c r="H832" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I832" s="6" t="inlineStr"/>
+      <c r="J832" s="6" t="inlineStr"/>
+      <c r="K832" s="6" t="inlineStr"/>
+      <c r="L832" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M832" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N832" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O832" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P832" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q832" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R832" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S832" s="6" t="n"/>
+      <c r="T832" s="6" t="n"/>
+      <c r="U832" s="6" t="n"/>
+      <c r="V832" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W832" s="6" t="inlineStr"/>
+      <c r="X832" s="6" t="n"/>
+      <c r="Y832" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z832" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA832" s="6" t="n"/>
+      <c r="AB832" s="6" t="n"/>
+      <c r="AC832" s="6" t="n"/>
+      <c r="AD832" s="6" t="n"/>
+      <c r="AE832" s="6" t="n"/>
+      <c r="AF832" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="833">
+      <c r="A833" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B833" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C833" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D833" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E833" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F833" s="4" t="n"/>
+      <c r="G833" s="4" t="n"/>
+      <c r="H833" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I833" s="4" t="inlineStr"/>
+      <c r="J833" s="4" t="inlineStr"/>
+      <c r="K833" s="4" t="inlineStr"/>
+      <c r="L833" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M833" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N833" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O833" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P833" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q833" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R833" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S833" s="4" t="n"/>
+      <c r="T833" s="4" t="n"/>
+      <c r="U833" s="4" t="n"/>
+      <c r="V833" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W833" s="4" t="inlineStr"/>
+      <c r="X833" s="4" t="n"/>
+      <c r="Y833" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z833" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA833" s="4" t="n"/>
+      <c r="AB833" s="4" t="n"/>
+      <c r="AC833" s="4" t="n"/>
+      <c r="AD833" s="4" t="n"/>
+      <c r="AE833" s="4" t="n"/>
+      <c r="AF833" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="834">
+      <c r="A834" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B834" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C834" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D834" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E834" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F834" s="6" t="n"/>
+      <c r="G834" s="6" t="n"/>
+      <c r="H834" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I834" s="6" t="inlineStr"/>
+      <c r="J834" s="6" t="inlineStr"/>
+      <c r="K834" s="6" t="inlineStr"/>
+      <c r="L834" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M834" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N834" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O834" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P834" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q834" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R834" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S834" s="6" t="n"/>
+      <c r="T834" s="6" t="n"/>
+      <c r="U834" s="6" t="n"/>
+      <c r="V834" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W834" s="6" t="inlineStr"/>
+      <c r="X834" s="6" t="n"/>
+      <c r="Y834" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z834" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA834" s="6" t="n"/>
+      <c r="AB834" s="6" t="n"/>
+      <c r="AC834" s="6" t="n"/>
+      <c r="AD834" s="6" t="n"/>
+      <c r="AE834" s="6" t="n"/>
+      <c r="AF834" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="835">
+      <c r="A835" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B835" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C835" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D835" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E835" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F835" s="4" t="n"/>
+      <c r="G835" s="4" t="n"/>
+      <c r="H835" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I835" s="4" t="inlineStr"/>
+      <c r="J835" s="4" t="inlineStr"/>
+      <c r="K835" s="4" t="inlineStr"/>
+      <c r="L835" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M835" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N835" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O835" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P835" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q835" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R835" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S835" s="4" t="n"/>
+      <c r="T835" s="4" t="n"/>
+      <c r="U835" s="4" t="n"/>
+      <c r="V835" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W835" s="4" t="inlineStr"/>
+      <c r="X835" s="4" t="n"/>
+      <c r="Y835" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z835" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA835" s="4" t="n"/>
+      <c r="AB835" s="4" t="n"/>
+      <c r="AC835" s="4" t="n"/>
+      <c r="AD835" s="4" t="n"/>
+      <c r="AE835" s="4" t="n"/>
+      <c r="AF835" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="836">
+      <c r="A836" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B836" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C836" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D836" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E836" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F836" s="6" t="n"/>
+      <c r="G836" s="6" t="n"/>
+      <c r="H836" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I836" s="6" t="inlineStr"/>
+      <c r="J836" s="6" t="inlineStr"/>
+      <c r="K836" s="6" t="inlineStr"/>
+      <c r="L836" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M836" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N836" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O836" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P836" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q836" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R836" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S836" s="6" t="n"/>
+      <c r="T836" s="6" t="n"/>
+      <c r="U836" s="6" t="n"/>
+      <c r="V836" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W836" s="6" t="inlineStr"/>
+      <c r="X836" s="6" t="n"/>
+      <c r="Y836" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z836" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA836" s="6" t="n"/>
+      <c r="AB836" s="6" t="n"/>
+      <c r="AC836" s="6" t="n"/>
+      <c r="AD836" s="6" t="n"/>
+      <c r="AE836" s="6" t="n"/>
+      <c r="AF836" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="837">
+      <c r="A837" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B837" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C837" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D837" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E837" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F837" s="4" t="n"/>
+      <c r="G837" s="4" t="n"/>
+      <c r="H837" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I837" s="4" t="inlineStr"/>
+      <c r="J837" s="4" t="inlineStr"/>
+      <c r="K837" s="4" t="inlineStr"/>
+      <c r="L837" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M837" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N837" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O837" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P837" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q837" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R837" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S837" s="4" t="n"/>
+      <c r="T837" s="4" t="n"/>
+      <c r="U837" s="4" t="n"/>
+      <c r="V837" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W837" s="4" t="inlineStr"/>
+      <c r="X837" s="4" t="n"/>
+      <c r="Y837" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z837" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA837" s="4" t="n"/>
+      <c r="AB837" s="4" t="n"/>
+      <c r="AC837" s="4" t="n"/>
+      <c r="AD837" s="4" t="n"/>
+      <c r="AE837" s="4" t="n"/>
+      <c r="AF837" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="838">
+      <c r="A838" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B838" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C838" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D838" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E838" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F838" s="6" t="n"/>
+      <c r="G838" s="6" t="n"/>
+      <c r="H838" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I838" s="6" t="inlineStr"/>
+      <c r="J838" s="6" t="inlineStr"/>
+      <c r="K838" s="6" t="inlineStr"/>
+      <c r="L838" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M838" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N838" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O838" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P838" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q838" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R838" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S838" s="6" t="n"/>
+      <c r="T838" s="6" t="n"/>
+      <c r="U838" s="6" t="n"/>
+      <c r="V838" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W838" s="6" t="inlineStr"/>
+      <c r="X838" s="6" t="n"/>
+      <c r="Y838" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z838" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA838" s="6" t="n"/>
+      <c r="AB838" s="6" t="n"/>
+      <c r="AC838" s="6" t="n"/>
+      <c r="AD838" s="6" t="n"/>
+      <c r="AE838" s="6" t="n"/>
+      <c r="AF838" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="839">
+      <c r="A839" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B839" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C839" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D839" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E839" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F839" s="4" t="n"/>
+      <c r="G839" s="4" t="n"/>
+      <c r="H839" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I839" s="4" t="inlineStr"/>
+      <c r="J839" s="4" t="inlineStr"/>
+      <c r="K839" s="4" t="inlineStr"/>
+      <c r="L839" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M839" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N839" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O839" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P839" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q839" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R839" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S839" s="4" t="n"/>
+      <c r="T839" s="4" t="n"/>
+      <c r="U839" s="4" t="n"/>
+      <c r="V839" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W839" s="4" t="inlineStr"/>
+      <c r="X839" s="4" t="n"/>
+      <c r="Y839" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z839" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA839" s="4" t="n"/>
+      <c r="AB839" s="4" t="n"/>
+      <c r="AC839" s="4" t="n"/>
+      <c r="AD839" s="4" t="n"/>
+      <c r="AE839" s="4" t="n"/>
+      <c r="AF839" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="840">
+      <c r="A840" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B840" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C840" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D840" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E840" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F840" s="6" t="n"/>
+      <c r="G840" s="6" t="n"/>
+      <c r="H840" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I840" s="6" t="inlineStr"/>
+      <c r="J840" s="6" t="inlineStr"/>
+      <c r="K840" s="6" t="inlineStr"/>
+      <c r="L840" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M840" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N840" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O840" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P840" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q840" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R840" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S840" s="6" t="n"/>
+      <c r="T840" s="6" t="n"/>
+      <c r="U840" s="6" t="n"/>
+      <c r="V840" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W840" s="6" t="inlineStr"/>
+      <c r="X840" s="6" t="n"/>
+      <c r="Y840" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z840" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA840" s="6" t="n"/>
+      <c r="AB840" s="6" t="n"/>
+      <c r="AC840" s="6" t="n"/>
+      <c r="AD840" s="6" t="n"/>
+      <c r="AE840" s="6" t="n"/>
+      <c r="AF840" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="841">
+      <c r="A841" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B841" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C841" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D841" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E841" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F841" s="4" t="n"/>
+      <c r="G841" s="4" t="n"/>
+      <c r="H841" s="4" t="n">
+        <v>71.40000000000001</v>
+      </c>
+      <c r="I841" s="4" t="inlineStr"/>
+      <c r="J841" s="4" t="inlineStr"/>
+      <c r="K841" s="4" t="inlineStr"/>
+      <c r="L841" s="4" t="n">
+        <v>90.38</v>
+      </c>
+      <c r="M841" s="4" t="n">
+        <v>2.711</v>
+      </c>
+      <c r="N841" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O841" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P841" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q841" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R841" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S841" s="4" t="n"/>
+      <c r="T841" s="4" t="n"/>
+      <c r="U841" s="4" t="n"/>
+      <c r="V841" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W841" s="4" t="inlineStr"/>
+      <c r="X841" s="4" t="n"/>
+      <c r="Y841" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z841" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA841" s="4" t="n"/>
+      <c r="AB841" s="4" t="n"/>
+      <c r="AC841" s="4" t="n"/>
+      <c r="AD841" s="4" t="n"/>
+      <c r="AE841" s="4" t="n"/>
+      <c r="AF841" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="842">
+      <c r="A842" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B842" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C842" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D842" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E842" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F842" s="6" t="n"/>
+      <c r="G842" s="6" t="n"/>
+      <c r="H842" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I842" s="6" t="inlineStr"/>
+      <c r="J842" s="6" t="inlineStr"/>
+      <c r="K842" s="6" t="inlineStr"/>
+      <c r="L842" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M842" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N842" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O842" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P842" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q842" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R842" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S842" s="6" t="n"/>
+      <c r="T842" s="6" t="n"/>
+      <c r="U842" s="6" t="n"/>
+      <c r="V842" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W842" s="6" t="inlineStr"/>
+      <c r="X842" s="6" t="n"/>
+      <c r="Y842" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z842" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA842" s="6" t="n"/>
+      <c r="AB842" s="6" t="n"/>
+      <c r="AC842" s="6" t="n"/>
+      <c r="AD842" s="6" t="n"/>
+      <c r="AE842" s="6" t="n"/>
+      <c r="AF842" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="843">
+      <c r="A843" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B843" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C843" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D843" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E843" s="4" t="n">
+        <v>54.99</v>
+      </c>
+      <c r="F843" s="4" t="n"/>
+      <c r="G843" s="4" t="n"/>
+      <c r="H843" s="4" t="n">
+        <v>62.85</v>
+      </c>
+      <c r="I843" s="4" t="inlineStr"/>
+      <c r="J843" s="4" t="inlineStr"/>
+      <c r="K843" s="4" t="inlineStr"/>
+      <c r="L843" s="4" t="n">
+        <v>79.56</v>
+      </c>
+      <c r="M843" s="4" t="n">
+        <v>2.387</v>
+      </c>
+      <c r="N843" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O843" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P843" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q843" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R843" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S843" s="4" t="n"/>
+      <c r="T843" s="4" t="n"/>
+      <c r="U843" s="4" t="n"/>
+      <c r="V843" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W843" s="4" t="inlineStr"/>
+      <c r="X843" s="4" t="n"/>
+      <c r="Y843" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z843" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA843" s="4" t="n"/>
+      <c r="AB843" s="4" t="n"/>
+      <c r="AC843" s="4" t="n"/>
+      <c r="AD843" s="4" t="n"/>
+      <c r="AE843" s="4" t="n"/>
+      <c r="AF843" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="844">
+      <c r="A844" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B844" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C844" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D844" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E844" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F844" s="6" t="n"/>
+      <c r="G844" s="6" t="n"/>
+      <c r="H844" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I844" s="6" t="inlineStr"/>
+      <c r="J844" s="6" t="inlineStr"/>
+      <c r="K844" s="6" t="inlineStr"/>
+      <c r="L844" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M844" s="6" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N844" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O844" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P844" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q844" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R844" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S844" s="6" t="n"/>
+      <c r="T844" s="6" t="n"/>
+      <c r="U844" s="6" t="n"/>
+      <c r="V844" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W844" s="6" t="inlineStr"/>
+      <c r="X844" s="6" t="n"/>
+      <c r="Y844" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z844" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA844" s="6" t="n"/>
+      <c r="AB844" s="6" t="n"/>
+      <c r="AC844" s="6" t="n"/>
+      <c r="AD844" s="6" t="n"/>
+      <c r="AE844" s="6" t="n"/>
+      <c r="AF844" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="845">
+      <c r="A845" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B845" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C845" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D845" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E845" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F845" s="4" t="n"/>
+      <c r="G845" s="4" t="n"/>
+      <c r="H845" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I845" s="4" t="inlineStr"/>
+      <c r="J845" s="4" t="inlineStr"/>
+      <c r="K845" s="4" t="inlineStr"/>
+      <c r="L845" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M845" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N845" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O845" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P845" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q845" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R845" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S845" s="4" t="n"/>
+      <c r="T845" s="4" t="n"/>
+      <c r="U845" s="4" t="n"/>
+      <c r="V845" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W845" s="4" t="inlineStr"/>
+      <c r="X845" s="4" t="n"/>
+      <c r="Y845" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z845" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA845" s="4" t="n"/>
+      <c r="AB845" s="4" t="n"/>
+      <c r="AC845" s="4" t="n"/>
+      <c r="AD845" s="4" t="n"/>
+      <c r="AE845" s="4" t="n"/>
+      <c r="AF845" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="846">
+      <c r="A846" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B846" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C846" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D846" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E846" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F846" s="6" t="n"/>
+      <c r="G846" s="6" t="n"/>
+      <c r="H846" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I846" s="6" t="inlineStr"/>
+      <c r="J846" s="6" t="inlineStr"/>
+      <c r="K846" s="6" t="inlineStr"/>
+      <c r="L846" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M846" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N846" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O846" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P846" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q846" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R846" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S846" s="6" t="n"/>
+      <c r="T846" s="6" t="n"/>
+      <c r="U846" s="6" t="n"/>
+      <c r="V846" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W846" s="6" t="inlineStr"/>
+      <c r="X846" s="6" t="n"/>
+      <c r="Y846" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z846" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA846" s="6" t="n"/>
+      <c r="AB846" s="6" t="n"/>
+      <c r="AC846" s="6" t="n"/>
+      <c r="AD846" s="6" t="n"/>
+      <c r="AE846" s="6" t="n"/>
+      <c r="AF846" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="847">
+      <c r="A847" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B847" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C847" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D847" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E847" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F847" s="4" t="n"/>
+      <c r="G847" s="4" t="n"/>
+      <c r="H847" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I847" s="4" t="inlineStr"/>
+      <c r="J847" s="4" t="inlineStr"/>
+      <c r="K847" s="4" t="inlineStr"/>
+      <c r="L847" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M847" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N847" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O847" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P847" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q847" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R847" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S847" s="4" t="n"/>
+      <c r="T847" s="4" t="n"/>
+      <c r="U847" s="4" t="n"/>
+      <c r="V847" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W847" s="4" t="inlineStr"/>
+      <c r="X847" s="4" t="n"/>
+      <c r="Y847" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z847" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA847" s="4" t="n"/>
+      <c r="AB847" s="4" t="n"/>
+      <c r="AC847" s="4" t="n"/>
+      <c r="AD847" s="4" t="n"/>
+      <c r="AE847" s="4" t="n"/>
+      <c r="AF847" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="848">
+      <c r="A848" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B848" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C848" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D848" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E848" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F848" s="6" t="n"/>
+      <c r="G848" s="6" t="n"/>
+      <c r="H848" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I848" s="6" t="inlineStr"/>
+      <c r="J848" s="6" t="inlineStr"/>
+      <c r="K848" s="6" t="inlineStr"/>
+      <c r="L848" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M848" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N848" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O848" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P848" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q848" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R848" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S848" s="6" t="n"/>
+      <c r="T848" s="6" t="n"/>
+      <c r="U848" s="6" t="n"/>
+      <c r="V848" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W848" s="6" t="inlineStr"/>
+      <c r="X848" s="6" t="n"/>
+      <c r="Y848" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z848" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA848" s="6" t="n"/>
+      <c r="AB848" s="6" t="n"/>
+      <c r="AC848" s="6" t="n"/>
+      <c r="AD848" s="6" t="n"/>
+      <c r="AE848" s="6" t="n"/>
+      <c r="AF848" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="849">
+      <c r="A849" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B849" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C849" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D849" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E849" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F849" s="4" t="n"/>
+      <c r="G849" s="4" t="n"/>
+      <c r="H849" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I849" s="4" t="inlineStr"/>
+      <c r="J849" s="4" t="inlineStr"/>
+      <c r="K849" s="4" t="inlineStr"/>
+      <c r="L849" s="4" t="n"/>
+      <c r="M849" s="4" t="n"/>
+      <c r="N849" s="4" t="n"/>
+      <c r="O849" s="4" t="n"/>
+      <c r="P849" s="4" t="n"/>
+      <c r="Q849" s="4" t="n"/>
+      <c r="R849" s="4" t="n"/>
+      <c r="S849" s="4" t="n"/>
+      <c r="T849" s="4" t="n"/>
+      <c r="U849" s="4" t="n"/>
+      <c r="V849" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W849" s="4" t="inlineStr"/>
+      <c r="X849" s="4" t="n"/>
+      <c r="Y849" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z849" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA849" s="4" t="n"/>
+      <c r="AB849" s="4" t="n"/>
+      <c r="AC849" s="4" t="n"/>
+      <c r="AD849" s="4" t="n"/>
+      <c r="AE849" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF849" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="850">
+      <c r="A850" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B850" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C850" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D850" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E850" s="6" t="n">
+        <v>8.289999999999999</v>
+      </c>
+      <c r="F850" s="6" t="n"/>
+      <c r="G850" s="6" t="n"/>
+      <c r="H850" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="I850" s="6" t="inlineStr"/>
+      <c r="J850" s="6" t="inlineStr"/>
+      <c r="K850" s="6" t="inlineStr"/>
+      <c r="L850" s="6" t="n"/>
+      <c r="M850" s="6" t="n"/>
+      <c r="N850" s="6" t="n"/>
+      <c r="O850" s="6" t="n"/>
+      <c r="P850" s="6" t="n"/>
+      <c r="Q850" s="6" t="n"/>
+      <c r="R850" s="6" t="n"/>
+      <c r="S850" s="6" t="n"/>
+      <c r="T850" s="6" t="n"/>
+      <c r="U850" s="6" t="n"/>
+      <c r="V850" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W850" s="6" t="inlineStr"/>
+      <c r="X850" s="6" t="n"/>
+      <c r="Y850" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z850" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA850" s="6" t="n"/>
+      <c r="AB850" s="6" t="n"/>
+      <c r="AC850" s="6" t="n"/>
+      <c r="AD850" s="6" t="n"/>
+      <c r="AE850" s="6" t="n">
+        <v>33.16</v>
+      </c>
+      <c r="AF850" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="851">
+      <c r="A851" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B851" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C851" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D851" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E851" s="4" t="n">
+        <v>13.79</v>
+      </c>
+      <c r="F851" s="4" t="n"/>
+      <c r="G851" s="4" t="n"/>
+      <c r="H851" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="I851" s="4" t="inlineStr"/>
+      <c r="J851" s="4" t="inlineStr"/>
+      <c r="K851" s="4" t="inlineStr"/>
+      <c r="L851" s="4" t="n"/>
+      <c r="M851" s="4" t="n"/>
+      <c r="N851" s="4" t="n"/>
+      <c r="O851" s="4" t="n"/>
+      <c r="P851" s="4" t="n"/>
+      <c r="Q851" s="4" t="n"/>
+      <c r="R851" s="4" t="n"/>
+      <c r="S851" s="4" t="n"/>
+      <c r="T851" s="4" t="n"/>
+      <c r="U851" s="4" t="n"/>
+      <c r="V851" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W851" s="4" t="inlineStr"/>
+      <c r="X851" s="4" t="n"/>
+      <c r="Y851" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z851" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA851" s="4" t="n"/>
+      <c r="AB851" s="4" t="n"/>
+      <c r="AC851" s="4" t="n"/>
+      <c r="AD851" s="4" t="n"/>
+      <c r="AE851" s="4" t="n">
+        <v>27.58</v>
+      </c>
+      <c r="AF851" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="852">
+      <c r="A852" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B852" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C852" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D852" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E852" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="F852" s="6" t="n"/>
+      <c r="G852" s="6" t="n"/>
+      <c r="H852" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="I852" s="6" t="inlineStr"/>
+      <c r="J852" s="6" t="inlineStr"/>
+      <c r="K852" s="6" t="inlineStr"/>
+      <c r="L852" s="6" t="n"/>
+      <c r="M852" s="6" t="n"/>
+      <c r="N852" s="6" t="n"/>
+      <c r="O852" s="6" t="n"/>
+      <c r="P852" s="6" t="n"/>
+      <c r="Q852" s="6" t="n"/>
+      <c r="R852" s="6" t="n"/>
+      <c r="S852" s="6" t="n"/>
+      <c r="T852" s="6" t="n"/>
+      <c r="U852" s="6" t="n"/>
+      <c r="V852" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W852" s="6" t="inlineStr"/>
+      <c r="X852" s="6" t="n"/>
+      <c r="Y852" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z852" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA852" s="6" t="n"/>
+      <c r="AB852" s="6" t="n"/>
+      <c r="AC852" s="6" t="n"/>
+      <c r="AD852" s="6" t="n"/>
+      <c r="AE852" s="6" t="n">
+        <v>25.49</v>
+      </c>
+      <c r="AF852" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="853">
+      <c r="A853" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B853" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C853" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D853" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E853" s="4" t="n">
+        <v>17.39</v>
+      </c>
+      <c r="F853" s="4" t="n"/>
+      <c r="G853" s="4" t="n"/>
+      <c r="H853" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="I853" s="4" t="inlineStr"/>
+      <c r="J853" s="4" t="inlineStr"/>
+      <c r="K853" s="4" t="inlineStr"/>
+      <c r="L853" s="4" t="n"/>
+      <c r="M853" s="4" t="n"/>
+      <c r="N853" s="4" t="n"/>
+      <c r="O853" s="4" t="n"/>
+      <c r="P853" s="4" t="n"/>
+      <c r="Q853" s="4" t="n"/>
+      <c r="R853" s="4" t="n"/>
+      <c r="S853" s="4" t="n"/>
+      <c r="T853" s="4" t="n"/>
+      <c r="U853" s="4" t="n"/>
+      <c r="V853" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W853" s="4" t="inlineStr"/>
+      <c r="X853" s="4" t="n"/>
+      <c r="Y853" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z853" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA853" s="4" t="n"/>
+      <c r="AB853" s="4" t="n"/>
+      <c r="AC853" s="4" t="n"/>
+      <c r="AD853" s="4" t="n"/>
+      <c r="AE853" s="4" t="n">
+        <v>69.56</v>
+      </c>
+      <c r="AF853" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="854">
+      <c r="A854" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B854" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C854" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D854" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E854" s="6" t="n">
+        <v>25.79</v>
+      </c>
+      <c r="F854" s="6" t="n"/>
+      <c r="G854" s="6" t="n"/>
+      <c r="H854" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="I854" s="6" t="inlineStr"/>
+      <c r="J854" s="6" t="inlineStr"/>
+      <c r="K854" s="6" t="inlineStr"/>
+      <c r="L854" s="6" t="n"/>
+      <c r="M854" s="6" t="n"/>
+      <c r="N854" s="6" t="n"/>
+      <c r="O854" s="6" t="n"/>
+      <c r="P854" s="6" t="n"/>
+      <c r="Q854" s="6" t="n"/>
+      <c r="R854" s="6" t="n"/>
+      <c r="S854" s="6" t="n"/>
+      <c r="T854" s="6" t="n"/>
+      <c r="U854" s="6" t="n"/>
+      <c r="V854" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W854" s="6" t="inlineStr"/>
+      <c r="X854" s="6" t="n"/>
+      <c r="Y854" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z854" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA854" s="6" t="n"/>
+      <c r="AB854" s="6" t="n"/>
+      <c r="AC854" s="6" t="n"/>
+      <c r="AD854" s="6" t="n"/>
+      <c r="AE854" s="6" t="n">
+        <v>51.58</v>
+      </c>
+      <c r="AF854" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="855">
+      <c r="A855" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B855" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C855" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D855" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E855" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F855" s="4" t="n"/>
+      <c r="G855" s="4" t="n"/>
+      <c r="H855" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I855" s="4" t="inlineStr"/>
+      <c r="J855" s="4" t="inlineStr"/>
+      <c r="K855" s="4" t="inlineStr"/>
+      <c r="L855" s="4" t="n"/>
+      <c r="M855" s="4" t="n"/>
+      <c r="N855" s="4" t="n"/>
+      <c r="O855" s="4" t="n"/>
+      <c r="P855" s="4" t="n"/>
+      <c r="Q855" s="4" t="n"/>
+      <c r="R855" s="4" t="n"/>
+      <c r="S855" s="4" t="n"/>
+      <c r="T855" s="4" t="n"/>
+      <c r="U855" s="4" t="n"/>
+      <c r="V855" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W855" s="4" t="inlineStr"/>
+      <c r="X855" s="4" t="n"/>
+      <c r="Y855" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z855" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA855" s="4" t="n"/>
+      <c r="AB855" s="4" t="n"/>
+      <c r="AC855" s="4" t="n"/>
+      <c r="AD855" s="4" t="n"/>
+      <c r="AE855" s="4" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="AF855" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="856">
+      <c r="A856" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B856" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C856" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D856" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E856" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F856" s="6" t="n"/>
+      <c r="G856" s="6" t="n"/>
+      <c r="H856" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I856" s="6" t="inlineStr"/>
+      <c r="J856" s="6" t="inlineStr"/>
+      <c r="K856" s="6" t="inlineStr"/>
+      <c r="L856" s="6" t="n"/>
+      <c r="M856" s="6" t="n"/>
+      <c r="N856" s="6" t="n"/>
+      <c r="O856" s="6" t="n"/>
+      <c r="P856" s="6" t="n"/>
+      <c r="Q856" s="6" t="n"/>
+      <c r="R856" s="6" t="n"/>
+      <c r="S856" s="6" t="n"/>
+      <c r="T856" s="6" t="n"/>
+      <c r="U856" s="6" t="n"/>
+      <c r="V856" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W856" s="6" t="inlineStr"/>
+      <c r="X856" s="6" t="n"/>
+      <c r="Y856" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z856" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA856" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB856" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC856" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD856" s="6" t="n"/>
+      <c r="AE856" s="6" t="n"/>
+      <c r="AF856" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="857">
+      <c r="A857" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B857" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C857" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D857" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E857" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F857" s="4" t="n"/>
+      <c r="G857" s="4" t="n"/>
+      <c r="H857" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I857" s="4" t="inlineStr"/>
+      <c r="J857" s="4" t="inlineStr"/>
+      <c r="K857" s="4" t="inlineStr"/>
+      <c r="L857" s="4" t="n"/>
+      <c r="M857" s="4" t="n"/>
+      <c r="N857" s="4" t="n"/>
+      <c r="O857" s="4" t="n"/>
+      <c r="P857" s="4" t="n"/>
+      <c r="Q857" s="4" t="n"/>
+      <c r="R857" s="4" t="n"/>
+      <c r="S857" s="4" t="n"/>
+      <c r="T857" s="4" t="n"/>
+      <c r="U857" s="4" t="n"/>
+      <c r="V857" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W857" s="4" t="inlineStr"/>
+      <c r="X857" s="4" t="n"/>
+      <c r="Y857" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z857" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA857" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB857" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC857" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD857" s="4" t="n"/>
+      <c r="AE857" s="4" t="n"/>
+      <c r="AF857" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="858">
+      <c r="A858" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B858" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C858" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D858" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E858" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F858" s="6" t="n"/>
+      <c r="G858" s="6" t="n"/>
+      <c r="H858" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I858" s="6" t="inlineStr"/>
+      <c r="J858" s="6" t="inlineStr"/>
+      <c r="K858" s="6" t="inlineStr"/>
+      <c r="L858" s="6" t="n"/>
+      <c r="M858" s="6" t="n"/>
+      <c r="N858" s="6" t="n"/>
+      <c r="O858" s="6" t="n"/>
+      <c r="P858" s="6" t="n"/>
+      <c r="Q858" s="6" t="n"/>
+      <c r="R858" s="6" t="n"/>
+      <c r="S858" s="6" t="n"/>
+      <c r="T858" s="6" t="n"/>
+      <c r="U858" s="6" t="n"/>
+      <c r="V858" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W858" s="6" t="inlineStr"/>
+      <c r="X858" s="6" t="n"/>
+      <c r="Y858" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z858" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA858" s="6" t="n"/>
+      <c r="AB858" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC858" s="6" t="n"/>
+      <c r="AD858" s="6" t="n"/>
+      <c r="AE858" s="6" t="n"/>
+      <c r="AF858" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="859">
+      <c r="A859" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B859" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C859" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D859" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E859" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F859" s="4" t="n"/>
+      <c r="G859" s="4" t="n"/>
+      <c r="H859" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I859" s="4" t="inlineStr"/>
+      <c r="J859" s="4" t="inlineStr"/>
+      <c r="K859" s="4" t="inlineStr"/>
+      <c r="L859" s="4" t="n"/>
+      <c r="M859" s="4" t="n"/>
+      <c r="N859" s="4" t="n"/>
+      <c r="O859" s="4" t="n"/>
+      <c r="P859" s="4" t="n"/>
+      <c r="Q859" s="4" t="n"/>
+      <c r="R859" s="4" t="n"/>
+      <c r="S859" s="4" t="n"/>
+      <c r="T859" s="4" t="n"/>
+      <c r="U859" s="4" t="n"/>
+      <c r="V859" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W859" s="4" t="inlineStr"/>
+      <c r="X859" s="4" t="n"/>
+      <c r="Y859" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z859" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA859" s="4" t="n"/>
+      <c r="AB859" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC859" s="4" t="n"/>
+      <c r="AD859" s="4" t="n"/>
+      <c r="AE859" s="4" t="n"/>
+      <c r="AF859" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Daily price update — 2026-07-13
</commit_message>
<xml_diff>
--- a/myprotein_prices.xlsx
+++ b/myprotein_prices.xlsx
@@ -467,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AF859"/>
+  <dimension ref="A1:AF894"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -68126,6 +68126,2754 @@
         <v>1</v>
       </c>
     </row>
+    <row r="860">
+      <c r="A860" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B860" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C860" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D860" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E860" s="4" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="F860" s="4" t="n"/>
+      <c r="G860" s="4" t="n"/>
+      <c r="H860" s="4" t="n">
+        <v>45.56</v>
+      </c>
+      <c r="I860" s="4" t="inlineStr"/>
+      <c r="J860" s="4" t="inlineStr"/>
+      <c r="K860" s="4" t="inlineStr"/>
+      <c r="L860" s="4" t="n">
+        <v>63.28</v>
+      </c>
+      <c r="M860" s="4" t="n">
+        <v>1.898</v>
+      </c>
+      <c r="N860" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O860" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P860" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q860" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R860" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S860" s="4" t="n"/>
+      <c r="T860" s="4" t="n"/>
+      <c r="U860" s="4" t="n"/>
+      <c r="V860" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W860" s="4" t="inlineStr"/>
+      <c r="X860" s="4" t="n"/>
+      <c r="Y860" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z860" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA860" s="4" t="n"/>
+      <c r="AB860" s="4" t="n"/>
+      <c r="AC860" s="4" t="n"/>
+      <c r="AD860" s="4" t="n"/>
+      <c r="AE860" s="4" t="n"/>
+      <c r="AF860" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="861">
+      <c r="A861" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B861" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C861" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D861" s="6" t="inlineStr">
+        <is>
+          <t>345g</t>
+        </is>
+      </c>
+      <c r="E861" s="6" t="n">
+        <v>16.19</v>
+      </c>
+      <c r="F861" s="6" t="n"/>
+      <c r="G861" s="6" t="n"/>
+      <c r="H861" s="6" t="n">
+        <v>46.93</v>
+      </c>
+      <c r="I861" s="6" t="inlineStr"/>
+      <c r="J861" s="6" t="inlineStr"/>
+      <c r="K861" s="6" t="inlineStr"/>
+      <c r="L861" s="6" t="n">
+        <v>65.18000000000001</v>
+      </c>
+      <c r="M861" s="6" t="n">
+        <v>1.955</v>
+      </c>
+      <c r="N861" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O861" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P861" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q861" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R861" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S861" s="6" t="n"/>
+      <c r="T861" s="6" t="n"/>
+      <c r="U861" s="6" t="n"/>
+      <c r="V861" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W861" s="6" t="inlineStr"/>
+      <c r="X861" s="6" t="n"/>
+      <c r="Y861" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z861" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA861" s="6" t="n"/>
+      <c r="AB861" s="6" t="n"/>
+      <c r="AC861" s="6" t="n"/>
+      <c r="AD861" s="6" t="n"/>
+      <c r="AE861" s="6" t="n"/>
+      <c r="AF861" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="862">
+      <c r="A862" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B862" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C862" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D862" s="4" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E862" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F862" s="4" t="n"/>
+      <c r="G862" s="4" t="n"/>
+      <c r="H862" s="4" t="n">
+        <v>35.98</v>
+      </c>
+      <c r="I862" s="4" t="inlineStr"/>
+      <c r="J862" s="4" t="inlineStr"/>
+      <c r="K862" s="4" t="inlineStr"/>
+      <c r="L862" s="4" t="n">
+        <v>49.97</v>
+      </c>
+      <c r="M862" s="4" t="n">
+        <v>1.499</v>
+      </c>
+      <c r="N862" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O862" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P862" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q862" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R862" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S862" s="4" t="n"/>
+      <c r="T862" s="4" t="n"/>
+      <c r="U862" s="4" t="n"/>
+      <c r="V862" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W862" s="4" t="inlineStr"/>
+      <c r="X862" s="4" t="n"/>
+      <c r="Y862" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z862" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA862" s="4" t="n"/>
+      <c r="AB862" s="4" t="n"/>
+      <c r="AC862" s="4" t="n"/>
+      <c r="AD862" s="4" t="n"/>
+      <c r="AE862" s="4" t="n"/>
+      <c r="AF862" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="863">
+      <c r="A863" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B863" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C863" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D863" s="6" t="inlineStr">
+        <is>
+          <t>750g</t>
+        </is>
+      </c>
+      <c r="E863" s="6" t="n">
+        <v>26.39</v>
+      </c>
+      <c r="F863" s="6" t="n"/>
+      <c r="G863" s="6" t="n"/>
+      <c r="H863" s="6" t="n">
+        <v>35.19</v>
+      </c>
+      <c r="I863" s="6" t="inlineStr"/>
+      <c r="J863" s="6" t="inlineStr"/>
+      <c r="K863" s="6" t="inlineStr"/>
+      <c r="L863" s="6" t="n">
+        <v>48.88</v>
+      </c>
+      <c r="M863" s="6" t="n">
+        <v>1.466</v>
+      </c>
+      <c r="N863" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O863" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P863" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q863" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R863" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S863" s="6" t="n"/>
+      <c r="T863" s="6" t="n"/>
+      <c r="U863" s="6" t="n"/>
+      <c r="V863" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W863" s="6" t="inlineStr"/>
+      <c r="X863" s="6" t="n"/>
+      <c r="Y863" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z863" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA863" s="6" t="n"/>
+      <c r="AB863" s="6" t="n"/>
+      <c r="AC863" s="6" t="n"/>
+      <c r="AD863" s="6" t="n"/>
+      <c r="AE863" s="6" t="n"/>
+      <c r="AF863" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="864">
+      <c r="A864" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B864" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C864" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D864" s="4" t="inlineStr">
+        <is>
+          <t>960g</t>
+        </is>
+      </c>
+      <c r="E864" s="4" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F864" s="4" t="n"/>
+      <c r="G864" s="4" t="n"/>
+      <c r="H864" s="4" t="n">
+        <v>32.49</v>
+      </c>
+      <c r="I864" s="4" t="inlineStr"/>
+      <c r="J864" s="4" t="inlineStr"/>
+      <c r="K864" s="4" t="inlineStr"/>
+      <c r="L864" s="4" t="n">
+        <v>45.13</v>
+      </c>
+      <c r="M864" s="4" t="n">
+        <v>1.354</v>
+      </c>
+      <c r="N864" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O864" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P864" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q864" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R864" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S864" s="4" t="n"/>
+      <c r="T864" s="4" t="n"/>
+      <c r="U864" s="4" t="n"/>
+      <c r="V864" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W864" s="4" t="inlineStr"/>
+      <c r="X864" s="4" t="n"/>
+      <c r="Y864" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z864" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA864" s="4" t="n"/>
+      <c r="AB864" s="4" t="n"/>
+      <c r="AC864" s="4" t="n"/>
+      <c r="AD864" s="4" t="n"/>
+      <c r="AE864" s="4" t="n"/>
+      <c r="AF864" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="865">
+      <c r="A865" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B865" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C865" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D865" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E865" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="F865" s="6" t="n"/>
+      <c r="G865" s="6" t="n"/>
+      <c r="H865" s="6" t="n">
+        <v>31.19</v>
+      </c>
+      <c r="I865" s="6" t="inlineStr"/>
+      <c r="J865" s="6" t="inlineStr"/>
+      <c r="K865" s="6" t="inlineStr"/>
+      <c r="L865" s="6" t="n">
+        <v>43.32</v>
+      </c>
+      <c r="M865" s="6" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="N865" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O865" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P865" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q865" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R865" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S865" s="6" t="n"/>
+      <c r="T865" s="6" t="n"/>
+      <c r="U865" s="6" t="n"/>
+      <c r="V865" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W865" s="6" t="inlineStr"/>
+      <c r="X865" s="6" t="n"/>
+      <c r="Y865" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z865" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA865" s="6" t="n"/>
+      <c r="AB865" s="6" t="n"/>
+      <c r="AC865" s="6" t="n"/>
+      <c r="AD865" s="6" t="n"/>
+      <c r="AE865" s="6" t="n"/>
+      <c r="AF865" s="6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="866">
+      <c r="A866" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B866" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C866" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D866" s="4" t="inlineStr">
+        <is>
+          <t>1.9kg</t>
+        </is>
+      </c>
+      <c r="E866" s="4" t="n">
+        <v>59.99</v>
+      </c>
+      <c r="F866" s="4" t="n"/>
+      <c r="G866" s="4" t="n"/>
+      <c r="H866" s="4" t="n">
+        <v>31.24</v>
+      </c>
+      <c r="I866" s="4" t="inlineStr"/>
+      <c r="J866" s="4" t="inlineStr"/>
+      <c r="K866" s="4" t="inlineStr"/>
+      <c r="L866" s="4" t="n">
+        <v>43.39</v>
+      </c>
+      <c r="M866" s="4" t="n">
+        <v>1.302</v>
+      </c>
+      <c r="N866" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O866" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P866" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q866" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R866" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S866" s="4" t="n"/>
+      <c r="T866" s="4" t="n"/>
+      <c r="U866" s="4" t="n"/>
+      <c r="V866" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W866" s="4" t="inlineStr"/>
+      <c r="X866" s="4" t="n"/>
+      <c r="Y866" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z866" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA866" s="4" t="n"/>
+      <c r="AB866" s="4" t="n"/>
+      <c r="AC866" s="4" t="n"/>
+      <c r="AD866" s="4" t="n"/>
+      <c r="AE866" s="4" t="n"/>
+      <c r="AF866" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B867" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C867" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D867" s="6" t="inlineStr">
+        <is>
+          <t>2.1kg</t>
+        </is>
+      </c>
+      <c r="E867" s="6" t="n">
+        <v>73.79000000000001</v>
+      </c>
+      <c r="F867" s="6" t="n"/>
+      <c r="G867" s="6" t="n"/>
+      <c r="H867" s="6" t="n">
+        <v>35.65</v>
+      </c>
+      <c r="I867" s="6" t="inlineStr"/>
+      <c r="J867" s="6" t="inlineStr"/>
+      <c r="K867" s="6" t="inlineStr"/>
+      <c r="L867" s="6" t="n">
+        <v>49.51</v>
+      </c>
+      <c r="M867" s="6" t="n">
+        <v>1.485</v>
+      </c>
+      <c r="N867" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O867" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P867" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q867" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R867" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S867" s="6" t="n"/>
+      <c r="T867" s="6" t="n"/>
+      <c r="U867" s="6" t="n"/>
+      <c r="V867" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W867" s="6" t="inlineStr"/>
+      <c r="X867" s="6" t="n"/>
+      <c r="Y867" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z867" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA867" s="6" t="n"/>
+      <c r="AB867" s="6" t="n"/>
+      <c r="AC867" s="6" t="n"/>
+      <c r="AD867" s="6" t="n"/>
+      <c r="AE867" s="6" t="n"/>
+      <c r="AF867" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="868">
+      <c r="A868" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B868" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C868" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D868" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E868" s="4" t="n">
+        <v>74.98999999999999</v>
+      </c>
+      <c r="F868" s="4" t="n"/>
+      <c r="G868" s="4" t="n"/>
+      <c r="H868" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="I868" s="4" t="inlineStr"/>
+      <c r="J868" s="4" t="inlineStr"/>
+      <c r="K868" s="4" t="inlineStr"/>
+      <c r="L868" s="4" t="n">
+        <v>41.67</v>
+      </c>
+      <c r="M868" s="4" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="N868" s="4" t="n">
+        <v>72</v>
+      </c>
+      <c r="O868" s="4" t="n">
+        <v>379</v>
+      </c>
+      <c r="P868" s="4" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q868" s="4" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R868" s="4" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S868" s="4" t="n"/>
+      <c r="T868" s="4" t="n"/>
+      <c r="U868" s="4" t="n"/>
+      <c r="V868" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W868" s="4" t="inlineStr"/>
+      <c r="X868" s="4" t="n"/>
+      <c r="Y868" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z868" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA868" s="4" t="n"/>
+      <c r="AB868" s="4" t="n"/>
+      <c r="AC868" s="4" t="n"/>
+      <c r="AD868" s="4" t="n"/>
+      <c r="AE868" s="4" t="n"/>
+      <c r="AF868" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="869">
+      <c r="A869" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B869" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Protein</t>
+        </is>
+      </c>
+      <c r="C869" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-protein/10530943/</t>
+        </is>
+      </c>
+      <c r="D869" s="6" t="inlineStr">
+        <is>
+          <t>3.6kg</t>
+        </is>
+      </c>
+      <c r="E869" s="6" t="n">
+        <v>118.19</v>
+      </c>
+      <c r="F869" s="6" t="n"/>
+      <c r="G869" s="6" t="n"/>
+      <c r="H869" s="6" t="n">
+        <v>32.83</v>
+      </c>
+      <c r="I869" s="6" t="inlineStr"/>
+      <c r="J869" s="6" t="inlineStr"/>
+      <c r="K869" s="6" t="inlineStr"/>
+      <c r="L869" s="6" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="M869" s="6" t="n">
+        <v>1.368</v>
+      </c>
+      <c r="N869" s="6" t="n">
+        <v>72</v>
+      </c>
+      <c r="O869" s="6" t="n">
+        <v>379</v>
+      </c>
+      <c r="P869" s="6" t="n">
+        <v>8.9</v>
+      </c>
+      <c r="Q869" s="6" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="R869" s="6" t="n">
+        <v>0.44</v>
+      </c>
+      <c r="S869" s="6" t="n"/>
+      <c r="T869" s="6" t="n"/>
+      <c r="U869" s="6" t="n"/>
+      <c r="V869" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Concentré de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants : lécithine de Soja, lécithine de tournesol), arôme, édulcorant (sucralose). Les allergènes apparaissent en gras dans la liste des ingrédients. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W869" s="6" t="inlineStr"/>
+      <c r="X869" s="6" t="n"/>
+      <c r="Y869" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z869" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA869" s="6" t="n"/>
+      <c r="AB869" s="6" t="n"/>
+      <c r="AC869" s="6" t="n"/>
+      <c r="AD869" s="6" t="n"/>
+      <c r="AE869" s="6" t="n"/>
+      <c r="AF869" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="870">
+      <c r="A870" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B870" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C870" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D870" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E870" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F870" s="4" t="n"/>
+      <c r="G870" s="4" t="n"/>
+      <c r="H870" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I870" s="4" t="inlineStr"/>
+      <c r="J870" s="4" t="inlineStr"/>
+      <c r="K870" s="4" t="inlineStr"/>
+      <c r="L870" s="4" t="n">
+        <v>93.78</v>
+      </c>
+      <c r="M870" s="4" t="n">
+        <v>2.813</v>
+      </c>
+      <c r="N870" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O870" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P870" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q870" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R870" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S870" s="4" t="n"/>
+      <c r="T870" s="4" t="n"/>
+      <c r="U870" s="4" t="n"/>
+      <c r="V870" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W870" s="4" t="inlineStr"/>
+      <c r="X870" s="4" t="n"/>
+      <c r="Y870" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z870" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA870" s="4" t="n"/>
+      <c r="AB870" s="4" t="n"/>
+      <c r="AC870" s="4" t="n"/>
+      <c r="AD870" s="4" t="n"/>
+      <c r="AE870" s="4" t="n"/>
+      <c r="AF870" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="871">
+      <c r="A871" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B871" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C871" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D871" s="6" t="inlineStr">
+        <is>
+          <t>600g</t>
+        </is>
+      </c>
+      <c r="E871" s="6" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F871" s="6" t="n"/>
+      <c r="G871" s="6" t="n"/>
+      <c r="H871" s="6" t="n">
+        <v>114.98</v>
+      </c>
+      <c r="I871" s="6" t="inlineStr"/>
+      <c r="J871" s="6" t="inlineStr"/>
+      <c r="K871" s="6" t="inlineStr"/>
+      <c r="L871" s="6" t="n">
+        <v>140.22</v>
+      </c>
+      <c r="M871" s="6" t="n">
+        <v>4.207</v>
+      </c>
+      <c r="N871" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O871" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P871" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q871" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R871" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S871" s="6" t="n"/>
+      <c r="T871" s="6" t="n"/>
+      <c r="U871" s="6" t="n"/>
+      <c r="V871" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W871" s="6" t="inlineStr"/>
+      <c r="X871" s="6" t="n"/>
+      <c r="Y871" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z871" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA871" s="6" t="n"/>
+      <c r="AB871" s="6" t="n"/>
+      <c r="AC871" s="6" t="n"/>
+      <c r="AD871" s="6" t="n"/>
+      <c r="AE871" s="6" t="n"/>
+      <c r="AF871" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="872">
+      <c r="A872" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B872" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C872" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D872" s="4" t="inlineStr">
+        <is>
+          <t>780g</t>
+        </is>
+      </c>
+      <c r="E872" s="4" t="n">
+        <v>47.99</v>
+      </c>
+      <c r="F872" s="4" t="n"/>
+      <c r="G872" s="4" t="n"/>
+      <c r="H872" s="4" t="n">
+        <v>61.53</v>
+      </c>
+      <c r="I872" s="4" t="inlineStr"/>
+      <c r="J872" s="4" t="inlineStr"/>
+      <c r="K872" s="4" t="inlineStr"/>
+      <c r="L872" s="4" t="n">
+        <v>75.04000000000001</v>
+      </c>
+      <c r="M872" s="4" t="n">
+        <v>2.251</v>
+      </c>
+      <c r="N872" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O872" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P872" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q872" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R872" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S872" s="4" t="n"/>
+      <c r="T872" s="4" t="n"/>
+      <c r="U872" s="4" t="n"/>
+      <c r="V872" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W872" s="4" t="inlineStr"/>
+      <c r="X872" s="4" t="n"/>
+      <c r="Y872" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z872" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA872" s="4" t="n"/>
+      <c r="AB872" s="4" t="n"/>
+      <c r="AC872" s="4" t="n"/>
+      <c r="AD872" s="4" t="n"/>
+      <c r="AE872" s="4" t="n"/>
+      <c r="AF872" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="873">
+      <c r="A873" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B873" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C873" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D873" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E873" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="F873" s="6" t="n"/>
+      <c r="G873" s="6" t="n"/>
+      <c r="H873" s="6" t="n">
+        <v>56.49</v>
+      </c>
+      <c r="I873" s="6" t="inlineStr"/>
+      <c r="J873" s="6" t="inlineStr"/>
+      <c r="K873" s="6" t="inlineStr"/>
+      <c r="L873" s="6" t="n">
+        <v>68.89</v>
+      </c>
+      <c r="M873" s="6" t="n">
+        <v>2.067</v>
+      </c>
+      <c r="N873" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O873" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P873" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q873" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R873" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S873" s="6" t="n"/>
+      <c r="T873" s="6" t="n"/>
+      <c r="U873" s="6" t="n"/>
+      <c r="V873" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W873" s="6" t="inlineStr"/>
+      <c r="X873" s="6" t="n"/>
+      <c r="Y873" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z873" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA873" s="6" t="n"/>
+      <c r="AB873" s="6" t="n"/>
+      <c r="AC873" s="6" t="n"/>
+      <c r="AD873" s="6" t="n"/>
+      <c r="AE873" s="6" t="n"/>
+      <c r="AF873" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="874">
+      <c r="A874" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B874" s="3" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C874" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D874" s="4" t="inlineStr">
+        <is>
+          <t>2.7kg</t>
+        </is>
+      </c>
+      <c r="E874" s="4" t="n">
+        <v>133.99</v>
+      </c>
+      <c r="F874" s="4" t="n"/>
+      <c r="G874" s="4" t="n"/>
+      <c r="H874" s="4" t="n">
+        <v>49.63</v>
+      </c>
+      <c r="I874" s="4" t="inlineStr"/>
+      <c r="J874" s="4" t="inlineStr"/>
+      <c r="K874" s="4" t="inlineStr"/>
+      <c r="L874" s="4" t="n">
+        <v>60.52</v>
+      </c>
+      <c r="M874" s="4" t="n">
+        <v>1.816</v>
+      </c>
+      <c r="N874" s="4" t="n">
+        <v>82</v>
+      </c>
+      <c r="O874" s="4" t="n">
+        <v>361</v>
+      </c>
+      <c r="P874" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q874" s="4" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R874" s="4" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S874" s="4" t="n"/>
+      <c r="T874" s="4" t="n"/>
+      <c r="U874" s="4" t="n"/>
+      <c r="V874" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W874" s="4" t="inlineStr"/>
+      <c r="X874" s="4" t="n"/>
+      <c r="Y874" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z874" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA874" s="4" t="n"/>
+      <c r="AB874" s="4" t="n"/>
+      <c r="AC874" s="4" t="n"/>
+      <c r="AD874" s="4" t="n"/>
+      <c r="AE874" s="4" t="n"/>
+      <c r="AF874" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="875">
+      <c r="A875" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B875" s="5" t="inlineStr">
+        <is>
+          <t>Impact Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C875" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-whey-isolate/10530911/</t>
+        </is>
+      </c>
+      <c r="D875" s="6" t="inlineStr">
+        <is>
+          <t>4.2kg</t>
+        </is>
+      </c>
+      <c r="E875" s="6" t="n">
+        <v>214.99</v>
+      </c>
+      <c r="F875" s="6" t="n"/>
+      <c r="G875" s="6" t="n"/>
+      <c r="H875" s="6" t="n">
+        <v>51.19</v>
+      </c>
+      <c r="I875" s="6" t="inlineStr"/>
+      <c r="J875" s="6" t="inlineStr"/>
+      <c r="K875" s="6" t="inlineStr"/>
+      <c r="L875" s="6" t="n">
+        <v>62.43</v>
+      </c>
+      <c r="M875" s="6" t="n">
+        <v>1.873</v>
+      </c>
+      <c r="N875" s="6" t="n">
+        <v>82</v>
+      </c>
+      <c r="O875" s="6" t="n">
+        <v>361</v>
+      </c>
+      <c r="P875" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="Q875" s="6" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="R875" s="6" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="S875" s="6" t="n"/>
+      <c r="T875" s="6" t="n"/>
+      <c r="U875" s="6" t="n"/>
+      <c r="V875" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum (Lait) (96 %) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Arôme, Édulcorant (Sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W875" s="6" t="inlineStr"/>
+      <c r="X875" s="6" t="n"/>
+      <c r="Y875" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z875" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA875" s="6" t="n"/>
+      <c r="AB875" s="6" t="n"/>
+      <c r="AC875" s="6" t="n"/>
+      <c r="AD875" s="6" t="n"/>
+      <c r="AE875" s="6" t="n"/>
+      <c r="AF875" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="876">
+      <c r="A876" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B876" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C876" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D876" s="4" t="inlineStr">
+        <is>
+          <t>390g</t>
+        </is>
+      </c>
+      <c r="E876" s="4" t="n">
+        <v>29.99</v>
+      </c>
+      <c r="F876" s="4" t="n"/>
+      <c r="G876" s="4" t="n"/>
+      <c r="H876" s="4" t="n">
+        <v>76.90000000000001</v>
+      </c>
+      <c r="I876" s="4" t="inlineStr"/>
+      <c r="J876" s="4" t="inlineStr"/>
+      <c r="K876" s="4" t="inlineStr"/>
+      <c r="L876" s="4" t="n">
+        <v>97.34</v>
+      </c>
+      <c r="M876" s="4" t="n">
+        <v>2.92</v>
+      </c>
+      <c r="N876" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O876" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P876" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q876" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R876" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S876" s="4" t="n"/>
+      <c r="T876" s="4" t="n"/>
+      <c r="U876" s="4" t="n"/>
+      <c r="V876" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W876" s="4" t="inlineStr"/>
+      <c r="X876" s="4" t="n"/>
+      <c r="Y876" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z876" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA876" s="4" t="n"/>
+      <c r="AB876" s="4" t="n"/>
+      <c r="AC876" s="4" t="n"/>
+      <c r="AD876" s="4" t="n"/>
+      <c r="AE876" s="4" t="n"/>
+      <c r="AF876" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="877">
+      <c r="A877" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B877" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C877" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D877" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E877" s="6" t="n">
+        <v>28.19</v>
+      </c>
+      <c r="F877" s="6" t="n"/>
+      <c r="G877" s="6" t="n"/>
+      <c r="H877" s="6" t="n">
+        <v>56.38</v>
+      </c>
+      <c r="I877" s="6" t="inlineStr"/>
+      <c r="J877" s="6" t="inlineStr"/>
+      <c r="K877" s="6" t="inlineStr"/>
+      <c r="L877" s="6" t="n">
+        <v>71.37</v>
+      </c>
+      <c r="M877" s="6" t="n">
+        <v>2.141</v>
+      </c>
+      <c r="N877" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O877" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P877" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q877" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R877" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S877" s="6" t="n"/>
+      <c r="T877" s="6" t="n"/>
+      <c r="U877" s="6" t="n"/>
+      <c r="V877" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W877" s="6" t="inlineStr"/>
+      <c r="X877" s="6" t="n"/>
+      <c r="Y877" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z877" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA877" s="6" t="n"/>
+      <c r="AB877" s="6" t="n"/>
+      <c r="AC877" s="6" t="n"/>
+      <c r="AD877" s="6" t="n"/>
+      <c r="AE877" s="6" t="n"/>
+      <c r="AF877" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="878">
+      <c r="A878" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B878" s="3" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C878" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D878" s="4" t="inlineStr">
+        <is>
+          <t>875g</t>
+        </is>
+      </c>
+      <c r="E878" s="4" t="n">
+        <v>54.99</v>
+      </c>
+      <c r="F878" s="4" t="n"/>
+      <c r="G878" s="4" t="n"/>
+      <c r="H878" s="4" t="n">
+        <v>62.85</v>
+      </c>
+      <c r="I878" s="4" t="inlineStr"/>
+      <c r="J878" s="4" t="inlineStr"/>
+      <c r="K878" s="4" t="inlineStr"/>
+      <c r="L878" s="4" t="n">
+        <v>79.56</v>
+      </c>
+      <c r="M878" s="4" t="n">
+        <v>2.387</v>
+      </c>
+      <c r="N878" s="4" t="n">
+        <v>79</v>
+      </c>
+      <c r="O878" s="4" t="n">
+        <v>331</v>
+      </c>
+      <c r="P878" s="4" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q878" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R878" s="4" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S878" s="4" t="n"/>
+      <c r="T878" s="4" t="n"/>
+      <c r="U878" s="4" t="n"/>
+      <c r="V878" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W878" s="4" t="inlineStr"/>
+      <c r="X878" s="4" t="n"/>
+      <c r="Y878" s="4" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z878" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA878" s="4" t="n"/>
+      <c r="AB878" s="4" t="n"/>
+      <c r="AC878" s="4" t="n"/>
+      <c r="AD878" s="4" t="n"/>
+      <c r="AE878" s="4" t="n"/>
+      <c r="AF878" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="879">
+      <c r="A879" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B879" s="5" t="inlineStr">
+        <is>
+          <t>Clear Whey Isolate</t>
+        </is>
+      </c>
+      <c r="C879" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/clear-whey-isolate/12081395/</t>
+        </is>
+      </c>
+      <c r="D879" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E879" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="F879" s="6" t="n"/>
+      <c r="G879" s="6" t="n"/>
+      <c r="H879" s="6" t="n">
+        <v>50.39</v>
+      </c>
+      <c r="I879" s="6" t="inlineStr"/>
+      <c r="J879" s="6" t="inlineStr"/>
+      <c r="K879" s="6" t="inlineStr"/>
+      <c r="L879" s="6" t="n">
+        <v>63.78</v>
+      </c>
+      <c r="M879" s="6" t="n">
+        <v>1.913</v>
+      </c>
+      <c r="N879" s="6" t="n">
+        <v>79</v>
+      </c>
+      <c r="O879" s="6" t="n">
+        <v>331</v>
+      </c>
+      <c r="P879" s="6" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="Q879" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R879" s="6" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="S879" s="6" t="n"/>
+      <c r="T879" s="6" t="n"/>
+      <c r="U879" s="6" t="n"/>
+      <c r="V879" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Isolat de protéines de lactosérum hydrolysé (Lait) (93 %) (contient un agent antimousse (dioxyde de silicium), huile de colza), arômes naturels, acidifiant (acide citrique), colorant (rouge de betterave), édulcorant (sucralose). Pour les allergènes, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W879" s="6" t="inlineStr"/>
+      <c r="X879" s="6" t="n"/>
+      <c r="Y879" s="6" t="inlineStr">
+        <is>
+          <t>Whey</t>
+        </is>
+      </c>
+      <c r="Z879" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA879" s="6" t="n"/>
+      <c r="AB879" s="6" t="n"/>
+      <c r="AC879" s="6" t="n"/>
+      <c r="AD879" s="6" t="n"/>
+      <c r="AE879" s="6" t="n"/>
+      <c r="AF879" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="880">
+      <c r="A880" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B880" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C880" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D880" s="4" t="inlineStr">
+        <is>
+          <t>420g</t>
+        </is>
+      </c>
+      <c r="E880" s="4" t="n">
+        <v>14.49</v>
+      </c>
+      <c r="F880" s="4" t="n"/>
+      <c r="G880" s="4" t="n"/>
+      <c r="H880" s="4" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="I880" s="4" t="inlineStr"/>
+      <c r="J880" s="4" t="inlineStr"/>
+      <c r="K880" s="4" t="inlineStr"/>
+      <c r="L880" s="4" t="n">
+        <v>58.47</v>
+      </c>
+      <c r="M880" s="4" t="n">
+        <v>1.754</v>
+      </c>
+      <c r="N880" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O880" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P880" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q880" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R880" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S880" s="4" t="n"/>
+      <c r="T880" s="4" t="n"/>
+      <c r="U880" s="4" t="n"/>
+      <c r="V880" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W880" s="4" t="inlineStr"/>
+      <c r="X880" s="4" t="n"/>
+      <c r="Y880" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z880" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA880" s="4" t="n"/>
+      <c r="AB880" s="4" t="n"/>
+      <c r="AC880" s="4" t="n"/>
+      <c r="AD880" s="4" t="n"/>
+      <c r="AE880" s="4" t="n"/>
+      <c r="AF880" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="881">
+      <c r="A881" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B881" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C881" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D881" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E881" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="F881" s="6" t="n"/>
+      <c r="G881" s="6" t="n"/>
+      <c r="H881" s="6" t="n">
+        <v>30.49</v>
+      </c>
+      <c r="I881" s="6" t="inlineStr"/>
+      <c r="J881" s="6" t="inlineStr"/>
+      <c r="K881" s="6" t="inlineStr"/>
+      <c r="L881" s="6" t="n">
+        <v>51.68</v>
+      </c>
+      <c r="M881" s="6" t="n">
+        <v>1.55</v>
+      </c>
+      <c r="N881" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O881" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P881" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q881" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R881" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S881" s="6" t="n"/>
+      <c r="T881" s="6" t="n"/>
+      <c r="U881" s="6" t="n"/>
+      <c r="V881" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W881" s="6" t="inlineStr"/>
+      <c r="X881" s="6" t="n"/>
+      <c r="Y881" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z881" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA881" s="6" t="n"/>
+      <c r="AB881" s="6" t="n"/>
+      <c r="AC881" s="6" t="n"/>
+      <c r="AD881" s="6" t="n"/>
+      <c r="AE881" s="6" t="n"/>
+      <c r="AF881" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="882">
+      <c r="A882" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B882" s="3" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C882" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D882" s="4" t="inlineStr">
+        <is>
+          <t>2.5kg</t>
+        </is>
+      </c>
+      <c r="E882" s="4" t="n">
+        <v>68.98999999999999</v>
+      </c>
+      <c r="F882" s="4" t="n"/>
+      <c r="G882" s="4" t="n"/>
+      <c r="H882" s="4" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="I882" s="4" t="inlineStr"/>
+      <c r="J882" s="4" t="inlineStr"/>
+      <c r="K882" s="4" t="inlineStr"/>
+      <c r="L882" s="4" t="n">
+        <v>46.78</v>
+      </c>
+      <c r="M882" s="4" t="n">
+        <v>1.403</v>
+      </c>
+      <c r="N882" s="4" t="n">
+        <v>59</v>
+      </c>
+      <c r="O882" s="4" t="n">
+        <v>359</v>
+      </c>
+      <c r="P882" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q882" s="4" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R882" s="4" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S882" s="4" t="n"/>
+      <c r="T882" s="4" t="n"/>
+      <c r="U882" s="4" t="n"/>
+      <c r="V882" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W882" s="4" t="inlineStr"/>
+      <c r="X882" s="4" t="n"/>
+      <c r="Y882" s="4" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z882" s="4" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA882" s="4" t="n"/>
+      <c r="AB882" s="4" t="n"/>
+      <c r="AC882" s="4" t="n"/>
+      <c r="AD882" s="4" t="n"/>
+      <c r="AE882" s="4" t="n"/>
+      <c r="AF882" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="883">
+      <c r="A883" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B883" s="5" t="inlineStr">
+        <is>
+          <t>Impact Diet Whey</t>
+        </is>
+      </c>
+      <c r="C883" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/impact-diet-whey/10530657/</t>
+        </is>
+      </c>
+      <c r="D883" s="6" t="inlineStr">
+        <is>
+          <t>5kg</t>
+        </is>
+      </c>
+      <c r="E883" s="6" t="n">
+        <v>128.99</v>
+      </c>
+      <c r="F883" s="6" t="n"/>
+      <c r="G883" s="6" t="n"/>
+      <c r="H883" s="6" t="n">
+        <v>25.8</v>
+      </c>
+      <c r="I883" s="6" t="inlineStr"/>
+      <c r="J883" s="6" t="inlineStr"/>
+      <c r="K883" s="6" t="inlineStr"/>
+      <c r="L883" s="6" t="n">
+        <v>43.73</v>
+      </c>
+      <c r="M883" s="6" t="n">
+        <v>1.312</v>
+      </c>
+      <c r="N883" s="6" t="n">
+        <v>59</v>
+      </c>
+      <c r="O883" s="6" t="n">
+        <v>359</v>
+      </c>
+      <c r="P883" s="6" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q883" s="6" t="n">
+        <v>6.1</v>
+      </c>
+      <c r="R883" s="6" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="S883" s="6" t="n"/>
+      <c r="T883" s="6" t="n"/>
+      <c r="U883" s="6" t="n"/>
+      <c r="V883" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Mélange de protéines (76 %) (Concentré de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol)), Lait Concentré de protéines de lait, Isolat de protéines de lactosérum (Lait) (contient des émulsifiants (Lécithine de Soja, Lécithine de tournesol))), Farine d'Avoine (8 %), Inuline (8 %), Arôme,L-Glutamine, Poudre de graines de lin (2 %), Préparation CLA (Triglycéride d'acide linoléique conjugué (Huile de carthame), Solides de sirop de maïs, Protéines de Lait, Stabilisant (Phosphate dipotassique), Anti-agglomérant (Dioxyde de silicium), Antioxydant (Tocophérols mixtes)), Extrait de thé vert (Camellia sinensis), Bitartrate de choline, Épaississant (Gomme xanthane), Édulcorant (Sucralose), Complexe enzymatique DigeZyme™ (0,1 %) (Alpha-amylase, Lactase, Cellulase, Protéase, Lipase). Pour les allergènes, y compris les céréales contenant du gluten, voir les ingrédients en gras. Convient aux végétariens.</t>
+        </is>
+      </c>
+      <c r="W883" s="6" t="inlineStr"/>
+      <c r="X883" s="6" t="n"/>
+      <c r="Y883" s="6" t="inlineStr">
+        <is>
+          <t>Aliments enrichis</t>
+        </is>
+      </c>
+      <c r="Z883" s="6" t="inlineStr">
+        <is>
+          <t>whey</t>
+        </is>
+      </c>
+      <c r="AA883" s="6" t="n"/>
+      <c r="AB883" s="6" t="n"/>
+      <c r="AC883" s="6" t="n"/>
+      <c r="AD883" s="6" t="n"/>
+      <c r="AE883" s="6" t="n"/>
+      <c r="AF883" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="884">
+      <c r="A884" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B884" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C884" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D884" s="4" t="inlineStr">
+        <is>
+          <t>100g</t>
+        </is>
+      </c>
+      <c r="E884" s="4" t="n">
+        <v>4.39</v>
+      </c>
+      <c r="F884" s="4" t="n"/>
+      <c r="G884" s="4" t="n"/>
+      <c r="H884" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="I884" s="4" t="inlineStr"/>
+      <c r="J884" s="4" t="inlineStr"/>
+      <c r="K884" s="4" t="inlineStr"/>
+      <c r="L884" s="4" t="n"/>
+      <c r="M884" s="4" t="n"/>
+      <c r="N884" s="4" t="n"/>
+      <c r="O884" s="4" t="n"/>
+      <c r="P884" s="4" t="n"/>
+      <c r="Q884" s="4" t="n"/>
+      <c r="R884" s="4" t="n"/>
+      <c r="S884" s="4" t="n"/>
+      <c r="T884" s="4" t="n"/>
+      <c r="U884" s="4" t="n"/>
+      <c r="V884" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W884" s="4" t="inlineStr"/>
+      <c r="X884" s="4" t="n"/>
+      <c r="Y884" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z884" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA884" s="4" t="n"/>
+      <c r="AB884" s="4" t="n"/>
+      <c r="AC884" s="4" t="n"/>
+      <c r="AD884" s="4" t="n"/>
+      <c r="AE884" s="4" t="n">
+        <v>43.9</v>
+      </c>
+      <c r="AF884" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="885">
+      <c r="A885" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B885" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C885" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D885" s="6" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E885" s="6" t="n">
+        <v>8.24</v>
+      </c>
+      <c r="F885" s="6" t="n"/>
+      <c r="G885" s="6" t="n"/>
+      <c r="H885" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="I885" s="6" t="inlineStr"/>
+      <c r="J885" s="6" t="inlineStr"/>
+      <c r="K885" s="6" t="inlineStr"/>
+      <c r="L885" s="6" t="n"/>
+      <c r="M885" s="6" t="n"/>
+      <c r="N885" s="6" t="n"/>
+      <c r="O885" s="6" t="n"/>
+      <c r="P885" s="6" t="n"/>
+      <c r="Q885" s="6" t="n"/>
+      <c r="R885" s="6" t="n"/>
+      <c r="S885" s="6" t="n"/>
+      <c r="T885" s="6" t="n"/>
+      <c r="U885" s="6" t="n"/>
+      <c r="V885" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W885" s="6" t="inlineStr"/>
+      <c r="X885" s="6" t="n"/>
+      <c r="Y885" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z885" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA885" s="6" t="n"/>
+      <c r="AB885" s="6" t="n"/>
+      <c r="AC885" s="6" t="n"/>
+      <c r="AD885" s="6" t="n"/>
+      <c r="AE885" s="6" t="n">
+        <v>32.96</v>
+      </c>
+      <c r="AF885" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="886">
+      <c r="A886" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B886" s="3" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C886" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D886" s="4" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E886" s="4" t="n">
+        <v>13.74</v>
+      </c>
+      <c r="F886" s="4" t="n"/>
+      <c r="G886" s="4" t="n"/>
+      <c r="H886" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="I886" s="4" t="inlineStr"/>
+      <c r="J886" s="4" t="inlineStr"/>
+      <c r="K886" s="4" t="inlineStr"/>
+      <c r="L886" s="4" t="n"/>
+      <c r="M886" s="4" t="n"/>
+      <c r="N886" s="4" t="n"/>
+      <c r="O886" s="4" t="n"/>
+      <c r="P886" s="4" t="n"/>
+      <c r="Q886" s="4" t="n"/>
+      <c r="R886" s="4" t="n"/>
+      <c r="S886" s="4" t="n"/>
+      <c r="T886" s="4" t="n"/>
+      <c r="U886" s="4" t="n"/>
+      <c r="V886" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W886" s="4" t="inlineStr"/>
+      <c r="X886" s="4" t="n"/>
+      <c r="Y886" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z886" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA886" s="4" t="n"/>
+      <c r="AB886" s="4" t="n"/>
+      <c r="AC886" s="4" t="n"/>
+      <c r="AD886" s="4" t="n"/>
+      <c r="AE886" s="4" t="n">
+        <v>27.48</v>
+      </c>
+      <c r="AF886" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="887">
+      <c r="A887" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B887" s="5" t="inlineStr">
+        <is>
+          <t>Créatine Monohydrate en poudre</t>
+        </is>
+      </c>
+      <c r="C887" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/creatine-monohydrate-en-poudre/10530050/</t>
+        </is>
+      </c>
+      <c r="D887" s="6" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E887" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="F887" s="6" t="n"/>
+      <c r="G887" s="6" t="n"/>
+      <c r="H887" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="I887" s="6" t="inlineStr"/>
+      <c r="J887" s="6" t="inlineStr"/>
+      <c r="K887" s="6" t="inlineStr"/>
+      <c r="L887" s="6" t="n"/>
+      <c r="M887" s="6" t="n"/>
+      <c r="N887" s="6" t="n"/>
+      <c r="O887" s="6" t="n"/>
+      <c r="P887" s="6" t="n"/>
+      <c r="Q887" s="6" t="n"/>
+      <c r="R887" s="6" t="n"/>
+      <c r="S887" s="6" t="n"/>
+      <c r="T887" s="6" t="n"/>
+      <c r="U887" s="6" t="n"/>
+      <c r="V887" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Créatine monohydrate. Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W887" s="6" t="inlineStr"/>
+      <c r="X887" s="6" t="n"/>
+      <c r="Y887" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z887" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA887" s="6" t="n"/>
+      <c r="AB887" s="6" t="n"/>
+      <c r="AC887" s="6" t="n"/>
+      <c r="AD887" s="6" t="n"/>
+      <c r="AE887" s="6" t="n">
+        <v>25.29</v>
+      </c>
+      <c r="AF887" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="888">
+      <c r="A888" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B888" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C888" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D888" s="4" t="inlineStr">
+        <is>
+          <t>250g</t>
+        </is>
+      </c>
+      <c r="E888" s="4" t="n">
+        <v>15.94</v>
+      </c>
+      <c r="F888" s="4" t="n"/>
+      <c r="G888" s="4" t="n"/>
+      <c r="H888" s="4" t="n">
+        <v>63.76</v>
+      </c>
+      <c r="I888" s="4" t="inlineStr"/>
+      <c r="J888" s="4" t="inlineStr"/>
+      <c r="K888" s="4" t="inlineStr"/>
+      <c r="L888" s="4" t="n"/>
+      <c r="M888" s="4" t="n"/>
+      <c r="N888" s="4" t="n"/>
+      <c r="O888" s="4" t="n"/>
+      <c r="P888" s="4" t="n"/>
+      <c r="Q888" s="4" t="n"/>
+      <c r="R888" s="4" t="n"/>
+      <c r="S888" s="4" t="n"/>
+      <c r="T888" s="4" t="n"/>
+      <c r="U888" s="4" t="n"/>
+      <c r="V888" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W888" s="4" t="inlineStr"/>
+      <c r="X888" s="4" t="n"/>
+      <c r="Y888" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z888" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA888" s="4" t="n"/>
+      <c r="AB888" s="4" t="n"/>
+      <c r="AC888" s="4" t="n"/>
+      <c r="AD888" s="4" t="n"/>
+      <c r="AE888" s="4" t="n">
+        <v>63.76</v>
+      </c>
+      <c r="AF888" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="889">
+      <c r="A889" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B889" s="5" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C889" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D889" s="6" t="inlineStr">
+        <is>
+          <t>500g</t>
+        </is>
+      </c>
+      <c r="E889" s="6" t="n">
+        <v>23.64</v>
+      </c>
+      <c r="F889" s="6" t="n"/>
+      <c r="G889" s="6" t="n"/>
+      <c r="H889" s="6" t="n">
+        <v>47.28</v>
+      </c>
+      <c r="I889" s="6" t="inlineStr"/>
+      <c r="J889" s="6" t="inlineStr"/>
+      <c r="K889" s="6" t="inlineStr"/>
+      <c r="L889" s="6" t="n"/>
+      <c r="M889" s="6" t="n"/>
+      <c r="N889" s="6" t="n"/>
+      <c r="O889" s="6" t="n"/>
+      <c r="P889" s="6" t="n"/>
+      <c r="Q889" s="6" t="n"/>
+      <c r="R889" s="6" t="n"/>
+      <c r="S889" s="6" t="n"/>
+      <c r="T889" s="6" t="n"/>
+      <c r="U889" s="6" t="n"/>
+      <c r="V889" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W889" s="6" t="inlineStr"/>
+      <c r="X889" s="6" t="n"/>
+      <c r="Y889" s="6" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z889" s="6" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA889" s="6" t="n"/>
+      <c r="AB889" s="6" t="n"/>
+      <c r="AC889" s="6" t="n"/>
+      <c r="AD889" s="6" t="n"/>
+      <c r="AE889" s="6" t="n">
+        <v>47.28</v>
+      </c>
+      <c r="AF889" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="890">
+      <c r="A890" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B890" s="3" t="inlineStr">
+        <is>
+          <t>THE Creatine Creapure®</t>
+        </is>
+      </c>
+      <c r="C890" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/the-creatine-creapure/10529740/</t>
+        </is>
+      </c>
+      <c r="D890" s="4" t="inlineStr">
+        <is>
+          <t>1kg</t>
+        </is>
+      </c>
+      <c r="E890" s="4" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="F890" s="4" t="n"/>
+      <c r="G890" s="4" t="n"/>
+      <c r="H890" s="4" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="I890" s="4" t="inlineStr"/>
+      <c r="J890" s="4" t="inlineStr"/>
+      <c r="K890" s="4" t="inlineStr"/>
+      <c r="L890" s="4" t="n"/>
+      <c r="M890" s="4" t="n"/>
+      <c r="N890" s="4" t="n"/>
+      <c r="O890" s="4" t="n"/>
+      <c r="P890" s="4" t="n"/>
+      <c r="Q890" s="4" t="n"/>
+      <c r="R890" s="4" t="n"/>
+      <c r="S890" s="4" t="n"/>
+      <c r="T890" s="4" t="n"/>
+      <c r="U890" s="4" t="n"/>
+      <c r="V890" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Creapure® (Monohydrate de Créatine). Produit dans une usine qui traite également du lait. Convient aux végétariens et aux végétaliens.</t>
+        </is>
+      </c>
+      <c r="W890" s="4" t="inlineStr"/>
+      <c r="X890" s="4" t="n"/>
+      <c r="Y890" s="4" t="inlineStr">
+        <is>
+          <t>Créatine</t>
+        </is>
+      </c>
+      <c r="Z890" s="4" t="inlineStr">
+        <is>
+          <t>creatine</t>
+        </is>
+      </c>
+      <c r="AA890" s="4" t="n"/>
+      <c r="AB890" s="4" t="n"/>
+      <c r="AC890" s="4" t="n"/>
+      <c r="AD890" s="4" t="n"/>
+      <c r="AE890" s="4" t="n">
+        <v>46.19</v>
+      </c>
+      <c r="AF890" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="891">
+      <c r="A891" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B891" s="5" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C891" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D891" s="6" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E891" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F891" s="6" t="n"/>
+      <c r="G891" s="6" t="n"/>
+      <c r="H891" s="6" t="n">
+        <v>99.89</v>
+      </c>
+      <c r="I891" s="6" t="inlineStr"/>
+      <c r="J891" s="6" t="inlineStr"/>
+      <c r="K891" s="6" t="inlineStr"/>
+      <c r="L891" s="6" t="n"/>
+      <c r="M891" s="6" t="n"/>
+      <c r="N891" s="6" t="n"/>
+      <c r="O891" s="6" t="n"/>
+      <c r="P891" s="6" t="n"/>
+      <c r="Q891" s="6" t="n"/>
+      <c r="R891" s="6" t="n"/>
+      <c r="S891" s="6" t="n"/>
+      <c r="T891" s="6" t="n"/>
+      <c r="U891" s="6" t="n"/>
+      <c r="V891" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W891" s="6" t="inlineStr"/>
+      <c r="X891" s="6" t="n"/>
+      <c r="Y891" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z891" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA891" s="6" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB891" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC891" s="6" t="n">
+        <v>0.333</v>
+      </c>
+      <c r="AD891" s="6" t="n"/>
+      <c r="AE891" s="6" t="n"/>
+      <c r="AF891" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="892">
+      <c r="A892" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B892" s="3" t="inlineStr">
+        <is>
+          <t>Oméga 3 en gélules</t>
+        </is>
+      </c>
+      <c r="C892" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omega-3-en-gelules/10529329/</t>
+        </is>
+      </c>
+      <c r="D892" s="4" t="inlineStr">
+        <is>
+          <t>250 gélules</t>
+        </is>
+      </c>
+      <c r="E892" s="4" t="n">
+        <v>21.59</v>
+      </c>
+      <c r="F892" s="4" t="n"/>
+      <c r="G892" s="4" t="n"/>
+      <c r="H892" s="4" t="n">
+        <v>86.36</v>
+      </c>
+      <c r="I892" s="4" t="inlineStr"/>
+      <c r="J892" s="4" t="inlineStr"/>
+      <c r="K892" s="4" t="inlineStr"/>
+      <c r="L892" s="4" t="n"/>
+      <c r="M892" s="4" t="n"/>
+      <c r="N892" s="4" t="n"/>
+      <c r="O892" s="4" t="n"/>
+      <c r="P892" s="4" t="n"/>
+      <c r="Q892" s="4" t="n"/>
+      <c r="R892" s="4" t="n"/>
+      <c r="S892" s="4" t="n"/>
+      <c r="T892" s="4" t="n"/>
+      <c r="U892" s="4" t="n"/>
+      <c r="V892" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Ingrédients :  Huile de Poisson Oméga 3, Enveloppe de capsule molle (Gélatine de bœuf, Humectant (Glycérol)), Antioxydant (D-Alpha-Tocophérol), Huile de Soja raffinée. Peut contenir du Lait. Pour les allergènes, voir les ingrédients en gras.</t>
+        </is>
+      </c>
+      <c r="W892" s="4" t="inlineStr"/>
+      <c r="X892" s="4" t="n"/>
+      <c r="Y892" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z892" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA892" s="4" t="n">
+        <v>180</v>
+      </c>
+      <c r="AB892" s="4" t="n">
+        <v>120</v>
+      </c>
+      <c r="AC892" s="4" t="n">
+        <v>0.288</v>
+      </c>
+      <c r="AD892" s="4" t="n"/>
+      <c r="AE892" s="4" t="n"/>
+      <c r="AF892" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="893">
+      <c r="A893" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B893" s="5" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C893" s="5" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D893" s="6" t="inlineStr">
+        <is>
+          <t>30 gélules</t>
+        </is>
+      </c>
+      <c r="E893" s="6" t="n">
+        <v>8.99</v>
+      </c>
+      <c r="F893" s="6" t="n"/>
+      <c r="G893" s="6" t="n"/>
+      <c r="H893" s="6" t="n">
+        <v>299.67</v>
+      </c>
+      <c r="I893" s="6" t="inlineStr"/>
+      <c r="J893" s="6" t="inlineStr"/>
+      <c r="K893" s="6" t="inlineStr"/>
+      <c r="L893" s="6" t="n"/>
+      <c r="M893" s="6" t="n"/>
+      <c r="N893" s="6" t="n"/>
+      <c r="O893" s="6" t="n"/>
+      <c r="P893" s="6" t="n"/>
+      <c r="Q893" s="6" t="n"/>
+      <c r="R893" s="6" t="n"/>
+      <c r="S893" s="6" t="n"/>
+      <c r="T893" s="6" t="n"/>
+      <c r="U893" s="6" t="n"/>
+      <c r="V893" s="6" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W893" s="6" t="inlineStr"/>
+      <c r="X893" s="6" t="n"/>
+      <c r="Y893" s="6" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z893" s="6" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA893" s="6" t="n"/>
+      <c r="AB893" s="6" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC893" s="6" t="n"/>
+      <c r="AD893" s="6" t="n"/>
+      <c r="AE893" s="6" t="n"/>
+      <c r="AF893" s="6" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="894">
+      <c r="A894" s="2" t="inlineStr">
+        <is>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B894" s="3" t="inlineStr">
+        <is>
+          <t>Omégas 3 végans</t>
+        </is>
+      </c>
+      <c r="C894" s="3" t="inlineStr">
+        <is>
+          <t>https://fr.myprotein.com/p/nutrition-sportive/omegas-3-vegans/13633515/</t>
+        </is>
+      </c>
+      <c r="D894" s="4" t="inlineStr">
+        <is>
+          <t>90 gélules</t>
+        </is>
+      </c>
+      <c r="E894" s="4" t="n">
+        <v>20.99</v>
+      </c>
+      <c r="F894" s="4" t="n"/>
+      <c r="G894" s="4" t="n"/>
+      <c r="H894" s="4" t="n">
+        <v>233.22</v>
+      </c>
+      <c r="I894" s="4" t="inlineStr"/>
+      <c r="J894" s="4" t="inlineStr"/>
+      <c r="K894" s="4" t="inlineStr"/>
+      <c r="L894" s="4" t="n"/>
+      <c r="M894" s="4" t="n"/>
+      <c r="N894" s="4" t="n"/>
+      <c r="O894" s="4" t="n"/>
+      <c r="P894" s="4" t="n"/>
+      <c r="Q894" s="4" t="n"/>
+      <c r="R894" s="4" t="n"/>
+      <c r="S894" s="4" t="n"/>
+      <c r="T894" s="4" t="n"/>
+      <c r="U894" s="4" t="n"/>
+      <c r="V894" s="4" t="inlineStr">
+        <is>
+          <t>Ingrédients          Acide docosahexaénoïque (DHA) d’huile d’algue, enrobage de la gélule (humectant [glycérine], excipient [amidon de maïs modifié], agent gélifiant [carraghénane], eau purifiée), vitamine E.
+ALLERGÈNES : produit dans des locaux utilisant également du lait.</t>
+        </is>
+      </c>
+      <c r="W894" s="4" t="inlineStr"/>
+      <c r="X894" s="4" t="n"/>
+      <c r="Y894" s="4" t="inlineStr">
+        <is>
+          <t>Oméga-3</t>
+        </is>
+      </c>
+      <c r="Z894" s="4" t="inlineStr">
+        <is>
+          <t>omega3</t>
+        </is>
+      </c>
+      <c r="AA894" s="4" t="n"/>
+      <c r="AB894" s="4" t="n">
+        <v>200</v>
+      </c>
+      <c r="AC894" s="4" t="n"/>
+      <c r="AD894" s="4" t="n"/>
+      <c r="AE894" s="4" t="n"/>
+      <c r="AF894" s="4" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>